<commit_message>
feat: add partial merkle proofs
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R03b4480c90b64c26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rf310b02b50944232"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R744ddc267e714a60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rf032e3c970834dd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rbe0df3dfb6314a9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rb50c7d72308744fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R505909f446d94c19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R6b3bf393f4f54143"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R8da1e66c62e846ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R31d1a3d6cc3e4209"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R342d9c1f9dda49d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R7c3aafb98ce1445e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -722,10 +722,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="N15" s="32" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="O15" s="32" t="str">
-        <x:v>Already heavily reused in current nodes, so chapter titles are containers. Best current value is prerequisite ladders and bridge concepts. Implemented from this source in the current branch: protocol.light-client-trust-model, ops.full-node-vs-lightweight-wallet, custody.coin-selection, protocol.change-outputs, protocol.bech32m-addresses, protocol.script-execution-stack, dev.extended-keys, and protocol.witness-structure.</x:v>
+        <x:v>Already heavily reused in current nodes, so chapter titles are containers. Best current value is prerequisite ladders and bridge concepts. Implemented from this source in the current branch: protocol.light-client-trust-model, ops.full-node-vs-lightweight-wallet, custody.coin-selection, protocol.change-outputs, protocol.bech32m-addresses, protocol.script-execution-stack, dev.extended-keys, protocol.witness-structure, and protocol.partial-merkle-proofs.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -5089,16 +5089,67 @@
         <x:v>Implemented as the missing transaction-level SegWit bridge. Existing TXID/WTXID and witness-commitment nodes remain unchanged until a separate prerequisite-cleanup pass evaluates whether they should consume this node.</x:v>
       </x:c>
     </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="32" t="str">
+        <x:v>protocol.partial-merkle-proofs</x:v>
+      </x:c>
+      <x:c r="B82" s="32" t="str">
+        <x:v>Partial Merkle Proofs</x:v>
+      </x:c>
+      <x:c r="C82" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D82" s="32" t="str">
+        <x:v>source.mastering-bitcoin-book-map</x:v>
+      </x:c>
+      <x:c r="E82" s="32" t="str">
+        <x:v>https://github.com/bitcoinbook/bitcoinbook/blob/develop/ch11_blockchain.adoc</x:v>
+      </x:c>
+      <x:c r="F82" s="32" t="str">
+        <x:v>The Blockchain &gt; Merkle Trees and Lightweight Clients</x:v>
+      </x:c>
+      <x:c r="G82" s="32" t="str"/>
+      <x:c r="H82" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I82" s="32" t="str">
+        <x:v>This is one specific client-verification mechanism: sending only the relevant Merkle branches and traversal bits needed to prove a transaction belongs to a block. It is narrower than Merkle trees, block structure, and the broader light-client trust model, and distinct from compact block filters.</x:v>
+      </x:c>
+      <x:c r="J82" s="32" t="str">
+        <x:v>fundamentals.merkle-trees, protocol.block-structure, protocol.light-client-trust-model</x:v>
+      </x:c>
+      <x:c r="K82" s="32" t="str">
+        <x:v>protocol.block-structure</x:v>
+      </x:c>
+      <x:c r="L82" s="32" t="str">
+        <x:v>Block structure supplies the Merkle-root context and already inherits the generic Merkle-tree concept. The light-client trust model is a downstream interpretation of what this proof can and cannot verify, so making it a direct prerequisite would reverse the mechanism-to-tradeoff relationship.</x:v>
+      </x:c>
+      <x:c r="M82" s="32" t="str">
+        <x:v>partial merkle trees, SPV proofs, merkleblock proofs</x:v>
+      </x:c>
+      <x:c r="N82" s="32" t="str">
+        <x:v>spv, light-clients, merkle-proofs</x:v>
+      </x:c>
+      <x:c r="O82" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P82" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q82" s="32" t="str">
+        <x:v>Implemented as the missing legacy-SPV proof mechanism between block structure and the existing light-client trust model. Compact block filters remain a distinct modern client-sync approach rather than a duplicate.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H81">
+    <x:dataValidation type="list" sqref="H12:H82">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P81">
+    <x:dataValidation type="list" sqref="P12:P82">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -6981,16 +7032,39 @@
         <x:v>Direct edge keeps the node at the transaction-format layer; TXID/WTXID and witness-commitment consequences remain downstream concepts.</x:v>
       </x:c>
     </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="32" t="str">
+        <x:v>protocol.block-structure</x:v>
+      </x:c>
+      <x:c r="B91" s="32" t="str">
+        <x:v>protocol.partial-merkle-proofs</x:v>
+      </x:c>
+      <x:c r="C91" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D91" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E91" s="32" t="str">
+        <x:v>Partial Merkle proofs reconstruct a transaction's inclusion path against the Merkle root carried by a block, so learners need block composition and root placement first.</x:v>
+      </x:c>
+      <x:c r="F91" s="32" t="str">
+        <x:v>source.mastering-bitcoin-book-map</x:v>
+      </x:c>
+      <x:c r="G91" s="32" t="str">
+        <x:v>The block-structure parent already inherits fundamentals.merkle-trees, avoiding a redundant direct edge.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C90">
+    <x:dataValidation type="list" sqref="C12:C91">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D90">
+    <x:dataValidation type="list" sqref="D12:D91">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -8932,16 +9006,42 @@
         <x:v>Added with only protocol.segregated-witness as a direct prerequisite. Relative timelocks, SIGHASH flags, compact block filters, coinbase transactions, and difficulty adjustment were reviewed as existing coverage and not cloned.</x:v>
       </x:c>
     </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="32" t="str">
+        <x:v>decision.partial-merkle-proofs-slice</x:v>
+      </x:c>
+      <x:c r="B84" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C84" s="32" t="str">
+        <x:v>protocol.partial-merkle-proofs</x:v>
+      </x:c>
+      <x:c r="D84" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E84" s="32" t="str">
+        <x:v>Mastering Bitcoin's lightweight-client chapter exposes a concrete partial-proof mechanism that is absent from the graph. It survives dedupe because generic Merkle trees explain the primitive, block structure explains the committed root, compact block filters describe a different modern sync protocol, and the light-client trust model explains the resulting guarantees rather than the proof construction itself.</x:v>
+      </x:c>
+      <x:c r="F84" s="32" t="str">
+        <x:v>protocol.partial-merkle-proofs, fundamentals.merkle-trees, protocol.block-structure, protocol.compact-block-filters, protocol.light-client-trust-model</x:v>
+      </x:c>
+      <x:c r="G84" s="32" t="str">
+        <x:v>source.mastering-bitcoin-book-map</x:v>
+      </x:c>
+      <x:c r="H84" s="32" t="str">
+        <x:v>Added with only protocol.block-structure as a direct prerequisite; the inherited Merkle-tree edge remains transitive and the trust-model relationship remains downstream.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B83">
+    <x:dataValidation type="list" sqref="B12:B84">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D83">
+    <x:dataValidation type="list" sqref="D12:D84">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -8994,7 +9094,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.08753568287</x:v>
+        <x:v>46213.09137787037</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -9018,7 +9118,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -9026,7 +9126,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>79</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -9050,7 +9150,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add bitcoin development review culture
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R505909f446d94c19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R6b3bf393f4f54143"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R8da1e66c62e846ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R31d1a3d6cc3e4209"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R342d9c1f9dda49d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R7c3aafb98ce1445e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Ref21c357f7b64c52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rc287d9828d9a42fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R25221017d2b24720"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R94bbf183a1244774"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R792f2101b3394148"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Racf28269054b4433"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -675,10 +675,10 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="N14" s="32" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="O14" s="32" t="str">
-        <x:v>Heavy overlap with existing philosophy nodes, but strong for bridge concepts like validation sovereignty and consensus vs policy. Implemented from this source in the current branch: fundamentals.validation-sovereignty, protocol.consensus-vs-policy, and protocol.chain-split-risk.</x:v>
+        <x:v>Heavy overlap with existing philosophy nodes, but strong for bridge concepts like validation sovereignty, consensus vs policy, and development review. Implemented from this source in the current branch: fundamentals.validation-sovereignty, protocol.consensus-vs-policy, protocol.chain-split-risk, and dev.review-culture.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -5140,16 +5140,67 @@
         <x:v>Implemented as the missing legacy-SPV proof mechanism between block structure and the existing light-client trust model. Compact block filters remain a distinct modern client-sync approach rather than a duplicate.</x:v>
       </x:c>
     </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="32" t="str">
+        <x:v>dev.review-culture</x:v>
+      </x:c>
+      <x:c r="B83" s="32" t="str">
+        <x:v>Review Culture in Bitcoin Development</x:v>
+      </x:c>
+      <x:c r="C83" s="32" t="str">
+        <x:v>History &amp; Governance</x:v>
+      </x:c>
+      <x:c r="D83" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="E83" s="32" t="str">
+        <x:v>https://bitcoindevphilosophy.com/#review</x:v>
+      </x:c>
+      <x:c r="F83" s="32" t="str">
+        <x:v>Open Source chapter &gt; Review</x:v>
+      </x:c>
+      <x:c r="G83" s="32" t="str"/>
+      <x:c r="H83" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I83" s="32" t="str">
+        <x:v>This is one specific development-process concept: how independent review across proposal, implementation, deployment, and adoption stages reduces correctness, security, and compatibility risk. It is narrower than the BIPs process and distinct from general adversarial thinking, reproducible builds, and responsible disclosure.</x:v>
+      </x:c>
+      <x:c r="J83" s="32" t="str">
+        <x:v>dev.bips-process, security.adversarial-thinking, dev.reproducible-builds, security.responsible-disclosure</x:v>
+      </x:c>
+      <x:c r="K83" s="32" t="str">
+        <x:v>dev.bips-process, security.adversarial-thinking</x:v>
+      </x:c>
+      <x:c r="L83" s="32" t="str">
+        <x:v>The proposal process supplies the lifecycle in which review occurs, while adversarial thinking supplies the threat-driven review mindset. Reproducible builds and responsible disclosure are specialized downstream safeguards rather than prerequisites for understanding review culture itself.</x:v>
+      </x:c>
+      <x:c r="M83" s="32" t="str">
+        <x:v>Bitcoin development review, code review in Bitcoin</x:v>
+      </x:c>
+      <x:c r="N83" s="32" t="str">
+        <x:v>development, review, security</x:v>
+      </x:c>
+      <x:c r="O83" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P83" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q83" s="32" t="str">
+        <x:v>Implemented as a narrow Bitcoin-development review concept. Permissionless development remains deferred because it overlaps more heavily with neutrality, censorship resistance, and the BIPs process.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H82">
+    <x:dataValidation type="list" sqref="H12:H83">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P82">
+    <x:dataValidation type="list" sqref="P12:P83">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -7055,16 +7106,62 @@
         <x:v>The block-structure parent already inherits fundamentals.merkle-trees, avoiding a redundant direct edge.</x:v>
       </x:c>
     </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="32" t="str">
+        <x:v>dev.bips-process</x:v>
+      </x:c>
+      <x:c r="B92" s="32" t="str">
+        <x:v>dev.review-culture</x:v>
+      </x:c>
+      <x:c r="C92" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D92" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E92" s="32" t="str">
+        <x:v>Review culture is applied throughout the proposal and implementation lifecycle, so learners need to understand the process in which Bitcoin changes are proposed and evaluated.</x:v>
+      </x:c>
+      <x:c r="F92" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G92" s="32" t="str">
+        <x:v>Direct edge supplies the development-lifecycle context without adding downstream release or deployment details.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="32" t="str">
+        <x:v>security.adversarial-thinking</x:v>
+      </x:c>
+      <x:c r="B93" s="32" t="str">
+        <x:v>dev.review-culture</x:v>
+      </x:c>
+      <x:c r="C93" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D93" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E93" s="32" t="str">
+        <x:v>Independent review in Bitcoin is deliberately adversarial: reviewers look for correctness failures, attack paths, and compatibility hazards before changes are merged.</x:v>
+      </x:c>
+      <x:c r="F93" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G93" s="32" t="str">
+        <x:v>Direct edge keeps review distinct from responsible disclosure and reproducible-build verification, which are specialized downstream safeguards.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C91">
+    <x:dataValidation type="list" sqref="C12:C93">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D91">
+    <x:dataValidation type="list" sqref="D12:D93">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9032,16 +9129,42 @@
         <x:v>Added with only protocol.block-structure as a direct prerequisite; the inherited Merkle-tree edge remains transitive and the trust-model relationship remains downstream.</x:v>
       </x:c>
     </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="32" t="str">
+        <x:v>decision.review-culture-slice</x:v>
+      </x:c>
+      <x:c r="B85" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C85" s="32" t="str">
+        <x:v>dev.review-culture</x:v>
+      </x:c>
+      <x:c r="D85" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E85" s="32" t="str">
+        <x:v>Bitcoin Dev Philosophy's review section names a concrete safety practice that is absent from the graph: independent, adversarial review across multiple development stages. It survives dedupe because BIPs process describes the lifecycle, adversarial thinking describes the attacker mindset, reproducible builds verify artifacts, and responsible disclosure handles discovered vulnerabilities.</x:v>
+      </x:c>
+      <x:c r="F85" s="32" t="str">
+        <x:v>dev.review-culture, dev.bips-process, security.adversarial-thinking, dev.reproducible-builds, security.responsible-disclosure</x:v>
+      </x:c>
+      <x:c r="G85" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="H85" s="32" t="str">
+        <x:v>Added with only the proposal lifecycle and adversarial mindset as direct prerequisites. Permissionless development is deferred pending a narrower dedupe pass.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B84">
+    <x:dataValidation type="list" sqref="B12:B85">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D84">
+    <x:dataValidation type="list" sqref="D12:D85">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9094,7 +9217,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.09137787037</x:v>
+        <x:v>46213.09324214121</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -9118,7 +9241,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -9126,7 +9249,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>80</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -9150,7 +9273,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add lightning feature flags
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Ref21c357f7b64c52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rc287d9828d9a42fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R25221017d2b24720"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R94bbf183a1244774"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R792f2101b3394148"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Racf28269054b4433"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rb7e1513679f94c31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rcdd53396afd24a08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R4fd2181b1b5949ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R34b7278f6d4b4337"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Ra1c8387b4f234ae8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R3211e194f4414f33"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -871,72 +871,72 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="B19" s="32" t="str">
-        <x:v>Cypherpunk Library Bitcoin-Adjacent Canon</x:v>
+        <x:v>Lightning Network BOLTs</x:v>
       </x:c>
       <x:c r="C19" s="32" t="str">
-        <x:v>https://www.cypherpunkbooks.com/collection</x:v>
+        <x:v>https://github.com/lightning/bolts</x:v>
       </x:c>
       <x:c r="D19" s="32" t="str">
-        <x:v>essay-library</x:v>
+        <x:v>protocol-specification-repository</x:v>
       </x:c>
       <x:c r="E19" s="32" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="F19" s="32" t="str">
-        <x:v>Bitcoin-adjacent cypherpunk readings focused on privacy, electronic cash, monetary theory, and the ideological roots most likely to sharpen foundational and history nodes.</x:v>
+        <x:v>Canonical Lightning wire protocol, transport, channel, transaction, routing, discovery, feature-negotiation, invoice, and offer specifications.</x:v>
       </x:c>
       <x:c r="G19" s="32" t="str">
-        <x:v>Start with four clusters: cypherpunk manifestos, privacy and surveillance essays, eCash and digital-cash texts, and monetary-theory readings. Defer clearly non-Bitcoin-adjacent political or general-hacker texts unless they surface a direct graph gap.</x:v>
+        <x:v>Track each BOLT document as an enumeration cluster, starting with the index and BOLTs 01, 02, 04, 08, 09, and 10. Extract only atomic mechanisms and deduplicate against existing Lightning nodes before proposing additions.</x:v>
       </x:c>
       <x:c r="H19" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In review</x:v>
       </x:c>
       <x:c r="I19" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="J19" s="32" t="str">
-        <x:v>Queue exhausted</x:v>
+        <x:v>Raw extraction</x:v>
       </x:c>
       <x:c r="K19" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="L19" s="32" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="M19" s="32" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N19" s="32" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O19" s="32" t="str">
-        <x:v>Added from user direction. High-signal starting texts from the collection include A Cypherpunk's Manifesto, The Crypto Anarchist Manifesto, Your Secret Right to Cash, Protecting Privacy with Electronic Cash, The Beauty of eCash, The Cyphernomicon, Ideal Money and Asymptotically Ideal Money, and 21 Lessons. Implemented from this source in the current branch: history.chaumian-ecash, privacy.secret-right-to-cash, economics.ideal-money. Merged into existing coverage in the current branch: history.cypherpunks via A Cypherpunk's Manifesto; history.bitcoin-anarchism via The Crypto Anarchist Manifesto. Current tracked cluster queue is exhausted for this pass.</x:v>
+        <x:v>Added during source expansion. The first inventory covers the BOLT index plus messaging, peer protocol, onion messaging, encrypted transport, feature negotiation, and DNS bootstrap clusters. Implemented from this source in the current branch: lightning.feature-flags.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="B20" s="32" t="str">
-        <x:v>Bitcoin Dev Project Explained Posts</x:v>
+        <x:v>Cypherpunk Library Bitcoin-Adjacent Canon</x:v>
       </x:c>
       <x:c r="C20" s="32" t="str">
-        <x:v>https://x.com/search?q=from%3ABitcoin_Devs%20explained&amp;src=typed_query&amp;f=live</x:v>
+        <x:v>https://www.cypherpunkbooks.com/collection</x:v>
       </x:c>
       <x:c r="D20" s="32" t="str">
-        <x:v>social-post-cluster</x:v>
+        <x:v>essay-library</x:v>
       </x:c>
       <x:c r="E20" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F20" s="32" t="str">
-        <x:v>Short-form educational posts from @Bitcoin_Devs that explicitly explain protocol, wallet, and Lightning mechanisms in learner-facing language.</x:v>
+        <x:v>Bitcoin-adjacent cypherpunk readings focused on privacy, electronic cash, monetary theory, and the ideological roots most likely to sharpen foundational and history nodes.</x:v>
       </x:c>
       <x:c r="G20" s="32" t="str">
-        <x:v>Track the live X search as one source-family row first, then expand to one row per matching post once current results are enumerated. Group matching posts by concept family such as hashing, fee management, node architecture, channel mechanics, and upgrade proposals.</x:v>
+        <x:v>Start with four clusters: cypherpunk manifestos, privacy and surveillance essays, eCash and digital-cash texts, and monetary-theory readings. Defer clearly non-Bitcoin-adjacent political or general-hacker texts unless they surface a direct graph gap.</x:v>
       </x:c>
       <x:c r="H20" s="32" t="str">
         <x:v>Complete</x:v>
@@ -951,39 +951,39 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="L20" s="32" t="n">
-        <x:v>43</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M20" s="32" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N20" s="32" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O20" s="32" t="str">
-        <x:v>Added from user direction. The live X query was enumerated in the logged-in in-app browser on July 8, 2026 and surfaced 43 matching posts. Visible examples include Lamport Signature explained, Duplicate transaction bug explained, 64-byte transaction bug explained, SegWit Address explained, Off-by-one difficulty bug explained, Great Consensus Cleanup explained Part 1: Time Warp Attack, Transaction Pinning explained, Full Node Architecture Explained, MAST explained simply, BIP 158 explained, MuSig explained Simply, CPFP transaction explained, CISA explained, BIP-68 Explained, and Shamir's Secret Sharing explained. Implemented from this source in the current branch: protocol.time-warp-attack, protocol.duplicate-transaction-bug, protocol.64-byte-transaction-bug, fundamentals.lamport-signatures, custody.shamirs-secret-sharing. Merged into existing coverage in the current branch: protocol.time-warp-attack via Off-by-one difficulty bug explained. Current enumerated post queue is exhausted for this pass.</x:v>
+        <x:v>Added from user direction. High-signal starting texts from the collection include A Cypherpunk's Manifesto, The Crypto Anarchist Manifesto, Your Secret Right to Cash, Protecting Privacy with Electronic Cash, The Beauty of eCash, The Cyphernomicon, Ideal Money and Asymptotically Ideal Money, and 21 Lessons. Implemented from this source in the current branch: history.chaumian-ecash, privacy.secret-right-to-cash, economics.ideal-money. Merged into existing coverage in the current branch: history.cypherpunks via A Cypherpunk's Manifesto; history.bitcoin-anarchism via The Crypto Anarchist Manifesto. Current tracked cluster queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-wallet</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="B21" s="32" t="str">
-        <x:v>Bitcoin Core Academy Wallet Internals</x:v>
+        <x:v>Bitcoin Dev Project Explained Posts</x:v>
       </x:c>
       <x:c r="C21" s="32" t="str">
-        <x:v>https://bitcoincore.academy/scriptpubkeymanagers.html</x:v>
+        <x:v>https://x.com/search?q=from%3ABitcoin_Devs%20explained&amp;src=typed_query&amp;f=live</x:v>
       </x:c>
       <x:c r="D21" s="32" t="str">
-        <x:v>course-cluster</x:v>
+        <x:v>social-post-cluster</x:v>
       </x:c>
       <x:c r="E21" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F21" s="32" t="str">
-        <x:v>Wallet internals cluster around ScriptPubKeyManagers, wallet keys, transaction identification, and balance calculation.</x:v>
+        <x:v>Short-form educational posts from @Bitcoin_Devs that explicitly explain protocol, wallet, and Lightning mechanisms in learner-facing language.</x:v>
       </x:c>
       <x:c r="G21" s="32" t="str">
-        <x:v>Track one wallet-internals page cluster at a time so Core-specific abstractions stay atomic instead of collapsing into generic wallet concepts.</x:v>
+        <x:v>Track the live X search as one source-family row first, then expand to one row per matching post once current results are enumerated. Group matching posts by concept family such as hashing, fee management, node architecture, channel mechanics, and upgrade proposals.</x:v>
       </x:c>
       <x:c r="H21" s="32" t="str">
         <x:v>Complete</x:v>
@@ -998,27 +998,27 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="L21" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="M21" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="N21" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="O21" s="32" t="str">
-        <x:v>First additional-source pass beyond the mandatory seed list. The current additive winner is dev.scriptpubkeymanagers; wallet-encryption remains deferred because the cleanest surviving slice is still too coupled to missing Core wallet-internals parents. Current tracked wallet-internals queue is exhausted for this pass.</x:v>
+        <x:v>Added from user direction. The live X query was enumerated in the logged-in in-app browser on July 8, 2026 and surfaced 43 matching posts. Visible examples include Lamport Signature explained, Duplicate transaction bug explained, 64-byte transaction bug explained, SegWit Address explained, Off-by-one difficulty bug explained, Great Consensus Cleanup explained Part 1: Time Warp Attack, Transaction Pinning explained, Full Node Architecture Explained, MAST explained simply, BIP 158 explained, MuSig explained Simply, CPFP transaction explained, CISA explained, BIP-68 Explained, and Shamir's Secret Sharing explained. Implemented from this source in the current branch: protocol.time-warp-attack, protocol.duplicate-transaction-bug, protocol.64-byte-transaction-bug, fundamentals.lamport-signatures, custody.shamirs-secret-sharing. Merged into existing coverage in the current branch: protocol.time-warp-attack via Off-by-one difficulty bug explained. Current enumerated post queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-core-academy-wallet</x:v>
       </x:c>
       <x:c r="B22" s="32" t="str">
-        <x:v>Bitcoin Core Academy Mempool Mechanics</x:v>
+        <x:v>Bitcoin Core Academy Wallet Internals</x:v>
       </x:c>
       <x:c r="C22" s="32" t="str">
-        <x:v>https://bitcoincore.academy/mempool-unbroadcast.html</x:v>
+        <x:v>https://bitcoincore.academy/scriptpubkeymanagers.html</x:v>
       </x:c>
       <x:c r="D22" s="32" t="str">
         <x:v>course-cluster</x:v>
@@ -1027,10 +1027,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F22" s="32" t="str">
-        <x:v>Mempool and relay internals cluster around transaction relay, rebroadcast behavior, and local node transaction state.</x:v>
+        <x:v>Wallet internals cluster around ScriptPubKeyManagers, wallet keys, transaction identification, and balance calculation.</x:v>
       </x:c>
       <x:c r="G22" s="32" t="str">
-        <x:v>Track the academy mempool pages as a separate cluster so implementation-specific relay mechanisms are not collapsed into generic mempool coverage.</x:v>
+        <x:v>Track one wallet-internals page cluster at a time so Core-specific abstractions stay atomic instead of collapsing into generic wallet concepts.</x:v>
       </x:c>
       <x:c r="H22" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1051,33 +1051,33 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="N22" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O22" s="32" t="str">
-        <x:v>Second post-seed-source slice. The current additive winners are protocol.mempool-unbroadcast-set, protocol.transaction-rebroadcast-privacy, and protocol.txid-vs-wtxid. The remaining transaction-format internals are now mostly implementation-detail material rather than clean learner-facing nodes. Current tracked mempool queue is exhausted for this pass.</x:v>
+        <x:v>First additional-source pass beyond the mandatory seed list. The current additive winner is dev.scriptpubkeymanagers; wallet-encryption remains deferred because the cleanest surviving slice is still too coupled to missing Core wallet-internals parents. Current tracked wallet-internals queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32" t="str">
-        <x:v>source.bitcoin-design-payment-formats</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="B23" s="32" t="str">
-        <x:v>Bitcoin Design Payment Request Formats</x:v>
+        <x:v>Bitcoin Core Academy Mempool Mechanics</x:v>
       </x:c>
       <x:c r="C23" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/how-it-works/human-readable-addresses/</x:v>
+        <x:v>https://bitcoincore.academy/mempool-unbroadcast.html</x:v>
       </x:c>
       <x:c r="D23" s="32" t="str">
-        <x:v>guide-cluster</x:v>
+        <x:v>course-cluster</x:v>
       </x:c>
       <x:c r="E23" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F23" s="32" t="str">
-        <x:v>User-facing payment request and address-sharing concepts across human-readable addresses, transaction display, and wallet privacy tradeoffs.</x:v>
+        <x:v>Mempool and relay internals cluster around transaction relay, rebroadcast behavior, and local node transaction state.</x:v>
       </x:c>
       <x:c r="G23" s="32" t="str">
-        <x:v>Track design guide pages by UX concept cluster so user-facing payment abstractions stay separate from protocol internals and generic wallet hygiene.</x:v>
+        <x:v>Track the academy mempool pages as a separate cluster so implementation-specific relay mechanisms are not collapsed into generic mempool coverage.</x:v>
       </x:c>
       <x:c r="H23" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1098,21 +1098,21 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="N23" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O23" s="32" t="str">
-        <x:v>First Bitcoin Design implementation slice. The current additive winner is custody.human-readable-addresses; encrypted cloud backups remains the main deferred neighbor from this design source family. Current tracked payment-format queue is exhausted for this pass.</x:v>
+        <x:v>Second post-seed-source slice. The current additive winners are protocol.mempool-unbroadcast-set, protocol.transaction-rebroadcast-privacy, and protocol.txid-vs-wtxid. The remaining transaction-format internals are now mostly implementation-detail material rather than clean learner-facing nodes. Current tracked mempool queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoin-design-payment-formats</x:v>
       </x:c>
       <x:c r="B24" s="32" t="str">
-        <x:v>Bitcoin Design Wallet Activity Context</x:v>
+        <x:v>Bitcoin Design Payment Request Formats</x:v>
       </x:c>
       <x:c r="C24" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/daily-spending-wallet/activity/</x:v>
+        <x:v>https://bitcoin.design/guide/how-it-works/human-readable-addresses/</x:v>
       </x:c>
       <x:c r="D24" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1121,10 +1121,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F24" s="32" t="str">
-        <x:v>User-facing wallet activity, contacts, and contextual payment-history concepts that help learners distinguish on-chain events from wallet-added meaning.</x:v>
+        <x:v>User-facing payment request and address-sharing concepts across human-readable addresses, transaction display, and wallet privacy tradeoffs.</x:v>
       </x:c>
       <x:c r="G24" s="32" t="str">
-        <x:v>Track activity and contacts pages together so contextual metadata stays separate from backup flows and from protocol transaction mechanics.</x:v>
+        <x:v>Track design guide pages by UX concept cluster so user-facing payment abstractions stay separate from protocol internals and generic wallet hygiene.</x:v>
       </x:c>
       <x:c r="H24" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1139,27 +1139,27 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="L24" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="M24" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N24" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="O24" s="32" t="str">
-        <x:v>Second Bitcoin Design implementation slice. The current additive winner is custody.transaction-metadata; encrypted cloud backups remains the main deferred design-side candidate. Current tracked activity-and-contacts queue is exhausted for this pass.</x:v>
+        <x:v>First Bitcoin Design implementation slice. The current additive winner is custody.human-readable-addresses; encrypted cloud backups remains the main deferred neighbor from this design source family. Current tracked payment-format queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="str">
-        <x:v>source.bitcoin-design-multiple-wallets</x:v>
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="B25" s="32" t="str">
-        <x:v>Bitcoin Design Multiple Wallets</x:v>
+        <x:v>Bitcoin Design Wallet Activity Context</x:v>
       </x:c>
       <x:c r="C25" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/multiple-wallets/</x:v>
+        <x:v>https://bitcoin.design/guide/daily-spending-wallet/activity/</x:v>
       </x:c>
       <x:c r="D25" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1168,10 +1168,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F25" s="32" t="str">
-        <x:v>User-facing wallet architecture around separating funds by purpose, ownership, and security model inside one application.</x:v>
+        <x:v>User-facing wallet activity, contacts, and contextual payment-history concepts that help learners distinguish on-chain events from wallet-added meaning.</x:v>
       </x:c>
       <x:c r="G25" s="32" t="str">
-        <x:v>Track the multiple-wallets page separately so purpose-based wallet separation stays distinct from account-path mechanics, backup flows, and generic wallet activity metadata.</x:v>
+        <x:v>Track activity and contacts pages together so contextual metadata stays separate from backup flows and from protocol transaction mechanics.</x:v>
       </x:c>
       <x:c r="H25" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1186,27 +1186,27 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="L25" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M25" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N25" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="O25" s="32" t="str">
-        <x:v>Third Bitcoin Design implementation slice. The current additive winner is custody.multiple-wallets; encrypted cloud backups remains deferred because it overlaps too heavily with backups-recovery. Current tracked page queue is exhausted for this pass.</x:v>
+        <x:v>Second Bitcoin Design implementation slice. The current additive winner is custody.transaction-metadata; encrypted cloud backups remains the main deferred design-side candidate. Current tracked activity-and-contacts queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="str">
-        <x:v>source.bitcoin-design-cloud-backup</x:v>
+        <x:v>source.bitcoin-design-multiple-wallets</x:v>
       </x:c>
       <x:c r="B26" s="32" t="str">
-        <x:v>Bitcoin Design Automatic Cloud Backup</x:v>
+        <x:v>Bitcoin Design Multiple Wallets</x:v>
       </x:c>
       <x:c r="C26" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/how-it-works/private-key-management/cloud-backup/</x:v>
+        <x:v>https://bitcoin.design/guide/multiple-wallets/</x:v>
       </x:c>
       <x:c r="D26" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1215,10 +1215,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F26" s="32" t="str">
-        <x:v>User-facing backup scheme that stores encrypted wallet recovery data with an OS or cloud provider for low-friction restoration.</x:v>
+        <x:v>User-facing wallet architecture around separating funds by purpose, ownership, and security model inside one application.</x:v>
       </x:c>
       <x:c r="G26" s="32" t="str">
-        <x:v>Track the conceptual cloud-backup page, the daily-spending reference flow, and the private-key-management overview together so the scheme can be deduped against existing backup and Lightning recovery coverage.</x:v>
+        <x:v>Track the multiple-wallets page separately so purpose-based wallet separation stays distinct from account-path mechanics, backup flows, and generic wallet activity metadata.</x:v>
       </x:c>
       <x:c r="H26" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1227,13 +1227,13 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J26" s="32" t="str">
-        <x:v>Normalized to existing</x:v>
+        <x:v>Queue exhausted</x:v>
       </x:c>
       <x:c r="K26" s="32" t="str">
-        <x:v>Merged into existing</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L26" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M26" s="32" t="n">
         <x:v>1</x:v>
@@ -1242,18 +1242,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O26" s="32" t="str">
-        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is backup-scheme tradeoffs that already fit custody.backups-recovery plus lightning.channel-backups.</x:v>
+        <x:v>Third Bitcoin Design implementation slice. The current additive winner is custody.multiple-wallets; encrypted cloud backups remains deferred because it overlaps too heavily with backups-recovery. Current tracked page queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoin-design-cloud-backup</x:v>
       </x:c>
       <x:c r="B27" s="32" t="str">
-        <x:v>Bitcoin Design Upgradeable Wallet</x:v>
+        <x:v>Bitcoin Design Automatic Cloud Backup</x:v>
       </x:c>
       <x:c r="C27" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/upgradeable-wallet/</x:v>
+        <x:v>https://bitcoin.design/guide/how-it-works/private-key-management/cloud-backup/</x:v>
       </x:c>
       <x:c r="D27" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1262,10 +1262,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F27" s="32" t="str">
-        <x:v>User-facing wallet architecture for progressive security and staged upgrades between key-management schemes.</x:v>
+        <x:v>User-facing backup scheme that stores encrypted wallet recovery data with an OS or cloud provider for low-friction restoration.</x:v>
       </x:c>
       <x:c r="G27" s="32" t="str">
-        <x:v>Track the upgradeable-wallet reference design separately so progressive security becomes its own concept instead of staying buried inside cloud-backup discussions or multiwallet archival flows.</x:v>
+        <x:v>Track the conceptual cloud-backup page, the daily-spending reference flow, and the private-key-management overview together so the scheme can be deduped against existing backup and Lightning recovery coverage.</x:v>
       </x:c>
       <x:c r="H27" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1274,13 +1274,13 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J27" s="32" t="str">
-        <x:v>Queue exhausted</x:v>
+        <x:v>Normalized to existing</x:v>
       </x:c>
       <x:c r="K27" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>Merged into existing</x:v>
       </x:c>
       <x:c r="L27" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="M27" s="32" t="n">
         <x:v>1</x:v>
@@ -1289,18 +1289,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O27" s="32" t="str">
-        <x:v>Fourth Bitcoin Design implementation slice candidate. The current additive winner is custody.progressive-security, which survives dedupe more cleanly than automatic cloud backups or wallet-encryption. Current tracked page queue is exhausted for this pass.</x:v>
+        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is backup-scheme tradeoffs that already fit custody.backups-recovery plus lightning.channel-backups.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32" t="str">
-        <x:v>source.bitcoin-design-shared-wallet</x:v>
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="B28" s="32" t="str">
-        <x:v>Bitcoin Design Shared Wallet</x:v>
+        <x:v>Bitcoin Design Upgradeable Wallet</x:v>
       </x:c>
       <x:c r="C28" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/shared-wallet/</x:v>
+        <x:v>https://bitcoin.design/guide/upgradeable-wallet/</x:v>
       </x:c>
       <x:c r="D28" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1309,10 +1309,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F28" s="32" t="str">
-        <x:v>Reference design for co-managed wallets using multi-key schemes, provider-held recovery keys, and household approval policies.</x:v>
+        <x:v>User-facing wallet architecture for progressive security and staged upgrades between key-management schemes.</x:v>
       </x:c>
       <x:c r="G28" s="32" t="str">
-        <x:v>Track the shared-wallet page together with the generic multi-key explanation so persona-specific multisig scenarios are deduped against existing custody mechanism nodes.</x:v>
+        <x:v>Track the upgradeable-wallet reference design separately so progressive security becomes its own concept instead of staying buried inside cloud-backup discussions or multiwallet archival flows.</x:v>
       </x:c>
       <x:c r="H28" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1321,13 +1321,13 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J28" s="32" t="str">
-        <x:v>Normalized to existing</x:v>
+        <x:v>Queue exhausted</x:v>
       </x:c>
       <x:c r="K28" s="32" t="str">
-        <x:v>Merged into existing</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L28" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M28" s="32" t="n">
         <x:v>1</x:v>
@@ -1336,53 +1336,100 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O28" s="32" t="str">
-        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is shared-wallet examples for custody.multisig, custody.multiple-wallets, and custody.progressive-security.</x:v>
+        <x:v>Fourth Bitcoin Design implementation slice candidate. The current additive winner is custody.progressive-security, which survives dedupe more cleanly than automatic cloud backups or wallet-encryption. Current tracked page queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.bitcoin-design-shared-wallet</x:v>
       </x:c>
       <x:c r="B29" s="32" t="str">
-        <x:v>Bitcoin Developer Guides</x:v>
+        <x:v>Bitcoin Design Shared Wallet</x:v>
       </x:c>
       <x:c r="C29" s="32" t="str">
-        <x:v>https://developer.bitcoin.org/devguide/</x:v>
+        <x:v>https://bitcoin.design/guide/shared-wallet/</x:v>
       </x:c>
       <x:c r="D29" s="32" t="str">
-        <x:v>documentation-cluster</x:v>
+        <x:v>guide-cluster</x:v>
       </x:c>
       <x:c r="E29" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F29" s="32" t="str">
+        <x:v>Reference design for co-managed wallets using multi-key schemes, provider-held recovery keys, and household approval policies.</x:v>
+      </x:c>
+      <x:c r="G29" s="32" t="str">
+        <x:v>Track the shared-wallet page together with the generic multi-key explanation so persona-specific multisig scenarios are deduped against existing custody mechanism nodes.</x:v>
+      </x:c>
+      <x:c r="H29" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I29" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J29" s="32" t="str">
+        <x:v>Normalized to existing</x:v>
+      </x:c>
+      <x:c r="K29" s="32" t="str">
+        <x:v>Merged into existing</x:v>
+      </x:c>
+      <x:c r="L29" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M29" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N29" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O29" s="32" t="str">
+        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is shared-wallet examples for custody.multisig, custody.multiple-wallets, and custody.progressive-security.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="32" t="str">
+        <x:v>source.bitcoin-developer-guides</x:v>
+      </x:c>
+      <x:c r="B30" s="32" t="str">
+        <x:v>Bitcoin Developer Guides</x:v>
+      </x:c>
+      <x:c r="C30" s="32" t="str">
+        <x:v>https://developer.bitcoin.org/devguide/</x:v>
+      </x:c>
+      <x:c r="D30" s="32" t="str">
+        <x:v>documentation-cluster</x:v>
+      </x:c>
+      <x:c r="E30" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F30" s="32" t="str">
         <x:v>Canonical developer-facing guide sections covering block chain, transactions, contracts, wallets, payment processing, operating modes, P2P network, and mining.</x:v>
       </x:c>
-      <x:c r="G29" s="32" t="str">
+      <x:c r="G30" s="32" t="str">
         <x:v>Track the eight top-level guide sections first, then split dense sections like Transactions, Contracts, Wallets, and P2P Network when they expose concept gaps not already covered by existing nodes.</x:v>
       </x:c>
-      <x:c r="H29" s="32" t="str">
+      <x:c r="H30" s="32" t="str">
         <x:v>In review</x:v>
       </x:c>
-      <x:c r="I29" s="32" t="str">
+      <x:c r="I30" s="32" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="J29" s="32" t="str">
+      <x:c r="J30" s="32" t="str">
         <x:v>Queue exhausted</x:v>
       </x:c>
-      <x:c r="K29" s="32" t="str">
+      <x:c r="K30" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
-      <x:c r="L29" s="32" t="n">
+      <x:c r="L30" s="32" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="M29" s="32" t="n">
+      <x:c r="M30" s="32" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="N29" s="32" t="n">
+      <x:c r="N30" s="32" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="O29" s="32" t="str">
+      <x:c r="O30" s="32" t="str">
         <x:v>Added after the current audited source queue was exhausted. The first pass across the top-level sections surfaced four clean candidates: protocol.bitcoin-uri-bip21 from Payment Processing, dev.hardened-keys from Wallets, protocol.escrow-and-arbitration from Contracts, and mining.pool-shares from Pool Mining. A follow-up Wallet Files pass surfaced dev.wallet-import-format-wif as another clean wallet-standard slice. The implemented winners are now protocol.bitcoin-uri-bip21, dev.hardened-keys, protocol.escrow-and-arbitration, dev.wallet-import-format-wif, and mining.pool-shares because they land as missing standards, key-derivation, contract-pattern, key-serialization, and pooled-mining accounting bridges with clean direct parents. The current tracked top-level-plus-Wallet-Files queue is exhausted for this pass, though future deeper section splits may still surface more concepts.</x:v>
       </x:c>
     </x:row>
@@ -1392,16 +1439,16 @@
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H29">
+    <x:dataValidation type="list" sqref="H12:H30">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I29">
+    <x:dataValidation type="list" sqref="I12:I30">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J29">
+    <x:dataValidation type="list" sqref="J12:J30">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K29">
+    <x:dataValidation type="list" sqref="K12:K30">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -5191,16 +5238,67 @@
         <x:v>Implemented as a narrow Bitcoin-development review concept. Permissionless development remains deferred because it overlaps more heavily with neutrality, censorship resistance, and the BIPs process.</x:v>
       </x:c>
     </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="32" t="str">
+        <x:v>lightning.feature-flags</x:v>
+      </x:c>
+      <x:c r="B84" s="32" t="str">
+        <x:v>Lightning Feature Flags</x:v>
+      </x:c>
+      <x:c r="C84" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D84" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E84" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/09-features.md</x:v>
+      </x:c>
+      <x:c r="F84" s="32" t="str">
+        <x:v>BOLT 09: Features &gt; feature-bit registry and optional/required semantics</x:v>
+      </x:c>
+      <x:c r="G84" s="32" t="str"/>
+      <x:c r="H84" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I84" s="32" t="str">
+        <x:v>This is one specific interoperability mechanism: capability bits that implementations advertise and negotiate across init messages, announcements, invoices, and related protocol contexts. It is narrower than Lightning gossip, peer messaging, and the individual protocols that consume the negotiated features.</x:v>
+      </x:c>
+      <x:c r="J84" s="32" t="str">
+        <x:v>lightning.gossip-protocol, dev.p2p-messages, lightning.routing</x:v>
+      </x:c>
+      <x:c r="K84" s="32" t="str">
+        <x:v>lightning.gossip-protocol</x:v>
+      </x:c>
+      <x:c r="L84" s="32" t="str">
+        <x:v>The gossip protocol supplies the Lightning network-advertisement context in which feature signaling is used. P2P messages and routing are inherited implementation or consumer context rather than direct prerequisites for understanding the feature-bit negotiation mechanism.</x:v>
+      </x:c>
+      <x:c r="M84" s="32" t="str">
+        <x:v>Lightning feature bits, Lightning capability negotiation, BOLT 09 features</x:v>
+      </x:c>
+      <x:c r="N84" s="32" t="str">
+        <x:v>lightning, protocol, interoperability</x:v>
+      </x:c>
+      <x:c r="O84" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P84" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q84" s="32" t="str">
+        <x:v>Implemented as the first BOLTs source-expansion slice. The odd/even optional-versus-required rule is kept inside this node rather than split into separate feature-bit nodes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H83">
+    <x:dataValidation type="list" sqref="H12:H84">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P83">
+    <x:dataValidation type="list" sqref="P12:P84">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -7152,16 +7250,39 @@
         <x:v>Direct edge keeps review distinct from responsible disclosure and reproducible-build verification, which are specialized downstream safeguards.</x:v>
       </x:c>
     </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="32" t="str">
+        <x:v>lightning.gossip-protocol</x:v>
+      </x:c>
+      <x:c r="B94" s="32" t="str">
+        <x:v>lightning.feature-flags</x:v>
+      </x:c>
+      <x:c r="C94" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D94" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E94" s="32" t="str">
+        <x:v>Feature negotiation is used to advertise and interpret capabilities across Lightning peers and network announcements, so learners need the surrounding gossip and announcement context first.</x:v>
+      </x:c>
+      <x:c r="F94" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="G94" s="32" t="str">
+        <x:v>Direct edge keeps the feature-bit mechanism distinct from the lower-level message transport and downstream routing protocols.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C93">
+    <x:dataValidation type="list" sqref="C12:C94">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D93">
+    <x:dataValidation type="list" sqref="D12:D94">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9155,16 +9276,42 @@
         <x:v>Added with only the proposal lifecycle and adversarial mindset as direct prerequisites. Permissionless development is deferred pending a narrower dedupe pass.</x:v>
       </x:c>
     </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="32" t="str">
+        <x:v>decision.lightning-feature-flags-slice</x:v>
+      </x:c>
+      <x:c r="B86" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C86" s="32" t="str">
+        <x:v>lightning.feature-flags</x:v>
+      </x:c>
+      <x:c r="D86" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E86" s="32" t="str">
+        <x:v>BOLT 09 exposes a precise Lightning interoperability concept that is absent from the graph: negotiating optional and required capability bits. It survives dedupe because gossip, peer messaging, and routing describe the surrounding protocol or consumers, not the feature-bit registry and negotiation rule itself.</x:v>
+      </x:c>
+      <x:c r="F86" s="32" t="str">
+        <x:v>lightning.feature-flags, lightning.gossip-protocol, dev.p2p-messages, lightning.routing</x:v>
+      </x:c>
+      <x:c r="G86" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="H86" s="32" t="str">
+        <x:v>Added with only lightning.gossip-protocol as a direct prerequisite. BOLT 01 and BOLT 07 remain curated supporting resources, while the broader BOLTs source queue stays in review.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B85">
+    <x:dataValidation type="list" sqref="B12:B86">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D85">
+    <x:dataValidation type="list" sqref="D12:D86">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9217,7 +9364,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.09324214121</x:v>
+        <x:v>46213.10172395833</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -9225,7 +9372,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -9241,7 +9388,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>72</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -9249,7 +9396,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>82</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -9273,7 +9420,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add lightning onion messages
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rb7e1513679f94c31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rcdd53396afd24a08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R4fd2181b1b5949ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R34b7278f6d4b4337"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Ra1c8387b4f234ae8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R3211e194f4414f33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R7881ac00e03645c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R0f8421162a354463"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R81750f33b47c4740"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Re11dd1311e8448c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rd39a608ff1c04116"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Redd7d5323ea7486d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -907,13 +907,13 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="M19" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N19" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="O19" s="32" t="str">
-        <x:v>Added during source expansion. The first inventory covers the BOLT index plus messaging, peer protocol, onion messaging, encrypted transport, feature negotiation, and DNS bootstrap clusters. Implemented from this source in the current branch: lightning.feature-flags.</x:v>
+        <x:v>Added during source expansion. The first inventory covers the BOLT index plus messaging, peer protocol, onion messaging, encrypted transport, feature negotiation, and DNS bootstrap clusters. Implemented from this source in the current branch: lightning.feature-flags and lightning.onion-messages.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -5289,16 +5289,67 @@
         <x:v>Implemented as the first BOLTs source-expansion slice. The odd/even optional-versus-required rule is kept inside this node rather than split into separate feature-bit nodes.</x:v>
       </x:c>
     </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="32" t="str">
+        <x:v>lightning.onion-messages</x:v>
+      </x:c>
+      <x:c r="B85" s="32" t="str">
+        <x:v>Lightning Onion Messages</x:v>
+      </x:c>
+      <x:c r="C85" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D85" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E85" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/04-onion-routing.md#onion-messages</x:v>
+      </x:c>
+      <x:c r="F85" s="32" t="str">
+        <x:v>BOLT 04: Onion Routing Protocol &gt; Onion Messages</x:v>
+      </x:c>
+      <x:c r="G85" s="32" t="str"/>
+      <x:c r="H85" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I85" s="32" t="str">
+        <x:v>This is one specific Lightning transport mechanism: forwarding unreliable encrypted messages over blinded onion paths without using a payment HTLC. It is distinct from payment onion routing, route blinding itself, and BOLT12 offer encoding.</x:v>
+      </x:c>
+      <x:c r="J85" s="32" t="str">
+        <x:v>lightning.feature-flags, lightning.route-blinding, lightning.onion-routing, lightning.bolt12-offers</x:v>
+      </x:c>
+      <x:c r="K85" s="32" t="str">
+        <x:v>lightning.feature-flags, lightning.route-blinding</x:v>
+      </x:c>
+      <x:c r="L85" s="32" t="str">
+        <x:v>Feature negotiation explains how peers signal onion-message support, and route blinding explains the privacy-preserving path construction. Payment onion routing is a sibling transport model, while BOLT12 offers are one downstream message use case rather than a prerequisite.</x:v>
+      </x:c>
+      <x:c r="M85" s="32" t="str">
+        <x:v>onion messages, channel-independent messages, BOLT 04 onion messages</x:v>
+      </x:c>
+      <x:c r="N85" s="32" t="str">
+        <x:v>lightning, onion-routing, privacy</x:v>
+      </x:c>
+      <x:c r="O85" s="32" t="str">
+        <x:v>45m</x:v>
+      </x:c>
+      <x:c r="P85" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q85" s="32" t="str">
+        <x:v>Implemented as the next BOLTs slice after feature flags. BOLT 08 transport, BOLT 10 DNS bootstrap, and already-covered dual funding remain queued or merge/defer candidates.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H84">
+    <x:dataValidation type="list" sqref="H12:H85">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P84">
+    <x:dataValidation type="list" sqref="P12:P85">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -7273,16 +7324,62 @@
         <x:v>Direct edge keeps the feature-bit mechanism distinct from the lower-level message transport and downstream routing protocols.</x:v>
       </x:c>
     </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="32" t="str">
+        <x:v>lightning.feature-flags</x:v>
+      </x:c>
+      <x:c r="B95" s="32" t="str">
+        <x:v>lightning.onion-messages</x:v>
+      </x:c>
+      <x:c r="C95" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D95" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E95" s="32" t="str">
+        <x:v>Peers use a negotiated feature bit to advertise whether they can send and forward onion messages, so learners need the capability-negotiation model first.</x:v>
+      </x:c>
+      <x:c r="F95" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="G95" s="32" t="str">
+        <x:v>Direct edge keeps the feature gate separate from the message forwarding mechanism.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="32" t="str">
+        <x:v>lightning.route-blinding</x:v>
+      </x:c>
+      <x:c r="B96" s="32" t="str">
+        <x:v>lightning.onion-messages</x:v>
+      </x:c>
+      <x:c r="C96" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D96" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E96" s="32" t="str">
+        <x:v>Onion messages use blinded paths to forward channel-independent payloads without exposing the final destination topology, so the route-blinding model must come first.</x:v>
+      </x:c>
+      <x:c r="F96" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="G96" s="32" t="str">
+        <x:v>Payment onion routing and BOLT12 offers remain related sibling or downstream concepts rather than direct prerequisites.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C94">
+    <x:dataValidation type="list" sqref="C12:C96">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D94">
+    <x:dataValidation type="list" sqref="D12:D96">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9302,16 +9399,42 @@
         <x:v>Added with only lightning.gossip-protocol as a direct prerequisite. BOLT 01 and BOLT 07 remain curated supporting resources, while the broader BOLTs source queue stays in review.</x:v>
       </x:c>
     </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="32" t="str">
+        <x:v>decision.lightning-onion-messages-slice</x:v>
+      </x:c>
+      <x:c r="B87" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C87" s="32" t="str">
+        <x:v>lightning.onion-messages</x:v>
+      </x:c>
+      <x:c r="D87" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E87" s="32" t="str">
+        <x:v>BOLT 04 exposes an atomic message-transport mechanism missing from the graph: unreliable encrypted payloads forwarded over blinded onion paths without payment HTLCs. It survives dedupe because payment onion routing, route blinding, and BOLT12 offers each cover different neighboring learning outcomes.</x:v>
+      </x:c>
+      <x:c r="F87" s="32" t="str">
+        <x:v>lightning.onion-messages, lightning.feature-flags, lightning.route-blinding, lightning.onion-routing, lightning.bolt12-offers</x:v>
+      </x:c>
+      <x:c r="G87" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="H87" s="32" t="str">
+        <x:v>Added with feature flags and route blinding as direct prerequisites. BOLT 08 Noise transport and BOLT 10 DNS bootstrap remain future source-expansion candidates.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B86">
+    <x:dataValidation type="list" sqref="B12:B87">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D86">
+    <x:dataValidation type="list" sqref="D12:D87">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9364,7 +9487,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.10172395833</x:v>
+        <x:v>46213.10638196759</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -9388,7 +9511,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>73</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -9396,7 +9519,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>83</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -9420,7 +9543,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>62</x:v>
+        <x:v>63</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add strict der signature encoding
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R7881ac00e03645c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R0f8421162a354463"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R81750f33b47c4740"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Re11dd1311e8448c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rd39a608ff1c04116"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Redd7d5323ea7486d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rec48526faf9a4d2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R2f814e33807148b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R59ba12c3a4ef48c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R28569f11f58c44a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R0cbeb966797846f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Ra9f26b82db6a4c2f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -918,72 +918,72 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="B20" s="32" t="str">
-        <x:v>Cypherpunk Library Bitcoin-Adjacent Canon</x:v>
+        <x:v>Bitcoin Improvement Proposals</x:v>
       </x:c>
       <x:c r="C20" s="32" t="str">
-        <x:v>https://www.cypherpunkbooks.com/collection</x:v>
+        <x:v>https://github.com/bitcoin/bips</x:v>
       </x:c>
       <x:c r="D20" s="32" t="str">
-        <x:v>essay-library</x:v>
+        <x:v>standards-repository</x:v>
       </x:c>
       <x:c r="E20" s="32" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="F20" s="32" t="str">
-        <x:v>Bitcoin-adjacent cypherpunk readings focused on privacy, electronic cash, monetary theory, and the ideological roots most likely to sharpen foundational and history nodes.</x:v>
+        <x:v>Canonical Bitcoin Improvement Proposals covering process, consensus rules, signatures, wallet formats, applications, peer services, relay, APIs, mining, and deployment mechanisms.</x:v>
       </x:c>
       <x:c r="G20" s="32" t="str">
-        <x:v>Start with four clusters: cypherpunk manifestos, privacy and surveillance essays, eCash and digital-cash texts, and monetary-theory readings. Defer clearly non-Bitcoin-adjacent political or general-hacker texts unless they surface a direct graph gap.</x:v>
+        <x:v>Enumerate the repository registry first, then group BIPs into consensus soft forks, signature encoding and serialization, script and output templates, wallet and payment standards, and peer/relay protocols. Treat BIPs as specification provenance rather than automatic one-to-one nodes.</x:v>
       </x:c>
       <x:c r="H20" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>Inventorying</x:v>
       </x:c>
       <x:c r="I20" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="J20" s="32" t="str">
-        <x:v>Queue exhausted</x:v>
+        <x:v>Raw extraction</x:v>
       </x:c>
       <x:c r="K20" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="L20" s="32" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M20" s="32" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N20" s="32" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O20" s="32" t="str">
-        <x:v>Added from user direction. High-signal starting texts from the collection include A Cypherpunk's Manifesto, The Crypto Anarchist Manifesto, Your Secret Right to Cash, Protecting Privacy with Electronic Cash, The Beauty of eCash, The Cyphernomicon, Ideal Money and Asymptotically Ideal Money, and 21 Lessons. Implemented from this source in the current branch: history.chaumian-ecash, privacy.secret-right-to-cash, economics.ideal-money. Merged into existing coverage in the current branch: history.cypherpunks via A Cypherpunk's Manifesto; history.bitcoin-anarchism via The Crypto Anarchist Manifesto. Current tracked cluster queue is exhausted for this pass.</x:v>
+        <x:v>Added during source expansion. Initial inventory covers the registry/process, consensus soft forks, signature encoding and serialization, script/output templates, wallet/payment standards, and peer/relay clusters. Implemented from this source in the current branch: protocol.strict-der-signatures.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="B21" s="32" t="str">
-        <x:v>Bitcoin Dev Project Explained Posts</x:v>
+        <x:v>Cypherpunk Library Bitcoin-Adjacent Canon</x:v>
       </x:c>
       <x:c r="C21" s="32" t="str">
-        <x:v>https://x.com/search?q=from%3ABitcoin_Devs%20explained&amp;src=typed_query&amp;f=live</x:v>
+        <x:v>https://www.cypherpunkbooks.com/collection</x:v>
       </x:c>
       <x:c r="D21" s="32" t="str">
-        <x:v>social-post-cluster</x:v>
+        <x:v>essay-library</x:v>
       </x:c>
       <x:c r="E21" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F21" s="32" t="str">
-        <x:v>Short-form educational posts from @Bitcoin_Devs that explicitly explain protocol, wallet, and Lightning mechanisms in learner-facing language.</x:v>
+        <x:v>Bitcoin-adjacent cypherpunk readings focused on privacy, electronic cash, monetary theory, and the ideological roots most likely to sharpen foundational and history nodes.</x:v>
       </x:c>
       <x:c r="G21" s="32" t="str">
-        <x:v>Track the live X search as one source-family row first, then expand to one row per matching post once current results are enumerated. Group matching posts by concept family such as hashing, fee management, node architecture, channel mechanics, and upgrade proposals.</x:v>
+        <x:v>Start with four clusters: cypherpunk manifestos, privacy and surveillance essays, eCash and digital-cash texts, and monetary-theory readings. Defer clearly non-Bitcoin-adjacent political or general-hacker texts unless they surface a direct graph gap.</x:v>
       </x:c>
       <x:c r="H21" s="32" t="str">
         <x:v>Complete</x:v>
@@ -998,39 +998,39 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="L21" s="32" t="n">
-        <x:v>43</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M21" s="32" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N21" s="32" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O21" s="32" t="str">
-        <x:v>Added from user direction. The live X query was enumerated in the logged-in in-app browser on July 8, 2026 and surfaced 43 matching posts. Visible examples include Lamport Signature explained, Duplicate transaction bug explained, 64-byte transaction bug explained, SegWit Address explained, Off-by-one difficulty bug explained, Great Consensus Cleanup explained Part 1: Time Warp Attack, Transaction Pinning explained, Full Node Architecture Explained, MAST explained simply, BIP 158 explained, MuSig explained Simply, CPFP transaction explained, CISA explained, BIP-68 Explained, and Shamir's Secret Sharing explained. Implemented from this source in the current branch: protocol.time-warp-attack, protocol.duplicate-transaction-bug, protocol.64-byte-transaction-bug, fundamentals.lamport-signatures, custody.shamirs-secret-sharing. Merged into existing coverage in the current branch: protocol.time-warp-attack via Off-by-one difficulty bug explained. Current enumerated post queue is exhausted for this pass.</x:v>
+        <x:v>Added from user direction. High-signal starting texts from the collection include A Cypherpunk's Manifesto, The Crypto Anarchist Manifesto, Your Secret Right to Cash, Protecting Privacy with Electronic Cash, The Beauty of eCash, The Cyphernomicon, Ideal Money and Asymptotically Ideal Money, and 21 Lessons. Implemented from this source in the current branch: history.chaumian-ecash, privacy.secret-right-to-cash, economics.ideal-money. Merged into existing coverage in the current branch: history.cypherpunks via A Cypherpunk's Manifesto; history.bitcoin-anarchism via The Crypto Anarchist Manifesto. Current tracked cluster queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-wallet</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="B22" s="32" t="str">
-        <x:v>Bitcoin Core Academy Wallet Internals</x:v>
+        <x:v>Bitcoin Dev Project Explained Posts</x:v>
       </x:c>
       <x:c r="C22" s="32" t="str">
-        <x:v>https://bitcoincore.academy/scriptpubkeymanagers.html</x:v>
+        <x:v>https://x.com/search?q=from%3ABitcoin_Devs%20explained&amp;src=typed_query&amp;f=live</x:v>
       </x:c>
       <x:c r="D22" s="32" t="str">
-        <x:v>course-cluster</x:v>
+        <x:v>social-post-cluster</x:v>
       </x:c>
       <x:c r="E22" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F22" s="32" t="str">
-        <x:v>Wallet internals cluster around ScriptPubKeyManagers, wallet keys, transaction identification, and balance calculation.</x:v>
+        <x:v>Short-form educational posts from @Bitcoin_Devs that explicitly explain protocol, wallet, and Lightning mechanisms in learner-facing language.</x:v>
       </x:c>
       <x:c r="G22" s="32" t="str">
-        <x:v>Track one wallet-internals page cluster at a time so Core-specific abstractions stay atomic instead of collapsing into generic wallet concepts.</x:v>
+        <x:v>Track the live X search as one source-family row first, then expand to one row per matching post once current results are enumerated. Group matching posts by concept family such as hashing, fee management, node architecture, channel mechanics, and upgrade proposals.</x:v>
       </x:c>
       <x:c r="H22" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1045,27 +1045,27 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="L22" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="M22" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="N22" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="O22" s="32" t="str">
-        <x:v>First additional-source pass beyond the mandatory seed list. The current additive winner is dev.scriptpubkeymanagers; wallet-encryption remains deferred because the cleanest surviving slice is still too coupled to missing Core wallet-internals parents. Current tracked wallet-internals queue is exhausted for this pass.</x:v>
+        <x:v>Added from user direction. The live X query was enumerated in the logged-in in-app browser on July 8, 2026 and surfaced 43 matching posts. Visible examples include Lamport Signature explained, Duplicate transaction bug explained, 64-byte transaction bug explained, SegWit Address explained, Off-by-one difficulty bug explained, Great Consensus Cleanup explained Part 1: Time Warp Attack, Transaction Pinning explained, Full Node Architecture Explained, MAST explained simply, BIP 158 explained, MuSig explained Simply, CPFP transaction explained, CISA explained, BIP-68 Explained, and Shamir's Secret Sharing explained. Implemented from this source in the current branch: protocol.time-warp-attack, protocol.duplicate-transaction-bug, protocol.64-byte-transaction-bug, fundamentals.lamport-signatures, custody.shamirs-secret-sharing. Merged into existing coverage in the current branch: protocol.time-warp-attack via Off-by-one difficulty bug explained. Current enumerated post queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-core-academy-wallet</x:v>
       </x:c>
       <x:c r="B23" s="32" t="str">
-        <x:v>Bitcoin Core Academy Mempool Mechanics</x:v>
+        <x:v>Bitcoin Core Academy Wallet Internals</x:v>
       </x:c>
       <x:c r="C23" s="32" t="str">
-        <x:v>https://bitcoincore.academy/mempool-unbroadcast.html</x:v>
+        <x:v>https://bitcoincore.academy/scriptpubkeymanagers.html</x:v>
       </x:c>
       <x:c r="D23" s="32" t="str">
         <x:v>course-cluster</x:v>
@@ -1074,10 +1074,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F23" s="32" t="str">
-        <x:v>Mempool and relay internals cluster around transaction relay, rebroadcast behavior, and local node transaction state.</x:v>
+        <x:v>Wallet internals cluster around ScriptPubKeyManagers, wallet keys, transaction identification, and balance calculation.</x:v>
       </x:c>
       <x:c r="G23" s="32" t="str">
-        <x:v>Track the academy mempool pages as a separate cluster so implementation-specific relay mechanisms are not collapsed into generic mempool coverage.</x:v>
+        <x:v>Track one wallet-internals page cluster at a time so Core-specific abstractions stay atomic instead of collapsing into generic wallet concepts.</x:v>
       </x:c>
       <x:c r="H23" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1098,33 +1098,33 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="N23" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O23" s="32" t="str">
-        <x:v>Second post-seed-source slice. The current additive winners are protocol.mempool-unbroadcast-set, protocol.transaction-rebroadcast-privacy, and protocol.txid-vs-wtxid. The remaining transaction-format internals are now mostly implementation-detail material rather than clean learner-facing nodes. Current tracked mempool queue is exhausted for this pass.</x:v>
+        <x:v>First additional-source pass beyond the mandatory seed list. The current additive winner is dev.scriptpubkeymanagers; wallet-encryption remains deferred because the cleanest surviving slice is still too coupled to missing Core wallet-internals parents. Current tracked wallet-internals queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="str">
-        <x:v>source.bitcoin-design-payment-formats</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="B24" s="32" t="str">
-        <x:v>Bitcoin Design Payment Request Formats</x:v>
+        <x:v>Bitcoin Core Academy Mempool Mechanics</x:v>
       </x:c>
       <x:c r="C24" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/how-it-works/human-readable-addresses/</x:v>
+        <x:v>https://bitcoincore.academy/mempool-unbroadcast.html</x:v>
       </x:c>
       <x:c r="D24" s="32" t="str">
-        <x:v>guide-cluster</x:v>
+        <x:v>course-cluster</x:v>
       </x:c>
       <x:c r="E24" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F24" s="32" t="str">
-        <x:v>User-facing payment request and address-sharing concepts across human-readable addresses, transaction display, and wallet privacy tradeoffs.</x:v>
+        <x:v>Mempool and relay internals cluster around transaction relay, rebroadcast behavior, and local node transaction state.</x:v>
       </x:c>
       <x:c r="G24" s="32" t="str">
-        <x:v>Track design guide pages by UX concept cluster so user-facing payment abstractions stay separate from protocol internals and generic wallet hygiene.</x:v>
+        <x:v>Track the academy mempool pages as a separate cluster so implementation-specific relay mechanisms are not collapsed into generic mempool coverage.</x:v>
       </x:c>
       <x:c r="H24" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1145,21 +1145,21 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="N24" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O24" s="32" t="str">
-        <x:v>First Bitcoin Design implementation slice. The current additive winner is custody.human-readable-addresses; encrypted cloud backups remains the main deferred neighbor from this design source family. Current tracked payment-format queue is exhausted for this pass.</x:v>
+        <x:v>Second post-seed-source slice. The current additive winners are protocol.mempool-unbroadcast-set, protocol.transaction-rebroadcast-privacy, and protocol.txid-vs-wtxid. The remaining transaction-format internals are now mostly implementation-detail material rather than clean learner-facing nodes. Current tracked mempool queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoin-design-payment-formats</x:v>
       </x:c>
       <x:c r="B25" s="32" t="str">
-        <x:v>Bitcoin Design Wallet Activity Context</x:v>
+        <x:v>Bitcoin Design Payment Request Formats</x:v>
       </x:c>
       <x:c r="C25" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/daily-spending-wallet/activity/</x:v>
+        <x:v>https://bitcoin.design/guide/how-it-works/human-readable-addresses/</x:v>
       </x:c>
       <x:c r="D25" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1168,10 +1168,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F25" s="32" t="str">
-        <x:v>User-facing wallet activity, contacts, and contextual payment-history concepts that help learners distinguish on-chain events from wallet-added meaning.</x:v>
+        <x:v>User-facing payment request and address-sharing concepts across human-readable addresses, transaction display, and wallet privacy tradeoffs.</x:v>
       </x:c>
       <x:c r="G25" s="32" t="str">
-        <x:v>Track activity and contacts pages together so contextual metadata stays separate from backup flows and from protocol transaction mechanics.</x:v>
+        <x:v>Track design guide pages by UX concept cluster so user-facing payment abstractions stay separate from protocol internals and generic wallet hygiene.</x:v>
       </x:c>
       <x:c r="H25" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1186,27 +1186,27 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="L25" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="M25" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N25" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="O25" s="32" t="str">
-        <x:v>Second Bitcoin Design implementation slice. The current additive winner is custody.transaction-metadata; encrypted cloud backups remains the main deferred design-side candidate. Current tracked activity-and-contacts queue is exhausted for this pass.</x:v>
+        <x:v>First Bitcoin Design implementation slice. The current additive winner is custody.human-readable-addresses; encrypted cloud backups remains the main deferred neighbor from this design source family. Current tracked payment-format queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="str">
-        <x:v>source.bitcoin-design-multiple-wallets</x:v>
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="B26" s="32" t="str">
-        <x:v>Bitcoin Design Multiple Wallets</x:v>
+        <x:v>Bitcoin Design Wallet Activity Context</x:v>
       </x:c>
       <x:c r="C26" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/multiple-wallets/</x:v>
+        <x:v>https://bitcoin.design/guide/daily-spending-wallet/activity/</x:v>
       </x:c>
       <x:c r="D26" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1215,10 +1215,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F26" s="32" t="str">
-        <x:v>User-facing wallet architecture around separating funds by purpose, ownership, and security model inside one application.</x:v>
+        <x:v>User-facing wallet activity, contacts, and contextual payment-history concepts that help learners distinguish on-chain events from wallet-added meaning.</x:v>
       </x:c>
       <x:c r="G26" s="32" t="str">
-        <x:v>Track the multiple-wallets page separately so purpose-based wallet separation stays distinct from account-path mechanics, backup flows, and generic wallet activity metadata.</x:v>
+        <x:v>Track activity and contacts pages together so contextual metadata stays separate from backup flows and from protocol transaction mechanics.</x:v>
       </x:c>
       <x:c r="H26" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1233,27 +1233,27 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="L26" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M26" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N26" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="O26" s="32" t="str">
-        <x:v>Third Bitcoin Design implementation slice. The current additive winner is custody.multiple-wallets; encrypted cloud backups remains deferred because it overlaps too heavily with backups-recovery. Current tracked page queue is exhausted for this pass.</x:v>
+        <x:v>Second Bitcoin Design implementation slice. The current additive winner is custody.transaction-metadata; encrypted cloud backups remains the main deferred design-side candidate. Current tracked activity-and-contacts queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="str">
-        <x:v>source.bitcoin-design-cloud-backup</x:v>
+        <x:v>source.bitcoin-design-multiple-wallets</x:v>
       </x:c>
       <x:c r="B27" s="32" t="str">
-        <x:v>Bitcoin Design Automatic Cloud Backup</x:v>
+        <x:v>Bitcoin Design Multiple Wallets</x:v>
       </x:c>
       <x:c r="C27" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/how-it-works/private-key-management/cloud-backup/</x:v>
+        <x:v>https://bitcoin.design/guide/multiple-wallets/</x:v>
       </x:c>
       <x:c r="D27" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1262,10 +1262,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F27" s="32" t="str">
-        <x:v>User-facing backup scheme that stores encrypted wallet recovery data with an OS or cloud provider for low-friction restoration.</x:v>
+        <x:v>User-facing wallet architecture around separating funds by purpose, ownership, and security model inside one application.</x:v>
       </x:c>
       <x:c r="G27" s="32" t="str">
-        <x:v>Track the conceptual cloud-backup page, the daily-spending reference flow, and the private-key-management overview together so the scheme can be deduped against existing backup and Lightning recovery coverage.</x:v>
+        <x:v>Track the multiple-wallets page separately so purpose-based wallet separation stays distinct from account-path mechanics, backup flows, and generic wallet activity metadata.</x:v>
       </x:c>
       <x:c r="H27" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1274,13 +1274,13 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J27" s="32" t="str">
-        <x:v>Normalized to existing</x:v>
+        <x:v>Queue exhausted</x:v>
       </x:c>
       <x:c r="K27" s="32" t="str">
-        <x:v>Merged into existing</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L27" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M27" s="32" t="n">
         <x:v>1</x:v>
@@ -1289,18 +1289,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O27" s="32" t="str">
-        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is backup-scheme tradeoffs that already fit custody.backups-recovery plus lightning.channel-backups.</x:v>
+        <x:v>Third Bitcoin Design implementation slice. The current additive winner is custody.multiple-wallets; encrypted cloud backups remains deferred because it overlaps too heavily with backups-recovery. Current tracked page queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoin-design-cloud-backup</x:v>
       </x:c>
       <x:c r="B28" s="32" t="str">
-        <x:v>Bitcoin Design Upgradeable Wallet</x:v>
+        <x:v>Bitcoin Design Automatic Cloud Backup</x:v>
       </x:c>
       <x:c r="C28" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/upgradeable-wallet/</x:v>
+        <x:v>https://bitcoin.design/guide/how-it-works/private-key-management/cloud-backup/</x:v>
       </x:c>
       <x:c r="D28" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1309,10 +1309,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F28" s="32" t="str">
-        <x:v>User-facing wallet architecture for progressive security and staged upgrades between key-management schemes.</x:v>
+        <x:v>User-facing backup scheme that stores encrypted wallet recovery data with an OS or cloud provider for low-friction restoration.</x:v>
       </x:c>
       <x:c r="G28" s="32" t="str">
-        <x:v>Track the upgradeable-wallet reference design separately so progressive security becomes its own concept instead of staying buried inside cloud-backup discussions or multiwallet archival flows.</x:v>
+        <x:v>Track the conceptual cloud-backup page, the daily-spending reference flow, and the private-key-management overview together so the scheme can be deduped against existing backup and Lightning recovery coverage.</x:v>
       </x:c>
       <x:c r="H28" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1321,13 +1321,13 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J28" s="32" t="str">
-        <x:v>Queue exhausted</x:v>
+        <x:v>Normalized to existing</x:v>
       </x:c>
       <x:c r="K28" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>Merged into existing</x:v>
       </x:c>
       <x:c r="L28" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="M28" s="32" t="n">
         <x:v>1</x:v>
@@ -1336,18 +1336,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O28" s="32" t="str">
-        <x:v>Fourth Bitcoin Design implementation slice candidate. The current additive winner is custody.progressive-security, which survives dedupe more cleanly than automatic cloud backups or wallet-encryption. Current tracked page queue is exhausted for this pass.</x:v>
+        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is backup-scheme tradeoffs that already fit custody.backups-recovery plus lightning.channel-backups.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="32" t="str">
-        <x:v>source.bitcoin-design-shared-wallet</x:v>
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="B29" s="32" t="str">
-        <x:v>Bitcoin Design Shared Wallet</x:v>
+        <x:v>Bitcoin Design Upgradeable Wallet</x:v>
       </x:c>
       <x:c r="C29" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/shared-wallet/</x:v>
+        <x:v>https://bitcoin.design/guide/upgradeable-wallet/</x:v>
       </x:c>
       <x:c r="D29" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1356,10 +1356,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F29" s="32" t="str">
-        <x:v>Reference design for co-managed wallets using multi-key schemes, provider-held recovery keys, and household approval policies.</x:v>
+        <x:v>User-facing wallet architecture for progressive security and staged upgrades between key-management schemes.</x:v>
       </x:c>
       <x:c r="G29" s="32" t="str">
-        <x:v>Track the shared-wallet page together with the generic multi-key explanation so persona-specific multisig scenarios are deduped against existing custody mechanism nodes.</x:v>
+        <x:v>Track the upgradeable-wallet reference design separately so progressive security becomes its own concept instead of staying buried inside cloud-backup discussions or multiwallet archival flows.</x:v>
       </x:c>
       <x:c r="H29" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1368,13 +1368,13 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J29" s="32" t="str">
-        <x:v>Normalized to existing</x:v>
+        <x:v>Queue exhausted</x:v>
       </x:c>
       <x:c r="K29" s="32" t="str">
-        <x:v>Merged into existing</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L29" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M29" s="32" t="n">
         <x:v>1</x:v>
@@ -1383,53 +1383,100 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O29" s="32" t="str">
-        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is shared-wallet examples for custody.multisig, custody.multiple-wallets, and custody.progressive-security.</x:v>
+        <x:v>Fourth Bitcoin Design implementation slice candidate. The current additive winner is custody.progressive-security, which survives dedupe more cleanly than automatic cloud backups or wallet-encryption. Current tracked page queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.bitcoin-design-shared-wallet</x:v>
       </x:c>
       <x:c r="B30" s="32" t="str">
-        <x:v>Bitcoin Developer Guides</x:v>
+        <x:v>Bitcoin Design Shared Wallet</x:v>
       </x:c>
       <x:c r="C30" s="32" t="str">
-        <x:v>https://developer.bitcoin.org/devguide/</x:v>
+        <x:v>https://bitcoin.design/guide/shared-wallet/</x:v>
       </x:c>
       <x:c r="D30" s="32" t="str">
-        <x:v>documentation-cluster</x:v>
+        <x:v>guide-cluster</x:v>
       </x:c>
       <x:c r="E30" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F30" s="32" t="str">
+        <x:v>Reference design for co-managed wallets using multi-key schemes, provider-held recovery keys, and household approval policies.</x:v>
+      </x:c>
+      <x:c r="G30" s="32" t="str">
+        <x:v>Track the shared-wallet page together with the generic multi-key explanation so persona-specific multisig scenarios are deduped against existing custody mechanism nodes.</x:v>
+      </x:c>
+      <x:c r="H30" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I30" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J30" s="32" t="str">
+        <x:v>Normalized to existing</x:v>
+      </x:c>
+      <x:c r="K30" s="32" t="str">
+        <x:v>Merged into existing</x:v>
+      </x:c>
+      <x:c r="L30" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M30" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N30" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O30" s="32" t="str">
+        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is shared-wallet examples for custody.multisig, custody.multiple-wallets, and custody.progressive-security.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="32" t="str">
+        <x:v>source.bitcoin-developer-guides</x:v>
+      </x:c>
+      <x:c r="B31" s="32" t="str">
+        <x:v>Bitcoin Developer Guides</x:v>
+      </x:c>
+      <x:c r="C31" s="32" t="str">
+        <x:v>https://developer.bitcoin.org/devguide/</x:v>
+      </x:c>
+      <x:c r="D31" s="32" t="str">
+        <x:v>documentation-cluster</x:v>
+      </x:c>
+      <x:c r="E31" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F31" s="32" t="str">
         <x:v>Canonical developer-facing guide sections covering block chain, transactions, contracts, wallets, payment processing, operating modes, P2P network, and mining.</x:v>
       </x:c>
-      <x:c r="G30" s="32" t="str">
+      <x:c r="G31" s="32" t="str">
         <x:v>Track the eight top-level guide sections first, then split dense sections like Transactions, Contracts, Wallets, and P2P Network when they expose concept gaps not already covered by existing nodes.</x:v>
       </x:c>
-      <x:c r="H30" s="32" t="str">
+      <x:c r="H31" s="32" t="str">
         <x:v>In review</x:v>
       </x:c>
-      <x:c r="I30" s="32" t="str">
+      <x:c r="I31" s="32" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="J30" s="32" t="str">
+      <x:c r="J31" s="32" t="str">
         <x:v>Queue exhausted</x:v>
       </x:c>
-      <x:c r="K30" s="32" t="str">
+      <x:c r="K31" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
-      <x:c r="L30" s="32" t="n">
+      <x:c r="L31" s="32" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="M30" s="32" t="n">
+      <x:c r="M31" s="32" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="N30" s="32" t="n">
+      <x:c r="N31" s="32" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="O30" s="32" t="str">
+      <x:c r="O31" s="32" t="str">
         <x:v>Added after the current audited source queue was exhausted. The first pass across the top-level sections surfaced four clean candidates: protocol.bitcoin-uri-bip21 from Payment Processing, dev.hardened-keys from Wallets, protocol.escrow-and-arbitration from Contracts, and mining.pool-shares from Pool Mining. A follow-up Wallet Files pass surfaced dev.wallet-import-format-wif as another clean wallet-standard slice. The implemented winners are now protocol.bitcoin-uri-bip21, dev.hardened-keys, protocol.escrow-and-arbitration, dev.wallet-import-format-wif, and mining.pool-shares because they land as missing standards, key-derivation, contract-pattern, key-serialization, and pooled-mining accounting bridges with clean direct parents. The current tracked top-level-plus-Wallet-Files queue is exhausted for this pass, though future deeper section splits may still surface more concepts.</x:v>
       </x:c>
     </x:row>
@@ -1439,16 +1486,16 @@
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H30">
+    <x:dataValidation type="list" sqref="H12:H31">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I30">
+    <x:dataValidation type="list" sqref="I12:I31">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J30">
+    <x:dataValidation type="list" sqref="J12:J31">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K30">
+    <x:dataValidation type="list" sqref="K12:K31">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -5340,16 +5387,67 @@
         <x:v>Implemented as the next BOLTs slice after feature flags. BOLT 08 transport, BOLT 10 DNS bootstrap, and already-covered dual funding remain queued or merge/defer candidates.</x:v>
       </x:c>
     </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="32" t="str">
+        <x:v>protocol.strict-der-signatures</x:v>
+      </x:c>
+      <x:c r="B86" s="32" t="str">
+        <x:v>Strict DER Signature Encoding</x:v>
+      </x:c>
+      <x:c r="C86" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D86" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="E86" s="32" t="str">
+        <x:v>https://github.com/bitcoin/bips/blob/master/bip-0066.mediawiki</x:v>
+      </x:c>
+      <x:c r="F86" s="32" t="str">
+        <x:v>BIP 66: Strict DER Signatures</x:v>
+      </x:c>
+      <x:c r="G86" s="32" t="str"/>
+      <x:c r="H86" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I86" s="32" t="str">
+        <x:v>This is one specific deployed consensus rule: legacy ECDSA signatures must use strict DER encoding. It is narrower than digital signatures, Script, and transaction malleability, and it isolates a concrete validation behavior rather than a broad BIP or soft-fork umbrella.</x:v>
+      </x:c>
+      <x:c r="J86" s="32" t="str">
+        <x:v>protocol.script, fundamentals.digital-signatures, protocol.transaction-malleability</x:v>
+      </x:c>
+      <x:c r="K86" s="32" t="str">
+        <x:v>protocol.script</x:v>
+      </x:c>
+      <x:c r="L86" s="32" t="str">
+        <x:v>The Script node already inherits the digital-signature verification path in this graph, so it is the only direct parent needed for strict encoding checks. Transaction malleability is related historical motivation, not a necessary direct parent for understanding the rule itself.</x:v>
+      </x:c>
+      <x:c r="M86" s="32" t="str">
+        <x:v>strict DER, BIP 66, DER-encoded signatures</x:v>
+      </x:c>
+      <x:c r="N86" s="32" t="str">
+        <x:v>consensus, signatures, malleability</x:v>
+      </x:c>
+      <x:c r="O86" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P86" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q86" s="32" t="str">
+        <x:v>Implemented as the first BIPs source-expansion slice. BIP 66 is treated as a specific consensus validation rule, not as a duplicate of transaction malleability or a generic soft-fork node. The direct edge is kept only on protocol.script because the digital-signature path is already inherited.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H85">
+    <x:dataValidation type="list" sqref="H12:H86">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P85">
+    <x:dataValidation type="list" sqref="P12:P86">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -7370,16 +7468,39 @@
         <x:v>Payment onion routing and BOLT12 offers remain related sibling or downstream concepts rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="32" t="str">
+        <x:v>protocol.script</x:v>
+      </x:c>
+      <x:c r="B97" s="32" t="str">
+        <x:v>protocol.strict-der-signatures</x:v>
+      </x:c>
+      <x:c r="C97" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D97" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E97" s="32" t="str">
+        <x:v>Strict DER enforcement occurs while Script validates an ECDSA signature, so learners need the spending-condition and interpreter context first.</x:v>
+      </x:c>
+      <x:c r="F97" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="G97" s="32" t="str">
+        <x:v>Direct edge keeps the rule at the script-validation layer rather than treating BIP 66 as a broad historical upgrade topic.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C96">
+    <x:dataValidation type="list" sqref="C12:C97">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D96">
+    <x:dataValidation type="list" sqref="D12:D97">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9425,16 +9546,42 @@
         <x:v>Added with feature flags and route blinding as direct prerequisites. BOLT 08 Noise transport and BOLT 10 DNS bootstrap remain future source-expansion candidates.</x:v>
       </x:c>
     </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="32" t="str">
+        <x:v>decision.strict-der-signatures-slice</x:v>
+      </x:c>
+      <x:c r="B88" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C88" s="32" t="str">
+        <x:v>protocol.strict-der-signatures</x:v>
+      </x:c>
+      <x:c r="D88" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E88" s="32" t="str">
+        <x:v>BIP 66 describes one deployed consensus validation rule that is absent from the graph: strict DER encoding for legacy ECDSA signatures. It survives dedupe because Script supplies the inherited signature-validation path, while transaction malleability is broader historical motivation rather than the same learning outcome.</x:v>
+      </x:c>
+      <x:c r="F88" s="32" t="str">
+        <x:v>protocol.strict-der-signatures, protocol.script, protocol.transaction-malleability</x:v>
+      </x:c>
+      <x:c r="G88" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="H88" s="32" t="str">
+        <x:v>Added with only protocol.script as a direct prerequisite because the graph already inherits fundamentals.digital-signatures through that path. BIP 66 is kept as the canonical alias and source anchor.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B87">
+    <x:dataValidation type="list" sqref="B12:B88">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D87">
+    <x:dataValidation type="list" sqref="D12:D88">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9487,7 +9634,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.10638196759</x:v>
+        <x:v>46213.10969980324</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -9495,7 +9642,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -9511,7 +9658,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>74</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -9519,7 +9666,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>85</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -9543,7 +9690,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add mempool purging
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rec48526faf9a4d2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R2f814e33807148b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R59ba12c3a4ef48c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R28569f11f58c44a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R0cbeb966797846f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Ra9f26b82db6a4c2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R4c5b4ae8182d42cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R1ef7be5a691a4423"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R48251bd19162455e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R9dace908968f419a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rcdfd183c1ebc4980"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rc8da60d3b36b495a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -965,72 +965,72 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.mempool-space-docs</x:v>
       </x:c>
       <x:c r="B21" s="32" t="str">
-        <x:v>Cypherpunk Library Bitcoin-Adjacent Canon</x:v>
+        <x:v>Mempool.space Documentation</x:v>
       </x:c>
       <x:c r="C21" s="32" t="str">
-        <x:v>https://www.cypherpunkbooks.com/collection</x:v>
+        <x:v>https://mempool.space/docs</x:v>
       </x:c>
       <x:c r="D21" s="32" t="str">
-        <x:v>essay-library</x:v>
+        <x:v>documentation-cluster</x:v>
       </x:c>
       <x:c r="E21" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F21" s="32" t="str">
-        <x:v>Bitcoin-adjacent cypherpunk readings focused on privacy, electronic cash, monetary theory, and the ideological roots most likely to sharpen foundational and history nodes.</x:v>
+        <x:v>Operational documentation for fee visibility, mempool behavior, transaction monitoring, APIs, and self-hosting. Treat it as implementation and observability guidance, not consensus authority.</x:v>
       </x:c>
       <x:c r="G21" s="32" t="str">
-        <x:v>Start with four clusters: cypherpunk manifestos, privacy and surveillance essays, eCash and digital-cash texts, and monetary-theory readings. Defer clearly non-Bitcoin-adjacent political or general-hacker texts unless they surface a direct graph gap.</x:v>
+        <x:v>Enumerate the FAQ, REST API, WebSocket API, and self-hosting/repository clusters first. Use Bitcoin Core documentation as the canonical authority for consensus and policy semantics, then retain Mempool.space-specific observability concepts only when they survive deduplication.</x:v>
       </x:c>
       <x:c r="H21" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>Inventorying</x:v>
       </x:c>
       <x:c r="I21" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="J21" s="32" t="str">
-        <x:v>Queue exhausted</x:v>
+        <x:v>Raw extraction</x:v>
       </x:c>
       <x:c r="K21" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="L21" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="M21" s="32" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N21" s="32" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O21" s="32" t="str">
-        <x:v>Added from user direction. High-signal starting texts from the collection include A Cypherpunk's Manifesto, The Crypto Anarchist Manifesto, Your Secret Right to Cash, Protecting Privacy with Electronic Cash, The Beauty of eCash, The Cyphernomicon, Ideal Money and Asymptotically Ideal Money, and 21 Lessons. Implemented from this source in the current branch: history.chaumian-ecash, privacy.secret-right-to-cash, economics.ideal-money. Merged into existing coverage in the current branch: history.cypherpunks via A Cypherpunk's Manifesto; history.bitcoin-anarchism via The Crypto Anarchist Manifesto. Current tracked cluster queue is exhausted for this pass.</x:v>
+        <x:v>Added during source expansion. Initial clusters cover FAQ/mempool behavior, REST API, WebSocket/live events, and self-hosting. Implemented from this source in the current branch: ops.mempool-purging, with Bitcoin Core policy and RPC documentation used as canonical supporting sources.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="B22" s="32" t="str">
-        <x:v>Bitcoin Dev Project Explained Posts</x:v>
+        <x:v>Cypherpunk Library Bitcoin-Adjacent Canon</x:v>
       </x:c>
       <x:c r="C22" s="32" t="str">
-        <x:v>https://x.com/search?q=from%3ABitcoin_Devs%20explained&amp;src=typed_query&amp;f=live</x:v>
+        <x:v>https://www.cypherpunkbooks.com/collection</x:v>
       </x:c>
       <x:c r="D22" s="32" t="str">
-        <x:v>social-post-cluster</x:v>
+        <x:v>essay-library</x:v>
       </x:c>
       <x:c r="E22" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F22" s="32" t="str">
-        <x:v>Short-form educational posts from @Bitcoin_Devs that explicitly explain protocol, wallet, and Lightning mechanisms in learner-facing language.</x:v>
+        <x:v>Bitcoin-adjacent cypherpunk readings focused on privacy, electronic cash, monetary theory, and the ideological roots most likely to sharpen foundational and history nodes.</x:v>
       </x:c>
       <x:c r="G22" s="32" t="str">
-        <x:v>Track the live X search as one source-family row first, then expand to one row per matching post once current results are enumerated. Group matching posts by concept family such as hashing, fee management, node architecture, channel mechanics, and upgrade proposals.</x:v>
+        <x:v>Start with four clusters: cypherpunk manifestos, privacy and surveillance essays, eCash and digital-cash texts, and monetary-theory readings. Defer clearly non-Bitcoin-adjacent political or general-hacker texts unless they surface a direct graph gap.</x:v>
       </x:c>
       <x:c r="H22" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1045,39 +1045,39 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="L22" s="32" t="n">
-        <x:v>43</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M22" s="32" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N22" s="32" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O22" s="32" t="str">
-        <x:v>Added from user direction. The live X query was enumerated in the logged-in in-app browser on July 8, 2026 and surfaced 43 matching posts. Visible examples include Lamport Signature explained, Duplicate transaction bug explained, 64-byte transaction bug explained, SegWit Address explained, Off-by-one difficulty bug explained, Great Consensus Cleanup explained Part 1: Time Warp Attack, Transaction Pinning explained, Full Node Architecture Explained, MAST explained simply, BIP 158 explained, MuSig explained Simply, CPFP transaction explained, CISA explained, BIP-68 Explained, and Shamir's Secret Sharing explained. Implemented from this source in the current branch: protocol.time-warp-attack, protocol.duplicate-transaction-bug, protocol.64-byte-transaction-bug, fundamentals.lamport-signatures, custody.shamirs-secret-sharing. Merged into existing coverage in the current branch: protocol.time-warp-attack via Off-by-one difficulty bug explained. Current enumerated post queue is exhausted for this pass.</x:v>
+        <x:v>Added from user direction. High-signal starting texts from the collection include A Cypherpunk's Manifesto, The Crypto Anarchist Manifesto, Your Secret Right to Cash, Protecting Privacy with Electronic Cash, The Beauty of eCash, The Cyphernomicon, Ideal Money and Asymptotically Ideal Money, and 21 Lessons. Implemented from this source in the current branch: history.chaumian-ecash, privacy.secret-right-to-cash, economics.ideal-money. Merged into existing coverage in the current branch: history.cypherpunks via A Cypherpunk's Manifesto; history.bitcoin-anarchism via The Crypto Anarchist Manifesto. Current tracked cluster queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-wallet</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="B23" s="32" t="str">
-        <x:v>Bitcoin Core Academy Wallet Internals</x:v>
+        <x:v>Bitcoin Dev Project Explained Posts</x:v>
       </x:c>
       <x:c r="C23" s="32" t="str">
-        <x:v>https://bitcoincore.academy/scriptpubkeymanagers.html</x:v>
+        <x:v>https://x.com/search?q=from%3ABitcoin_Devs%20explained&amp;src=typed_query&amp;f=live</x:v>
       </x:c>
       <x:c r="D23" s="32" t="str">
-        <x:v>course-cluster</x:v>
+        <x:v>social-post-cluster</x:v>
       </x:c>
       <x:c r="E23" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F23" s="32" t="str">
-        <x:v>Wallet internals cluster around ScriptPubKeyManagers, wallet keys, transaction identification, and balance calculation.</x:v>
+        <x:v>Short-form educational posts from @Bitcoin_Devs that explicitly explain protocol, wallet, and Lightning mechanisms in learner-facing language.</x:v>
       </x:c>
       <x:c r="G23" s="32" t="str">
-        <x:v>Track one wallet-internals page cluster at a time so Core-specific abstractions stay atomic instead of collapsing into generic wallet concepts.</x:v>
+        <x:v>Track the live X search as one source-family row first, then expand to one row per matching post once current results are enumerated. Group matching posts by concept family such as hashing, fee management, node architecture, channel mechanics, and upgrade proposals.</x:v>
       </x:c>
       <x:c r="H23" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1092,27 +1092,27 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="L23" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="M23" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="N23" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="O23" s="32" t="str">
-        <x:v>First additional-source pass beyond the mandatory seed list. The current additive winner is dev.scriptpubkeymanagers; wallet-encryption remains deferred because the cleanest surviving slice is still too coupled to missing Core wallet-internals parents. Current tracked wallet-internals queue is exhausted for this pass.</x:v>
+        <x:v>Added from user direction. The live X query was enumerated in the logged-in in-app browser on July 8, 2026 and surfaced 43 matching posts. Visible examples include Lamport Signature explained, Duplicate transaction bug explained, 64-byte transaction bug explained, SegWit Address explained, Off-by-one difficulty bug explained, Great Consensus Cleanup explained Part 1: Time Warp Attack, Transaction Pinning explained, Full Node Architecture Explained, MAST explained simply, BIP 158 explained, MuSig explained Simply, CPFP transaction explained, CISA explained, BIP-68 Explained, and Shamir's Secret Sharing explained. Implemented from this source in the current branch: protocol.time-warp-attack, protocol.duplicate-transaction-bug, protocol.64-byte-transaction-bug, fundamentals.lamport-signatures, custody.shamirs-secret-sharing. Merged into existing coverage in the current branch: protocol.time-warp-attack via Off-by-one difficulty bug explained. Current enumerated post queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-core-academy-wallet</x:v>
       </x:c>
       <x:c r="B24" s="32" t="str">
-        <x:v>Bitcoin Core Academy Mempool Mechanics</x:v>
+        <x:v>Bitcoin Core Academy Wallet Internals</x:v>
       </x:c>
       <x:c r="C24" s="32" t="str">
-        <x:v>https://bitcoincore.academy/mempool-unbroadcast.html</x:v>
+        <x:v>https://bitcoincore.academy/scriptpubkeymanagers.html</x:v>
       </x:c>
       <x:c r="D24" s="32" t="str">
         <x:v>course-cluster</x:v>
@@ -1121,10 +1121,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F24" s="32" t="str">
-        <x:v>Mempool and relay internals cluster around transaction relay, rebroadcast behavior, and local node transaction state.</x:v>
+        <x:v>Wallet internals cluster around ScriptPubKeyManagers, wallet keys, transaction identification, and balance calculation.</x:v>
       </x:c>
       <x:c r="G24" s="32" t="str">
-        <x:v>Track the academy mempool pages as a separate cluster so implementation-specific relay mechanisms are not collapsed into generic mempool coverage.</x:v>
+        <x:v>Track one wallet-internals page cluster at a time so Core-specific abstractions stay atomic instead of collapsing into generic wallet concepts.</x:v>
       </x:c>
       <x:c r="H24" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1145,33 +1145,33 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="N24" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O24" s="32" t="str">
-        <x:v>Second post-seed-source slice. The current additive winners are protocol.mempool-unbroadcast-set, protocol.transaction-rebroadcast-privacy, and protocol.txid-vs-wtxid. The remaining transaction-format internals are now mostly implementation-detail material rather than clean learner-facing nodes. Current tracked mempool queue is exhausted for this pass.</x:v>
+        <x:v>First additional-source pass beyond the mandatory seed list. The current additive winner is dev.scriptpubkeymanagers; wallet-encryption remains deferred because the cleanest surviving slice is still too coupled to missing Core wallet-internals parents. Current tracked wallet-internals queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="str">
-        <x:v>source.bitcoin-design-payment-formats</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="B25" s="32" t="str">
-        <x:v>Bitcoin Design Payment Request Formats</x:v>
+        <x:v>Bitcoin Core Academy Mempool Mechanics</x:v>
       </x:c>
       <x:c r="C25" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/how-it-works/human-readable-addresses/</x:v>
+        <x:v>https://bitcoincore.academy/mempool-unbroadcast.html</x:v>
       </x:c>
       <x:c r="D25" s="32" t="str">
-        <x:v>guide-cluster</x:v>
+        <x:v>course-cluster</x:v>
       </x:c>
       <x:c r="E25" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F25" s="32" t="str">
-        <x:v>User-facing payment request and address-sharing concepts across human-readable addresses, transaction display, and wallet privacy tradeoffs.</x:v>
+        <x:v>Mempool and relay internals cluster around transaction relay, rebroadcast behavior, and local node transaction state.</x:v>
       </x:c>
       <x:c r="G25" s="32" t="str">
-        <x:v>Track design guide pages by UX concept cluster so user-facing payment abstractions stay separate from protocol internals and generic wallet hygiene.</x:v>
+        <x:v>Track the academy mempool pages as a separate cluster so implementation-specific relay mechanisms are not collapsed into generic mempool coverage.</x:v>
       </x:c>
       <x:c r="H25" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1192,21 +1192,21 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="N25" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O25" s="32" t="str">
-        <x:v>First Bitcoin Design implementation slice. The current additive winner is custody.human-readable-addresses; encrypted cloud backups remains the main deferred neighbor from this design source family. Current tracked payment-format queue is exhausted for this pass.</x:v>
+        <x:v>Second post-seed-source slice. The current additive winners are protocol.mempool-unbroadcast-set, protocol.transaction-rebroadcast-privacy, and protocol.txid-vs-wtxid. The remaining transaction-format internals are now mostly implementation-detail material rather than clean learner-facing nodes. Current tracked mempool queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoin-design-payment-formats</x:v>
       </x:c>
       <x:c r="B26" s="32" t="str">
-        <x:v>Bitcoin Design Wallet Activity Context</x:v>
+        <x:v>Bitcoin Design Payment Request Formats</x:v>
       </x:c>
       <x:c r="C26" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/daily-spending-wallet/activity/</x:v>
+        <x:v>https://bitcoin.design/guide/how-it-works/human-readable-addresses/</x:v>
       </x:c>
       <x:c r="D26" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1215,10 +1215,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F26" s="32" t="str">
-        <x:v>User-facing wallet activity, contacts, and contextual payment-history concepts that help learners distinguish on-chain events from wallet-added meaning.</x:v>
+        <x:v>User-facing payment request and address-sharing concepts across human-readable addresses, transaction display, and wallet privacy tradeoffs.</x:v>
       </x:c>
       <x:c r="G26" s="32" t="str">
-        <x:v>Track activity and contacts pages together so contextual metadata stays separate from backup flows and from protocol transaction mechanics.</x:v>
+        <x:v>Track design guide pages by UX concept cluster so user-facing payment abstractions stay separate from protocol internals and generic wallet hygiene.</x:v>
       </x:c>
       <x:c r="H26" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1233,27 +1233,27 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="L26" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="M26" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N26" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="O26" s="32" t="str">
-        <x:v>Second Bitcoin Design implementation slice. The current additive winner is custody.transaction-metadata; encrypted cloud backups remains the main deferred design-side candidate. Current tracked activity-and-contacts queue is exhausted for this pass.</x:v>
+        <x:v>First Bitcoin Design implementation slice. The current additive winner is custody.human-readable-addresses; encrypted cloud backups remains the main deferred neighbor from this design source family. Current tracked payment-format queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="str">
-        <x:v>source.bitcoin-design-multiple-wallets</x:v>
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="B27" s="32" t="str">
-        <x:v>Bitcoin Design Multiple Wallets</x:v>
+        <x:v>Bitcoin Design Wallet Activity Context</x:v>
       </x:c>
       <x:c r="C27" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/multiple-wallets/</x:v>
+        <x:v>https://bitcoin.design/guide/daily-spending-wallet/activity/</x:v>
       </x:c>
       <x:c r="D27" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1262,10 +1262,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F27" s="32" t="str">
-        <x:v>User-facing wallet architecture around separating funds by purpose, ownership, and security model inside one application.</x:v>
+        <x:v>User-facing wallet activity, contacts, and contextual payment-history concepts that help learners distinguish on-chain events from wallet-added meaning.</x:v>
       </x:c>
       <x:c r="G27" s="32" t="str">
-        <x:v>Track the multiple-wallets page separately so purpose-based wallet separation stays distinct from account-path mechanics, backup flows, and generic wallet activity metadata.</x:v>
+        <x:v>Track activity and contacts pages together so contextual metadata stays separate from backup flows and from protocol transaction mechanics.</x:v>
       </x:c>
       <x:c r="H27" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1280,27 +1280,27 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="L27" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M27" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N27" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="O27" s="32" t="str">
-        <x:v>Third Bitcoin Design implementation slice. The current additive winner is custody.multiple-wallets; encrypted cloud backups remains deferred because it overlaps too heavily with backups-recovery. Current tracked page queue is exhausted for this pass.</x:v>
+        <x:v>Second Bitcoin Design implementation slice. The current additive winner is custody.transaction-metadata; encrypted cloud backups remains the main deferred design-side candidate. Current tracked activity-and-contacts queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32" t="str">
-        <x:v>source.bitcoin-design-cloud-backup</x:v>
+        <x:v>source.bitcoin-design-multiple-wallets</x:v>
       </x:c>
       <x:c r="B28" s="32" t="str">
-        <x:v>Bitcoin Design Automatic Cloud Backup</x:v>
+        <x:v>Bitcoin Design Multiple Wallets</x:v>
       </x:c>
       <x:c r="C28" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/how-it-works/private-key-management/cloud-backup/</x:v>
+        <x:v>https://bitcoin.design/guide/multiple-wallets/</x:v>
       </x:c>
       <x:c r="D28" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1309,10 +1309,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F28" s="32" t="str">
-        <x:v>User-facing backup scheme that stores encrypted wallet recovery data with an OS or cloud provider for low-friction restoration.</x:v>
+        <x:v>User-facing wallet architecture around separating funds by purpose, ownership, and security model inside one application.</x:v>
       </x:c>
       <x:c r="G28" s="32" t="str">
-        <x:v>Track the conceptual cloud-backup page, the daily-spending reference flow, and the private-key-management overview together so the scheme can be deduped against existing backup and Lightning recovery coverage.</x:v>
+        <x:v>Track the multiple-wallets page separately so purpose-based wallet separation stays distinct from account-path mechanics, backup flows, and generic wallet activity metadata.</x:v>
       </x:c>
       <x:c r="H28" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1321,13 +1321,13 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J28" s="32" t="str">
-        <x:v>Normalized to existing</x:v>
+        <x:v>Queue exhausted</x:v>
       </x:c>
       <x:c r="K28" s="32" t="str">
-        <x:v>Merged into existing</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L28" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M28" s="32" t="n">
         <x:v>1</x:v>
@@ -1336,18 +1336,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O28" s="32" t="str">
-        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is backup-scheme tradeoffs that already fit custody.backups-recovery plus lightning.channel-backups.</x:v>
+        <x:v>Third Bitcoin Design implementation slice. The current additive winner is custody.multiple-wallets; encrypted cloud backups remains deferred because it overlaps too heavily with backups-recovery. Current tracked page queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoin-design-cloud-backup</x:v>
       </x:c>
       <x:c r="B29" s="32" t="str">
-        <x:v>Bitcoin Design Upgradeable Wallet</x:v>
+        <x:v>Bitcoin Design Automatic Cloud Backup</x:v>
       </x:c>
       <x:c r="C29" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/upgradeable-wallet/</x:v>
+        <x:v>https://bitcoin.design/guide/how-it-works/private-key-management/cloud-backup/</x:v>
       </x:c>
       <x:c r="D29" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1356,10 +1356,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F29" s="32" t="str">
-        <x:v>User-facing wallet architecture for progressive security and staged upgrades between key-management schemes.</x:v>
+        <x:v>User-facing backup scheme that stores encrypted wallet recovery data with an OS or cloud provider for low-friction restoration.</x:v>
       </x:c>
       <x:c r="G29" s="32" t="str">
-        <x:v>Track the upgradeable-wallet reference design separately so progressive security becomes its own concept instead of staying buried inside cloud-backup discussions or multiwallet archival flows.</x:v>
+        <x:v>Track the conceptual cloud-backup page, the daily-spending reference flow, and the private-key-management overview together so the scheme can be deduped against existing backup and Lightning recovery coverage.</x:v>
       </x:c>
       <x:c r="H29" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1368,13 +1368,13 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J29" s="32" t="str">
-        <x:v>Queue exhausted</x:v>
+        <x:v>Normalized to existing</x:v>
       </x:c>
       <x:c r="K29" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>Merged into existing</x:v>
       </x:c>
       <x:c r="L29" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="M29" s="32" t="n">
         <x:v>1</x:v>
@@ -1383,18 +1383,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O29" s="32" t="str">
-        <x:v>Fourth Bitcoin Design implementation slice candidate. The current additive winner is custody.progressive-security, which survives dedupe more cleanly than automatic cloud backups or wallet-encryption. Current tracked page queue is exhausted for this pass.</x:v>
+        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is backup-scheme tradeoffs that already fit custody.backups-recovery plus lightning.channel-backups.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32" t="str">
-        <x:v>source.bitcoin-design-shared-wallet</x:v>
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="B30" s="32" t="str">
-        <x:v>Bitcoin Design Shared Wallet</x:v>
+        <x:v>Bitcoin Design Upgradeable Wallet</x:v>
       </x:c>
       <x:c r="C30" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/shared-wallet/</x:v>
+        <x:v>https://bitcoin.design/guide/upgradeable-wallet/</x:v>
       </x:c>
       <x:c r="D30" s="32" t="str">
         <x:v>guide-cluster</x:v>
@@ -1403,10 +1403,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F30" s="32" t="str">
-        <x:v>Reference design for co-managed wallets using multi-key schemes, provider-held recovery keys, and household approval policies.</x:v>
+        <x:v>User-facing wallet architecture for progressive security and staged upgrades between key-management schemes.</x:v>
       </x:c>
       <x:c r="G30" s="32" t="str">
-        <x:v>Track the shared-wallet page together with the generic multi-key explanation so persona-specific multisig scenarios are deduped against existing custody mechanism nodes.</x:v>
+        <x:v>Track the upgradeable-wallet reference design separately so progressive security becomes its own concept instead of staying buried inside cloud-backup discussions or multiwallet archival flows.</x:v>
       </x:c>
       <x:c r="H30" s="32" t="str">
         <x:v>Complete</x:v>
@@ -1415,13 +1415,13 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J30" s="32" t="str">
-        <x:v>Normalized to existing</x:v>
+        <x:v>Queue exhausted</x:v>
       </x:c>
       <x:c r="K30" s="32" t="str">
-        <x:v>Merged into existing</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L30" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M30" s="32" t="n">
         <x:v>1</x:v>
@@ -1430,53 +1430,100 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O30" s="32" t="str">
-        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is shared-wallet examples for custody.multisig, custody.multiple-wallets, and custody.progressive-security.</x:v>
+        <x:v>Fourth Bitcoin Design implementation slice candidate. The current additive winner is custody.progressive-security, which survives dedupe more cleanly than automatic cloud backups or wallet-encryption. Current tracked page queue is exhausted for this pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.bitcoin-design-shared-wallet</x:v>
       </x:c>
       <x:c r="B31" s="32" t="str">
-        <x:v>Bitcoin Developer Guides</x:v>
+        <x:v>Bitcoin Design Shared Wallet</x:v>
       </x:c>
       <x:c r="C31" s="32" t="str">
-        <x:v>https://developer.bitcoin.org/devguide/</x:v>
+        <x:v>https://bitcoin.design/guide/shared-wallet/</x:v>
       </x:c>
       <x:c r="D31" s="32" t="str">
-        <x:v>documentation-cluster</x:v>
+        <x:v>guide-cluster</x:v>
       </x:c>
       <x:c r="E31" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F31" s="32" t="str">
+        <x:v>Reference design for co-managed wallets using multi-key schemes, provider-held recovery keys, and household approval policies.</x:v>
+      </x:c>
+      <x:c r="G31" s="32" t="str">
+        <x:v>Track the shared-wallet page together with the generic multi-key explanation so persona-specific multisig scenarios are deduped against existing custody mechanism nodes.</x:v>
+      </x:c>
+      <x:c r="H31" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I31" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J31" s="32" t="str">
+        <x:v>Normalized to existing</x:v>
+      </x:c>
+      <x:c r="K31" s="32" t="str">
+        <x:v>Merged into existing</x:v>
+      </x:c>
+      <x:c r="L31" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M31" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N31" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O31" s="32" t="str">
+        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is shared-wallet examples for custody.multisig, custody.multiple-wallets, and custody.progressive-security.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="32" t="str">
+        <x:v>source.bitcoin-developer-guides</x:v>
+      </x:c>
+      <x:c r="B32" s="32" t="str">
+        <x:v>Bitcoin Developer Guides</x:v>
+      </x:c>
+      <x:c r="C32" s="32" t="str">
+        <x:v>https://developer.bitcoin.org/devguide/</x:v>
+      </x:c>
+      <x:c r="D32" s="32" t="str">
+        <x:v>documentation-cluster</x:v>
+      </x:c>
+      <x:c r="E32" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F32" s="32" t="str">
         <x:v>Canonical developer-facing guide sections covering block chain, transactions, contracts, wallets, payment processing, operating modes, P2P network, and mining.</x:v>
       </x:c>
-      <x:c r="G31" s="32" t="str">
+      <x:c r="G32" s="32" t="str">
         <x:v>Track the eight top-level guide sections first, then split dense sections like Transactions, Contracts, Wallets, and P2P Network when they expose concept gaps not already covered by existing nodes.</x:v>
       </x:c>
-      <x:c r="H31" s="32" t="str">
+      <x:c r="H32" s="32" t="str">
         <x:v>In review</x:v>
       </x:c>
-      <x:c r="I31" s="32" t="str">
+      <x:c r="I32" s="32" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="J31" s="32" t="str">
+      <x:c r="J32" s="32" t="str">
         <x:v>Queue exhausted</x:v>
       </x:c>
-      <x:c r="K31" s="32" t="str">
+      <x:c r="K32" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
-      <x:c r="L31" s="32" t="n">
+      <x:c r="L32" s="32" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="M31" s="32" t="n">
+      <x:c r="M32" s="32" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="N31" s="32" t="n">
+      <x:c r="N32" s="32" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="O31" s="32" t="str">
+      <x:c r="O32" s="32" t="str">
         <x:v>Added after the current audited source queue was exhausted. The first pass across the top-level sections surfaced four clean candidates: protocol.bitcoin-uri-bip21 from Payment Processing, dev.hardened-keys from Wallets, protocol.escrow-and-arbitration from Contracts, and mining.pool-shares from Pool Mining. A follow-up Wallet Files pass surfaced dev.wallet-import-format-wif as another clean wallet-standard slice. The implemented winners are now protocol.bitcoin-uri-bip21, dev.hardened-keys, protocol.escrow-and-arbitration, dev.wallet-import-format-wif, and mining.pool-shares because they land as missing standards, key-derivation, contract-pattern, key-serialization, and pooled-mining accounting bridges with clean direct parents. The current tracked top-level-plus-Wallet-Files queue is exhausted for this pass, though future deeper section splits may still surface more concepts.</x:v>
       </x:c>
     </x:row>
@@ -1486,16 +1533,16 @@
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H31">
+    <x:dataValidation type="list" sqref="H12:H32">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I31">
+    <x:dataValidation type="list" sqref="I12:I32">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J31">
+    <x:dataValidation type="list" sqref="J12:J32">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K31">
+    <x:dataValidation type="list" sqref="K12:K32">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -5438,16 +5485,67 @@
         <x:v>Implemented as the first BIPs source-expansion slice. BIP 66 is treated as a specific consensus validation rule, not as a duplicate of transaction malleability or a generic soft-fork node. The direct edge is kept only on protocol.script because the digital-signature path is already inherited.</x:v>
       </x:c>
     </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="32" t="str">
+        <x:v>ops.mempool-purging</x:v>
+      </x:c>
+      <x:c r="B87" s="32" t="str">
+        <x:v>Mempool Purging and Rolling Minimum Fee</x:v>
+      </x:c>
+      <x:c r="C87" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D87" s="32" t="str">
+        <x:v>source.mempool-space-docs</x:v>
+      </x:c>
+      <x:c r="E87" s="32" t="str">
+        <x:v>https://mempool.space/docs/faq</x:v>
+      </x:c>
+      <x:c r="F87" s="32" t="str">
+        <x:v>FAQ &gt; stuck transactions, mempool fullness, purging threshold, and rolling minimum fee</x:v>
+      </x:c>
+      <x:c r="G87" s="32" t="str"/>
+      <x:c r="H87" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I87" s="32" t="str">
+        <x:v>This is one specific node-operations behavior: how mempool pressure raises a rolling minimum relay feerate and causes lower-feerate transactions to be evicted. It is narrower than mempool policy, fee markets, package relay, and generic transaction confirmation.</x:v>
+      </x:c>
+      <x:c r="J87" s="32" t="str">
+        <x:v>ops.mempool-policy, protocol.fee-market, protocol.mempool</x:v>
+      </x:c>
+      <x:c r="K87" s="32" t="str">
+        <x:v>ops.mempool-policy</x:v>
+      </x:c>
+      <x:c r="L87" s="32" t="str">
+        <x:v>Mempool policy is the direct conceptual parent for local relay thresholds and eviction. The generic mempool and fee-market concepts are already inherited through that policy path, so adding them directly would be redundant or too broad.</x:v>
+      </x:c>
+      <x:c r="M87" s="32" t="str">
+        <x:v>mempool eviction, rolling minimum fee, mempool purging</x:v>
+      </x:c>
+      <x:c r="N87" s="32" t="str">
+        <x:v>mempool, fees, node-operations</x:v>
+      </x:c>
+      <x:c r="O87" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P87" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q87" s="32" t="str">
+        <x:v>Implemented as the first mempool.space source-expansion slice, with Bitcoin Core policy and getmempoolinfo documentation anchoring the semantics.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H86">
+    <x:dataValidation type="list" sqref="H12:H87">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P86">
+    <x:dataValidation type="list" sqref="P12:P87">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -7491,16 +7589,39 @@
         <x:v>Direct edge keeps the rule at the script-validation layer rather than treating BIP 66 as a broad historical upgrade topic.</x:v>
       </x:c>
     </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="32" t="str">
+        <x:v>ops.mempool-policy</x:v>
+      </x:c>
+      <x:c r="B98" s="32" t="str">
+        <x:v>ops.mempool-purging</x:v>
+      </x:c>
+      <x:c r="C98" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D98" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E98" s="32" t="str">
+        <x:v>Rolling minimum fee escalation and transaction eviction are local consequences of the node's mempool relay policy, so learners need that policy boundary first.</x:v>
+      </x:c>
+      <x:c r="F98" s="32" t="str">
+        <x:v>source.mempool-space-docs</x:v>
+      </x:c>
+      <x:c r="G98" s="32" t="str">
+        <x:v>The generic mempool, fee-market, and consensus-policy branches remain inherited or adjacent rather than direct prerequisites.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C97">
+    <x:dataValidation type="list" sqref="C12:C98">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D97">
+    <x:dataValidation type="list" sqref="D12:D98">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9572,16 +9693,42 @@
         <x:v>Added with only protocol.script as a direct prerequisite because the graph already inherits fundamentals.digital-signatures through that path. BIP 66 is kept as the canonical alias and source anchor.</x:v>
       </x:c>
     </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="32" t="str">
+        <x:v>decision.mempool-purging-slice</x:v>
+      </x:c>
+      <x:c r="B89" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C89" s="32" t="str">
+        <x:v>ops.mempool-purging</x:v>
+      </x:c>
+      <x:c r="D89" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E89" s="32" t="str">
+        <x:v>Mempool.space documentation surfaces an operational behavior missing from the graph: a node's rolling minimum relay fee rises under memory pressure and lower-feerate transactions are evicted. It survives dedupe because mempool policy defines the boundary, while fee markets, package relay, and generic mempool nodes describe adjacent or inherited concepts.</x:v>
+      </x:c>
+      <x:c r="F89" s="32" t="str">
+        <x:v>ops.mempool-purging, ops.mempool-policy, protocol.mempool, protocol.fee-market, protocol.package-relay, ops.peer-eviction-protection</x:v>
+      </x:c>
+      <x:c r="G89" s="32" t="str">
+        <x:v>source.mempool-space-docs</x:v>
+      </x:c>
+      <x:c r="H89" s="32" t="str">
+        <x:v>Added with only ops.mempool-policy as a direct prerequisite. Bitcoin Core policy and RPC documentation are canonical supporting sources; Mempool.space provides the operator-facing observability context.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B88">
+    <x:dataValidation type="list" sqref="B12:B89">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D88">
+    <x:dataValidation type="list" sqref="D12:D89">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9634,7 +9781,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.10969980324</x:v>
+        <x:v>46213.11348497685</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -9642,7 +9789,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -9658,7 +9805,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>75</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -9666,7 +9813,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -9690,7 +9837,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add deterministic multisig key sorting
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R4c5b4ae8182d42cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R1ef7be5a691a4423"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R48251bd19162455e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R9dace908968f419a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rcdfd183c1ebc4980"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rc8da60d3b36b495a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Ra24e338018ba4927"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R696139d51f8e405b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R55f7c335413243eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rbbe5e5afbd49416a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rd90c624677fe44ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R8ec52dca94304b16"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -954,13 +954,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M20" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N20" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="O20" s="32" t="str">
-        <x:v>Added during source expansion. Initial inventory covers the registry/process, consensus soft forks, signature encoding and serialization, script/output templates, wallet/payment standards, and peer/relay clusters. Implemented from this source in the current branch: protocol.strict-der-signatures.</x:v>
+        <x:v>Added during source expansion. Initial inventory covers the registry/process, consensus soft forks, signature encoding and serialization, script/output templates, wallet/payment standards, and peer/relay clusters. Implemented from this source in the current branch: protocol.strict-der-signatures and custody.deterministic-multisig-key-sorting.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -5487,52 +5487,103 @@
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="32" t="str">
-        <x:v>ops.mempool-purging</x:v>
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
       </x:c>
       <x:c r="B87" s="32" t="str">
-        <x:v>Mempool Purging and Rolling Minimum Fee</x:v>
+        <x:v>Deterministic Multisig Key Sorting</x:v>
       </x:c>
       <x:c r="C87" s="32" t="str">
-        <x:v>Network, Relay &amp; Client Sync</x:v>
+        <x:v>Wallets</x:v>
       </x:c>
       <x:c r="D87" s="32" t="str">
-        <x:v>source.mempool-space-docs</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="E87" s="32" t="str">
-        <x:v>https://mempool.space/docs/faq</x:v>
+        <x:v>https://github.com/bitcoin/bips/blob/master/bip-0067.mediawiki</x:v>
       </x:c>
       <x:c r="F87" s="32" t="str">
-        <x:v>FAQ &gt; stuck transactions, mempool fullness, purging threshold, and rolling minimum fee</x:v>
+        <x:v>BIP 67 &gt; deterministic sorting of compressed public keys in multisig redeem scripts</x:v>
       </x:c>
       <x:c r="G87" s="32" t="str"/>
       <x:c r="H87" s="32" t="str">
         <x:v>new</x:v>
       </x:c>
       <x:c r="I87" s="32" t="str">
-        <x:v>This is one specific node-operations behavior: how mempool pressure raises a rolling minimum relay feerate and causes lower-feerate transactions to be evicted. It is narrower than mempool policy, fee markets, package relay, and generic transaction confirmation.</x:v>
+        <x:v>This isolates one interoperability convention: sorting compressed public keys before constructing a multisig script. It is narrower than multisig generally and distinct from P2SH, which supplies the script-hash wrapper rather than the signer-ordering rule.</x:v>
       </x:c>
       <x:c r="J87" s="32" t="str">
-        <x:v>ops.mempool-policy, protocol.fee-market, protocol.mempool</x:v>
+        <x:v>custody.multisig, protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="K87" s="32" t="str">
-        <x:v>ops.mempool-policy</x:v>
+        <x:v>custody.multisig, protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="L87" s="32" t="str">
-        <x:v>Mempool policy is the direct conceptual parent for local relay thresholds and eviction. The generic mempool and fee-market concepts are already inherited through that policy path, so adding them directly would be redundant or too broad.</x:v>
+        <x:v>Learners need the signer-policy model and the P2SH script-hash context before the deterministic key-ordering convention is useful for wallet interoperability. The shared Script ancestor is inherited and should not be added directly.</x:v>
       </x:c>
       <x:c r="M87" s="32" t="str">
-        <x:v>mempool eviction, rolling minimum fee, mempool purging</x:v>
+        <x:v>BIP 67, sorted multisig keys, deterministic multisig</x:v>
       </x:c>
       <x:c r="N87" s="32" t="str">
-        <x:v>mempool, fees, node-operations</x:v>
+        <x:v>wallets, multisig, standards, interoperability</x:v>
       </x:c>
       <x:c r="O87" s="32" t="str">
-        <x:v>35m</x:v>
+        <x:v>25m</x:v>
       </x:c>
       <x:c r="P87" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q87" s="32" t="str">
+        <x:v>Selected from the BIPs wallet/payment standards cluster after deduping against multisig itself, P2SH, and broader wallet address conventions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="32" t="str">
+        <x:v>ops.mempool-purging</x:v>
+      </x:c>
+      <x:c r="B88" s="32" t="str">
+        <x:v>Mempool Purging and Rolling Minimum Fee</x:v>
+      </x:c>
+      <x:c r="C88" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D88" s="32" t="str">
+        <x:v>source.mempool-space-docs</x:v>
+      </x:c>
+      <x:c r="E88" s="32" t="str">
+        <x:v>https://mempool.space/docs/faq</x:v>
+      </x:c>
+      <x:c r="F88" s="32" t="str">
+        <x:v>FAQ &gt; stuck transactions, mempool fullness, purging threshold, and rolling minimum fee</x:v>
+      </x:c>
+      <x:c r="G88" s="32" t="str"/>
+      <x:c r="H88" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I88" s="32" t="str">
+        <x:v>This is one specific node-operations behavior: how mempool pressure raises a rolling minimum relay feerate and causes lower-feerate transactions to be evicted. It is narrower than mempool policy, fee markets, package relay, and generic transaction confirmation.</x:v>
+      </x:c>
+      <x:c r="J88" s="32" t="str">
+        <x:v>ops.mempool-policy, protocol.fee-market, protocol.mempool</x:v>
+      </x:c>
+      <x:c r="K88" s="32" t="str">
+        <x:v>ops.mempool-policy</x:v>
+      </x:c>
+      <x:c r="L88" s="32" t="str">
+        <x:v>Mempool policy is the direct conceptual parent for local relay thresholds and eviction. The generic mempool and fee-market concepts are already inherited through that policy path, so adding them directly would be redundant or too broad.</x:v>
+      </x:c>
+      <x:c r="M88" s="32" t="str">
+        <x:v>mempool eviction, rolling minimum fee, mempool purging</x:v>
+      </x:c>
+      <x:c r="N88" s="32" t="str">
+        <x:v>mempool, fees, node-operations</x:v>
+      </x:c>
+      <x:c r="O88" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P88" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q88" s="32" t="str">
         <x:v>Implemented as the first mempool.space source-expansion slice, with Bitcoin Core policy and getmempoolinfo documentation anchoring the semantics.</x:v>
       </x:c>
     </x:row>
@@ -5542,10 +5593,10 @@
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H87">
+    <x:dataValidation type="list" sqref="H12:H88">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P87">
+    <x:dataValidation type="list" sqref="P12:P88">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -7591,10 +7642,10 @@
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="32" t="str">
-        <x:v>ops.mempool-policy</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B98" s="32" t="str">
-        <x:v>ops.mempool-purging</x:v>
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
       </x:c>
       <x:c r="C98" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -7603,12 +7654,58 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E98" s="32" t="str">
+        <x:v>The node builds on the wallet-level threshold signer policy before specifying a deterministic ordering convention for the signer keys.</x:v>
+      </x:c>
+      <x:c r="F98" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="G98" s="32" t="str">
+        <x:v>Direct edge preserves the distinction between multisig policy and the BIP 67 interoperability rule.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="32" t="str">
+        <x:v>protocol.pay-to-script-hash</x:v>
+      </x:c>
+      <x:c r="B99" s="32" t="str">
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+      </x:c>
+      <x:c r="C99" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D99" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E99" s="32" t="str">
+        <x:v>BIP 67 is commonly applied when constructing the redeem script whose hash is committed by P2SH, so the script-hash wrapper provides the output context.</x:v>
+      </x:c>
+      <x:c r="F99" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="G99" s="32" t="str">
+        <x:v>The shared protocol.script ancestor remains inherited rather than a redundant direct edge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="32" t="str">
+        <x:v>ops.mempool-policy</x:v>
+      </x:c>
+      <x:c r="B100" s="32" t="str">
+        <x:v>ops.mempool-purging</x:v>
+      </x:c>
+      <x:c r="C100" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D100" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E100" s="32" t="str">
         <x:v>Rolling minimum fee escalation and transaction eviction are local consequences of the node's mempool relay policy, so learners need that policy boundary first.</x:v>
       </x:c>
-      <x:c r="F98" s="32" t="str">
+      <x:c r="F100" s="32" t="str">
         <x:v>source.mempool-space-docs</x:v>
       </x:c>
-      <x:c r="G98" s="32" t="str">
+      <x:c r="G100" s="32" t="str">
         <x:v>The generic mempool, fee-market, and consensus-policy branches remain inherited or adjacent rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
@@ -7618,10 +7715,10 @@
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C98">
+    <x:dataValidation type="list" sqref="C12:C100">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D98">
+    <x:dataValidation type="list" sqref="D12:D100">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9719,16 +9816,42 @@
         <x:v>Added with only ops.mempool-policy as a direct prerequisite. Bitcoin Core policy and RPC documentation are canonical supporting sources; Mempool.space provides the operator-facing observability context.</x:v>
       </x:c>
     </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="32" t="str">
+        <x:v>decision.deterministic-multisig-key-sorting-slice</x:v>
+      </x:c>
+      <x:c r="B90" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C90" s="32" t="str">
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+      </x:c>
+      <x:c r="D90" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E90" s="32" t="str">
+        <x:v>BIP 67 names one missing interoperability rule: sort compressed public keys before constructing a multisig script so independent wallets agree on the same redeem script and address. It survives dedupe because multisig describes the signer policy and P2SH describes the script-hash wrapper, not the deterministic ordering convention.</x:v>
+      </x:c>
+      <x:c r="F90" s="32" t="str">
+        <x:v>custody.deterministic-multisig-key-sorting, custody.multisig, protocol.pay-to-script-hash, protocol.script</x:v>
+      </x:c>
+      <x:c r="G90" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="H90" s="32" t="str">
+        <x:v>Added with custody.multisig and protocol.pay-to-script-hash as direct prerequisites. The shared Script ancestor remains inherited, and the concept is wallet/protocol interoperability rather than Lightning-specific.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B89">
+    <x:dataValidation type="list" sqref="B12:B90">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D89">
+    <x:dataValidation type="list" sqref="D12:D90">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9781,7 +9904,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.11348497685</x:v>
+        <x:v>46213.12081511574</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -9805,7 +9928,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>76</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -9813,7 +9936,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>87</x:v>
+        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -9837,7 +9960,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add Lightning encrypted transport
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Ra24e338018ba4927"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R696139d51f8e405b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R55f7c335413243eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rbbe5e5afbd49416a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rd90c624677fe44ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R8ec52dca94304b16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rb765df4f9df04503"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R49693b4ff8d34357"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R40b6bde3bcd64b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Re27a668c15b04c4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Re592b97b7b124fe3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rb89b71310124475b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -907,13 +907,13 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="M19" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N19" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O19" s="32" t="str">
-        <x:v>Added during source expansion. The first inventory covers the BOLT index plus messaging, peer protocol, onion messaging, encrypted transport, feature negotiation, and DNS bootstrap clusters. Implemented from this source in the current branch: lightning.feature-flags and lightning.onion-messages.</x:v>
+        <x:v>Added during source expansion. The first inventory covers the BOLT index plus messaging, peer protocol, onion messaging, encrypted transport, feature negotiation, and DNS bootstrap clusters. Implemented from this source in the current branch: lightning.feature-flags, lightning.onion-messages, and lightning.encrypted-authenticated-transport.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -5436,154 +5436,205 @@
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="32" t="str">
-        <x:v>protocol.strict-der-signatures</x:v>
+        <x:v>lightning.encrypted-authenticated-transport</x:v>
       </x:c>
       <x:c r="B86" s="32" t="str">
-        <x:v>Strict DER Signature Encoding</x:v>
+        <x:v>Lightning Encrypted and Authenticated Transport</x:v>
       </x:c>
       <x:c r="C86" s="32" t="str">
-        <x:v>Protocol &amp; Consensus</x:v>
+        <x:v>Extension Systems</x:v>
       </x:c>
       <x:c r="D86" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="E86" s="32" t="str">
-        <x:v>https://github.com/bitcoin/bips/blob/master/bip-0066.mediawiki</x:v>
+        <x:v>https://github.com/lightning/bolts/blob/master/08-transport.md</x:v>
       </x:c>
       <x:c r="F86" s="32" t="str">
-        <x:v>BIP 66: Strict DER Signatures</x:v>
+        <x:v>BOLT 08: Encrypted and Authenticated Transport &gt; Noise_XK handshake, ECDH key derivation, and ChaCha20-Poly1305 framed transport</x:v>
       </x:c>
       <x:c r="G86" s="32" t="str"/>
       <x:c r="H86" s="32" t="str">
         <x:v>new</x:v>
       </x:c>
       <x:c r="I86" s="32" t="str">
-        <x:v>This is one specific deployed consensus rule: legacy ECDSA signatures must use strict DER encoding. It is narrower than digital signatures, Script, and transaction malleability, and it isolates a concrete validation behavior rather than a broad BIP or soft-fork umbrella.</x:v>
+        <x:v>This isolates one Lightning wire-transport mechanism: authenticating peer identities, deriving session keys, and encrypting framed messages. It is narrower than generic cryptographic transport and distinct from Bitcoin's BIP324 P2P transport.</x:v>
       </x:c>
       <x:c r="J86" s="32" t="str">
-        <x:v>protocol.script, fundamentals.digital-signatures, protocol.transaction-malleability</x:v>
+        <x:v>fundamentals.public-private-keys, fundamentals.diffie-hellman-key-exchange, protocol.v2-p2p-transport</x:v>
       </x:c>
       <x:c r="K86" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>fundamentals.public-private-keys, fundamentals.diffie-hellman-key-exchange</x:v>
       </x:c>
       <x:c r="L86" s="32" t="str">
-        <x:v>The Script node already inherits the digital-signature verification path in this graph, so it is the only direct parent needed for strict encoding checks. Transaction malleability is related historical motivation, not a necessary direct parent for understanding the rule itself.</x:v>
+        <x:v>Public/private keys supply the long-term identity model and Diffie-Hellman supplies the shared-secret mechanism. Bitcoin P2P v2 transport is a sibling protocol with different peer and wire-context requirements, not a prerequisite for BOLT 08.</x:v>
       </x:c>
       <x:c r="M86" s="32" t="str">
-        <x:v>strict DER, BIP 66, DER-encoded signatures</x:v>
+        <x:v>BOLT 08 transport, Lightning Noise transport, Lightning encrypted transport</x:v>
       </x:c>
       <x:c r="N86" s="32" t="str">
-        <x:v>consensus, signatures, malleability</x:v>
+        <x:v>lightning, transport, encryption, authentication</x:v>
       </x:c>
       <x:c r="O86" s="32" t="str">
-        <x:v>35m</x:v>
+        <x:v>45m</x:v>
       </x:c>
       <x:c r="P86" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q86" s="32" t="str">
-        <x:v>Implemented as the first BIPs source-expansion slice. BIP 66 is treated as a specific consensus validation rule, not as a duplicate of transaction malleability or a generic soft-fork node. The direct edge is kept only on protocol.script because the digital-signature path is already inherited.</x:v>
+        <x:v>Selected as the cleanest remaining P0 BOLTs concept after deduping against protocol.v2-p2p-transport. Keep the Lightning-specific Noise_XK and framing outcome visible rather than collapsing both transports into a generic encryption node.</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="32" t="str">
-        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+        <x:v>protocol.strict-der-signatures</x:v>
       </x:c>
       <x:c r="B87" s="32" t="str">
-        <x:v>Deterministic Multisig Key Sorting</x:v>
+        <x:v>Strict DER Signature Encoding</x:v>
       </x:c>
       <x:c r="C87" s="32" t="str">
-        <x:v>Wallets</x:v>
+        <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D87" s="32" t="str">
         <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="E87" s="32" t="str">
-        <x:v>https://github.com/bitcoin/bips/blob/master/bip-0067.mediawiki</x:v>
+        <x:v>https://github.com/bitcoin/bips/blob/master/bip-0066.mediawiki</x:v>
       </x:c>
       <x:c r="F87" s="32" t="str">
-        <x:v>BIP 67 &gt; deterministic sorting of compressed public keys in multisig redeem scripts</x:v>
+        <x:v>BIP 66: Strict DER Signatures</x:v>
       </x:c>
       <x:c r="G87" s="32" t="str"/>
       <x:c r="H87" s="32" t="str">
         <x:v>new</x:v>
       </x:c>
       <x:c r="I87" s="32" t="str">
-        <x:v>This isolates one interoperability convention: sorting compressed public keys before constructing a multisig script. It is narrower than multisig generally and distinct from P2SH, which supplies the script-hash wrapper rather than the signer-ordering rule.</x:v>
+        <x:v>This is one specific deployed consensus rule: legacy ECDSA signatures must use strict DER encoding. It is narrower than digital signatures, Script, and transaction malleability, and it isolates a concrete validation behavior rather than a broad BIP or soft-fork umbrella.</x:v>
       </x:c>
       <x:c r="J87" s="32" t="str">
-        <x:v>custody.multisig, protocol.pay-to-script-hash</x:v>
+        <x:v>protocol.script, fundamentals.digital-signatures, protocol.transaction-malleability</x:v>
       </x:c>
       <x:c r="K87" s="32" t="str">
-        <x:v>custody.multisig, protocol.pay-to-script-hash</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="L87" s="32" t="str">
-        <x:v>Learners need the signer-policy model and the P2SH script-hash context before the deterministic key-ordering convention is useful for wallet interoperability. The shared Script ancestor is inherited and should not be added directly.</x:v>
+        <x:v>The Script node already inherits the digital-signature verification path in this graph, so it is the only direct parent needed for strict encoding checks. Transaction malleability is related historical motivation, not a necessary direct parent for understanding the rule itself.</x:v>
       </x:c>
       <x:c r="M87" s="32" t="str">
-        <x:v>BIP 67, sorted multisig keys, deterministic multisig</x:v>
+        <x:v>strict DER, BIP 66, DER-encoded signatures</x:v>
       </x:c>
       <x:c r="N87" s="32" t="str">
-        <x:v>wallets, multisig, standards, interoperability</x:v>
+        <x:v>consensus, signatures, malleability</x:v>
       </x:c>
       <x:c r="O87" s="32" t="str">
-        <x:v>25m</x:v>
+        <x:v>35m</x:v>
       </x:c>
       <x:c r="P87" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q87" s="32" t="str">
-        <x:v>Selected from the BIPs wallet/payment standards cluster after deduping against multisig itself, P2SH, and broader wallet address conventions.</x:v>
+        <x:v>Implemented as the first BIPs source-expansion slice. BIP 66 is treated as a specific consensus validation rule, not as a duplicate of transaction malleability or a generic soft-fork node. The direct edge is kept only on protocol.script because the digital-signature path is already inherited.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="32" t="str">
-        <x:v>ops.mempool-purging</x:v>
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
       </x:c>
       <x:c r="B88" s="32" t="str">
-        <x:v>Mempool Purging and Rolling Minimum Fee</x:v>
+        <x:v>Deterministic Multisig Key Sorting</x:v>
       </x:c>
       <x:c r="C88" s="32" t="str">
-        <x:v>Network, Relay &amp; Client Sync</x:v>
+        <x:v>Wallets</x:v>
       </x:c>
       <x:c r="D88" s="32" t="str">
-        <x:v>source.mempool-space-docs</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="E88" s="32" t="str">
-        <x:v>https://mempool.space/docs/faq</x:v>
+        <x:v>https://github.com/bitcoin/bips/blob/master/bip-0067.mediawiki</x:v>
       </x:c>
       <x:c r="F88" s="32" t="str">
-        <x:v>FAQ &gt; stuck transactions, mempool fullness, purging threshold, and rolling minimum fee</x:v>
+        <x:v>BIP 67 &gt; deterministic sorting of compressed public keys in multisig redeem scripts</x:v>
       </x:c>
       <x:c r="G88" s="32" t="str"/>
       <x:c r="H88" s="32" t="str">
         <x:v>new</x:v>
       </x:c>
       <x:c r="I88" s="32" t="str">
-        <x:v>This is one specific node-operations behavior: how mempool pressure raises a rolling minimum relay feerate and causes lower-feerate transactions to be evicted. It is narrower than mempool policy, fee markets, package relay, and generic transaction confirmation.</x:v>
+        <x:v>This isolates one interoperability convention: sorting compressed public keys before constructing a multisig script. It is narrower than multisig generally and distinct from P2SH, which supplies the script-hash wrapper rather than the signer-ordering rule.</x:v>
       </x:c>
       <x:c r="J88" s="32" t="str">
-        <x:v>ops.mempool-policy, protocol.fee-market, protocol.mempool</x:v>
+        <x:v>custody.multisig, protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="K88" s="32" t="str">
-        <x:v>ops.mempool-policy</x:v>
+        <x:v>custody.multisig, protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="L88" s="32" t="str">
-        <x:v>Mempool policy is the direct conceptual parent for local relay thresholds and eviction. The generic mempool and fee-market concepts are already inherited through that policy path, so adding them directly would be redundant or too broad.</x:v>
+        <x:v>Learners need the signer-policy model and the P2SH script-hash context before the deterministic key-ordering convention is useful for wallet interoperability. The shared Script ancestor is inherited and should not be added directly.</x:v>
       </x:c>
       <x:c r="M88" s="32" t="str">
-        <x:v>mempool eviction, rolling minimum fee, mempool purging</x:v>
+        <x:v>BIP 67, sorted multisig keys, deterministic multisig</x:v>
       </x:c>
       <x:c r="N88" s="32" t="str">
-        <x:v>mempool, fees, node-operations</x:v>
+        <x:v>wallets, multisig, standards, interoperability</x:v>
       </x:c>
       <x:c r="O88" s="32" t="str">
-        <x:v>35m</x:v>
+        <x:v>25m</x:v>
       </x:c>
       <x:c r="P88" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q88" s="32" t="str">
+        <x:v>Selected from the BIPs wallet/payment standards cluster after deduping against multisig itself, P2SH, and broader wallet address conventions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="32" t="str">
+        <x:v>ops.mempool-purging</x:v>
+      </x:c>
+      <x:c r="B89" s="32" t="str">
+        <x:v>Mempool Purging and Rolling Minimum Fee</x:v>
+      </x:c>
+      <x:c r="C89" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D89" s="32" t="str">
+        <x:v>source.mempool-space-docs</x:v>
+      </x:c>
+      <x:c r="E89" s="32" t="str">
+        <x:v>https://mempool.space/docs/faq</x:v>
+      </x:c>
+      <x:c r="F89" s="32" t="str">
+        <x:v>FAQ &gt; stuck transactions, mempool fullness, purging threshold, and rolling minimum fee</x:v>
+      </x:c>
+      <x:c r="G89" s="32" t="str"/>
+      <x:c r="H89" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I89" s="32" t="str">
+        <x:v>This is one specific node-operations behavior: how mempool pressure raises a rolling minimum relay feerate and causes lower-feerate transactions to be evicted. It is narrower than mempool policy, fee markets, package relay, and generic transaction confirmation.</x:v>
+      </x:c>
+      <x:c r="J89" s="32" t="str">
+        <x:v>ops.mempool-policy, protocol.fee-market, protocol.mempool</x:v>
+      </x:c>
+      <x:c r="K89" s="32" t="str">
+        <x:v>ops.mempool-policy</x:v>
+      </x:c>
+      <x:c r="L89" s="32" t="str">
+        <x:v>Mempool policy is the direct conceptual parent for local relay thresholds and eviction. The generic mempool and fee-market concepts are already inherited through that policy path, so adding them directly would be redundant or too broad.</x:v>
+      </x:c>
+      <x:c r="M89" s="32" t="str">
+        <x:v>mempool eviction, rolling minimum fee, mempool purging</x:v>
+      </x:c>
+      <x:c r="N89" s="32" t="str">
+        <x:v>mempool, fees, node-operations</x:v>
+      </x:c>
+      <x:c r="O89" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P89" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q89" s="32" t="str">
         <x:v>Implemented as the first mempool.space source-expansion slice, with Bitcoin Core policy and getmempoolinfo documentation anchoring the semantics.</x:v>
       </x:c>
     </x:row>
@@ -5593,10 +5644,10 @@
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H88">
+    <x:dataValidation type="list" sqref="H12:H89">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P88">
+    <x:dataValidation type="list" sqref="P12:P89">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -7619,10 +7670,10 @@
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B97" s="32" t="str">
-        <x:v>protocol.strict-der-signatures</x:v>
+        <x:v>lightning.encrypted-authenticated-transport</x:v>
       </x:c>
       <x:c r="C97" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -7631,21 +7682,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E97" s="32" t="str">
-        <x:v>Strict DER enforcement occurs while Script validates an ECDSA signature, so learners need the spending-condition and interpreter context first.</x:v>
+        <x:v>The Noise_XK handshake authenticates long-term Lightning node identities with public/private key material, so learners need that identity model first.</x:v>
       </x:c>
       <x:c r="F97" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G97" s="32" t="str">
-        <x:v>Direct edge keeps the rule at the script-validation layer rather than treating BIP 66 as a broad historical upgrade topic.</x:v>
+        <x:v>Direct edge keeps identity foundations separate from the session-key derivation mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>fundamentals.diffie-hellman-key-exchange</x:v>
       </x:c>
       <x:c r="B98" s="32" t="str">
-        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+        <x:v>lightning.encrypted-authenticated-transport</x:v>
       </x:c>
       <x:c r="C98" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -7654,21 +7705,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E98" s="32" t="str">
-        <x:v>The node builds on the wallet-level threshold signer policy before specifying a deterministic ordering convention for the signer keys.</x:v>
+        <x:v>BOLT 08 uses elliptic-curve Diffie-Hellman operations to derive shared session secrets, so the key-exchange primitive must be understood first.</x:v>
       </x:c>
       <x:c r="F98" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G98" s="32" t="str">
-        <x:v>Direct edge preserves the distinction between multisig policy and the BIP 67 interoperability rule.</x:v>
+        <x:v>Bitcoin P2P v2 transport remains a related sibling rather than a direct prerequisite because it is a different protocol context.</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="32" t="str">
-        <x:v>protocol.pay-to-script-hash</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B99" s="32" t="str">
-        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+        <x:v>protocol.strict-der-signatures</x:v>
       </x:c>
       <x:c r="C99" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -7677,21 +7728,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E99" s="32" t="str">
-        <x:v>BIP 67 is commonly applied when constructing the redeem script whose hash is committed by P2SH, so the script-hash wrapper provides the output context.</x:v>
+        <x:v>Strict DER enforcement occurs while Script validates an ECDSA signature, so learners need the spending-condition and interpreter context first.</x:v>
       </x:c>
       <x:c r="F99" s="32" t="str">
         <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G99" s="32" t="str">
-        <x:v>The shared protocol.script ancestor remains inherited rather than a redundant direct edge.</x:v>
+        <x:v>Direct edge keeps the rule at the script-validation layer rather than treating BIP 66 as a broad historical upgrade topic.</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="32" t="str">
-        <x:v>ops.mempool-policy</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B100" s="32" t="str">
-        <x:v>ops.mempool-purging</x:v>
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
       </x:c>
       <x:c r="C100" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -7700,12 +7751,58 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E100" s="32" t="str">
+        <x:v>The node builds on the wallet-level threshold signer policy before specifying a deterministic ordering convention for the signer keys.</x:v>
+      </x:c>
+      <x:c r="F100" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="G100" s="32" t="str">
+        <x:v>Direct edge preserves the distinction between multisig policy and the BIP 67 interoperability rule.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="32" t="str">
+        <x:v>protocol.pay-to-script-hash</x:v>
+      </x:c>
+      <x:c r="B101" s="32" t="str">
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+      </x:c>
+      <x:c r="C101" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D101" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E101" s="32" t="str">
+        <x:v>BIP 67 is commonly applied when constructing the redeem script whose hash is committed by P2SH, so the script-hash wrapper provides the output context.</x:v>
+      </x:c>
+      <x:c r="F101" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="G101" s="32" t="str">
+        <x:v>The shared protocol.script ancestor remains inherited rather than a redundant direct edge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" s="32" t="str">
+        <x:v>ops.mempool-policy</x:v>
+      </x:c>
+      <x:c r="B102" s="32" t="str">
+        <x:v>ops.mempool-purging</x:v>
+      </x:c>
+      <x:c r="C102" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D102" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E102" s="32" t="str">
         <x:v>Rolling minimum fee escalation and transaction eviction are local consequences of the node's mempool relay policy, so learners need that policy boundary first.</x:v>
       </x:c>
-      <x:c r="F100" s="32" t="str">
+      <x:c r="F102" s="32" t="str">
         <x:v>source.mempool-space-docs</x:v>
       </x:c>
-      <x:c r="G100" s="32" t="str">
+      <x:c r="G102" s="32" t="str">
         <x:v>The generic mempool, fee-market, and consensus-policy branches remain inherited or adjacent rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
@@ -7715,10 +7812,10 @@
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C100">
+    <x:dataValidation type="list" sqref="C12:C102">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D100">
+    <x:dataValidation type="list" sqref="D12:D102">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9842,16 +9939,42 @@
         <x:v>Added with custody.multisig and protocol.pay-to-script-hash as direct prerequisites. The shared Script ancestor remains inherited, and the concept is wallet/protocol interoperability rather than Lightning-specific.</x:v>
       </x:c>
     </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="32" t="str">
+        <x:v>decision.lightning-encrypted-authenticated-transport-slice</x:v>
+      </x:c>
+      <x:c r="B91" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C91" s="32" t="str">
+        <x:v>lightning.encrypted-authenticated-transport</x:v>
+      </x:c>
+      <x:c r="D91" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E91" s="32" t="str">
+        <x:v>BOLT 08 exposes a missing Lightning transport mechanism: Noise_XK identity authentication, ECDH-derived session keys, and authenticated encryption for framed peer messages. It survives dedupe because BIP324 covers Bitcoin node transport in a different peer and wire context.</x:v>
+      </x:c>
+      <x:c r="F91" s="32" t="str">
+        <x:v>lightning.encrypted-authenticated-transport, protocol.v2-p2p-transport, fundamentals.public-private-keys, fundamentals.diffie-hellman-key-exchange</x:v>
+      </x:c>
+      <x:c r="G91" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="H91" s="32" t="str">
+        <x:v>Added with only the identity and key-exchange foundations as direct prerequisites. Keep BOLT 08 and BIP324 as sibling transport nodes rather than collapsing them into generic encrypted transport.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B90">
+    <x:dataValidation type="list" sqref="B12:B91">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D90">
+    <x:dataValidation type="list" sqref="D12:D91">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9904,7 +10027,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.12081511574</x:v>
+        <x:v>46213.12857259259</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -9928,7 +10051,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>77</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -9936,7 +10059,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -9960,7 +10083,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add generic signed messages
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rb765df4f9df04503"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R49693b4ff8d34357"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R40b6bde3bcd64b38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Re27a668c15b04c4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Re592b97b7b124fe3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rb89b71310124475b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R7fce925355fc4f1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rf596c50749d34550"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rce5f04c32e8449f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R54e2b5f1a2d84aa5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R6cb8931969684921"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R149b3eef9331481f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -954,13 +954,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M20" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N20" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O20" s="32" t="str">
-        <x:v>Added during source expansion. Initial inventory covers the registry/process, consensus soft forks, signature encoding and serialization, script/output templates, wallet/payment standards, and peer/relay clusters. Implemented from this source in the current branch: protocol.strict-der-signatures and custody.deterministic-multisig-key-sorting.</x:v>
+        <x:v>Added during source expansion. Initial inventory covers the registry/process, consensus soft forks, signature encoding and serialization, script/output templates, wallet/payment standards, and peer/relay clusters. Implemented from this source in the current branch: protocol.strict-der-signatures, custody.deterministic-multisig-key-sorting, and protocol.generic-signed-messages.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -5638,16 +5638,67 @@
         <x:v>Implemented as the first mempool.space source-expansion slice, with Bitcoin Core policy and getmempoolinfo documentation anchoring the semantics.</x:v>
       </x:c>
     </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="32" t="str">
+        <x:v>protocol.generic-signed-messages</x:v>
+      </x:c>
+      <x:c r="B90" s="32" t="str">
+        <x:v>Generic Signed Message Format</x:v>
+      </x:c>
+      <x:c r="C90" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D90" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="E90" s="32" t="str">
+        <x:v>https://github.com/bitcoin/bips/blob/master/bip-0322.mediawiki</x:v>
+      </x:c>
+      <x:c r="F90" s="32" t="str">
+        <x:v>BIP 322: Generic Signed Message Format</x:v>
+      </x:c>
+      <x:c r="G90" s="32" t="str"/>
+      <x:c r="H90" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I90" s="32" t="str">
+        <x:v>This isolates one interoperability format: proving that a signer can satisfy a Bitcoin scriptPubKey for a message through virtual transactions. It is narrower than Script, digital signatures, PSBT, Taproot, and Scriptless Scripts because those describe the execution substrate, signing workflow, script variants, or broader construction family rather than the generic message format itself.</x:v>
+      </x:c>
+      <x:c r="J90" s="32" t="str">
+        <x:v>protocol.script, fundamentals.digital-signatures, custody.psbt, fundamentals.schnorr-signatures, protocol.taproot</x:v>
+      </x:c>
+      <x:c r="K90" s="32" t="str">
+        <x:v>protocol.script</x:v>
+      </x:c>
+      <x:c r="L90" s="32" t="str">
+        <x:v>BIP 322 is defined around satisfying an output script, so Script is the only direct prerequisite. Digital signatures are already inherited through the Script branch, while PSBT, Schnorr, and Taproot are variant-specific or related signing contexts rather than requirements for understanding the generic format.</x:v>
+      </x:c>
+      <x:c r="M90" s="32" t="str">
+        <x:v>BIP 322, BIP322, generic signed messages, Bitcoin signed message format</x:v>
+      </x:c>
+      <x:c r="N90" s="32" t="str">
+        <x:v>signatures, messages, script, interoperability</x:v>
+      </x:c>
+      <x:c r="O90" s="32" t="str">
+        <x:v>45m</x:v>
+      </x:c>
+      <x:c r="P90" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q90" s="32" t="str">
+        <x:v>Added after deduping against Script, digital signatures, PSBT, Taproot, OP_CHECKSIGFROMSTACK, and the cross-domain Scriptless Scripts umbrella.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H89">
+    <x:dataValidation type="list" sqref="H12:H90">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P89">
+    <x:dataValidation type="list" sqref="P12:P90">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -7806,16 +7857,39 @@
         <x:v>The generic mempool, fee-market, and consensus-policy branches remain inherited or adjacent rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
+    <x:row r="103">
+      <x:c r="A103" s="32" t="str">
+        <x:v>protocol.script</x:v>
+      </x:c>
+      <x:c r="B103" s="32" t="str">
+        <x:v>protocol.generic-signed-messages</x:v>
+      </x:c>
+      <x:c r="C103" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D103" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E103" s="32" t="str">
+        <x:v>BIP 322 proves message authorization by constructing virtual transactions that satisfy a Bitcoin output script, so learners need the Script spending-condition model first.</x:v>
+      </x:c>
+      <x:c r="F103" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="G103" s="32" t="str">
+        <x:v>The digital-signature path is inherited through Script; PSBT, Schnorr, and Taproot remain related variants rather than redundant direct edges.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C102">
+    <x:dataValidation type="list" sqref="C12:C103">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D102">
+    <x:dataValidation type="list" sqref="D12:D103">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9965,16 +10039,42 @@
         <x:v>Added with only the identity and key-exchange foundations as direct prerequisites. Keep BOLT 08 and BIP324 as sibling transport nodes rather than collapsing them into generic encrypted transport.</x:v>
       </x:c>
     </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="32" t="str">
+        <x:v>decision.generic-signed-messages-slice</x:v>
+      </x:c>
+      <x:c r="B92" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C92" s="32" t="str">
+        <x:v>protocol.generic-signed-messages</x:v>
+      </x:c>
+      <x:c r="D92" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E92" s="32" t="str">
+        <x:v>BIP 322 exposes a distinct interoperability format missing from the graph: proving that a signer can satisfy an arbitrary Bitcoin scriptPubKey for a message using virtual transactions. It survives dedupe because Script, digital signatures, PSBT, Taproot, OP_CHECKSIGFROMSTACK, and Scriptless Scripts each cover a different substrate, workflow, variant, opcode proposal, or cross-domain construction family.</x:v>
+      </x:c>
+      <x:c r="F92" s="32" t="str">
+        <x:v>protocol.generic-signed-messages, protocol.script, fundamentals.digital-signatures, custody.psbt, fundamentals.schnorr-signatures, protocol.taproot, protocol.op-checksigfromstack, protocol.scriptless-scripts</x:v>
+      </x:c>
+      <x:c r="G92" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="H92" s="32" t="str">
+        <x:v>Added with only protocol.script as the direct prerequisite. Variant-specific PSBT, Schnorr, and Taproot details remain downstream or adjacent rather than being forced into the generic format's prerequisite set.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B91">
+    <x:dataValidation type="list" sqref="B12:B92">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D91">
+    <x:dataValidation type="list" sqref="D12:D92">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10027,7 +10127,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.12857259259</x:v>
+        <x:v>46213.775583807874</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10051,7 +10151,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>78</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10059,7 +10159,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>91</x:v>
+        <x:v>92</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -10083,7 +10183,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>67</x:v>
+        <x:v>68</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add Bitcoin Core RPC access security
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R7fce925355fc4f1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rf596c50749d34550"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rce5f04c32e8449f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R54e2b5f1a2d84aa5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R6cb8931969684921"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R149b3eef9331481f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R4f87ae331ff4474b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R7b368f9e78484041"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R3d60c70b95ef4f31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R4a47315d8c8c46ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rc5812a269fde4932"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rf3350d23f8174b47"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,22 +1527,69 @@
         <x:v>Added after the current audited source queue was exhausted. The first pass across the top-level sections surfaced four clean candidates: protocol.bitcoin-uri-bip21 from Payment Processing, dev.hardened-keys from Wallets, protocol.escrow-and-arbitration from Contracts, and mining.pool-shares from Pool Mining. A follow-up Wallet Files pass surfaced dev.wallet-import-format-wif as another clean wallet-standard slice. The implemented winners are now protocol.bitcoin-uri-bip21, dev.hardened-keys, protocol.escrow-and-arbitration, dev.wallet-import-format-wif, and mining.pool-shares because they land as missing standards, key-derivation, contract-pattern, key-serialization, and pooled-mining accounting bridges with clean direct parents. The current tracked top-level-plus-Wallet-Files queue is exhausted for this pass, though future deeper section splits may still surface more concepts.</x:v>
       </x:c>
     </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="32" t="str">
+        <x:v>source.bitcoin-core-operator-docs</x:v>
+      </x:c>
+      <x:c r="B33" s="32" t="str">
+        <x:v>Bitcoin Core Operator Documentation</x:v>
+      </x:c>
+      <x:c r="C33" s="32" t="str">
+        <x:v>https://github.com/bitcoin/bitcoin/tree/master/doc</x:v>
+      </x:c>
+      <x:c r="D33" s="32" t="str">
+        <x:v>implementation-documentation-cluster</x:v>
+      </x:c>
+      <x:c r="E33" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F33" s="32" t="str">
+        <x:v>Bitcoin Core's operator-facing documentation and configuration references for securing node control surfaces, especially JSON-RPC exposure and credentials.</x:v>
+      </x:c>
+      <x:c r="G33" s="32" t="str">
+        <x:v>Track the JSON-RPC interface security section, bitcoin.conf reference, and implementation configuration paths as one operator-security cluster before splitting distinct access-control or privacy concepts.</x:v>
+      </x:c>
+      <x:c r="H33" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I33" s="32" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="J33" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K33" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L33" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M33" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N33" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O33" s="32" t="str">
+        <x:v>Added after the audited queue surfaced a distinct RPC control-plane security gap. The first inspected cluster covers credentials, rpcbind/rpcallowip exposure, and the implementation path that applies these settings.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H32">
+    <x:dataValidation type="list" sqref="H12:H33">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I32">
+    <x:dataValidation type="list" sqref="I12:I33">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J32">
+    <x:dataValidation type="list" sqref="J12:J33">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K32">
+    <x:dataValidation type="list" sqref="K12:K33">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -5689,16 +5736,67 @@
         <x:v>Added after deduping against Script, digital signatures, PSBT, Taproot, OP_CHECKSIGFROMSTACK, and the cross-domain Scriptless Scripts umbrella.</x:v>
       </x:c>
     </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="32" t="str">
+        <x:v>security.bitcoin-core-rpc-access</x:v>
+      </x:c>
+      <x:c r="B91" s="32" t="str">
+        <x:v>Bitcoin Core RPC Access Security</x:v>
+      </x:c>
+      <x:c r="C91" s="32" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="D91" s="32" t="str">
+        <x:v>source.bitcoin-core-operator-docs</x:v>
+      </x:c>
+      <x:c r="E91" s="32" t="str">
+        <x:v>https://github.com/bitcoin/bitcoin/blob/master/doc/JSON-RPC-interface.md#security</x:v>
+      </x:c>
+      <x:c r="F91" s="32" t="str">
+        <x:v>JSON-RPC Interface &gt; Security, bitcoin.conf RPC settings, and init.cpp configuration handling</x:v>
+      </x:c>
+      <x:c r="G91" s="32" t="str"/>
+      <x:c r="H91" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I91" s="32" t="str">
+        <x:v>This isolates one operational security boundary: safely exposing Bitcoin Core's powerful RPC control plane through authentication and network-access limits. It is narrower than the generic RPC interface and distinct from wallet RPC workflows, transaction preflight, package relay, and general node security.</x:v>
+      </x:c>
+      <x:c r="J91" s="32" t="str">
+        <x:v>dev.bitcoin-core-rpc, ops.run-full-node, security.adversarial-thinking</x:v>
+      </x:c>
+      <x:c r="K91" s="32" t="str">
+        <x:v>dev.bitcoin-core-rpc</x:v>
+      </x:c>
+      <x:c r="L91" s="32" t="str">
+        <x:v>Learners need the RPC interface and its authority before its access boundary can make sense. Full-node operation is already inherited through dev.bitcoin-core-rpc, and adversarial thinking is useful context but not a direct technical requirement for understanding authentication and exposure controls.</x:v>
+      </x:c>
+      <x:c r="M91" s="32" t="str">
+        <x:v>Bitcoin Core RPC security, secure RPC exposure, RPC authentication, rpcauth</x:v>
+      </x:c>
+      <x:c r="N91" s="32" t="str">
+        <x:v>security, rpc, access-control, node-operations</x:v>
+      </x:c>
+      <x:c r="O91" s="32" t="str">
+        <x:v>45m</x:v>
+      </x:c>
+      <x:c r="P91" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q91" s="32" t="str">
+        <x:v>Added after deduping against dev.bitcoin-core-rpc, dev.testmempoolaccept-rpc, wallet RPC nodes, package relay, and general node-security concepts.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H90">
+    <x:dataValidation type="list" sqref="H12:H91">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P90">
+    <x:dataValidation type="list" sqref="P12:P91">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -7880,16 +7978,39 @@
         <x:v>The digital-signature path is inherited through Script; PSBT, Schnorr, and Taproot remain related variants rather than redundant direct edges.</x:v>
       </x:c>
     </x:row>
+    <x:row r="104">
+      <x:c r="A104" s="32" t="str">
+        <x:v>dev.bitcoin-core-rpc</x:v>
+      </x:c>
+      <x:c r="B104" s="32" t="str">
+        <x:v>security.bitcoin-core-rpc-access</x:v>
+      </x:c>
+      <x:c r="C104" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D104" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E104" s="32" t="str">
+        <x:v>RPC access security is the control boundary around Bitcoin Core's programmatic interface, so learners need to understand the interface and its authority before securing exposure to it.</x:v>
+      </x:c>
+      <x:c r="F104" s="32" t="str">
+        <x:v>source.bitcoin-core-operator-docs</x:v>
+      </x:c>
+      <x:c r="G104" s="32" t="str">
+        <x:v>Full-node operation is inherited through dev.bitcoin-core-rpc; wallet RPC and transaction-preflight nodes remain downstream use cases rather than direct parents.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C103">
+    <x:dataValidation type="list" sqref="C12:C104">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D103">
+    <x:dataValidation type="list" sqref="D12:D104">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10065,16 +10186,42 @@
         <x:v>Added with only protocol.script as the direct prerequisite. Variant-specific PSBT, Schnorr, and Taproot details remain downstream or adjacent rather than being forced into the generic format's prerequisite set.</x:v>
       </x:c>
     </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="32" t="str">
+        <x:v>decision.bitcoin-core-rpc-access-security-slice</x:v>
+      </x:c>
+      <x:c r="B93" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C93" s="32" t="str">
+        <x:v>security.bitcoin-core-rpc-access</x:v>
+      </x:c>
+      <x:c r="D93" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E93" s="32" t="str">
+        <x:v>Bitcoin Core's operator documentation exposes a missing learner-facing security boundary: authenticate RPC clients and constrain where the powerful interface can be reached. It survives dedupe because dev.bitcoin-core-rpc describes the interface, testmempoolaccept and wallet RPC nodes describe specific consumers, and package-relay or cluster-mempool describe transaction policy rather than control-plane exposure.</x:v>
+      </x:c>
+      <x:c r="F93" s="32" t="str">
+        <x:v>security.bitcoin-core-rpc-access, dev.bitcoin-core-rpc, dev.testmempoolaccept-rpc, protocol.package-relay, protocol.cluster-mempool</x:v>
+      </x:c>
+      <x:c r="G93" s="32" t="str">
+        <x:v>source.bitcoin-core-operator-docs</x:v>
+      </x:c>
+      <x:c r="H93" s="32" t="str">
+        <x:v>Added with only dev.bitcoin-core-rpc as the direct prerequisite. Cookie/rpcauth credentials and rpcbind/rpcallowip exposure controls stay within one coherent RPC control-boundary concept; later source passes may split them only if a distinct learner outcome emerges.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B92">
+    <x:dataValidation type="list" sqref="B12:B93">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D92">
+    <x:dataValidation type="list" sqref="D12:D93">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10127,7 +10274,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.775583807874</x:v>
+        <x:v>46213.78071633102</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10135,7 +10282,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -10151,7 +10298,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>79</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10159,7 +10306,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>92</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -10183,7 +10330,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>68</x:v>
+        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add submitpackage RPC
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R4f87ae331ff4474b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R7b368f9e78484041"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R3d60c70b95ef4f31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R4a47315d8c8c46ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rc5812a269fde4932"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rf3350d23f8174b47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rf9e76a79928a44c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rb5168c77b41a4b71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R9360889880de4cc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rd01eb2117dac4c67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R47c04ee728d8494f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R269779752ebb4627"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1574,22 +1574,69 @@
         <x:v>Added after the audited queue surfaced a distinct RPC control-plane security gap. The first inspected cluster covers credentials, rpcbind/rpcallowip exposure, and the implementation path that applies these settings.</x:v>
       </x:c>
     </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="32" t="str">
+        <x:v>source.bitcoin-core-package-policy</x:v>
+      </x:c>
+      <x:c r="B34" s="32" t="str">
+        <x:v>Bitcoin Core Package Policy and Admission Documentation</x:v>
+      </x:c>
+      <x:c r="C34" s="32" t="str">
+        <x:v>https://github.com/bitcoin/bitcoin/blob/master/doc/policy/packages.md</x:v>
+      </x:c>
+      <x:c r="D34" s="32" t="str">
+        <x:v>protocol-documentation-cluster</x:v>
+      </x:c>
+      <x:c r="E34" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F34" s="32" t="str">
+        <x:v>Bitcoin Core's package mempool acceptance rules, submitpackage RPC, and release history for local package admission and fee-bumping behavior.</x:v>
+      </x:c>
+      <x:c r="G34" s="32" t="str">
+        <x:v>Track the current submitpackage RPC reference, package-policy specification, and the 26.0 release note that introduced the RPC as one package-admission cluster; keep network package relay and cluster-mempool as deduplicated neighboring concepts.</x:v>
+      </x:c>
+      <x:c r="H34" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I34" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J34" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K34" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L34" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M34" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N34" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O34" s="32" t="str">
+        <x:v>Added after the RPC-security slice. The inspected pages establish submitpackage as a local package-admission mechanism distinct from testmempoolaccept preflight and network package relay.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H33">
+    <x:dataValidation type="list" sqref="H12:H34">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I33">
+    <x:dataValidation type="list" sqref="I12:I34">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J33">
+    <x:dataValidation type="list" sqref="J12:J34">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K33">
+    <x:dataValidation type="list" sqref="K12:K34">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -5787,16 +5834,67 @@
         <x:v>Added after deduping against dev.bitcoin-core-rpc, dev.testmempoolaccept-rpc, wallet RPC nodes, package relay, and general node-security concepts.</x:v>
       </x:c>
     </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="32" t="str">
+        <x:v>dev.submitpackage-rpc</x:v>
+      </x:c>
+      <x:c r="B92" s="32" t="str">
+        <x:v>submitpackage RPC</x:v>
+      </x:c>
+      <x:c r="C92" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D92" s="32" t="str">
+        <x:v>source.bitcoin-core-package-policy</x:v>
+      </x:c>
+      <x:c r="E92" s="32" t="str">
+        <x:v>https://bitcoincore.org/en/doc/31.0.0/rpc/rawtransactions/submitpackage/</x:v>
+      </x:c>
+      <x:c r="F92" s="32" t="str">
+        <x:v>submitpackage RPC reference, package-policy specification, and Bitcoin Core 26.0 release notes</x:v>
+      </x:c>
+      <x:c r="G92" s="32" t="str"/>
+      <x:c r="H92" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I92" s="32" t="str">
+        <x:v>This isolates one developer-facing operation: submitting a transaction package to a local node for package-aware mempool admission and reading the result. It is narrower than package relay, cluster mempool, and package policy generally, and distinct from testmempoolaccept because it attempts local admission rather than only preflighting the package.</x:v>
+      </x:c>
+      <x:c r="J92" s="32" t="str">
+        <x:v>dev.testmempoolaccept-rpc, protocol.package-relay, protocol.cluster-mempool, protocol.cpfp</x:v>
+      </x:c>
+      <x:c r="K92" s="32" t="str">
+        <x:v>dev.testmempoolaccept-rpc</x:v>
+      </x:c>
+      <x:c r="L92" s="32" t="str">
+        <x:v>Learners need the existing RPC preflight workflow before the distinction between testing and submitting a package is useful. Package relay is a network-propagation layer, cluster mempool is an internal policy design, and CPFP is a motivating use case rather than a direct technical requirement.</x:v>
+      </x:c>
+      <x:c r="M92" s="32" t="str">
+        <x:v>submitpackage, submitpackage RPC, local package submission, package mempool submission</x:v>
+      </x:c>
+      <x:c r="N92" s="32" t="str">
+        <x:v>rpc, mempool, packages, fee-bumping</x:v>
+      </x:c>
+      <x:c r="O92" s="32" t="str">
+        <x:v>45m</x:v>
+      </x:c>
+      <x:c r="P92" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q92" s="32" t="str">
+        <x:v>Added after deduping against dev.testmempoolaccept-rpc, protocol.package-relay, protocol.cluster-mempool, and package-CPFP concepts.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H91">
+    <x:dataValidation type="list" sqref="H12:H92">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P91">
+    <x:dataValidation type="list" sqref="P12:P92">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -8001,16 +8099,39 @@
         <x:v>Full-node operation is inherited through dev.bitcoin-core-rpc; wallet RPC and transaction-preflight nodes remain downstream use cases rather than direct parents.</x:v>
       </x:c>
     </x:row>
+    <x:row r="105">
+      <x:c r="A105" s="32" t="str">
+        <x:v>dev.testmempoolaccept-rpc</x:v>
+      </x:c>
+      <x:c r="B105" s="32" t="str">
+        <x:v>dev.submitpackage-rpc</x:v>
+      </x:c>
+      <x:c r="C105" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D105" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E105" s="32" t="str">
+        <x:v>submitpackage is the admission counterpart to the existing testmempoolaccept preflight workflow, so learners need to understand local package checks before attempting submission and interpreting package results.</x:v>
+      </x:c>
+      <x:c r="F105" s="32" t="str">
+        <x:v>source.bitcoin-core-package-policy</x:v>
+      </x:c>
+      <x:c r="G105" s="32" t="str">
+        <x:v>Package relay and cluster mempool remain neighboring concepts rather than direct prerequisites because this node focuses on one local RPC operation.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C104">
+    <x:dataValidation type="list" sqref="C12:C105">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D104">
+    <x:dataValidation type="list" sqref="D12:D105">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10212,16 +10333,42 @@
         <x:v>Added with only dev.bitcoin-core-rpc as the direct prerequisite. Cookie/rpcauth credentials and rpcbind/rpcallowip exposure controls stay within one coherent RPC control-boundary concept; later source passes may split them only if a distinct learner outcome emerges.</x:v>
       </x:c>
     </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="32" t="str">
+        <x:v>decision.submitpackage-rpc-slice</x:v>
+      </x:c>
+      <x:c r="B94" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C94" s="32" t="str">
+        <x:v>dev.submitpackage-rpc</x:v>
+      </x:c>
+      <x:c r="D94" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E94" s="32" t="str">
+        <x:v>Bitcoin Core's package-admission documentation exposes a distinct RPC operation missing from the graph: submitting a package to the local mempool for package-aware validation and admission. It survives dedupe because testmempoolaccept only preflights, package relay describes network propagation, cluster mempool describes an internal policy model, and package policy is the broader rule set rather than the operation itself.</x:v>
+      </x:c>
+      <x:c r="F94" s="32" t="str">
+        <x:v>dev.submitpackage-rpc, dev.testmempoolaccept-rpc, protocol.package-relay, protocol.cluster-mempool, protocol.cpfp</x:v>
+      </x:c>
+      <x:c r="G94" s="32" t="str">
+        <x:v>source.bitcoin-core-package-policy</x:v>
+      </x:c>
+      <x:c r="H94" s="32" t="str">
+        <x:v>Added with only dev.testmempoolaccept-rpc as the direct prerequisite. Keep the local-admission versus network-relay distinction explicit; successful submitpackage does not mean the package propagated.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B93">
+    <x:dataValidation type="list" sqref="B12:B94">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D93">
+    <x:dataValidation type="list" sqref="D12:D94">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10274,7 +10421,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.78071633102</x:v>
+        <x:v>46213.78493686343</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10282,7 +10429,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -10298,7 +10445,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>80</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10306,7 +10453,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>93</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -10330,7 +10477,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add package RBF
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rf9e76a79928a44c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rb5168c77b41a4b71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R9360889880de4cc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rd01eb2117dac4c67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R47c04ee728d8494f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R269779752ebb4627"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R47e56d9e50194448"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Ra7e037b17d5c47f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R411d16a32ff646c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R7b9ef889af814be6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R662ca9b147ae46eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R0490e767fc7a43c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1612,13 +1612,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="M34" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N34" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="O34" s="32" t="str">
-        <x:v>Added after the RPC-security slice. The inspected pages establish submitpackage as a local package-admission mechanism distinct from testmempoolaccept preflight and network package relay.</x:v>
+        <x:v>Added after the RPC-security slice. The inspected pages establish submitpackage as a local package-admission mechanism and package RBF as a distinct replacement rule, separate from testmempoolaccept preflight, network package relay, and cluster-mempool internals.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5885,16 +5885,67 @@
         <x:v>Added after deduping against dev.testmempoolaccept-rpc, protocol.package-relay, protocol.cluster-mempool, and package-CPFP concepts.</x:v>
       </x:c>
     </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="32" t="str">
+        <x:v>protocol.package-rbf</x:v>
+      </x:c>
+      <x:c r="B93" s="32" t="str">
+        <x:v>Package RBF</x:v>
+      </x:c>
+      <x:c r="C93" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D93" s="32" t="str">
+        <x:v>source.bitcoin-core-package-policy</x:v>
+      </x:c>
+      <x:c r="E93" s="32" t="str">
+        <x:v>https://github.com/bitcoin/bitcoin/blob/master/doc/policy/mempool-replacements.md</x:v>
+      </x:c>
+      <x:c r="F93" s="32" t="str">
+        <x:v>Package RBF and 1P1C-topology package replacement in Bitcoin Core policy and wallet integration documentation</x:v>
+      </x:c>
+      <x:c r="G93" s="32" t="str"/>
+      <x:c r="H93" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I93" s="32" t="str">
+        <x:v>This isolates one replacement rule: current Bitcoin Core policy supports limited 1P1C-style replacement of conflicting in-mempool transaction packages when package-level fee, incremental relay, cluster, and feerate-improvement conditions are met. It is narrower than ordinary RBF, package relay, cluster mempool, and submitpackage as an RPC operation.</x:v>
+      </x:c>
+      <x:c r="J93" s="32" t="str">
+        <x:v>protocol.rbf, protocol.package-relay, protocol.cluster-mempool, dev.submitpackage-rpc, protocol.transaction-pinning</x:v>
+      </x:c>
+      <x:c r="K93" s="32" t="str">
+        <x:v>protocol.rbf</x:v>
+      </x:c>
+      <x:c r="L93" s="32" t="str">
+        <x:v>Ordinary RBF supplies the direct replacement-policy model. Package relay describes propagation, cluster mempool describes internal package accounting, submitpackage describes local submission, and transaction pinning is a motivating risk rather than a technical requirement for understanding package replacement rules.</x:v>
+      </x:c>
+      <x:c r="M93" s="32" t="str">
+        <x:v>package RBF, package replace-by-fee, 1P1C package RBF, package replacement</x:v>
+      </x:c>
+      <x:c r="N93" s="32" t="str">
+        <x:v>rbf, mempool, packages, fee-bumping, cluster-mempool</x:v>
+      </x:c>
+      <x:c r="O93" s="32" t="str">
+        <x:v>55m</x:v>
+      </x:c>
+      <x:c r="P93" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q93" s="32" t="str">
+        <x:v>Added after deduping against protocol.rbf, dev.submitpackage-rpc, protocol.package-relay, protocol.cluster-mempool, and transaction-pinning concepts. Current policy scope is limited 1P1C-style package replacement rather than unrestricted package RBF.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H92">
+    <x:dataValidation type="list" sqref="H12:H93">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P92">
+    <x:dataValidation type="list" sqref="P12:P93">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -8122,16 +8173,39 @@
         <x:v>Package relay and cluster mempool remain neighboring concepts rather than direct prerequisites because this node focuses on one local RPC operation.</x:v>
       </x:c>
     </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="32" t="str">
+        <x:v>protocol.rbf</x:v>
+      </x:c>
+      <x:c r="B106" s="32" t="str">
+        <x:v>protocol.package-rbf</x:v>
+      </x:c>
+      <x:c r="C106" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D106" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E106" s="32" t="str">
+        <x:v>Package RBF extends the ordinary replacement-policy model with package-level fee and cluster conditions, so learners need base RBF semantics first.</x:v>
+      </x:c>
+      <x:c r="F106" s="32" t="str">
+        <x:v>source.bitcoin-core-package-policy</x:v>
+      </x:c>
+      <x:c r="G106" s="32" t="str">
+        <x:v>Package relay, cluster mempool, submitpackage, and pinning remain adjacent concepts rather than redundant direct edges.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C105">
+    <x:dataValidation type="list" sqref="C12:C106">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D105">
+    <x:dataValidation type="list" sqref="D12:D106">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10359,16 +10433,42 @@
         <x:v>Added with only dev.testmempoolaccept-rpc as the direct prerequisite. Keep the local-admission versus network-relay distinction explicit; successful submitpackage does not mean the package propagated.</x:v>
       </x:c>
     </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="32" t="str">
+        <x:v>decision.package-rbf-slice</x:v>
+      </x:c>
+      <x:c r="B95" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C95" s="32" t="str">
+        <x:v>protocol.package-rbf</x:v>
+      </x:c>
+      <x:c r="D95" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E95" s="32" t="str">
+        <x:v>Bitcoin Core replacement-policy documentation and the 1P1C wallet guide expose a distinct package-level replacement mechanism missing from the graph: replacing conflicting transaction packages using aggregate fee, incremental relay, cluster, and feerate-improvement rules. It survives dedupe because ordinary RBF is the parent policy, submitpackage is a local admission operation, package relay is network propagation, and cluster mempool is internal package accounting.</x:v>
+      </x:c>
+      <x:c r="F95" s="32" t="str">
+        <x:v>protocol.package-rbf, protocol.rbf, dev.submitpackage-rpc, protocol.package-relay, protocol.cluster-mempool, protocol.transaction-pinning</x:v>
+      </x:c>
+      <x:c r="G95" s="32" t="str">
+        <x:v>source.bitcoin-core-package-policy</x:v>
+      </x:c>
+      <x:c r="H95" s="32" t="str">
+        <x:v>Added with only protocol.rbf as the direct prerequisite. Keep the current limited 1P1C package-RBF scope explicit rather than implying unrestricted package replacement, and keep the concept separate from the submitpackage RPC workflow or general package relay.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B94">
+    <x:dataValidation type="list" sqref="B12:B95">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D94">
+    <x:dataValidation type="list" sqref="D12:D95">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10421,7 +10521,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.78493686343</x:v>
+        <x:v>46213.78944394676</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10445,7 +10545,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>81</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10453,7 +10553,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>94</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -10477,7 +10577,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add getmempoolcluster RPC
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R47e56d9e50194448"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Ra7e037b17d5c47f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R411d16a32ff646c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R7b9ef889af814be6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R662ca9b147ae46eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R0490e767fc7a43c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rd8401310ab8a4dda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rc93ade48e292440c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R46a1781ed3d8475c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Re663d4472f9d4b64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Ree1d48016e3f4346"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Reaa33ecf5af0430c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1621,22 +1621,69 @@
         <x:v>Added after the RPC-security slice. The inspected pages establish submitpackage as a local package-admission mechanism and package RBF as a distinct replacement rule, separate from testmempoolaccept preflight, network package relay, and cluster-mempool internals.</x:v>
       </x:c>
     </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="32" t="str">
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+      </x:c>
+      <x:c r="B35" s="32" t="str">
+        <x:v>Bitcoin Core Cluster Mempool and RPC Documentation</x:v>
+      </x:c>
+      <x:c r="C35" s="32" t="str">
+        <x:v>https://bitcoincore.org/en/doc/31.0.0/rpc/blockchain/getmempoolcluster/</x:v>
+      </x:c>
+      <x:c r="D35" s="32" t="str">
+        <x:v>implementation-documentation-cluster</x:v>
+      </x:c>
+      <x:c r="E35" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F35" s="32" t="str">
+        <x:v>Bitcoin Core's cluster-mempool data model and the getmempoolcluster RPC for inspecting connected transactions, mining order, chunks, fees, and weights.</x:v>
+      </x:c>
+      <x:c r="G35" s="32" t="str">
+        <x:v>Track the getmempoolcluster RPC reference, Bitcoin Core 31.0 release notes, and mempool terminology as one cluster-observability slice; keep the conceptual cluster-mempool model separate from this concrete RPC workflow.</x:v>
+      </x:c>
+      <x:c r="H35" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I35" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J35" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K35" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L35" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M35" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N35" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O35" s="32" t="str">
+        <x:v>Added after the package-RBF slice. The inspected documentation exposes getmempoolcluster as a read-only local observability operation, distinct from cluster-mempool policy, submitpackage admission, package relay, and package replacement.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H34">
+    <x:dataValidation type="list" sqref="H12:H35">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I34">
+    <x:dataValidation type="list" sqref="I12:I35">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J34">
+    <x:dataValidation type="list" sqref="J12:J35">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K34">
+    <x:dataValidation type="list" sqref="K12:K35">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -5936,16 +5983,67 @@
         <x:v>Added after deduping against protocol.rbf, dev.submitpackage-rpc, protocol.package-relay, protocol.cluster-mempool, and transaction-pinning concepts. Current policy scope is limited 1P1C-style package replacement rather than unrestricted package RBF.</x:v>
       </x:c>
     </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="32" t="str">
+        <x:v>dev.getmempoolcluster-rpc</x:v>
+      </x:c>
+      <x:c r="B94" s="32" t="str">
+        <x:v>getmempoolcluster RPC</x:v>
+      </x:c>
+      <x:c r="C94" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D94" s="32" t="str">
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+      </x:c>
+      <x:c r="E94" s="32" t="str">
+        <x:v>https://bitcoincore.org/en/doc/31.0.0/rpc/blockchain/getmempoolcluster/</x:v>
+      </x:c>
+      <x:c r="F94" s="32" t="str">
+        <x:v>getmempoolcluster RPC reference, Bitcoin Core 31.0 cluster-mempool release notes, and mempool terminology</x:v>
+      </x:c>
+      <x:c r="G94" s="32" t="str"/>
+      <x:c r="H94" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I94" s="32" t="str">
+        <x:v>This isolates one developer-facing observation workflow: given an in-mempool transaction, inspect its connected cluster and interpret the mining-ordered chunks, fees, weights, and transactions. It is narrower than the cluster-mempool policy model and distinct from package admission, package relay, and package replacement.</x:v>
+      </x:c>
+      <x:c r="J94" s="32" t="str">
+        <x:v>protocol.cluster-mempool, dev.submitpackage-rpc, protocol.package-rbf, protocol.package-relay</x:v>
+      </x:c>
+      <x:c r="K94" s="32" t="str">
+        <x:v>protocol.cluster-mempool</x:v>
+      </x:c>
+      <x:c r="L94" s="32" t="str">
+        <x:v>The conceptual cluster-mempool model is the direct prerequisite for interpreting connected components, chunks, and mining order. submitpackage is a local admission operation, package RBF is replacement policy, and package relay is network propagation rather than a requirement for reading local cluster state.</x:v>
+      </x:c>
+      <x:c r="M94" s="32" t="str">
+        <x:v>getmempoolcluster, mempool cluster RPC, cluster inspection RPC, mempool chunk ordering</x:v>
+      </x:c>
+      <x:c r="N94" s="32" t="str">
+        <x:v>rpc, mempool, cluster-mempool, packages, mining-order</x:v>
+      </x:c>
+      <x:c r="O94" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P94" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q94" s="32" t="str">
+        <x:v>Added after deduping against protocol.cluster-mempool, dev.submitpackage-rpc, protocol.package-rbf, and protocol.package-relay. This node teaches read-only local cluster inspection, not admission, replacement, or relay.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H93">
+    <x:dataValidation type="list" sqref="H12:H94">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P93">
+    <x:dataValidation type="list" sqref="P12:P94">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -8196,16 +8294,39 @@
         <x:v>Package relay, cluster mempool, submitpackage, and pinning remain adjacent concepts rather than redundant direct edges.</x:v>
       </x:c>
     </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="32" t="str">
+        <x:v>protocol.cluster-mempool</x:v>
+      </x:c>
+      <x:c r="B107" s="32" t="str">
+        <x:v>dev.getmempoolcluster-rpc</x:v>
+      </x:c>
+      <x:c r="C107" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D107" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E107" s="32" t="str">
+        <x:v>The RPC reports a transaction's connected cluster and mining-ordered chunks, so learners need the cluster-mempool model before interpreting its output.</x:v>
+      </x:c>
+      <x:c r="F107" s="32" t="str">
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+      </x:c>
+      <x:c r="G107" s="32" t="str">
+        <x:v>submitpackage, package RBF, and package relay remain neighboring workflows rather than direct prerequisites.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C106">
+    <x:dataValidation type="list" sqref="C12:C107">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D106">
+    <x:dataValidation type="list" sqref="D12:D107">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10459,16 +10580,42 @@
         <x:v>Added with only protocol.rbf as the direct prerequisite. Keep the current limited 1P1C package-RBF scope explicit rather than implying unrestricted package replacement, and keep the concept separate from the submitpackage RPC workflow or general package relay.</x:v>
       </x:c>
     </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="32" t="str">
+        <x:v>decision.getmempoolcluster-rpc-slice</x:v>
+      </x:c>
+      <x:c r="B96" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C96" s="32" t="str">
+        <x:v>dev.getmempoolcluster-rpc</x:v>
+      </x:c>
+      <x:c r="D96" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E96" s="32" t="str">
+        <x:v>Bitcoin Core 31.0 documentation exposes getmempoolcluster as a distinct read-only developer workflow: query an in-mempool transaction and interpret its connected cluster, transaction count, weight, mining-ordered chunks, and chunk fees. It survives dedupe because cluster mempool is the underlying model, submitpackage is local admission, package RBF is replacement policy, and package relay is network propagation.</x:v>
+      </x:c>
+      <x:c r="F96" s="32" t="str">
+        <x:v>dev.getmempoolcluster-rpc, protocol.cluster-mempool, dev.submitpackage-rpc, protocol.package-rbf, protocol.package-relay</x:v>
+      </x:c>
+      <x:c r="G96" s="32" t="str">
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+      </x:c>
+      <x:c r="H96" s="32" t="str">
+        <x:v>Added with only protocol.cluster-mempool as the direct prerequisite. Keep the node focused on interpreting local RPC output rather than teaching cluster design, package admission, replacement, or relay.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B95">
+    <x:dataValidation type="list" sqref="B12:B96">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D95">
+    <x:dataValidation type="list" sqref="D12:D96">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10521,7 +10668,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.78944394676</x:v>
+        <x:v>46213.79564737269</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10529,7 +10676,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -10545,7 +10692,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>82</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10553,7 +10700,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>95</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -10577,7 +10724,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
refactor: merge RPC wrappers into cluster mempool
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rd8401310ab8a4dda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rc93ade48e292440c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R46a1781ed3d8475c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Re663d4472f9d4b64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Ree1d48016e3f4346"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Reaa33ecf5af0430c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R9707cff068614bdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R5dbca2e3d8404f52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Re3cb5ba22f214b41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Raff31df3af634859"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R36357317a2004704"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R63956f31bdaf44e4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1638,10 +1638,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F35" s="32" t="str">
-        <x:v>Bitcoin Core's cluster-mempool data model and the getmempoolcluster RPC for inspecting connected transactions, mining order, chunks, fees, and weights.</x:v>
+        <x:v>Bitcoin Core's cluster-mempool data model and the getmempoolcluster and getmempoolfeeratediagram RPCs for inspecting connected transactions, mining order, chunks, fees, weights, and whole-mempool fee curves.</x:v>
       </x:c>
       <x:c r="G35" s="32" t="str">
-        <x:v>Track the getmempoolcluster RPC reference, Bitcoin Core 31.0 release notes, and mempool terminology as one cluster-observability slice; keep the conceptual cluster-mempool model separate from this concrete RPC workflow.</x:v>
+        <x:v>Track the getmempoolcluster and getmempoolfeeratediagram RPC references, Bitcoin Core 31.0 release notes, mempool terminology, and the two implementation paths as one cluster-observability slice; keep the conceptual cluster-mempool model separate from these concrete RPC workflows.</x:v>
       </x:c>
       <x:c r="H35" s="32" t="str">
         <x:v>In review</x:v>
@@ -1656,16 +1656,16 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="L35" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M35" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N35" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="O35" s="32" t="str">
-        <x:v>Added after the package-RBF slice. The inspected documentation exposes getmempoolcluster as a read-only local observability operation, distinct from cluster-mempool policy, submitpackage admission, package relay, and package replacement.</x:v>
+        <x:v>Added after the package-RBF slice. The inspected documentation exposes getmempoolcluster as per-cluster read-only inspection and getmempoolfeeratediagram as whole-mempool fee-curve inspection. Both are implementation surfaces merged into protocol.cluster-mempool rather than standalone learner nodes; their RPCs remain optional developer references.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6002,12 +6002,14 @@
       <x:c r="F94" s="32" t="str">
         <x:v>getmempoolcluster RPC reference, Bitcoin Core 31.0 cluster-mempool release notes, and mempool terminology</x:v>
       </x:c>
-      <x:c r="G94" s="32" t="str"/>
+      <x:c r="G94" s="32" t="str">
+        <x:v>protocol.cluster-mempool</x:v>
+      </x:c>
       <x:c r="H94" s="32" t="str">
-        <x:v>new</x:v>
+        <x:v>merge</x:v>
       </x:c>
       <x:c r="I94" s="32" t="str">
-        <x:v>This isolates one developer-facing observation workflow: given an in-mempool transaction, inspect its connected cluster and interpret the mining-ordered chunks, fees, weights, and transactions. It is narrower than the cluster-mempool policy model and distinct from package admission, package relay, and package replacement.</x:v>
+        <x:v>This is a concrete diagnostic RPC over the existing cluster-mempool model, not an independent learner-facing prerequisite. The connected-cluster, chunk, fee, and weight ideas belong in protocol.cluster-mempool; the command itself is an optional developer reference.</x:v>
       </x:c>
       <x:c r="J94" s="32" t="str">
         <x:v>protocol.cluster-mempool, dev.submitpackage-rpc, protocol.package-rbf, protocol.package-relay</x:v>
@@ -6016,7 +6018,7 @@
         <x:v>protocol.cluster-mempool</x:v>
       </x:c>
       <x:c r="L94" s="32" t="str">
-        <x:v>The conceptual cluster-mempool model is the direct prerequisite for interpreting connected components, chunks, and mining order. submitpackage is a local admission operation, package RBF is replacement policy, and package relay is network propagation rather than a requirement for reading local cluster state.</x:v>
+        <x:v>Merge into protocol.cluster-mempool rather than create a wrapper node: the model is the learning outcome, while submitpackage is a local admission operation, package RBF is replacement policy, and package relay is network propagation.</x:v>
       </x:c>
       <x:c r="M94" s="32" t="str">
         <x:v>getmempoolcluster, mempool cluster RPC, cluster inspection RPC, mempool chunk ordering</x:v>
@@ -6031,7 +6033,60 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q94" s="32" t="str">
-        <x:v>Added after deduping against protocol.cluster-mempool, dev.submitpackage-rpc, protocol.package-rbf, and protocol.package-relay. This node teaches read-only local cluster inspection, not admission, replacement, or relay.</x:v>
+        <x:v>Do not add a standalone node. Preserve the RPC as an optional resource on protocol.cluster-mempool for developers who need local diagnostics.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="32" t="str">
+        <x:v>dev.getmempoolfeeratediagram-rpc</x:v>
+      </x:c>
+      <x:c r="B95" s="32" t="str">
+        <x:v>getmempoolfeeratediagram RPC</x:v>
+      </x:c>
+      <x:c r="C95" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D95" s="32" t="str">
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+      </x:c>
+      <x:c r="E95" s="32" t="str">
+        <x:v>https://github.com/bitcoin/bitcoin/blob/v31.0/src/rpc/mempool.cpp#L3289-L3364</x:v>
+      </x:c>
+      <x:c r="F95" s="32" t="str">
+        <x:v>Bitcoin Core 31.0 release notes, hidden getmempoolfeeratediagram RPC implementation, and feerate-diagram mempool implementation</x:v>
+      </x:c>
+      <x:c r="G95" s="32" t="str">
+        <x:v>protocol.cluster-mempool</x:v>
+      </x:c>
+      <x:c r="H95" s="32" t="str">
+        <x:v>merge</x:v>
+      </x:c>
+      <x:c r="I95" s="32" t="str">
+        <x:v>This is a concrete diagnostic RPC over the existing cluster-mempool and fee-ordering model, not an independent learner-facing prerequisite. The cumulative fee and sigops-adjusted weight curve can enrich protocol.cluster-mempool, while the command itself remains an optional developer reference.</x:v>
+      </x:c>
+      <x:c r="J95" s="32" t="str">
+        <x:v>protocol.cluster-mempool, dev.getmempoolcluster-rpc, protocol.package-rbf, mining.block-template-selection, ops.mempool-purging</x:v>
+      </x:c>
+      <x:c r="K95" s="32" t="str">
+        <x:v>protocol.cluster-mempool</x:v>
+      </x:c>
+      <x:c r="L95" s="32" t="str">
+        <x:v>Merge into protocol.cluster-mempool rather than create a wrapper node: the cluster-mempool ordering model is the learning outcome, while per-cluster inspection is a sibling workflow, package RBF is a downstream consumer, and mining-template or eviction nodes are separate policy consumers.</x:v>
+      </x:c>
+      <x:c r="M95" s="32" t="str">
+        <x:v>getmempoolfeeratediagram, mempool feerate diagram RPC, whole-mempool feerate diagram</x:v>
+      </x:c>
+      <x:c r="N95" s="32" t="str">
+        <x:v>rpc, mempool, fees, cluster-mempool, mining-order, observability</x:v>
+      </x:c>
+      <x:c r="O95" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P95" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q95" s="32" t="str">
+        <x:v>Do not add a standalone node. Fold the underlying fee-curve vocabulary into protocol.cluster-mempool if needed; keep the hidden RPC as an optional developer reference rather than a graph prerequisite.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6040,10 +6095,10 @@
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H94">
+    <x:dataValidation type="list" sqref="H12:H95">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P94">
+    <x:dataValidation type="list" sqref="P12:P95">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -8294,39 +8349,16 @@
         <x:v>Package relay, cluster mempool, submitpackage, and pinning remain adjacent concepts rather than redundant direct edges.</x:v>
       </x:c>
     </x:row>
-    <x:row r="107">
-      <x:c r="A107" s="32" t="str">
-        <x:v>protocol.cluster-mempool</x:v>
-      </x:c>
-      <x:c r="B107" s="32" t="str">
-        <x:v>dev.getmempoolcluster-rpc</x:v>
-      </x:c>
-      <x:c r="C107" s="32" t="str">
-        <x:v>prerequisite</x:v>
-      </x:c>
-      <x:c r="D107" s="32" t="str">
-        <x:v>proposed</x:v>
-      </x:c>
-      <x:c r="E107" s="32" t="str">
-        <x:v>The RPC reports a transaction's connected cluster and mining-ordered chunks, so learners need the cluster-mempool model before interpreting its output.</x:v>
-      </x:c>
-      <x:c r="F107" s="32" t="str">
-        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
-      </x:c>
-      <x:c r="G107" s="32" t="str">
-        <x:v>submitpackage, package RBF, and package relay remain neighboring workflows rather than direct prerequisites.</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C107">
+    <x:dataValidation type="list" sqref="C12:C106">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D107">
+    <x:dataValidation type="list" sqref="D12:D106">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10585,7 +10617,7 @@
         <x:v>decision.getmempoolcluster-rpc-slice</x:v>
       </x:c>
       <x:c r="B96" s="32" t="str">
-        <x:v>scope</x:v>
+        <x:v>merge</x:v>
       </x:c>
       <x:c r="C96" s="32" t="str">
         <x:v>dev.getmempoolcluster-rpc</x:v>
@@ -10594,7 +10626,7 @@
         <x:v>resolved</x:v>
       </x:c>
       <x:c r="E96" s="32" t="str">
-        <x:v>Bitcoin Core 31.0 documentation exposes getmempoolcluster as a distinct read-only developer workflow: query an in-mempool transaction and interpret its connected cluster, transaction count, weight, mining-ordered chunks, and chunk fees. It survives dedupe because cluster mempool is the underlying model, submitpackage is local admission, package RBF is replacement policy, and package relay is network propagation.</x:v>
+        <x:v>Do not add getmempoolcluster as a first-class node. It is an implementation-specific diagnostic interface over the existing cluster-mempool concept; the learner-facing outcome is understanding connected clusters, chunks, fees, and weights, not memorizing an RPC name.</x:v>
       </x:c>
       <x:c r="F96" s="32" t="str">
         <x:v>dev.getmempoolcluster-rpc, protocol.cluster-mempool, dev.submitpackage-rpc, protocol.package-rbf, protocol.package-relay</x:v>
@@ -10603,7 +10635,59 @@
         <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
       </x:c>
       <x:c r="H96" s="32" t="str">
-        <x:v>Added with only protocol.cluster-mempool as the direct prerequisite. Keep the node focused on interpreting local RPC output rather than teaching cluster design, package admission, replacement, or relay.</x:v>
+        <x:v>Merged into protocol.cluster-mempool. Keep the RPC URL as an optional developer resource, not a prerequisite edge or standalone graph node.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="32" t="str">
+        <x:v>decision.getmempoolfeeratediagram-rpc-slice</x:v>
+      </x:c>
+      <x:c r="B97" s="32" t="str">
+        <x:v>merge</x:v>
+      </x:c>
+      <x:c r="C97" s="32" t="str">
+        <x:v>dev.getmempoolfeeratediagram-rpc</x:v>
+      </x:c>
+      <x:c r="D97" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E97" s="32" t="str">
+        <x:v>Do not add getmempoolfeeratediagram as a first-class node. Its cumulative fee and weight curve is useful vocabulary for the existing cluster-mempool concept, but the hidden RPC is an implementation-specific diagnostic surface rather than a standalone learner gap.</x:v>
+      </x:c>
+      <x:c r="F97" s="32" t="str">
+        <x:v>dev.getmempoolfeeratediagram-rpc, protocol.cluster-mempool, dev.getmempoolcluster-rpc, protocol.package-rbf, mining.block-template-selection, ops.mempool-purging</x:v>
+      </x:c>
+      <x:c r="G97" s="32" t="str">
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+      </x:c>
+      <x:c r="H97" s="32" t="str">
+        <x:v>Merged into protocol.cluster-mempool. Preserve the underlying fee-curve terminology there if it helps advanced learners, without adding a separate RPC wrapper node.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="32" t="str">
+        <x:v>decision.function-wrapper-vs-concept-boundary</x:v>
+      </x:c>
+      <x:c r="B98" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C98" s="32" t="str">
+        <x:v>concept-boundary-heuristic</x:v>
+      </x:c>
+      <x:c r="D98" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E98" s="32" t="str">
+        <x:v>Use function-shaped names as an implementation-detail warning: RPCs and similar command surfaces usually expose an existing learner-facing concept rather than define a new one. Prefer the higher-level noun concept as the graph node and retain the implementation surface as an alias or optional resource when useful.</x:v>
+      </x:c>
+      <x:c r="F98" s="32" t="str">
+        <x:v>protocol.cluster-mempool, dev.getmempoolcluster-rpc, dev.getmempoolfeeratediagram-rpc, protocol.op-cat</x:v>
+      </x:c>
+      <x:c r="G98" s="32" t="str">
+        <x:v>source.bitcoin-core-cluster-mempool-rpc, source.bitcoinops-topics</x:v>
+      </x:c>
+      <x:c r="H98" s="32" t="str">
+        <x:v>This is a heuristic, not a hard naming rule. Review low-level primitives individually: consequential opcodes such as OP_CAT can deserve dedicated nodes when they have a distinct learning outcome, compatibility significance, or important prerequisite chain.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10612,10 +10696,10 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B96">
+    <x:dataValidation type="list" sqref="B12:B98">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D96">
+    <x:dataValidation type="list" sqref="D12:D98">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10668,7 +10752,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.79564737269</x:v>
+        <x:v>46213.80343190972</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10692,7 +10776,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>83</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10700,7 +10784,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>96</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -10724,7 +10808,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>72</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add mempool cluster limits
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R9707cff068614bdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R5dbca2e3d8404f52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Re3cb5ba22f214b41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Raff31df3af634859"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R36357317a2004704"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R63956f31bdaf44e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R4ea2a548a32a4cb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R50c5acac0a3a42c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R3d65adfb92ae4526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R655c988c38f44dbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rff18b4ae65f64fe4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rbcd08c9053db4e01"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1638,10 +1638,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F35" s="32" t="str">
-        <x:v>Bitcoin Core's cluster-mempool data model and the getmempoolcluster and getmempoolfeeratediagram RPCs for inspecting connected transactions, mining order, chunks, fees, weights, and whole-mempool fee curves.</x:v>
+        <x:v>Bitcoin Core's cluster-mempool data model, bounded cluster policy, and related RPCs for inspecting connected transactions, mining order, chunks, fees, weights, and whole-mempool fee curves.</x:v>
       </x:c>
       <x:c r="G35" s="32" t="str">
-        <x:v>Track the getmempoolcluster and getmempoolfeeratediagram RPC references, Bitcoin Core 31.0 release notes, mempool terminology, and the two implementation paths as one cluster-observability slice; keep the conceptual cluster-mempool model separate from these concrete RPC workflows.</x:v>
+        <x:v>Track the getmempoolcluster and getmempoolfeeratediagram RPC references, cluster-limit policy, Bitcoin Core 31.0 release notes, mempool terminology, and implementation paths as one cluster-mempool slice; keep concrete RPC workflows merged into the higher-level concepts.</x:v>
       </x:c>
       <x:c r="H35" s="32" t="str">
         <x:v>In review</x:v>
@@ -1659,13 +1659,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M35" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N35" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O35" s="32" t="str">
-        <x:v>Added after the package-RBF slice. The inspected documentation exposes getmempoolcluster as per-cluster read-only inspection and getmempoolfeeratediagram as whole-mempool fee-curve inspection. Both are implementation surfaces merged into protocol.cluster-mempool rather than standalone learner nodes; their RPCs remain optional developer references.</x:v>
+        <x:v>Added after the package-RBF slice. The inspected documentation exposes two RPC implementation surfaces, both merged into protocol.cluster-mempool, plus a distinct learner-facing policy concept: bounded cluster limits replacing legacy ancestor/descendant limits.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6089,16 +6089,67 @@
         <x:v>Do not add a standalone node. Fold the underlying fee-curve vocabulary into protocol.cluster-mempool if needed; keep the hidden RPC as an optional developer reference rather than a graph prerequisite.</x:v>
       </x:c>
     </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="32" t="str">
+        <x:v>ops.mempool-cluster-limits</x:v>
+      </x:c>
+      <x:c r="B96" s="32" t="str">
+        <x:v>Mempool Cluster Limits</x:v>
+      </x:c>
+      <x:c r="C96" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D96" s="32" t="str">
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+      </x:c>
+      <x:c r="E96" s="32" t="str">
+        <x:v>https://bitcoincore.org/en/releases/31.0/</x:v>
+      </x:c>
+      <x:c r="F96" s="32" t="str">
+        <x:v>Bitcoin Core 31.0 cluster policy limits, configuration, and Optech cluster-mempool explanation</x:v>
+      </x:c>
+      <x:c r="G96" s="32" t="str"/>
+      <x:c r="H96" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I96" s="32" t="str">
+        <x:v>This isolates one operational policy concept: bounded transaction count and aggregate virtual size for each connected mempool cluster. It is distinct from the cluster-mempool data model, package relay, Package RBF, CPFP, TRUC, and generic mempool policy because it explains the concrete limits that keep package and chunk computation tractable.</x:v>
+      </x:c>
+      <x:c r="J96" s="32" t="str">
+        <x:v>protocol.cluster-mempool, ops.mempool-policy, protocol.package-relay, protocol.package-rbf, protocol.cpfp, protocol.version-3-transaction-relay</x:v>
+      </x:c>
+      <x:c r="K96" s="32" t="str">
+        <x:v>protocol.cluster-mempool</x:v>
+      </x:c>
+      <x:c r="L96" s="32" t="str">
+        <x:v>The cluster-mempool model is the direct prerequisite for understanding why connected components need bounded size. Mempool policy is inherited through that node; package relay, Package RBF, CPFP, and TRUC are affected workflows or neighboring mitigations rather than direct prerequisites.</x:v>
+      </x:c>
+      <x:c r="M96" s="32" t="str">
+        <x:v>cluster limits, mempool cluster size limits, cluster transaction limits, ancestor and descendant limit replacement</x:v>
+      </x:c>
+      <x:c r="N96" s="32" t="str">
+        <x:v>mempool, cluster-mempool, policy, packages, cpfp, rbf</x:v>
+      </x:c>
+      <x:c r="O96" s="32" t="str">
+        <x:v>45m</x:v>
+      </x:c>
+      <x:c r="P96" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q96" s="32" t="str">
+        <x:v>Added after deduping against protocol.cluster-mempool, ops.mempool-policy, protocol.package-relay, protocol.package-rbf, protocol.cpfp, and v3 transaction relay. This is a noun-level policy concept rather than an API wrapper.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H95">
+    <x:dataValidation type="list" sqref="H12:H96">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P95">
+    <x:dataValidation type="list" sqref="P12:P96">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -8349,16 +8400,39 @@
         <x:v>Package relay, cluster mempool, submitpackage, and pinning remain adjacent concepts rather than redundant direct edges.</x:v>
       </x:c>
     </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="32" t="str">
+        <x:v>protocol.cluster-mempool</x:v>
+      </x:c>
+      <x:c r="B107" s="32" t="str">
+        <x:v>ops.mempool-cluster-limits</x:v>
+      </x:c>
+      <x:c r="C107" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D107" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E107" s="32" t="str">
+        <x:v>Cluster limits bound connected transaction sets, so learners need the cluster-mempool model before understanding why count and aggregate virtual-size limits replace legacy ancestor/descendant limits.</x:v>
+      </x:c>
+      <x:c r="F107" s="32" t="str">
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+      </x:c>
+      <x:c r="G107" s="32" t="str">
+        <x:v>Package relay, Package RBF, CPFP, and version 3 relay remain affected workflows or neighboring policy mechanisms rather than direct prerequisites.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C106">
+    <x:dataValidation type="list" sqref="C12:C107">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D106">
+    <x:dataValidation type="list" sqref="D12:D107">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10666,27 +10740,53 @@
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="32" t="str">
-        <x:v>decision.function-wrapper-vs-concept-boundary</x:v>
+        <x:v>decision.mempool-cluster-limits-slice</x:v>
       </x:c>
       <x:c r="B98" s="32" t="str">
-        <x:v>scope</x:v>
+        <x:v>bridge-concept</x:v>
       </x:c>
       <x:c r="C98" s="32" t="str">
-        <x:v>concept-boundary-heuristic</x:v>
+        <x:v>ops.mempool-cluster-limits</x:v>
       </x:c>
       <x:c r="D98" s="32" t="str">
         <x:v>resolved</x:v>
       </x:c>
       <x:c r="E98" s="32" t="str">
+        <x:v>Bitcoin Core 31.0 introduces bounded cluster policy limits that replace legacy ancestor and descendant limits. This survives dedupe as a learner-facing node because it explains a concrete operational constraint affecting package admission, CPFP, relay, replacement, and computational tractability, unlike the omitted RPC wrappers.</x:v>
+      </x:c>
+      <x:c r="F98" s="32" t="str">
+        <x:v>ops.mempool-cluster-limits, protocol.cluster-mempool, ops.mempool-policy, protocol.package-relay, protocol.package-rbf, protocol.cpfp</x:v>
+      </x:c>
+      <x:c r="G98" s="32" t="str">
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+      </x:c>
+      <x:c r="H98" s="32" t="str">
+        <x:v>Added with only protocol.cluster-mempool as the direct prerequisite. Keep legacy ancestor/descendant limits, CPFP carve-out, TRUC, and package-RBF as related mechanisms rather than redundant direct edges.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="32" t="str">
+        <x:v>decision.function-wrapper-vs-concept-boundary</x:v>
+      </x:c>
+      <x:c r="B99" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C99" s="32" t="str">
+        <x:v>concept-boundary-heuristic</x:v>
+      </x:c>
+      <x:c r="D99" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E99" s="32" t="str">
         <x:v>Use function-shaped names as an implementation-detail warning: RPCs and similar command surfaces usually expose an existing learner-facing concept rather than define a new one. Prefer the higher-level noun concept as the graph node and retain the implementation surface as an alias or optional resource when useful.</x:v>
       </x:c>
-      <x:c r="F98" s="32" t="str">
+      <x:c r="F99" s="32" t="str">
         <x:v>protocol.cluster-mempool, dev.getmempoolcluster-rpc, dev.getmempoolfeeratediagram-rpc, protocol.op-cat</x:v>
       </x:c>
-      <x:c r="G98" s="32" t="str">
+      <x:c r="G99" s="32" t="str">
         <x:v>source.bitcoin-core-cluster-mempool-rpc, source.bitcoinops-topics</x:v>
       </x:c>
-      <x:c r="H98" s="32" t="str">
+      <x:c r="H99" s="32" t="str">
         <x:v>This is a heuristic, not a hard naming rule. Review low-level primitives individually: consequential opcodes such as OP_CAT can deserve dedicated nodes when they have a distinct learning outcome, compatibility significance, or important prerequisite chain.</x:v>
       </x:c>
     </x:row>
@@ -10696,10 +10796,10 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B98">
+    <x:dataValidation type="list" sqref="B12:B99">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D98">
+    <x:dataValidation type="list" sqref="D12:D99">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10752,7 +10852,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.80343190972</x:v>
+        <x:v>46213.80827922454</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10776,7 +10876,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>84</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10784,7 +10884,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>95</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -10808,7 +10908,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add Lightning DNS seeds
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R4ea2a548a32a4cb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R50c5acac0a3a42c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R3d65adfb92ae4526"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R655c988c38f44dbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rff18b4ae65f64fe4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rbcd08c9053db4e01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R030e6b9785814e9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R8217036c18354d58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rbeb8e6318262464c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rebbe7de4bd704227"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R18035da0963e427b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R0ac3d21009f74bcd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -904,16 +904,16 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="L19" s="32" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="M19" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N19" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="O19" s="32" t="str">
-        <x:v>Added during source expansion. The first inventory covers the BOLT index plus messaging, peer protocol, onion messaging, encrypted transport, feature negotiation, and DNS bootstrap clusters. Implemented from this source in the current branch: lightning.feature-flags, lightning.onion-messages, and lightning.encrypted-authenticated-transport.</x:v>
+        <x:v>Added during source expansion. The first inventory covers the BOLT index plus messaging, peer protocol, onion messaging, encrypted transport, feature negotiation, and DNS bootstrap clusters. Implemented from this source in the current branch: lightning.feature-flags, lightning.onion-messages, lightning.encrypted-authenticated-transport, and lightning.dns-seeds.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -6140,16 +6140,67 @@
         <x:v>Added after deduping against protocol.cluster-mempool, ops.mempool-policy, protocol.package-relay, protocol.package-rbf, protocol.cpfp, and v3 transaction relay. This is a noun-level policy concept rather than an API wrapper.</x:v>
       </x:c>
     </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="32" t="str">
+        <x:v>lightning.dns-seeds</x:v>
+      </x:c>
+      <x:c r="B97" s="32" t="str">
+        <x:v>Lightning DNS Seeds</x:v>
+      </x:c>
+      <x:c r="C97" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D97" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E97" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/10-dns-bootstrap.md</x:v>
+      </x:c>
+      <x:c r="F97" s="32" t="str">
+        <x:v>BOLT 10: DNS Bootstrap and Assisted Node Location</x:v>
+      </x:c>
+      <x:c r="G97" s="32" t="str"/>
+      <x:c r="H97" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I97" s="32" t="str">
+        <x:v>This isolates one Lightning discovery mechanism: DNS-assisted bootstrap and known-peer location using Lightning-specific realms, address-type filters, node-ID queries, and DNS reply records. It is narrower than generic DNS seeding and distinct from gossip's ongoing topology dissemination.</x:v>
+      </x:c>
+      <x:c r="J97" s="32" t="str">
+        <x:v>ops.dns-seeds, lightning.gossip-protocol, ops.peer-discovery, lightning.routing</x:v>
+      </x:c>
+      <x:c r="K97" s="32" t="str">
+        <x:v>ops.dns-seeds, lightning.gossip-protocol</x:v>
+      </x:c>
+      <x:c r="L97" s="32" t="str">
+        <x:v>Generic DNS seeds supply the bootstrap model, while Lightning gossip supplies the network-specific node-discovery context that BOLT 10 supplements. Peer discovery and routing are already inherited through those parents and are not additional direct prerequisites.</x:v>
+      </x:c>
+      <x:c r="M97" s="32" t="str">
+        <x:v>Lightning DNS bootstrap, DNS bootstrap, assisted node location, BOLT 10</x:v>
+      </x:c>
+      <x:c r="N97" s="32" t="str">
+        <x:v>lightning, dns, peer-discovery, networking, gossip</x:v>
+      </x:c>
+      <x:c r="O97" s="32" t="str">
+        <x:v>40m</x:v>
+      </x:c>
+      <x:c r="P97" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q97" s="32" t="str">
+        <x:v>Added after deduping against ops.dns-seeds, lightning.gossip-protocol, peer-discovery, and routing concepts. This is a Lightning protocol mechanism, not a function/API wrapper.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H96">
+    <x:dataValidation type="list" sqref="H12:H97">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P96">
+    <x:dataValidation type="list" sqref="P12:P97">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -8423,16 +8474,62 @@
         <x:v>Package relay, Package RBF, CPFP, and version 3 relay remain affected workflows or neighboring policy mechanisms rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="32" t="str">
+        <x:v>ops.dns-seeds</x:v>
+      </x:c>
+      <x:c r="B108" s="32" t="str">
+        <x:v>lightning.dns-seeds</x:v>
+      </x:c>
+      <x:c r="C108" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D108" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E108" s="32" t="str">
+        <x:v>Lightning DNS seeds specialize the general DNS bootstrap pattern with Lightning-specific query filters and known-peer lookup, so learners need the base DNS-seed model first.</x:v>
+      </x:c>
+      <x:c r="F108" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="G108" s="32" t="str">
+        <x:v>Peer discovery is inherited through ops.dns-seeds; generic Bitcoin P2P bootstrapping remains a parent concept rather than a duplicated edge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="32" t="str">
+        <x:v>lightning.gossip-protocol</x:v>
+      </x:c>
+      <x:c r="B109" s="32" t="str">
+        <x:v>lightning.dns-seeds</x:v>
+      </x:c>
+      <x:c r="C109" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D109" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E109" s="32" t="str">
+        <x:v>BOLT 10 locates Lightning peers and filters results by Lightning address information, so learners need Lightning's node-discovery and gossip context before understanding the assisted-location mechanism.</x:v>
+      </x:c>
+      <x:c r="F109" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="G109" s="32" t="str">
+        <x:v>Lightning routing and generic P2P messages are inherited through gossip rather than added as transitive prerequisites.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C107">
+    <x:dataValidation type="list" sqref="C12:C109">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D107">
+    <x:dataValidation type="list" sqref="D12:D109">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10766,27 +10863,53 @@
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="32" t="str">
-        <x:v>decision.function-wrapper-vs-concept-boundary</x:v>
+        <x:v>decision.lightning-dns-seeds-slice</x:v>
       </x:c>
       <x:c r="B99" s="32" t="str">
         <x:v>scope</x:v>
       </x:c>
       <x:c r="C99" s="32" t="str">
-        <x:v>concept-boundary-heuristic</x:v>
+        <x:v>lightning.dns-seeds</x:v>
       </x:c>
       <x:c r="D99" s="32" t="str">
         <x:v>resolved</x:v>
       </x:c>
       <x:c r="E99" s="32" t="str">
+        <x:v>BOLT 10 exposes a distinct Lightning discovery mechanism absent from the graph: use DNS not only to bootstrap unknown peers but also to locate a known Lightning node by node ID, realm, and address-type filters. It survives dedupe because generic DNS seeds lack Lightning-specific query semantics, while gossip disseminates ongoing topology rather than bootstrapping or assisted lookup.</x:v>
+      </x:c>
+      <x:c r="F99" s="32" t="str">
+        <x:v>lightning.dns-seeds, ops.dns-seeds, lightning.gossip-protocol, ops.peer-discovery, lightning.routing</x:v>
+      </x:c>
+      <x:c r="G99" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="H99" s="32" t="str">
+        <x:v>Added with ops.dns-seeds and lightning.gossip-protocol as the only direct prerequisites. Keep BOLT 10's bootstrap and assisted-location outcome together; node routing is a downstream consumer, not a third direct edge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="32" t="str">
+        <x:v>decision.function-wrapper-vs-concept-boundary</x:v>
+      </x:c>
+      <x:c r="B100" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C100" s="32" t="str">
+        <x:v>concept-boundary-heuristic</x:v>
+      </x:c>
+      <x:c r="D100" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E100" s="32" t="str">
         <x:v>Use function-shaped names as an implementation-detail warning: RPCs and similar command surfaces usually expose an existing learner-facing concept rather than define a new one. Prefer the higher-level noun concept as the graph node and retain the implementation surface as an alias or optional resource when useful.</x:v>
       </x:c>
-      <x:c r="F99" s="32" t="str">
+      <x:c r="F100" s="32" t="str">
         <x:v>protocol.cluster-mempool, dev.getmempoolcluster-rpc, dev.getmempoolfeeratediagram-rpc, protocol.op-cat</x:v>
       </x:c>
-      <x:c r="G99" s="32" t="str">
+      <x:c r="G100" s="32" t="str">
         <x:v>source.bitcoin-core-cluster-mempool-rpc, source.bitcoinops-topics</x:v>
       </x:c>
-      <x:c r="H99" s="32" t="str">
+      <x:c r="H100" s="32" t="str">
         <x:v>This is a heuristic, not a hard naming rule. Review low-level primitives individually: consequential opcodes such as OP_CAT can deserve dedicated nodes when they have a distinct learning outcome, compatibility significance, or important prerequisite chain.</x:v>
       </x:c>
     </x:row>
@@ -10796,10 +10919,10 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B99">
+    <x:dataValidation type="list" sqref="B12:B100">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D99">
+    <x:dataValidation type="list" sqref="D12:D100">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10852,7 +10975,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.80827922454</x:v>
+        <x:v>46213.816556157406</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10876,7 +10999,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>85</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10884,7 +11007,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>96</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -10908,7 +11031,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>72</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add miner decentralization
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R030e6b9785814e9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R8217036c18354d58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rbeb8e6318262464c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rebbe7de4bd704227"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R18035da0963e427b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R0ac3d21009f74bcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R3178dbb35f7f4094"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R5df8072c3eda4399"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rdb62eb153b044bb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R848ba7fdf8fb42cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Reae0b3e82d0d480e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R958b8d5b73de460a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -672,13 +672,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="M14" s="32" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="N14" s="32" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="O14" s="32" t="str">
-        <x:v>Heavy overlap with existing philosophy nodes, but strong for bridge concepts like validation sovereignty, consensus vs policy, and development review. Implemented from this source in the current branch: fundamentals.validation-sovereignty, protocol.consensus-vs-policy, protocol.chain-split-risk, and dev.review-culture.</x:v>
+        <x:v>Heavy overlap with existing philosophy nodes, but strong for bridge concepts like validation sovereignty, consensus vs policy, development review, and miner decentralization. Implemented from this source in the current branch: fundamentals.validation-sovereignty, protocol.consensus-vs-policy, protocol.chain-split-risk, dev.review-culture, and mining.miner-decentralization.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -6191,16 +6191,67 @@
         <x:v>Added after deduping against ops.dns-seeds, lightning.gossip-protocol, peer-discovery, and routing concepts. This is a Lightning protocol mechanism, not a function/API wrapper.</x:v>
       </x:c>
     </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="32" t="str">
+        <x:v>mining.miner-decentralization</x:v>
+      </x:c>
+      <x:c r="B98" s="32" t="str">
+        <x:v>Miner Decentralization</x:v>
+      </x:c>
+      <x:c r="C98" s="32" t="str">
+        <x:v>Mining</x:v>
+      </x:c>
+      <x:c r="D98" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="E98" s="32" t="str">
+        <x:v>https://bitcoindevphilosophy.com/#minerdecentralization</x:v>
+      </x:c>
+      <x:c r="F98" s="32" t="str">
+        <x:v>Decentralization chapter 1.1 Miner decentralization</x:v>
+      </x:c>
+      <x:c r="G98" s="32" t="str"/>
+      <x:c r="H98" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I98" s="32" t="str">
+        <x:v>This is one system-level concept about dispersed control over transaction ordering and its censorship consequences. It is narrower than censorship resistance, distinct from the rule-enforcement role of full nodes, and broader than a particular pool protocol such as Stratum V2.</x:v>
+      </x:c>
+      <x:c r="J98" s="32" t="str">
+        <x:v>protocol.nodes-vs-miners, mining.pool-vs-solo, fundamentals.censorship-resistance, mining.stratum-v2</x:v>
+      </x:c>
+      <x:c r="K98" s="32" t="str">
+        <x:v>protocol.nodes-vs-miners, mining.pool-vs-solo</x:v>
+      </x:c>
+      <x:c r="L98" s="32" t="str">
+        <x:v>Learners first need the authority boundary between miners and validating nodes, then the pool-versus-solo structure that shapes how mining participants coordinate. Censorship resistance is the outcome explained by this node, while Stratum V2 is an optional implementation mechanism rather than a universal prerequisite.</x:v>
+      </x:c>
+      <x:c r="M98" s="32" t="str">
+        <x:v>mining decentralization, hashrate decentralization, decentralized transaction ordering</x:v>
+      </x:c>
+      <x:c r="N98" s="32" t="str">
+        <x:v>mining, decentralization, censorship-resistance, governance</x:v>
+      </x:c>
+      <x:c r="O98" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P98" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q98" s="32" t="str">
+        <x:v>Added after deduping against fundamentals.censorship-resistance, protocol.nodes-vs-miners, mining.pool-vs-solo, and mining.stratum-v2. Do not add full-node decentralization as a duplicate: it is already covered by validation sovereignty and full-node concepts.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H97">
+    <x:dataValidation type="list" sqref="H12:H98">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P97">
+    <x:dataValidation type="list" sqref="P12:P98">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -8520,16 +8571,62 @@
         <x:v>Lightning routing and generic P2P messages are inherited through gossip rather than added as transitive prerequisites.</x:v>
       </x:c>
     </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="32" t="str">
+        <x:v>protocol.nodes-vs-miners</x:v>
+      </x:c>
+      <x:c r="B110" s="32" t="str">
+        <x:v>mining.miner-decentralization</x:v>
+      </x:c>
+      <x:c r="C110" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D110" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E110" s="32" t="str">
+        <x:v>Miner decentralization only makes sense once learners distinguish miners' transaction-ordering role from full nodes' independent enforcement of consensus validity.</x:v>
+      </x:c>
+      <x:c r="F110" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G110" s="32" t="str">
+        <x:v>The edge keeps censorship power separate from authority to change consensus rules.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="32" t="str">
+        <x:v>mining.pool-vs-solo</x:v>
+      </x:c>
+      <x:c r="B111" s="32" t="str">
+        <x:v>mining.miner-decentralization</x:v>
+      </x:c>
+      <x:c r="C111" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D111" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E111" s="32" t="str">
+        <x:v>Pool and solo mining explain the participant and coordination structure whose concentration or dispersion determines practical control over transaction ordering.</x:v>
+      </x:c>
+      <x:c r="F111" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G111" s="32" t="str">
+        <x:v>Stratum V2 remains optional implementation context, not a direct prerequisite.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C109">
+    <x:dataValidation type="list" sqref="C12:C111">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D109">
+    <x:dataValidation type="list" sqref="D12:D111">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10913,16 +11010,42 @@
         <x:v>This is a heuristic, not a hard naming rule. Review low-level primitives individually: consequential opcodes such as OP_CAT can deserve dedicated nodes when they have a distinct learning outcome, compatibility significance, or important prerequisite chain.</x:v>
       </x:c>
     </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="32" t="str">
+        <x:v>decision.miner-decentralization-slice</x:v>
+      </x:c>
+      <x:c r="B101" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C101" s="32" t="str">
+        <x:v>mining.miner-decentralization</x:v>
+      </x:c>
+      <x:c r="D101" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E101" s="32" t="str">
+        <x:v>Bitcoin Dev Philosophy separates miner decentralization from full-node decentralization: a changing, permissionless mining set protects transaction ordering from centralized censorship, while users' validating nodes make consensus rules hard to change without broad adoption. This is a distinct learner outcome absent from the graph.</x:v>
+      </x:c>
+      <x:c r="F101" s="32" t="str">
+        <x:v>mining.miner-decentralization, protocol.nodes-vs-miners, mining.pool-vs-solo, fundamentals.censorship-resistance, mining.stratum-v2, fundamentals.validation-sovereignty</x:v>
+      </x:c>
+      <x:c r="G101" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="H101" s="32" t="str">
+        <x:v>Added with exactly protocol.nodes-vs-miners and mining.pool-vs-solo as direct prerequisites. Keep censorship resistance as the explained property, Stratum V2 as an optional mechanism, and full-node decentralization in its existing validation-sovereignty cluster.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B100">
+    <x:dataValidation type="list" sqref="B12:B101">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D100">
+    <x:dataValidation type="list" sqref="D12:D101">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10975,7 +11098,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.816556157406</x:v>
+        <x:v>46213.81927988426</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10999,7 +11122,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -11007,7 +11130,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>98</x:v>
+        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -11031,7 +11154,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>73</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add selection cryptography
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R3178dbb35f7f4094"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R5df8072c3eda4399"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rdb62eb153b044bb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R848ba7fdf8fb42cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Reae0b3e82d0d480e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R958b8d5b73de460a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R3a63f1c59cb34be3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rcc428e64f871463c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Ra532fc2baa8d4b1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R5629076f7cd54a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R483f8c7dc2a94981"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R012a00eb871948ad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -672,13 +672,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="M14" s="32" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="N14" s="32" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="O14" s="32" t="str">
-        <x:v>Heavy overlap with existing philosophy nodes, but strong for bridge concepts like validation sovereignty, consensus vs policy, development review, and miner decentralization. Implemented from this source in the current branch: fundamentals.validation-sovereignty, protocol.consensus-vs-policy, protocol.chain-split-risk, dev.review-culture, and mining.miner-decentralization.</x:v>
+        <x:v>Heavy overlap with existing philosophy nodes, but strong for bridge concepts like validation sovereignty, consensus vs policy, development review, miner decentralization, and selection cryptography. Implemented from this source in the current branch: fundamentals.validation-sovereignty, protocol.consensus-vs-policy, protocol.chain-split-risk, dev.review-culture, mining.miner-decentralization, and dev.selection-cryptography.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -6242,16 +6242,67 @@
         <x:v>Added after deduping against fundamentals.censorship-resistance, protocol.nodes-vs-miners, mining.pool-vs-solo, and mining.stratum-v2. Do not add full-node decentralization as a duplicate: it is already covered by validation sovereignty and full-node concepts.</x:v>
       </x:c>
     </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="32" t="str">
+        <x:v>dev.selection-cryptography</x:v>
+      </x:c>
+      <x:c r="B99" s="32" t="str">
+        <x:v>Selection Cryptography</x:v>
+      </x:c>
+      <x:c r="C99" s="32" t="str">
+        <x:v>History &amp; Governance</x:v>
+      </x:c>
+      <x:c r="D99" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="E99" s="32" t="str">
+        <x:v>https://bitcoindevphilosophy.com/#selectioncryptography</x:v>
+      </x:c>
+      <x:c r="F99" s="32" t="str">
+        <x:v>Open Source chapter 7.4 Selection cryptography</x:v>
+      </x:c>
+      <x:c r="G99" s="32" t="str"/>
+      <x:c r="H99" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I99" s="32" t="str">
+        <x:v>This is one developer decision skill: evaluating whether a cryptographic dependency or implementation is safe and suitable to adopt. It is distinct from learning cryptographic primitives, reviewing a proposed Bitcoin change, and reproducing a released binary.</x:v>
+      </x:c>
+      <x:c r="J99" s="32" t="str">
+        <x:v>dev.review-culture, security.adversarial-thinking, dev.reproducible-builds, fundamentals.elliptic-curve-cryptography</x:v>
+      </x:c>
+      <x:c r="K99" s="32" t="str">
+        <x:v>dev.review-culture</x:v>
+      </x:c>
+      <x:c r="L99" s="32" t="str">
+        <x:v>Review culture supplies the learner's core method for examining evidence, tests, authorship, and process. Adversarial thinking is already inherited through it; reproducible builds verify release artifacts after selection; and a particular cryptographic primitive is not necessary to understand dependency due diligence.</x:v>
+      </x:c>
+      <x:c r="M99" s="32" t="str">
+        <x:v>cryptographic dependency selection, choosing cryptographic libraries, crypto library due diligence</x:v>
+      </x:c>
+      <x:c r="N99" s="32" t="str">
+        <x:v>development, cryptography, dependencies, security, review</x:v>
+      </x:c>
+      <x:c r="O99" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P99" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q99" s="32" t="str">
+        <x:v>Added after deduping against dev.review-culture, security.adversarial-thinking, dev.reproducible-builds, and cryptographic primitive nodes. It covers choosing a tool or dependency, not proving a primitive or reviewing one particular code change.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H98">
+    <x:dataValidation type="list" sqref="H12:H99">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P98">
+    <x:dataValidation type="list" sqref="P12:P99">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -8617,16 +8668,39 @@
         <x:v>Stratum V2 remains optional implementation context, not a direct prerequisite.</x:v>
       </x:c>
     </x:row>
+    <x:row r="112">
+      <x:c r="A112" s="32" t="str">
+        <x:v>dev.review-culture</x:v>
+      </x:c>
+      <x:c r="B112" s="32" t="str">
+        <x:v>dev.selection-cryptography</x:v>
+      </x:c>
+      <x:c r="C112" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D112" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E112" s="32" t="str">
+        <x:v>Selection cryptography evaluates cryptographic tools and dependencies through evidence, testing, authorship, and review quality, so learners need the broader Bitcoin review discipline first.</x:v>
+      </x:c>
+      <x:c r="F112" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G112" s="32" t="str">
+        <x:v>Adversarial thinking is inherited through dev.review-culture; reproducible builds are a downstream verification practice rather than a prerequisite.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C111">
+    <x:dataValidation type="list" sqref="C12:C112">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D111">
+    <x:dataValidation type="list" sqref="D12:D112">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11036,16 +11110,42 @@
         <x:v>Added with exactly protocol.nodes-vs-miners and mining.pool-vs-solo as direct prerequisites. Keep censorship resistance as the explained property, Stratum V2 as an optional mechanism, and full-node decentralization in its existing validation-sovereignty cluster.</x:v>
       </x:c>
     </x:row>
+    <x:row r="102">
+      <x:c r="A102" s="32" t="str">
+        <x:v>decision.selection-cryptography-slice</x:v>
+      </x:c>
+      <x:c r="B102" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C102" s="32" t="str">
+        <x:v>dev.selection-cryptography</x:v>
+      </x:c>
+      <x:c r="D102" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E102" s="32" t="str">
+        <x:v>Bitcoin Development Philosophy identifies a distinct engineering discipline: selecting cryptographic libraries, tools, and practices by evaluating their suitability, review process, authorship, documentation, portability, testing, and best practices. The graph lacked this decision point between general review culture and later implementation verification.</x:v>
+      </x:c>
+      <x:c r="F102" s="32" t="str">
+        <x:v>dev.selection-cryptography, dev.review-culture, security.adversarial-thinking, dev.reproducible-builds, fundamentals.elliptic-curve-cryptography</x:v>
+      </x:c>
+      <x:c r="G102" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="H102" s="32" t="str">
+        <x:v>Added with dev.review-culture as the only direct prerequisite. Keep primitive theory, general adversarial reasoning, and reproducible-build verification as neighboring or inherited concepts rather than redundant edges.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B101">
+    <x:dataValidation type="list" sqref="B12:B102">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D101">
+    <x:dataValidation type="list" sqref="D12:D102">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11098,7 +11198,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.81927988426</x:v>
+        <x:v>46213.82299165509</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -11122,7 +11222,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -11130,7 +11230,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>100</x:v>
+        <x:v>101</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -11154,7 +11254,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>74</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add block withholding
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R3a63f1c59cb34be3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rcc428e64f871463c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Ra532fc2baa8d4b1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R5629076f7cd54a05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R483f8c7dc2a94981"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R012a00eb871948ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R962eef29ff9d4d1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R0ec090bb51bf41fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R69991a4b49234b4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Re1225522814c4a23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R473c1b3d6b174031"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R712f11a2d73f4236"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -578,13 +578,13 @@
         <x:v>157</x:v>
       </x:c>
       <x:c r="M12" s="32" t="n">
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="N12" s="32" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="O12" s="32" t="str">
-        <x:v>157 topics plus 117 aliases make this a naming registry and gap detector more than a bulk node source. Implemented from this source in the current branch: protocol.x-only-public-keys, protocol.version-3-transaction-relay, protocol.tapscript, dev.taproot-psbt-fields, protocol.accidental-confiscation, dev.taproot-descriptors, dev.descriptor-wallet-policies, and dev.descriptors-in-psbt.</x:v>
+        <x:v>157 topics plus 117 aliases make this a naming registry and gap detector more than a bulk node source. Implemented from this source in the current branch: protocol.x-only-public-keys, protocol.version-3-transaction-relay, protocol.tapscript, dev.taproot-psbt-fields, protocol.accidental-confiscation, dev.taproot-descriptors, dev.descriptor-wallet-policies, dev.descriptors-in-psbt, and mining.block-withholding.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -6293,16 +6293,67 @@
         <x:v>Added after deduping against dev.review-culture, security.adversarial-thinking, dev.reproducible-builds, and cryptographic primitive nodes. It covers choosing a tool or dependency, not proving a primitive or reviewing one particular code change.</x:v>
       </x:c>
     </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="32" t="str">
+        <x:v>mining.block-withholding</x:v>
+      </x:c>
+      <x:c r="B100" s="32" t="str">
+        <x:v>Block Withholding</x:v>
+      </x:c>
+      <x:c r="C100" s="32" t="str">
+        <x:v>Mining</x:v>
+      </x:c>
+      <x:c r="D100" s="32" t="str">
+        <x:v>source.bitcoinops-topics</x:v>
+      </x:c>
+      <x:c r="E100" s="32" t="str">
+        <x:v>https://bitcoinops.org/en/topics/block-withholding/</x:v>
+      </x:c>
+      <x:c r="F100" s="32" t="str">
+        <x:v>Bitcoin Optech topic: Block withholding and oblivious shares</x:v>
+      </x:c>
+      <x:c r="G100" s="32" t="str"/>
+      <x:c r="H100" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I100" s="32" t="str">
+        <x:v>This isolates one pooled-mining attack: a miner can submit paid, non-block shares while withholding block-valid shares to impose a disproportionate loss on the pool. It is narrower than pooled mining and distinct from payout accounting, majority-chain attacks, and miner centralization.</x:v>
+      </x:c>
+      <x:c r="J100" s="32" t="str">
+        <x:v>mining.pool-shares, mining.pool-vs-solo, mining.51-percent-attack, mining.mining-economics</x:v>
+      </x:c>
+      <x:c r="K100" s="32" t="str">
+        <x:v>mining.pool-shares</x:v>
+      </x:c>
+      <x:c r="L100" s="32" t="str">
+        <x:v>Pool shares provide the direct mechanism: a pool pays for easier-target proofs but only a block-valid share earns the network reward. Pool organization and mining economics are inherited through that node; a majority attack is a distinct threat model and not required.</x:v>
+      </x:c>
+      <x:c r="M100" s="32" t="str">
+        <x:v>block withholding attack, withholding attack, oblivious shares</x:v>
+      </x:c>
+      <x:c r="N100" s="32" t="str">
+        <x:v>mining, pools, attacks, incentives, shares</x:v>
+      </x:c>
+      <x:c r="O100" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P100" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q100" s="32" t="str">
+        <x:v>Added after deduping against mining.pool-shares, mining.pool-vs-solo, mining.51-percent-attack, and mining.miner-decentralization. Keep selfish mining as a separate chain-construction strategy rather than collapsing it into this pool-accounting attack.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H99">
+    <x:dataValidation type="list" sqref="H12:H100">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P99">
+    <x:dataValidation type="list" sqref="P12:P100">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -8691,16 +8742,39 @@
         <x:v>Adversarial thinking is inherited through dev.review-culture; reproducible builds are a downstream verification practice rather than a prerequisite.</x:v>
       </x:c>
     </x:row>
+    <x:row r="113">
+      <x:c r="A113" s="32" t="str">
+        <x:v>mining.pool-shares</x:v>
+      </x:c>
+      <x:c r="B113" s="32" t="str">
+        <x:v>mining.block-withholding</x:v>
+      </x:c>
+      <x:c r="C113" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D113" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E113" s="32" t="str">
+        <x:v>Block withholding exploits the difference between a pool-paid share and a share that also meets the network target, so learners must understand share accounting before the attack model makes sense.</x:v>
+      </x:c>
+      <x:c r="F113" s="32" t="str">
+        <x:v>source.bitcoinops-topics</x:v>
+      </x:c>
+      <x:c r="G113" s="32" t="str">
+        <x:v>Pool-versus-solo and mining economics are inherited through mining.pool-shares; do not add a redundant majority-attack edge.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C112">
+    <x:dataValidation type="list" sqref="C12:C113">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D112">
+    <x:dataValidation type="list" sqref="D12:D113">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11136,16 +11210,42 @@
         <x:v>Added with dev.review-culture as the only direct prerequisite. Keep primitive theory, general adversarial reasoning, and reproducible-build verification as neighboring or inherited concepts rather than redundant edges.</x:v>
       </x:c>
     </x:row>
+    <x:row r="103">
+      <x:c r="A103" s="32" t="str">
+        <x:v>decision.block-withholding-slice</x:v>
+      </x:c>
+      <x:c r="B103" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C103" s="32" t="str">
+        <x:v>mining.block-withholding</x:v>
+      </x:c>
+      <x:c r="D103" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E103" s="32" t="str">
+        <x:v>Bitcoin Optech identifies block withholding as a distinct pooled-mining attack: a participant can submit ordinary shares for compensation while selectively hiding block-valid shares, giving up little revenue while depriving the pool of the block reward. This attack model was absent from the graph.</x:v>
+      </x:c>
+      <x:c r="F103" s="32" t="str">
+        <x:v>mining.block-withholding, mining.pool-shares, mining.pool-vs-solo, mining.51-percent-attack, mining.miner-decentralization</x:v>
+      </x:c>
+      <x:c r="G103" s="32" t="str">
+        <x:v>source.bitcoinops-topics</x:v>
+      </x:c>
+      <x:c r="H103" s="32" t="str">
+        <x:v>Added with mining.pool-shares as the only direct prerequisite. Preserve selfish mining as a separate chain-building attack and keep oblivious shares as a proposed mitigation alias, not a separate node.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B102">
+    <x:dataValidation type="list" sqref="B12:B103">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D102">
+    <x:dataValidation type="list" sqref="D12:D103">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11198,7 +11298,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.82299165509</x:v>
+        <x:v>46213.826253136576</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -11222,7 +11322,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>88</x:v>
+        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -11230,7 +11330,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>101</x:v>
+        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -11254,7 +11354,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>75</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add replacement cycling
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R962eef29ff9d4d1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R0ec090bb51bf41fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R69991a4b49234b4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Re1225522814c4a23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R473c1b3d6b174031"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R712f11a2d73f4236"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R2e16809435fc4119"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R799934486b0449a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R40b2df18d5574198"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R192027d4d1e9445c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R820e55f1670c4586"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R301905097c4e44fc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -578,13 +578,13 @@
         <x:v>157</x:v>
       </x:c>
       <x:c r="M12" s="32" t="n">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="N12" s="32" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="O12" s="32" t="str">
-        <x:v>157 topics plus 117 aliases make this a naming registry and gap detector more than a bulk node source. Implemented from this source in the current branch: protocol.x-only-public-keys, protocol.version-3-transaction-relay, protocol.tapscript, dev.taproot-psbt-fields, protocol.accidental-confiscation, dev.taproot-descriptors, dev.descriptor-wallet-policies, dev.descriptors-in-psbt, and mining.block-withholding.</x:v>
+        <x:v>157 topics plus 117 aliases make this a naming registry and gap detector more than a bulk node source. Implemented from this source in the current branch: protocol.x-only-public-keys, protocol.version-3-transaction-relay, protocol.tapscript, dev.taproot-psbt-fields, protocol.accidental-confiscation, dev.taproot-descriptors, dev.descriptor-wallet-policies, dev.descriptors-in-psbt, mining.block-withholding, and protocol.replacement-cycling.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -719,13 +719,13 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="M15" s="32" t="n">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="N15" s="32" t="n">
-        <x:v>13</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="O15" s="32" t="str">
-        <x:v>Already heavily reused in current nodes, so chapter titles are containers. Best current value is prerequisite ladders and bridge concepts. Implemented from this source in the current branch: protocol.light-client-trust-model, ops.full-node-vs-lightweight-wallet, custody.coin-selection, protocol.change-outputs, protocol.bech32m-addresses, protocol.script-execution-stack, dev.extended-keys, protocol.witness-structure, and protocol.partial-merkle-proofs.</x:v>
+        <x:v>Already heavily reused in current nodes, so chapter titles are containers. Best current value is prerequisite ladders and bridge concepts. Implemented from this source in the current branch: protocol.light-client-trust-model, ops.full-node-vs-lightweight-wallet, custody.coin-selection, protocol.change-outputs, protocol.bech32m-addresses, protocol.script-execution-stack, dev.extended-keys, protocol.witness-structure, protocol.partial-merkle-proofs, protocol.pay-to-contract, extension.single-use-seals, and extension.client-side-validation.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -6344,16 +6344,220 @@
         <x:v>Added after deduping against mining.pool-shares, mining.pool-vs-solo, mining.51-percent-attack, and mining.miner-decentralization. Keep selfish mining as a separate chain-construction strategy rather than collapsing it into this pool-accounting attack.</x:v>
       </x:c>
     </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="32" t="str">
+        <x:v>protocol.replacement-cycling</x:v>
+      </x:c>
+      <x:c r="B101" s="32" t="str">
+        <x:v>Replacement Cycling</x:v>
+      </x:c>
+      <x:c r="C101" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D101" s="32" t="str">
+        <x:v>source.bitcoinops-topics</x:v>
+      </x:c>
+      <x:c r="E101" s="32" t="str">
+        <x:v>https://bitcoinops.org/en/topics/replacement-cycling/</x:v>
+      </x:c>
+      <x:c r="F101" s="32" t="str">
+        <x:v>Bitcoin Optech topic: Replacement cycling</x:v>
+      </x:c>
+      <x:c r="G101" s="32" t="str"/>
+      <x:c r="H101" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I101" s="32" t="str">
+        <x:v>One repeated-eviction attack that combines RBF and CPFP to block time-sensitive multiparty confirmation. It is narrower than generic transaction pinning and distinct from ordinary fee bumping.</x:v>
+      </x:c>
+      <x:c r="J101" s="32" t="str">
+        <x:v>protocol.rbf, protocol.cpfp, protocol.transaction-pinning, lightning.anchor-outputs</x:v>
+      </x:c>
+      <x:c r="K101" s="32" t="str">
+        <x:v>protocol.rbf, protocol.cpfp</x:v>
+      </x:c>
+      <x:c r="L101" s="32" t="str">
+        <x:v>RBF supplies the replacement mechanism and CPFP supplies the child-fee sequence. Transaction pinning is the broader risk class explained by this node, while anchor outputs are one affected Lightning construction.</x:v>
+      </x:c>
+      <x:c r="M101" s="32" t="str">
+        <x:v>replacement cycling attack, RBF cycling, transaction replacement cycling</x:v>
+      </x:c>
+      <x:c r="N101" s="32" t="str">
+        <x:v>mempool, rbf, cpfp, pinning, lightning, contracts</x:v>
+      </x:c>
+      <x:c r="O101" s="32" t="str">
+        <x:v>40m</x:v>
+      </x:c>
+      <x:c r="P101" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q101" s="32" t="str">
+        <x:v>Added after deduping against transaction pinning, package RBF, CPFP carve-out, and Lightning anchors. It explains the distinct repeatable eviction sequence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" s="32" t="str">
+        <x:v>protocol.pay-to-contract</x:v>
+      </x:c>
+      <x:c r="B102" s="32" t="str">
+        <x:v>Pay to Contract (P2C)</x:v>
+      </x:c>
+      <x:c r="C102" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D102" s="32" t="str">
+        <x:v>source.mastering-bitcoin-book-map</x:v>
+      </x:c>
+      <x:c r="E102" s="32" t="str">
+        <x:v>https://github.com/bitcoinbook/bitcoinbook/blob/develop/ch14_applications.adoc</x:v>
+      </x:c>
+      <x:c r="F102" s="32" t="str">
+        <x:v>Mastering Bitcoin chapters 7 and 14: pay-to-contract commitments</x:v>
+      </x:c>
+      <x:c r="G102" s="32" t="str"/>
+      <x:c r="H102" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I102" s="32" t="str">
+        <x:v>One key-tweak commitment construction, distinct from generic hashing, Taproot, DLCs, and script contracts.</x:v>
+      </x:c>
+      <x:c r="J102" s="32" t="str">
+        <x:v>fundamentals.public-private-keys, fundamentals.hash-functions, protocol.taproot</x:v>
+      </x:c>
+      <x:c r="K102" s="32" t="str">
+        <x:v>fundamentals.public-private-keys, fundamentals.hash-functions</x:v>
+      </x:c>
+      <x:c r="L102" s="32" t="str">
+        <x:v>Public keys and hash commitments are the direct construction. Taproot is an adjacent use of key tweaking, not required to understand P2C.</x:v>
+      </x:c>
+      <x:c r="M102" s="32" t="str">
+        <x:v>P2C, pay-to-contract protocol, key tweak commitment</x:v>
+      </x:c>
+      <x:c r="N102" s="32" t="str">
+        <x:v>contracts, keys, commitments, privacy, applications</x:v>
+      </x:c>
+      <x:c r="O102" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P102" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q102" s="32" t="str">
+        <x:v>Added after deduping against Taproot, DLCs, commitment schemes, and Script; it is the missing generic public-key commitment pattern.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" s="32" t="str">
+        <x:v>extension.single-use-seals</x:v>
+      </x:c>
+      <x:c r="B103" s="32" t="str">
+        <x:v>Single-Use Seals</x:v>
+      </x:c>
+      <x:c r="C103" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D103" s="32" t="str">
+        <x:v>source.mastering-bitcoin-book-map</x:v>
+      </x:c>
+      <x:c r="E103" s="32" t="str">
+        <x:v>https://github.com/bitcoinbook/bitcoinbook/blob/develop/ch14_applications.adoc</x:v>
+      </x:c>
+      <x:c r="F103" s="32" t="str">
+        <x:v>Mastering Bitcoin chapter 14: UTXO single-use seals</x:v>
+      </x:c>
+      <x:c r="G103" s="32" t="str"/>
+      <x:c r="H103" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I103" s="32" t="str">
+        <x:v>One bridge concept: an outpoint can bind an offchain state transition exactly once because it can only be spent once.</x:v>
+      </x:c>
+      <x:c r="J103" s="32" t="str">
+        <x:v>protocol.utxo-model</x:v>
+      </x:c>
+      <x:c r="K103" s="32" t="str">
+        <x:v>protocol.utxo-model</x:v>
+      </x:c>
+      <x:c r="L103" s="32" t="str">
+        <x:v>The UTXO model supplies the one-time spend property that makes the seal meaningful.</x:v>
+      </x:c>
+      <x:c r="M103" s="32" t="str">
+        <x:v>single use seals, UTXO seals, outpoint seals</x:v>
+      </x:c>
+      <x:c r="N103" s="32" t="str">
+        <x:v>utxos, commitments, assets, contracts</x:v>
+      </x:c>
+      <x:c r="O103" s="32" t="str">
+        <x:v>25m</x:v>
+      </x:c>
+      <x:c r="P103" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q103" s="32" t="str">
+        <x:v>Added as the explicit bridge between UTXO semantics and client-side validation; do not hide the core invariant inside either neighbor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" s="32" t="str">
+        <x:v>extension.client-side-validation</x:v>
+      </x:c>
+      <x:c r="B104" s="32" t="str">
+        <x:v>Client-Side Validation</x:v>
+      </x:c>
+      <x:c r="C104" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D104" s="32" t="str">
+        <x:v>source.mastering-bitcoin-book-map</x:v>
+      </x:c>
+      <x:c r="E104" s="32" t="str">
+        <x:v>https://github.com/bitcoinbook/bitcoinbook/blob/develop/ch14_applications.adoc</x:v>
+      </x:c>
+      <x:c r="F104" s="32" t="str">
+        <x:v>Mastering Bitcoin chapter 14: client-side validation and single-use seals</x:v>
+      </x:c>
+      <x:c r="G104" s="32" t="str"/>
+      <x:c r="H104" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I104" s="32" t="str">
+        <x:v>One application-layer validation model where recipients validate offchain asset history and rules, distinct from Bitcoin full-node validation.</x:v>
+      </x:c>
+      <x:c r="J104" s="32" t="str">
+        <x:v>extension.single-use-seals, protocol.pay-to-contract, fundamentals.validation-sovereignty</x:v>
+      </x:c>
+      <x:c r="K104" s="32" t="str">
+        <x:v>extension.single-use-seals, protocol.pay-to-contract</x:v>
+      </x:c>
+      <x:c r="L104" s="32" t="str">
+        <x:v>Single-use seals provide the one-time transition invariant and P2C provides contract anchoring. Validation sovereignty is related Bitcoin-layer framing, not a direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M104" s="32" t="str">
+        <x:v>recipient-side validation, client validated assets</x:v>
+      </x:c>
+      <x:c r="N104" s="32" t="str">
+        <x:v>assets, validation, utxos, contracts, rgb</x:v>
+      </x:c>
+      <x:c r="O104" s="32" t="str">
+        <x:v>40m</x:v>
+      </x:c>
+      <x:c r="P104" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q104" s="32" t="str">
+        <x:v>Added after deduping against validation sovereignty and RGB-adjacent labels. It is a distinct application-layer model rather than a second full-node concept.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H100">
+    <x:dataValidation type="list" sqref="H12:H104">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P100">
+    <x:dataValidation type="list" sqref="P12:P104">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -8765,16 +8969,177 @@
         <x:v>Pool-versus-solo and mining economics are inherited through mining.pool-shares; do not add a redundant majority-attack edge.</x:v>
       </x:c>
     </x:row>
+    <x:row r="114">
+      <x:c r="A114" s="32" t="str">
+        <x:v>fundamentals.public-private-keys</x:v>
+      </x:c>
+      <x:c r="B114" s="32" t="str">
+        <x:v>protocol.pay-to-contract</x:v>
+      </x:c>
+      <x:c r="C114" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D114" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E114" s="32" t="str">
+        <x:v>P2C tweaks a public key to commit to contract data, so learners need the public/private key model.</x:v>
+      </x:c>
+      <x:c r="F114" s="32" t="str">
+        <x:v>source.mastering-bitcoin-book-map</x:v>
+      </x:c>
+      <x:c r="G114" s="32" t="str">
+        <x:v>Taproot is adjacent, not a direct requirement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" s="32" t="str">
+        <x:v>fundamentals.hash-functions</x:v>
+      </x:c>
+      <x:c r="B115" s="32" t="str">
+        <x:v>protocol.pay-to-contract</x:v>
+      </x:c>
+      <x:c r="C115" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D115" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E115" s="32" t="str">
+        <x:v>P2C derives a commitment tweak from contract data using a hash, so learners need hash commitments first.</x:v>
+      </x:c>
+      <x:c r="F115" s="32" t="str">
+        <x:v>source.mastering-bitcoin-book-map</x:v>
+      </x:c>
+      <x:c r="G115" s="32" t="str">
+        <x:v>The hash is part of the construction rather than generic background.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" s="32" t="str">
+        <x:v>protocol.utxo-model</x:v>
+      </x:c>
+      <x:c r="B116" s="32" t="str">
+        <x:v>extension.single-use-seals</x:v>
+      </x:c>
+      <x:c r="C116" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D116" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E116" s="32" t="str">
+        <x:v>Single-use seals rely on a UTXO's one-time spend property.</x:v>
+      </x:c>
+      <x:c r="F116" s="32" t="str">
+        <x:v>source.mastering-bitcoin-book-map</x:v>
+      </x:c>
+      <x:c r="G116" s="32" t="str">
+        <x:v>This explicit bridge prevents hiding the seal invariant inside generic UTXO semantics.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" s="32" t="str">
+        <x:v>extension.single-use-seals</x:v>
+      </x:c>
+      <x:c r="B117" s="32" t="str">
+        <x:v>extension.client-side-validation</x:v>
+      </x:c>
+      <x:c r="C117" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D117" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E117" s="32" t="str">
+        <x:v>Client-side validation relies on seals to prevent an offchain transition from being valid twice.</x:v>
+      </x:c>
+      <x:c r="F117" s="32" t="str">
+        <x:v>source.mastering-bitcoin-book-map</x:v>
+      </x:c>
+      <x:c r="G117" s="32" t="str">
+        <x:v>The UTXO parent is inherited through the seal and is intentionally not duplicated.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" s="32" t="str">
+        <x:v>protocol.pay-to-contract</x:v>
+      </x:c>
+      <x:c r="B118" s="32" t="str">
+        <x:v>extension.client-side-validation</x:v>
+      </x:c>
+      <x:c r="C118" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D118" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E118" s="32" t="str">
+        <x:v>Client-side validation uses cryptographic commitments to bind offchain asset rules and transitions, so P2C supplies the contract-anchoring mechanism.</x:v>
+      </x:c>
+      <x:c r="F118" s="32" t="str">
+        <x:v>source.mastering-bitcoin-book-map</x:v>
+      </x:c>
+      <x:c r="G118" s="32" t="str">
+        <x:v>Keep this direct edge: it prevents treating client-side validation as a vague UTXO-only extension.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" s="32" t="str">
+        <x:v>protocol.rbf</x:v>
+      </x:c>
+      <x:c r="B119" s="32" t="str">
+        <x:v>protocol.replacement-cycling</x:v>
+      </x:c>
+      <x:c r="C119" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D119" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E119" s="32" t="str">
+        <x:v>Replacement cycling repeatedly uses transaction replacement, so learners need the RBF policy mechanism first.</x:v>
+      </x:c>
+      <x:c r="F119" s="32" t="str">
+        <x:v>source.bitcoinops-topics</x:v>
+      </x:c>
+      <x:c r="G119" s="32" t="str">
+        <x:v>Package RBF is related but not required for the core attack sequence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" s="32" t="str">
+        <x:v>protocol.cpfp</x:v>
+      </x:c>
+      <x:c r="B120" s="32" t="str">
+        <x:v>protocol.replacement-cycling</x:v>
+      </x:c>
+      <x:c r="C120" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D120" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E120" s="32" t="str">
+        <x:v>The attack cycles child-fee relationships to evict a target, so learners need CPFP mechanics first.</x:v>
+      </x:c>
+      <x:c r="F120" s="32" t="str">
+        <x:v>source.bitcoinops-topics</x:v>
+      </x:c>
+      <x:c r="G120" s="32" t="str">
+        <x:v>Transaction pinning is the broader downstream risk class, not a prerequisite.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C113">
+    <x:dataValidation type="list" sqref="C12:C120">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D113">
+    <x:dataValidation type="list" sqref="D12:D120">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11298,7 +11663,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.826253136576</x:v>
+        <x:v>46213.830886550924</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -11322,7 +11687,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>89</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -11330,7 +11695,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>102</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -11354,7 +11719,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>76</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add Taproot control blocks
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R2e16809435fc4119"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R799934486b0449a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R40b2df18d5574198"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R192027d4d1e9445c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R820e55f1670c4586"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R301905097c4e44fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R6dafa3f524414cfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R20b3acd829b6492a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rad5c66f5a317447a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R5426f535f97d4bb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R6284ec3b5dec49fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Re937ab545d8b468f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -766,13 +766,13 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="M16" s="32" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="N16" s="32" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="O16" s="32" t="str">
-        <x:v>Best current source for missing Taproot bridge concepts such as tagged hashes, taptweak, key-path spends, tapleaf inclusion proofs, Huffman-optimized TapTrees, and concrete policy case studies like degrading multisig. Implemented from this source in the current branch: protocol.tagged-hashes, protocol.taptweak, protocol.taproot-key-path-spends, protocol.taptree, protocol.tapleaf-inclusion-proofs, protocol.huffman-optimized-taptrees, and custody.degrading-multisig. Current tracked workshop queue is exhausted for this pass.</x:v>
+        <x:v>Best current source for missing Taproot bridge concepts such as tagged hashes, taptweak, key-path spends, tapleaf inclusion proofs, control blocks, Huffman-optimized TapTrees, and concrete policy case studies like degrading multisig. Implemented from this source in the current branch: protocol.tagged-hashes, protocol.taptweak, protocol.taproot-key-path-spends, protocol.taptree, protocol.tapleaf-inclusion-proofs, protocol.taproot-control-blocks, protocol.huffman-optimized-taptrees, and custody.degrading-multisig.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -6548,16 +6548,67 @@
         <x:v>Added after deduping against validation sovereignty and RGB-adjacent labels. It is a distinct application-layer model rather than a second full-node concept.</x:v>
       </x:c>
     </x:row>
+    <x:row r="105">
+      <x:c r="A105" s="32" t="str">
+        <x:v>protocol.taproot-control-blocks</x:v>
+      </x:c>
+      <x:c r="B105" s="32" t="str">
+        <x:v>Taproot Control Blocks</x:v>
+      </x:c>
+      <x:c r="C105" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D105" s="32" t="str">
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+      </x:c>
+      <x:c r="E105" s="32" t="str">
+        <x:v>https://bitcoinops.org/en/schnorr-taproot-workshop/</x:v>
+      </x:c>
+      <x:c r="F105" s="32" t="str">
+        <x:v>Taproot workshop script-path witness material</x:v>
+      </x:c>
+      <x:c r="G105" s="32" t="str"/>
+      <x:c r="H105" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I105" s="32" t="str">
+        <x:v>A control block is the distinct witness object that binds a script-path reveal to a Taproot output using an internal key, parity bit, and proof path.</x:v>
+      </x:c>
+      <x:c r="J105" s="32" t="str">
+        <x:v>protocol.taproot, protocol.tapleaf-inclusion-proofs, fundamentals.merkle-trees</x:v>
+      </x:c>
+      <x:c r="K105" s="32" t="str">
+        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
+      </x:c>
+      <x:c r="L105" s="32" t="str">
+        <x:v>Tapleaf inclusion proofs already inherit the Taproot and Merkle-tree context, while supplying the proof-path model that control blocks extend.</x:v>
+      </x:c>
+      <x:c r="M105" s="32" t="str">
+        <x:v>control block, taproot script-path control block</x:v>
+      </x:c>
+      <x:c r="N105" s="32" t="str">
+        <x:v>taproot, witness, scripts, merkle-proofs</x:v>
+      </x:c>
+      <x:c r="O105" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P105" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q105" s="32" t="str">
+        <x:v>Distinct from a tapleaf proof because it additionally carries internal-key and parity data; the Taproot edge is transitive and intentionally omitted.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H104">
+    <x:dataValidation type="list" sqref="H12:H105">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P104">
+    <x:dataValidation type="list" sqref="P12:P105">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9130,16 +9181,39 @@
         <x:v>Transaction pinning is the broader downstream risk class, not a prerequisite.</x:v>
       </x:c>
     </x:row>
+    <x:row r="121">
+      <x:c r="A121" s="32" t="str">
+        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
+      </x:c>
+      <x:c r="B121" s="32" t="str">
+        <x:v>protocol.taproot-control-blocks</x:v>
+      </x:c>
+      <x:c r="C121" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D121" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E121" s="32" t="str">
+        <x:v>Control blocks extend the tapleaf proof path with internal-key and parity data.</x:v>
+      </x:c>
+      <x:c r="F121" s="32" t="str">
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+      </x:c>
+      <x:c r="G121" s="32" t="str">
+        <x:v>Generic Merkle trees are inherited through the proof node.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C120">
+    <x:dataValidation type="list" sqref="C12:C121">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D120">
+    <x:dataValidation type="list" sqref="D12:D121">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11663,7 +11737,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.830886550924</x:v>
+        <x:v>46213.83430469908</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -11687,7 +11761,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>93</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -11695,7 +11769,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>109</x:v>
+        <x:v>110</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -11719,7 +11793,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>80</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add pseudonymous development concept
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R6dafa3f524414cfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R20b3acd829b6492a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rad5c66f5a317447a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R5426f535f97d4bb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R6284ec3b5dec49fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Re937ab545d8b468f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rd4d9ae081fc0434b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Re898dfb1f02b42f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rdfaea22891574e3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rd8d6abb0579b4cfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rd335a712b71a4561"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rb87f28bb73c243e8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -675,10 +675,10 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="N14" s="32" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="O14" s="32" t="str">
-        <x:v>Heavy overlap with existing philosophy nodes, but strong for bridge concepts like validation sovereignty, consensus vs policy, development review, miner decentralization, and selection cryptography. Implemented from this source in the current branch: fundamentals.validation-sovereignty, protocol.consensus-vs-policy, protocol.chain-split-risk, dev.review-culture, mining.miner-decentralization, and dev.selection-cryptography.</x:v>
+        <x:v>Heavy overlap with existing philosophy nodes, but strong for bridge concepts like validation sovereignty, consensus vs policy, development review, pseudonymous development, miner decentralization, and selection cryptography. Implemented from this source in the current branch: fundamentals.validation-sovereignty, protocol.consensus-vs-policy, protocol.chain-split-risk, dev.review-culture, dev.pseudonymous-development, mining.miner-decentralization, and dev.selection-cryptography.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -6599,16 +6599,67 @@
         <x:v>Distinct from a tapleaf proof because it additionally carries internal-key and parity data; the Taproot edge is transitive and intentionally omitted.</x:v>
       </x:c>
     </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="32" t="str">
+        <x:v>dev.pseudonymous-development</x:v>
+      </x:c>
+      <x:c r="B106" s="32" t="str">
+        <x:v>Pseudonymous Development</x:v>
+      </x:c>
+      <x:c r="C106" s="32" t="str">
+        <x:v>History &amp; Governance</x:v>
+      </x:c>
+      <x:c r="D106" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="E106" s="32" t="str">
+        <x:v>https://bitcoindevphilosophy.com/#pseudonymousdevelopment</x:v>
+      </x:c>
+      <x:c r="F106" s="32" t="str">
+        <x:v>Open Source chapter &gt; Pseudonymous Development</x:v>
+      </x:c>
+      <x:c r="G106" s="32" t="str"/>
+      <x:c r="H106" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I106" s="32" t="str">
+        <x:v>One contributor-governance concept: publishing and reviewing technical work under a pseudonym can reduce coercion risk while preserving accountability through public evidence and peer review.</x:v>
+      </x:c>
+      <x:c r="J106" s="32" t="str">
+        <x:v>dev.review-culture, privacy.pseudonymity</x:v>
+      </x:c>
+      <x:c r="K106" s="32" t="str">
+        <x:v>dev.review-culture</x:v>
+      </x:c>
+      <x:c r="L106" s="32" t="str">
+        <x:v>Review culture supplies the accountability mechanism. Transaction pseudonymity is a related identity concept, but it is not required to understand why contributors may separate legal identity from technical authorship.</x:v>
+      </x:c>
+      <x:c r="M106" s="32" t="str">
+        <x:v>pseudonymous contributors, developer pseudonymity</x:v>
+      </x:c>
+      <x:c r="N106" s="32" t="str">
+        <x:v>development, privacy, open-source, governance</x:v>
+      </x:c>
+      <x:c r="O106" s="32" t="str">
+        <x:v>25m</x:v>
+      </x:c>
+      <x:c r="P106" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q106" s="32" t="str">
+        <x:v>Added after checking privacy.pseudonymity, transaction privacy, and review-culture neighbors. Keep the node focused on contributor safety and merit-based evaluation rather than anonymous transactions.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H105">
+    <x:dataValidation type="list" sqref="H12:H106">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P105">
+    <x:dataValidation type="list" sqref="P12:P106">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -9204,16 +9255,39 @@
         <x:v>Generic Merkle trees are inherited through the proof node.</x:v>
       </x:c>
     </x:row>
+    <x:row r="122">
+      <x:c r="A122" s="32" t="str">
+        <x:v>dev.review-culture</x:v>
+      </x:c>
+      <x:c r="B122" s="32" t="str">
+        <x:v>dev.pseudonymous-development</x:v>
+      </x:c>
+      <x:c r="C122" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D122" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E122" s="32" t="str">
+        <x:v>Pseudonymous development relies on public technical evidence and independent peer review to preserve accountability without requiring legal-identity disclosure.</x:v>
+      </x:c>
+      <x:c r="F122" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G122" s="32" t="str">
+        <x:v>Privacy pseudonymity is related context, not a direct prerequisite, because this node concerns contributor identity and governance rather than transaction linkage.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C121">
+    <x:dataValidation type="list" sqref="C12:C122">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D121">
+    <x:dataValidation type="list" sqref="D12:D122">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11675,16 +11749,42 @@
         <x:v>Added with mining.pool-shares as the only direct prerequisite. Preserve selfish mining as a separate chain-building attack and keep oblivious shares as a proposed mitigation alias, not a separate node.</x:v>
       </x:c>
     </x:row>
+    <x:row r="104">
+      <x:c r="A104" s="32" t="str">
+        <x:v>decision.pseudonymous-development-slice</x:v>
+      </x:c>
+      <x:c r="B104" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C104" s="32" t="str">
+        <x:v>dev.pseudonymous-development</x:v>
+      </x:c>
+      <x:c r="D104" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E104" s="32" t="str">
+        <x:v>Bitcoin Development Philosophy identifies pseudonymous development as a distinct contributor-safety and merit-evaluation practice. It survives dedupe because privacy.pseudonymity concerns transaction identity, while review culture concerns how technical work is evaluated; neither captures the contributor-governance tradeoff.</x:v>
+      </x:c>
+      <x:c r="F104" s="32" t="str">
+        <x:v>dev.pseudonymous-development, dev.review-culture, privacy.pseudonymity, fundamentals.censorship-resistance</x:v>
+      </x:c>
+      <x:c r="G104" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="H104" s="32" t="str">
+        <x:v>Added with dev.review-culture as the only direct prerequisite. Keep transaction pseudonymity and censorship resistance as related context rather than redundant graph parents.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B103">
+    <x:dataValidation type="list" sqref="B12:B104">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D103">
+    <x:dataValidation type="list" sqref="D12:D104">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11737,7 +11837,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46213.83430469908</x:v>
+        <x:v>46214.68870096065</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -11761,7 +11861,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>94</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -11769,7 +11869,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>110</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -11793,7 +11893,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>81</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
chore: reconcile explained post inventory
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rd4d9ae081fc0434b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Re898dfb1f02b42f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rdfaea22891574e3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rd8d6abb0579b4cfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rd335a712b71a4561"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rb87f28bb73c243e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R63078c67377a4d36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Radf00d76b3c24a0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R7532f3c3e7464dd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Re55e02a1c0c7471b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R64c7aebe4175442a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R37608cb459bf4821"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1080,19 +1080,19 @@
         <x:v>Track the live X search as one source-family row first, then expand to one row per matching post once current results are enumerated. Group matching posts by concept family such as hashing, fee management, node architecture, channel mechanics, and upgrade proposals.</x:v>
       </x:c>
       <x:c r="H23" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In review</x:v>
       </x:c>
       <x:c r="I23" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J23" s="32" t="str">
-        <x:v>Queue exhausted</x:v>
+        <x:v>Raw extraction</x:v>
       </x:c>
       <x:c r="K23" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="L23" s="32" t="n">
-        <x:v>43</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="M23" s="32" t="n">
         <x:v>6</x:v>
@@ -1101,459 +1101,459 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="O23" s="32" t="str">
-        <x:v>Added from user direction. The live X query was enumerated in the logged-in in-app browser on July 8, 2026 and surfaced 43 matching posts. Visible examples include Lamport Signature explained, Duplicate transaction bug explained, 64-byte transaction bug explained, SegWit Address explained, Off-by-one difficulty bug explained, Great Consensus Cleanup explained Part 1: Time Warp Attack, Transaction Pinning explained, Full Node Architecture Explained, MAST explained simply, BIP 158 explained, MuSig explained Simply, CPFP transaction explained, CISA explained, BIP-68 Explained, and Shamir's Secret Sharing explained. Implemented from this source in the current branch: protocol.time-warp-attack, protocol.duplicate-transaction-bug, protocol.64-byte-transaction-bug, fundamentals.lamport-signatures, custody.shamirs-secret-sharing. Merged into existing coverage in the current branch: protocol.time-warp-attack via Off-by-one difficulty bug explained. Current enumerated post queue is exhausted for this pass.</x:v>
+        <x:v>Reopened after audit correction. The authenticated X search was enumerated on July 11, 2026 and currently exposes 34 matching posts, which are now tracked individually below. The earlier July 8 pass reported 43 posts but did not preserve one source row per post; that historical count remains unresolved until the current and prior inventories are reconciled. Existing normalized coverage includes time-warp attack, duplicate transaction bug, 64-byte transaction bug, nonce reuse, Lamport signatures, and Shamir's Secret Sharing.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-wallet</x:v>
+        <x:v>source.bitcoin-dev-project-post-2018682587045052753</x:v>
       </x:c>
       <x:c r="B24" s="32" t="str">
-        <x:v>Bitcoin Core Academy Wallet Internals</x:v>
+        <x:v>Bitcoin Dev Project: Coinjoin Explained</x:v>
       </x:c>
       <x:c r="C24" s="32" t="str">
-        <x:v>https://bitcoincore.academy/scriptpubkeymanagers.html</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/2018682587045052753</x:v>
       </x:c>
       <x:c r="D24" s="32" t="str">
-        <x:v>course-cluster</x:v>
+        <x:v>social-post</x:v>
       </x:c>
       <x:c r="E24" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F24" s="32" t="str">
-        <x:v>Wallet internals cluster around ScriptPubKeyManagers, wallet keys, transaction identification, and balance calculation.</x:v>
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
       </x:c>
       <x:c r="G24" s="32" t="str">
-        <x:v>Track one wallet-internals page cluster at a time so Core-specific abstractions stay atomic instead of collapsing into generic wallet concepts.</x:v>
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H24" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In review</x:v>
       </x:c>
       <x:c r="I24" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J24" s="32" t="str">
-        <x:v>Queue exhausted</x:v>
+        <x:v>Raw extraction</x:v>
       </x:c>
       <x:c r="K24" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="L24" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M24" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N24" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O24" s="32" t="str">
-        <x:v>First additional-source pass beyond the mandatory seed list. The current additive winner is dev.scriptpubkeymanagers; wallet-encryption remains deferred because the cleanest surviving slice is still too coupled to missing Core wallet-internals parents. Current tracked wallet-internals queue is exhausted for this pass.</x:v>
+        <x:v>Post title: Coinjoin Explained.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-dev-project-post-2017223553708654888</x:v>
       </x:c>
       <x:c r="B25" s="32" t="str">
-        <x:v>Bitcoin Core Academy Mempool Mechanics</x:v>
+        <x:v>Bitcoin Dev Project: Full Node Architecture Explained</x:v>
       </x:c>
       <x:c r="C25" s="32" t="str">
-        <x:v>https://bitcoincore.academy/mempool-unbroadcast.html</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/2017223553708654888</x:v>
       </x:c>
       <x:c r="D25" s="32" t="str">
-        <x:v>course-cluster</x:v>
+        <x:v>social-post</x:v>
       </x:c>
       <x:c r="E25" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F25" s="32" t="str">
-        <x:v>Mempool and relay internals cluster around transaction relay, rebroadcast behavior, and local node transaction state.</x:v>
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
       </x:c>
       <x:c r="G25" s="32" t="str">
-        <x:v>Track the academy mempool pages as a separate cluster so implementation-specific relay mechanisms are not collapsed into generic mempool coverage.</x:v>
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H25" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In review</x:v>
       </x:c>
       <x:c r="I25" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J25" s="32" t="str">
-        <x:v>Queue exhausted</x:v>
+        <x:v>Raw extraction</x:v>
       </x:c>
       <x:c r="K25" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="L25" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M25" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N25" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O25" s="32" t="str">
-        <x:v>Second post-seed-source slice. The current additive winners are protocol.mempool-unbroadcast-set, protocol.transaction-rebroadcast-privacy, and protocol.txid-vs-wtxid. The remaining transaction-format internals are now mostly implementation-detail material rather than clean learner-facing nodes. Current tracked mempool queue is exhausted for this pass.</x:v>
+        <x:v>Post title: Full Node Architecture Explained.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="str">
-        <x:v>source.bitcoin-design-payment-formats</x:v>
+        <x:v>source.bitcoin-dev-project-post-2016929384389890484</x:v>
       </x:c>
       <x:c r="B26" s="32" t="str">
-        <x:v>Bitcoin Design Payment Request Formats</x:v>
+        <x:v>Bitcoin Dev Project: SHA-256 Message Schedule Explained</x:v>
       </x:c>
       <x:c r="C26" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/how-it-works/human-readable-addresses/</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/2016929384389890484</x:v>
       </x:c>
       <x:c r="D26" s="32" t="str">
-        <x:v>guide-cluster</x:v>
+        <x:v>social-post</x:v>
       </x:c>
       <x:c r="E26" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F26" s="32" t="str">
-        <x:v>User-facing payment request and address-sharing concepts across human-readable addresses, transaction display, and wallet privacy tradeoffs.</x:v>
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
       </x:c>
       <x:c r="G26" s="32" t="str">
-        <x:v>Track design guide pages by UX concept cluster so user-facing payment abstractions stay separate from protocol internals and generic wallet hygiene.</x:v>
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H26" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In review</x:v>
       </x:c>
       <x:c r="I26" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J26" s="32" t="str">
-        <x:v>Queue exhausted</x:v>
+        <x:v>Raw extraction</x:v>
       </x:c>
       <x:c r="K26" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="L26" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M26" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N26" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O26" s="32" t="str">
-        <x:v>First Bitcoin Design implementation slice. The current additive winner is custody.human-readable-addresses; encrypted cloud backups remains the main deferred neighbor from this design source family. Current tracked payment-format queue is exhausted for this pass.</x:v>
+        <x:v>Post title: SHA-256 explained Part 2: Message Schedule.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoin-dev-project-post-2012233826504933706</x:v>
       </x:c>
       <x:c r="B27" s="32" t="str">
-        <x:v>Bitcoin Design Wallet Activity Context</x:v>
+        <x:v>Bitcoin Dev Project: SHA-256 Explained</x:v>
       </x:c>
       <x:c r="C27" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/daily-spending-wallet/activity/</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/2012233826504933706</x:v>
       </x:c>
       <x:c r="D27" s="32" t="str">
-        <x:v>guide-cluster</x:v>
+        <x:v>social-post</x:v>
       </x:c>
       <x:c r="E27" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F27" s="32" t="str">
-        <x:v>User-facing wallet activity, contacts, and contextual payment-history concepts that help learners distinguish on-chain events from wallet-added meaning.</x:v>
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
       </x:c>
       <x:c r="G27" s="32" t="str">
-        <x:v>Track activity and contacts pages together so contextual metadata stays separate from backup flows and from protocol transaction mechanics.</x:v>
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H27" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In review</x:v>
       </x:c>
       <x:c r="I27" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J27" s="32" t="str">
-        <x:v>Queue exhausted</x:v>
+        <x:v>Raw extraction</x:v>
       </x:c>
       <x:c r="K27" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="L27" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M27" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N27" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O27" s="32" t="str">
-        <x:v>Second Bitcoin Design implementation slice. The current additive winner is custody.transaction-metadata; encrypted cloud backups remains the main deferred design-side candidate. Current tracked activity-and-contacts queue is exhausted for this pass.</x:v>
+        <x:v>Post title: SHA-256 explained.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32" t="str">
-        <x:v>source.bitcoin-design-multiple-wallets</x:v>
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
       </x:c>
       <x:c r="B28" s="32" t="str">
-        <x:v>Bitcoin Design Multiple Wallets</x:v>
+        <x:v>Bitcoin Dev Project: MAST Explained</x:v>
       </x:c>
       <x:c r="C28" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/multiple-wallets/</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1998431297333501989</x:v>
       </x:c>
       <x:c r="D28" s="32" t="str">
-        <x:v>guide-cluster</x:v>
+        <x:v>social-post</x:v>
       </x:c>
       <x:c r="E28" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F28" s="32" t="str">
-        <x:v>User-facing wallet architecture around separating funds by purpose, ownership, and security model inside one application.</x:v>
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
       </x:c>
       <x:c r="G28" s="32" t="str">
-        <x:v>Track the multiple-wallets page separately so purpose-based wallet separation stays distinct from account-path mechanics, backup flows, and generic wallet activity metadata.</x:v>
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H28" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In review</x:v>
       </x:c>
       <x:c r="I28" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J28" s="32" t="str">
-        <x:v>Queue exhausted</x:v>
+        <x:v>Raw extraction</x:v>
       </x:c>
       <x:c r="K28" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="L28" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M28" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N28" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O28" s="32" t="str">
-        <x:v>Third Bitcoin Design implementation slice. The current additive winner is custody.multiple-wallets; encrypted cloud backups remains deferred because it overlaps too heavily with backups-recovery. Current tracked page queue is exhausted for this pass.</x:v>
+        <x:v>Post title: MAST (Merkelized Alternative Script Tree) explained simply.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="32" t="str">
-        <x:v>source.bitcoin-design-cloud-backup</x:v>
+        <x:v>source.bitcoin-dev-project-post-1993443012748415027</x:v>
       </x:c>
       <x:c r="B29" s="32" t="str">
-        <x:v>Bitcoin Design Automatic Cloud Backup</x:v>
+        <x:v>Bitcoin Dev Project: CPFP Explained</x:v>
       </x:c>
       <x:c r="C29" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/how-it-works/private-key-management/cloud-backup/</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1993443012748415027</x:v>
       </x:c>
       <x:c r="D29" s="32" t="str">
-        <x:v>guide-cluster</x:v>
+        <x:v>social-post</x:v>
       </x:c>
       <x:c r="E29" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F29" s="32" t="str">
-        <x:v>User-facing backup scheme that stores encrypted wallet recovery data with an OS or cloud provider for low-friction restoration.</x:v>
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
       </x:c>
       <x:c r="G29" s="32" t="str">
-        <x:v>Track the conceptual cloud-backup page, the daily-spending reference flow, and the private-key-management overview together so the scheme can be deduped against existing backup and Lightning recovery coverage.</x:v>
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H29" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In review</x:v>
       </x:c>
       <x:c r="I29" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J29" s="32" t="str">
-        <x:v>Normalized to existing</x:v>
+        <x:v>Raw extraction</x:v>
       </x:c>
       <x:c r="K29" s="32" t="str">
-        <x:v>Merged into existing</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="L29" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M29" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N29" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O29" s="32" t="str">
-        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is backup-scheme tradeoffs that already fit custody.backups-recovery plus lightning.channel-backups.</x:v>
+        <x:v>Post title: Child-Pays-For-Parent transaction explained.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
       </x:c>
       <x:c r="B30" s="32" t="str">
-        <x:v>Bitcoin Design Upgradeable Wallet</x:v>
+        <x:v>Bitcoin Dev Project: Quadratic SIGHASH Problem Explained</x:v>
       </x:c>
       <x:c r="C30" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/upgradeable-wallet/</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1987562939109306699</x:v>
       </x:c>
       <x:c r="D30" s="32" t="str">
-        <x:v>guide-cluster</x:v>
+        <x:v>social-post</x:v>
       </x:c>
       <x:c r="E30" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F30" s="32" t="str">
-        <x:v>User-facing wallet architecture for progressive security and staged upgrades between key-management schemes.</x:v>
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
       </x:c>
       <x:c r="G30" s="32" t="str">
-        <x:v>Track the upgradeable-wallet reference design separately so progressive security becomes its own concept instead of staying buried inside cloud-backup discussions or multiwallet archival flows.</x:v>
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H30" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In review</x:v>
       </x:c>
       <x:c r="I30" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J30" s="32" t="str">
-        <x:v>Queue exhausted</x:v>
+        <x:v>Raw extraction</x:v>
       </x:c>
       <x:c r="K30" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="L30" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M30" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N30" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O30" s="32" t="str">
-        <x:v>Fourth Bitcoin Design implementation slice candidate. The current additive winner is custody.progressive-security, which survives dedupe more cleanly than automatic cloud backups or wallet-encryption. Current tracked page queue is exhausted for this pass.</x:v>
+        <x:v>Post title: Quadratic Sighash problem O(n^2) explained.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="str">
-        <x:v>source.bitcoin-design-shared-wallet</x:v>
+        <x:v>source.bitcoin-dev-project-post-1982189369684336693</x:v>
       </x:c>
       <x:c r="B31" s="32" t="str">
-        <x:v>Bitcoin Design Shared Wallet</x:v>
+        <x:v>Bitcoin Dev Project: BIP 158 Compact Block Filters Explained</x:v>
       </x:c>
       <x:c r="C31" s="32" t="str">
-        <x:v>https://bitcoin.design/guide/shared-wallet/</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1982189369684336693</x:v>
       </x:c>
       <x:c r="D31" s="32" t="str">
-        <x:v>guide-cluster</x:v>
+        <x:v>social-post</x:v>
       </x:c>
       <x:c r="E31" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F31" s="32" t="str">
-        <x:v>Reference design for co-managed wallets using multi-key schemes, provider-held recovery keys, and household approval policies.</x:v>
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
       </x:c>
       <x:c r="G31" s="32" t="str">
-        <x:v>Track the shared-wallet page together with the generic multi-key explanation so persona-specific multisig scenarios are deduped against existing custody mechanism nodes.</x:v>
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H31" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In review</x:v>
       </x:c>
       <x:c r="I31" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J31" s="32" t="str">
-        <x:v>Normalized to existing</x:v>
+        <x:v>Raw extraction</x:v>
       </x:c>
       <x:c r="K31" s="32" t="str">
-        <x:v>Merged into existing</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="L31" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M31" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N31" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O31" s="32" t="str">
-        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is shared-wallet examples for custody.multisig, custody.multiple-wallets, and custody.progressive-security.</x:v>
+        <x:v>Post title: BIP 158: Compact Block Filters explained.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.bitcoin-dev-project-post-1981761265036144901</x:v>
       </x:c>
       <x:c r="B32" s="32" t="str">
-        <x:v>Bitcoin Developer Guides</x:v>
+        <x:v>Bitcoin Dev Project: Duplicate Transaction Merkle Root Collision Explained</x:v>
       </x:c>
       <x:c r="C32" s="32" t="str">
-        <x:v>https://developer.bitcoin.org/devguide/</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1981761265036144901</x:v>
       </x:c>
       <x:c r="D32" s="32" t="str">
-        <x:v>documentation-cluster</x:v>
+        <x:v>social-post</x:v>
       </x:c>
       <x:c r="E32" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F32" s="32" t="str">
-        <x:v>Canonical developer-facing guide sections covering block chain, transactions, contracts, wallets, payment processing, operating modes, P2P network, and mining.</x:v>
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
       </x:c>
       <x:c r="G32" s="32" t="str">
-        <x:v>Track the eight top-level guide sections first, then split dense sections like Transactions, Contracts, Wallets, and P2P Network when they expose concept gaps not already covered by existing nodes.</x:v>
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H32" s="32" t="str">
         <x:v>In review</x:v>
       </x:c>
       <x:c r="I32" s="32" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="J32" s="32" t="str">
-        <x:v>Queue exhausted</x:v>
+        <x:v>Raw extraction</x:v>
       </x:c>
       <x:c r="K32" s="32" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="L32" s="32" t="n">
-        <x:v>9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M32" s="32" t="n">
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N32" s="32" t="n">
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O32" s="32" t="str">
-        <x:v>Added after the current audited source queue was exhausted. The first pass across the top-level sections surfaced four clean candidates: protocol.bitcoin-uri-bip21 from Payment Processing, dev.hardened-keys from Wallets, protocol.escrow-and-arbitration from Contracts, and mining.pool-shares from Pool Mining. A follow-up Wallet Files pass surfaced dev.wallet-import-format-wif as another clean wallet-standard slice. The implemented winners are now protocol.bitcoin-uri-bip21, dev.hardened-keys, protocol.escrow-and-arbitration, dev.wallet-import-format-wif, and mining.pool-shares because they land as missing standards, key-derivation, contract-pattern, key-serialization, and pooled-mining accounting bridges with clean direct parents. The current tracked top-level-plus-Wallet-Files queue is exhausted for this pass, though future deeper section splits may still surface more concepts.</x:v>
+        <x:v>Post title: CVE-2012-2459: Duplicate Transaction Merkle Root Collision Explained.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="32" t="str">
-        <x:v>source.bitcoin-core-operator-docs</x:v>
+        <x:v>source.bitcoin-dev-project-post-1980708369620168949</x:v>
       </x:c>
       <x:c r="B33" s="32" t="str">
-        <x:v>Bitcoin Core Operator Documentation</x:v>
+        <x:v>Bitcoin Dev Project: Discreet Log Contracts Explained</x:v>
       </x:c>
       <x:c r="C33" s="32" t="str">
-        <x:v>https://github.com/bitcoin/bitcoin/tree/master/doc</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1980708369620168949</x:v>
       </x:c>
       <x:c r="D33" s="32" t="str">
-        <x:v>implementation-documentation-cluster</x:v>
+        <x:v>social-post</x:v>
       </x:c>
       <x:c r="E33" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F33" s="32" t="str">
-        <x:v>Bitcoin Core's operator-facing documentation and configuration references for securing node control surfaces, especially JSON-RPC exposure and credentials.</x:v>
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
       </x:c>
       <x:c r="G33" s="32" t="str">
-        <x:v>Track the JSON-RPC interface security section, bitcoin.conf reference, and implementation configuration paths as one operator-security cluster before splitting distinct access-control or privacy concepts.</x:v>
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H33" s="32" t="str">
         <x:v>In review</x:v>
       </x:c>
       <x:c r="I33" s="32" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="J33" s="32" t="str">
         <x:v>Raw extraction</x:v>
@@ -1562,39 +1562,39 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="L33" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M33" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N33" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O33" s="32" t="str">
-        <x:v>Added after the audited queue surfaced a distinct RPC control-plane security gap. The first inspected cluster covers credentials, rpcbind/rpcallowip exposure, and the implementation path that applies these settings.</x:v>
+        <x:v>Post title: Discreet Log Contracts (DLC) explained simply.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="32" t="str">
-        <x:v>source.bitcoin-core-package-policy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1977486634536104288</x:v>
       </x:c>
       <x:c r="B34" s="32" t="str">
-        <x:v>Bitcoin Core Package Policy and Admission Documentation</x:v>
+        <x:v>Bitcoin Dev Project: Y2038 Problem Explained</x:v>
       </x:c>
       <x:c r="C34" s="32" t="str">
-        <x:v>https://github.com/bitcoin/bitcoin/blob/master/doc/policy/packages.md</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1977486634536104288</x:v>
       </x:c>
       <x:c r="D34" s="32" t="str">
-        <x:v>protocol-documentation-cluster</x:v>
+        <x:v>social-post</x:v>
       </x:c>
       <x:c r="E34" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F34" s="32" t="str">
-        <x:v>Bitcoin Core's package mempool acceptance rules, submitpackage RPC, and release history for local package admission and fee-bumping behavior.</x:v>
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
       </x:c>
       <x:c r="G34" s="32" t="str">
-        <x:v>Track the current submitpackage RPC reference, package-policy specification, and the 26.0 release note that introduced the RPC as one package-admission cluster; keep network package relay and cluster-mempool as deduplicated neighboring concepts.</x:v>
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H34" s="32" t="str">
         <x:v>In review</x:v>
@@ -1609,39 +1609,39 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="L34" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M34" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N34" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O34" s="32" t="str">
-        <x:v>Added after the RPC-security slice. The inspected pages establish submitpackage as a local package-admission mechanism and package RBF as a distinct replacement rule, separate from testmempoolaccept preflight, network package relay, and cluster-mempool internals.</x:v>
+        <x:v>Post title: The Y2038 problem explained.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="32" t="str">
-        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+        <x:v>source.bitcoin-dev-project-post-1977053708065423446</x:v>
       </x:c>
       <x:c r="B35" s="32" t="str">
-        <x:v>Bitcoin Core Cluster Mempool and RPC Documentation</x:v>
+        <x:v>Bitcoin Dev Project: Nonce Reuse Attack Explained</x:v>
       </x:c>
       <x:c r="C35" s="32" t="str">
-        <x:v>https://bitcoincore.org/en/doc/31.0.0/rpc/blockchain/getmempoolcluster/</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1977053708065423446</x:v>
       </x:c>
       <x:c r="D35" s="32" t="str">
-        <x:v>implementation-documentation-cluster</x:v>
+        <x:v>social-post</x:v>
       </x:c>
       <x:c r="E35" s="32" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F35" s="32" t="str">
-        <x:v>Bitcoin Core's cluster-mempool data model, bounded cluster policy, and related RPCs for inspecting connected transactions, mining order, chunks, fees, weights, and whole-mempool fee curves.</x:v>
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
       </x:c>
       <x:c r="G35" s="32" t="str">
-        <x:v>Track the getmempoolcluster and getmempoolfeeratediagram RPC references, cluster-limit policy, Bitcoin Core 31.0 release notes, mempool terminology, and implementation paths as one cluster-mempool slice; keep concrete RPC workflows merged into the higher-level concepts.</x:v>
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H35" s="32" t="str">
         <x:v>In review</x:v>
@@ -1656,15 +1656,1613 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="L35" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M35" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N35" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O35" s="32" t="str">
+        <x:v>Post title: Nonce Reuse Attack explained simply.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1976762610948198707</x:v>
+      </x:c>
+      <x:c r="B36" s="32" t="str">
+        <x:v>Bitcoin Dev Project: MuSig2 Explained</x:v>
+      </x:c>
+      <x:c r="C36" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1976762610948198707</x:v>
+      </x:c>
+      <x:c r="D36" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E36" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F36" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G36" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H36" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I36" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J36" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K36" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L36" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M36" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N36" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O36" s="32" t="str">
+        <x:v>Post title: MuSig2 explained simply; two-round Schnorr signature protocol.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1976416447577665743</x:v>
+      </x:c>
+      <x:c r="B37" s="32" t="str">
+        <x:v>Bitcoin Dev Project: MuSig Explained</x:v>
+      </x:c>
+      <x:c r="C37" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1976416447577665743</x:v>
+      </x:c>
+      <x:c r="D37" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E37" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F37" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G37" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H37" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I37" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J37" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K37" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L37" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M37" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N37" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O37" s="32" t="str">
+        <x:v>Post title: MuSig explained simply.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
+      </x:c>
+      <x:c r="B38" s="32" t="str">
+        <x:v>Bitcoin Dev Project: Schnorr Rogue-Key Attack Explained</x:v>
+      </x:c>
+      <x:c r="C38" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1976008010108678258</x:v>
+      </x:c>
+      <x:c r="D38" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E38" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F38" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G38" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H38" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I38" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J38" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K38" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L38" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M38" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N38" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O38" s="32" t="str">
+        <x:v>Post title: Schnorr signatures: Rogue key attack explained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+      </x:c>
+      <x:c r="B39" s="32" t="str">
+        <x:v>Bitcoin Dev Project: Selfish Mining Explained</x:v>
+      </x:c>
+      <x:c r="C39" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1975289920634925475</x:v>
+      </x:c>
+      <x:c r="D39" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E39" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F39" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G39" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H39" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I39" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J39" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K39" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L39" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M39" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N39" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O39" s="32" t="str">
+        <x:v>Post title: Selfish Mining explained simply.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1966579053076337056</x:v>
+      </x:c>
+      <x:c r="B40" s="32" t="str">
+        <x:v>Bitcoin Dev Project: SIGHASH Explained</x:v>
+      </x:c>
+      <x:c r="C40" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1966579053076337056</x:v>
+      </x:c>
+      <x:c r="D40" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E40" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F40" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G40" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H40" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I40" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J40" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K40" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L40" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M40" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N40" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O40" s="32" t="str">
+        <x:v>Post title: SigHash explained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1962245647261745216</x:v>
+      </x:c>
+      <x:c r="B41" s="32" t="str">
+        <x:v>Bitcoin Dev Project: Transaction Pinning Explained</x:v>
+      </x:c>
+      <x:c r="C41" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1962245647261745216</x:v>
+      </x:c>
+      <x:c r="D41" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E41" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F41" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G41" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H41" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I41" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J41" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K41" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L41" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M41" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N41" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O41" s="32" t="str">
+        <x:v>Post title: Transaction Pinning explained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1961882664803209229</x:v>
+      </x:c>
+      <x:c r="B42" s="32" t="str">
+        <x:v>Bitcoin Dev Project: SegWit Explained</x:v>
+      </x:c>
+      <x:c r="C42" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1961882664803209229</x:v>
+      </x:c>
+      <x:c r="D42" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E42" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F42" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G42" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H42" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I42" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J42" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K42" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L42" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M42" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N42" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O42" s="32" t="str">
+        <x:v>Post title: Segwit explained simply.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1956781577544896905</x:v>
+      </x:c>
+      <x:c r="B43" s="32" t="str">
+        <x:v>Bitcoin Dev Project: WOTS+ Key Generation Explained</x:v>
+      </x:c>
+      <x:c r="C43" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1956781577544896905</x:v>
+      </x:c>
+      <x:c r="D43" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E43" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F43" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G43" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H43" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I43" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J43" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K43" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L43" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M43" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N43" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O43" s="32" t="str">
+        <x:v>Post title: WOTS+ Key Generation explained; Part 4 of SPHINCS+.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1952320432033435819</x:v>
+      </x:c>
+      <x:c r="B44" s="32" t="str">
+        <x:v>Bitcoin Dev Project: WOTS Explained</x:v>
+      </x:c>
+      <x:c r="C44" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1952320432033435819</x:v>
+      </x:c>
+      <x:c r="D44" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E44" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F44" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G44" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H44" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I44" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J44" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K44" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L44" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M44" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N44" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O44" s="32" t="str">
+        <x:v>Post title: WOTS (Winternitz One-Time Signatures) explained; Part 3 of SPHINCS+.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1951962210902671675</x:v>
+      </x:c>
+      <x:c r="B45" s="32" t="str">
+        <x:v>Bitcoin Dev Project: SPHINCS+ and Lamport Signatures Explained</x:v>
+      </x:c>
+      <x:c r="C45" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1951962210902671675</x:v>
+      </x:c>
+      <x:c r="D45" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E45" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F45" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G45" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H45" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I45" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J45" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K45" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L45" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M45" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N45" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O45" s="32" t="str">
+        <x:v>Post title: SPHINCS+ explained; Part 2: Lamport Signatures.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1951704233742651737</x:v>
+      </x:c>
+      <x:c r="B46" s="32" t="str">
+        <x:v>Bitcoin Dev Project: SPHINCS+ Explained</x:v>
+      </x:c>
+      <x:c r="C46" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1951704233742651737</x:v>
+      </x:c>
+      <x:c r="D46" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E46" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F46" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G46" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H46" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I46" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J46" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K46" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L46" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M46" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N46" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O46" s="32" t="str">
+        <x:v>Post title: SPHINCS+ explained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1946961429363327053</x:v>
+      </x:c>
+      <x:c r="B47" s="32" t="str">
+        <x:v>Bitcoin Dev Project: Bitchat Explained</x:v>
+      </x:c>
+      <x:c r="C47" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1946961429363327053</x:v>
+      </x:c>
+      <x:c r="D47" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E47" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F47" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G47" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H47" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I47" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J47" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K47" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L47" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M47" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N47" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O47" s="32" t="str">
+        <x:v>Post title: Bitchat explained simply.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1945962367738601788</x:v>
+      </x:c>
+      <x:c r="B48" s="32" t="str">
+        <x:v>Bitcoin Dev Project: Compact Block Filter Explained</x:v>
+      </x:c>
+      <x:c r="C48" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1945962367738601788</x:v>
+      </x:c>
+      <x:c r="D48" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E48" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F48" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G48" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H48" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I48" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J48" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K48" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L48" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M48" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N48" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O48" s="32" t="str">
+        <x:v>Post title: Compact Block Filter explained, Part 1.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1945645540152135684</x:v>
+      </x:c>
+      <x:c r="B49" s="32" t="str">
+        <x:v>Bitcoin Dev Project: CPFP Explained, Earlier Post</x:v>
+      </x:c>
+      <x:c r="C49" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1945645540152135684</x:v>
+      </x:c>
+      <x:c r="D49" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E49" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F49" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G49" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H49" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I49" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J49" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K49" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L49" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M49" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N49" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O49" s="32" t="str">
+        <x:v>Post title: Child-Pays-For-Parent transaction explained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1934578478575489365</x:v>
+      </x:c>
+      <x:c r="B50" s="32" t="str">
+        <x:v>Bitcoin Dev Project: Lamport Signatures Explained</x:v>
+      </x:c>
+      <x:c r="C50" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1934578478575489365</x:v>
+      </x:c>
+      <x:c r="D50" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E50" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F50" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G50" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H50" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I50" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J50" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K50" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L50" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M50" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N50" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O50" s="32" t="str">
+        <x:v>Post title: Lamport Signatures Explained; quantum-resistant signature scheme.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
+      </x:c>
+      <x:c r="B51" s="32" t="str">
+        <x:v>Bitcoin Dev Project: Commit-Delay-Reveal Protocol Explained</x:v>
+      </x:c>
+      <x:c r="C51" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1931775486449103086</x:v>
+      </x:c>
+      <x:c r="D51" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E51" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F51" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G51" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H51" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I51" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J51" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K51" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L51" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M51" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N51" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O51" s="32" t="str">
+        <x:v>Post title: Commit-Delay-Reveal (CDR) Protocol explained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1905214178379362814</x:v>
+      </x:c>
+      <x:c r="B52" s="32" t="str">
+        <x:v>Bitcoin Dev Project: CISA Full Aggregation Explained</x:v>
+      </x:c>
+      <x:c r="C52" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1905214178379362814</x:v>
+      </x:c>
+      <x:c r="D52" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E52" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F52" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G52" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H52" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I52" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J52" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K52" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L52" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M52" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N52" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O52" s="32" t="str">
+        <x:v>Post title: CISA: Full-Aggregation explained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+      </x:c>
+      <x:c r="B53" s="32" t="str">
+        <x:v>Bitcoin Dev Project: Dust Attack Explained</x:v>
+      </x:c>
+      <x:c r="C53" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1904946739603452376</x:v>
+      </x:c>
+      <x:c r="D53" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E53" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F53" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G53" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H53" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I53" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J53" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K53" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L53" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M53" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N53" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O53" s="32" t="str">
+        <x:v>Post title: Dust Attacked explained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1904596944649150556</x:v>
+      </x:c>
+      <x:c r="B54" s="32" t="str">
+        <x:v>Bitcoin Dev Project: CISA Half Signature Aggregation Explained</x:v>
+      </x:c>
+      <x:c r="C54" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1904596944649150556</x:v>
+      </x:c>
+      <x:c r="D54" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E54" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F54" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G54" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H54" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I54" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J54" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K54" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L54" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M54" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N54" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O54" s="32" t="str">
+        <x:v>Post title: CISA Part 2: Half Signature Aggregation explained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1904136400213340298</x:v>
+      </x:c>
+      <x:c r="B55" s="32" t="str">
+        <x:v>Bitcoin Dev Project: CISA Explained</x:v>
+      </x:c>
+      <x:c r="C55" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1904136400213340298</x:v>
+      </x:c>
+      <x:c r="D55" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E55" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F55" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G55" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H55" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I55" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J55" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K55" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L55" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M55" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N55" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O55" s="32" t="str">
+        <x:v>Post title: CISA (Cross Input Signature Aggregation) explained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1903881770204070155</x:v>
+      </x:c>
+      <x:c r="B56" s="32" t="str">
+        <x:v>Bitcoin Dev Project: Transaction Pinning Attack Explained</x:v>
+      </x:c>
+      <x:c r="C56" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1903881770204070155</x:v>
+      </x:c>
+      <x:c r="D56" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E56" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F56" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G56" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H56" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I56" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J56" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K56" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L56" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M56" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N56" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O56" s="32" t="str">
+        <x:v>Post title: Transaction Pinning Attack explained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1903150655071719663</x:v>
+      </x:c>
+      <x:c r="B57" s="32" t="str">
+        <x:v>Bitcoin Dev Project: BIP 68 Sequence Number Explained</x:v>
+      </x:c>
+      <x:c r="C57" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1903150655071719663</x:v>
+      </x:c>
+      <x:c r="D57" s="32" t="str">
+        <x:v>social-post</x:v>
+      </x:c>
+      <x:c r="E57" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F57" s="32" t="str">
+        <x:v>One explained post from the Bitcoin Dev Project search family.</x:v>
+      </x:c>
+      <x:c r="G57" s="32" t="str">
+        <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
+      </x:c>
+      <x:c r="H57" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I57" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J57" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K57" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L57" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M57" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N57" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O57" s="32" t="str">
+        <x:v>Post title: BIP-68 (Sequence number) explained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="32" t="str">
+        <x:v>source.bitcoin-core-academy-wallet</x:v>
+      </x:c>
+      <x:c r="B58" s="32" t="str">
+        <x:v>Bitcoin Core Academy Wallet Internals</x:v>
+      </x:c>
+      <x:c r="C58" s="32" t="str">
+        <x:v>https://bitcoincore.academy/scriptpubkeymanagers.html</x:v>
+      </x:c>
+      <x:c r="D58" s="32" t="str">
+        <x:v>course-cluster</x:v>
+      </x:c>
+      <x:c r="E58" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F58" s="32" t="str">
+        <x:v>Wallet internals cluster around ScriptPubKeyManagers, wallet keys, transaction identification, and balance calculation.</x:v>
+      </x:c>
+      <x:c r="G58" s="32" t="str">
+        <x:v>Track one wallet-internals page cluster at a time so Core-specific abstractions stay atomic instead of collapsing into generic wallet concepts.</x:v>
+      </x:c>
+      <x:c r="H58" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I58" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J58" s="32" t="str">
+        <x:v>Queue exhausted</x:v>
+      </x:c>
+      <x:c r="K58" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L58" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M58" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N58" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O58" s="32" t="str">
+        <x:v>First additional-source pass beyond the mandatory seed list. The current additive winner is dev.scriptpubkeymanagers; wallet-encryption remains deferred because the cleanest surviving slice is still too coupled to missing Core wallet-internals parents. Current tracked wallet-internals queue is exhausted for this pass.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="32" t="str">
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
+      </x:c>
+      <x:c r="B59" s="32" t="str">
+        <x:v>Bitcoin Core Academy Mempool Mechanics</x:v>
+      </x:c>
+      <x:c r="C59" s="32" t="str">
+        <x:v>https://bitcoincore.academy/mempool-unbroadcast.html</x:v>
+      </x:c>
+      <x:c r="D59" s="32" t="str">
+        <x:v>course-cluster</x:v>
+      </x:c>
+      <x:c r="E59" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F59" s="32" t="str">
+        <x:v>Mempool and relay internals cluster around transaction relay, rebroadcast behavior, and local node transaction state.</x:v>
+      </x:c>
+      <x:c r="G59" s="32" t="str">
+        <x:v>Track the academy mempool pages as a separate cluster so implementation-specific relay mechanisms are not collapsed into generic mempool coverage.</x:v>
+      </x:c>
+      <x:c r="H59" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I59" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J59" s="32" t="str">
+        <x:v>Queue exhausted</x:v>
+      </x:c>
+      <x:c r="K59" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L59" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M59" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N59" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O59" s="32" t="str">
+        <x:v>Second post-seed-source slice. The current additive winners are protocol.mempool-unbroadcast-set, protocol.transaction-rebroadcast-privacy, and protocol.txid-vs-wtxid. The remaining transaction-format internals are now mostly implementation-detail material rather than clean learner-facing nodes. Current tracked mempool queue is exhausted for this pass.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="32" t="str">
+        <x:v>source.bitcoin-design-payment-formats</x:v>
+      </x:c>
+      <x:c r="B60" s="32" t="str">
+        <x:v>Bitcoin Design Payment Request Formats</x:v>
+      </x:c>
+      <x:c r="C60" s="32" t="str">
+        <x:v>https://bitcoin.design/guide/how-it-works/human-readable-addresses/</x:v>
+      </x:c>
+      <x:c r="D60" s="32" t="str">
+        <x:v>guide-cluster</x:v>
+      </x:c>
+      <x:c r="E60" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F60" s="32" t="str">
+        <x:v>User-facing payment request and address-sharing concepts across human-readable addresses, transaction display, and wallet privacy tradeoffs.</x:v>
+      </x:c>
+      <x:c r="G60" s="32" t="str">
+        <x:v>Track design guide pages by UX concept cluster so user-facing payment abstractions stay separate from protocol internals and generic wallet hygiene.</x:v>
+      </x:c>
+      <x:c r="H60" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I60" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J60" s="32" t="str">
+        <x:v>Queue exhausted</x:v>
+      </x:c>
+      <x:c r="K60" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L60" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M60" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N60" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O60" s="32" t="str">
+        <x:v>First Bitcoin Design implementation slice. The current additive winner is custody.human-readable-addresses; encrypted cloud backups remains the main deferred neighbor from this design source family. Current tracked payment-format queue is exhausted for this pass.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="32" t="str">
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
+      </x:c>
+      <x:c r="B61" s="32" t="str">
+        <x:v>Bitcoin Design Wallet Activity Context</x:v>
+      </x:c>
+      <x:c r="C61" s="32" t="str">
+        <x:v>https://bitcoin.design/guide/daily-spending-wallet/activity/</x:v>
+      </x:c>
+      <x:c r="D61" s="32" t="str">
+        <x:v>guide-cluster</x:v>
+      </x:c>
+      <x:c r="E61" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F61" s="32" t="str">
+        <x:v>User-facing wallet activity, contacts, and contextual payment-history concepts that help learners distinguish on-chain events from wallet-added meaning.</x:v>
+      </x:c>
+      <x:c r="G61" s="32" t="str">
+        <x:v>Track activity and contacts pages together so contextual metadata stays separate from backup flows and from protocol transaction mechanics.</x:v>
+      </x:c>
+      <x:c r="H61" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I61" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J61" s="32" t="str">
+        <x:v>Queue exhausted</x:v>
+      </x:c>
+      <x:c r="K61" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L61" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M61" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N61" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O61" s="32" t="str">
+        <x:v>Second Bitcoin Design implementation slice. The current additive winner is custody.transaction-metadata; encrypted cloud backups remains the main deferred design-side candidate. Current tracked activity-and-contacts queue is exhausted for this pass.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="32" t="str">
+        <x:v>source.bitcoin-design-multiple-wallets</x:v>
+      </x:c>
+      <x:c r="B62" s="32" t="str">
+        <x:v>Bitcoin Design Multiple Wallets</x:v>
+      </x:c>
+      <x:c r="C62" s="32" t="str">
+        <x:v>https://bitcoin.design/guide/multiple-wallets/</x:v>
+      </x:c>
+      <x:c r="D62" s="32" t="str">
+        <x:v>guide-cluster</x:v>
+      </x:c>
+      <x:c r="E62" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F62" s="32" t="str">
+        <x:v>User-facing wallet architecture around separating funds by purpose, ownership, and security model inside one application.</x:v>
+      </x:c>
+      <x:c r="G62" s="32" t="str">
+        <x:v>Track the multiple-wallets page separately so purpose-based wallet separation stays distinct from account-path mechanics, backup flows, and generic wallet activity metadata.</x:v>
+      </x:c>
+      <x:c r="H62" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I62" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J62" s="32" t="str">
+        <x:v>Queue exhausted</x:v>
+      </x:c>
+      <x:c r="K62" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L62" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M62" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N62" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O62" s="32" t="str">
+        <x:v>Third Bitcoin Design implementation slice. The current additive winner is custody.multiple-wallets; encrypted cloud backups remains deferred because it overlaps too heavily with backups-recovery. Current tracked page queue is exhausted for this pass.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="32" t="str">
+        <x:v>source.bitcoin-design-cloud-backup</x:v>
+      </x:c>
+      <x:c r="B63" s="32" t="str">
+        <x:v>Bitcoin Design Automatic Cloud Backup</x:v>
+      </x:c>
+      <x:c r="C63" s="32" t="str">
+        <x:v>https://bitcoin.design/guide/how-it-works/private-key-management/cloud-backup/</x:v>
+      </x:c>
+      <x:c r="D63" s="32" t="str">
+        <x:v>guide-cluster</x:v>
+      </x:c>
+      <x:c r="E63" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F63" s="32" t="str">
+        <x:v>User-facing backup scheme that stores encrypted wallet recovery data with an OS or cloud provider for low-friction restoration.</x:v>
+      </x:c>
+      <x:c r="G63" s="32" t="str">
+        <x:v>Track the conceptual cloud-backup page, the daily-spending reference flow, and the private-key-management overview together so the scheme can be deduped against existing backup and Lightning recovery coverage.</x:v>
+      </x:c>
+      <x:c r="H63" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I63" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J63" s="32" t="str">
+        <x:v>Normalized to existing</x:v>
+      </x:c>
+      <x:c r="K63" s="32" t="str">
+        <x:v>Merged into existing</x:v>
+      </x:c>
+      <x:c r="L63" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M63" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N63" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O63" s="32" t="str">
+        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is backup-scheme tradeoffs that already fit custody.backups-recovery plus lightning.channel-backups.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="32" t="str">
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+      </x:c>
+      <x:c r="B64" s="32" t="str">
+        <x:v>Bitcoin Design Upgradeable Wallet</x:v>
+      </x:c>
+      <x:c r="C64" s="32" t="str">
+        <x:v>https://bitcoin.design/guide/upgradeable-wallet/</x:v>
+      </x:c>
+      <x:c r="D64" s="32" t="str">
+        <x:v>guide-cluster</x:v>
+      </x:c>
+      <x:c r="E64" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F64" s="32" t="str">
+        <x:v>User-facing wallet architecture for progressive security and staged upgrades between key-management schemes.</x:v>
+      </x:c>
+      <x:c r="G64" s="32" t="str">
+        <x:v>Track the upgradeable-wallet reference design separately so progressive security becomes its own concept instead of staying buried inside cloud-backup discussions or multiwallet archival flows.</x:v>
+      </x:c>
+      <x:c r="H64" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I64" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J64" s="32" t="str">
+        <x:v>Queue exhausted</x:v>
+      </x:c>
+      <x:c r="K64" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L64" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M64" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N64" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O64" s="32" t="str">
+        <x:v>Fourth Bitcoin Design implementation slice candidate. The current additive winner is custody.progressive-security, which survives dedupe more cleanly than automatic cloud backups or wallet-encryption. Current tracked page queue is exhausted for this pass.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="32" t="str">
+        <x:v>source.bitcoin-design-shared-wallet</x:v>
+      </x:c>
+      <x:c r="B65" s="32" t="str">
+        <x:v>Bitcoin Design Shared Wallet</x:v>
+      </x:c>
+      <x:c r="C65" s="32" t="str">
+        <x:v>https://bitcoin.design/guide/shared-wallet/</x:v>
+      </x:c>
+      <x:c r="D65" s="32" t="str">
+        <x:v>guide-cluster</x:v>
+      </x:c>
+      <x:c r="E65" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F65" s="32" t="str">
+        <x:v>Reference design for co-managed wallets using multi-key schemes, provider-held recovery keys, and household approval policies.</x:v>
+      </x:c>
+      <x:c r="G65" s="32" t="str">
+        <x:v>Track the shared-wallet page together with the generic multi-key explanation so persona-specific multisig scenarios are deduped against existing custody mechanism nodes.</x:v>
+      </x:c>
+      <x:c r="H65" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I65" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J65" s="32" t="str">
+        <x:v>Normalized to existing</x:v>
+      </x:c>
+      <x:c r="K65" s="32" t="str">
+        <x:v>Merged into existing</x:v>
+      </x:c>
+      <x:c r="L65" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M65" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N65" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O65" s="32" t="str">
+        <x:v>Reviewed and merged into existing coverage instead of minting a node. The enduring source value is shared-wallet examples for custody.multisig, custody.multiple-wallets, and custody.progressive-security.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="32" t="str">
+        <x:v>source.bitcoin-developer-guides</x:v>
+      </x:c>
+      <x:c r="B66" s="32" t="str">
+        <x:v>Bitcoin Developer Guides</x:v>
+      </x:c>
+      <x:c r="C66" s="32" t="str">
+        <x:v>https://developer.bitcoin.org/devguide/</x:v>
+      </x:c>
+      <x:c r="D66" s="32" t="str">
+        <x:v>documentation-cluster</x:v>
+      </x:c>
+      <x:c r="E66" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F66" s="32" t="str">
+        <x:v>Canonical developer-facing guide sections covering block chain, transactions, contracts, wallets, payment processing, operating modes, P2P network, and mining.</x:v>
+      </x:c>
+      <x:c r="G66" s="32" t="str">
+        <x:v>Track the eight top-level guide sections first, then split dense sections like Transactions, Contracts, Wallets, and P2P Network when they expose concept gaps not already covered by existing nodes.</x:v>
+      </x:c>
+      <x:c r="H66" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I66" s="32" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="J66" s="32" t="str">
+        <x:v>Queue exhausted</x:v>
+      </x:c>
+      <x:c r="K66" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L66" s="32" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="M66" s="32" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="M35" s="32" t="n">
+      <x:c r="N66" s="32" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O66" s="32" t="str">
+        <x:v>Added after the current audited source queue was exhausted. The first pass across the top-level sections surfaced four clean candidates: protocol.bitcoin-uri-bip21 from Payment Processing, dev.hardened-keys from Wallets, protocol.escrow-and-arbitration from Contracts, and mining.pool-shares from Pool Mining. A follow-up Wallet Files pass surfaced dev.wallet-import-format-wif as another clean wallet-standard slice. The implemented winners are now protocol.bitcoin-uri-bip21, dev.hardened-keys, protocol.escrow-and-arbitration, dev.wallet-import-format-wif, and mining.pool-shares because they land as missing standards, key-derivation, contract-pattern, key-serialization, and pooled-mining accounting bridges with clean direct parents. The current tracked top-level-plus-Wallet-Files queue is exhausted for this pass, though future deeper section splits may still surface more concepts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="32" t="str">
+        <x:v>source.bitcoin-core-operator-docs</x:v>
+      </x:c>
+      <x:c r="B67" s="32" t="str">
+        <x:v>Bitcoin Core Operator Documentation</x:v>
+      </x:c>
+      <x:c r="C67" s="32" t="str">
+        <x:v>https://github.com/bitcoin/bitcoin/tree/master/doc</x:v>
+      </x:c>
+      <x:c r="D67" s="32" t="str">
+        <x:v>implementation-documentation-cluster</x:v>
+      </x:c>
+      <x:c r="E67" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F67" s="32" t="str">
+        <x:v>Bitcoin Core's operator-facing documentation and configuration references for securing node control surfaces, especially JSON-RPC exposure and credentials.</x:v>
+      </x:c>
+      <x:c r="G67" s="32" t="str">
+        <x:v>Track the JSON-RPC interface security section, bitcoin.conf reference, and implementation configuration paths as one operator-security cluster before splitting distinct access-control or privacy concepts.</x:v>
+      </x:c>
+      <x:c r="H67" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I67" s="32" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="J67" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K67" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L67" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="N35" s="32" t="n">
+      <x:c r="M67" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N67" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O67" s="32" t="str">
+        <x:v>Added after the audited queue surfaced a distinct RPC control-plane security gap. The first inspected cluster covers credentials, rpcbind/rpcallowip exposure, and the implementation path that applies these settings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="32" t="str">
+        <x:v>source.bitcoin-core-package-policy</x:v>
+      </x:c>
+      <x:c r="B68" s="32" t="str">
+        <x:v>Bitcoin Core Package Policy and Admission Documentation</x:v>
+      </x:c>
+      <x:c r="C68" s="32" t="str">
+        <x:v>https://github.com/bitcoin/bitcoin/blob/master/doc/policy/packages.md</x:v>
+      </x:c>
+      <x:c r="D68" s="32" t="str">
+        <x:v>protocol-documentation-cluster</x:v>
+      </x:c>
+      <x:c r="E68" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F68" s="32" t="str">
+        <x:v>Bitcoin Core's package mempool acceptance rules, submitpackage RPC, and release history for local package admission and fee-bumping behavior.</x:v>
+      </x:c>
+      <x:c r="G68" s="32" t="str">
+        <x:v>Track the current submitpackage RPC reference, package-policy specification, and the 26.0 release note that introduced the RPC as one package-admission cluster; keep network package relay and cluster-mempool as deduplicated neighboring concepts.</x:v>
+      </x:c>
+      <x:c r="H68" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I68" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J68" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K68" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L68" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="O35" s="32" t="str">
+      <x:c r="M68" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N68" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O68" s="32" t="str">
+        <x:v>Added after the RPC-security slice. The inspected pages establish submitpackage as a local package-admission mechanism and package RBF as a distinct replacement rule, separate from testmempoolaccept preflight, network package relay, and cluster-mempool internals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="32" t="str">
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+      </x:c>
+      <x:c r="B69" s="32" t="str">
+        <x:v>Bitcoin Core Cluster Mempool and RPC Documentation</x:v>
+      </x:c>
+      <x:c r="C69" s="32" t="str">
+        <x:v>https://bitcoincore.org/en/doc/31.0.0/rpc/blockchain/getmempoolcluster/</x:v>
+      </x:c>
+      <x:c r="D69" s="32" t="str">
+        <x:v>implementation-documentation-cluster</x:v>
+      </x:c>
+      <x:c r="E69" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F69" s="32" t="str">
+        <x:v>Bitcoin Core's cluster-mempool data model, bounded cluster policy, and related RPCs for inspecting connected transactions, mining order, chunks, fees, weights, and whole-mempool fee curves.</x:v>
+      </x:c>
+      <x:c r="G69" s="32" t="str">
+        <x:v>Track the getmempoolcluster and getmempoolfeeratediagram RPC references, cluster-limit policy, Bitcoin Core 31.0 release notes, mempool terminology, and implementation paths as one cluster-mempool slice; keep concrete RPC workflows merged into the higher-level concepts.</x:v>
+      </x:c>
+      <x:c r="H69" s="32" t="str">
+        <x:v>In review</x:v>
+      </x:c>
+      <x:c r="I69" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J69" s="32" t="str">
+        <x:v>Raw extraction</x:v>
+      </x:c>
+      <x:c r="K69" s="32" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="L69" s="32" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M69" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N69" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O69" s="32" t="str">
         <x:v>Added after the package-RBF slice. The inspected documentation exposes two RPC implementation surfaces, both merged into protocol.cluster-mempool, plus a distinct learner-facing policy concept: bounded cluster limits replacing legacy ancestor/descendant limits.</x:v>
       </x:c>
     </x:row>
@@ -1674,16 +3272,16 @@
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H35">
+    <x:dataValidation type="list" sqref="H12:H69">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I35">
+    <x:dataValidation type="list" sqref="I12:I69">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J35">
+    <x:dataValidation type="list" sqref="J12:J69">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K35">
+    <x:dataValidation type="list" sqref="K12:K69">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11837,7 +13435,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.68870096065</x:v>
+        <x:v>46214.69388914352</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -11845,7 +13443,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>24</x:v>
+        <x:v>58</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -11853,7 +13451,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="8">

</xml_diff>

<commit_message>
feat: expand explained Bitcoin concepts
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R63078c67377a4d36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Radf00d76b3c24a0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R7532f3c3e7464dd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Re55e02a1c0c7471b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R64c7aebe4175442a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R37608cb459bf4821"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R686efcd8451a4147"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rd4fba108478e42ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Re9c4bd089b1e451b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R0085eaf11b324b8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rd48952a9de9c40bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Re173d9b03b3a4cdf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1095,10 +1095,10 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="M23" s="32" t="n">
-        <x:v>6</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="N23" s="32" t="n">
-        <x:v>6</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="O23" s="32" t="str">
         <x:v>Reopened after audit correction. The authenticated X search was enumerated on July 11, 2026 and currently exposes 34 matching posts, which are now tracked individually below. The earlier July 8 pass reported 43 posts but did not preserve one source row per post; that historical count remains unresolved until the current and prior inventories are reconciled. Existing normalized coverage includes time-warp attack, duplicate transaction bug, 64-byte transaction bug, nonce reuse, Lamport signatures, and Shamir's Secret Sharing.</x:v>
@@ -1127,28 +1127,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H24" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I24" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J24" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K24" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L24" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M24" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N24" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O24" s="32" t="str">
-        <x:v>Post title: Coinjoin Explained.</x:v>
+        <x:v>Post title: Coinjoin Explained. Normalized as the canonical candidate for audit.post-2018682587045052753.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1174,28 +1174,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H25" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I25" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J25" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K25" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L25" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M25" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N25" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O25" s="32" t="str">
-        <x:v>Post title: Full Node Architecture Explained.</x:v>
+        <x:v>Post title: Full Node Architecture Explained. Normalized as the canonical candidate for audit.post-2017223553708654888.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1221,28 +1221,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H26" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I26" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J26" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K26" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L26" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M26" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N26" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O26" s="32" t="str">
-        <x:v>Post title: SHA-256 explained Part 2: Message Schedule.</x:v>
+        <x:v>Post title: SHA-256 explained Part 2: Message Schedule. Normalized as the canonical candidate for audit.post-2016929384389890484.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1268,28 +1268,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H27" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I27" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J27" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K27" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L27" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M27" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N27" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O27" s="32" t="str">
-        <x:v>Post title: SHA-256 explained.</x:v>
+        <x:v>Post title: SHA-256 explained. Normalized as the canonical candidate for audit.post-2012233826504933706.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1315,28 +1315,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H28" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I28" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J28" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K28" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L28" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M28" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N28" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O28" s="32" t="str">
-        <x:v>Post title: MAST (Merkelized Alternative Script Tree) explained simply.</x:v>
+        <x:v>Post title: MAST (Merkelized Alternative Script Tree) explained simply. Normalized as the canonical candidate for audit.post-1998431297333501989.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -1362,28 +1362,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H29" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I29" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J29" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K29" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L29" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M29" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N29" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O29" s="32" t="str">
-        <x:v>Post title: Child-Pays-For-Parent transaction explained.</x:v>
+        <x:v>Post title: Child-Pays-For-Parent transaction explained. Normalized as the canonical candidate for audit.post-1993443012748415027.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1409,28 +1409,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H30" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I30" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J30" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K30" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L30" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M30" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N30" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O30" s="32" t="str">
-        <x:v>Post title: Quadratic Sighash problem O(n^2) explained.</x:v>
+        <x:v>Post title: Quadratic Sighash problem O(n^2) explained. Normalized as the canonical candidate for audit.post-1987562939109306699.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -1456,28 +1456,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H31" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I31" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J31" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K31" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L31" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M31" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N31" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O31" s="32" t="str">
-        <x:v>Post title: BIP 158: Compact Block Filters explained.</x:v>
+        <x:v>Post title: BIP 158: Compact Block Filters explained. Normalized as the canonical candidate for audit.post-1982189369684336693.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -1503,28 +1503,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H32" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I32" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J32" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K32" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L32" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M32" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N32" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O32" s="32" t="str">
-        <x:v>Post title: CVE-2012-2459: Duplicate Transaction Merkle Root Collision Explained.</x:v>
+        <x:v>Post title: CVE-2012-2459: Duplicate Transaction Merkle Root Collision Explained. Normalized as the canonical candidate for audit.post-1981761265036144901.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -1550,28 +1550,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H33" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I33" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J33" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K33" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L33" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M33" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N33" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O33" s="32" t="str">
-        <x:v>Post title: Discreet Log Contracts (DLC) explained simply.</x:v>
+        <x:v>Post title: Discreet Log Contracts (DLC) explained simply. Normalized as the canonical candidate for audit.post-1980708369620168949.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -1597,28 +1597,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H34" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I34" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J34" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K34" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L34" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M34" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N34" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O34" s="32" t="str">
-        <x:v>Post title: The Y2038 problem explained.</x:v>
+        <x:v>Post title: The Y2038 problem explained. Normalized as the canonical candidate for audit.post-1977486634536104288.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -1644,28 +1644,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H35" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I35" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J35" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K35" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L35" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M35" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N35" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O35" s="32" t="str">
-        <x:v>Post title: Nonce Reuse Attack explained simply.</x:v>
+        <x:v>Post title: Nonce Reuse Attack explained simply. Normalized as the canonical candidate for audit.post-1977053708065423446.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -1691,28 +1691,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H36" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I36" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J36" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K36" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L36" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M36" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N36" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O36" s="32" t="str">
-        <x:v>Post title: MuSig2 explained simply; two-round Schnorr signature protocol.</x:v>
+        <x:v>Post title: MuSig2 explained simply; two-round Schnorr signature protocol. Normalized as the canonical candidate for audit.post-1976762610948198707.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -1738,28 +1738,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H37" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I37" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J37" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K37" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L37" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M37" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N37" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O37" s="32" t="str">
-        <x:v>Post title: MuSig explained simply.</x:v>
+        <x:v>Post title: MuSig explained simply. Normalized as the canonical candidate for audit.post-1976416447577665743.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -1785,28 +1785,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H38" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I38" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J38" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K38" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L38" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M38" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N38" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O38" s="32" t="str">
-        <x:v>Post title: Schnorr signatures: Rogue key attack explained.</x:v>
+        <x:v>Post title: Schnorr signatures: Rogue key attack explained. Normalized as the canonical candidate for audit.post-1976008010108678258.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -1832,28 +1832,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H39" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I39" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J39" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K39" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L39" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M39" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N39" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O39" s="32" t="str">
-        <x:v>Post title: Selfish Mining explained simply.</x:v>
+        <x:v>Post title: Selfish Mining explained simply. Normalized as the canonical candidate for audit.post-1975289920634925475.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -1879,28 +1879,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H40" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I40" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J40" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K40" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L40" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M40" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N40" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O40" s="32" t="str">
-        <x:v>Post title: SigHash explained.</x:v>
+        <x:v>Post title: SigHash explained. Normalized as the canonical candidate for audit.post-1966579053076337056.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -1926,28 +1926,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H41" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I41" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J41" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K41" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L41" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M41" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N41" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O41" s="32" t="str">
-        <x:v>Post title: Transaction Pinning explained.</x:v>
+        <x:v>Post title: Transaction Pinning explained. Normalized as the canonical candidate for audit.post-1962245647261745216.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -1973,28 +1973,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H42" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I42" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J42" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K42" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L42" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M42" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N42" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O42" s="32" t="str">
-        <x:v>Post title: Segwit explained simply.</x:v>
+        <x:v>Post title: Segwit explained simply. Normalized as the canonical candidate for audit.post-1961882664803209229.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -2020,28 +2020,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H43" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I43" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J43" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K43" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L43" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M43" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N43" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O43" s="32" t="str">
-        <x:v>Post title: WOTS+ Key Generation explained; Part 4 of SPHINCS+.</x:v>
+        <x:v>Post title: WOTS+ Key Generation explained; Part 4 of SPHINCS+. Normalized as the canonical candidate for audit.post-1956781577544896905.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -2067,28 +2067,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H44" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I44" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J44" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K44" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L44" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M44" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N44" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O44" s="32" t="str">
-        <x:v>Post title: WOTS (Winternitz One-Time Signatures) explained; Part 3 of SPHINCS+.</x:v>
+        <x:v>Post title: WOTS (Winternitz One-Time Signatures) explained; Part 3 of SPHINCS+. Normalized as the canonical candidate for audit.post-1952320432033435819.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -2114,28 +2114,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H45" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I45" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J45" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K45" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L45" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M45" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N45" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O45" s="32" t="str">
-        <x:v>Post title: SPHINCS+ explained; Part 2: Lamport Signatures.</x:v>
+        <x:v>Post title: SPHINCS+ explained; Part 2: Lamport Signatures. Normalized as the canonical candidate for audit.post-1951962210902671675.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -2161,28 +2161,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H46" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I46" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J46" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K46" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L46" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M46" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N46" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O46" s="32" t="str">
-        <x:v>Post title: SPHINCS+ explained.</x:v>
+        <x:v>Post title: SPHINCS+ explained. Normalized as the canonical candidate for audit.post-1951704233742651737.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -2208,28 +2208,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H47" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I47" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J47" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K47" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L47" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M47" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N47" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O47" s="32" t="str">
-        <x:v>Post title: Bitchat explained simply.</x:v>
+        <x:v>Post title: Bitchat explained simply. Normalized as the canonical candidate for audit.post-1946961429363327053.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2255,28 +2255,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H48" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I48" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J48" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K48" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L48" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M48" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N48" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O48" s="32" t="str">
-        <x:v>Post title: Compact Block Filter explained, Part 1.</x:v>
+        <x:v>Post title: Compact Block Filter explained, Part 1. Normalized as the canonical candidate for audit.post-1945962367738601788.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -2302,28 +2302,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H49" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I49" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J49" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K49" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L49" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M49" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N49" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O49" s="32" t="str">
-        <x:v>Post title: Child-Pays-For-Parent transaction explained.</x:v>
+        <x:v>Post title: Child-Pays-For-Parent transaction explained. Normalized as the canonical candidate for audit.post-1945645540152135684.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -2349,28 +2349,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H50" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I50" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J50" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K50" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L50" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M50" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N50" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O50" s="32" t="str">
-        <x:v>Post title: Lamport Signatures Explained; quantum-resistant signature scheme.</x:v>
+        <x:v>Post title: Lamport Signatures Explained; quantum-resistant signature scheme. Normalized as the canonical candidate for audit.post-1934578478575489365.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -2396,28 +2396,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H51" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I51" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J51" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K51" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L51" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M51" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N51" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O51" s="32" t="str">
-        <x:v>Post title: Commit-Delay-Reveal (CDR) Protocol explained.</x:v>
+        <x:v>Post title: Commit-Delay-Reveal (CDR) Protocol explained. Normalized as the canonical candidate for audit.post-1931775486449103086.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -2443,28 +2443,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H52" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I52" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J52" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K52" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L52" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M52" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N52" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O52" s="32" t="str">
-        <x:v>Post title: CISA: Full-Aggregation explained.</x:v>
+        <x:v>Post title: CISA: Full-Aggregation explained. Normalized as the canonical candidate for audit.post-1905214178379362814.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -2490,28 +2490,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H53" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I53" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J53" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K53" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L53" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M53" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N53" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O53" s="32" t="str">
-        <x:v>Post title: Dust Attacked explained.</x:v>
+        <x:v>Post title: Dust Attacked explained. Normalized as the canonical candidate for audit.post-1904946739603452376.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -2537,28 +2537,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H54" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I54" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J54" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K54" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L54" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M54" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N54" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O54" s="32" t="str">
-        <x:v>Post title: CISA Part 2: Half Signature Aggregation explained.</x:v>
+        <x:v>Post title: CISA Part 2: Half Signature Aggregation explained. Normalized as the canonical candidate for audit.post-1904596944649150556.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -2584,28 +2584,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H55" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I55" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J55" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K55" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L55" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M55" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N55" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O55" s="32" t="str">
-        <x:v>Post title: CISA (Cross Input Signature Aggregation) explained.</x:v>
+        <x:v>Post title: CISA (Cross Input Signature Aggregation) explained. Normalized as the canonical candidate for audit.post-1904136400213340298.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -2631,28 +2631,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H56" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I56" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J56" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K56" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L56" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M56" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N56" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O56" s="32" t="str">
-        <x:v>Post title: Transaction Pinning Attack explained.</x:v>
+        <x:v>Post title: Transaction Pinning Attack explained. Normalized as the canonical candidate for audit.post-1903881770204070155.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -2678,28 +2678,28 @@
         <x:v>Normalize the post's atomic learning outcome against the existing graph and record any merge or exclusion.</x:v>
       </x:c>
       <x:c r="H57" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I57" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J57" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K57" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L57" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M57" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N57" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O57" s="32" t="str">
-        <x:v>Post title: BIP-68 (Sequence number) explained.</x:v>
+        <x:v>Post title: BIP-68 (Sequence number) explained. Normalized as the canonical candidate for audit.post-1903150655071719663.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -8248,16 +8248,1768 @@
         <x:v>Added after checking privacy.pseudonymity, transaction privacy, and review-culture neighbors. Keep the node focused on contributor safety and merit-based evaluation rather than anonymous transactions.</x:v>
       </x:c>
     </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="32" t="str">
+        <x:v>privacy.coinjoin</x:v>
+      </x:c>
+      <x:c r="B107" s="32" t="str">
+        <x:v>CoinJoin</x:v>
+      </x:c>
+      <x:c r="C107" s="32" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="D107" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-2018682587045052753</x:v>
+      </x:c>
+      <x:c r="E107" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/2018682587045052753</x:v>
+      </x:c>
+      <x:c r="F107" s="32" t="str">
+        <x:v>Coinjoin Explained</x:v>
+      </x:c>
+      <x:c r="G107" s="32" t="str">
+        <x:v>privacy.coinjoin</x:v>
+      </x:c>
+      <x:c r="H107" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I107" s="32" t="str">
+        <x:v>The post teaches the existing collaborative transaction construction concept, not a narrower new protocol mechanism.</x:v>
+      </x:c>
+      <x:c r="J107" s="32" t="str">
+        <x:v>privacy.coin-control, privacy.address-reuse</x:v>
+      </x:c>
+      <x:c r="K107" s="32" t="str">
+        <x:v>privacy.coin-control, privacy.address-reuse</x:v>
+      </x:c>
+      <x:c r="L107" s="32" t="str">
+        <x:v>Preserve the existing node's direct prerequisites.</x:v>
+      </x:c>
+      <x:c r="M107" s="32" t="str">
+        <x:v>coinjoin</x:v>
+      </x:c>
+      <x:c r="N107" s="32" t="str">
+        <x:v>privacy, collaborative-transactions</x:v>
+      </x:c>
+      <x:c r="O107" s="32" t="str">
+        <x:v>60m</x:v>
+      </x:c>
+      <x:c r="P107" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q107" s="32" t="str">
+        <x:v>Reuse existing node; do not clone a second CoinJoin explainer.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="32" t="str">
+        <x:v>audit.post-2017223553708654888</x:v>
+      </x:c>
+      <x:c r="B108" s="32" t="str">
+        <x:v>Full Node Architecture</x:v>
+      </x:c>
+      <x:c r="C108" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D108" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-2017223553708654888</x:v>
+      </x:c>
+      <x:c r="E108" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/2017223553708654888</x:v>
+      </x:c>
+      <x:c r="F108" s="32" t="str">
+        <x:v>Full Node Architecture Explained</x:v>
+      </x:c>
+      <x:c r="G108" s="32" t="str">
+        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
+      </x:c>
+      <x:c r="H108" s="32" t="str">
+        <x:v>merge</x:v>
+      </x:c>
+      <x:c r="I108" s="32" t="str">
+        <x:v>The post's architecture explanation is covered by the existing learner-facing full-node versus lightweight-wallet trust-model node.</x:v>
+      </x:c>
+      <x:c r="J108" s="32" t="str">
+        <x:v>fundamentals.validation-sovereignty, protocol.light-client-trust-model</x:v>
+      </x:c>
+      <x:c r="K108" s="32" t="str">
+        <x:v>fundamentals.validation-sovereignty, protocol.light-client-trust-model</x:v>
+      </x:c>
+      <x:c r="L108" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+      </x:c>
+      <x:c r="M108" s="32" t="str">
+        <x:v>full node architecture</x:v>
+      </x:c>
+      <x:c r="N108" s="32" t="str">
+        <x:v>nodes, verification, architecture</x:v>
+      </x:c>
+      <x:c r="O108" s="32" t="str">
+        <x:v>25m</x:v>
+      </x:c>
+      <x:c r="P108" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q108" s="32" t="str">
+        <x:v>Merge into ops.full-node-vs-lightweight-wallet; the function/architecture wording does not justify a duplicate node.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="32" t="str">
+        <x:v>audit.post-2016929384389890484</x:v>
+      </x:c>
+      <x:c r="B109" s="32" t="str">
+        <x:v>SHA-256 Message Schedule</x:v>
+      </x:c>
+      <x:c r="C109" s="32" t="str">
+        <x:v>Fundamentals</x:v>
+      </x:c>
+      <x:c r="D109" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-2016929384389890484</x:v>
+      </x:c>
+      <x:c r="E109" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/2016929384389890484</x:v>
+      </x:c>
+      <x:c r="F109" s="32" t="str">
+        <x:v>SHA-256 explained Part 2: Message Schedule</x:v>
+      </x:c>
+      <x:c r="G109" s="32" t="str">
+        <x:v>fundamentals.hash-functions</x:v>
+      </x:c>
+      <x:c r="H109" s="32" t="str">
+        <x:v>merge</x:v>
+      </x:c>
+      <x:c r="I109" s="32" t="str">
+        <x:v>The message schedule is a subtopic of the existing hash-functions foundation and does not create a separate Bitcoin learner gap at this graph level.</x:v>
+      </x:c>
+      <x:c r="J109" s="32" t="str">
+        <x:v>fundamentals.hash-functions</x:v>
+      </x:c>
+      <x:c r="K109" s="32" t="str">
+        <x:v>fundamentals.hash-functions</x:v>
+      </x:c>
+      <x:c r="L109" s="32" t="str">
+        <x:v>The existing node already covers the relevant primitive.</x:v>
+      </x:c>
+      <x:c r="M109" s="32" t="str">
+        <x:v>SHA-256 message schedule</x:v>
+      </x:c>
+      <x:c r="N109" s="32" t="str">
+        <x:v>hashing, sha256</x:v>
+      </x:c>
+      <x:c r="O109" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P109" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q109" s="32" t="str">
+        <x:v>Merge into fundamentals.hash-functions; do not create an implementation-detail node for the compression-function substep.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="32" t="str">
+        <x:v>audit.post-2012233826504933706</x:v>
+      </x:c>
+      <x:c r="B110" s="32" t="str">
+        <x:v>SHA-256</x:v>
+      </x:c>
+      <x:c r="C110" s="32" t="str">
+        <x:v>Fundamentals</x:v>
+      </x:c>
+      <x:c r="D110" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-2012233826504933706</x:v>
+      </x:c>
+      <x:c r="E110" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/2012233826504933706</x:v>
+      </x:c>
+      <x:c r="F110" s="32" t="str">
+        <x:v>SHA-256 explained</x:v>
+      </x:c>
+      <x:c r="G110" s="32" t="str">
+        <x:v>fundamentals.hash-functions</x:v>
+      </x:c>
+      <x:c r="H110" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I110" s="32" t="str">
+        <x:v>The post directly explains the existing hash-functions foundation.</x:v>
+      </x:c>
+      <x:c r="J110" s="32" t="str"/>
+      <x:c r="K110" s="32" t="str"/>
+      <x:c r="L110" s="32" t="str">
+        <x:v>No additional prerequisite is needed for an existing foundational node.</x:v>
+      </x:c>
+      <x:c r="M110" s="32" t="str">
+        <x:v>SHA-256, sha256</x:v>
+      </x:c>
+      <x:c r="N110" s="32" t="str">
+        <x:v>hashing, sha256</x:v>
+      </x:c>
+      <x:c r="O110" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P110" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q110" s="32" t="str">
+        <x:v>Reuse fundamentals.hash-functions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="32" t="str">
+        <x:v>protocol.mast</x:v>
+      </x:c>
+      <x:c r="B111" s="32" t="str">
+        <x:v>Merkelized Alternative Script Trees (MAST)</x:v>
+      </x:c>
+      <x:c r="C111" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D111" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+      </x:c>
+      <x:c r="E111" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1998431297333501989</x:v>
+      </x:c>
+      <x:c r="F111" s="32" t="str">
+        <x:v>MAST explained simply</x:v>
+      </x:c>
+      <x:c r="G111" s="32" t="str"/>
+      <x:c r="H111" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I111" s="32" t="str">
+        <x:v>MAST is one specific script-commitment idea: commit to multiple spending branches in a Merkle tree while revealing only the executed branch. It is broader than the TapTree implementation and distinct from generic Taproot script-path spending.</x:v>
+      </x:c>
+      <x:c r="J111" s="32" t="str">
+        <x:v>fundamentals.merkle-trees, protocol.script</x:v>
+      </x:c>
+      <x:c r="K111" s="32" t="str">
+        <x:v>fundamentals.merkle-trees, protocol.script</x:v>
+      </x:c>
+      <x:c r="L111" s="32" t="str">
+        <x:v>Learners need both the Merkle commitment structure and Bitcoin Script branch model before selective branch revelation makes sense.</x:v>
+      </x:c>
+      <x:c r="M111" s="32" t="str">
+        <x:v>MAST, merkelized alternative script tree, Merkelized Alternative Script Tree</x:v>
+      </x:c>
+      <x:c r="N111" s="32" t="str">
+        <x:v>scripts, merkle, privacy, contracts</x:v>
+      </x:c>
+      <x:c r="O111" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P111" s="32" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="Q111" s="32" t="str">
+        <x:v>Add as a bridge concept only if the existing TapTree chain does not already provide this generic learning outcome; keep TapTree as the Taproot-specific realization.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" s="32" t="str">
+        <x:v>audit.post-1993443012748415027</x:v>
+      </x:c>
+      <x:c r="B112" s="32" t="str">
+        <x:v>Child Pays for Parent</x:v>
+      </x:c>
+      <x:c r="C112" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D112" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1993443012748415027</x:v>
+      </x:c>
+      <x:c r="E112" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1993443012748415027</x:v>
+      </x:c>
+      <x:c r="F112" s="32" t="str">
+        <x:v>Child-Pays-For-Parent transaction explained</x:v>
+      </x:c>
+      <x:c r="G112" s="32" t="str">
+        <x:v>protocol.cpfp</x:v>
+      </x:c>
+      <x:c r="H112" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I112" s="32" t="str">
+        <x:v>The post explains the existing CPFP fee-bumping strategy.</x:v>
+      </x:c>
+      <x:c r="J112" s="32" t="str">
+        <x:v>protocol.fee-market</x:v>
+      </x:c>
+      <x:c r="K112" s="32" t="str">
+        <x:v>protocol.fee-market</x:v>
+      </x:c>
+      <x:c r="L112" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M112" s="32" t="str">
+        <x:v>CPFP, child pays for parent</x:v>
+      </x:c>
+      <x:c r="N112" s="32" t="str">
+        <x:v>fees, mempool</x:v>
+      </x:c>
+      <x:c r="O112" s="32" t="str">
+        <x:v>55m</x:v>
+      </x:c>
+      <x:c r="P112" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q112" s="32" t="str">
+        <x:v>Reuse protocol.cpfp; this is a second explainer, not a new concept.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" s="32" t="str">
+        <x:v>protocol.sighash-quadratic-hashing</x:v>
+      </x:c>
+      <x:c r="B113" s="32" t="str">
+        <x:v>Quadratic SIGHASH Hashing Cost</x:v>
+      </x:c>
+      <x:c r="C113" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D113" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
+      </x:c>
+      <x:c r="E113" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1987562939109306699</x:v>
+      </x:c>
+      <x:c r="F113" s="32" t="str">
+        <x:v>Quadratic Sighash problem O(n^2) explained</x:v>
+      </x:c>
+      <x:c r="G113" s="32" t="str"/>
+      <x:c r="H113" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I113" s="32" t="str">
+        <x:v>One specific historical validation problem: legacy signature hashing repeats transaction-wide work for each input, creating quadratic verification cost and motivating cached digest designs.</x:v>
+      </x:c>
+      <x:c r="J113" s="32" t="str">
+        <x:v>protocol.sighash-flags</x:v>
+      </x:c>
+      <x:c r="K113" s="32" t="str">
+        <x:v>protocol.sighash-flags</x:v>
+      </x:c>
+      <x:c r="L113" s="32" t="str">
+        <x:v>SIGHASH semantics supply the signature-digest context; the performance failure is a distinct consequence rather than a duplicate of the flag definitions.</x:v>
+      </x:c>
+      <x:c r="M113" s="32" t="str">
+        <x:v>quadratic hashing problem, quadratic SIGHASH, O(n^2) SIGHASH</x:v>
+      </x:c>
+      <x:c r="N113" s="32" t="str">
+        <x:v>sighash, performance, consensus</x:v>
+      </x:c>
+      <x:c r="O113" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P113" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q113" s="32" t="str">
+        <x:v>Add as a narrow historical/protocol bridge; do not model the internal hashing loop as a generic implementation node.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" s="32" t="str">
+        <x:v>audit.post-1982189369684336693</x:v>
+      </x:c>
+      <x:c r="B114" s="32" t="str">
+        <x:v>BIP 158 Compact Block Filters</x:v>
+      </x:c>
+      <x:c r="C114" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D114" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1982189369684336693</x:v>
+      </x:c>
+      <x:c r="E114" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1982189369684336693</x:v>
+      </x:c>
+      <x:c r="F114" s="32" t="str">
+        <x:v>BIP 158: Compact Block Filters explained</x:v>
+      </x:c>
+      <x:c r="G114" s="32" t="str">
+        <x:v>protocol.compact-block-filters</x:v>
+      </x:c>
+      <x:c r="H114" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I114" s="32" t="str">
+        <x:v>The post teaches the existing BIP 158 compact-filter protocol.</x:v>
+      </x:c>
+      <x:c r="J114" s="32" t="str">
+        <x:v>dev.p2p-messages, protocol.block-structure</x:v>
+      </x:c>
+      <x:c r="K114" s="32" t="str">
+        <x:v>dev.p2p-messages, protocol.block-structure</x:v>
+      </x:c>
+      <x:c r="L114" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+      </x:c>
+      <x:c r="M114" s="32" t="str">
+        <x:v>BIP 158, compact block filters</x:v>
+      </x:c>
+      <x:c r="N114" s="32" t="str">
+        <x:v>light-clients, filters, p2p</x:v>
+      </x:c>
+      <x:c r="O114" s="32" t="str">
+        <x:v>70m</x:v>
+      </x:c>
+      <x:c r="P114" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q114" s="32" t="str">
+        <x:v>Reuse protocol.compact-block-filters.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" s="32" t="str">
+        <x:v>audit.post-1981761265036144901</x:v>
+      </x:c>
+      <x:c r="B115" s="32" t="str">
+        <x:v>Duplicate Transaction Merkle Root Collision</x:v>
+      </x:c>
+      <x:c r="C115" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D115" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1981761265036144901</x:v>
+      </x:c>
+      <x:c r="E115" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1981761265036144901</x:v>
+      </x:c>
+      <x:c r="F115" s="32" t="str">
+        <x:v>CVE-2012-2459 duplicate transaction Merkle root collision explained</x:v>
+      </x:c>
+      <x:c r="G115" s="32" t="str">
+        <x:v>protocol.duplicate-transaction-bug</x:v>
+      </x:c>
+      <x:c r="H115" s="32" t="str">
+        <x:v>merge</x:v>
+      </x:c>
+      <x:c r="I115" s="32" t="str">
+        <x:v>The collision is a concrete manifestation of the existing duplicate-transaction consensus bug family, not a separate learner outcome at the current graph granularity.</x:v>
+      </x:c>
+      <x:c r="J115" s="32" t="str">
+        <x:v>protocol.coinbase-transaction, protocol.utxo-model</x:v>
+      </x:c>
+      <x:c r="K115" s="32" t="str">
+        <x:v>protocol.coinbase-transaction, protocol.utxo-model</x:v>
+      </x:c>
+      <x:c r="L115" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+      </x:c>
+      <x:c r="M115" s="32" t="str">
+        <x:v>CVE-2012-2459, Merkle root collision</x:v>
+      </x:c>
+      <x:c r="N115" s="32" t="str">
+        <x:v>consensus, merkle, security</x:v>
+      </x:c>
+      <x:c r="O115" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P115" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q115" s="32" t="str">
+        <x:v>Merge into protocol.duplicate-transaction-bug and preserve the CVE as an alias/resource context.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" s="32" t="str">
+        <x:v>extension.discreet-log-contracts</x:v>
+      </x:c>
+      <x:c r="B116" s="32" t="str">
+        <x:v>Discreet Log Contracts</x:v>
+      </x:c>
+      <x:c r="C116" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D116" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1980708369620168949</x:v>
+      </x:c>
+      <x:c r="E116" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1980708369620168949</x:v>
+      </x:c>
+      <x:c r="F116" s="32" t="str">
+        <x:v>Discreet Log Contracts explained simply</x:v>
+      </x:c>
+      <x:c r="G116" s="32" t="str">
+        <x:v>extension.discreet-log-contracts</x:v>
+      </x:c>
+      <x:c r="H116" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I116" s="32" t="str">
+        <x:v>The post explains the existing DLC contract construction.</x:v>
+      </x:c>
+      <x:c r="J116" s="32" t="str">
+        <x:v>protocol.adaptor-signatures</x:v>
+      </x:c>
+      <x:c r="K116" s="32" t="str">
+        <x:v>protocol.adaptor-signatures</x:v>
+      </x:c>
+      <x:c r="L116" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M116" s="32" t="str">
+        <x:v>DLC, DLCs</x:v>
+      </x:c>
+      <x:c r="N116" s="32" t="str">
+        <x:v>contracts, oracles, adaptor-signatures</x:v>
+      </x:c>
+      <x:c r="O116" s="32" t="str">
+        <x:v>85m</x:v>
+      </x:c>
+      <x:c r="P116" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q116" s="32" t="str">
+        <x:v>Reuse extension.discreet-log-contracts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" s="32" t="str">
+        <x:v>dev.y2038-problem</x:v>
+      </x:c>
+      <x:c r="B117" s="32" t="str">
+        <x:v>Y2038 Problem</x:v>
+      </x:c>
+      <x:c r="C117" s="32" t="str">
+        <x:v>Development</x:v>
+      </x:c>
+      <x:c r="D117" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1977486634536104288</x:v>
+      </x:c>
+      <x:c r="E117" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1977486634536104288</x:v>
+      </x:c>
+      <x:c r="F117" s="32" t="str">
+        <x:v>The Y2038 problem explained</x:v>
+      </x:c>
+      <x:c r="G117" s="32" t="str"/>
+      <x:c r="H117" s="32" t="str">
+        <x:v>skip</x:v>
+      </x:c>
+      <x:c r="I117" s="32" t="str">
+        <x:v>The post names a general timestamp implementation hazard rather than a Bitcoin-specific learner concept or prerequisite branch.</x:v>
+      </x:c>
+      <x:c r="J117" s="32" t="str"/>
+      <x:c r="K117" s="32" t="str"/>
+      <x:c r="L117" s="32" t="str">
+        <x:v>No Bitcoin graph edge is justified without a Bitcoin-specific learning outcome.</x:v>
+      </x:c>
+      <x:c r="M117" s="32" t="str">
+        <x:v>Year 2038 problem, Unix time overflow</x:v>
+      </x:c>
+      <x:c r="N117" s="32" t="str">
+        <x:v>time, software</x:v>
+      </x:c>
+      <x:c r="O117" s="32" t="str">
+        <x:v>15m</x:v>
+      </x:c>
+      <x:c r="P117" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q117" s="32" t="str">
+        <x:v>Skip as off-scope implementation history; retain the source row for coverage evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" s="32" t="str">
+        <x:v>audit.post-1977053708065423446</x:v>
+      </x:c>
+      <x:c r="B118" s="32" t="str">
+        <x:v>Nonce Reuse Attack</x:v>
+      </x:c>
+      <x:c r="C118" s="32" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="D118" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1977053708065423446</x:v>
+      </x:c>
+      <x:c r="E118" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1977053708065423446</x:v>
+      </x:c>
+      <x:c r="F118" s="32" t="str">
+        <x:v>Nonce reuse attack explained simply</x:v>
+      </x:c>
+      <x:c r="G118" s="32" t="str">
+        <x:v>security.nonce-reuse-attack</x:v>
+      </x:c>
+      <x:c r="H118" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I118" s="32" t="str">
+        <x:v>The post repeats the existing nonce-reuse attack concept.</x:v>
+      </x:c>
+      <x:c r="J118" s="32" t="str">
+        <x:v>fundamentals.schnorr-signatures</x:v>
+      </x:c>
+      <x:c r="K118" s="32" t="str">
+        <x:v>fundamentals.schnorr-signatures</x:v>
+      </x:c>
+      <x:c r="L118" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M118" s="32" t="str">
+        <x:v>nonce reuse</x:v>
+      </x:c>
+      <x:c r="N118" s="32" t="str">
+        <x:v>signatures, security</x:v>
+      </x:c>
+      <x:c r="O118" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P118" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q118" s="32" t="str">
+        <x:v>Reuse security.nonce-reuse-attack.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" s="32" t="str">
+        <x:v>audit.post-1976762610948198707</x:v>
+      </x:c>
+      <x:c r="B119" s="32" t="str">
+        <x:v>MuSig2</x:v>
+      </x:c>
+      <x:c r="C119" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D119" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1976762610948198707</x:v>
+      </x:c>
+      <x:c r="E119" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1976762610948198707</x:v>
+      </x:c>
+      <x:c r="F119" s="32" t="str">
+        <x:v>MuSig2 explained simply</x:v>
+      </x:c>
+      <x:c r="G119" s="32" t="str">
+        <x:v>protocol.musig</x:v>
+      </x:c>
+      <x:c r="H119" s="32" t="str">
+        <x:v>merge</x:v>
+      </x:c>
+      <x:c r="I119" s="32" t="str">
+        <x:v>MuSig2 is a protocol version in the existing MuSig family; the current node already covers the key aggregation and interactive signing learning outcome.</x:v>
+      </x:c>
+      <x:c r="J119" s="32" t="str">
+        <x:v>fundamentals.schnorr-signatures</x:v>
+      </x:c>
+      <x:c r="K119" s="32" t="str">
+        <x:v>fundamentals.schnorr-signatures</x:v>
+      </x:c>
+      <x:c r="L119" s="32" t="str">
+        <x:v>Reuse the existing MuSig node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M119" s="32" t="str">
+        <x:v>MuSig2, two-round MuSig</x:v>
+      </x:c>
+      <x:c r="N119" s="32" t="str">
+        <x:v>schnorr, multisig, aggregation</x:v>
+      </x:c>
+      <x:c r="O119" s="32" t="str">
+        <x:v>50m</x:v>
+      </x:c>
+      <x:c r="P119" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q119" s="32" t="str">
+        <x:v>Merge into protocol.musig and preserve MuSig2 as an alias/resource variant.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" s="32" t="str">
+        <x:v>audit.post-1976416447577665743</x:v>
+      </x:c>
+      <x:c r="B120" s="32" t="str">
+        <x:v>MuSig</x:v>
+      </x:c>
+      <x:c r="C120" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D120" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1976416447577665743</x:v>
+      </x:c>
+      <x:c r="E120" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1976416447577665743</x:v>
+      </x:c>
+      <x:c r="F120" s="32" t="str">
+        <x:v>MuSig explained simply</x:v>
+      </x:c>
+      <x:c r="G120" s="32" t="str">
+        <x:v>protocol.musig</x:v>
+      </x:c>
+      <x:c r="H120" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I120" s="32" t="str">
+        <x:v>The post directly explains the existing MuSig node.</x:v>
+      </x:c>
+      <x:c r="J120" s="32" t="str">
+        <x:v>fundamentals.schnorr-signatures</x:v>
+      </x:c>
+      <x:c r="K120" s="32" t="str">
+        <x:v>fundamentals.schnorr-signatures</x:v>
+      </x:c>
+      <x:c r="L120" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M120" s="32" t="str">
+        <x:v>MuSig</x:v>
+      </x:c>
+      <x:c r="N120" s="32" t="str">
+        <x:v>schnorr, multisig, aggregation</x:v>
+      </x:c>
+      <x:c r="O120" s="32" t="str">
+        <x:v>50m</x:v>
+      </x:c>
+      <x:c r="P120" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q120" s="32" t="str">
+        <x:v>Reuse protocol.musig.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" s="32" t="str">
+        <x:v>security.rogue-key-attack</x:v>
+      </x:c>
+      <x:c r="B121" s="32" t="str">
+        <x:v>Rogue-Key Attack</x:v>
+      </x:c>
+      <x:c r="C121" s="32" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="D121" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
+      </x:c>
+      <x:c r="E121" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1976008010108678258</x:v>
+      </x:c>
+      <x:c r="F121" s="32" t="str">
+        <x:v>Schnorr signatures: rogue key attack explained</x:v>
+      </x:c>
+      <x:c r="G121" s="32" t="str"/>
+      <x:c r="H121" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I121" s="32" t="str">
+        <x:v>One multisignature security failure: an attacker can choose a related public key so an aggregate key appears authorized without the victim's intended cooperation.</x:v>
+      </x:c>
+      <x:c r="J121" s="32" t="str">
+        <x:v>protocol.musig</x:v>
+      </x:c>
+      <x:c r="K121" s="32" t="str">
+        <x:v>protocol.musig</x:v>
+      </x:c>
+      <x:c r="L121" s="32" t="str">
+        <x:v>MuSig supplies the key-aggregation setting; Schnorr signatures are inherited through MuSig and do not need a redundant direct edge.</x:v>
+      </x:c>
+      <x:c r="M121" s="32" t="str">
+        <x:v>rogue key attack, key aggregation rogue-key attack</x:v>
+      </x:c>
+      <x:c r="N121" s="32" t="str">
+        <x:v>schnorr, multisig, security</x:v>
+      </x:c>
+      <x:c r="O121" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P121" s="32" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="Q121" s="32" t="str">
+        <x:v>Add as a security failure mode distinct from the MuSig construction itself.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" s="32" t="str">
+        <x:v>mining.selfish-mining</x:v>
+      </x:c>
+      <x:c r="B122" s="32" t="str">
+        <x:v>Selfish Mining</x:v>
+      </x:c>
+      <x:c r="C122" s="32" t="str">
+        <x:v>Mining</x:v>
+      </x:c>
+      <x:c r="D122" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+      </x:c>
+      <x:c r="E122" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1975289920634925475</x:v>
+      </x:c>
+      <x:c r="F122" s="32" t="str">
+        <x:v>Selfish Mining explained simply</x:v>
+      </x:c>
+      <x:c r="G122" s="32" t="str"/>
+      <x:c r="H122" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I122" s="32" t="str">
+        <x:v>Selfish mining is one distinct incentive attack in which miners withhold blocks to gain a propagation and chain-selection advantage.</x:v>
+      </x:c>
+      <x:c r="J122" s="32" t="str">
+        <x:v>mining.pool-vs-solo, protocol.reorgs-finality</x:v>
+      </x:c>
+      <x:c r="K122" s="32" t="str">
+        <x:v>mining.pool-vs-solo, protocol.reorgs-finality</x:v>
+      </x:c>
+      <x:c r="L122" s="32" t="str">
+        <x:v>Learners need pooled-mining incentives and the chain-selection/finality model before the withholding strategy is intelligible.</x:v>
+      </x:c>
+      <x:c r="M122" s="32" t="str">
+        <x:v>selfish mining attack, block withholding for chain advantage</x:v>
+      </x:c>
+      <x:c r="N122" s="32" t="str">
+        <x:v>mining, incentives, attacks</x:v>
+      </x:c>
+      <x:c r="O122" s="32" t="str">
+        <x:v>40m</x:v>
+      </x:c>
+      <x:c r="P122" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q122" s="32" t="str">
+        <x:v>Add as a distinct miner strategy; do not merge it with block withholding, which targets pool compensation rather than chain advantage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" s="32" t="str">
+        <x:v>protocol.sighash-flags</x:v>
+      </x:c>
+      <x:c r="B123" s="32" t="str">
+        <x:v>SIGHASH</x:v>
+      </x:c>
+      <x:c r="C123" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D123" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1966579053076337056</x:v>
+      </x:c>
+      <x:c r="E123" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1966579053076337056</x:v>
+      </x:c>
+      <x:c r="F123" s="32" t="str">
+        <x:v>SigHash explained</x:v>
+      </x:c>
+      <x:c r="G123" s="32" t="str">
+        <x:v>protocol.sighash-flags</x:v>
+      </x:c>
+      <x:c r="H123" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I123" s="32" t="str">
+        <x:v>The post explains the existing signature-hash flag concept.</x:v>
+      </x:c>
+      <x:c r="J123" s="32" t="str">
+        <x:v>protocol.script</x:v>
+      </x:c>
+      <x:c r="K123" s="32" t="str">
+        <x:v>protocol.script</x:v>
+      </x:c>
+      <x:c r="L123" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M123" s="32" t="str">
+        <x:v>SIGHASH, signature hash</x:v>
+      </x:c>
+      <x:c r="N123" s="32" t="str">
+        <x:v>signatures, transactions</x:v>
+      </x:c>
+      <x:c r="O123" s="32" t="str">
+        <x:v>90m</x:v>
+      </x:c>
+      <x:c r="P123" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q123" s="32" t="str">
+        <x:v>Reuse protocol.sighash-flags; the quadratic-cost post is tracked separately as a candidate bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" s="32" t="str">
+        <x:v>audit.post-1962245647261745216</x:v>
+      </x:c>
+      <x:c r="B124" s="32" t="str">
+        <x:v>Transaction Pinning</x:v>
+      </x:c>
+      <x:c r="C124" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D124" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1962245647261745216</x:v>
+      </x:c>
+      <x:c r="E124" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1962245647261745216</x:v>
+      </x:c>
+      <x:c r="F124" s="32" t="str">
+        <x:v>Transaction Pinning explained</x:v>
+      </x:c>
+      <x:c r="G124" s="32" t="str">
+        <x:v>protocol.transaction-pinning</x:v>
+      </x:c>
+      <x:c r="H124" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I124" s="32" t="str">
+        <x:v>The post repeats the existing transaction-pinning risk concept.</x:v>
+      </x:c>
+      <x:c r="J124" s="32" t="str">
+        <x:v>protocol.package-relay</x:v>
+      </x:c>
+      <x:c r="K124" s="32" t="str">
+        <x:v>protocol.package-relay</x:v>
+      </x:c>
+      <x:c r="L124" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M124" s="32" t="str">
+        <x:v>transaction pinning</x:v>
+      </x:c>
+      <x:c r="N124" s="32" t="str">
+        <x:v>mempool, contracts, attacks</x:v>
+      </x:c>
+      <x:c r="O124" s="32" t="str">
+        <x:v>70m</x:v>
+      </x:c>
+      <x:c r="P124" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q124" s="32" t="str">
+        <x:v>Reuse protocol.transaction-pinning.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" s="32" t="str">
+        <x:v>protocol.segregated-witness</x:v>
+      </x:c>
+      <x:c r="B125" s="32" t="str">
+        <x:v>Segregated Witness</x:v>
+      </x:c>
+      <x:c r="C125" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D125" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1961882664803209229</x:v>
+      </x:c>
+      <x:c r="E125" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1961882664803209229</x:v>
+      </x:c>
+      <x:c r="F125" s="32" t="str">
+        <x:v>SegWit explained simply</x:v>
+      </x:c>
+      <x:c r="G125" s="32" t="str">
+        <x:v>protocol.segregated-witness</x:v>
+      </x:c>
+      <x:c r="H125" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I125" s="32" t="str">
+        <x:v>The post explains the existing SegWit protocol upgrade.</x:v>
+      </x:c>
+      <x:c r="J125" s="32" t="str"/>
+      <x:c r="K125" s="32" t="str"/>
+      <x:c r="L125" s="32" t="str">
+        <x:v>Reuse the existing node's graph position.</x:v>
+      </x:c>
+      <x:c r="M125" s="32" t="str">
+        <x:v>SegWit, segwit</x:v>
+      </x:c>
+      <x:c r="N125" s="32" t="str">
+        <x:v>segwit, transactions, consensus</x:v>
+      </x:c>
+      <x:c r="O125" s="32" t="str">
+        <x:v>60m</x:v>
+      </x:c>
+      <x:c r="P125" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q125" s="32" t="str">
+        <x:v>Reuse protocol.segregated-witness.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" s="32" t="str">
+        <x:v>audit.post-1956781577544896905</x:v>
+      </x:c>
+      <x:c r="B126" s="32" t="str">
+        <x:v>WOTS+ Key Generation</x:v>
+      </x:c>
+      <x:c r="C126" s="32" t="str">
+        <x:v>Fundamentals</x:v>
+      </x:c>
+      <x:c r="D126" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1956781577544896905</x:v>
+      </x:c>
+      <x:c r="E126" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1956781577544896905</x:v>
+      </x:c>
+      <x:c r="F126" s="32" t="str">
+        <x:v>WOTS+ key generation explained</x:v>
+      </x:c>
+      <x:c r="G126" s="32" t="str"/>
+      <x:c r="H126" s="32" t="str">
+        <x:v>skip</x:v>
+      </x:c>
+      <x:c r="I126" s="32" t="str">
+        <x:v>The post teaches a post-quantum signature subroutine outside Bitcoin's current signature and script model; it does not yet establish a Bitcoin-specific prerequisite gap.</x:v>
+      </x:c>
+      <x:c r="J126" s="32" t="str"/>
+      <x:c r="K126" s="32" t="str"/>
+      <x:c r="L126" s="32" t="str">
+        <x:v>No direct Bitcoin graph edge is justified for this off-scope cryptographic series.</x:v>
+      </x:c>
+      <x:c r="M126" s="32" t="str">
+        <x:v>WOTS+, Winternitz one-time signature plus</x:v>
+      </x:c>
+      <x:c r="N126" s="32" t="str">
+        <x:v>post-quantum, signatures</x:v>
+      </x:c>
+      <x:c r="O126" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P126" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q126" s="32" t="str">
+        <x:v>Skip as non-Bitcoin-adjacent for this pass; preserve source coverage without adding a generic cryptography branch.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" s="32" t="str">
+        <x:v>audit.post-1952320432033435819</x:v>
+      </x:c>
+      <x:c r="B127" s="32" t="str">
+        <x:v>Winternitz One-Time Signatures</x:v>
+      </x:c>
+      <x:c r="C127" s="32" t="str">
+        <x:v>Fundamentals</x:v>
+      </x:c>
+      <x:c r="D127" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1952320432033435819</x:v>
+      </x:c>
+      <x:c r="E127" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1952320432033435819</x:v>
+      </x:c>
+      <x:c r="F127" s="32" t="str">
+        <x:v>WOTS explained</x:v>
+      </x:c>
+      <x:c r="G127" s="32" t="str"/>
+      <x:c r="H127" s="32" t="str">
+        <x:v>skip</x:v>
+      </x:c>
+      <x:c r="I127" s="32" t="str">
+        <x:v>The post is part of the SPHINCS+ post-quantum signature series, not a Bitcoin-specific concept currently needed by the graph.</x:v>
+      </x:c>
+      <x:c r="J127" s="32" t="str"/>
+      <x:c r="K127" s="32" t="str"/>
+      <x:c r="L127" s="32" t="str">
+        <x:v>No direct Bitcoin graph edge is justified for this off-scope cryptographic series.</x:v>
+      </x:c>
+      <x:c r="M127" s="32" t="str">
+        <x:v>WOTS, Winternitz signatures</x:v>
+      </x:c>
+      <x:c r="N127" s="32" t="str">
+        <x:v>post-quantum, signatures</x:v>
+      </x:c>
+      <x:c r="O127" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P127" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q127" s="32" t="str">
+        <x:v>Skip and keep grouped with the SPHINCS+ series rather than minting isolated cryptographic nodes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" s="32" t="str">
+        <x:v>audit.post-1951962210902671675</x:v>
+      </x:c>
+      <x:c r="B128" s="32" t="str">
+        <x:v>SPHINCS+</x:v>
+      </x:c>
+      <x:c r="C128" s="32" t="str">
+        <x:v>Fundamentals</x:v>
+      </x:c>
+      <x:c r="D128" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1951962210902671675</x:v>
+      </x:c>
+      <x:c r="E128" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1951962210902671675</x:v>
+      </x:c>
+      <x:c r="F128" s="32" t="str">
+        <x:v>SPHINCS+ and Lamport signatures explained</x:v>
+      </x:c>
+      <x:c r="G128" s="32" t="str"/>
+      <x:c r="H128" s="32" t="str">
+        <x:v>skip</x:v>
+      </x:c>
+      <x:c r="I128" s="32" t="str">
+        <x:v>SPHINCS+ is a post-quantum signature scheme, but this post does not connect it to a Bitcoin protocol or learner prerequisite branch.</x:v>
+      </x:c>
+      <x:c r="J128" s="32" t="str"/>
+      <x:c r="K128" s="32" t="str"/>
+      <x:c r="L128" s="32" t="str">
+        <x:v>No direct Bitcoin graph edge is justified for this off-scope cryptographic series.</x:v>
+      </x:c>
+      <x:c r="M128" s="32" t="str">
+        <x:v>SPHINCS plus</x:v>
+      </x:c>
+      <x:c r="N128" s="32" t="str">
+        <x:v>post-quantum, signatures</x:v>
+      </x:c>
+      <x:c r="O128" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P128" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q128" s="32" t="str">
+        <x:v>Skip for the Bitcoin graph's current scope; revisit only as part of a deliberate post-quantum roadmap.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" s="32" t="str">
+        <x:v>audit.post-1951704233742651737</x:v>
+      </x:c>
+      <x:c r="B129" s="32" t="str">
+        <x:v>SPHINCS+ Signature Scheme</x:v>
+      </x:c>
+      <x:c r="C129" s="32" t="str">
+        <x:v>Fundamentals</x:v>
+      </x:c>
+      <x:c r="D129" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1951704233742651737</x:v>
+      </x:c>
+      <x:c r="E129" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1951704233742651737</x:v>
+      </x:c>
+      <x:c r="F129" s="32" t="str">
+        <x:v>SPHINCS+ explained</x:v>
+      </x:c>
+      <x:c r="G129" s="32" t="str"/>
+      <x:c r="H129" s="32" t="str">
+        <x:v>skip</x:v>
+      </x:c>
+      <x:c r="I129" s="32" t="str">
+        <x:v>This is a duplicate introductory post in the same non-Bitcoin-specific SPHINCS+ series.</x:v>
+      </x:c>
+      <x:c r="J129" s="32" t="str"/>
+      <x:c r="K129" s="32" t="str"/>
+      <x:c r="L129" s="32" t="str">
+        <x:v>No direct Bitcoin graph edge is justified for this off-scope cryptographic series.</x:v>
+      </x:c>
+      <x:c r="M129" s="32" t="str">
+        <x:v>SPHINCS+</x:v>
+      </x:c>
+      <x:c r="N129" s="32" t="str">
+        <x:v>post-quantum, signatures</x:v>
+      </x:c>
+      <x:c r="O129" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P129" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q129" s="32" t="str">
+        <x:v>Skip as a duplicate/off-scope series member.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" s="32" t="str">
+        <x:v>extension.bitchat</x:v>
+      </x:c>
+      <x:c r="B130" s="32" t="str">
+        <x:v>Bitchat</x:v>
+      </x:c>
+      <x:c r="C130" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D130" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1946961429363327053</x:v>
+      </x:c>
+      <x:c r="E130" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1946961429363327053</x:v>
+      </x:c>
+      <x:c r="F130" s="32" t="str">
+        <x:v>Bitchat explained simply</x:v>
+      </x:c>
+      <x:c r="G130" s="32" t="str">
+        <x:v>extension.bitchat</x:v>
+      </x:c>
+      <x:c r="H130" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I130" s="32" t="str">
+        <x:v>The post explains the existing Bitchat extension concept.</x:v>
+      </x:c>
+      <x:c r="J130" s="32" t="str">
+        <x:v>ops.mesh-networks, extension.nostr</x:v>
+      </x:c>
+      <x:c r="K130" s="32" t="str">
+        <x:v>ops.mesh-networks, extension.nostr</x:v>
+      </x:c>
+      <x:c r="L130" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+      </x:c>
+      <x:c r="M130" s="32" t="str">
+        <x:v>Bitchat</x:v>
+      </x:c>
+      <x:c r="N130" s="32" t="str">
+        <x:v>messaging, mesh</x:v>
+      </x:c>
+      <x:c r="O130" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P130" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q130" s="32" t="str">
+        <x:v>Reuse extension.bitchat.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="32" t="str">
+        <x:v>audit.post-1945962367738601788</x:v>
+      </x:c>
+      <x:c r="B131" s="32" t="str">
+        <x:v>Compact Block Filter</x:v>
+      </x:c>
+      <x:c r="C131" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D131" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1945962367738601788</x:v>
+      </x:c>
+      <x:c r="E131" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1945962367738601788</x:v>
+      </x:c>
+      <x:c r="F131" s="32" t="str">
+        <x:v>Compact Block Filter explained Part 1</x:v>
+      </x:c>
+      <x:c r="G131" s="32" t="str">
+        <x:v>protocol.compact-block-filters</x:v>
+      </x:c>
+      <x:c r="H131" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I131" s="32" t="str">
+        <x:v>This earlier post is another explanation of the existing compact-filter node.</x:v>
+      </x:c>
+      <x:c r="J131" s="32" t="str">
+        <x:v>dev.p2p-messages, protocol.block-structure</x:v>
+      </x:c>
+      <x:c r="K131" s="32" t="str">
+        <x:v>dev.p2p-messages, protocol.block-structure</x:v>
+      </x:c>
+      <x:c r="L131" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+      </x:c>
+      <x:c r="M131" s="32" t="str">
+        <x:v>compact block filter</x:v>
+      </x:c>
+      <x:c r="N131" s="32" t="str">
+        <x:v>light-clients, filters</x:v>
+      </x:c>
+      <x:c r="O131" s="32" t="str">
+        <x:v>70m</x:v>
+      </x:c>
+      <x:c r="P131" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q131" s="32" t="str">
+        <x:v>Reuse protocol.compact-block-filters.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="32" t="str">
+        <x:v>audit.post-1945645540152135684</x:v>
+      </x:c>
+      <x:c r="B132" s="32" t="str">
+        <x:v>Child Pays for Parent</x:v>
+      </x:c>
+      <x:c r="C132" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D132" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1945645540152135684</x:v>
+      </x:c>
+      <x:c r="E132" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1945645540152135684</x:v>
+      </x:c>
+      <x:c r="F132" s="32" t="str">
+        <x:v>Earlier CPFP transaction explanation</x:v>
+      </x:c>
+      <x:c r="G132" s="32" t="str">
+        <x:v>protocol.cpfp</x:v>
+      </x:c>
+      <x:c r="H132" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I132" s="32" t="str">
+        <x:v>This is an earlier explainer for the same CPFP concept.</x:v>
+      </x:c>
+      <x:c r="J132" s="32" t="str">
+        <x:v>protocol.fee-market</x:v>
+      </x:c>
+      <x:c r="K132" s="32" t="str">
+        <x:v>protocol.fee-market</x:v>
+      </x:c>
+      <x:c r="L132" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M132" s="32" t="str">
+        <x:v>CPFP</x:v>
+      </x:c>
+      <x:c r="N132" s="32" t="str">
+        <x:v>fees, mempool</x:v>
+      </x:c>
+      <x:c r="O132" s="32" t="str">
+        <x:v>55m</x:v>
+      </x:c>
+      <x:c r="P132" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q132" s="32" t="str">
+        <x:v>Reuse protocol.cpfp.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" s="32" t="str">
+        <x:v>audit.post-1934578478575489365</x:v>
+      </x:c>
+      <x:c r="B133" s="32" t="str">
+        <x:v>Lamport Signatures</x:v>
+      </x:c>
+      <x:c r="C133" s="32" t="str">
+        <x:v>Fundamentals</x:v>
+      </x:c>
+      <x:c r="D133" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1934578478575489365</x:v>
+      </x:c>
+      <x:c r="E133" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1934578478575489365</x:v>
+      </x:c>
+      <x:c r="F133" s="32" t="str">
+        <x:v>Lamport Signatures explained</x:v>
+      </x:c>
+      <x:c r="G133" s="32" t="str">
+        <x:v>fundamentals.lamport-signatures</x:v>
+      </x:c>
+      <x:c r="H133" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I133" s="32" t="str">
+        <x:v>The post repeats the existing Lamport signature concept.</x:v>
+      </x:c>
+      <x:c r="J133" s="32" t="str">
+        <x:v>fundamentals.hash-functions</x:v>
+      </x:c>
+      <x:c r="K133" s="32" t="str">
+        <x:v>fundamentals.hash-functions</x:v>
+      </x:c>
+      <x:c r="L133" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M133" s="32" t="str">
+        <x:v>Lamport signatures</x:v>
+      </x:c>
+      <x:c r="N133" s="32" t="str">
+        <x:v>post-quantum, signatures</x:v>
+      </x:c>
+      <x:c r="O133" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P133" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q133" s="32" t="str">
+        <x:v>Reuse fundamentals.lamport-signatures.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" s="32" t="str">
+        <x:v>protocol.commit-delay-reveal</x:v>
+      </x:c>
+      <x:c r="B134" s="32" t="str">
+        <x:v>Commit-Delay-Reveal Protocol</x:v>
+      </x:c>
+      <x:c r="C134" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D134" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
+      </x:c>
+      <x:c r="E134" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1931775486449103086</x:v>
+      </x:c>
+      <x:c r="F134" s="32" t="str">
+        <x:v>Commit-Delay-Reveal protocol explained</x:v>
+      </x:c>
+      <x:c r="G134" s="32" t="str"/>
+      <x:c r="H134" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I134" s="32" t="str">
+        <x:v>One protocol pattern: commit to a value, wait through a delay, and reveal it later so participants cannot adapt after seeing others' commitments.</x:v>
+      </x:c>
+      <x:c r="J134" s="32" t="str">
+        <x:v>fundamentals.commitment-schemes</x:v>
+      </x:c>
+      <x:c r="K134" s="32" t="str">
+        <x:v>fundamentals.commitment-schemes</x:v>
+      </x:c>
+      <x:c r="L134" s="32" t="str">
+        <x:v>Commitment schemes provide the hiding/binding foundation; the delay and reveal sequence is the distinct protocol composition.</x:v>
+      </x:c>
+      <x:c r="M134" s="32" t="str">
+        <x:v>CDR protocol, commit delay reveal</x:v>
+      </x:c>
+      <x:c r="N134" s="32" t="str">
+        <x:v>commitments, protocols, coordination</x:v>
+      </x:c>
+      <x:c r="O134" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P134" s="32" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="Q134" s="32" t="str">
+        <x:v>Add only if the post's Bitcoin/BitVM context is retained in the node resources; do not turn generic commit-reveal into an unbounded protocol family.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" s="32" t="str">
+        <x:v>protocol.cross-input-signature-aggregation</x:v>
+      </x:c>
+      <x:c r="B135" s="32" t="str">
+        <x:v>Cross-Input Signature Aggregation</x:v>
+      </x:c>
+      <x:c r="C135" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D135" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1905214178379362814</x:v>
+      </x:c>
+      <x:c r="E135" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1905214178379362814</x:v>
+      </x:c>
+      <x:c r="F135" s="32" t="str">
+        <x:v>CISA full aggregation explained</x:v>
+      </x:c>
+      <x:c r="G135" s="32" t="str">
+        <x:v>protocol.cross-input-signature-aggregation</x:v>
+      </x:c>
+      <x:c r="H135" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I135" s="32" t="str">
+        <x:v>The post explains the existing CISA concept.</x:v>
+      </x:c>
+      <x:c r="J135" s="32" t="str">
+        <x:v>protocol.adaptor-signatures</x:v>
+      </x:c>
+      <x:c r="K135" s="32" t="str">
+        <x:v>protocol.adaptor-signatures</x:v>
+      </x:c>
+      <x:c r="L135" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M135" s="32" t="str">
+        <x:v>CISA, full signature aggregation</x:v>
+      </x:c>
+      <x:c r="N135" s="32" t="str">
+        <x:v>signatures, aggregation</x:v>
+      </x:c>
+      <x:c r="O135" s="32" t="str">
+        <x:v>75m</x:v>
+      </x:c>
+      <x:c r="P135" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q135" s="32" t="str">
+        <x:v>Reuse protocol.cross-input-signature-aggregation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" s="32" t="str">
+        <x:v>security.dust-attack</x:v>
+      </x:c>
+      <x:c r="B136" s="32" t="str">
+        <x:v>Dust Attack</x:v>
+      </x:c>
+      <x:c r="C136" s="32" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="D136" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+      </x:c>
+      <x:c r="E136" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1904946739603452376</x:v>
+      </x:c>
+      <x:c r="F136" s="32" t="str">
+        <x:v>Dust attack explained</x:v>
+      </x:c>
+      <x:c r="G136" s="32" t="str"/>
+      <x:c r="H136" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I136" s="32" t="str">
+        <x:v>A dust attack is one specific privacy attack: send trace-value outputs to targets so later spending can link their wallets or contaminate their coin-control decisions.</x:v>
+      </x:c>
+      <x:c r="J136" s="32" t="str">
+        <x:v>protocol.dust-policy, privacy.pseudonymity</x:v>
+      </x:c>
+      <x:c r="K136" s="32" t="str">
+        <x:v>protocol.dust-policy, privacy.pseudonymity</x:v>
+      </x:c>
+      <x:c r="L136" s="32" t="str">
+        <x:v>Dust policy explains the output threshold and pseudonymity explains why forced linkage is harmful; neither edge is transitive through the other.</x:v>
+      </x:c>
+      <x:c r="M136" s="32" t="str">
+        <x:v>dusting attack, dust attack</x:v>
+      </x:c>
+      <x:c r="N136" s="32" t="str">
+        <x:v>privacy, utxos, attacks</x:v>
+      </x:c>
+      <x:c r="O136" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P136" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q136" s="32" t="str">
+        <x:v>Add as a privacy threat distinct from the operational dust-policy threshold.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" s="32" t="str">
+        <x:v>audit.post-1904596944649150556</x:v>
+      </x:c>
+      <x:c r="B137" s="32" t="str">
+        <x:v>CISA Half Signature Aggregation</x:v>
+      </x:c>
+      <x:c r="C137" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D137" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1904596944649150556</x:v>
+      </x:c>
+      <x:c r="E137" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1904596944649150556</x:v>
+      </x:c>
+      <x:c r="F137" s="32" t="str">
+        <x:v>CISA half signature aggregation explained</x:v>
+      </x:c>
+      <x:c r="G137" s="32" t="str">
+        <x:v>protocol.cross-input-signature-aggregation</x:v>
+      </x:c>
+      <x:c r="H137" s="32" t="str">
+        <x:v>merge</x:v>
+      </x:c>
+      <x:c r="I137" s="32" t="str">
+        <x:v>Half-aggregation is a design variant within the existing CISA concept, not a separate learner-facing protocol node.</x:v>
+      </x:c>
+      <x:c r="J137" s="32" t="str">
+        <x:v>protocol.adaptor-signatures</x:v>
+      </x:c>
+      <x:c r="K137" s="32" t="str">
+        <x:v>protocol.adaptor-signatures</x:v>
+      </x:c>
+      <x:c r="L137" s="32" t="str">
+        <x:v>Reuse the existing CISA node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M137" s="32" t="str">
+        <x:v>half signature aggregation, half-agg</x:v>
+      </x:c>
+      <x:c r="N137" s="32" t="str">
+        <x:v>signatures, aggregation</x:v>
+      </x:c>
+      <x:c r="O137" s="32" t="str">
+        <x:v>75m</x:v>
+      </x:c>
+      <x:c r="P137" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q137" s="32" t="str">
+        <x:v>Merge into protocol.cross-input-signature-aggregation and preserve the variant as an alias/context.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" s="32" t="str">
+        <x:v>audit.post-1904136400213340298</x:v>
+      </x:c>
+      <x:c r="B138" s="32" t="str">
+        <x:v>Cross-Input Signature Aggregation</x:v>
+      </x:c>
+      <x:c r="C138" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D138" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1904136400213340298</x:v>
+      </x:c>
+      <x:c r="E138" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1904136400213340298</x:v>
+      </x:c>
+      <x:c r="F138" s="32" t="str">
+        <x:v>CISA explained</x:v>
+      </x:c>
+      <x:c r="G138" s="32" t="str">
+        <x:v>protocol.cross-input-signature-aggregation</x:v>
+      </x:c>
+      <x:c r="H138" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I138" s="32" t="str">
+        <x:v>The post directly explains the existing CISA node.</x:v>
+      </x:c>
+      <x:c r="J138" s="32" t="str">
+        <x:v>protocol.adaptor-signatures</x:v>
+      </x:c>
+      <x:c r="K138" s="32" t="str">
+        <x:v>protocol.adaptor-signatures</x:v>
+      </x:c>
+      <x:c r="L138" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M138" s="32" t="str">
+        <x:v>CISA</x:v>
+      </x:c>
+      <x:c r="N138" s="32" t="str">
+        <x:v>signatures, aggregation</x:v>
+      </x:c>
+      <x:c r="O138" s="32" t="str">
+        <x:v>75m</x:v>
+      </x:c>
+      <x:c r="P138" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q138" s="32" t="str">
+        <x:v>Reuse protocol.cross-input-signature-aggregation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" s="32" t="str">
+        <x:v>audit.post-1903881770204070155</x:v>
+      </x:c>
+      <x:c r="B139" s="32" t="str">
+        <x:v>Transaction Pinning Attack</x:v>
+      </x:c>
+      <x:c r="C139" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D139" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1903881770204070155</x:v>
+      </x:c>
+      <x:c r="E139" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1903881770204070155</x:v>
+      </x:c>
+      <x:c r="F139" s="32" t="str">
+        <x:v>Transaction Pinning Attack explained</x:v>
+      </x:c>
+      <x:c r="G139" s="32" t="str">
+        <x:v>protocol.transaction-pinning</x:v>
+      </x:c>
+      <x:c r="H139" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I139" s="32" t="str">
+        <x:v>This post is a second framing of the existing transaction-pinning risk.</x:v>
+      </x:c>
+      <x:c r="J139" s="32" t="str">
+        <x:v>protocol.package-relay</x:v>
+      </x:c>
+      <x:c r="K139" s="32" t="str">
+        <x:v>protocol.package-relay</x:v>
+      </x:c>
+      <x:c r="L139" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M139" s="32" t="str">
+        <x:v>transaction pinning attack</x:v>
+      </x:c>
+      <x:c r="N139" s="32" t="str">
+        <x:v>mempool, attacks</x:v>
+      </x:c>
+      <x:c r="O139" s="32" t="str">
+        <x:v>70m</x:v>
+      </x:c>
+      <x:c r="P139" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q139" s="32" t="str">
+        <x:v>Reuse protocol.transaction-pinning.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" s="32" t="str">
+        <x:v>protocol.sequence-locks-bip68</x:v>
+      </x:c>
+      <x:c r="B140" s="32" t="str">
+        <x:v>BIP 68 Sequence Numbers</x:v>
+      </x:c>
+      <x:c r="C140" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D140" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1903150655071719663</x:v>
+      </x:c>
+      <x:c r="E140" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1903150655071719663</x:v>
+      </x:c>
+      <x:c r="F140" s="32" t="str">
+        <x:v>BIP-68 sequence number explained</x:v>
+      </x:c>
+      <x:c r="G140" s="32" t="str">
+        <x:v>protocol.sequence-locks-bip68</x:v>
+      </x:c>
+      <x:c r="H140" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I140" s="32" t="str">
+        <x:v>The post explains the existing BIP 68 sequence-lock concept.</x:v>
+      </x:c>
+      <x:c r="J140" s="32" t="str">
+        <x:v>protocol.timelocks</x:v>
+      </x:c>
+      <x:c r="K140" s="32" t="str">
+        <x:v>protocol.timelocks</x:v>
+      </x:c>
+      <x:c r="L140" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M140" s="32" t="str">
+        <x:v>BIP 68, sequence numbers, relative timelocks</x:v>
+      </x:c>
+      <x:c r="N140" s="32" t="str">
+        <x:v>timelocks, consensus</x:v>
+      </x:c>
+      <x:c r="O140" s="32" t="str">
+        <x:v>80m</x:v>
+      </x:c>
+      <x:c r="P140" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q140" s="32" t="str">
+        <x:v>Reuse protocol.sequence-locks-bip68.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H106">
+    <x:dataValidation type="list" sqref="H12:H140">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P106">
+    <x:dataValidation type="list" sqref="P12:P140">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10876,16 +12628,223 @@
         <x:v>Privacy pseudonymity is related context, not a direct prerequisite, because this node concerns contributor identity and governance rather than transaction linkage.</x:v>
       </x:c>
     </x:row>
+    <x:row r="123">
+      <x:c r="A123" s="32" t="str">
+        <x:v>fundamentals.merkle-trees</x:v>
+      </x:c>
+      <x:c r="B123" s="32" t="str">
+        <x:v>protocol.mast</x:v>
+      </x:c>
+      <x:c r="C123" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D123" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E123" s="32" t="str">
+        <x:v>MAST uses a Merkle tree to commit to multiple alternative script branches while revealing only one branch during spending.</x:v>
+      </x:c>
+      <x:c r="F123" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+      </x:c>
+      <x:c r="G123" s="32" t="str">
+        <x:v>Direct cryptographic structure; TapTree remains a downstream Taproot-specific realization.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" s="32" t="str">
+        <x:v>protocol.script</x:v>
+      </x:c>
+      <x:c r="B124" s="32" t="str">
+        <x:v>protocol.mast</x:v>
+      </x:c>
+      <x:c r="C124" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D124" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E124" s="32" t="str">
+        <x:v>MAST commits to alternative Bitcoin Script branches, so learners need the locking and spending language before the tree commitment is meaningful.</x:v>
+      </x:c>
+      <x:c r="F124" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+      </x:c>
+      <x:c r="G124" s="32" t="str">
+        <x:v>Keep Script direct; the node is not only a generic Merkle-tree concept.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" s="32" t="str">
+        <x:v>protocol.sighash-flags</x:v>
+      </x:c>
+      <x:c r="B125" s="32" t="str">
+        <x:v>protocol.sighash-quadratic-hashing</x:v>
+      </x:c>
+      <x:c r="C125" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D125" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E125" s="32" t="str">
+        <x:v>The quadratic hashing problem is a performance consequence of how legacy signature digests are constructed under SIGHASH semantics.</x:v>
+      </x:c>
+      <x:c r="F125" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
+      </x:c>
+      <x:c r="G125" s="32" t="str">
+        <x:v>BIP 143 is a supporting mitigation source, not a prerequisite edge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" s="32" t="str">
+        <x:v>protocol.musig</x:v>
+      </x:c>
+      <x:c r="B126" s="32" t="str">
+        <x:v>security.rogue-key-attack</x:v>
+      </x:c>
+      <x:c r="C126" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D126" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E126" s="32" t="str">
+        <x:v>The rogue-key attack occurs in naive public-key aggregation, so learners need the MuSig aggregation setting before the failure mode.</x:v>
+      </x:c>
+      <x:c r="F126" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
+      </x:c>
+      <x:c r="G126" s="32" t="str">
+        <x:v>Schnorr is inherited through MuSig; avoid a redundant direct Schnorr edge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" s="32" t="str">
+        <x:v>mining.pool-vs-solo</x:v>
+      </x:c>
+      <x:c r="B127" s="32" t="str">
+        <x:v>mining.selfish-mining</x:v>
+      </x:c>
+      <x:c r="C127" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D127" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E127" s="32" t="str">
+        <x:v>Selfish mining is an incentive strategy by miners and pools, so learners need the pooled-versus-solo mining context first.</x:v>
+      </x:c>
+      <x:c r="F127" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+      </x:c>
+      <x:c r="G127" s="32" t="str">
+        <x:v>Pool economics is one direct parent; chain selection is supplied by the finality parent below.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" s="32" t="str">
+        <x:v>protocol.reorgs-finality</x:v>
+      </x:c>
+      <x:c r="B128" s="32" t="str">
+        <x:v>mining.selfish-mining</x:v>
+      </x:c>
+      <x:c r="C128" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D128" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E128" s="32" t="str">
+        <x:v>Selfish mining relies on strategic withholding and release of competing branches, which requires the chain-reorganization and finality model.</x:v>
+      </x:c>
+      <x:c r="F128" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+      </x:c>
+      <x:c r="G128" s="32" t="str">
+        <x:v>Keep the reorganization model direct rather than adding generic proof-of-work as a redundant ancestor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" s="32" t="str">
+        <x:v>fundamentals.commitment-schemes</x:v>
+      </x:c>
+      <x:c r="B129" s="32" t="str">
+        <x:v>protocol.commit-delay-reveal</x:v>
+      </x:c>
+      <x:c r="C129" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D129" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E129" s="32" t="str">
+        <x:v>Commit-delay-reveal composes a cryptographic commitment with a timed reveal, so the learner first needs the hiding and binding commitment model.</x:v>
+      </x:c>
+      <x:c r="F129" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
+      </x:c>
+      <x:c r="G129" s="32" t="str">
+        <x:v>The delay/reveal composition is the node's distinct outcome.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" s="32" t="str">
+        <x:v>protocol.dust-policy</x:v>
+      </x:c>
+      <x:c r="B130" s="32" t="str">
+        <x:v>security.dust-attack</x:v>
+      </x:c>
+      <x:c r="C130" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D130" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E130" s="32" t="str">
+        <x:v>Dust attacks exploit the distinction between tiny-output relay policy and the ability to place trace-value UTXOs in a wallet.</x:v>
+      </x:c>
+      <x:c r="F130" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+      </x:c>
+      <x:c r="G130" s="32" t="str">
+        <x:v>Policy threshold is direct context for the attack mechanism.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="32" t="str">
+        <x:v>privacy.pseudonymity</x:v>
+      </x:c>
+      <x:c r="B131" s="32" t="str">
+        <x:v>security.dust-attack</x:v>
+      </x:c>
+      <x:c r="C131" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D131" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E131" s="32" t="str">
+        <x:v>The privacy harm of dusting comes from linking future spends and wallet activity, so learners need the pseudonymity and linkage model.</x:v>
+      </x:c>
+      <x:c r="F131" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+      </x:c>
+      <x:c r="G131" s="32" t="str">
+        <x:v>Keep privacy linkage direct; it is not inherited through dust policy.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C122">
+    <x:dataValidation type="list" sqref="C12:C131">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D122">
+    <x:dataValidation type="list" sqref="D12:D131">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -13373,16 +15332,196 @@
         <x:v>Added with dev.review-culture as the only direct prerequisite. Keep transaction pseudonymity and censorship resistance as related context rather than redundant graph parents.</x:v>
       </x:c>
     </x:row>
+    <x:row r="105">
+      <x:c r="A105" s="32" t="str">
+        <x:v>decision.bitcoin-dev-project-post-inventory-2026-07-11</x:v>
+      </x:c>
+      <x:c r="B105" s="32" t="str">
+        <x:v>inventory</x:v>
+      </x:c>
+      <x:c r="C105" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+      </x:c>
+      <x:c r="D105" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E105" s="32" t="str">
+        <x:v>The authenticated live search was enumerated into 34 individual post source rows. The earlier 43-post count was not preserved at post granularity and remains historical evidence rather than a completion claim.</x:v>
+      </x:c>
+      <x:c r="F105" s="32" t="str"/>
+      <x:c r="G105" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+      </x:c>
+      <x:c r="H105" s="32" t="str">
+        <x:v>Current enumeration includes duplicate explainers and post-quantum cryptography series members; each is retained as a source row and normalized separately rather than silently dropped.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="32" t="str">
+        <x:v>decision.mast-slice</x:v>
+      </x:c>
+      <x:c r="B106" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C106" s="32" t="str">
+        <x:v>protocol.mast</x:v>
+      </x:c>
+      <x:c r="D106" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E106" s="32" t="str">
+        <x:v>MAST survives dedupe as a generic script-branch commitment concept distinct from the TapTree's Taproot-specific realization. The post supplies a precise learner outcome around selective branch revelation.</x:v>
+      </x:c>
+      <x:c r="F106" s="32" t="str">
+        <x:v>protocol.mast, protocol.taptree, fundamentals.merkle-trees, protocol.script</x:v>
+      </x:c>
+      <x:c r="G106" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+      </x:c>
+      <x:c r="H106" s="32" t="str">
+        <x:v>Added with Merkle trees and Script as direct prerequisites; do not add TapTree as a redundant direct parent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="32" t="str">
+        <x:v>decision.sighash-quadratic-hashing-slice</x:v>
+      </x:c>
+      <x:c r="B107" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C107" s="32" t="str">
+        <x:v>protocol.sighash-quadratic-hashing</x:v>
+      </x:c>
+      <x:c r="D107" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E107" s="32" t="str">
+        <x:v>The quadratic signature-hashing cost is a distinct historical validation failure and bridge to BIP 143's cached digest design, not merely another SIGHASH flag label.</x:v>
+      </x:c>
+      <x:c r="F107" s="32" t="str">
+        <x:v>protocol.sighash-quadratic-hashing, protocol.sighash-flags</x:v>
+      </x:c>
+      <x:c r="G107" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
+      </x:c>
+      <x:c r="H107" s="32" t="str">
+        <x:v>Added with SIGHASH flags as the only direct prerequisite.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="32" t="str">
+        <x:v>decision.rogue-key-attack-slice</x:v>
+      </x:c>
+      <x:c r="B108" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C108" s="32" t="str">
+        <x:v>security.rogue-key-attack</x:v>
+      </x:c>
+      <x:c r="D108" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E108" s="32" t="str">
+        <x:v>The rogue-key attack has a distinct security learning outcome: naive key aggregation can authorize an attacker-controlled relation. It should not be hidden inside the MuSig construction node.</x:v>
+      </x:c>
+      <x:c r="F108" s="32" t="str">
+        <x:v>security.rogue-key-attack, protocol.musig, fundamentals.schnorr-signatures</x:v>
+      </x:c>
+      <x:c r="G108" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
+      </x:c>
+      <x:c r="H108" s="32" t="str">
+        <x:v>Added after dedupe against MuSig and Schnorr; MuSig is the sole direct graph parent because Schnorr is inherited.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="32" t="str">
+        <x:v>decision.selfish-mining-slice</x:v>
+      </x:c>
+      <x:c r="B109" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C109" s="32" t="str">
+        <x:v>mining.selfish-mining</x:v>
+      </x:c>
+      <x:c r="D109" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E109" s="32" t="str">
+        <x:v>Selfish mining is a chain-selection incentive attack distinct from block withholding, which attacks pool compensation by hiding valid shares. The post fills a missing mining attack branch.</x:v>
+      </x:c>
+      <x:c r="F109" s="32" t="str">
+        <x:v>mining.selfish-mining, mining.block-withholding, mining.pool-vs-solo, protocol.reorgs-finality</x:v>
+      </x:c>
+      <x:c r="G109" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+      </x:c>
+      <x:c r="H109" s="32" t="str">
+        <x:v>Added with pool-versus-solo mining and reorg/finality as direct prerequisites.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="32" t="str">
+        <x:v>decision.commit-delay-reveal-slice</x:v>
+      </x:c>
+      <x:c r="B110" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C110" s="32" t="str">
+        <x:v>protocol.commit-delay-reveal</x:v>
+      </x:c>
+      <x:c r="D110" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E110" s="32" t="str">
+        <x:v>Commit-delay-reveal is a reusable protocol composition that adds timing and anti-adaptation semantics to a commitment scheme. It is narrower than generic commitments and does not duplicate existing commit/reveal-adjacent nodes.</x:v>
+      </x:c>
+      <x:c r="F110" s="32" t="str">
+        <x:v>protocol.commit-delay-reveal, fundamentals.commitment-schemes</x:v>
+      </x:c>
+      <x:c r="G110" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
+      </x:c>
+      <x:c r="H110" s="32" t="str">
+        <x:v>Added with commitment schemes as the only direct prerequisite; preserve the CDR source context in resources.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="32" t="str">
+        <x:v>decision.dust-attack-slice</x:v>
+      </x:c>
+      <x:c r="B111" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C111" s="32" t="str">
+        <x:v>security.dust-attack</x:v>
+      </x:c>
+      <x:c r="D111" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E111" s="32" t="str">
+        <x:v>Dust attack is a privacy threat that is not equivalent to the dust-policy threshold. It explains why unsolicited tiny outputs can create wallet-linkage and coin-control risks.</x:v>
+      </x:c>
+      <x:c r="F111" s="32" t="str">
+        <x:v>security.dust-attack, protocol.dust-policy, privacy.pseudonymity</x:v>
+      </x:c>
+      <x:c r="G111" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+      </x:c>
+      <x:c r="H111" s="32" t="str">
+        <x:v>Added with dust policy and pseudonymity as direct prerequisites.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B104">
+    <x:dataValidation type="list" sqref="B12:B111">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D104">
+    <x:dataValidation type="list" sqref="D12:D111">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -13435,7 +15574,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.69388914352</x:v>
+        <x:v>46214.70099293981</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -13451,7 +15590,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>12</x:v>
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -13459,7 +15598,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>95</x:v>
+        <x:v>129</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -13467,7 +15606,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>111</x:v>
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -13483,7 +15622,7 @@
         <x:v>Existing Matches</x:v>
       </x:c>
       <x:c r="B11" s="22" t="n">
-        <x:v>5</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -13491,7 +15630,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>82</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
docs: complete explained post audit
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R686efcd8451a4147"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rd4fba108478e42ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Re9c4bd089b1e451b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R0085eaf11b324b8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rd48952a9de9c40bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Re173d9b03b3a4cdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rccc897f34c9244f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R38b0e591bd5f4eaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rd15c44f46e10476d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Raad14bf2906f4c56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R00159176b73246f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R3486e0f21fec4d20"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -563,16 +563,16 @@
         <x:v>Track the index views plus individual topic pages for canonical naming, aliases, see-also links, and primary docs.</x:v>
       </x:c>
       <x:c r="H12" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I12" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J12" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K12" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L12" s="32" t="n">
         <x:v>157</x:v>
@@ -1080,16 +1080,16 @@
         <x:v>Track the live X search as one source-family row first, then expand to one row per matching post once current results are enumerated. Group matching posts by concept family such as hashing, fee management, node architecture, channel mechanics, and upgrade proposals.</x:v>
       </x:c>
       <x:c r="H23" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I23" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J23" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K23" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L23" s="32" t="n">
         <x:v>34</x:v>
@@ -1101,7 +1101,7 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="O23" s="32" t="str">
-        <x:v>Reopened after audit correction. The authenticated X search was enumerated on July 11, 2026 and currently exposes 34 matching posts, which are now tracked individually below. The earlier July 8 pass reported 43 posts but did not preserve one source row per post; that historical count remains unresolved until the current and prior inventories are reconciled. Existing normalized coverage includes time-warp attack, duplicate transaction bug, 64-byte transaction bug, nonce reuse, Lamport signatures, and Shamir's Secret Sharing.</x:v>
+        <x:v>Completed for the current authenticated enumeration on July 11, 2026: 34 matching posts are tracked individually below and each has a normalized candidate classification. The earlier July 8 pass reported 43 posts but did not preserve one source row per post; that historical discrepancy is documented in Decisions and is not treated as evidence for nine additional unobserved posts. Existing coverage includes time-warp attack, duplicate transaction bug, 64-byte transaction bug, nonce reuse, Lamport signatures, and Shamir's Secret Sharing.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -15574,7 +15574,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.70099293981</x:v>
+        <x:v>46214.70172208334</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -15590,7 +15590,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>46</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="8">

</xml_diff>

<commit_message>
feat: add permissionless development
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rccc897f34c9244f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R38b0e591bd5f4eaa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rd15c44f46e10476d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Raad14bf2906f4c56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R00159176b73246f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R3486e0f21fec4d20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R92062feb650448e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rf86c0bc4236b4f91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R8c3d428bc609435e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rfbd5f4b25ee34637"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rba019b7d83fc4ee7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R60bfc346291b4ad5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -675,10 +675,10 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="N14" s="32" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="O14" s="32" t="str">
-        <x:v>Heavy overlap with existing philosophy nodes, but strong for bridge concepts like validation sovereignty, consensus vs policy, development review, pseudonymous development, miner decentralization, and selection cryptography. Implemented from this source in the current branch: fundamentals.validation-sovereignty, protocol.consensus-vs-policy, protocol.chain-split-risk, dev.review-culture, dev.pseudonymous-development, mining.miner-decentralization, and dev.selection-cryptography.</x:v>
+        <x:v>Heavy overlap with existing philosophy nodes, but strong for bridge concepts like validation sovereignty, consensus vs policy, development review, permissionless development, pseudonymous development, miner decentralization, and selection cryptography. Implemented from this source in the current branch: fundamentals.validation-sovereignty, protocol.consensus-vs-policy, protocol.chain-split-risk, dev.review-culture, dev.permissionless-development, dev.pseudonymous-development, mining.miner-decentralization, and dev.selection-cryptography.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -8250,198 +8250,200 @@
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="32" t="str">
-        <x:v>privacy.coinjoin</x:v>
+        <x:v>dev.permissionless-development</x:v>
       </x:c>
       <x:c r="B107" s="32" t="str">
-        <x:v>CoinJoin</x:v>
+        <x:v>Permissionless Development</x:v>
       </x:c>
       <x:c r="C107" s="32" t="str">
-        <x:v>Security</x:v>
+        <x:v>History &amp; Governance</x:v>
       </x:c>
       <x:c r="D107" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-2018682587045052753</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="E107" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/2018682587045052753</x:v>
+        <x:v>https://bitcoindevphilosophy.com/#permissionlessdevelopment</x:v>
       </x:c>
       <x:c r="F107" s="32" t="str">
-        <x:v>Coinjoin Explained</x:v>
-      </x:c>
-      <x:c r="G107" s="32" t="str">
-        <x:v>privacy.coinjoin</x:v>
-      </x:c>
+        <x:v>Open Source chapter &gt; Permissionless Development</x:v>
+      </x:c>
+      <x:c r="G107" s="32" t="str"/>
       <x:c r="H107" s="32" t="str">
-        <x:v>existing</x:v>
+        <x:v>new</x:v>
       </x:c>
       <x:c r="I107" s="32" t="str">
-        <x:v>The post teaches the existing collaborative transaction construction concept, not a narrower new protocol mechanism.</x:v>
+        <x:v>One governance concept: anyone can build around Bitcoin without approval from a central authority, while protocol rules and voluntary adoption define the actual constraints.</x:v>
       </x:c>
       <x:c r="J107" s="32" t="str">
-        <x:v>privacy.coin-control, privacy.address-reuse</x:v>
+        <x:v>fundamentals.neutrality, dev.bips-process, dev.review-culture</x:v>
       </x:c>
       <x:c r="K107" s="32" t="str">
-        <x:v>privacy.coin-control, privacy.address-reuse</x:v>
+        <x:v>fundamentals.neutrality, dev.bips-process</x:v>
       </x:c>
       <x:c r="L107" s="32" t="str">
-        <x:v>Preserve the existing node's direct prerequisites.</x:v>
+        <x:v>Neutrality explains permissionless participation as a protocol property, while the BIPs process explains how changes and extensions are proposed. Review culture is an accountability practice rather than a prerequisite for understanding permissionless access.</x:v>
       </x:c>
       <x:c r="M107" s="32" t="str">
-        <x:v>coinjoin</x:v>
+        <x:v>permissionless development, permissionless building, permissionless innovation</x:v>
       </x:c>
       <x:c r="N107" s="32" t="str">
-        <x:v>privacy, collaborative-transactions</x:v>
+        <x:v>development, governance, neutrality, open-source</x:v>
       </x:c>
       <x:c r="O107" s="32" t="str">
-        <x:v>60m</x:v>
+        <x:v>30m</x:v>
       </x:c>
       <x:c r="P107" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q107" s="32" t="str">
-        <x:v>Reuse existing node; do not clone a second CoinJoin explainer.</x:v>
+        <x:v>Add as a governance bridge distinct from protocol neutrality, BIPs process, and review culture.</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="32" t="str">
-        <x:v>audit.post-2017223553708654888</x:v>
+        <x:v>privacy.coinjoin</x:v>
       </x:c>
       <x:c r="B108" s="32" t="str">
-        <x:v>Full Node Architecture</x:v>
+        <x:v>CoinJoin</x:v>
       </x:c>
       <x:c r="C108" s="32" t="str">
-        <x:v>Network, Relay &amp; Client Sync</x:v>
+        <x:v>Security</x:v>
       </x:c>
       <x:c r="D108" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-2017223553708654888</x:v>
+        <x:v>source.bitcoin-dev-project-post-2018682587045052753</x:v>
       </x:c>
       <x:c r="E108" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/2017223553708654888</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/2018682587045052753</x:v>
       </x:c>
       <x:c r="F108" s="32" t="str">
-        <x:v>Full Node Architecture Explained</x:v>
+        <x:v>Coinjoin Explained</x:v>
       </x:c>
       <x:c r="G108" s="32" t="str">
-        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
+        <x:v>privacy.coinjoin</x:v>
       </x:c>
       <x:c r="H108" s="32" t="str">
-        <x:v>merge</x:v>
+        <x:v>existing</x:v>
       </x:c>
       <x:c r="I108" s="32" t="str">
-        <x:v>The post's architecture explanation is covered by the existing learner-facing full-node versus lightweight-wallet trust-model node.</x:v>
+        <x:v>The post teaches the existing collaborative transaction construction concept, not a narrower new protocol mechanism.</x:v>
       </x:c>
       <x:c r="J108" s="32" t="str">
-        <x:v>fundamentals.validation-sovereignty, protocol.light-client-trust-model</x:v>
+        <x:v>privacy.coin-control, privacy.address-reuse</x:v>
       </x:c>
       <x:c r="K108" s="32" t="str">
-        <x:v>fundamentals.validation-sovereignty, protocol.light-client-trust-model</x:v>
+        <x:v>privacy.coin-control, privacy.address-reuse</x:v>
       </x:c>
       <x:c r="L108" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+        <x:v>Preserve the existing node's direct prerequisites.</x:v>
       </x:c>
       <x:c r="M108" s="32" t="str">
-        <x:v>full node architecture</x:v>
+        <x:v>coinjoin</x:v>
       </x:c>
       <x:c r="N108" s="32" t="str">
-        <x:v>nodes, verification, architecture</x:v>
+        <x:v>privacy, collaborative-transactions</x:v>
       </x:c>
       <x:c r="O108" s="32" t="str">
-        <x:v>25m</x:v>
+        <x:v>60m</x:v>
       </x:c>
       <x:c r="P108" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q108" s="32" t="str">
-        <x:v>Merge into ops.full-node-vs-lightweight-wallet; the function/architecture wording does not justify a duplicate node.</x:v>
+        <x:v>Reuse existing node; do not clone a second CoinJoin explainer.</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="32" t="str">
-        <x:v>audit.post-2016929384389890484</x:v>
+        <x:v>audit.post-2017223553708654888</x:v>
       </x:c>
       <x:c r="B109" s="32" t="str">
-        <x:v>SHA-256 Message Schedule</x:v>
+        <x:v>Full Node Architecture</x:v>
       </x:c>
       <x:c r="C109" s="32" t="str">
-        <x:v>Fundamentals</x:v>
+        <x:v>Network, Relay &amp; Client Sync</x:v>
       </x:c>
       <x:c r="D109" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-2016929384389890484</x:v>
+        <x:v>source.bitcoin-dev-project-post-2017223553708654888</x:v>
       </x:c>
       <x:c r="E109" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/2016929384389890484</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/2017223553708654888</x:v>
       </x:c>
       <x:c r="F109" s="32" t="str">
-        <x:v>SHA-256 explained Part 2: Message Schedule</x:v>
+        <x:v>Full Node Architecture Explained</x:v>
       </x:c>
       <x:c r="G109" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
       </x:c>
       <x:c r="H109" s="32" t="str">
         <x:v>merge</x:v>
       </x:c>
       <x:c r="I109" s="32" t="str">
-        <x:v>The message schedule is a subtopic of the existing hash-functions foundation and does not create a separate Bitcoin learner gap at this graph level.</x:v>
+        <x:v>The post's architecture explanation is covered by the existing learner-facing full-node versus lightweight-wallet trust-model node.</x:v>
       </x:c>
       <x:c r="J109" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>fundamentals.validation-sovereignty, protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="K109" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>fundamentals.validation-sovereignty, protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="L109" s="32" t="str">
-        <x:v>The existing node already covers the relevant primitive.</x:v>
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
       </x:c>
       <x:c r="M109" s="32" t="str">
-        <x:v>SHA-256 message schedule</x:v>
+        <x:v>full node architecture</x:v>
       </x:c>
       <x:c r="N109" s="32" t="str">
-        <x:v>hashing, sha256</x:v>
+        <x:v>nodes, verification, architecture</x:v>
       </x:c>
       <x:c r="O109" s="32" t="str">
-        <x:v>30m</x:v>
+        <x:v>25m</x:v>
       </x:c>
       <x:c r="P109" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q109" s="32" t="str">
-        <x:v>Merge into fundamentals.hash-functions; do not create an implementation-detail node for the compression-function substep.</x:v>
+        <x:v>Merge into ops.full-node-vs-lightweight-wallet; the function/architecture wording does not justify a duplicate node.</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="32" t="str">
-        <x:v>audit.post-2012233826504933706</x:v>
+        <x:v>audit.post-2016929384389890484</x:v>
       </x:c>
       <x:c r="B110" s="32" t="str">
-        <x:v>SHA-256</x:v>
+        <x:v>SHA-256 Message Schedule</x:v>
       </x:c>
       <x:c r="C110" s="32" t="str">
         <x:v>Fundamentals</x:v>
       </x:c>
       <x:c r="D110" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-2012233826504933706</x:v>
+        <x:v>source.bitcoin-dev-project-post-2016929384389890484</x:v>
       </x:c>
       <x:c r="E110" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/2012233826504933706</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/2016929384389890484</x:v>
       </x:c>
       <x:c r="F110" s="32" t="str">
-        <x:v>SHA-256 explained</x:v>
+        <x:v>SHA-256 explained Part 2: Message Schedule</x:v>
       </x:c>
       <x:c r="G110" s="32" t="str">
         <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="H110" s="32" t="str">
-        <x:v>existing</x:v>
+        <x:v>merge</x:v>
       </x:c>
       <x:c r="I110" s="32" t="str">
-        <x:v>The post directly explains the existing hash-functions foundation.</x:v>
-      </x:c>
-      <x:c r="J110" s="32" t="str"/>
-      <x:c r="K110" s="32" t="str"/>
+        <x:v>The message schedule is a subtopic of the existing hash-functions foundation and does not create a separate Bitcoin learner gap at this graph level.</x:v>
+      </x:c>
+      <x:c r="J110" s="32" t="str">
+        <x:v>fundamentals.hash-functions</x:v>
+      </x:c>
+      <x:c r="K110" s="32" t="str">
+        <x:v>fundamentals.hash-functions</x:v>
+      </x:c>
       <x:c r="L110" s="32" t="str">
-        <x:v>No additional prerequisite is needed for an existing foundational node.</x:v>
+        <x:v>The existing node already covers the relevant primitive.</x:v>
       </x:c>
       <x:c r="M110" s="32" t="str">
-        <x:v>SHA-256, sha256</x:v>
+        <x:v>SHA-256 message schedule</x:v>
       </x:c>
       <x:c r="N110" s="32" t="str">
         <x:v>hashing, sha256</x:v>
@@ -8453,450 +8455,446 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q110" s="32" t="str">
-        <x:v>Reuse fundamentals.hash-functions.</x:v>
+        <x:v>Merge into fundamentals.hash-functions; do not create an implementation-detail node for the compression-function substep.</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="32" t="str">
-        <x:v>protocol.mast</x:v>
+        <x:v>audit.post-2012233826504933706</x:v>
       </x:c>
       <x:c r="B111" s="32" t="str">
-        <x:v>Merkelized Alternative Script Trees (MAST)</x:v>
+        <x:v>SHA-256</x:v>
       </x:c>
       <x:c r="C111" s="32" t="str">
-        <x:v>Protocol &amp; Consensus</x:v>
+        <x:v>Fundamentals</x:v>
       </x:c>
       <x:c r="D111" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+        <x:v>source.bitcoin-dev-project-post-2012233826504933706</x:v>
       </x:c>
       <x:c r="E111" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1998431297333501989</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/2012233826504933706</x:v>
       </x:c>
       <x:c r="F111" s="32" t="str">
-        <x:v>MAST explained simply</x:v>
-      </x:c>
-      <x:c r="G111" s="32" t="str"/>
+        <x:v>SHA-256 explained</x:v>
+      </x:c>
+      <x:c r="G111" s="32" t="str">
+        <x:v>fundamentals.hash-functions</x:v>
+      </x:c>
       <x:c r="H111" s="32" t="str">
-        <x:v>new</x:v>
+        <x:v>existing</x:v>
       </x:c>
       <x:c r="I111" s="32" t="str">
-        <x:v>MAST is one specific script-commitment idea: commit to multiple spending branches in a Merkle tree while revealing only the executed branch. It is broader than the TapTree implementation and distinct from generic Taproot script-path spending.</x:v>
-      </x:c>
-      <x:c r="J111" s="32" t="str">
-        <x:v>fundamentals.merkle-trees, protocol.script</x:v>
-      </x:c>
-      <x:c r="K111" s="32" t="str">
-        <x:v>fundamentals.merkle-trees, protocol.script</x:v>
-      </x:c>
+        <x:v>The post directly explains the existing hash-functions foundation.</x:v>
+      </x:c>
+      <x:c r="J111" s="32" t="str"/>
+      <x:c r="K111" s="32" t="str"/>
       <x:c r="L111" s="32" t="str">
-        <x:v>Learners need both the Merkle commitment structure and Bitcoin Script branch model before selective branch revelation makes sense.</x:v>
+        <x:v>No additional prerequisite is needed for an existing foundational node.</x:v>
       </x:c>
       <x:c r="M111" s="32" t="str">
-        <x:v>MAST, merkelized alternative script tree, Merkelized Alternative Script Tree</x:v>
+        <x:v>SHA-256, sha256</x:v>
       </x:c>
       <x:c r="N111" s="32" t="str">
-        <x:v>scripts, merkle, privacy, contracts</x:v>
+        <x:v>hashing, sha256</x:v>
       </x:c>
       <x:c r="O111" s="32" t="str">
-        <x:v>35m</x:v>
+        <x:v>30m</x:v>
       </x:c>
       <x:c r="P111" s="32" t="str">
-        <x:v>medium</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="Q111" s="32" t="str">
-        <x:v>Add as a bridge concept only if the existing TapTree chain does not already provide this generic learning outcome; keep TapTree as the Taproot-specific realization.</x:v>
+        <x:v>Reuse fundamentals.hash-functions.</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="32" t="str">
-        <x:v>audit.post-1993443012748415027</x:v>
+        <x:v>protocol.mast</x:v>
       </x:c>
       <x:c r="B112" s="32" t="str">
-        <x:v>Child Pays for Parent</x:v>
+        <x:v>Merkelized Alternative Script Trees (MAST)</x:v>
       </x:c>
       <x:c r="C112" s="32" t="str">
-        <x:v>Network, Relay &amp; Client Sync</x:v>
+        <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D112" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1993443012748415027</x:v>
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
       </x:c>
       <x:c r="E112" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1993443012748415027</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1998431297333501989</x:v>
       </x:c>
       <x:c r="F112" s="32" t="str">
-        <x:v>Child-Pays-For-Parent transaction explained</x:v>
-      </x:c>
-      <x:c r="G112" s="32" t="str">
-        <x:v>protocol.cpfp</x:v>
-      </x:c>
+        <x:v>MAST explained simply</x:v>
+      </x:c>
+      <x:c r="G112" s="32" t="str"/>
       <x:c r="H112" s="32" t="str">
-        <x:v>existing</x:v>
+        <x:v>new</x:v>
       </x:c>
       <x:c r="I112" s="32" t="str">
-        <x:v>The post explains the existing CPFP fee-bumping strategy.</x:v>
+        <x:v>MAST is one specific script-commitment idea: commit to multiple spending branches in a Merkle tree while revealing only the executed branch. It is broader than the TapTree implementation and distinct from generic Taproot script-path spending.</x:v>
       </x:c>
       <x:c r="J112" s="32" t="str">
-        <x:v>protocol.fee-market</x:v>
+        <x:v>fundamentals.merkle-trees, protocol.script</x:v>
       </x:c>
       <x:c r="K112" s="32" t="str">
-        <x:v>protocol.fee-market</x:v>
+        <x:v>fundamentals.merkle-trees, protocol.script</x:v>
       </x:c>
       <x:c r="L112" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+        <x:v>Learners need both the Merkle commitment structure and Bitcoin Script branch model before selective branch revelation makes sense.</x:v>
       </x:c>
       <x:c r="M112" s="32" t="str">
-        <x:v>CPFP, child pays for parent</x:v>
+        <x:v>MAST, merkelized alternative script tree, Merkelized Alternative Script Tree</x:v>
       </x:c>
       <x:c r="N112" s="32" t="str">
-        <x:v>fees, mempool</x:v>
+        <x:v>scripts, merkle, privacy, contracts</x:v>
       </x:c>
       <x:c r="O112" s="32" t="str">
-        <x:v>55m</x:v>
+        <x:v>35m</x:v>
       </x:c>
       <x:c r="P112" s="32" t="str">
-        <x:v>high</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="Q112" s="32" t="str">
-        <x:v>Reuse protocol.cpfp; this is a second explainer, not a new concept.</x:v>
+        <x:v>Add as a bridge concept only if the existing TapTree chain does not already provide this generic learning outcome; keep TapTree as the Taproot-specific realization.</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="32" t="str">
-        <x:v>protocol.sighash-quadratic-hashing</x:v>
+        <x:v>audit.post-1993443012748415027</x:v>
       </x:c>
       <x:c r="B113" s="32" t="str">
-        <x:v>Quadratic SIGHASH Hashing Cost</x:v>
+        <x:v>Child Pays for Parent</x:v>
       </x:c>
       <x:c r="C113" s="32" t="str">
-        <x:v>Protocol &amp; Consensus</x:v>
+        <x:v>Network, Relay &amp; Client Sync</x:v>
       </x:c>
       <x:c r="D113" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
+        <x:v>source.bitcoin-dev-project-post-1993443012748415027</x:v>
       </x:c>
       <x:c r="E113" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1987562939109306699</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1993443012748415027</x:v>
       </x:c>
       <x:c r="F113" s="32" t="str">
-        <x:v>Quadratic Sighash problem O(n^2) explained</x:v>
-      </x:c>
-      <x:c r="G113" s="32" t="str"/>
+        <x:v>Child-Pays-For-Parent transaction explained</x:v>
+      </x:c>
+      <x:c r="G113" s="32" t="str">
+        <x:v>protocol.cpfp</x:v>
+      </x:c>
       <x:c r="H113" s="32" t="str">
-        <x:v>new</x:v>
+        <x:v>existing</x:v>
       </x:c>
       <x:c r="I113" s="32" t="str">
-        <x:v>One specific historical validation problem: legacy signature hashing repeats transaction-wide work for each input, creating quadratic verification cost and motivating cached digest designs.</x:v>
+        <x:v>The post explains the existing CPFP fee-bumping strategy.</x:v>
       </x:c>
       <x:c r="J113" s="32" t="str">
-        <x:v>protocol.sighash-flags</x:v>
+        <x:v>protocol.fee-market</x:v>
       </x:c>
       <x:c r="K113" s="32" t="str">
-        <x:v>protocol.sighash-flags</x:v>
+        <x:v>protocol.fee-market</x:v>
       </x:c>
       <x:c r="L113" s="32" t="str">
-        <x:v>SIGHASH semantics supply the signature-digest context; the performance failure is a distinct consequence rather than a duplicate of the flag definitions.</x:v>
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M113" s="32" t="str">
-        <x:v>quadratic hashing problem, quadratic SIGHASH, O(n^2) SIGHASH</x:v>
+        <x:v>CPFP, child pays for parent</x:v>
       </x:c>
       <x:c r="N113" s="32" t="str">
-        <x:v>sighash, performance, consensus</x:v>
+        <x:v>fees, mempool</x:v>
       </x:c>
       <x:c r="O113" s="32" t="str">
-        <x:v>35m</x:v>
+        <x:v>55m</x:v>
       </x:c>
       <x:c r="P113" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q113" s="32" t="str">
-        <x:v>Add as a narrow historical/protocol bridge; do not model the internal hashing loop as a generic implementation node.</x:v>
+        <x:v>Reuse protocol.cpfp; this is a second explainer, not a new concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="32" t="str">
-        <x:v>audit.post-1982189369684336693</x:v>
+        <x:v>protocol.sighash-quadratic-hashing</x:v>
       </x:c>
       <x:c r="B114" s="32" t="str">
-        <x:v>BIP 158 Compact Block Filters</x:v>
+        <x:v>Quadratic SIGHASH Hashing Cost</x:v>
       </x:c>
       <x:c r="C114" s="32" t="str">
-        <x:v>Network, Relay &amp; Client Sync</x:v>
+        <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D114" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1982189369684336693</x:v>
+        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
       </x:c>
       <x:c r="E114" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1982189369684336693</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1987562939109306699</x:v>
       </x:c>
       <x:c r="F114" s="32" t="str">
-        <x:v>BIP 158: Compact Block Filters explained</x:v>
-      </x:c>
-      <x:c r="G114" s="32" t="str">
-        <x:v>protocol.compact-block-filters</x:v>
-      </x:c>
+        <x:v>Quadratic Sighash problem O(n^2) explained</x:v>
+      </x:c>
+      <x:c r="G114" s="32" t="str"/>
       <x:c r="H114" s="32" t="str">
-        <x:v>existing</x:v>
+        <x:v>new</x:v>
       </x:c>
       <x:c r="I114" s="32" t="str">
-        <x:v>The post teaches the existing BIP 158 compact-filter protocol.</x:v>
+        <x:v>One specific historical validation problem: legacy signature hashing repeats transaction-wide work for each input, creating quadratic verification cost and motivating cached digest designs.</x:v>
       </x:c>
       <x:c r="J114" s="32" t="str">
-        <x:v>dev.p2p-messages, protocol.block-structure</x:v>
+        <x:v>protocol.sighash-flags</x:v>
       </x:c>
       <x:c r="K114" s="32" t="str">
-        <x:v>dev.p2p-messages, protocol.block-structure</x:v>
+        <x:v>protocol.sighash-flags</x:v>
       </x:c>
       <x:c r="L114" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+        <x:v>SIGHASH semantics supply the signature-digest context; the performance failure is a distinct consequence rather than a duplicate of the flag definitions.</x:v>
       </x:c>
       <x:c r="M114" s="32" t="str">
-        <x:v>BIP 158, compact block filters</x:v>
+        <x:v>quadratic hashing problem, quadratic SIGHASH, O(n^2) SIGHASH</x:v>
       </x:c>
       <x:c r="N114" s="32" t="str">
-        <x:v>light-clients, filters, p2p</x:v>
+        <x:v>sighash, performance, consensus</x:v>
       </x:c>
       <x:c r="O114" s="32" t="str">
-        <x:v>70m</x:v>
+        <x:v>35m</x:v>
       </x:c>
       <x:c r="P114" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q114" s="32" t="str">
-        <x:v>Reuse protocol.compact-block-filters.</x:v>
+        <x:v>Add as a narrow historical/protocol bridge; do not model the internal hashing loop as a generic implementation node.</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="32" t="str">
-        <x:v>audit.post-1981761265036144901</x:v>
+        <x:v>audit.post-1982189369684336693</x:v>
       </x:c>
       <x:c r="B115" s="32" t="str">
-        <x:v>Duplicate Transaction Merkle Root Collision</x:v>
+        <x:v>BIP 158 Compact Block Filters</x:v>
       </x:c>
       <x:c r="C115" s="32" t="str">
-        <x:v>Protocol &amp; Consensus</x:v>
+        <x:v>Network, Relay &amp; Client Sync</x:v>
       </x:c>
       <x:c r="D115" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1981761265036144901</x:v>
+        <x:v>source.bitcoin-dev-project-post-1982189369684336693</x:v>
       </x:c>
       <x:c r="E115" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1981761265036144901</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1982189369684336693</x:v>
       </x:c>
       <x:c r="F115" s="32" t="str">
-        <x:v>CVE-2012-2459 duplicate transaction Merkle root collision explained</x:v>
+        <x:v>BIP 158: Compact Block Filters explained</x:v>
       </x:c>
       <x:c r="G115" s="32" t="str">
-        <x:v>protocol.duplicate-transaction-bug</x:v>
+        <x:v>protocol.compact-block-filters</x:v>
       </x:c>
       <x:c r="H115" s="32" t="str">
-        <x:v>merge</x:v>
+        <x:v>existing</x:v>
       </x:c>
       <x:c r="I115" s="32" t="str">
-        <x:v>The collision is a concrete manifestation of the existing duplicate-transaction consensus bug family, not a separate learner outcome at the current graph granularity.</x:v>
+        <x:v>The post teaches the existing BIP 158 compact-filter protocol.</x:v>
       </x:c>
       <x:c r="J115" s="32" t="str">
-        <x:v>protocol.coinbase-transaction, protocol.utxo-model</x:v>
+        <x:v>dev.p2p-messages, protocol.block-structure</x:v>
       </x:c>
       <x:c r="K115" s="32" t="str">
-        <x:v>protocol.coinbase-transaction, protocol.utxo-model</x:v>
+        <x:v>dev.p2p-messages, protocol.block-structure</x:v>
       </x:c>
       <x:c r="L115" s="32" t="str">
         <x:v>Reuse the existing node's direct prerequisites.</x:v>
       </x:c>
       <x:c r="M115" s="32" t="str">
-        <x:v>CVE-2012-2459, Merkle root collision</x:v>
+        <x:v>BIP 158, compact block filters</x:v>
       </x:c>
       <x:c r="N115" s="32" t="str">
-        <x:v>consensus, merkle, security</x:v>
+        <x:v>light-clients, filters, p2p</x:v>
       </x:c>
       <x:c r="O115" s="32" t="str">
-        <x:v>35m</x:v>
+        <x:v>70m</x:v>
       </x:c>
       <x:c r="P115" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q115" s="32" t="str">
-        <x:v>Merge into protocol.duplicate-transaction-bug and preserve the CVE as an alias/resource context.</x:v>
+        <x:v>Reuse protocol.compact-block-filters.</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="32" t="str">
-        <x:v>extension.discreet-log-contracts</x:v>
+        <x:v>audit.post-1981761265036144901</x:v>
       </x:c>
       <x:c r="B116" s="32" t="str">
-        <x:v>Discreet Log Contracts</x:v>
+        <x:v>Duplicate Transaction Merkle Root Collision</x:v>
       </x:c>
       <x:c r="C116" s="32" t="str">
-        <x:v>Extension Systems</x:v>
+        <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D116" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1980708369620168949</x:v>
+        <x:v>source.bitcoin-dev-project-post-1981761265036144901</x:v>
       </x:c>
       <x:c r="E116" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1980708369620168949</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1981761265036144901</x:v>
       </x:c>
       <x:c r="F116" s="32" t="str">
-        <x:v>Discreet Log Contracts explained simply</x:v>
+        <x:v>CVE-2012-2459 duplicate transaction Merkle root collision explained</x:v>
       </x:c>
       <x:c r="G116" s="32" t="str">
-        <x:v>extension.discreet-log-contracts</x:v>
+        <x:v>protocol.duplicate-transaction-bug</x:v>
       </x:c>
       <x:c r="H116" s="32" t="str">
-        <x:v>existing</x:v>
+        <x:v>merge</x:v>
       </x:c>
       <x:c r="I116" s="32" t="str">
-        <x:v>The post explains the existing DLC contract construction.</x:v>
+        <x:v>The collision is a concrete manifestation of the existing duplicate-transaction consensus bug family, not a separate learner outcome at the current graph granularity.</x:v>
       </x:c>
       <x:c r="J116" s="32" t="str">
-        <x:v>protocol.adaptor-signatures</x:v>
+        <x:v>protocol.coinbase-transaction, protocol.utxo-model</x:v>
       </x:c>
       <x:c r="K116" s="32" t="str">
-        <x:v>protocol.adaptor-signatures</x:v>
+        <x:v>protocol.coinbase-transaction, protocol.utxo-model</x:v>
       </x:c>
       <x:c r="L116" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
       </x:c>
       <x:c r="M116" s="32" t="str">
-        <x:v>DLC, DLCs</x:v>
+        <x:v>CVE-2012-2459, Merkle root collision</x:v>
       </x:c>
       <x:c r="N116" s="32" t="str">
-        <x:v>contracts, oracles, adaptor-signatures</x:v>
+        <x:v>consensus, merkle, security</x:v>
       </x:c>
       <x:c r="O116" s="32" t="str">
-        <x:v>85m</x:v>
+        <x:v>35m</x:v>
       </x:c>
       <x:c r="P116" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q116" s="32" t="str">
-        <x:v>Reuse extension.discreet-log-contracts.</x:v>
+        <x:v>Merge into protocol.duplicate-transaction-bug and preserve the CVE as an alias/resource context.</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="32" t="str">
-        <x:v>dev.y2038-problem</x:v>
+        <x:v>extension.discreet-log-contracts</x:v>
       </x:c>
       <x:c r="B117" s="32" t="str">
-        <x:v>Y2038 Problem</x:v>
+        <x:v>Discreet Log Contracts</x:v>
       </x:c>
       <x:c r="C117" s="32" t="str">
-        <x:v>Development</x:v>
+        <x:v>Extension Systems</x:v>
       </x:c>
       <x:c r="D117" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1977486634536104288</x:v>
+        <x:v>source.bitcoin-dev-project-post-1980708369620168949</x:v>
       </x:c>
       <x:c r="E117" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1977486634536104288</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1980708369620168949</x:v>
       </x:c>
       <x:c r="F117" s="32" t="str">
-        <x:v>The Y2038 problem explained</x:v>
-      </x:c>
-      <x:c r="G117" s="32" t="str"/>
+        <x:v>Discreet Log Contracts explained simply</x:v>
+      </x:c>
+      <x:c r="G117" s="32" t="str">
+        <x:v>extension.discreet-log-contracts</x:v>
+      </x:c>
       <x:c r="H117" s="32" t="str">
-        <x:v>skip</x:v>
+        <x:v>existing</x:v>
       </x:c>
       <x:c r="I117" s="32" t="str">
-        <x:v>The post names a general timestamp implementation hazard rather than a Bitcoin-specific learner concept or prerequisite branch.</x:v>
-      </x:c>
-      <x:c r="J117" s="32" t="str"/>
-      <x:c r="K117" s="32" t="str"/>
+        <x:v>The post explains the existing DLC contract construction.</x:v>
+      </x:c>
+      <x:c r="J117" s="32" t="str">
+        <x:v>protocol.adaptor-signatures</x:v>
+      </x:c>
+      <x:c r="K117" s="32" t="str">
+        <x:v>protocol.adaptor-signatures</x:v>
+      </x:c>
       <x:c r="L117" s="32" t="str">
-        <x:v>No Bitcoin graph edge is justified without a Bitcoin-specific learning outcome.</x:v>
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M117" s="32" t="str">
-        <x:v>Year 2038 problem, Unix time overflow</x:v>
+        <x:v>DLC, DLCs</x:v>
       </x:c>
       <x:c r="N117" s="32" t="str">
-        <x:v>time, software</x:v>
+        <x:v>contracts, oracles, adaptor-signatures</x:v>
       </x:c>
       <x:c r="O117" s="32" t="str">
-        <x:v>15m</x:v>
+        <x:v>85m</x:v>
       </x:c>
       <x:c r="P117" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q117" s="32" t="str">
-        <x:v>Skip as off-scope implementation history; retain the source row for coverage evidence.</x:v>
+        <x:v>Reuse extension.discreet-log-contracts.</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="32" t="str">
-        <x:v>audit.post-1977053708065423446</x:v>
+        <x:v>dev.y2038-problem</x:v>
       </x:c>
       <x:c r="B118" s="32" t="str">
-        <x:v>Nonce Reuse Attack</x:v>
+        <x:v>Y2038 Problem</x:v>
       </x:c>
       <x:c r="C118" s="32" t="str">
-        <x:v>Security</x:v>
+        <x:v>Development</x:v>
       </x:c>
       <x:c r="D118" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1977053708065423446</x:v>
+        <x:v>source.bitcoin-dev-project-post-1977486634536104288</x:v>
       </x:c>
       <x:c r="E118" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1977053708065423446</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1977486634536104288</x:v>
       </x:c>
       <x:c r="F118" s="32" t="str">
-        <x:v>Nonce reuse attack explained simply</x:v>
-      </x:c>
-      <x:c r="G118" s="32" t="str">
-        <x:v>security.nonce-reuse-attack</x:v>
-      </x:c>
+        <x:v>The Y2038 problem explained</x:v>
+      </x:c>
+      <x:c r="G118" s="32" t="str"/>
       <x:c r="H118" s="32" t="str">
-        <x:v>existing</x:v>
+        <x:v>skip</x:v>
       </x:c>
       <x:c r="I118" s="32" t="str">
-        <x:v>The post repeats the existing nonce-reuse attack concept.</x:v>
-      </x:c>
-      <x:c r="J118" s="32" t="str">
-        <x:v>fundamentals.schnorr-signatures</x:v>
-      </x:c>
-      <x:c r="K118" s="32" t="str">
-        <x:v>fundamentals.schnorr-signatures</x:v>
-      </x:c>
+        <x:v>The post names a general timestamp implementation hazard rather than a Bitcoin-specific learner concept or prerequisite branch.</x:v>
+      </x:c>
+      <x:c r="J118" s="32" t="str"/>
+      <x:c r="K118" s="32" t="str"/>
       <x:c r="L118" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+        <x:v>No Bitcoin graph edge is justified without a Bitcoin-specific learning outcome.</x:v>
       </x:c>
       <x:c r="M118" s="32" t="str">
-        <x:v>nonce reuse</x:v>
+        <x:v>Year 2038 problem, Unix time overflow</x:v>
       </x:c>
       <x:c r="N118" s="32" t="str">
-        <x:v>signatures, security</x:v>
+        <x:v>time, software</x:v>
       </x:c>
       <x:c r="O118" s="32" t="str">
-        <x:v>30m</x:v>
+        <x:v>15m</x:v>
       </x:c>
       <x:c r="P118" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q118" s="32" t="str">
-        <x:v>Reuse security.nonce-reuse-attack.</x:v>
+        <x:v>Skip as off-scope implementation history; retain the source row for coverage evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="32" t="str">
-        <x:v>audit.post-1976762610948198707</x:v>
+        <x:v>audit.post-1977053708065423446</x:v>
       </x:c>
       <x:c r="B119" s="32" t="str">
-        <x:v>MuSig2</x:v>
+        <x:v>Nonce Reuse Attack</x:v>
       </x:c>
       <x:c r="C119" s="32" t="str">
-        <x:v>Protocol &amp; Consensus</x:v>
+        <x:v>Security</x:v>
       </x:c>
       <x:c r="D119" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1976762610948198707</x:v>
+        <x:v>source.bitcoin-dev-project-post-1977053708065423446</x:v>
       </x:c>
       <x:c r="E119" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1976762610948198707</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1977053708065423446</x:v>
       </x:c>
       <x:c r="F119" s="32" t="str">
-        <x:v>MuSig2 explained simply</x:v>
+        <x:v>Nonce reuse attack explained simply</x:v>
       </x:c>
       <x:c r="G119" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>security.nonce-reuse-attack</x:v>
       </x:c>
       <x:c r="H119" s="32" t="str">
-        <x:v>merge</x:v>
+        <x:v>existing</x:v>
       </x:c>
       <x:c r="I119" s="32" t="str">
-        <x:v>MuSig2 is a protocol version in the existing MuSig family; the current node already covers the key aggregation and interactive signing learning outcome.</x:v>
+        <x:v>The post repeats the existing nonce-reuse attack concept.</x:v>
       </x:c>
       <x:c r="J119" s="32" t="str">
         <x:v>fundamentals.schnorr-signatures</x:v>
@@ -8905,51 +8903,51 @@
         <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="L119" s="32" t="str">
-        <x:v>Reuse the existing MuSig node's direct prerequisite.</x:v>
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M119" s="32" t="str">
-        <x:v>MuSig2, two-round MuSig</x:v>
+        <x:v>nonce reuse</x:v>
       </x:c>
       <x:c r="N119" s="32" t="str">
-        <x:v>schnorr, multisig, aggregation</x:v>
+        <x:v>signatures, security</x:v>
       </x:c>
       <x:c r="O119" s="32" t="str">
-        <x:v>50m</x:v>
+        <x:v>30m</x:v>
       </x:c>
       <x:c r="P119" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q119" s="32" t="str">
-        <x:v>Merge into protocol.musig and preserve MuSig2 as an alias/resource variant.</x:v>
+        <x:v>Reuse security.nonce-reuse-attack.</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="32" t="str">
-        <x:v>audit.post-1976416447577665743</x:v>
+        <x:v>audit.post-1976762610948198707</x:v>
       </x:c>
       <x:c r="B120" s="32" t="str">
-        <x:v>MuSig</x:v>
+        <x:v>MuSig2</x:v>
       </x:c>
       <x:c r="C120" s="32" t="str">
         <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D120" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1976416447577665743</x:v>
+        <x:v>source.bitcoin-dev-project-post-1976762610948198707</x:v>
       </x:c>
       <x:c r="E120" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1976416447577665743</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1976762610948198707</x:v>
       </x:c>
       <x:c r="F120" s="32" t="str">
-        <x:v>MuSig explained simply</x:v>
+        <x:v>MuSig2 explained simply</x:v>
       </x:c>
       <x:c r="G120" s="32" t="str">
         <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="H120" s="32" t="str">
-        <x:v>existing</x:v>
+        <x:v>merge</x:v>
       </x:c>
       <x:c r="I120" s="32" t="str">
-        <x:v>The post directly explains the existing MuSig node.</x:v>
+        <x:v>MuSig2 is a protocol version in the existing MuSig family; the current node already covers the key aggregation and interactive signing learning outcome.</x:v>
       </x:c>
       <x:c r="J120" s="32" t="str">
         <x:v>fundamentals.schnorr-signatures</x:v>
@@ -8958,10 +8956,10 @@
         <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="L120" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+        <x:v>Reuse the existing MuSig node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M120" s="32" t="str">
-        <x:v>MuSig</x:v>
+        <x:v>MuSig2, two-round MuSig</x:v>
       </x:c>
       <x:c r="N120" s="32" t="str">
         <x:v>schnorr, multisig, aggregation</x:v>
@@ -8973,338 +8971,344 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q120" s="32" t="str">
-        <x:v>Reuse protocol.musig.</x:v>
+        <x:v>Merge into protocol.musig and preserve MuSig2 as an alias/resource variant.</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="32" t="str">
-        <x:v>security.rogue-key-attack</x:v>
+        <x:v>audit.post-1976416447577665743</x:v>
       </x:c>
       <x:c r="B121" s="32" t="str">
-        <x:v>Rogue-Key Attack</x:v>
+        <x:v>MuSig</x:v>
       </x:c>
       <x:c r="C121" s="32" t="str">
-        <x:v>Security</x:v>
+        <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D121" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
+        <x:v>source.bitcoin-dev-project-post-1976416447577665743</x:v>
       </x:c>
       <x:c r="E121" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1976008010108678258</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1976416447577665743</x:v>
       </x:c>
       <x:c r="F121" s="32" t="str">
-        <x:v>Schnorr signatures: rogue key attack explained</x:v>
-      </x:c>
-      <x:c r="G121" s="32" t="str"/>
+        <x:v>MuSig explained simply</x:v>
+      </x:c>
+      <x:c r="G121" s="32" t="str">
+        <x:v>protocol.musig</x:v>
+      </x:c>
       <x:c r="H121" s="32" t="str">
-        <x:v>new</x:v>
+        <x:v>existing</x:v>
       </x:c>
       <x:c r="I121" s="32" t="str">
-        <x:v>One multisignature security failure: an attacker can choose a related public key so an aggregate key appears authorized without the victim's intended cooperation.</x:v>
+        <x:v>The post directly explains the existing MuSig node.</x:v>
       </x:c>
       <x:c r="J121" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="K121" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="L121" s="32" t="str">
-        <x:v>MuSig supplies the key-aggregation setting; Schnorr signatures are inherited through MuSig and do not need a redundant direct edge.</x:v>
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M121" s="32" t="str">
-        <x:v>rogue key attack, key aggregation rogue-key attack</x:v>
+        <x:v>MuSig</x:v>
       </x:c>
       <x:c r="N121" s="32" t="str">
-        <x:v>schnorr, multisig, security</x:v>
+        <x:v>schnorr, multisig, aggregation</x:v>
       </x:c>
       <x:c r="O121" s="32" t="str">
-        <x:v>35m</x:v>
+        <x:v>50m</x:v>
       </x:c>
       <x:c r="P121" s="32" t="str">
-        <x:v>medium</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="Q121" s="32" t="str">
-        <x:v>Add as a security failure mode distinct from the MuSig construction itself.</x:v>
+        <x:v>Reuse protocol.musig.</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="32" t="str">
-        <x:v>mining.selfish-mining</x:v>
+        <x:v>security.rogue-key-attack</x:v>
       </x:c>
       <x:c r="B122" s="32" t="str">
-        <x:v>Selfish Mining</x:v>
+        <x:v>Rogue-Key Attack</x:v>
       </x:c>
       <x:c r="C122" s="32" t="str">
-        <x:v>Mining</x:v>
+        <x:v>Security</x:v>
       </x:c>
       <x:c r="D122" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
       </x:c>
       <x:c r="E122" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1975289920634925475</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1976008010108678258</x:v>
       </x:c>
       <x:c r="F122" s="32" t="str">
-        <x:v>Selfish Mining explained simply</x:v>
+        <x:v>Schnorr signatures: rogue key attack explained</x:v>
       </x:c>
       <x:c r="G122" s="32" t="str"/>
       <x:c r="H122" s="32" t="str">
         <x:v>new</x:v>
       </x:c>
       <x:c r="I122" s="32" t="str">
-        <x:v>Selfish mining is one distinct incentive attack in which miners withhold blocks to gain a propagation and chain-selection advantage.</x:v>
+        <x:v>One multisignature security failure: an attacker can choose a related public key so an aggregate key appears authorized without the victim's intended cooperation.</x:v>
       </x:c>
       <x:c r="J122" s="32" t="str">
-        <x:v>mining.pool-vs-solo, protocol.reorgs-finality</x:v>
+        <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="K122" s="32" t="str">
-        <x:v>mining.pool-vs-solo, protocol.reorgs-finality</x:v>
+        <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="L122" s="32" t="str">
-        <x:v>Learners need pooled-mining incentives and the chain-selection/finality model before the withholding strategy is intelligible.</x:v>
+        <x:v>MuSig supplies the key-aggregation setting; Schnorr signatures are inherited through MuSig and do not need a redundant direct edge.</x:v>
       </x:c>
       <x:c r="M122" s="32" t="str">
-        <x:v>selfish mining attack, block withholding for chain advantage</x:v>
+        <x:v>rogue key attack, key aggregation rogue-key attack</x:v>
       </x:c>
       <x:c r="N122" s="32" t="str">
-        <x:v>mining, incentives, attacks</x:v>
+        <x:v>schnorr, multisig, security</x:v>
       </x:c>
       <x:c r="O122" s="32" t="str">
-        <x:v>40m</x:v>
+        <x:v>35m</x:v>
       </x:c>
       <x:c r="P122" s="32" t="str">
-        <x:v>high</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="Q122" s="32" t="str">
-        <x:v>Add as a distinct miner strategy; do not merge it with block withholding, which targets pool compensation rather than chain advantage.</x:v>
+        <x:v>Add as a security failure mode distinct from the MuSig construction itself.</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="32" t="str">
-        <x:v>protocol.sighash-flags</x:v>
+        <x:v>mining.selfish-mining</x:v>
       </x:c>
       <x:c r="B123" s="32" t="str">
-        <x:v>SIGHASH</x:v>
+        <x:v>Selfish Mining</x:v>
       </x:c>
       <x:c r="C123" s="32" t="str">
-        <x:v>Protocol &amp; Consensus</x:v>
+        <x:v>Mining</x:v>
       </x:c>
       <x:c r="D123" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1966579053076337056</x:v>
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
       </x:c>
       <x:c r="E123" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1966579053076337056</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1975289920634925475</x:v>
       </x:c>
       <x:c r="F123" s="32" t="str">
-        <x:v>SigHash explained</x:v>
-      </x:c>
-      <x:c r="G123" s="32" t="str">
-        <x:v>protocol.sighash-flags</x:v>
-      </x:c>
+        <x:v>Selfish Mining explained simply</x:v>
+      </x:c>
+      <x:c r="G123" s="32" t="str"/>
       <x:c r="H123" s="32" t="str">
-        <x:v>existing</x:v>
+        <x:v>new</x:v>
       </x:c>
       <x:c r="I123" s="32" t="str">
-        <x:v>The post explains the existing signature-hash flag concept.</x:v>
+        <x:v>Selfish mining is one distinct incentive attack in which miners withhold blocks to gain a propagation and chain-selection advantage.</x:v>
       </x:c>
       <x:c r="J123" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>mining.pool-vs-solo, protocol.reorgs-finality</x:v>
       </x:c>
       <x:c r="K123" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>mining.pool-vs-solo, protocol.reorgs-finality</x:v>
       </x:c>
       <x:c r="L123" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+        <x:v>Learners need pooled-mining incentives and the chain-selection/finality model before the withholding strategy is intelligible.</x:v>
       </x:c>
       <x:c r="M123" s="32" t="str">
-        <x:v>SIGHASH, signature hash</x:v>
+        <x:v>selfish mining attack, block withholding for chain advantage</x:v>
       </x:c>
       <x:c r="N123" s="32" t="str">
-        <x:v>signatures, transactions</x:v>
+        <x:v>mining, incentives, attacks</x:v>
       </x:c>
       <x:c r="O123" s="32" t="str">
-        <x:v>90m</x:v>
+        <x:v>40m</x:v>
       </x:c>
       <x:c r="P123" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q123" s="32" t="str">
-        <x:v>Reuse protocol.sighash-flags; the quadratic-cost post is tracked separately as a candidate bridge.</x:v>
+        <x:v>Add as a distinct miner strategy; do not merge it with block withholding, which targets pool compensation rather than chain advantage.</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="32" t="str">
-        <x:v>audit.post-1962245647261745216</x:v>
+        <x:v>protocol.sighash-flags</x:v>
       </x:c>
       <x:c r="B124" s="32" t="str">
-        <x:v>Transaction Pinning</x:v>
+        <x:v>SIGHASH</x:v>
       </x:c>
       <x:c r="C124" s="32" t="str">
         <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D124" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1962245647261745216</x:v>
+        <x:v>source.bitcoin-dev-project-post-1966579053076337056</x:v>
       </x:c>
       <x:c r="E124" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1962245647261745216</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1966579053076337056</x:v>
       </x:c>
       <x:c r="F124" s="32" t="str">
-        <x:v>Transaction Pinning explained</x:v>
+        <x:v>SigHash explained</x:v>
       </x:c>
       <x:c r="G124" s="32" t="str">
-        <x:v>protocol.transaction-pinning</x:v>
+        <x:v>protocol.sighash-flags</x:v>
       </x:c>
       <x:c r="H124" s="32" t="str">
         <x:v>existing</x:v>
       </x:c>
       <x:c r="I124" s="32" t="str">
-        <x:v>The post repeats the existing transaction-pinning risk concept.</x:v>
+        <x:v>The post explains the existing signature-hash flag concept.</x:v>
       </x:c>
       <x:c r="J124" s="32" t="str">
-        <x:v>protocol.package-relay</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="K124" s="32" t="str">
-        <x:v>protocol.package-relay</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="L124" s="32" t="str">
         <x:v>Reuse the existing node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M124" s="32" t="str">
-        <x:v>transaction pinning</x:v>
+        <x:v>SIGHASH, signature hash</x:v>
       </x:c>
       <x:c r="N124" s="32" t="str">
-        <x:v>mempool, contracts, attacks</x:v>
+        <x:v>signatures, transactions</x:v>
       </x:c>
       <x:c r="O124" s="32" t="str">
-        <x:v>70m</x:v>
+        <x:v>90m</x:v>
       </x:c>
       <x:c r="P124" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q124" s="32" t="str">
-        <x:v>Reuse protocol.transaction-pinning.</x:v>
+        <x:v>Reuse protocol.sighash-flags; the quadratic-cost post is tracked separately as a candidate bridge.</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="32" t="str">
-        <x:v>protocol.segregated-witness</x:v>
+        <x:v>audit.post-1962245647261745216</x:v>
       </x:c>
       <x:c r="B125" s="32" t="str">
-        <x:v>Segregated Witness</x:v>
+        <x:v>Transaction Pinning</x:v>
       </x:c>
       <x:c r="C125" s="32" t="str">
         <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D125" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1961882664803209229</x:v>
+        <x:v>source.bitcoin-dev-project-post-1962245647261745216</x:v>
       </x:c>
       <x:c r="E125" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1961882664803209229</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1962245647261745216</x:v>
       </x:c>
       <x:c r="F125" s="32" t="str">
-        <x:v>SegWit explained simply</x:v>
+        <x:v>Transaction Pinning explained</x:v>
       </x:c>
       <x:c r="G125" s="32" t="str">
-        <x:v>protocol.segregated-witness</x:v>
+        <x:v>protocol.transaction-pinning</x:v>
       </x:c>
       <x:c r="H125" s="32" t="str">
         <x:v>existing</x:v>
       </x:c>
       <x:c r="I125" s="32" t="str">
-        <x:v>The post explains the existing SegWit protocol upgrade.</x:v>
-      </x:c>
-      <x:c r="J125" s="32" t="str"/>
-      <x:c r="K125" s="32" t="str"/>
+        <x:v>The post repeats the existing transaction-pinning risk concept.</x:v>
+      </x:c>
+      <x:c r="J125" s="32" t="str">
+        <x:v>protocol.package-relay</x:v>
+      </x:c>
+      <x:c r="K125" s="32" t="str">
+        <x:v>protocol.package-relay</x:v>
+      </x:c>
       <x:c r="L125" s="32" t="str">
-        <x:v>Reuse the existing node's graph position.</x:v>
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M125" s="32" t="str">
-        <x:v>SegWit, segwit</x:v>
+        <x:v>transaction pinning</x:v>
       </x:c>
       <x:c r="N125" s="32" t="str">
-        <x:v>segwit, transactions, consensus</x:v>
+        <x:v>mempool, contracts, attacks</x:v>
       </x:c>
       <x:c r="O125" s="32" t="str">
-        <x:v>60m</x:v>
+        <x:v>70m</x:v>
       </x:c>
       <x:c r="P125" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q125" s="32" t="str">
-        <x:v>Reuse protocol.segregated-witness.</x:v>
+        <x:v>Reuse protocol.transaction-pinning.</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="32" t="str">
-        <x:v>audit.post-1956781577544896905</x:v>
+        <x:v>protocol.segregated-witness</x:v>
       </x:c>
       <x:c r="B126" s="32" t="str">
-        <x:v>WOTS+ Key Generation</x:v>
+        <x:v>Segregated Witness</x:v>
       </x:c>
       <x:c r="C126" s="32" t="str">
-        <x:v>Fundamentals</x:v>
+        <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D126" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1956781577544896905</x:v>
+        <x:v>source.bitcoin-dev-project-post-1961882664803209229</x:v>
       </x:c>
       <x:c r="E126" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1956781577544896905</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1961882664803209229</x:v>
       </x:c>
       <x:c r="F126" s="32" t="str">
-        <x:v>WOTS+ key generation explained</x:v>
-      </x:c>
-      <x:c r="G126" s="32" t="str"/>
+        <x:v>SegWit explained simply</x:v>
+      </x:c>
+      <x:c r="G126" s="32" t="str">
+        <x:v>protocol.segregated-witness</x:v>
+      </x:c>
       <x:c r="H126" s="32" t="str">
-        <x:v>skip</x:v>
+        <x:v>existing</x:v>
       </x:c>
       <x:c r="I126" s="32" t="str">
-        <x:v>The post teaches a post-quantum signature subroutine outside Bitcoin's current signature and script model; it does not yet establish a Bitcoin-specific prerequisite gap.</x:v>
+        <x:v>The post explains the existing SegWit protocol upgrade.</x:v>
       </x:c>
       <x:c r="J126" s="32" t="str"/>
       <x:c r="K126" s="32" t="str"/>
       <x:c r="L126" s="32" t="str">
-        <x:v>No direct Bitcoin graph edge is justified for this off-scope cryptographic series.</x:v>
+        <x:v>Reuse the existing node's graph position.</x:v>
       </x:c>
       <x:c r="M126" s="32" t="str">
-        <x:v>WOTS+, Winternitz one-time signature plus</x:v>
+        <x:v>SegWit, segwit</x:v>
       </x:c>
       <x:c r="N126" s="32" t="str">
-        <x:v>post-quantum, signatures</x:v>
+        <x:v>segwit, transactions, consensus</x:v>
       </x:c>
       <x:c r="O126" s="32" t="str">
-        <x:v>30m</x:v>
+        <x:v>60m</x:v>
       </x:c>
       <x:c r="P126" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q126" s="32" t="str">
-        <x:v>Skip as non-Bitcoin-adjacent for this pass; preserve source coverage without adding a generic cryptography branch.</x:v>
+        <x:v>Reuse protocol.segregated-witness.</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="32" t="str">
-        <x:v>audit.post-1952320432033435819</x:v>
+        <x:v>audit.post-1956781577544896905</x:v>
       </x:c>
       <x:c r="B127" s="32" t="str">
-        <x:v>Winternitz One-Time Signatures</x:v>
+        <x:v>WOTS+ Key Generation</x:v>
       </x:c>
       <x:c r="C127" s="32" t="str">
         <x:v>Fundamentals</x:v>
       </x:c>
       <x:c r="D127" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1952320432033435819</x:v>
+        <x:v>source.bitcoin-dev-project-post-1956781577544896905</x:v>
       </x:c>
       <x:c r="E127" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1952320432033435819</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1956781577544896905</x:v>
       </x:c>
       <x:c r="F127" s="32" t="str">
-        <x:v>WOTS explained</x:v>
+        <x:v>WOTS+ key generation explained</x:v>
       </x:c>
       <x:c r="G127" s="32" t="str"/>
       <x:c r="H127" s="32" t="str">
         <x:v>skip</x:v>
       </x:c>
       <x:c r="I127" s="32" t="str">
-        <x:v>The post is part of the SPHINCS+ post-quantum signature series, not a Bitcoin-specific concept currently needed by the graph.</x:v>
+        <x:v>The post teaches a post-quantum signature subroutine outside Bitcoin's current signature and script model; it does not yet establish a Bitcoin-specific prerequisite gap.</x:v>
       </x:c>
       <x:c r="J127" s="32" t="str"/>
       <x:c r="K127" s="32" t="str"/>
@@ -9312,7 +9316,7 @@
         <x:v>No direct Bitcoin graph edge is justified for this off-scope cryptographic series.</x:v>
       </x:c>
       <x:c r="M127" s="32" t="str">
-        <x:v>WOTS, Winternitz signatures</x:v>
+        <x:v>WOTS+, Winternitz one-time signature plus</x:v>
       </x:c>
       <x:c r="N127" s="32" t="str">
         <x:v>post-quantum, signatures</x:v>
@@ -9324,34 +9328,34 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q127" s="32" t="str">
-        <x:v>Skip and keep grouped with the SPHINCS+ series rather than minting isolated cryptographic nodes.</x:v>
+        <x:v>Skip as non-Bitcoin-adjacent for this pass; preserve source coverage without adding a generic cryptography branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="32" t="str">
-        <x:v>audit.post-1951962210902671675</x:v>
+        <x:v>audit.post-1952320432033435819</x:v>
       </x:c>
       <x:c r="B128" s="32" t="str">
-        <x:v>SPHINCS+</x:v>
+        <x:v>Winternitz One-Time Signatures</x:v>
       </x:c>
       <x:c r="C128" s="32" t="str">
         <x:v>Fundamentals</x:v>
       </x:c>
       <x:c r="D128" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1951962210902671675</x:v>
+        <x:v>source.bitcoin-dev-project-post-1952320432033435819</x:v>
       </x:c>
       <x:c r="E128" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1951962210902671675</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1952320432033435819</x:v>
       </x:c>
       <x:c r="F128" s="32" t="str">
-        <x:v>SPHINCS+ and Lamport signatures explained</x:v>
+        <x:v>WOTS explained</x:v>
       </x:c>
       <x:c r="G128" s="32" t="str"/>
       <x:c r="H128" s="32" t="str">
         <x:v>skip</x:v>
       </x:c>
       <x:c r="I128" s="32" t="str">
-        <x:v>SPHINCS+ is a post-quantum signature scheme, but this post does not connect it to a Bitcoin protocol or learner prerequisite branch.</x:v>
+        <x:v>The post is part of the SPHINCS+ post-quantum signature series, not a Bitcoin-specific concept currently needed by the graph.</x:v>
       </x:c>
       <x:c r="J128" s="32" t="str"/>
       <x:c r="K128" s="32" t="str"/>
@@ -9359,7 +9363,7 @@
         <x:v>No direct Bitcoin graph edge is justified for this off-scope cryptographic series.</x:v>
       </x:c>
       <x:c r="M128" s="32" t="str">
-        <x:v>SPHINCS plus</x:v>
+        <x:v>WOTS, Winternitz signatures</x:v>
       </x:c>
       <x:c r="N128" s="32" t="str">
         <x:v>post-quantum, signatures</x:v>
@@ -9371,34 +9375,34 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q128" s="32" t="str">
-        <x:v>Skip for the Bitcoin graph's current scope; revisit only as part of a deliberate post-quantum roadmap.</x:v>
+        <x:v>Skip and keep grouped with the SPHINCS+ series rather than minting isolated cryptographic nodes.</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="32" t="str">
-        <x:v>audit.post-1951704233742651737</x:v>
+        <x:v>audit.post-1951962210902671675</x:v>
       </x:c>
       <x:c r="B129" s="32" t="str">
-        <x:v>SPHINCS+ Signature Scheme</x:v>
+        <x:v>SPHINCS+</x:v>
       </x:c>
       <x:c r="C129" s="32" t="str">
         <x:v>Fundamentals</x:v>
       </x:c>
       <x:c r="D129" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1951704233742651737</x:v>
+        <x:v>source.bitcoin-dev-project-post-1951962210902671675</x:v>
       </x:c>
       <x:c r="E129" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1951704233742651737</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1951962210902671675</x:v>
       </x:c>
       <x:c r="F129" s="32" t="str">
-        <x:v>SPHINCS+ explained</x:v>
+        <x:v>SPHINCS+ and Lamport signatures explained</x:v>
       </x:c>
       <x:c r="G129" s="32" t="str"/>
       <x:c r="H129" s="32" t="str">
         <x:v>skip</x:v>
       </x:c>
       <x:c r="I129" s="32" t="str">
-        <x:v>This is a duplicate introductory post in the same non-Bitcoin-specific SPHINCS+ series.</x:v>
+        <x:v>SPHINCS+ is a post-quantum signature scheme, but this post does not connect it to a Bitcoin protocol or learner prerequisite branch.</x:v>
       </x:c>
       <x:c r="J129" s="32" t="str"/>
       <x:c r="K129" s="32" t="str"/>
@@ -9406,7 +9410,7 @@
         <x:v>No direct Bitcoin graph edge is justified for this off-scope cryptographic series.</x:v>
       </x:c>
       <x:c r="M129" s="32" t="str">
-        <x:v>SPHINCS+</x:v>
+        <x:v>SPHINCS plus</x:v>
       </x:c>
       <x:c r="N129" s="32" t="str">
         <x:v>post-quantum, signatures</x:v>
@@ -9418,456 +9422,450 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q129" s="32" t="str">
-        <x:v>Skip as a duplicate/off-scope series member.</x:v>
+        <x:v>Skip for the Bitcoin graph's current scope; revisit only as part of a deliberate post-quantum roadmap.</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="32" t="str">
-        <x:v>extension.bitchat</x:v>
+        <x:v>audit.post-1951704233742651737</x:v>
       </x:c>
       <x:c r="B130" s="32" t="str">
-        <x:v>Bitchat</x:v>
+        <x:v>SPHINCS+ Signature Scheme</x:v>
       </x:c>
       <x:c r="C130" s="32" t="str">
-        <x:v>Extension Systems</x:v>
+        <x:v>Fundamentals</x:v>
       </x:c>
       <x:c r="D130" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1946961429363327053</x:v>
+        <x:v>source.bitcoin-dev-project-post-1951704233742651737</x:v>
       </x:c>
       <x:c r="E130" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1946961429363327053</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1951704233742651737</x:v>
       </x:c>
       <x:c r="F130" s="32" t="str">
-        <x:v>Bitchat explained simply</x:v>
-      </x:c>
-      <x:c r="G130" s="32" t="str">
-        <x:v>extension.bitchat</x:v>
-      </x:c>
+        <x:v>SPHINCS+ explained</x:v>
+      </x:c>
+      <x:c r="G130" s="32" t="str"/>
       <x:c r="H130" s="32" t="str">
-        <x:v>existing</x:v>
+        <x:v>skip</x:v>
       </x:c>
       <x:c r="I130" s="32" t="str">
-        <x:v>The post explains the existing Bitchat extension concept.</x:v>
-      </x:c>
-      <x:c r="J130" s="32" t="str">
-        <x:v>ops.mesh-networks, extension.nostr</x:v>
-      </x:c>
-      <x:c r="K130" s="32" t="str">
-        <x:v>ops.mesh-networks, extension.nostr</x:v>
-      </x:c>
+        <x:v>This is a duplicate introductory post in the same non-Bitcoin-specific SPHINCS+ series.</x:v>
+      </x:c>
+      <x:c r="J130" s="32" t="str"/>
+      <x:c r="K130" s="32" t="str"/>
       <x:c r="L130" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+        <x:v>No direct Bitcoin graph edge is justified for this off-scope cryptographic series.</x:v>
       </x:c>
       <x:c r="M130" s="32" t="str">
-        <x:v>Bitchat</x:v>
+        <x:v>SPHINCS+</x:v>
       </x:c>
       <x:c r="N130" s="32" t="str">
-        <x:v>messaging, mesh</x:v>
+        <x:v>post-quantum, signatures</x:v>
       </x:c>
       <x:c r="O130" s="32" t="str">
-        <x:v>35m</x:v>
+        <x:v>30m</x:v>
       </x:c>
       <x:c r="P130" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q130" s="32" t="str">
-        <x:v>Reuse extension.bitchat.</x:v>
+        <x:v>Skip as a duplicate/off-scope series member.</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="32" t="str">
-        <x:v>audit.post-1945962367738601788</x:v>
+        <x:v>extension.bitchat</x:v>
       </x:c>
       <x:c r="B131" s="32" t="str">
-        <x:v>Compact Block Filter</x:v>
+        <x:v>Bitchat</x:v>
       </x:c>
       <x:c r="C131" s="32" t="str">
-        <x:v>Network, Relay &amp; Client Sync</x:v>
+        <x:v>Extension Systems</x:v>
       </x:c>
       <x:c r="D131" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1945962367738601788</x:v>
+        <x:v>source.bitcoin-dev-project-post-1946961429363327053</x:v>
       </x:c>
       <x:c r="E131" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1945962367738601788</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1946961429363327053</x:v>
       </x:c>
       <x:c r="F131" s="32" t="str">
-        <x:v>Compact Block Filter explained Part 1</x:v>
+        <x:v>Bitchat explained simply</x:v>
       </x:c>
       <x:c r="G131" s="32" t="str">
-        <x:v>protocol.compact-block-filters</x:v>
+        <x:v>extension.bitchat</x:v>
       </x:c>
       <x:c r="H131" s="32" t="str">
         <x:v>existing</x:v>
       </x:c>
       <x:c r="I131" s="32" t="str">
-        <x:v>This earlier post is another explanation of the existing compact-filter node.</x:v>
+        <x:v>The post explains the existing Bitchat extension concept.</x:v>
       </x:c>
       <x:c r="J131" s="32" t="str">
-        <x:v>dev.p2p-messages, protocol.block-structure</x:v>
+        <x:v>ops.mesh-networks, extension.nostr</x:v>
       </x:c>
       <x:c r="K131" s="32" t="str">
-        <x:v>dev.p2p-messages, protocol.block-structure</x:v>
+        <x:v>ops.mesh-networks, extension.nostr</x:v>
       </x:c>
       <x:c r="L131" s="32" t="str">
         <x:v>Reuse the existing node's direct prerequisites.</x:v>
       </x:c>
       <x:c r="M131" s="32" t="str">
-        <x:v>compact block filter</x:v>
+        <x:v>Bitchat</x:v>
       </x:c>
       <x:c r="N131" s="32" t="str">
-        <x:v>light-clients, filters</x:v>
+        <x:v>messaging, mesh</x:v>
       </x:c>
       <x:c r="O131" s="32" t="str">
-        <x:v>70m</x:v>
+        <x:v>35m</x:v>
       </x:c>
       <x:c r="P131" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q131" s="32" t="str">
-        <x:v>Reuse protocol.compact-block-filters.</x:v>
+        <x:v>Reuse extension.bitchat.</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="32" t="str">
-        <x:v>audit.post-1945645540152135684</x:v>
+        <x:v>audit.post-1945962367738601788</x:v>
       </x:c>
       <x:c r="B132" s="32" t="str">
-        <x:v>Child Pays for Parent</x:v>
+        <x:v>Compact Block Filter</x:v>
       </x:c>
       <x:c r="C132" s="32" t="str">
         <x:v>Network, Relay &amp; Client Sync</x:v>
       </x:c>
       <x:c r="D132" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1945645540152135684</x:v>
+        <x:v>source.bitcoin-dev-project-post-1945962367738601788</x:v>
       </x:c>
       <x:c r="E132" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1945645540152135684</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1945962367738601788</x:v>
       </x:c>
       <x:c r="F132" s="32" t="str">
-        <x:v>Earlier CPFP transaction explanation</x:v>
+        <x:v>Compact Block Filter explained Part 1</x:v>
       </x:c>
       <x:c r="G132" s="32" t="str">
-        <x:v>protocol.cpfp</x:v>
+        <x:v>protocol.compact-block-filters</x:v>
       </x:c>
       <x:c r="H132" s="32" t="str">
         <x:v>existing</x:v>
       </x:c>
       <x:c r="I132" s="32" t="str">
-        <x:v>This is an earlier explainer for the same CPFP concept.</x:v>
+        <x:v>This earlier post is another explanation of the existing compact-filter node.</x:v>
       </x:c>
       <x:c r="J132" s="32" t="str">
-        <x:v>protocol.fee-market</x:v>
+        <x:v>dev.p2p-messages, protocol.block-structure</x:v>
       </x:c>
       <x:c r="K132" s="32" t="str">
-        <x:v>protocol.fee-market</x:v>
+        <x:v>dev.p2p-messages, protocol.block-structure</x:v>
       </x:c>
       <x:c r="L132" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
       </x:c>
       <x:c r="M132" s="32" t="str">
-        <x:v>CPFP</x:v>
+        <x:v>compact block filter</x:v>
       </x:c>
       <x:c r="N132" s="32" t="str">
-        <x:v>fees, mempool</x:v>
+        <x:v>light-clients, filters</x:v>
       </x:c>
       <x:c r="O132" s="32" t="str">
-        <x:v>55m</x:v>
+        <x:v>70m</x:v>
       </x:c>
       <x:c r="P132" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q132" s="32" t="str">
-        <x:v>Reuse protocol.cpfp.</x:v>
+        <x:v>Reuse protocol.compact-block-filters.</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="32" t="str">
-        <x:v>audit.post-1934578478575489365</x:v>
+        <x:v>audit.post-1945645540152135684</x:v>
       </x:c>
       <x:c r="B133" s="32" t="str">
-        <x:v>Lamport Signatures</x:v>
+        <x:v>Child Pays for Parent</x:v>
       </x:c>
       <x:c r="C133" s="32" t="str">
-        <x:v>Fundamentals</x:v>
+        <x:v>Network, Relay &amp; Client Sync</x:v>
       </x:c>
       <x:c r="D133" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1934578478575489365</x:v>
+        <x:v>source.bitcoin-dev-project-post-1945645540152135684</x:v>
       </x:c>
       <x:c r="E133" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1934578478575489365</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1945645540152135684</x:v>
       </x:c>
       <x:c r="F133" s="32" t="str">
-        <x:v>Lamport Signatures explained</x:v>
+        <x:v>Earlier CPFP transaction explanation</x:v>
       </x:c>
       <x:c r="G133" s="32" t="str">
-        <x:v>fundamentals.lamport-signatures</x:v>
+        <x:v>protocol.cpfp</x:v>
       </x:c>
       <x:c r="H133" s="32" t="str">
         <x:v>existing</x:v>
       </x:c>
       <x:c r="I133" s="32" t="str">
-        <x:v>The post repeats the existing Lamport signature concept.</x:v>
+        <x:v>This is an earlier explainer for the same CPFP concept.</x:v>
       </x:c>
       <x:c r="J133" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>protocol.fee-market</x:v>
       </x:c>
       <x:c r="K133" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>protocol.fee-market</x:v>
       </x:c>
       <x:c r="L133" s="32" t="str">
         <x:v>Reuse the existing node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M133" s="32" t="str">
-        <x:v>Lamport signatures</x:v>
+        <x:v>CPFP</x:v>
       </x:c>
       <x:c r="N133" s="32" t="str">
-        <x:v>post-quantum, signatures</x:v>
+        <x:v>fees, mempool</x:v>
       </x:c>
       <x:c r="O133" s="32" t="str">
-        <x:v>30m</x:v>
+        <x:v>55m</x:v>
       </x:c>
       <x:c r="P133" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q133" s="32" t="str">
-        <x:v>Reuse fundamentals.lamport-signatures.</x:v>
+        <x:v>Reuse protocol.cpfp.</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="32" t="str">
-        <x:v>protocol.commit-delay-reveal</x:v>
+        <x:v>audit.post-1934578478575489365</x:v>
       </x:c>
       <x:c r="B134" s="32" t="str">
-        <x:v>Commit-Delay-Reveal Protocol</x:v>
+        <x:v>Lamport Signatures</x:v>
       </x:c>
       <x:c r="C134" s="32" t="str">
-        <x:v>Protocol &amp; Consensus</x:v>
+        <x:v>Fundamentals</x:v>
       </x:c>
       <x:c r="D134" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
+        <x:v>source.bitcoin-dev-project-post-1934578478575489365</x:v>
       </x:c>
       <x:c r="E134" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1931775486449103086</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1934578478575489365</x:v>
       </x:c>
       <x:c r="F134" s="32" t="str">
-        <x:v>Commit-Delay-Reveal protocol explained</x:v>
-      </x:c>
-      <x:c r="G134" s="32" t="str"/>
+        <x:v>Lamport Signatures explained</x:v>
+      </x:c>
+      <x:c r="G134" s="32" t="str">
+        <x:v>fundamentals.lamport-signatures</x:v>
+      </x:c>
       <x:c r="H134" s="32" t="str">
-        <x:v>new</x:v>
+        <x:v>existing</x:v>
       </x:c>
       <x:c r="I134" s="32" t="str">
-        <x:v>One protocol pattern: commit to a value, wait through a delay, and reveal it later so participants cannot adapt after seeing others' commitments.</x:v>
+        <x:v>The post repeats the existing Lamport signature concept.</x:v>
       </x:c>
       <x:c r="J134" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="K134" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="L134" s="32" t="str">
-        <x:v>Commitment schemes provide the hiding/binding foundation; the delay and reveal sequence is the distinct protocol composition.</x:v>
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M134" s="32" t="str">
-        <x:v>CDR protocol, commit delay reveal</x:v>
+        <x:v>Lamport signatures</x:v>
       </x:c>
       <x:c r="N134" s="32" t="str">
-        <x:v>commitments, protocols, coordination</x:v>
+        <x:v>post-quantum, signatures</x:v>
       </x:c>
       <x:c r="O134" s="32" t="str">
-        <x:v>35m</x:v>
+        <x:v>30m</x:v>
       </x:c>
       <x:c r="P134" s="32" t="str">
-        <x:v>medium</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="Q134" s="32" t="str">
-        <x:v>Add only if the post's Bitcoin/BitVM context is retained in the node resources; do not turn generic commit-reveal into an unbounded protocol family.</x:v>
+        <x:v>Reuse fundamentals.lamport-signatures.</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="32" t="str">
-        <x:v>protocol.cross-input-signature-aggregation</x:v>
+        <x:v>protocol.commit-delay-reveal</x:v>
       </x:c>
       <x:c r="B135" s="32" t="str">
-        <x:v>Cross-Input Signature Aggregation</x:v>
+        <x:v>Commit-Delay-Reveal Protocol</x:v>
       </x:c>
       <x:c r="C135" s="32" t="str">
         <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D135" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1905214178379362814</x:v>
+        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
       </x:c>
       <x:c r="E135" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1905214178379362814</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1931775486449103086</x:v>
       </x:c>
       <x:c r="F135" s="32" t="str">
-        <x:v>CISA full aggregation explained</x:v>
-      </x:c>
-      <x:c r="G135" s="32" t="str">
-        <x:v>protocol.cross-input-signature-aggregation</x:v>
-      </x:c>
+        <x:v>Commit-Delay-Reveal protocol explained</x:v>
+      </x:c>
+      <x:c r="G135" s="32" t="str"/>
       <x:c r="H135" s="32" t="str">
-        <x:v>existing</x:v>
+        <x:v>new</x:v>
       </x:c>
       <x:c r="I135" s="32" t="str">
-        <x:v>The post explains the existing CISA concept.</x:v>
+        <x:v>One protocol pattern: commit to a value, wait through a delay, and reveal it later so participants cannot adapt after seeing others' commitments.</x:v>
       </x:c>
       <x:c r="J135" s="32" t="str">
-        <x:v>protocol.adaptor-signatures</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="K135" s="32" t="str">
-        <x:v>protocol.adaptor-signatures</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="L135" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+        <x:v>Commitment schemes provide the hiding/binding foundation; the delay and reveal sequence is the distinct protocol composition.</x:v>
       </x:c>
       <x:c r="M135" s="32" t="str">
-        <x:v>CISA, full signature aggregation</x:v>
+        <x:v>CDR protocol, commit delay reveal</x:v>
       </x:c>
       <x:c r="N135" s="32" t="str">
-        <x:v>signatures, aggregation</x:v>
+        <x:v>commitments, protocols, coordination</x:v>
       </x:c>
       <x:c r="O135" s="32" t="str">
-        <x:v>75m</x:v>
+        <x:v>35m</x:v>
       </x:c>
       <x:c r="P135" s="32" t="str">
-        <x:v>high</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="Q135" s="32" t="str">
-        <x:v>Reuse protocol.cross-input-signature-aggregation.</x:v>
+        <x:v>Add only if the post's Bitcoin/BitVM context is retained in the node resources; do not turn generic commit-reveal into an unbounded protocol family.</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="32" t="str">
-        <x:v>security.dust-attack</x:v>
+        <x:v>protocol.cross-input-signature-aggregation</x:v>
       </x:c>
       <x:c r="B136" s="32" t="str">
-        <x:v>Dust Attack</x:v>
+        <x:v>Cross-Input Signature Aggregation</x:v>
       </x:c>
       <x:c r="C136" s="32" t="str">
-        <x:v>Security</x:v>
+        <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D136" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+        <x:v>source.bitcoin-dev-project-post-1905214178379362814</x:v>
       </x:c>
       <x:c r="E136" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1904946739603452376</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1905214178379362814</x:v>
       </x:c>
       <x:c r="F136" s="32" t="str">
-        <x:v>Dust attack explained</x:v>
-      </x:c>
-      <x:c r="G136" s="32" t="str"/>
+        <x:v>CISA full aggregation explained</x:v>
+      </x:c>
+      <x:c r="G136" s="32" t="str">
+        <x:v>protocol.cross-input-signature-aggregation</x:v>
+      </x:c>
       <x:c r="H136" s="32" t="str">
-        <x:v>new</x:v>
+        <x:v>existing</x:v>
       </x:c>
       <x:c r="I136" s="32" t="str">
-        <x:v>A dust attack is one specific privacy attack: send trace-value outputs to targets so later spending can link their wallets or contaminate their coin-control decisions.</x:v>
+        <x:v>The post explains the existing CISA concept.</x:v>
       </x:c>
       <x:c r="J136" s="32" t="str">
-        <x:v>protocol.dust-policy, privacy.pseudonymity</x:v>
+        <x:v>protocol.adaptor-signatures</x:v>
       </x:c>
       <x:c r="K136" s="32" t="str">
-        <x:v>protocol.dust-policy, privacy.pseudonymity</x:v>
+        <x:v>protocol.adaptor-signatures</x:v>
       </x:c>
       <x:c r="L136" s="32" t="str">
-        <x:v>Dust policy explains the output threshold and pseudonymity explains why forced linkage is harmful; neither edge is transitive through the other.</x:v>
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M136" s="32" t="str">
-        <x:v>dusting attack, dust attack</x:v>
+        <x:v>CISA, full signature aggregation</x:v>
       </x:c>
       <x:c r="N136" s="32" t="str">
-        <x:v>privacy, utxos, attacks</x:v>
+        <x:v>signatures, aggregation</x:v>
       </x:c>
       <x:c r="O136" s="32" t="str">
-        <x:v>30m</x:v>
+        <x:v>75m</x:v>
       </x:c>
       <x:c r="P136" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q136" s="32" t="str">
-        <x:v>Add as a privacy threat distinct from the operational dust-policy threshold.</x:v>
+        <x:v>Reuse protocol.cross-input-signature-aggregation.</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="32" t="str">
-        <x:v>audit.post-1904596944649150556</x:v>
+        <x:v>security.dust-attack</x:v>
       </x:c>
       <x:c r="B137" s="32" t="str">
-        <x:v>CISA Half Signature Aggregation</x:v>
+        <x:v>Dust Attack</x:v>
       </x:c>
       <x:c r="C137" s="32" t="str">
-        <x:v>Protocol &amp; Consensus</x:v>
+        <x:v>Security</x:v>
       </x:c>
       <x:c r="D137" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1904596944649150556</x:v>
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
       </x:c>
       <x:c r="E137" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1904596944649150556</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1904946739603452376</x:v>
       </x:c>
       <x:c r="F137" s="32" t="str">
-        <x:v>CISA half signature aggregation explained</x:v>
-      </x:c>
-      <x:c r="G137" s="32" t="str">
-        <x:v>protocol.cross-input-signature-aggregation</x:v>
-      </x:c>
+        <x:v>Dust attack explained</x:v>
+      </x:c>
+      <x:c r="G137" s="32" t="str"/>
       <x:c r="H137" s="32" t="str">
-        <x:v>merge</x:v>
+        <x:v>new</x:v>
       </x:c>
       <x:c r="I137" s="32" t="str">
-        <x:v>Half-aggregation is a design variant within the existing CISA concept, not a separate learner-facing protocol node.</x:v>
+        <x:v>A dust attack is one specific privacy attack: send trace-value outputs to targets so later spending can link their wallets or contaminate their coin-control decisions.</x:v>
       </x:c>
       <x:c r="J137" s="32" t="str">
-        <x:v>protocol.adaptor-signatures</x:v>
+        <x:v>protocol.dust-policy, privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="K137" s="32" t="str">
-        <x:v>protocol.adaptor-signatures</x:v>
+        <x:v>protocol.dust-policy, privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="L137" s="32" t="str">
-        <x:v>Reuse the existing CISA node's direct prerequisite.</x:v>
+        <x:v>Dust policy explains the output threshold and pseudonymity explains why forced linkage is harmful; neither edge is transitive through the other.</x:v>
       </x:c>
       <x:c r="M137" s="32" t="str">
-        <x:v>half signature aggregation, half-agg</x:v>
+        <x:v>dusting attack, dust attack</x:v>
       </x:c>
       <x:c r="N137" s="32" t="str">
-        <x:v>signatures, aggregation</x:v>
+        <x:v>privacy, utxos, attacks</x:v>
       </x:c>
       <x:c r="O137" s="32" t="str">
-        <x:v>75m</x:v>
+        <x:v>30m</x:v>
       </x:c>
       <x:c r="P137" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q137" s="32" t="str">
-        <x:v>Merge into protocol.cross-input-signature-aggregation and preserve the variant as an alias/context.</x:v>
+        <x:v>Add as a privacy threat distinct from the operational dust-policy threshold.</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="32" t="str">
-        <x:v>audit.post-1904136400213340298</x:v>
+        <x:v>audit.post-1904596944649150556</x:v>
       </x:c>
       <x:c r="B138" s="32" t="str">
-        <x:v>Cross-Input Signature Aggregation</x:v>
+        <x:v>CISA Half Signature Aggregation</x:v>
       </x:c>
       <x:c r="C138" s="32" t="str">
         <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D138" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1904136400213340298</x:v>
+        <x:v>source.bitcoin-dev-project-post-1904596944649150556</x:v>
       </x:c>
       <x:c r="E138" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1904136400213340298</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1904596944649150556</x:v>
       </x:c>
       <x:c r="F138" s="32" t="str">
-        <x:v>CISA explained</x:v>
+        <x:v>CISA half signature aggregation explained</x:v>
       </x:c>
       <x:c r="G138" s="32" t="str">
         <x:v>protocol.cross-input-signature-aggregation</x:v>
       </x:c>
       <x:c r="H138" s="32" t="str">
-        <x:v>existing</x:v>
+        <x:v>merge</x:v>
       </x:c>
       <x:c r="I138" s="32" t="str">
-        <x:v>The post directly explains the existing CISA node.</x:v>
+        <x:v>Half-aggregation is a design variant within the existing CISA concept, not a separate learner-facing protocol node.</x:v>
       </x:c>
       <x:c r="J138" s="32" t="str">
         <x:v>protocol.adaptor-signatures</x:v>
@@ -9876,10 +9874,10 @@
         <x:v>protocol.adaptor-signatures</x:v>
       </x:c>
       <x:c r="L138" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+        <x:v>Reuse the existing CISA node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M138" s="32" t="str">
-        <x:v>CISA</x:v>
+        <x:v>half signature aggregation, half-agg</x:v>
       </x:c>
       <x:c r="N138" s="32" t="str">
         <x:v>signatures, aggregation</x:v>
@@ -9891,112 +9889,165 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q138" s="32" t="str">
-        <x:v>Reuse protocol.cross-input-signature-aggregation.</x:v>
+        <x:v>Merge into protocol.cross-input-signature-aggregation and preserve the variant as an alias/context.</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="32" t="str">
-        <x:v>audit.post-1903881770204070155</x:v>
+        <x:v>audit.post-1904136400213340298</x:v>
       </x:c>
       <x:c r="B139" s="32" t="str">
-        <x:v>Transaction Pinning Attack</x:v>
+        <x:v>Cross-Input Signature Aggregation</x:v>
       </x:c>
       <x:c r="C139" s="32" t="str">
         <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D139" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1903881770204070155</x:v>
+        <x:v>source.bitcoin-dev-project-post-1904136400213340298</x:v>
       </x:c>
       <x:c r="E139" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1903881770204070155</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1904136400213340298</x:v>
       </x:c>
       <x:c r="F139" s="32" t="str">
-        <x:v>Transaction Pinning Attack explained</x:v>
+        <x:v>CISA explained</x:v>
       </x:c>
       <x:c r="G139" s="32" t="str">
-        <x:v>protocol.transaction-pinning</x:v>
+        <x:v>protocol.cross-input-signature-aggregation</x:v>
       </x:c>
       <x:c r="H139" s="32" t="str">
         <x:v>existing</x:v>
       </x:c>
       <x:c r="I139" s="32" t="str">
-        <x:v>This post is a second framing of the existing transaction-pinning risk.</x:v>
+        <x:v>The post directly explains the existing CISA node.</x:v>
       </x:c>
       <x:c r="J139" s="32" t="str">
-        <x:v>protocol.package-relay</x:v>
+        <x:v>protocol.adaptor-signatures</x:v>
       </x:c>
       <x:c r="K139" s="32" t="str">
-        <x:v>protocol.package-relay</x:v>
+        <x:v>protocol.adaptor-signatures</x:v>
       </x:c>
       <x:c r="L139" s="32" t="str">
         <x:v>Reuse the existing node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M139" s="32" t="str">
-        <x:v>transaction pinning attack</x:v>
+        <x:v>CISA</x:v>
       </x:c>
       <x:c r="N139" s="32" t="str">
-        <x:v>mempool, attacks</x:v>
+        <x:v>signatures, aggregation</x:v>
       </x:c>
       <x:c r="O139" s="32" t="str">
-        <x:v>70m</x:v>
+        <x:v>75m</x:v>
       </x:c>
       <x:c r="P139" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q139" s="32" t="str">
-        <x:v>Reuse protocol.transaction-pinning.</x:v>
+        <x:v>Reuse protocol.cross-input-signature-aggregation.</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="32" t="str">
-        <x:v>protocol.sequence-locks-bip68</x:v>
+        <x:v>audit.post-1903881770204070155</x:v>
       </x:c>
       <x:c r="B140" s="32" t="str">
-        <x:v>BIP 68 Sequence Numbers</x:v>
+        <x:v>Transaction Pinning Attack</x:v>
       </x:c>
       <x:c r="C140" s="32" t="str">
         <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D140" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1903150655071719663</x:v>
+        <x:v>source.bitcoin-dev-project-post-1903881770204070155</x:v>
       </x:c>
       <x:c r="E140" s="32" t="str">
-        <x:v>https://x.com/Bitcoin_Devs/status/1903150655071719663</x:v>
+        <x:v>https://x.com/Bitcoin_Devs/status/1903881770204070155</x:v>
       </x:c>
       <x:c r="F140" s="32" t="str">
-        <x:v>BIP-68 sequence number explained</x:v>
+        <x:v>Transaction Pinning Attack explained</x:v>
       </x:c>
       <x:c r="G140" s="32" t="str">
-        <x:v>protocol.sequence-locks-bip68</x:v>
+        <x:v>protocol.transaction-pinning</x:v>
       </x:c>
       <x:c r="H140" s="32" t="str">
         <x:v>existing</x:v>
       </x:c>
       <x:c r="I140" s="32" t="str">
-        <x:v>The post explains the existing BIP 68 sequence-lock concept.</x:v>
+        <x:v>This post is a second framing of the existing transaction-pinning risk.</x:v>
       </x:c>
       <x:c r="J140" s="32" t="str">
-        <x:v>protocol.timelocks</x:v>
+        <x:v>protocol.package-relay</x:v>
       </x:c>
       <x:c r="K140" s="32" t="str">
-        <x:v>protocol.timelocks</x:v>
+        <x:v>protocol.package-relay</x:v>
       </x:c>
       <x:c r="L140" s="32" t="str">
         <x:v>Reuse the existing node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M140" s="32" t="str">
-        <x:v>BIP 68, sequence numbers, relative timelocks</x:v>
+        <x:v>transaction pinning attack</x:v>
       </x:c>
       <x:c r="N140" s="32" t="str">
-        <x:v>timelocks, consensus</x:v>
+        <x:v>mempool, attacks</x:v>
       </x:c>
       <x:c r="O140" s="32" t="str">
-        <x:v>80m</x:v>
+        <x:v>70m</x:v>
       </x:c>
       <x:c r="P140" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q140" s="32" t="str">
+        <x:v>Reuse protocol.transaction-pinning.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" s="32" t="str">
+        <x:v>protocol.sequence-locks-bip68</x:v>
+      </x:c>
+      <x:c r="B141" s="32" t="str">
+        <x:v>BIP 68 Sequence Numbers</x:v>
+      </x:c>
+      <x:c r="C141" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D141" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1903150655071719663</x:v>
+      </x:c>
+      <x:c r="E141" s="32" t="str">
+        <x:v>https://x.com/Bitcoin_Devs/status/1903150655071719663</x:v>
+      </x:c>
+      <x:c r="F141" s="32" t="str">
+        <x:v>BIP-68 sequence number explained</x:v>
+      </x:c>
+      <x:c r="G141" s="32" t="str">
+        <x:v>protocol.sequence-locks-bip68</x:v>
+      </x:c>
+      <x:c r="H141" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I141" s="32" t="str">
+        <x:v>The post explains the existing BIP 68 sequence-lock concept.</x:v>
+      </x:c>
+      <x:c r="J141" s="32" t="str">
+        <x:v>protocol.timelocks</x:v>
+      </x:c>
+      <x:c r="K141" s="32" t="str">
+        <x:v>protocol.timelocks</x:v>
+      </x:c>
+      <x:c r="L141" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M141" s="32" t="str">
+        <x:v>BIP 68, sequence numbers, relative timelocks</x:v>
+      </x:c>
+      <x:c r="N141" s="32" t="str">
+        <x:v>timelocks, consensus</x:v>
+      </x:c>
+      <x:c r="O141" s="32" t="str">
+        <x:v>80m</x:v>
+      </x:c>
+      <x:c r="P141" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q141" s="32" t="str">
         <x:v>Reuse protocol.sequence-locks-bip68.</x:v>
       </x:c>
     </x:row>
@@ -10006,10 +10057,10 @@
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H140">
+    <x:dataValidation type="list" sqref="H12:H141">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P140">
+    <x:dataValidation type="list" sqref="P12:P141">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -12835,16 +12886,62 @@
         <x:v>Keep privacy linkage direct; it is not inherited through dust policy.</x:v>
       </x:c>
     </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="32" t="str">
+        <x:v>fundamentals.neutrality</x:v>
+      </x:c>
+      <x:c r="B132" s="32" t="str">
+        <x:v>dev.permissionless-development</x:v>
+      </x:c>
+      <x:c r="C132" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D132" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E132" s="32" t="str">
+        <x:v>Permissionless development depends on a neutral protocol that does not select which users or applications may participate.</x:v>
+      </x:c>
+      <x:c r="F132" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G132" s="32" t="str">
+        <x:v>Neutrality supplies the protocol property; the BIPs process supplies the change/proposal lifecycle below.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" s="32" t="str">
+        <x:v>dev.bips-process</x:v>
+      </x:c>
+      <x:c r="B133" s="32" t="str">
+        <x:v>dev.permissionless-development</x:v>
+      </x:c>
+      <x:c r="C133" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D133" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E133" s="32" t="str">
+        <x:v>Learners need the proposal and deployment process to distinguish building permissionlessly from changing Bitcoin's consensus rules without broad adoption.</x:v>
+      </x:c>
+      <x:c r="F133" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G133" s="32" t="str">
+        <x:v>Review culture remains related but is not a direct prerequisite for permissionless access.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C131">
+    <x:dataValidation type="list" sqref="C12:C133">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D131">
+    <x:dataValidation type="list" sqref="D12:D133">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -15512,16 +15609,42 @@
         <x:v>Added with dust policy and pseudonymity as direct prerequisites.</x:v>
       </x:c>
     </x:row>
+    <x:row r="112">
+      <x:c r="A112" s="32" t="str">
+        <x:v>decision.permissionless-development-slice</x:v>
+      </x:c>
+      <x:c r="B112" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C112" s="32" t="str">
+        <x:v>dev.permissionless-development</x:v>
+      </x:c>
+      <x:c r="D112" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E112" s="32" t="str">
+        <x:v>Permissionless development is a distinct governance outcome: anyone can build around Bitcoin without an approval authority. It survives dedupe against protocol neutrality, the BIPs process, and review culture because those nodes explain adjacent protocol and process properties rather than the access boundary itself.</x:v>
+      </x:c>
+      <x:c r="F112" s="32" t="str">
+        <x:v>dev.permissionless-development, fundamentals.neutrality, dev.bips-process, dev.review-culture</x:v>
+      </x:c>
+      <x:c r="G112" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="H112" s="32" t="str">
+        <x:v>Added with neutrality and the BIPs process as direct prerequisites; review culture remains related context rather than a redundant parent.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B111">
+    <x:dataValidation type="list" sqref="B12:B112">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D111">
+    <x:dataValidation type="list" sqref="D12:D112">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -15574,7 +15697,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.70172208334</x:v>
+        <x:v>46214.70437629629</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -15598,7 +15721,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -15606,7 +15729,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>120</x:v>
+        <x:v>122</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -15630,7 +15753,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>88</x:v>
+        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add bootstrappable builds
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R92062feb650448e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rf86c0bc4236b4f91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R8c3d428bc609435e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rfbd5f4b25ee34637"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rba019b7d83fc4ee7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R60bfc346291b4ad5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R2ce5ec39d46e4d91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R3f32133a23a34e07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rc47dc4d57cfd4167"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R717c87a8260a444e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R2745259bca1c43d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R153dfb8856c54bce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -672,10 +672,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="M14" s="32" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="N14" s="32" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="O14" s="32" t="str">
         <x:v>Heavy overlap with existing philosophy nodes, but strong for bridge concepts like validation sovereignty, consensus vs policy, development review, permissionless development, pseudonymous development, miner decentralization, and selection cryptography. Implemented from this source in the current branch: fundamentals.validation-sovereignty, protocol.consensus-vs-policy, protocol.chain-split-risk, dev.review-culture, dev.permissionless-development, dev.pseudonymous-development, mining.miner-decentralization, and dev.selection-cryptography.</x:v>
@@ -10051,16 +10051,67 @@
         <x:v>Reuse protocol.sequence-locks-bip68.</x:v>
       </x:c>
     </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="32" t="str">
+        <x:v>dev.bootstrappable-builds</x:v>
+      </x:c>
+      <x:c r="B142" s="32" t="str">
+        <x:v>Bootstrappable Builds</x:v>
+      </x:c>
+      <x:c r="C142" s="32" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="D142" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="E142" s="32" t="str">
+        <x:v>https://bitcoindevphilosophy.com/#trustlessness</x:v>
+      </x:c>
+      <x:c r="F142" s="32" t="str">
+        <x:v>Trustlessness chapter: bootstrappable toolchains</x:v>
+      </x:c>
+      <x:c r="G142" s="32" t="str"/>
+      <x:c r="H142" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I142" s="32" t="str">
+        <x:v>Bootstrappable builds are one supply-chain verification concept: rebuild the compiler and build tools from a small trusted base instead of treating reproducibility of the final binary as sufficient.</x:v>
+      </x:c>
+      <x:c r="J142" s="32" t="str">
+        <x:v>dev.reproducible-builds</x:v>
+      </x:c>
+      <x:c r="K142" s="32" t="str">
+        <x:v>dev.reproducible-builds</x:v>
+      </x:c>
+      <x:c r="L142" s="32" t="str">
+        <x:v>Reproducible builds establish identical output across independent builders; bootstrapping addresses the remaining trust in the builders' compilers and toolchain binaries.</x:v>
+      </x:c>
+      <x:c r="M142" s="32" t="str">
+        <x:v>bootstrappable toolchains, bootstrapable builds, trust-minimized builds</x:v>
+      </x:c>
+      <x:c r="N142" s="32" t="str">
+        <x:v>builds, supply-chain, toolchains, verification</x:v>
+      </x:c>
+      <x:c r="O142" s="32" t="str">
+        <x:v>45m</x:v>
+      </x:c>
+      <x:c r="P142" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q142" s="32" t="str">
+        <x:v>Add as a distinct downstream verification concept, not an alias of reproducible builds.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H141">
+    <x:dataValidation type="list" sqref="H12:H142">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P141">
+    <x:dataValidation type="list" sqref="P12:P142">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -12932,16 +12983,39 @@
         <x:v>Review culture remains related but is not a direct prerequisite for permissionless access.</x:v>
       </x:c>
     </x:row>
+    <x:row r="134">
+      <x:c r="A134" s="32" t="str">
+        <x:v>dev.reproducible-builds</x:v>
+      </x:c>
+      <x:c r="B134" s="32" t="str">
+        <x:v>dev.bootstrappable-builds</x:v>
+      </x:c>
+      <x:c r="C134" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D134" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E134" s="32" t="str">
+        <x:v>Bootstrappable builds extend reproducible builds by reducing trust in the compiler and build-tool binaries used to produce the reproducible output.</x:v>
+      </x:c>
+      <x:c r="F134" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G134" s="32" t="str">
+        <x:v>Keep this as a direct downstream edge; the node is not a duplicate alias for reproducible builds.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C133">
+    <x:dataValidation type="list" sqref="C12:C134">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D133">
+    <x:dataValidation type="list" sqref="D12:D134">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -15635,16 +15709,42 @@
         <x:v>Added with neutrality and the BIPs process as direct prerequisites; review culture remains related context rather than a redundant parent.</x:v>
       </x:c>
     </x:row>
+    <x:row r="113">
+      <x:c r="A113" s="32" t="str">
+        <x:v>decision.bootstrappable-builds-slice</x:v>
+      </x:c>
+      <x:c r="B113" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C113" s="32" t="str">
+        <x:v>dev.bootstrappable-builds</x:v>
+      </x:c>
+      <x:c r="D113" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E113" s="32" t="str">
+        <x:v>Bootstrappable builds survive dedupe against reproducible builds because identical output does not by itself remove trust in the compilers and build tools that produced it. The concept has a distinct supply-chain verification outcome and a clear prerequisite relation.</x:v>
+      </x:c>
+      <x:c r="F113" s="32" t="str">
+        <x:v>dev.bootstrappable-builds, dev.reproducible-builds</x:v>
+      </x:c>
+      <x:c r="G113" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="H113" s="32" t="str">
+        <x:v>Added as a downstream concept with reproducible builds as the only direct prerequisite; Guix is implementation context, not a separate node.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B112">
+    <x:dataValidation type="list" sqref="B12:B113">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D112">
+    <x:dataValidation type="list" sqref="D12:D113">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -15697,7 +15797,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.70437629629</x:v>
+        <x:v>46214.70756951389</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -15721,7 +15821,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>131</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -15729,7 +15829,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>122</x:v>
+        <x:v>123</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -15753,7 +15853,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>89</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add short channel id concept
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R2ce5ec39d46e4d91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R3f32133a23a34e07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rc47dc4d57cfd4167"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R717c87a8260a444e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R2745259bca1c43d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R153dfb8856c54bce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rb352f582a9df456f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R54d64153b63c4a14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Re4ee8fd36f414269"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rb367ef1668a948cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R38f9fbb929e44f6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R53a7bb54a7ff415b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -892,28 +892,28 @@
         <x:v>Track each BOLT document as an enumeration cluster, starting with the index and BOLTs 01, 02, 04, 08, 09, and 10. Extract only atomic mechanisms and deduplicate against existing Lightning nodes before proposing additions.</x:v>
       </x:c>
       <x:c r="H19" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I19" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="J19" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K19" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L19" s="32" t="n">
-        <x:v>7</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="M19" s="32" t="n">
-        <x:v>4</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="N19" s="32" t="n">
-        <x:v>4</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="O19" s="32" t="str">
-        <x:v>Added during source expansion. The first inventory covers the BOLT index plus messaging, peer protocol, onion messaging, encrypted transport, feature negotiation, and DNS bootstrap clusters. Implemented from this source in the current branch: lightning.feature-flags, lightning.onion-messages, lightning.encrypted-authenticated-transport, and lightning.dns-seeds.</x:v>
+        <x:v>Complete first-pass enumeration of all 12 current BOLT documents (00, 01, 02, 03, 04, 05, 07, 08, 09, 10, 11, and 12). Existing commitment, closure, gossip, fee-policy, invoice, and offer nodes were confirmed; lightning.short-channel-id was added as the only missing learner-facing bridge. Message names, TLV fields, and query workflows remain inside their parent protocol concepts rather than becoming implementation-shaped nodes.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -10102,16 +10102,438 @@
         <x:v>Add as a distinct downstream verification concept, not an alias of reproducible builds.</x:v>
       </x:c>
     </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="32" t="str">
+        <x:v>lightning.commitment-transactions</x:v>
+      </x:c>
+      <x:c r="B143" s="32" t="str">
+        <x:v>Lightning Commitment Transactions</x:v>
+      </x:c>
+      <x:c r="C143" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D143" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E143" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/03-transactions.md</x:v>
+      </x:c>
+      <x:c r="F143" s="32" t="str">
+        <x:v>BOLT 03 commitment transaction and output formats</x:v>
+      </x:c>
+      <x:c r="G143" s="32" t="str">
+        <x:v>lightning.commitment-transactions</x:v>
+      </x:c>
+      <x:c r="H143" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I143" s="32" t="str">
+        <x:v>BOLT 03 specifies the existing commitment-transaction concept and its channel-state outputs.</x:v>
+      </x:c>
+      <x:c r="J143" s="32" t="str">
+        <x:v>lightning.payment-channels, protocol.timelocks</x:v>
+      </x:c>
+      <x:c r="K143" s="32" t="str">
+        <x:v>lightning.payment-channels, protocol.timelocks</x:v>
+      </x:c>
+      <x:c r="L143" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+      </x:c>
+      <x:c r="M143" s="32" t="str">
+        <x:v>BOLT 3 transactions, commitment transaction</x:v>
+      </x:c>
+      <x:c r="N143" s="32" t="str">
+        <x:v>lightning, channels, transactions</x:v>
+      </x:c>
+      <x:c r="O143" s="32" t="str">
+        <x:v>80m</x:v>
+      </x:c>
+      <x:c r="P143" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q143" s="32" t="str">
+        <x:v>Existing node confirmed after inspecting BOLT 03.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" s="32" t="str">
+        <x:v>lightning.force-closures</x:v>
+      </x:c>
+      <x:c r="B144" s="32" t="str">
+        <x:v>Lightning Force Closures</x:v>
+      </x:c>
+      <x:c r="C144" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D144" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E144" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/05-onchain.md</x:v>
+      </x:c>
+      <x:c r="F144" s="32" t="str">
+        <x:v>BOLT 05 on-chain transaction handling</x:v>
+      </x:c>
+      <x:c r="G144" s="32" t="str">
+        <x:v>lightning.force-closures</x:v>
+      </x:c>
+      <x:c r="H144" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I144" s="32" t="str">
+        <x:v>BOLT 05 specifies the existing unilateral and on-chain close-handling concept.</x:v>
+      </x:c>
+      <x:c r="J144" s="32" t="str">
+        <x:v>lightning.commitment-transactions, lightning.watchtowers</x:v>
+      </x:c>
+      <x:c r="K144" s="32" t="str">
+        <x:v>lightning.commitment-transactions, lightning.watchtowers</x:v>
+      </x:c>
+      <x:c r="L144" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+      </x:c>
+      <x:c r="M144" s="32" t="str">
+        <x:v>unilateral close, BOLT 5 on-chain handling</x:v>
+      </x:c>
+      <x:c r="N144" s="32" t="str">
+        <x:v>lightning, channels, on-chain</x:v>
+      </x:c>
+      <x:c r="O144" s="32" t="str">
+        <x:v>70m</x:v>
+      </x:c>
+      <x:c r="P144" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q144" s="32" t="str">
+        <x:v>Existing node confirmed after inspecting BOLT 05.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" s="32" t="str">
+        <x:v>lightning.revocation-penalty-keys</x:v>
+      </x:c>
+      <x:c r="B145" s="32" t="str">
+        <x:v>Revocation and Penalty Keys</x:v>
+      </x:c>
+      <x:c r="C145" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D145" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E145" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/05-onchain.md</x:v>
+      </x:c>
+      <x:c r="F145" s="32" t="str">
+        <x:v>BOLT 05 revoked transaction close handling</x:v>
+      </x:c>
+      <x:c r="G145" s="32" t="str">
+        <x:v>lightning.revocation-penalty-keys</x:v>
+      </x:c>
+      <x:c r="H145" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I145" s="32" t="str">
+        <x:v>BOLT 05 specifies the existing revocation and penalty mechanism for outdated commitment states.</x:v>
+      </x:c>
+      <x:c r="J145" s="32" t="str">
+        <x:v>lightning.commitment-transactions</x:v>
+      </x:c>
+      <x:c r="K145" s="32" t="str">
+        <x:v>lightning.commitment-transactions</x:v>
+      </x:c>
+      <x:c r="L145" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M145" s="32" t="str">
+        <x:v>penalty transactions, revoked transaction handling</x:v>
+      </x:c>
+      <x:c r="N145" s="32" t="str">
+        <x:v>lightning, security, channels</x:v>
+      </x:c>
+      <x:c r="O145" s="32" t="str">
+        <x:v>85m</x:v>
+      </x:c>
+      <x:c r="P145" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q145" s="32" t="str">
+        <x:v>Existing node confirmed after inspecting BOLT 05.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" s="32" t="str">
+        <x:v>lightning.gossip-protocol</x:v>
+      </x:c>
+      <x:c r="B146" s="32" t="str">
+        <x:v>Lightning Gossip Protocol</x:v>
+      </x:c>
+      <x:c r="C146" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D146" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E146" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/07-routing-gossip.md</x:v>
+      </x:c>
+      <x:c r="F146" s="32" t="str">
+        <x:v>BOLT 07 node and channel discovery</x:v>
+      </x:c>
+      <x:c r="G146" s="32" t="str">
+        <x:v>lightning.gossip-protocol</x:v>
+      </x:c>
+      <x:c r="H146" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I146" s="32" t="str">
+        <x:v>BOLT 07 specifies the existing gossip concept for node announcements, channel announcements, and routing updates.</x:v>
+      </x:c>
+      <x:c r="J146" s="32" t="str">
+        <x:v>lightning.routing, dev.p2p-messages</x:v>
+      </x:c>
+      <x:c r="K146" s="32" t="str">
+        <x:v>lightning.routing, dev.p2p-messages</x:v>
+      </x:c>
+      <x:c r="L146" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+      </x:c>
+      <x:c r="M146" s="32" t="str">
+        <x:v>channel announcements, node announcements, routing gossip</x:v>
+      </x:c>
+      <x:c r="N146" s="32" t="str">
+        <x:v>lightning, routing, discovery</x:v>
+      </x:c>
+      <x:c r="O146" s="32" t="str">
+        <x:v>85m</x:v>
+      </x:c>
+      <x:c r="P146" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q146" s="32" t="str">
+        <x:v>The message family is kept together; individual announcement messages are implementation-level protocol surfaces, not separate learner nodes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" s="32" t="str">
+        <x:v>lightning.channel-fee-policies</x:v>
+      </x:c>
+      <x:c r="B147" s="32" t="str">
+        <x:v>Lightning Channel Fee Policies</x:v>
+      </x:c>
+      <x:c r="C147" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D147" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E147" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/07-routing-gossip.md#the-channel_update-message</x:v>
+      </x:c>
+      <x:c r="F147" s="32" t="str">
+        <x:v>BOLT 07 channel_update fee and HTLC policy fields</x:v>
+      </x:c>
+      <x:c r="G147" s="32" t="str">
+        <x:v>lightning.channel-fee-policies</x:v>
+      </x:c>
+      <x:c r="H147" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I147" s="32" t="str">
+        <x:v>BOLT 07 specifies the existing learner-facing concept of channel forwarding fees and HTLC policy limits.</x:v>
+      </x:c>
+      <x:c r="J147" s="32" t="str">
+        <x:v>lightning.liquidity</x:v>
+      </x:c>
+      <x:c r="K147" s="32" t="str">
+        <x:v>lightning.liquidity</x:v>
+      </x:c>
+      <x:c r="L147" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M147" s="32" t="str">
+        <x:v>channel_update fees, routing fee policy</x:v>
+      </x:c>
+      <x:c r="N147" s="32" t="str">
+        <x:v>lightning, routing, fees</x:v>
+      </x:c>
+      <x:c r="O147" s="32" t="str">
+        <x:v>70m</x:v>
+      </x:c>
+      <x:c r="P147" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q147" s="32" t="str">
+        <x:v>Existing node confirmed; channel_update itself remains a protocol message rather than a separate node.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" s="32" t="str">
+        <x:v>lightning.short-channel-id</x:v>
+      </x:c>
+      <x:c r="B148" s="32" t="str">
+        <x:v>Short Channel IDs</x:v>
+      </x:c>
+      <x:c r="C148" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D148" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E148" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/07-routing-gossip.md#definition-of-short_channel_id</x:v>
+      </x:c>
+      <x:c r="F148" s="32" t="str">
+        <x:v>BOLT 07 short_channel_id definition</x:v>
+      </x:c>
+      <x:c r="G148" s="32" t="str"/>
+      <x:c r="H148" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I148" s="32" t="str">
+        <x:v>A Short Channel ID is one precise identifier encoding a channel funding output as block height, transaction index, and output index; it is a prerequisite for interpreting Lightning gossip references.</x:v>
+      </x:c>
+      <x:c r="J148" s="32" t="str">
+        <x:v>lightning.payment-channels, protocol.block-height</x:v>
+      </x:c>
+      <x:c r="K148" s="32" t="str">
+        <x:v>lightning.payment-channels, protocol.block-height</x:v>
+      </x:c>
+      <x:c r="L148" s="32" t="str">
+        <x:v>Learners need the channel funding context and the block-height component before the compact on-chain identifier is meaningful.</x:v>
+      </x:c>
+      <x:c r="M148" s="32" t="str">
+        <x:v>short_channel_id, SCID, short channel identifier</x:v>
+      </x:c>
+      <x:c r="N148" s="32" t="str">
+        <x:v>lightning, channels, gossip, identifiers</x:v>
+      </x:c>
+      <x:c r="O148" s="32" t="str">
+        <x:v>25m</x:v>
+      </x:c>
+      <x:c r="P148" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q148" s="32" t="str">
+        <x:v>Add as the only new node from the complete BOLT 07 pass; announcement and query messages remain part of gossip.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" s="32" t="str">
+        <x:v>lightning.invoices</x:v>
+      </x:c>
+      <x:c r="B149" s="32" t="str">
+        <x:v>Invoices and Payment Requests</x:v>
+      </x:c>
+      <x:c r="C149" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D149" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E149" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/11-payment-encoding.md</x:v>
+      </x:c>
+      <x:c r="F149" s="32" t="str">
+        <x:v>BOLT 11 invoice protocol</x:v>
+      </x:c>
+      <x:c r="G149" s="32" t="str">
+        <x:v>lightning.invoices</x:v>
+      </x:c>
+      <x:c r="H149" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I149" s="32" t="str">
+        <x:v>BOLT 11 specifies the existing invoice and payment-request concept.</x:v>
+      </x:c>
+      <x:c r="J149" s="32" t="str">
+        <x:v>lightning.routing</x:v>
+      </x:c>
+      <x:c r="K149" s="32" t="str">
+        <x:v>lightning.routing</x:v>
+      </x:c>
+      <x:c r="L149" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M149" s="32" t="str">
+        <x:v>BOLT 11 invoices, payment requests</x:v>
+      </x:c>
+      <x:c r="N149" s="32" t="str">
+        <x:v>lightning, payments</x:v>
+      </x:c>
+      <x:c r="O149" s="32" t="str">
+        <x:v>50m</x:v>
+      </x:c>
+      <x:c r="P149" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q149" s="32" t="str">
+        <x:v>Existing node confirmed after inspecting BOLT 11 encoding and payer/payee flow.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" s="32" t="str">
+        <x:v>lightning.bolt12-offers</x:v>
+      </x:c>
+      <x:c r="B150" s="32" t="str">
+        <x:v>BOLT12 Offers</x:v>
+      </x:c>
+      <x:c r="C150" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D150" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E150" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/12-offer-encoding.md</x:v>
+      </x:c>
+      <x:c r="F150" s="32" t="str">
+        <x:v>BOLT 12 offers, invoice requests, and invoices</x:v>
+      </x:c>
+      <x:c r="G150" s="32" t="str">
+        <x:v>lightning.bolt12-offers</x:v>
+      </x:c>
+      <x:c r="H150" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I150" s="32" t="str">
+        <x:v>BOLT 12 specifies the existing reusable offers and invoice-request protocol concept.</x:v>
+      </x:c>
+      <x:c r="J150" s="32" t="str">
+        <x:v>lightning.invoices, lightning.route-blinding</x:v>
+      </x:c>
+      <x:c r="K150" s="32" t="str">
+        <x:v>lightning.invoices, lightning.route-blinding</x:v>
+      </x:c>
+      <x:c r="L150" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+      </x:c>
+      <x:c r="M150" s="32" t="str">
+        <x:v>offers, invoice requests, BOLT 12</x:v>
+      </x:c>
+      <x:c r="N150" s="32" t="str">
+        <x:v>lightning, payments, privacy</x:v>
+      </x:c>
+      <x:c r="O150" s="32" t="str">
+        <x:v>75m</x:v>
+      </x:c>
+      <x:c r="P150" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q150" s="32" t="str">
+        <x:v>Existing node confirmed; payment proofs and TLV fields remain internal parts of the BOLT 12 flow rather than standalone learner nodes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H142">
+    <x:dataValidation type="list" sqref="H12:H150">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P142">
+    <x:dataValidation type="list" sqref="P12:P150">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -12433,10 +12855,10 @@
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="32" t="str">
-        <x:v>protocol.nodes-vs-miners</x:v>
+        <x:v>lightning.payment-channels</x:v>
       </x:c>
       <x:c r="B110" s="32" t="str">
-        <x:v>mining.miner-decentralization</x:v>
+        <x:v>lightning.short-channel-id</x:v>
       </x:c>
       <x:c r="C110" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12445,21 +12867,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E110" s="32" t="str">
-        <x:v>Miner decentralization only makes sense once learners distinguish miners' transaction-ordering role from full nodes' independent enforcement of consensus validity.</x:v>
+        <x:v>The identifier names a Lightning channel's on-chain funding output, so learners need the channel and funding relationship first.</x:v>
       </x:c>
       <x:c r="F110" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G110" s="32" t="str">
-        <x:v>The edge keeps censorship power separate from authority to change consensus rules.</x:v>
+        <x:v>Direct channel context; the gossip protocol is a downstream consumer rather than a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>protocol.block-height</x:v>
       </x:c>
       <x:c r="B111" s="32" t="str">
-        <x:v>mining.miner-decentralization</x:v>
+        <x:v>lightning.short-channel-id</x:v>
       </x:c>
       <x:c r="C111" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12468,21 +12890,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E111" s="32" t="str">
-        <x:v>Pool and solo mining explain the participant and coordination structure whose concentration or dispersion determines practical control over transaction ordering.</x:v>
+        <x:v>Short Channel IDs encode block height as their first component, so learners need the block-height concept before decoding the identifier.</x:v>
       </x:c>
       <x:c r="F111" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G111" s="32" t="str">
-        <x:v>Stratum V2 remains optional implementation context, not a direct prerequisite.</x:v>
+        <x:v>The transaction-index and output-index components remain part of the identifier's own outcome rather than extra transitive edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>protocol.nodes-vs-miners</x:v>
       </x:c>
       <x:c r="B112" s="32" t="str">
-        <x:v>dev.selection-cryptography</x:v>
+        <x:v>mining.miner-decentralization</x:v>
       </x:c>
       <x:c r="C112" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12491,21 +12913,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E112" s="32" t="str">
-        <x:v>Selection cryptography evaluates cryptographic tools and dependencies through evidence, testing, authorship, and review quality, so learners need the broader Bitcoin review discipline first.</x:v>
+        <x:v>Miner decentralization only makes sense once learners distinguish miners' transaction-ordering role from full nodes' independent enforcement of consensus validity.</x:v>
       </x:c>
       <x:c r="F112" s="32" t="str">
         <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G112" s="32" t="str">
-        <x:v>Adversarial thinking is inherited through dev.review-culture; reproducible builds are a downstream verification practice rather than a prerequisite.</x:v>
+        <x:v>The edge keeps censorship power separate from authority to change consensus rules.</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="32" t="str">
-        <x:v>mining.pool-shares</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B113" s="32" t="str">
-        <x:v>mining.block-withholding</x:v>
+        <x:v>mining.miner-decentralization</x:v>
       </x:c>
       <x:c r="C113" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12514,21 +12936,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E113" s="32" t="str">
-        <x:v>Block withholding exploits the difference between a pool-paid share and a share that also meets the network target, so learners must understand share accounting before the attack model makes sense.</x:v>
+        <x:v>Pool and solo mining explain the participant and coordination structure whose concentration or dispersion determines practical control over transaction ordering.</x:v>
       </x:c>
       <x:c r="F113" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G113" s="32" t="str">
-        <x:v>Pool-versus-solo and mining economics are inherited through mining.pool-shares; do not add a redundant majority-attack edge.</x:v>
+        <x:v>Stratum V2 remains optional implementation context, not a direct prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="B114" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>dev.selection-cryptography</x:v>
       </x:c>
       <x:c r="C114" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12537,21 +12959,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E114" s="32" t="str">
-        <x:v>P2C tweaks a public key to commit to contract data, so learners need the public/private key model.</x:v>
+        <x:v>Selection cryptography evaluates cryptographic tools and dependencies through evidence, testing, authorship, and review quality, so learners need the broader Bitcoin review discipline first.</x:v>
       </x:c>
       <x:c r="F114" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G114" s="32" t="str">
-        <x:v>Taproot is adjacent, not a direct requirement.</x:v>
+        <x:v>Adversarial thinking is inherited through dev.review-culture; reproducible builds are a downstream verification practice rather than a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>mining.pool-shares</x:v>
       </x:c>
       <x:c r="B115" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>mining.block-withholding</x:v>
       </x:c>
       <x:c r="C115" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12560,21 +12982,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E115" s="32" t="str">
-        <x:v>P2C derives a commitment tweak from contract data using a hash, so learners need hash commitments first.</x:v>
+        <x:v>Block withholding exploits the difference between a pool-paid share and a share that also meets the network target, so learners must understand share accounting before the attack model makes sense.</x:v>
       </x:c>
       <x:c r="F115" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G115" s="32" t="str">
-        <x:v>The hash is part of the construction rather than generic background.</x:v>
+        <x:v>Pool-versus-solo and mining economics are inherited through mining.pool-shares; do not add a redundant majority-attack edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="32" t="str">
-        <x:v>protocol.utxo-model</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B116" s="32" t="str">
-        <x:v>extension.single-use-seals</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="C116" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12583,21 +13005,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E116" s="32" t="str">
-        <x:v>Single-use seals rely on a UTXO's one-time spend property.</x:v>
+        <x:v>P2C tweaks a public key to commit to contract data, so learners need the public/private key model.</x:v>
       </x:c>
       <x:c r="F116" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G116" s="32" t="str">
-        <x:v>This explicit bridge prevents hiding the seal invariant inside generic UTXO semantics.</x:v>
+        <x:v>Taproot is adjacent, not a direct requirement.</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="32" t="str">
-        <x:v>extension.single-use-seals</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B117" s="32" t="str">
-        <x:v>extension.client-side-validation</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="C117" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12606,21 +13028,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E117" s="32" t="str">
-        <x:v>Client-side validation relies on seals to prevent an offchain transition from being valid twice.</x:v>
+        <x:v>P2C derives a commitment tweak from contract data using a hash, so learners need hash commitments first.</x:v>
       </x:c>
       <x:c r="F117" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G117" s="32" t="str">
-        <x:v>The UTXO parent is inherited through the seal and is intentionally not duplicated.</x:v>
+        <x:v>The hash is part of the construction rather than generic background.</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>protocol.utxo-model</x:v>
       </x:c>
       <x:c r="B118" s="32" t="str">
-        <x:v>extension.client-side-validation</x:v>
+        <x:v>extension.single-use-seals</x:v>
       </x:c>
       <x:c r="C118" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12629,21 +13051,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E118" s="32" t="str">
-        <x:v>Client-side validation uses cryptographic commitments to bind offchain asset rules and transitions, so P2C supplies the contract-anchoring mechanism.</x:v>
+        <x:v>Single-use seals rely on a UTXO's one-time spend property.</x:v>
       </x:c>
       <x:c r="F118" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G118" s="32" t="str">
-        <x:v>Keep this direct edge: it prevents treating client-side validation as a vague UTXO-only extension.</x:v>
+        <x:v>This explicit bridge prevents hiding the seal invariant inside generic UTXO semantics.</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="32" t="str">
-        <x:v>protocol.rbf</x:v>
+        <x:v>extension.single-use-seals</x:v>
       </x:c>
       <x:c r="B119" s="32" t="str">
-        <x:v>protocol.replacement-cycling</x:v>
+        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="C119" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12652,21 +13074,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E119" s="32" t="str">
-        <x:v>Replacement cycling repeatedly uses transaction replacement, so learners need the RBF policy mechanism first.</x:v>
+        <x:v>Client-side validation relies on seals to prevent an offchain transition from being valid twice.</x:v>
       </x:c>
       <x:c r="F119" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G119" s="32" t="str">
-        <x:v>Package RBF is related but not required for the core attack sequence.</x:v>
+        <x:v>The UTXO parent is inherited through the seal and is intentionally not duplicated.</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="32" t="str">
-        <x:v>protocol.cpfp</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="B120" s="32" t="str">
-        <x:v>protocol.replacement-cycling</x:v>
+        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="C120" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12675,21 +13097,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E120" s="32" t="str">
-        <x:v>The attack cycles child-fee relationships to evict a target, so learners need CPFP mechanics first.</x:v>
+        <x:v>Client-side validation uses cryptographic commitments to bind offchain asset rules and transitions, so P2C supplies the contract-anchoring mechanism.</x:v>
       </x:c>
       <x:c r="F120" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G120" s="32" t="str">
-        <x:v>Transaction pinning is the broader downstream risk class, not a prerequisite.</x:v>
+        <x:v>Keep this direct edge: it prevents treating client-side validation as a vague UTXO-only extension.</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="32" t="str">
-        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
+        <x:v>protocol.rbf</x:v>
       </x:c>
       <x:c r="B121" s="32" t="str">
-        <x:v>protocol.taproot-control-blocks</x:v>
+        <x:v>protocol.replacement-cycling</x:v>
       </x:c>
       <x:c r="C121" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12698,21 +13120,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E121" s="32" t="str">
-        <x:v>Control blocks extend the tapleaf proof path with internal-key and parity data.</x:v>
+        <x:v>Replacement cycling repeatedly uses transaction replacement, so learners need the RBF policy mechanism first.</x:v>
       </x:c>
       <x:c r="F121" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G121" s="32" t="str">
-        <x:v>Generic Merkle trees are inherited through the proof node.</x:v>
+        <x:v>Package RBF is related but not required for the core attack sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>protocol.cpfp</x:v>
       </x:c>
       <x:c r="B122" s="32" t="str">
-        <x:v>dev.pseudonymous-development</x:v>
+        <x:v>protocol.replacement-cycling</x:v>
       </x:c>
       <x:c r="C122" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12721,21 +13143,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E122" s="32" t="str">
-        <x:v>Pseudonymous development relies on public technical evidence and independent peer review to preserve accountability without requiring legal-identity disclosure.</x:v>
+        <x:v>The attack cycles child-fee relationships to evict a target, so learners need CPFP mechanics first.</x:v>
       </x:c>
       <x:c r="F122" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G122" s="32" t="str">
-        <x:v>Privacy pseudonymity is related context, not a direct prerequisite, because this node concerns contributor identity and governance rather than transaction linkage.</x:v>
+        <x:v>Transaction pinning is the broader downstream risk class, not a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="32" t="str">
-        <x:v>fundamentals.merkle-trees</x:v>
+        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
       </x:c>
       <x:c r="B123" s="32" t="str">
-        <x:v>protocol.mast</x:v>
+        <x:v>protocol.taproot-control-blocks</x:v>
       </x:c>
       <x:c r="C123" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12744,21 +13166,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E123" s="32" t="str">
-        <x:v>MAST uses a Merkle tree to commit to multiple alternative script branches while revealing only one branch during spending.</x:v>
+        <x:v>Control blocks extend the tapleaf proof path with internal-key and parity data.</x:v>
       </x:c>
       <x:c r="F123" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G123" s="32" t="str">
-        <x:v>Direct cryptographic structure; TapTree remains a downstream Taproot-specific realization.</x:v>
+        <x:v>Generic Merkle trees are inherited through the proof node.</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="B124" s="32" t="str">
-        <x:v>protocol.mast</x:v>
+        <x:v>dev.pseudonymous-development</x:v>
       </x:c>
       <x:c r="C124" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12767,21 +13189,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E124" s="32" t="str">
-        <x:v>MAST commits to alternative Bitcoin Script branches, so learners need the locking and spending language before the tree commitment is meaningful.</x:v>
+        <x:v>Pseudonymous development relies on public technical evidence and independent peer review to preserve accountability without requiring legal-identity disclosure.</x:v>
       </x:c>
       <x:c r="F124" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G124" s="32" t="str">
-        <x:v>Keep Script direct; the node is not only a generic Merkle-tree concept.</x:v>
+        <x:v>Privacy pseudonymity is related context, not a direct prerequisite, because this node concerns contributor identity and governance rather than transaction linkage.</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="32" t="str">
-        <x:v>protocol.sighash-flags</x:v>
+        <x:v>fundamentals.merkle-trees</x:v>
       </x:c>
       <x:c r="B125" s="32" t="str">
-        <x:v>protocol.sighash-quadratic-hashing</x:v>
+        <x:v>protocol.mast</x:v>
       </x:c>
       <x:c r="C125" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12790,21 +13212,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E125" s="32" t="str">
-        <x:v>The quadratic hashing problem is a performance consequence of how legacy signature digests are constructed under SIGHASH semantics.</x:v>
+        <x:v>MAST uses a Merkle tree to commit to multiple alternative script branches while revealing only one branch during spending.</x:v>
       </x:c>
       <x:c r="F125" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
       </x:c>
       <x:c r="G125" s="32" t="str">
-        <x:v>BIP 143 is a supporting mitigation source, not a prerequisite edge.</x:v>
+        <x:v>Direct cryptographic structure; TapTree remains a downstream Taproot-specific realization.</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B126" s="32" t="str">
-        <x:v>security.rogue-key-attack</x:v>
+        <x:v>protocol.mast</x:v>
       </x:c>
       <x:c r="C126" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12813,21 +13235,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E126" s="32" t="str">
-        <x:v>The rogue-key attack occurs in naive public-key aggregation, so learners need the MuSig aggregation setting before the failure mode.</x:v>
+        <x:v>MAST commits to alternative Bitcoin Script branches, so learners need the locking and spending language before the tree commitment is meaningful.</x:v>
       </x:c>
       <x:c r="F126" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
       </x:c>
       <x:c r="G126" s="32" t="str">
-        <x:v>Schnorr is inherited through MuSig; avoid a redundant direct Schnorr edge.</x:v>
+        <x:v>Keep Script direct; the node is not only a generic Merkle-tree concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>protocol.sighash-flags</x:v>
       </x:c>
       <x:c r="B127" s="32" t="str">
-        <x:v>mining.selfish-mining</x:v>
+        <x:v>protocol.sighash-quadratic-hashing</x:v>
       </x:c>
       <x:c r="C127" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12836,21 +13258,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E127" s="32" t="str">
-        <x:v>Selfish mining is an incentive strategy by miners and pools, so learners need the pooled-versus-solo mining context first.</x:v>
+        <x:v>The quadratic hashing problem is a performance consequence of how legacy signature digests are constructed under SIGHASH semantics.</x:v>
       </x:c>
       <x:c r="F127" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
       </x:c>
       <x:c r="G127" s="32" t="str">
-        <x:v>Pool economics is one direct parent; chain selection is supplied by the finality parent below.</x:v>
+        <x:v>BIP 143 is a supporting mitigation source, not a prerequisite edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="32" t="str">
-        <x:v>protocol.reorgs-finality</x:v>
+        <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="B128" s="32" t="str">
-        <x:v>mining.selfish-mining</x:v>
+        <x:v>security.rogue-key-attack</x:v>
       </x:c>
       <x:c r="C128" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12859,21 +13281,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E128" s="32" t="str">
-        <x:v>Selfish mining relies on strategic withholding and release of competing branches, which requires the chain-reorganization and finality model.</x:v>
+        <x:v>The rogue-key attack occurs in naive public-key aggregation, so learners need the MuSig aggregation setting before the failure mode.</x:v>
       </x:c>
       <x:c r="F128" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
       </x:c>
       <x:c r="G128" s="32" t="str">
-        <x:v>Keep the reorganization model direct rather than adding generic proof-of-work as a redundant ancestor.</x:v>
+        <x:v>Schnorr is inherited through MuSig; avoid a redundant direct Schnorr edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B129" s="32" t="str">
-        <x:v>protocol.commit-delay-reveal</x:v>
+        <x:v>mining.selfish-mining</x:v>
       </x:c>
       <x:c r="C129" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12882,21 +13304,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E129" s="32" t="str">
-        <x:v>Commit-delay-reveal composes a cryptographic commitment with a timed reveal, so the learner first needs the hiding and binding commitment model.</x:v>
+        <x:v>Selfish mining is an incentive strategy by miners and pools, so learners need the pooled-versus-solo mining context first.</x:v>
       </x:c>
       <x:c r="F129" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
       </x:c>
       <x:c r="G129" s="32" t="str">
-        <x:v>The delay/reveal composition is the node's distinct outcome.</x:v>
+        <x:v>Pool economics is one direct parent; chain selection is supplied by the finality parent below.</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="32" t="str">
-        <x:v>protocol.dust-policy</x:v>
+        <x:v>protocol.reorgs-finality</x:v>
       </x:c>
       <x:c r="B130" s="32" t="str">
-        <x:v>security.dust-attack</x:v>
+        <x:v>mining.selfish-mining</x:v>
       </x:c>
       <x:c r="C130" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12905,21 +13327,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E130" s="32" t="str">
-        <x:v>Dust attacks exploit the distinction between tiny-output relay policy and the ability to place trace-value UTXOs in a wallet.</x:v>
+        <x:v>Selfish mining relies on strategic withholding and release of competing branches, which requires the chain-reorganization and finality model.</x:v>
       </x:c>
       <x:c r="F130" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
       </x:c>
       <x:c r="G130" s="32" t="str">
-        <x:v>Policy threshold is direct context for the attack mechanism.</x:v>
+        <x:v>Keep the reorganization model direct rather than adding generic proof-of-work as a redundant ancestor.</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="B131" s="32" t="str">
-        <x:v>security.dust-attack</x:v>
+        <x:v>protocol.commit-delay-reveal</x:v>
       </x:c>
       <x:c r="C131" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12928,21 +13350,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E131" s="32" t="str">
-        <x:v>The privacy harm of dusting comes from linking future spends and wallet activity, so learners need the pseudonymity and linkage model.</x:v>
+        <x:v>Commit-delay-reveal composes a cryptographic commitment with a timed reveal, so the learner first needs the hiding and binding commitment model.</x:v>
       </x:c>
       <x:c r="F131" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
       </x:c>
       <x:c r="G131" s="32" t="str">
-        <x:v>Keep privacy linkage direct; it is not inherited through dust policy.</x:v>
+        <x:v>The delay/reveal composition is the node's distinct outcome.</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="32" t="str">
-        <x:v>fundamentals.neutrality</x:v>
+        <x:v>protocol.dust-policy</x:v>
       </x:c>
       <x:c r="B132" s="32" t="str">
-        <x:v>dev.permissionless-development</x:v>
+        <x:v>security.dust-attack</x:v>
       </x:c>
       <x:c r="C132" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12951,21 +13373,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E132" s="32" t="str">
-        <x:v>Permissionless development depends on a neutral protocol that does not select which users or applications may participate.</x:v>
+        <x:v>Dust attacks exploit the distinction between tiny-output relay policy and the ability to place trace-value UTXOs in a wallet.</x:v>
       </x:c>
       <x:c r="F132" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
       </x:c>
       <x:c r="G132" s="32" t="str">
-        <x:v>Neutrality supplies the protocol property; the BIPs process supplies the change/proposal lifecycle below.</x:v>
+        <x:v>Policy threshold is direct context for the attack mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="32" t="str">
-        <x:v>dev.bips-process</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B133" s="32" t="str">
-        <x:v>dev.permissionless-development</x:v>
+        <x:v>security.dust-attack</x:v>
       </x:c>
       <x:c r="C133" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12974,21 +13396,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E133" s="32" t="str">
-        <x:v>Learners need the proposal and deployment process to distinguish building permissionlessly from changing Bitcoin's consensus rules without broad adoption.</x:v>
+        <x:v>The privacy harm of dusting comes from linking future spends and wallet activity, so learners need the pseudonymity and linkage model.</x:v>
       </x:c>
       <x:c r="F133" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
       </x:c>
       <x:c r="G133" s="32" t="str">
-        <x:v>Review culture remains related but is not a direct prerequisite for permissionless access.</x:v>
+        <x:v>Keep privacy linkage direct; it is not inherited through dust policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="32" t="str">
-        <x:v>dev.reproducible-builds</x:v>
+        <x:v>fundamentals.neutrality</x:v>
       </x:c>
       <x:c r="B134" s="32" t="str">
-        <x:v>dev.bootstrappable-builds</x:v>
+        <x:v>dev.permissionless-development</x:v>
       </x:c>
       <x:c r="C134" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12997,12 +13419,58 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E134" s="32" t="str">
-        <x:v>Bootstrappable builds extend reproducible builds by reducing trust in the compiler and build-tool binaries used to produce the reproducible output.</x:v>
+        <x:v>Permissionless development depends on a neutral protocol that does not select which users or applications may participate.</x:v>
       </x:c>
       <x:c r="F134" s="32" t="str">
         <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G134" s="32" t="str">
+        <x:v>Neutrality supplies the protocol property; the BIPs process supplies the change/proposal lifecycle below.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" s="32" t="str">
+        <x:v>dev.bips-process</x:v>
+      </x:c>
+      <x:c r="B135" s="32" t="str">
+        <x:v>dev.permissionless-development</x:v>
+      </x:c>
+      <x:c r="C135" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D135" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E135" s="32" t="str">
+        <x:v>Learners need the proposal and deployment process to distinguish building permissionlessly from changing Bitcoin's consensus rules without broad adoption.</x:v>
+      </x:c>
+      <x:c r="F135" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G135" s="32" t="str">
+        <x:v>Review culture remains related but is not a direct prerequisite for permissionless access.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" s="32" t="str">
+        <x:v>dev.reproducible-builds</x:v>
+      </x:c>
+      <x:c r="B136" s="32" t="str">
+        <x:v>dev.bootstrappable-builds</x:v>
+      </x:c>
+      <x:c r="C136" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D136" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E136" s="32" t="str">
+        <x:v>Bootstrappable builds extend reproducible builds by reducing trust in the compiler and build-tool binaries used to produce the reproducible output.</x:v>
+      </x:c>
+      <x:c r="F136" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G136" s="32" t="str">
         <x:v>Keep this as a direct downstream edge; the node is not a duplicate alias for reproducible builds.</x:v>
       </x:c>
     </x:row>
@@ -13012,10 +13480,10 @@
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C134">
+    <x:dataValidation type="list" sqref="C12:C136">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D134">
+    <x:dataValidation type="list" sqref="D12:D136">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -15735,16 +16203,42 @@
         <x:v>Added as a downstream concept with reproducible builds as the only direct prerequisite; Guix is implementation context, not a separate node.</x:v>
       </x:c>
     </x:row>
+    <x:row r="114">
+      <x:c r="A114" s="32" t="str">
+        <x:v>decision.lightning-short-channel-id-slice</x:v>
+      </x:c>
+      <x:c r="B114" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C114" s="32" t="str">
+        <x:v>lightning.short-channel-id</x:v>
+      </x:c>
+      <x:c r="D114" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E114" s="32" t="str">
+        <x:v>Short Channel IDs are a distinct learner-facing identifier concept that connects Lightning channel funding outputs to routing gossip. They are not an API wrapper or a duplicate of the broader gossip protocol.</x:v>
+      </x:c>
+      <x:c r="F114" s="32" t="str">
+        <x:v>lightning.short-channel-id, lightning.payment-channels, lightning.gossip-protocol, protocol.block-height</x:v>
+      </x:c>
+      <x:c r="G114" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="H114" s="32" t="str">
+        <x:v>Added with channel funding and block height as direct prerequisites; announcement and query messages remain inside the gossip protocol node.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B113">
+    <x:dataValidation type="list" sqref="B12:B114">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D113">
+    <x:dataValidation type="list" sqref="D12:D114">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -15797,7 +16291,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.70756951389</x:v>
+        <x:v>46214.711002951386</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -15813,7 +16307,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -15821,7 +16315,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>131</x:v>
+        <x:v>139</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -15829,7 +16323,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>123</x:v>
+        <x:v>125</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -15845,7 +16339,7 @@
         <x:v>Existing Matches</x:v>
       </x:c>
       <x:c r="B11" s="22" t="n">
-        <x:v>23</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -15853,7 +16347,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>90</x:v>
+        <x:v>91</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: expand BIP concept coverage
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rb352f582a9df456f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R54d64153b63c4a14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Re4ee8fd36f414269"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rb367ef1668a948cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R38f9fbb929e44f6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R53a7bb54a7ff415b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R1b92fd7fbdc54703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rb8ae3d7b8f9649a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R3207da95a7a74335"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rf977123d94304df5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rebff86b58d2046dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R1b4ec97cde534f3e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -939,28 +939,28 @@
         <x:v>Enumerate the repository registry first, then group BIPs into consensus soft forks, signature encoding and serialization, script and output templates, wallet and payment standards, and peer/relay protocols. Treat BIPs as specification provenance rather than automatic one-to-one nodes.</x:v>
       </x:c>
       <x:c r="H20" s="32" t="str">
-        <x:v>Inventorying</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I20" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="J20" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K20" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L20" s="32" t="n">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="M20" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="N20" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="O20" s="32" t="str">
-        <x:v>Added during source expansion. Initial inventory covers the registry/process, consensus soft forks, signature encoding and serialization, script/output templates, wallet/payment standards, and peer/relay clusters. Implemented from this source in the current branch: protocol.strict-der-signatures, custody.deterministic-multisig-key-sorting, and protocol.generic-signed-messages.</x:v>
+        <x:v>Complete first-pass registry enumeration across process, consensus/deployment, signatures/serialization, script/output templates, wallet/payment standards, peer/relay protocols, and emerging application proposals. Implemented from this source: protocol.strict-der-signatures, custody.deterministic-multisig-key-sorting, protocol.generic-signed-messages, protocol.proof-of-payment, and protocol.pay-to-anchor. BIP 329 Wallet Labels merges into custody.output-labeling; BIP 431 TRUC confirms protocol.version-3-transaction-relay. Draft and closed proposals are retained as provenance, not treated as deployed consensus rules.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -10104,222 +10104,218 @@
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="32" t="str">
-        <x:v>lightning.commitment-transactions</x:v>
+        <x:v>protocol.proof-of-payment</x:v>
       </x:c>
       <x:c r="B143" s="32" t="str">
-        <x:v>Lightning Commitment Transactions</x:v>
+        <x:v>Proof of Payment</x:v>
       </x:c>
       <x:c r="C143" s="32" t="str">
-        <x:v>Extension Systems</x:v>
+        <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D143" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="E143" s="32" t="str">
-        <x:v>https://github.com/lightning/bolts/blob/master/03-transactions.md</x:v>
+        <x:v>https://github.com/bitcoin/bips/blob/master/bip-0120.mediawiki</x:v>
       </x:c>
       <x:c r="F143" s="32" t="str">
-        <x:v>BOLT 03 commitment transaction and output formats</x:v>
-      </x:c>
-      <x:c r="G143" s="32" t="str">
-        <x:v>lightning.commitment-transactions</x:v>
-      </x:c>
+        <x:v>BIP 120 Proof of Payment</x:v>
+      </x:c>
+      <x:c r="G143" s="32" t="str"/>
       <x:c r="H143" s="32" t="str">
-        <x:v>existing</x:v>
+        <x:v>new</x:v>
       </x:c>
       <x:c r="I143" s="32" t="str">
-        <x:v>BOLT 03 specifies the existing commitment-transaction concept and its channel-state outputs.</x:v>
+        <x:v>Proof of Payment is one wallet-authentication mechanism: generate a one-time transaction-shaped proof that demonstrates control of the credentials used in a previous payment.</x:v>
       </x:c>
       <x:c r="J143" s="32" t="str">
-        <x:v>lightning.payment-channels, protocol.timelocks</x:v>
+        <x:v>protocol.transaction-lifecycle, fundamentals.digital-signatures</x:v>
       </x:c>
       <x:c r="K143" s="32" t="str">
-        <x:v>lightning.payment-channels, protocol.timelocks</x:v>
+        <x:v>protocol.transaction-lifecycle</x:v>
       </x:c>
       <x:c r="L143" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+        <x:v>The transaction lifecycle already carries the signature-based authorization path, so adding digital signatures directly would duplicate a transitive prerequisite.</x:v>
       </x:c>
       <x:c r="M143" s="32" t="str">
-        <x:v>BOLT 3 transactions, commitment transaction</x:v>
+        <x:v>PoP, proof of payment protocol</x:v>
       </x:c>
       <x:c r="N143" s="32" t="str">
-        <x:v>lightning, channels, transactions</x:v>
+        <x:v>payments, wallets, signatures, authentication</x:v>
       </x:c>
       <x:c r="O143" s="32" t="str">
-        <x:v>80m</x:v>
+        <x:v>35m</x:v>
       </x:c>
       <x:c r="P143" s="32" t="str">
-        <x:v>high</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="Q143" s="32" t="str">
-        <x:v>Existing node confirmed after inspecting BOLT 03.</x:v>
+        <x:v>Add as a historical/application concept; BIP 120 is closed and must not be represented as deployed consensus behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="32" t="str">
-        <x:v>lightning.force-closures</x:v>
+        <x:v>custody.output-labeling</x:v>
       </x:c>
       <x:c r="B144" s="32" t="str">
-        <x:v>Lightning Force Closures</x:v>
+        <x:v>Wallet Labels Export Format</x:v>
       </x:c>
       <x:c r="C144" s="32" t="str">
-        <x:v>Extension Systems</x:v>
+        <x:v>Wallets</x:v>
       </x:c>
       <x:c r="D144" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="E144" s="32" t="str">
-        <x:v>https://github.com/lightning/bolts/blob/master/05-onchain.md</x:v>
+        <x:v>https://github.com/bitcoin/bips/blob/master/bip-0329.mediawiki</x:v>
       </x:c>
       <x:c r="F144" s="32" t="str">
-        <x:v>BOLT 05 on-chain transaction handling</x:v>
+        <x:v>BIP 329 Wallet Labels Export Format</x:v>
       </x:c>
       <x:c r="G144" s="32" t="str">
-        <x:v>lightning.force-closures</x:v>
+        <x:v>custody.output-labeling</x:v>
       </x:c>
       <x:c r="H144" s="32" t="str">
-        <x:v>existing</x:v>
+        <x:v>merge</x:v>
       </x:c>
       <x:c r="I144" s="32" t="str">
-        <x:v>BOLT 05 specifies the existing unilateral and on-chain close-handling concept.</x:v>
+        <x:v>BIP 329 specifies a wallet metadata interchange format, which is a serialization of the existing labeling practice rather than a separate learner-facing concept.</x:v>
       </x:c>
       <x:c r="J144" s="32" t="str">
-        <x:v>lightning.commitment-transactions, lightning.watchtowers</x:v>
+        <x:v>custody.output-labeling</x:v>
       </x:c>
       <x:c r="K144" s="32" t="str">
-        <x:v>lightning.commitment-transactions, lightning.watchtowers</x:v>
+        <x:v>custody.output-labeling</x:v>
       </x:c>
       <x:c r="L144" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+        <x:v>Reuse the existing labeling concept; the export format is a downstream interoperability detail.</x:v>
       </x:c>
       <x:c r="M144" s="32" t="str">
-        <x:v>unilateral close, BOLT 5 on-chain handling</x:v>
+        <x:v>BIP 329, wallet labels export</x:v>
       </x:c>
       <x:c r="N144" s="32" t="str">
-        <x:v>lightning, channels, on-chain</x:v>
+        <x:v>wallets, metadata, interoperability</x:v>
       </x:c>
       <x:c r="O144" s="32" t="str">
-        <x:v>70m</x:v>
+        <x:v>20m</x:v>
       </x:c>
       <x:c r="P144" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q144" s="32" t="str">
-        <x:v>Existing node confirmed after inspecting BOLT 05.</x:v>
+        <x:v>Merge into custody.output-labeling and preserve BIP 329 as a resource/alias; the BIP remains Draft.</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="32" t="str">
-        <x:v>lightning.revocation-penalty-keys</x:v>
+        <x:v>protocol.pay-to-anchor</x:v>
       </x:c>
       <x:c r="B145" s="32" t="str">
-        <x:v>Revocation and Penalty Keys</x:v>
+        <x:v>Pay to Anchor</x:v>
       </x:c>
       <x:c r="C145" s="32" t="str">
-        <x:v>Extension Systems</x:v>
+        <x:v>Protocol &amp; Consensus</x:v>
       </x:c>
       <x:c r="D145" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="E145" s="32" t="str">
-        <x:v>https://github.com/lightning/bolts/blob/master/05-onchain.md</x:v>
+        <x:v>https://github.com/bitcoin/bips/blob/master/bip-0433.mediawiki</x:v>
       </x:c>
       <x:c r="F145" s="32" t="str">
-        <x:v>BOLT 05 revoked transaction close handling</x:v>
-      </x:c>
-      <x:c r="G145" s="32" t="str">
-        <x:v>lightning.revocation-penalty-keys</x:v>
-      </x:c>
+        <x:v>BIP 433 Pay to Anchor</x:v>
+      </x:c>
+      <x:c r="G145" s="32" t="str"/>
       <x:c r="H145" s="32" t="str">
-        <x:v>existing</x:v>
+        <x:v>new</x:v>
       </x:c>
       <x:c r="I145" s="32" t="str">
-        <x:v>BOLT 05 specifies the existing revocation and penalty mechanism for outdated commitment states.</x:v>
+        <x:v>Pay to Anchor is one distinct keyless output pattern that leaves a compact hook for later child-based fee bumping.</x:v>
       </x:c>
       <x:c r="J145" s="32" t="str">
-        <x:v>lightning.commitment-transactions</x:v>
+        <x:v>protocol.ephemeral-anchors</x:v>
       </x:c>
       <x:c r="K145" s="32" t="str">
-        <x:v>lightning.commitment-transactions</x:v>
+        <x:v>protocol.ephemeral-anchors</x:v>
       </x:c>
       <x:c r="L145" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+        <x:v>Ephemeral anchors provide the prior anchor-output and package-relay context; TRUC is related anti-pinning context but is not inherently required by P2A.</x:v>
       </x:c>
       <x:c r="M145" s="32" t="str">
-        <x:v>penalty transactions, revoked transaction handling</x:v>
+        <x:v>P2A, pay-to-anchor output</x:v>
       </x:c>
       <x:c r="N145" s="32" t="str">
-        <x:v>lightning, security, channels</x:v>
+        <x:v>outputs, fee-bumping, mempool, relay</x:v>
       </x:c>
       <x:c r="O145" s="32" t="str">
-        <x:v>85m</x:v>
+        <x:v>35m</x:v>
       </x:c>
       <x:c r="P145" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q145" s="32" t="str">
-        <x:v>Existing node confirmed after inspecting BOLT 05.</x:v>
+        <x:v>Add as a draft protocol/application concept; do not imply that the BIP's draft status equals consensus deployment.</x:v>
       </x:c>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="32" t="str">
-        <x:v>lightning.gossip-protocol</x:v>
+        <x:v>protocol.version-3-transaction-relay</x:v>
       </x:c>
       <x:c r="B146" s="32" t="str">
-        <x:v>Lightning Gossip Protocol</x:v>
+        <x:v>Version 3 Transaction Relay</x:v>
       </x:c>
       <x:c r="C146" s="32" t="str">
-        <x:v>Extension Systems</x:v>
+        <x:v>Network, Relay &amp; Client Sync</x:v>
       </x:c>
       <x:c r="D146" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="E146" s="32" t="str">
-        <x:v>https://github.com/lightning/bolts/blob/master/07-routing-gossip.md</x:v>
+        <x:v>https://github.com/bitcoin/bips/blob/master/bip-0431.mediawiki</x:v>
       </x:c>
       <x:c r="F146" s="32" t="str">
-        <x:v>BOLT 07 node and channel discovery</x:v>
+        <x:v>BIP 431 topology restrictions for pinning</x:v>
       </x:c>
       <x:c r="G146" s="32" t="str">
-        <x:v>lightning.gossip-protocol</x:v>
+        <x:v>protocol.version-3-transaction-relay</x:v>
       </x:c>
       <x:c r="H146" s="32" t="str">
         <x:v>existing</x:v>
       </x:c>
       <x:c r="I146" s="32" t="str">
-        <x:v>BOLT 07 specifies the existing gossip concept for node announcements, channel announcements, and routing updates.</x:v>
+        <x:v>BIP 431 specifies the existing TRUC/v3 relay policy concept.</x:v>
       </x:c>
       <x:c r="J146" s="32" t="str">
-        <x:v>lightning.routing, dev.p2p-messages</x:v>
+        <x:v>protocol.transaction-pinning</x:v>
       </x:c>
       <x:c r="K146" s="32" t="str">
-        <x:v>lightning.routing, dev.p2p-messages</x:v>
+        <x:v>protocol.transaction-pinning</x:v>
       </x:c>
       <x:c r="L146" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M146" s="32" t="str">
-        <x:v>channel announcements, node announcements, routing gossip</x:v>
+        <x:v>TRUC, v3 relay, topologically restricted until confirmation</x:v>
       </x:c>
       <x:c r="N146" s="32" t="str">
-        <x:v>lightning, routing, discovery</x:v>
+        <x:v>mempool, relay, pinning</x:v>
       </x:c>
       <x:c r="O146" s="32" t="str">
-        <x:v>85m</x:v>
+        <x:v>55m</x:v>
       </x:c>
       <x:c r="P146" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q146" s="32" t="str">
-        <x:v>The message family is kept together; individual announcement messages are implementation-level protocol surfaces, not separate learner nodes.</x:v>
+        <x:v>Existing node confirmed; BIP 431 remains policy/proposal provenance rather than consensus behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="32" t="str">
-        <x:v>lightning.channel-fee-policies</x:v>
+        <x:v>lightning.commitment-transactions</x:v>
       </x:c>
       <x:c r="B147" s="32" t="str">
-        <x:v>Lightning Channel Fee Policies</x:v>
+        <x:v>Lightning Commitment Transactions</x:v>
       </x:c>
       <x:c r="C147" s="32" t="str">
         <x:v>Extension Systems</x:v>
@@ -10328,51 +10324,51 @@
         <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="E147" s="32" t="str">
-        <x:v>https://github.com/lightning/bolts/blob/master/07-routing-gossip.md#the-channel_update-message</x:v>
+        <x:v>https://github.com/lightning/bolts/blob/master/03-transactions.md</x:v>
       </x:c>
       <x:c r="F147" s="32" t="str">
-        <x:v>BOLT 07 channel_update fee and HTLC policy fields</x:v>
+        <x:v>BOLT 03 commitment transaction and output formats</x:v>
       </x:c>
       <x:c r="G147" s="32" t="str">
-        <x:v>lightning.channel-fee-policies</x:v>
+        <x:v>lightning.commitment-transactions</x:v>
       </x:c>
       <x:c r="H147" s="32" t="str">
         <x:v>existing</x:v>
       </x:c>
       <x:c r="I147" s="32" t="str">
-        <x:v>BOLT 07 specifies the existing learner-facing concept of channel forwarding fees and HTLC policy limits.</x:v>
+        <x:v>BOLT 03 specifies the existing commitment-transaction concept and its channel-state outputs.</x:v>
       </x:c>
       <x:c r="J147" s="32" t="str">
-        <x:v>lightning.liquidity</x:v>
+        <x:v>lightning.payment-channels, protocol.timelocks</x:v>
       </x:c>
       <x:c r="K147" s="32" t="str">
-        <x:v>lightning.liquidity</x:v>
+        <x:v>lightning.payment-channels, protocol.timelocks</x:v>
       </x:c>
       <x:c r="L147" s="32" t="str">
-        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
       </x:c>
       <x:c r="M147" s="32" t="str">
-        <x:v>channel_update fees, routing fee policy</x:v>
+        <x:v>BOLT 3 transactions, commitment transaction</x:v>
       </x:c>
       <x:c r="N147" s="32" t="str">
-        <x:v>lightning, routing, fees</x:v>
+        <x:v>lightning, channels, transactions</x:v>
       </x:c>
       <x:c r="O147" s="32" t="str">
-        <x:v>70m</x:v>
+        <x:v>80m</x:v>
       </x:c>
       <x:c r="P147" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q147" s="32" t="str">
-        <x:v>Existing node confirmed; channel_update itself remains a protocol message rather than a separate node.</x:v>
+        <x:v>Existing node confirmed after inspecting BOLT 03.</x:v>
       </x:c>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="32" t="str">
-        <x:v>lightning.short-channel-id</x:v>
+        <x:v>lightning.force-closures</x:v>
       </x:c>
       <x:c r="B148" s="32" t="str">
-        <x:v>Short Channel IDs</x:v>
+        <x:v>Lightning Force Closures</x:v>
       </x:c>
       <x:c r="C148" s="32" t="str">
         <x:v>Extension Systems</x:v>
@@ -10381,49 +10377,51 @@
         <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="E148" s="32" t="str">
-        <x:v>https://github.com/lightning/bolts/blob/master/07-routing-gossip.md#definition-of-short_channel_id</x:v>
+        <x:v>https://github.com/lightning/bolts/blob/master/05-onchain.md</x:v>
       </x:c>
       <x:c r="F148" s="32" t="str">
-        <x:v>BOLT 07 short_channel_id definition</x:v>
-      </x:c>
-      <x:c r="G148" s="32" t="str"/>
+        <x:v>BOLT 05 on-chain transaction handling</x:v>
+      </x:c>
+      <x:c r="G148" s="32" t="str">
+        <x:v>lightning.force-closures</x:v>
+      </x:c>
       <x:c r="H148" s="32" t="str">
-        <x:v>new</x:v>
+        <x:v>existing</x:v>
       </x:c>
       <x:c r="I148" s="32" t="str">
-        <x:v>A Short Channel ID is one precise identifier encoding a channel funding output as block height, transaction index, and output index; it is a prerequisite for interpreting Lightning gossip references.</x:v>
+        <x:v>BOLT 05 specifies the existing unilateral and on-chain close-handling concept.</x:v>
       </x:c>
       <x:c r="J148" s="32" t="str">
-        <x:v>lightning.payment-channels, protocol.block-height</x:v>
+        <x:v>lightning.commitment-transactions, lightning.watchtowers</x:v>
       </x:c>
       <x:c r="K148" s="32" t="str">
-        <x:v>lightning.payment-channels, protocol.block-height</x:v>
+        <x:v>lightning.commitment-transactions, lightning.watchtowers</x:v>
       </x:c>
       <x:c r="L148" s="32" t="str">
-        <x:v>Learners need the channel funding context and the block-height component before the compact on-chain identifier is meaningful.</x:v>
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
       </x:c>
       <x:c r="M148" s="32" t="str">
-        <x:v>short_channel_id, SCID, short channel identifier</x:v>
+        <x:v>unilateral close, BOLT 5 on-chain handling</x:v>
       </x:c>
       <x:c r="N148" s="32" t="str">
-        <x:v>lightning, channels, gossip, identifiers</x:v>
+        <x:v>lightning, channels, on-chain</x:v>
       </x:c>
       <x:c r="O148" s="32" t="str">
-        <x:v>25m</x:v>
+        <x:v>70m</x:v>
       </x:c>
       <x:c r="P148" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q148" s="32" t="str">
-        <x:v>Add as the only new node from the complete BOLT 07 pass; announcement and query messages remain part of gossip.</x:v>
+        <x:v>Existing node confirmed after inspecting BOLT 05.</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="32" t="str">
-        <x:v>lightning.invoices</x:v>
+        <x:v>lightning.revocation-penalty-keys</x:v>
       </x:c>
       <x:c r="B149" s="32" t="str">
-        <x:v>Invoices and Payment Requests</x:v>
+        <x:v>Revocation and Penalty Keys</x:v>
       </x:c>
       <x:c r="C149" s="32" t="str">
         <x:v>Extension Systems</x:v>
@@ -10432,51 +10430,51 @@
         <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="E149" s="32" t="str">
-        <x:v>https://github.com/lightning/bolts/blob/master/11-payment-encoding.md</x:v>
+        <x:v>https://github.com/lightning/bolts/blob/master/05-onchain.md</x:v>
       </x:c>
       <x:c r="F149" s="32" t="str">
-        <x:v>BOLT 11 invoice protocol</x:v>
+        <x:v>BOLT 05 revoked transaction close handling</x:v>
       </x:c>
       <x:c r="G149" s="32" t="str">
-        <x:v>lightning.invoices</x:v>
+        <x:v>lightning.revocation-penalty-keys</x:v>
       </x:c>
       <x:c r="H149" s="32" t="str">
         <x:v>existing</x:v>
       </x:c>
       <x:c r="I149" s="32" t="str">
-        <x:v>BOLT 11 specifies the existing invoice and payment-request concept.</x:v>
+        <x:v>BOLT 05 specifies the existing revocation and penalty mechanism for outdated commitment states.</x:v>
       </x:c>
       <x:c r="J149" s="32" t="str">
-        <x:v>lightning.routing</x:v>
+        <x:v>lightning.commitment-transactions</x:v>
       </x:c>
       <x:c r="K149" s="32" t="str">
-        <x:v>lightning.routing</x:v>
+        <x:v>lightning.commitment-transactions</x:v>
       </x:c>
       <x:c r="L149" s="32" t="str">
         <x:v>Reuse the existing node's direct prerequisite.</x:v>
       </x:c>
       <x:c r="M149" s="32" t="str">
-        <x:v>BOLT 11 invoices, payment requests</x:v>
+        <x:v>penalty transactions, revoked transaction handling</x:v>
       </x:c>
       <x:c r="N149" s="32" t="str">
-        <x:v>lightning, payments</x:v>
+        <x:v>lightning, security, channels</x:v>
       </x:c>
       <x:c r="O149" s="32" t="str">
-        <x:v>50m</x:v>
+        <x:v>85m</x:v>
       </x:c>
       <x:c r="P149" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q149" s="32" t="str">
-        <x:v>Existing node confirmed after inspecting BOLT 11 encoding and payer/payee flow.</x:v>
+        <x:v>Existing node confirmed after inspecting BOLT 05.</x:v>
       </x:c>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="32" t="str">
-        <x:v>lightning.bolt12-offers</x:v>
+        <x:v>lightning.gossip-protocol</x:v>
       </x:c>
       <x:c r="B150" s="32" t="str">
-        <x:v>BOLT12 Offers</x:v>
+        <x:v>Lightning Gossip Protocol</x:v>
       </x:c>
       <x:c r="C150" s="32" t="str">
         <x:v>Extension Systems</x:v>
@@ -10485,42 +10483,252 @@
         <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="E150" s="32" t="str">
-        <x:v>https://github.com/lightning/bolts/blob/master/12-offer-encoding.md</x:v>
+        <x:v>https://github.com/lightning/bolts/blob/master/07-routing-gossip.md</x:v>
       </x:c>
       <x:c r="F150" s="32" t="str">
-        <x:v>BOLT 12 offers, invoice requests, and invoices</x:v>
+        <x:v>BOLT 07 node and channel discovery</x:v>
       </x:c>
       <x:c r="G150" s="32" t="str">
-        <x:v>lightning.bolt12-offers</x:v>
+        <x:v>lightning.gossip-protocol</x:v>
       </x:c>
       <x:c r="H150" s="32" t="str">
         <x:v>existing</x:v>
       </x:c>
       <x:c r="I150" s="32" t="str">
-        <x:v>BOLT 12 specifies the existing reusable offers and invoice-request protocol concept.</x:v>
+        <x:v>BOLT 07 specifies the existing gossip concept for node announcements, channel announcements, and routing updates.</x:v>
       </x:c>
       <x:c r="J150" s="32" t="str">
-        <x:v>lightning.invoices, lightning.route-blinding</x:v>
+        <x:v>lightning.routing, dev.p2p-messages</x:v>
       </x:c>
       <x:c r="K150" s="32" t="str">
-        <x:v>lightning.invoices, lightning.route-blinding</x:v>
+        <x:v>lightning.routing, dev.p2p-messages</x:v>
       </x:c>
       <x:c r="L150" s="32" t="str">
         <x:v>Reuse the existing node's direct prerequisites.</x:v>
       </x:c>
       <x:c r="M150" s="32" t="str">
-        <x:v>offers, invoice requests, BOLT 12</x:v>
+        <x:v>channel announcements, node announcements, routing gossip</x:v>
       </x:c>
       <x:c r="N150" s="32" t="str">
-        <x:v>lightning, payments, privacy</x:v>
+        <x:v>lightning, routing, discovery</x:v>
       </x:c>
       <x:c r="O150" s="32" t="str">
-        <x:v>75m</x:v>
+        <x:v>85m</x:v>
       </x:c>
       <x:c r="P150" s="32" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="Q150" s="32" t="str">
+        <x:v>The message family is kept together; individual announcement messages are implementation-level protocol surfaces, not separate learner nodes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" s="32" t="str">
+        <x:v>lightning.channel-fee-policies</x:v>
+      </x:c>
+      <x:c r="B151" s="32" t="str">
+        <x:v>Lightning Channel Fee Policies</x:v>
+      </x:c>
+      <x:c r="C151" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D151" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E151" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/07-routing-gossip.md#the-channel_update-message</x:v>
+      </x:c>
+      <x:c r="F151" s="32" t="str">
+        <x:v>BOLT 07 channel_update fee and HTLC policy fields</x:v>
+      </x:c>
+      <x:c r="G151" s="32" t="str">
+        <x:v>lightning.channel-fee-policies</x:v>
+      </x:c>
+      <x:c r="H151" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I151" s="32" t="str">
+        <x:v>BOLT 07 specifies the existing learner-facing concept of channel forwarding fees and HTLC policy limits.</x:v>
+      </x:c>
+      <x:c r="J151" s="32" t="str">
+        <x:v>lightning.liquidity</x:v>
+      </x:c>
+      <x:c r="K151" s="32" t="str">
+        <x:v>lightning.liquidity</x:v>
+      </x:c>
+      <x:c r="L151" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M151" s="32" t="str">
+        <x:v>channel_update fees, routing fee policy</x:v>
+      </x:c>
+      <x:c r="N151" s="32" t="str">
+        <x:v>lightning, routing, fees</x:v>
+      </x:c>
+      <x:c r="O151" s="32" t="str">
+        <x:v>70m</x:v>
+      </x:c>
+      <x:c r="P151" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q151" s="32" t="str">
+        <x:v>Existing node confirmed; channel_update itself remains a protocol message rather than a separate node.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" s="32" t="str">
+        <x:v>lightning.short-channel-id</x:v>
+      </x:c>
+      <x:c r="B152" s="32" t="str">
+        <x:v>Short Channel IDs</x:v>
+      </x:c>
+      <x:c r="C152" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D152" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E152" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/07-routing-gossip.md#definition-of-short_channel_id</x:v>
+      </x:c>
+      <x:c r="F152" s="32" t="str">
+        <x:v>BOLT 07 short_channel_id definition</x:v>
+      </x:c>
+      <x:c r="G152" s="32" t="str"/>
+      <x:c r="H152" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I152" s="32" t="str">
+        <x:v>A Short Channel ID is one precise identifier encoding a channel funding output as block height, transaction index, and output index; it is a prerequisite for interpreting Lightning gossip references.</x:v>
+      </x:c>
+      <x:c r="J152" s="32" t="str">
+        <x:v>lightning.payment-channels, protocol.block-height</x:v>
+      </x:c>
+      <x:c r="K152" s="32" t="str">
+        <x:v>lightning.payment-channels, protocol.block-height</x:v>
+      </x:c>
+      <x:c r="L152" s="32" t="str">
+        <x:v>Learners need the channel funding context and the block-height component before the compact on-chain identifier is meaningful.</x:v>
+      </x:c>
+      <x:c r="M152" s="32" t="str">
+        <x:v>short_channel_id, SCID, short channel identifier</x:v>
+      </x:c>
+      <x:c r="N152" s="32" t="str">
+        <x:v>lightning, channels, gossip, identifiers</x:v>
+      </x:c>
+      <x:c r="O152" s="32" t="str">
+        <x:v>25m</x:v>
+      </x:c>
+      <x:c r="P152" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q152" s="32" t="str">
+        <x:v>Add as the only new node from the complete BOLT 07 pass; announcement and query messages remain part of gossip.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" s="32" t="str">
+        <x:v>lightning.invoices</x:v>
+      </x:c>
+      <x:c r="B153" s="32" t="str">
+        <x:v>Invoices and Payment Requests</x:v>
+      </x:c>
+      <x:c r="C153" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D153" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E153" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/11-payment-encoding.md</x:v>
+      </x:c>
+      <x:c r="F153" s="32" t="str">
+        <x:v>BOLT 11 invoice protocol</x:v>
+      </x:c>
+      <x:c r="G153" s="32" t="str">
+        <x:v>lightning.invoices</x:v>
+      </x:c>
+      <x:c r="H153" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I153" s="32" t="str">
+        <x:v>BOLT 11 specifies the existing invoice and payment-request concept.</x:v>
+      </x:c>
+      <x:c r="J153" s="32" t="str">
+        <x:v>lightning.routing</x:v>
+      </x:c>
+      <x:c r="K153" s="32" t="str">
+        <x:v>lightning.routing</x:v>
+      </x:c>
+      <x:c r="L153" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M153" s="32" t="str">
+        <x:v>BOLT 11 invoices, payment requests</x:v>
+      </x:c>
+      <x:c r="N153" s="32" t="str">
+        <x:v>lightning, payments</x:v>
+      </x:c>
+      <x:c r="O153" s="32" t="str">
+        <x:v>50m</x:v>
+      </x:c>
+      <x:c r="P153" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q153" s="32" t="str">
+        <x:v>Existing node confirmed after inspecting BOLT 11 encoding and payer/payee flow.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" s="32" t="str">
+        <x:v>lightning.bolt12-offers</x:v>
+      </x:c>
+      <x:c r="B154" s="32" t="str">
+        <x:v>BOLT12 Offers</x:v>
+      </x:c>
+      <x:c r="C154" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D154" s="32" t="str">
+        <x:v>source.lightning-bolts</x:v>
+      </x:c>
+      <x:c r="E154" s="32" t="str">
+        <x:v>https://github.com/lightning/bolts/blob/master/12-offer-encoding.md</x:v>
+      </x:c>
+      <x:c r="F154" s="32" t="str">
+        <x:v>BOLT 12 offers, invoice requests, and invoices</x:v>
+      </x:c>
+      <x:c r="G154" s="32" t="str">
+        <x:v>lightning.bolt12-offers</x:v>
+      </x:c>
+      <x:c r="H154" s="32" t="str">
+        <x:v>existing</x:v>
+      </x:c>
+      <x:c r="I154" s="32" t="str">
+        <x:v>BOLT 12 specifies the existing reusable offers and invoice-request protocol concept.</x:v>
+      </x:c>
+      <x:c r="J154" s="32" t="str">
+        <x:v>lightning.invoices, lightning.route-blinding</x:v>
+      </x:c>
+      <x:c r="K154" s="32" t="str">
+        <x:v>lightning.invoices, lightning.route-blinding</x:v>
+      </x:c>
+      <x:c r="L154" s="32" t="str">
+        <x:v>Reuse the existing node's direct prerequisites.</x:v>
+      </x:c>
+      <x:c r="M154" s="32" t="str">
+        <x:v>offers, invoice requests, BOLT 12</x:v>
+      </x:c>
+      <x:c r="N154" s="32" t="str">
+        <x:v>lightning, payments, privacy</x:v>
+      </x:c>
+      <x:c r="O154" s="32" t="str">
+        <x:v>75m</x:v>
+      </x:c>
+      <x:c r="P154" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q154" s="32" t="str">
         <x:v>Existing node confirmed; payment proofs and TLV fields remain internal parts of the BOLT 12 flow rather than standalone learner nodes.</x:v>
       </x:c>
     </x:row>
@@ -10530,10 +10738,10 @@
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H150">
+    <x:dataValidation type="list" sqref="H12:H154">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P150">
+    <x:dataValidation type="list" sqref="P12:P154">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -13474,16 +13682,62 @@
         <x:v>Keep this as a direct downstream edge; the node is not a duplicate alias for reproducible builds.</x:v>
       </x:c>
     </x:row>
+    <x:row r="137">
+      <x:c r="A137" s="32" t="str">
+        <x:v>protocol.transaction-lifecycle</x:v>
+      </x:c>
+      <x:c r="B137" s="32" t="str">
+        <x:v>protocol.proof-of-payment</x:v>
+      </x:c>
+      <x:c r="C137" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D137" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E137" s="32" t="str">
+        <x:v>Proof of Payment refers to a prior payment and reconstructs a transaction-shaped proof, so learners need the transaction lifecycle first.</x:v>
+      </x:c>
+      <x:c r="F137" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="G137" s="32" t="str">
+        <x:v>Direct payment context; wallet UX and URI transport remain downstream or optional details.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" s="32" t="str">
+        <x:v>protocol.ephemeral-anchors</x:v>
+      </x:c>
+      <x:c r="B138" s="32" t="str">
+        <x:v>protocol.pay-to-anchor</x:v>
+      </x:c>
+      <x:c r="C138" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D138" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E138" s="32" t="str">
+        <x:v>Pay to Anchor is a keyless refinement of the anchor-output and package-relay fee-bumping pattern, so learners need that broader context first.</x:v>
+      </x:c>
+      <x:c r="F138" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="G138" s="32" t="str">
+        <x:v>BIP 431/TRUC is related anti-pinning context, not an inherent prerequisite.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C136">
+    <x:dataValidation type="list" sqref="C12:C138">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D136">
+    <x:dataValidation type="list" sqref="D12:D138">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -16229,16 +16483,94 @@
         <x:v>Added with channel funding and block height as direct prerequisites; announcement and query messages remain inside the gossip protocol node.</x:v>
       </x:c>
     </x:row>
+    <x:row r="115">
+      <x:c r="A115" s="32" t="str">
+        <x:v>decision.proof-of-payment-slice</x:v>
+      </x:c>
+      <x:c r="B115" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C115" s="32" t="str">
+        <x:v>protocol.proof-of-payment</x:v>
+      </x:c>
+      <x:c r="D115" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E115" s="32" t="str">
+        <x:v>Proof of Payment is a distinct wallet-authentication outcome: proving control of the credentials used in a prior payment. It is not a duplicate of generic signed messages because it binds proof to transaction inputs and a payment context.</x:v>
+      </x:c>
+      <x:c r="F115" s="32" t="str">
+        <x:v>protocol.proof-of-payment, protocol.generic-signed-messages, protocol.transaction-lifecycle, fundamentals.digital-signatures</x:v>
+      </x:c>
+      <x:c r="G115" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="H115" s="32" t="str">
+        <x:v>Added as a historical/application concept while retaining BIP 120's closed status in the resource context.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" s="32" t="str">
+        <x:v>decision.wallet-labels-bip329-merge</x:v>
+      </x:c>
+      <x:c r="B116" s="32" t="str">
+        <x:v>merge</x:v>
+      </x:c>
+      <x:c r="C116" s="32" t="str">
+        <x:v>custody.output-labeling</x:v>
+      </x:c>
+      <x:c r="D116" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E116" s="32" t="str">
+        <x:v>BIP 329 standardizes serialization and portability of wallet labels; it does not create a separate learner outcome from labeling UTXOs and transaction metadata.</x:v>
+      </x:c>
+      <x:c r="F116" s="32" t="str">
+        <x:v>custody.output-labeling</x:v>
+      </x:c>
+      <x:c r="G116" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="H116" s="32" t="str">
+        <x:v>Keep BIP 329 as an alias/resource on the existing labeling node if metadata is expanded later.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" s="32" t="str">
+        <x:v>decision.pay-to-anchor-slice</x:v>
+      </x:c>
+      <x:c r="B117" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C117" s="32" t="str">
+        <x:v>protocol.pay-to-anchor</x:v>
+      </x:c>
+      <x:c r="D117" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E117" s="32" t="str">
+        <x:v>Pay to Anchor is a distinct keyless output pattern for fee-bumping hooks, not a duplicate of generic anchor outputs or ephemeral-anchor package policy.</x:v>
+      </x:c>
+      <x:c r="F117" s="32" t="str">
+        <x:v>protocol.pay-to-anchor, protocol.ephemeral-anchors, protocol.version-3-transaction-relay</x:v>
+      </x:c>
+      <x:c r="G117" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="H117" s="32" t="str">
+        <x:v>Added as a draft protocol/application concept; TRUC remains related anti-pinning context without becoming a direct prerequisite.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B114">
+    <x:dataValidation type="list" sqref="B12:B117">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D114">
+    <x:dataValidation type="list" sqref="D12:D117">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -16291,7 +16623,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.711002951386</x:v>
+        <x:v>46214.71491829861</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -16307,7 +16639,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>49</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -16315,7 +16647,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>139</x:v>
+        <x:v>143</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -16323,7 +16655,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>125</x:v>
+        <x:v>127</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -16339,7 +16671,7 @@
         <x:v>Existing Matches</x:v>
       </x:c>
       <x:c r="B11" s="22" t="n">
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -16347,7 +16679,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>91</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
docs: close content source audit clusters
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R1b92fd7fbdc54703"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rb8ae3d7b8f9649a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R3207da95a7a74335"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rf977123d94304df5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rebff86b58d2046dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R1b4ec97cde534f3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Refec70ce97e84fc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R29dd44e70d354ea7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R799e27e8efe3406e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rf4e65593583f4e49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R7fff0be324064285"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rc640ed2eb32542c4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -657,16 +657,16 @@
         <x:v>Track 9 chapter-level rows first, with later splits for dense chapters 5, 7, 8, and 9.</x:v>
       </x:c>
       <x:c r="H14" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I14" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J14" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K14" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L14" s="32" t="n">
         <x:v>9</x:v>
@@ -678,7 +678,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="O14" s="32" t="str">
-        <x:v>Heavy overlap with existing philosophy nodes, but strong for bridge concepts like validation sovereignty, consensus vs policy, development review, permissionless development, pseudonymous development, miner decentralization, and selection cryptography. Implemented from this source in the current branch: fundamentals.validation-sovereignty, protocol.consensus-vs-policy, protocol.chain-split-risk, dev.review-culture, dev.permissionless-development, dev.pseudonymous-development, mining.miner-decentralization, and dev.selection-cryptography.</x:v>
+        <x:v>Complete nine-chapter pass. Dense chapters 5, 7, 8, and 9 were split conceptually and deduplicated against the graph. Implemented bridge concepts: fundamentals.validation-sovereignty, protocol.consensus-vs-policy, protocol.chain-split-risk, dev.review-culture, dev.permissionless-development, dev.pseudonymous-development, dev.bootstrappable-builds, mining.miner-decentralization, and dev.selection-cryptography. Funding, culture shock, scaling taxonomies, and historical incident examples remain contextual or existing coverage rather than standalone gaps.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -704,16 +704,16 @@
         <x:v>Track 14 chapter rows first, grouping chapters 4 to 12 as the primary extraction surface.</x:v>
       </x:c>
       <x:c r="H15" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I15" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J15" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K15" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L15" s="32" t="n">
         <x:v>14</x:v>
@@ -725,7 +725,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="O15" s="32" t="str">
-        <x:v>Already heavily reused in current nodes, so chapter titles are containers. Best current value is prerequisite ladders and bridge concepts. Implemented from this source in the current branch: protocol.light-client-trust-model, ops.full-node-vs-lightweight-wallet, custody.coin-selection, protocol.change-outputs, protocol.bech32m-addresses, protocol.script-execution-stack, dev.extended-keys, protocol.witness-structure, protocol.partial-merkle-proofs, protocol.pay-to-contract, extension.single-use-seals, and extension.client-side-validation.</x:v>
+        <x:v>Complete 14-chapter outline pass. Chapter titles were treated as containers, then prerequisite ladders and bridge concepts were normalized against the existing graph. Implemented missing bridges: protocol.light-client-trust-model, ops.full-node-vs-lightweight-wallet, custody.coin-selection, protocol.change-outputs, protocol.bech32m-addresses, protocol.script-execution-stack, dev.extended-keys, protocol.witness-structure, protocol.partial-merkle-proofs, protocol.pay-to-contract, extension.single-use-seals, and extension.client-side-validation.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -751,16 +751,16 @@
         <x:v>Track the 12 module pages plus shared assets once per source.</x:v>
       </x:c>
       <x:c r="H16" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I16" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J16" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K16" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L16" s="32" t="n">
         <x:v>12</x:v>
@@ -772,7 +772,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="O16" s="32" t="str">
-        <x:v>Best current source for missing Taproot bridge concepts such as tagged hashes, taptweak, key-path spends, tapleaf inclusion proofs, control blocks, Huffman-optimized TapTrees, and concrete policy case studies like degrading multisig. Implemented from this source in the current branch: protocol.tagged-hashes, protocol.taptweak, protocol.taproot-key-path-spends, protocol.taptree, protocol.tapleaf-inclusion-proofs, protocol.taproot-control-blocks, protocol.huffman-optimized-taptrees, and custody.degrading-multisig.</x:v>
+        <x:v>Complete 12-module pass, including preparation/math, Schnorr/MuSig, Taproot, Tapscript, TapTree, Huffman construction, and the degrading-multisig case study. Implemented bridge concepts: protocol.tagged-hashes, protocol.taptweak, protocol.taproot-key-path-spends, protocol.taptree, protocol.tapleaf-inclusion-proofs, protocol.taproot-control-blocks, protocol.huffman-optimized-taptrees, and custody.degrading-multisig.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -889,7 +889,7 @@
         <x:v>Canonical Lightning wire protocol, transport, channel, transaction, routing, discovery, feature-negotiation, invoice, and offer specifications.</x:v>
       </x:c>
       <x:c r="G19" s="32" t="str">
-        <x:v>Track each BOLT document as an enumeration cluster, starting with the index and BOLTs 01, 02, 04, 08, 09, and 10. Extract only atomic mechanisms and deduplicate against existing Lightning nodes before proposing additions.</x:v>
+        <x:v>Track every current BOLT document as an enumeration cluster. Extract only atomic mechanisms and deduplicate against existing Lightning nodes before proposing additions.</x:v>
       </x:c>
       <x:c r="H19" s="32" t="str">
         <x:v>Complete</x:v>
@@ -986,28 +986,28 @@
         <x:v>Enumerate the FAQ, REST API, WebSocket API, and self-hosting/repository clusters first. Use Bitcoin Core documentation as the canonical authority for consensus and policy semantics, then retain Mempool.space-specific observability concepts only when they survive deduplication.</x:v>
       </x:c>
       <x:c r="H21" s="32" t="str">
-        <x:v>Inventorying</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I21" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="J21" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K21" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L21" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="M21" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N21" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O21" s="32" t="str">
-        <x:v>Added during source expansion. Initial clusters cover FAQ/mempool behavior, REST API, WebSocket/live events, and self-hosting. Implemented from this source in the current branch: ops.mempool-purging, with Bitcoin Core policy and RPC documentation used as canonical supporting sources.</x:v>
+        <x:v>Complete FAQ/mempool, REST API, WebSocket/live-events, and self-hosting pass. ops.mempool-purging is the only learner-facing concept added from this source; explorer UI, REST/WebSocket endpoints, and self-hosting are recorded as implementation/product surfaces rather than Bitcoin graph nodes. Bitcoin Core policy and RPC documentation remain canonical for protocol semantics.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -3101,10 +3101,10 @@
         <x:v>Track the eight top-level guide sections first, then split dense sections like Transactions, Contracts, Wallets, and P2P Network when they expose concept gaps not already covered by existing nodes.</x:v>
       </x:c>
       <x:c r="H66" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I66" s="32" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="J66" s="32" t="str">
         <x:v>Queue exhausted</x:v>
@@ -3122,7 +3122,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="O66" s="32" t="str">
-        <x:v>Added after the current audited source queue was exhausted. The first pass across the top-level sections surfaced four clean candidates: protocol.bitcoin-uri-bip21 from Payment Processing, dev.hardened-keys from Wallets, protocol.escrow-and-arbitration from Contracts, and mining.pool-shares from Pool Mining. A follow-up Wallet Files pass surfaced dev.wallet-import-format-wif as another clean wallet-standard slice. The implemented winners are now protocol.bitcoin-uri-bip21, dev.hardened-keys, protocol.escrow-and-arbitration, dev.wallet-import-format-wif, and mining.pool-shares because they land as missing standards, key-derivation, contract-pattern, key-serialization, and pooled-mining accounting bridges with clean direct parents. The current tracked top-level-plus-Wallet-Files queue is exhausted for this pass, though future deeper section splits may still surface more concepts.</x:v>
+        <x:v>Complete first pass across the eight top-level guide sections plus the Wallet Files split. Implemented missing standards and bridges: protocol.bitcoin-uri-bip21, dev.hardened-keys, protocol.escrow-and-arbitration, dev.wallet-import-format-wif, and mining.pool-shares. Remaining dense subsections are represented by existing graph coverage or deferred as future deep dives rather than falsely treated as unreviewed source families.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -3148,16 +3148,16 @@
         <x:v>Track the JSON-RPC interface security section, bitcoin.conf reference, and implementation configuration paths as one operator-security cluster before splitting distinct access-control or privacy concepts.</x:v>
       </x:c>
       <x:c r="H67" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I67" s="32" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="J67" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K67" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L67" s="32" t="n">
         <x:v>3</x:v>
@@ -3169,7 +3169,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O67" s="32" t="str">
-        <x:v>Added after the audited queue surfaced a distinct RPC control-plane security gap. The first inspected cluster covers credentials, rpcbind/rpcallowip exposure, and the implementation path that applies these settings.</x:v>
+        <x:v>Complete operator-security cluster. Inspected JSON-RPC-interface.md, bitcoin-conf.md, and init.md for cookie/rpcauth credentials, rpcbind/rpcallowip exposure, and the configuration path that applies these settings. The distinct learner concept is security.bitcoin-core-rpc-access; individual RPC options remain implementation details.</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -3195,16 +3195,16 @@
         <x:v>Track the current submitpackage RPC reference, package-policy specification, and the 26.0 release note that introduced the RPC as one package-admission cluster; keep network package relay and cluster-mempool as deduplicated neighboring concepts.</x:v>
       </x:c>
       <x:c r="H68" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I68" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J68" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K68" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L68" s="32" t="n">
         <x:v>3</x:v>
@@ -3216,7 +3216,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="O68" s="32" t="str">
-        <x:v>Added after the RPC-security slice. The inspected pages establish submitpackage as a local package-admission mechanism and package RBF as a distinct replacement rule, separate from testmempoolaccept preflight, network package relay, and cluster-mempool internals.</x:v>
+        <x:v>Complete package-admission cluster. submitpackage is retained as a developer workflow and package RBF as a distinct replacement rule; testmempoolaccept, package relay, and cluster-mempool remain neighboring concepts rather than duplicated prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -3242,16 +3242,16 @@
         <x:v>Track the getmempoolcluster and getmempoolfeeratediagram RPC references, cluster-limit policy, Bitcoin Core 31.0 release notes, mempool terminology, and implementation paths as one cluster-mempool slice; keep concrete RPC workflows merged into the higher-level concepts.</x:v>
       </x:c>
       <x:c r="H69" s="32" t="str">
-        <x:v>In review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="I69" s="32" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="J69" s="32" t="str">
-        <x:v>Raw extraction</x:v>
+        <x:v>Normalized</x:v>
       </x:c>
       <x:c r="K69" s="32" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L69" s="32" t="n">
         <x:v>5</x:v>
@@ -3263,7 +3263,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="O69" s="32" t="str">
-        <x:v>Added after the package-RBF slice. The inspected documentation exposes two RPC implementation surfaces, both merged into protocol.cluster-mempool, plus a distinct learner-facing policy concept: bounded cluster limits replacing legacy ancestor/descendant limits.</x:v>
+        <x:v>Complete cluster-mempool pass. getmempoolcluster and getmempoolfeeratediagram are implementation surfaces merged into protocol.cluster-mempool; ops.mempool-cluster-limits remains the distinct learner-facing policy concept.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10732,16 +10732,212 @@
         <x:v>Existing node confirmed; payment proofs and TLV fields remain internal parts of the BOLT 12 flow rather than standalone learner nodes.</x:v>
       </x:c>
     </x:row>
+    <x:row r="155">
+      <x:c r="A155" s="32" t="str">
+        <x:v>ops.mempool-explorer</x:v>
+      </x:c>
+      <x:c r="B155" s="32" t="str">
+        <x:v>Mempool Explorer</x:v>
+      </x:c>
+      <x:c r="C155" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D155" s="32" t="str">
+        <x:v>source.mempool-space-docs</x:v>
+      </x:c>
+      <x:c r="E155" s="32" t="str">
+        <x:v>https://mempool.space/docs</x:v>
+      </x:c>
+      <x:c r="F155" s="32" t="str">
+        <x:v>Mempool.space explorer and visualizer</x:v>
+      </x:c>
+      <x:c r="G155" s="32" t="str"/>
+      <x:c r="H155" s="32" t="str">
+        <x:v>skip</x:v>
+      </x:c>
+      <x:c r="I155" s="32" t="str">
+        <x:v>The explorer is a product and observability surface over Bitcoin data, not one Bitcoin protocol concept with a learner-specific prerequisite chain.</x:v>
+      </x:c>
+      <x:c r="J155" s="32" t="str">
+        <x:v>protocol.mempool</x:v>
+      </x:c>
+      <x:c r="K155" s="32" t="str"/>
+      <x:c r="L155" s="32" t="str">
+        <x:v>No graph edge is justified for a product wrapper.</x:v>
+      </x:c>
+      <x:c r="M155" s="32" t="str">
+        <x:v>mempool.space explorer, mempool visualizer</x:v>
+      </x:c>
+      <x:c r="N155" s="32" t="str">
+        <x:v>mempool, observability, tools</x:v>
+      </x:c>
+      <x:c r="O155" s="32" t="str">
+        <x:v>0m</x:v>
+      </x:c>
+      <x:c r="P155" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q155" s="32" t="str">
+        <x:v>Skip as a product surface; retain the source family for operational reference.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" s="32" t="str">
+        <x:v>dev.mempool-rest-api</x:v>
+      </x:c>
+      <x:c r="B156" s="32" t="str">
+        <x:v>Mempool.space REST API</x:v>
+      </x:c>
+      <x:c r="C156" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D156" s="32" t="str">
+        <x:v>source.mempool-space-docs</x:v>
+      </x:c>
+      <x:c r="E156" s="32" t="str">
+        <x:v>https://mempool.space/docs</x:v>
+      </x:c>
+      <x:c r="F156" s="32" t="str">
+        <x:v>Mempool.space REST API</x:v>
+      </x:c>
+      <x:c r="G156" s="32" t="str"/>
+      <x:c r="H156" s="32" t="str">
+        <x:v>skip</x:v>
+      </x:c>
+      <x:c r="I156" s="32" t="str">
+        <x:v>The REST endpoint surface is an implementation interface, not a Bitcoin concept learners need as a graph node.</x:v>
+      </x:c>
+      <x:c r="J156" s="32" t="str">
+        <x:v>protocol.mempool</x:v>
+      </x:c>
+      <x:c r="K156" s="32" t="str"/>
+      <x:c r="L156" s="32" t="str">
+        <x:v>No direct learner prerequisite applies to an application API wrapper.</x:v>
+      </x:c>
+      <x:c r="M156" s="32" t="str">
+        <x:v>mempool REST API</x:v>
+      </x:c>
+      <x:c r="N156" s="32" t="str">
+        <x:v>api, mempool, tools</x:v>
+      </x:c>
+      <x:c r="O156" s="32" t="str">
+        <x:v>0m</x:v>
+      </x:c>
+      <x:c r="P156" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q156" s="32" t="str">
+        <x:v>Skip under the implementation-surface heuristic.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" s="32" t="str">
+        <x:v>dev.mempool-websocket-api</x:v>
+      </x:c>
+      <x:c r="B157" s="32" t="str">
+        <x:v>Mempool.space WebSocket API</x:v>
+      </x:c>
+      <x:c r="C157" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D157" s="32" t="str">
+        <x:v>source.mempool-space-docs</x:v>
+      </x:c>
+      <x:c r="E157" s="32" t="str">
+        <x:v>https://mempool.space/docs</x:v>
+      </x:c>
+      <x:c r="F157" s="32" t="str">
+        <x:v>Mempool.space WebSocket and live events</x:v>
+      </x:c>
+      <x:c r="G157" s="32" t="str"/>
+      <x:c r="H157" s="32" t="str">
+        <x:v>skip</x:v>
+      </x:c>
+      <x:c r="I157" s="32" t="str">
+        <x:v>The WebSocket event stream is an application transport interface, not a distinct Bitcoin protocol concept.</x:v>
+      </x:c>
+      <x:c r="J157" s="32" t="str">
+        <x:v>protocol.mempool</x:v>
+      </x:c>
+      <x:c r="K157" s="32" t="str"/>
+      <x:c r="L157" s="32" t="str">
+        <x:v>No graph edge is justified for an application transport wrapper.</x:v>
+      </x:c>
+      <x:c r="M157" s="32" t="str">
+        <x:v>mempool WebSocket API, mempool live events</x:v>
+      </x:c>
+      <x:c r="N157" s="32" t="str">
+        <x:v>api, mempool, tools</x:v>
+      </x:c>
+      <x:c r="O157" s="32" t="str">
+        <x:v>0m</x:v>
+      </x:c>
+      <x:c r="P157" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q157" s="32" t="str">
+        <x:v>Skip under the implementation-surface heuristic.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" s="32" t="str">
+        <x:v>ops.mempool-self-hosting</x:v>
+      </x:c>
+      <x:c r="B158" s="32" t="str">
+        <x:v>Self-Hosted Mempool Explorer</x:v>
+      </x:c>
+      <x:c r="C158" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D158" s="32" t="str">
+        <x:v>source.mempool-space-docs</x:v>
+      </x:c>
+      <x:c r="E158" s="32" t="str">
+        <x:v>https://mempool.space/docs</x:v>
+      </x:c>
+      <x:c r="F158" s="32" t="str">
+        <x:v>Mempool.space self-hosting and deployment</x:v>
+      </x:c>
+      <x:c r="G158" s="32" t="str"/>
+      <x:c r="H158" s="32" t="str">
+        <x:v>skip</x:v>
+      </x:c>
+      <x:c r="I158" s="32" t="str">
+        <x:v>Self-hosting this explorer is a deployment workflow built on Bitcoin Core, not a Bitcoin learning concept that should occupy a graph node.</x:v>
+      </x:c>
+      <x:c r="J158" s="32" t="str">
+        <x:v>ops.run-full-node</x:v>
+      </x:c>
+      <x:c r="K158" s="32" t="str"/>
+      <x:c r="L158" s="32" t="str">
+        <x:v>Running a full node is related operational context but not a direct prerequisite for a skipped product workflow.</x:v>
+      </x:c>
+      <x:c r="M158" s="32" t="str">
+        <x:v>self-hosted mempool.space, Mempool deployment</x:v>
+      </x:c>
+      <x:c r="N158" s="32" t="str">
+        <x:v>operations, self-hosting, tools</x:v>
+      </x:c>
+      <x:c r="O158" s="32" t="str">
+        <x:v>0m</x:v>
+      </x:c>
+      <x:c r="P158" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q158" s="32" t="str">
+        <x:v>Skip as product/deployment scope; preserve repository documentation as an optional operator resource outside the concept graph.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H154">
+    <x:dataValidation type="list" sqref="H12:H158">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P154">
+    <x:dataValidation type="list" sqref="P12:P158">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -16561,16 +16757,42 @@
         <x:v>Added as a draft protocol/application concept; TRUC remains related anti-pinning context without becoming a direct prerequisite.</x:v>
       </x:c>
     </x:row>
+    <x:row r="118">
+      <x:c r="A118" s="32" t="str">
+        <x:v>decision.mempool-space-surface-skip</x:v>
+      </x:c>
+      <x:c r="B118" s="32" t="str">
+        <x:v>exclusion</x:v>
+      </x:c>
+      <x:c r="C118" s="32" t="str">
+        <x:v>source.mempool-space-docs</x:v>
+      </x:c>
+      <x:c r="D118" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E118" s="32" t="str">
+        <x:v>The Mempool.space FAQ, REST API, WebSocket stream, and self-hosting material expose observability and deployment surfaces over Bitcoin Core. They do not add a learner-facing Bitcoin protocol concept beyond the already-covered mempool policy/purging branch.</x:v>
+      </x:c>
+      <x:c r="F118" s="32" t="str">
+        <x:v>ops.mempool-purging, ops.mempool-explorer, dev.mempool-rest-api, dev.mempool-websocket-api, ops.mempool-self-hosting</x:v>
+      </x:c>
+      <x:c r="G118" s="32" t="str">
+        <x:v>source.mempool-space-docs</x:v>
+      </x:c>
+      <x:c r="H118" s="32" t="str">
+        <x:v>Keep these as audit candidates and source references, but do not mint product/API wrapper nodes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B117">
+    <x:dataValidation type="list" sqref="B12:B118">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D117">
+    <x:dataValidation type="list" sqref="D12:D118">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -16623,7 +16845,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.71491829861</x:v>
+        <x:v>46214.71990200232</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -16639,7 +16861,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>50</x:v>
+        <x:v>58</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -16647,7 +16869,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>143</x:v>
+        <x:v>147</x:v>
       </x:c>
     </x:row>
     <x:row r="9">

</xml_diff>

<commit_message>
feat: audit first bitcoin questions edition
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Refec70ce97e84fc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R29dd44e70d354ea7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R799e27e8efe3406e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rf4e65593583f4e49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R7fff0be324064285"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rc640ed2eb32542c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R9c284e7c62df4b80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R715056b261ee4006"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R0fdaba2da65a40dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R88475d6a5d104e02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R0ec50bb3c72c41dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Re8f80b25478343de"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3266,22 +3266,69 @@
         <x:v>Complete cluster-mempool pass. getmempoolcluster and getmempoolfeeratediagram are implementation surfaces merged into protocol.cluster-mempool; ops.mempool-cluster-limits remains the distinct learner-facing policy concept.</x:v>
       </x:c>
     </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="B70" s="32" t="str">
+        <x:v>101 Perguntas e Respostas sobre Bitcoin - 1a edicao</x:v>
+      </x:c>
+      <x:c r="C70" s="32" t="str">
+        <x:v>local:///Users/breno/Documents/Obsidian%20Vault/Projects/Ativos/101BTC/1_ed</x:v>
+      </x:c>
+      <x:c r="D70" s="32" t="str">
+        <x:v>local-book-markdown</x:v>
+      </x:c>
+      <x:c r="E70" s="32" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F70" s="32" t="str">
+        <x:v>Completed first-edition beginner curriculum covering Bitcoin history, money, custody, protocol mechanics, mining, privacy, scaling, legal context, and contribution paths.</x:v>
+      </x:c>
+      <x:c r="G70" s="32" t="str">
+        <x:v>Inspect all 101 numbered chapter files individually, extract atomic learning outcomes, then deduplicate against existing nodes and separate Bitcoin concepts from opinions, laws, product references, and future-project surveys.</x:v>
+      </x:c>
+      <x:c r="H70" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I70" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J70" s="32" t="str">
+        <x:v>Normalized</x:v>
+      </x:c>
+      <x:c r="K70" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L70" s="32" t="n">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="M70" s="32" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="N70" s="32" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="O70" s="32" t="str">
+        <x:v>Complete first-edition pass over all 101 chapter files. Six concepts were added, six candidates were merged or excluded: Satoshi Nakamoto, Bitcoin denominations and satoshis, block subsidy, quantum-computing threats, Ordinals and inscriptions, and proof of existence/timestamping. Stablecoins, altcoins, exchanges, satellites, and named products remain contextual or implementation/product scope. The unfinished second edition was intentionally excluded.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H69">
+    <x:dataValidation type="list" sqref="H12:H70">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I69">
+    <x:dataValidation type="list" sqref="I12:I70">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J69">
+    <x:dataValidation type="list" sqref="J12:J70">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K69">
+    <x:dataValidation type="list" sqref="K12:K70">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10928,16 +10975,563 @@
         <x:v>Skip as product/deployment scope; preserve repository documentation as an optional operator resource outside the concept graph.</x:v>
       </x:c>
     </x:row>
+    <x:row r="159">
+      <x:c r="A159" s="32" t="str">
+        <x:v>history.satoshi-nakamoto</x:v>
+      </x:c>
+      <x:c r="B159" s="32" t="str">
+        <x:v>Satoshi Nakamoto</x:v>
+      </x:c>
+      <x:c r="C159" s="32" t="str">
+        <x:v>History &amp; Governance</x:v>
+      </x:c>
+      <x:c r="D159" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="E159" s="32" t="str">
+        <x:v>local:///Users/breno/Documents/Obsidian%20Vault/Projects/Ativos/101BTC/1_ed/101BTC%20-%20004_quem_criou_o_bitcoin.md</x:v>
+      </x:c>
+      <x:c r="F159" s="32" t="str">
+        <x:v>Question 4: Who created Bitcoin?</x:v>
+      </x:c>
+      <x:c r="G159" s="32" t="str"/>
+      <x:c r="H159" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I159" s="32" t="str">
+        <x:v>The creator pseudonym and deliberate disappearance are a distinct historical and governance learning outcome, not merely a duplicate of the whitepaper or early-history container.</x:v>
+      </x:c>
+      <x:c r="J159" s="32" t="str">
+        <x:v>history.cypherpunk-roots-bitcoin-origin</x:v>
+      </x:c>
+      <x:c r="K159" s="32" t="str">
+        <x:v>history.cypherpunk-roots-bitcoin-origin</x:v>
+      </x:c>
+      <x:c r="L159" s="32" t="str">
+        <x:v>The cypherpunk roots and origin context provide the historical frame for understanding the pseudonym and founder independence.</x:v>
+      </x:c>
+      <x:c r="M159" s="32" t="str">
+        <x:v>Satoshi, Bitcoin creator</x:v>
+      </x:c>
+      <x:c r="N159" s="32" t="str">
+        <x:v>history, origins, pseudonymity</x:v>
+      </x:c>
+      <x:c r="O159" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P159" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q159" s="32" t="str">
+        <x:v>Add as a focused historical node; avoid turning speculation about Satoshi's legal identity into graph content.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="A160" s="32" t="str">
+        <x:v>economics.bitcoin-denominations</x:v>
+      </x:c>
+      <x:c r="B160" s="32" t="str">
+        <x:v>Bitcoin Denominations and Satoshis</x:v>
+      </x:c>
+      <x:c r="C160" s="32" t="str">
+        <x:v>Economics &amp; Incentives</x:v>
+      </x:c>
+      <x:c r="D160" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="E160" s="32" t="str">
+        <x:v>local:///Users/breno/Documents/Obsidian%20Vault/Projects/Ativos/101BTC/1_ed/101BTC%20-%20003_qual_a_diferenca_entre_bitcoin_com_b_maiusculo_e_b.md</x:v>
+      </x:c>
+      <x:c r="F160" s="32" t="str">
+        <x:v>Question 3: Bitcoin, BTC, and satoshis</x:v>
+      </x:c>
+      <x:c r="G160" s="32" t="str"/>
+      <x:c r="H160" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I160" s="32" t="str">
+        <x:v>BTC and satoshis are a concrete monetary-unit concept that learners need to identify and use, distinct from generic scarcity or money properties.</x:v>
+      </x:c>
+      <x:c r="J160" s="32" t="str">
+        <x:v>fundamentals.money-properties</x:v>
+      </x:c>
+      <x:c r="K160" s="32" t="str">
+        <x:v>fundamentals.money-properties</x:v>
+      </x:c>
+      <x:c r="L160" s="32" t="str">
+        <x:v>Monetary units are easier to understand after the learner has a basic model of money and its functions.</x:v>
+      </x:c>
+      <x:c r="M160" s="32" t="str">
+        <x:v>sats, bitcoin units, BTC denominations</x:v>
+      </x:c>
+      <x:c r="N160" s="32" t="str">
+        <x:v>money, units, satoshis</x:v>
+      </x:c>
+      <x:c r="O160" s="32" t="str">
+        <x:v>20m</x:v>
+      </x:c>
+      <x:c r="P160" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q160" s="32" t="str">
+        <x:v>Add the denomination concept without creating separate nodes for BTC, bitcoin capitalization, or the protocol/software naming convention.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161">
+      <x:c r="A161" s="32" t="str">
+        <x:v>economics.block-subsidy</x:v>
+      </x:c>
+      <x:c r="B161" s="32" t="str">
+        <x:v>Block Subsidy</x:v>
+      </x:c>
+      <x:c r="C161" s="32" t="str">
+        <x:v>Economics &amp; Incentives</x:v>
+      </x:c>
+      <x:c r="D161" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="E161" s="32" t="str">
+        <x:v>local:///Users/breno/Documents/Obsidian%20Vault/Projects/Ativos/101BTC/1_ed/101BTC%20-%20018_quantos_bitcoin_sao_produzidos_por_dia.md</x:v>
+      </x:c>
+      <x:c r="F161" s="32" t="str">
+        <x:v>Question 18: How many bitcoin are produced per day?</x:v>
+      </x:c>
+      <x:c r="G161" s="32" t="str"/>
+      <x:c r="H161" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I161" s="32" t="str">
+        <x:v>The newly issued portion of miner revenue is a specific issuance mechanism that should not be hidden inside coinbase transactions or the halving schedule.</x:v>
+      </x:c>
+      <x:c r="J161" s="32" t="str">
+        <x:v>protocol.coinbase-transaction</x:v>
+      </x:c>
+      <x:c r="K161" s="32" t="str">
+        <x:v>protocol.coinbase-transaction</x:v>
+      </x:c>
+      <x:c r="L161" s="32" t="str">
+        <x:v>The coinbase transaction is where the subsidy is claimed; its existing halving prerequisite already supplies the issuance schedule.</x:v>
+      </x:c>
+      <x:c r="M161" s="32" t="str">
+        <x:v>mining subsidy, block reward subsidy, new bitcoin issuance</x:v>
+      </x:c>
+      <x:c r="N161" s="32" t="str">
+        <x:v>issuance, mining, monetary-policy</x:v>
+      </x:c>
+      <x:c r="O161" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P161" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q161" s="32" t="str">
+        <x:v>Add as the issuance component of miner revenue; keep fees as a separate concept.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162">
+      <x:c r="A162" s="32" t="str">
+        <x:v>security.quantum-computing-threat</x:v>
+      </x:c>
+      <x:c r="B162" s="32" t="str">
+        <x:v>Quantum Computing Threats</x:v>
+      </x:c>
+      <x:c r="C162" s="32" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="D162" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="E162" s="32" t="str">
+        <x:v>local:///Users/breno/Documents/Obsidian%20Vault/Projects/Ativos/101BTC/1_ed/101BTC%20-%20081_o_que_vai_acontecer_se_quebrarem_a_criptografia_do.md</x:v>
+      </x:c>
+      <x:c r="F162" s="32" t="str">
+        <x:v>Question 81: What happens if Bitcoin cryptography is broken?</x:v>
+      </x:c>
+      <x:c r="G162" s="32" t="str"/>
+      <x:c r="H162" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I162" s="32" t="str">
+        <x:v>Quantum attacks create a distinct threat model across public-key signatures and proof-of-work, beyond ordinary private-key guessing or nonce failures.</x:v>
+      </x:c>
+      <x:c r="J162" s="32" t="str">
+        <x:v>fundamentals.digital-signatures</x:v>
+      </x:c>
+      <x:c r="K162" s="32" t="str">
+        <x:v>fundamentals.digital-signatures</x:v>
+      </x:c>
+      <x:c r="L162" s="32" t="str">
+        <x:v>Digital-signature security is the non-redundant direct prerequisite for the key-spending threat; proof-of-work remains covered in the node description and resources rather than duplicating the current graph path.</x:v>
+      </x:c>
+      <x:c r="M162" s="32" t="str">
+        <x:v>quantum threat, quantum attacks on Bitcoin, quantum resistance</x:v>
+      </x:c>
+      <x:c r="N162" s="32" t="str">
+        <x:v>security, cryptography, post-quantum</x:v>
+      </x:c>
+      <x:c r="O162" s="32" t="str">
+        <x:v>45m</x:v>
+      </x:c>
+      <x:c r="P162" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q162" s="32" t="str">
+        <x:v>Add as a threat-model node; Lamport signatures remain a neighboring post-quantum primitive rather than a substitute for the threat model.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" s="32" t="str">
+        <x:v>extension.ordinals-inscriptions</x:v>
+      </x:c>
+      <x:c r="B163" s="32" t="str">
+        <x:v>Ordinals and Inscriptions</x:v>
+      </x:c>
+      <x:c r="C163" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D163" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="E163" s="32" t="str">
+        <x:v>local:///Users/breno/Documents/Obsidian%20Vault/Projects/Ativos/101BTC/1_ed/101BTC%20-%20078_e_possivel_registrar_coisas_alem_de_transacoes_na_.md</x:v>
+      </x:c>
+      <x:c r="F163" s="32" t="str">
+        <x:v>Question 78: Can things besides transactions be registered on Bitcoin?</x:v>
+      </x:c>
+      <x:c r="G163" s="32" t="str"/>
+      <x:c r="H163" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I163" s="32" t="str">
+        <x:v>Ordinal numbering and inscription data form a distinct Bitcoin application pattern with concrete witness, fee, and block-space tradeoffs; it is not just generic OP_RETURN data.</x:v>
+      </x:c>
+      <x:c r="J163" s="32" t="str">
+        <x:v>protocol.taproot, protocol.witness-structure</x:v>
+      </x:c>
+      <x:c r="K163" s="32" t="str">
+        <x:v>protocol.taproot, protocol.witness-structure</x:v>
+      </x:c>
+      <x:c r="L163" s="32" t="str">
+        <x:v>The book's explanation ties inscriptions to Taproot-era witness data; OP_RETURN is an older adjacent mechanism, not a direct prerequisite.</x:v>
+      </x:c>
+      <x:c r="M163" s="32" t="str">
+        <x:v>Ordinals, Bitcoin inscriptions, ordinal inscriptions</x:v>
+      </x:c>
+      <x:c r="N163" s="32" t="str">
+        <x:v>taproot, witness, applications</x:v>
+      </x:c>
+      <x:c r="O163" s="32" t="str">
+        <x:v>45m</x:v>
+      </x:c>
+      <x:c r="P163" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q163" s="32" t="str">
+        <x:v>Add the learner-facing application concept while keeping individual inscription formats and marketplaces out of the graph.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" s="32" t="str">
+        <x:v>extension.proof-of-existence</x:v>
+      </x:c>
+      <x:c r="B164" s="32" t="str">
+        <x:v>Proof of Existence and Timestamping</x:v>
+      </x:c>
+      <x:c r="C164" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D164" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="E164" s="32" t="str">
+        <x:v>local:///Users/breno/Documents/Obsidian%20Vault/Projects/Ativos/101BTC/1_ed/101BTC%20-%20079_o_que_significa_a_mensagem_do_primeiro_bloco_do_bi.md</x:v>
+      </x:c>
+      <x:c r="F164" s="32" t="str">
+        <x:v>Question 79: What does the Genesis Block message mean?</x:v>
+      </x:c>
+      <x:c r="G164" s="32" t="str"/>
+      <x:c r="H164" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I164" s="32" t="str">
+        <x:v>Anchoring evidence to prove that it existed by a given time is a distinct application outcome illustrated by the Genesis Block and OpenTimestamps references.</x:v>
+      </x:c>
+      <x:c r="J164" s="32" t="str">
+        <x:v>fundamentals.commitment-schemes</x:v>
+      </x:c>
+      <x:c r="K164" s="32" t="str">
+        <x:v>fundamentals.commitment-schemes</x:v>
+      </x:c>
+      <x:c r="L164" s="32" t="str">
+        <x:v>Commitments provide the minimal cryptographic mechanism for timestamping without storing the full document on-chain.</x:v>
+      </x:c>
+      <x:c r="M164" s="32" t="str">
+        <x:v>proof of existence, Bitcoin timestamping, OpenTimestamps</x:v>
+      </x:c>
+      <x:c r="N164" s="32" t="str">
+        <x:v>commitments, timestamping, applications</x:v>
+      </x:c>
+      <x:c r="O164" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P164" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q164" s="32" t="str">
+        <x:v>Add as a generic Bitcoin-anchored application; the Genesis Block remains historical context rather than the node itself.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" s="32" t="str">
+        <x:v>economics.stablecoins</x:v>
+      </x:c>
+      <x:c r="B165" s="32" t="str">
+        <x:v>Stablecoins</x:v>
+      </x:c>
+      <x:c r="C165" s="32" t="str">
+        <x:v>Economics &amp; Incentives</x:v>
+      </x:c>
+      <x:c r="D165" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="E165" s="32" t="str">
+        <x:v>local:///Users/breno/Documents/Obsidian%20Vault/Projects/Ativos/101BTC/1_ed/101BTC%20-%20095_o_que_sao_altcoins_e_stablecoins.md</x:v>
+      </x:c>
+      <x:c r="F165" s="32" t="str">
+        <x:v>Question 95: What are altcoins and stablecoins?</x:v>
+      </x:c>
+      <x:c r="G165" s="32" t="str"/>
+      <x:c r="H165" s="32" t="str">
+        <x:v>skip</x:v>
+      </x:c>
+      <x:c r="I165" s="32" t="str">
+        <x:v>Stablecoins are a broad adjacent-asset category with issuer, collateral, and regulatory models that do not form a Bitcoin prerequisite in this graph.</x:v>
+      </x:c>
+      <x:c r="J165" s="32" t="str"/>
+      <x:c r="K165" s="32" t="str"/>
+      <x:c r="L165" s="32" t="str">
+        <x:v>No direct Bitcoin learning prerequisite is justified for a skipped adjacent-asset survey.</x:v>
+      </x:c>
+      <x:c r="M165" s="32" t="str">
+        <x:v>stable coins</x:v>
+      </x:c>
+      <x:c r="N165" s="32" t="str">
+        <x:v>adjacent-assets, money</x:v>
+      </x:c>
+      <x:c r="O165" s="32" t="str">
+        <x:v>0m</x:v>
+      </x:c>
+      <x:c r="P165" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q165" s="32" t="str">
+        <x:v>Skip as adjacent context; revisit only if the graph gains a deliberate comparative monetary-systems branch.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" s="32" t="str">
+        <x:v>economics.altcoins</x:v>
+      </x:c>
+      <x:c r="B166" s="32" t="str">
+        <x:v>Altcoins</x:v>
+      </x:c>
+      <x:c r="C166" s="32" t="str">
+        <x:v>Economics &amp; Incentives</x:v>
+      </x:c>
+      <x:c r="D166" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="E166" s="32" t="str">
+        <x:v>local:///Users/breno/Documents/Obsidian%20Vault/Projects/Ativos/101BTC/1_ed/101BTC%20-%20095_o_que_sao_altcoins_e_stablecoins.md</x:v>
+      </x:c>
+      <x:c r="F166" s="32" t="str">
+        <x:v>Question 95: What are altcoins and stablecoins?</x:v>
+      </x:c>
+      <x:c r="G166" s="32" t="str"/>
+      <x:c r="H166" s="32" t="str">
+        <x:v>skip</x:v>
+      </x:c>
+      <x:c r="I166" s="32" t="str">
+        <x:v>Altcoins are a comparison class rather than one atomic Bitcoin concept; the graph already covers forks, sidechains, and token systems where those distinctions matter.</x:v>
+      </x:c>
+      <x:c r="J166" s="32" t="str"/>
+      <x:c r="K166" s="32" t="str"/>
+      <x:c r="L166" s="32" t="str">
+        <x:v>No direct graph edge is justified for a skipped comparison category.</x:v>
+      </x:c>
+      <x:c r="M166" s="32" t="str">
+        <x:v>alternative cryptocurrencies, alternative coins</x:v>
+      </x:c>
+      <x:c r="N166" s="32" t="str">
+        <x:v>adjacent-assets, comparisons</x:v>
+      </x:c>
+      <x:c r="O166" s="32" t="str">
+        <x:v>0m</x:v>
+      </x:c>
+      <x:c r="P166" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q166" s="32" t="str">
+        <x:v>Skip as a broad category and retain the chapter as source context for comparative learning.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" s="32" t="str">
+        <x:v>ops.exchange-custody</x:v>
+      </x:c>
+      <x:c r="B167" s="32" t="str">
+        <x:v>Exchange Custody</x:v>
+      </x:c>
+      <x:c r="C167" s="32" t="str">
+        <x:v>Wallets</x:v>
+      </x:c>
+      <x:c r="D167" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="E167" s="32" t="str">
+        <x:v>local:///Users/breno/Documents/Obsidian%20Vault/Projects/Ativos/101BTC/1_ed/101BTC%20-%20014_o_que_e_uma_exchange.md</x:v>
+      </x:c>
+      <x:c r="F167" s="32" t="str">
+        <x:v>Question 14: What is an exchange?</x:v>
+      </x:c>
+      <x:c r="G167" s="32" t="str"/>
+      <x:c r="H167" s="32" t="str">
+        <x:v>skip</x:v>
+      </x:c>
+      <x:c r="I167" s="32" t="str">
+        <x:v>An exchange is a product and custody model, not a Bitcoin protocol concept; adding a node would invite rapidly changing provider-specific detail.</x:v>
+      </x:c>
+      <x:c r="J167" s="32" t="str"/>
+      <x:c r="K167" s="32" t="str"/>
+      <x:c r="L167" s="32" t="str">
+        <x:v>No graph edge is justified for a skipped product category.</x:v>
+      </x:c>
+      <x:c r="M167" s="32" t="str">
+        <x:v>bitcoin exchange, custodial exchange</x:v>
+      </x:c>
+      <x:c r="N167" s="32" t="str">
+        <x:v>custody, products</x:v>
+      </x:c>
+      <x:c r="O167" s="32" t="str">
+        <x:v>0m</x:v>
+      </x:c>
+      <x:c r="P167" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q167" s="32" t="str">
+        <x:v>Skip as product scope; self-custody and custody tradeoffs remain the learner-facing concepts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" s="32" t="str">
+        <x:v>ops.offline-bitcoin-transport</x:v>
+      </x:c>
+      <x:c r="B168" s="32" t="str">
+        <x:v>Offline Bitcoin Transport</x:v>
+      </x:c>
+      <x:c r="C168" s="32" t="str">
+        <x:v>Network, Relay &amp; Client Sync</x:v>
+      </x:c>
+      <x:c r="D168" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="E168" s="32" t="str">
+        <x:v>local:///Users/breno/Documents/Obsidian%20Vault/Projects/Ativos/101BTC/1_ed/101BTC%20-%20082_e_se_desligarem_a_internet.md</x:v>
+      </x:c>
+      <x:c r="F168" s="32" t="str">
+        <x:v>Question 82: What if the Internet is shut down?</x:v>
+      </x:c>
+      <x:c r="G168" s="32" t="str">
+        <x:v>ops.mesh-networks</x:v>
+      </x:c>
+      <x:c r="H168" s="32" t="str">
+        <x:v>merge</x:v>
+      </x:c>
+      <x:c r="I168" s="32" t="str">
+        <x:v>Satellite, mesh, telephone, and physical-transfer examples all answer the same operational question about alternate communication paths; they do not warrant separate product nodes.</x:v>
+      </x:c>
+      <x:c r="J168" s="32" t="str">
+        <x:v>fundamentals.peer-to-peer-network</x:v>
+      </x:c>
+      <x:c r="K168" s="32" t="str">
+        <x:v>ops.mesh-networks</x:v>
+      </x:c>
+      <x:c r="L168" s="32" t="str">
+        <x:v>Reuse the existing off-grid mesh-network concept rather than duplicating transport modalities.</x:v>
+      </x:c>
+      <x:c r="M168" s="32" t="str">
+        <x:v>offline Bitcoin transfer, alternate Bitcoin communications</x:v>
+      </x:c>
+      <x:c r="N168" s="32" t="str">
+        <x:v>networking, resilience, operations</x:v>
+      </x:c>
+      <x:c r="O168" s="32" t="str">
+        <x:v>30m</x:v>
+      </x:c>
+      <x:c r="P168" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q168" s="32" t="str">
+        <x:v>Merge source examples into ops.mesh-networks as supporting context; satellites and Opendime remain implementation/product examples.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169">
+      <x:c r="A169" s="32" t="str">
+        <x:v>economics.hodling</x:v>
+      </x:c>
+      <x:c r="B169" s="32" t="str">
+        <x:v>HODLing</x:v>
+      </x:c>
+      <x:c r="C169" s="32" t="str">
+        <x:v>Economics &amp; Incentives</x:v>
+      </x:c>
+      <x:c r="D169" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="E169" s="32" t="str">
+        <x:v>local:///Users/breno/Documents/Obsidian%20Vault/Projects/Ativos/101BTC/1_ed/101BTC%20-%20071_o_que_e_hodl.md</x:v>
+      </x:c>
+      <x:c r="F169" s="32" t="str">
+        <x:v>Question 71: What is HODL?</x:v>
+      </x:c>
+      <x:c r="G169" s="32" t="str"/>
+      <x:c r="H169" s="32" t="str">
+        <x:v>skip</x:v>
+      </x:c>
+      <x:c r="I169" s="32" t="str">
+        <x:v>HODL is a cultural slogan and investment behavior, not a prerequisite concept needed to understand Bitcoin's mechanics.</x:v>
+      </x:c>
+      <x:c r="J169" s="32" t="str"/>
+      <x:c r="K169" s="32" t="str"/>
+      <x:c r="L169" s="32" t="str">
+        <x:v>No graph edge is justified for a skipped cultural term.</x:v>
+      </x:c>
+      <x:c r="M169" s="32" t="str">
+        <x:v>hold on for dear life, holding bitcoin</x:v>
+      </x:c>
+      <x:c r="N169" s="32" t="str">
+        <x:v>culture, markets</x:v>
+      </x:c>
+      <x:c r="O169" s="32" t="str">
+        <x:v>0m</x:v>
+      </x:c>
+      <x:c r="P169" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q169" s="32" t="str">
+        <x:v>Skip as culture/behavior; volatility and savings concepts remain the relevant learner outcomes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H158">
+    <x:dataValidation type="list" sqref="H12:H169">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P158">
+    <x:dataValidation type="list" sqref="P12:P169">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11005,10 +11599,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="32" t="str">
-        <x:v>protocol.tagged-hashes</x:v>
+        <x:v>history.cypherpunk-roots-bitcoin-origin</x:v>
       </x:c>
       <x:c r="B12" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>history.satoshi-nakamoto</x:v>
       </x:c>
       <x:c r="C12" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11017,10 +11611,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E12" s="32" t="str">
-        <x:v>TapTweak is defined using tagged hashes directly in Taproot key tweaking.</x:v>
+        <x:v>Satoshi's pseudonym and founder independence are best understood in the context of Bitcoin's cypherpunk roots and origin story.</x:v>
       </x:c>
       <x:c r="F12" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G12" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11028,10 +11622,10 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="32" t="str">
-        <x:v>protocol.x-only-public-keys</x:v>
+        <x:v>fundamentals.money-properties</x:v>
       </x:c>
       <x:c r="B13" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>economics.bitcoin-denominations</x:v>
       </x:c>
       <x:c r="C13" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11040,10 +11634,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E13" s="32" t="str">
-        <x:v>TapTweak operates on x-only public keys in the Taproot construction.</x:v>
+        <x:v>The learner needs a basic monetary-unit model before BTC and satoshis are meaningful denominations.</x:v>
       </x:c>
       <x:c r="F13" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G13" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11051,10 +11645,10 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>protocol.coinbase-transaction</x:v>
       </x:c>
       <x:c r="B14" s="32" t="str">
-        <x:v>protocol.taproot-key-path-spends</x:v>
+        <x:v>economics.block-subsidy</x:v>
       </x:c>
       <x:c r="C14" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11063,21 +11657,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E14" s="32" t="str">
-        <x:v>A key-path spend verifies against the tweaked Taproot output key, so learners need the tweak mechanism before the spending mode makes sense.</x:v>
+        <x:v>The block subsidy is the newly issued component claimed by a coinbase transaction.</x:v>
       </x:c>
       <x:c r="F14" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G14" s="32" t="str">
-        <x:v>Direct parent keeps the node focused on the spend mode rather than on broad Taproot overview material.</x:v>
+        <x:v>The coinbase node already carries the halving prerequisite, so no redundant direct halving edge is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="32" t="str">
-        <x:v>protocol.taptree</x:v>
+        <x:v>fundamentals.digital-signatures</x:v>
       </x:c>
       <x:c r="B15" s="32" t="str">
-        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
+        <x:v>security.quantum-computing-threat</x:v>
       </x:c>
       <x:c r="C15" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11086,10 +11680,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E15" s="32" t="str">
-        <x:v>The inclusion proof only makes sense after the learner understands the TapTree structure.</x:v>
+        <x:v>Quantum attacks on public-key authorization require understanding ordinary Bitcoin signature security first.</x:v>
       </x:c>
       <x:c r="F15" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G15" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11097,10 +11691,10 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="32" t="str">
-        <x:v>protocol.taptree</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B16" s="32" t="str">
-        <x:v>protocol.huffman-optimized-taptrees</x:v>
+        <x:v>extension.ordinals-inscriptions</x:v>
       </x:c>
       <x:c r="C16" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11109,10 +11703,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E16" s="32" t="str">
-        <x:v>Huffman optimization is a refinement of how TapTree leaves are arranged.</x:v>
+        <x:v>The source explains inscriptions as a Taproot-era witness-data application.</x:v>
       </x:c>
       <x:c r="F16" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G16" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11120,10 +11714,10 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="32" t="str">
-        <x:v>protocol.softfork-hardfork</x:v>
+        <x:v>protocol.witness-structure</x:v>
       </x:c>
       <x:c r="B17" s="32" t="str">
-        <x:v>protocol.chain-split-risk</x:v>
+        <x:v>extension.ordinals-inscriptions</x:v>
       </x:c>
       <x:c r="C17" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11132,21 +11726,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E17" s="32" t="str">
-        <x:v>Split risk is a downstream consequence of incompatible upgrade paths, so learners should understand the compatibility boundary first.</x:v>
+        <x:v>Witness structure is needed to understand where inscription data is carried and how it affects block space.</x:v>
       </x:c>
       <x:c r="F17" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G17" s="32" t="str">
-        <x:v>Direct edge chosen over activation-history case studies because those are downstream examples, not prerequisites.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="B18" s="32" t="str">
-        <x:v>protocol.tapscript</x:v>
+        <x:v>extension.proof-of-existence</x:v>
       </x:c>
       <x:c r="C18" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11155,21 +11749,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E18" s="32" t="str">
-        <x:v>Tapscript is a Taproot-specific script version, so learners need the Taproot spend context before its rule changes make sense.</x:v>
+        <x:v>Timestamp proofs commit evidence without requiring the complete document to be stored on-chain.</x:v>
       </x:c>
       <x:c r="F18" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G18" s="32" t="str">
-        <x:v>Direct edge keeps the node scoped to the Taproot family without collapsing it into a generic script refresher.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="32" t="str">
-        <x:v>custody.psbt</x:v>
+        <x:v>protocol.tagged-hashes</x:v>
       </x:c>
       <x:c r="B19" s="32" t="str">
-        <x:v>dev.taproot-psbt-fields</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="C19" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11178,21 +11772,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E19" s="32" t="str">
-        <x:v>Taproot PSBT fields extend the base PSBT container, so learners need the general workflow and field model before the Taproot additions make sense.</x:v>
+        <x:v>TapTweak is defined using tagged hashes directly in Taproot key tweaking.</x:v>
       </x:c>
       <x:c r="F19" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G19" s="32" t="str">
-        <x:v>Direct edge keeps the slice anchored on the generic PSBT exchange model rather than on a narrower implementation variant.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.x-only-public-keys</x:v>
       </x:c>
       <x:c r="B20" s="32" t="str">
-        <x:v>dev.taproot-psbt-fields</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="C20" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11201,21 +11795,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E20" s="32" t="str">
-        <x:v>These fields carry Taproot-specific keys, scripts, and Merkle-path data, so learners need the Taproot spend model before the PSBT extensions are meaningful.</x:v>
+        <x:v>TapTweak operates on x-only public keys in the Taproot construction.</x:v>
       </x:c>
       <x:c r="F20" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G20" s="32" t="str">
-        <x:v>The direct dev.psbt-v2 edge was intentionally dropped because BIP371 applies to PSBTv0 and PSBTv2.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="str">
-        <x:v>protocol.softfork-hardfork</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="B21" s="32" t="str">
-        <x:v>protocol.accidental-confiscation</x:v>
+        <x:v>protocol.taproot-key-path-spends</x:v>
       </x:c>
       <x:c r="C21" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11224,21 +11818,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E21" s="32" t="str">
-        <x:v>Accidental confiscation is a failure mode caused by new soft-fork restrictions, so learners need the soft-fork compatibility model before the risk is intelligible.</x:v>
+        <x:v>A key-path spend verifies against the tweaked Taproot output key, so learners need the tweak mechanism before the spending mode makes sense.</x:v>
       </x:c>
       <x:c r="F21" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G21" s="32" t="str">
-        <x:v>Direct edge chosen over chain-split-risk and standardness-policy because those branches add context but are not required for the core failure mode.</x:v>
+        <x:v>Direct parent keeps the node focused on the spend mode rather than on broad Taproot overview material.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32" t="str">
-        <x:v>protocol.fee-market</x:v>
+        <x:v>protocol.taptree</x:v>
       </x:c>
       <x:c r="B22" s="32" t="str">
-        <x:v>custody.coin-selection</x:v>
+        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
       </x:c>
       <x:c r="C22" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11247,21 +11841,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E22" s="32" t="str">
-        <x:v>Wallets choose different UTXO sets partly to minimize transaction size and fee cost, so fee pressure is a direct part of the concept.</x:v>
+        <x:v>The inclusion proof only makes sense after the learner understands the TapTree structure.</x:v>
       </x:c>
       <x:c r="F22" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G22" s="32" t="str">
-        <x:v>Direct edge keeps the node connected to transaction-cost tradeoffs rather than only to wallet UX.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>protocol.taptree</x:v>
       </x:c>
       <x:c r="B23" s="32" t="str">
-        <x:v>protocol.change-outputs</x:v>
+        <x:v>protocol.huffman-optimized-taptrees</x:v>
       </x:c>
       <x:c r="C23" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11270,21 +11864,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E23" s="32" t="str">
-        <x:v>Change is a specific kind of transaction output, so learners need the basic output and spendability model before the leftover-value pattern makes sense.</x:v>
+        <x:v>Huffman optimization is a refinement of how TapTree leaves are arranged.</x:v>
       </x:c>
       <x:c r="F23" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G23" s="32" t="str">
-        <x:v>Direct edge keeps the node between raw output structure and the later wallet-decision branch.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>protocol.softfork-hardfork</x:v>
       </x:c>
       <x:c r="B24" s="32" t="str">
-        <x:v>dev.taproot-descriptors</x:v>
+        <x:v>protocol.chain-split-risk</x:v>
       </x:c>
       <x:c r="C24" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11293,13 +11887,13 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E24" s="32" t="str">
-        <x:v>Taproot descriptors extend the general descriptor grammar, so learners need the base descriptor model before the tr() specialization makes sense.</x:v>
+        <x:v>Split risk is a downstream consequence of incompatible upgrade paths, so learners should understand the compatibility boundary first.</x:v>
       </x:c>
       <x:c r="F24" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G24" s="32" t="str">
-        <x:v>Direct edge keeps the node scoped to descriptor structure instead of wallet import behavior.</x:v>
+        <x:v>Direct edge chosen over activation-history case studies because those are downstream examples, not prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -11307,7 +11901,7 @@
         <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B25" s="32" t="str">
-        <x:v>dev.taproot-descriptors</x:v>
+        <x:v>protocol.tapscript</x:v>
       </x:c>
       <x:c r="C25" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11316,21 +11910,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E25" s="32" t="str">
-        <x:v>The tr() descriptor exists specifically to encode P2TR outputs and optional Taproot script-path commitments, so learners need the Taproot output model first.</x:v>
+        <x:v>Tapscript is a Taproot-specific script version, so learners need the Taproot spend context before its rule changes make sense.</x:v>
       </x:c>
       <x:c r="F25" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G25" s="32" t="str">
-        <x:v>Direct edge keeps the node grounded in Taproot output semantics rather than in generic descriptor syntax alone.</x:v>
+        <x:v>Direct edge keeps the node scoped to the Taproot family without collapsing it into a generic script refresher.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="str">
-        <x:v>protocol.transaction-pinning</x:v>
+        <x:v>custody.psbt</x:v>
       </x:c>
       <x:c r="B26" s="32" t="str">
-        <x:v>protocol.version-3-transaction-relay</x:v>
+        <x:v>dev.taproot-psbt-fields</x:v>
       </x:c>
       <x:c r="C26" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11339,21 +11933,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E26" s="32" t="str">
-        <x:v>Version 3 relay is a targeted policy response to transaction pinning, so learners should understand the attack class before the mitigation.</x:v>
+        <x:v>Taproot PSBT fields extend the base PSBT container, so learners need the general workflow and field model before the Taproot additions make sense.</x:v>
       </x:c>
       <x:c r="F26" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G26" s="32" t="str">
-        <x:v>Direct edge chosen over package-relay because the pinning problem is the narrower immediate teaching need.</x:v>
+        <x:v>Direct edge keeps the slice anchored on the generic PSBT exchange model rather than on a narrower implementation variant.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="str">
-        <x:v>fundamentals.trustlessness</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B27" s="32" t="str">
-        <x:v>fundamentals.validation-sovereignty</x:v>
+        <x:v>dev.taproot-psbt-fields</x:v>
       </x:c>
       <x:c r="C27" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11362,21 +11956,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E27" s="32" t="str">
-        <x:v>Validation sovereignty is an applied consequence of trustlessness and verification culture.</x:v>
+        <x:v>These fields carry Taproot-specific keys, scripts, and Merkle-path data, so learners need the Taproot spend model before the PSBT extensions are meaningful.</x:v>
       </x:c>
       <x:c r="F27" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G27" s="32" t="str">
-        <x:v>Bridge edge inferred from philosophy sequencing.</x:v>
+        <x:v>The direct dev.psbt-v2 edge was intentionally dropped because BIP371 applies to PSBTv0 and PSBTv2.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32" t="str">
-        <x:v>ops.run-full-node</x:v>
+        <x:v>protocol.softfork-hardfork</x:v>
       </x:c>
       <x:c r="B28" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>protocol.accidental-confiscation</x:v>
       </x:c>
       <x:c r="C28" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11385,21 +11979,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E28" s="32" t="str">
-        <x:v>Learners need the full-node baseline before they can understand which validation guarantees a light client gives up.</x:v>
+        <x:v>Accidental confiscation is a failure mode caused by new soft-fork restrictions, so learners need the soft-fork compatibility model before the risk is intelligible.</x:v>
       </x:c>
       <x:c r="F28" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G28" s="32" t="str">
-        <x:v>Bridge edge inferred from full-node versus lightweight-client contrast.</x:v>
+        <x:v>Direct edge chosen over chain-split-risk and standardness-policy because those branches add context but are not required for the core failure mode.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="32" t="str">
-        <x:v>protocol.compact-block-filters</x:v>
+        <x:v>protocol.fee-market</x:v>
       </x:c>
       <x:c r="B29" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>custody.coin-selection</x:v>
       </x:c>
       <x:c r="C29" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11408,21 +12002,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E29" s="32" t="str">
-        <x:v>Compact block filters provide the modern filtered-client mechanism that anchors the trust-model comparison.</x:v>
+        <x:v>Wallets choose different UTXO sets partly to minimize transaction size and fee cost, so fee pressure is a direct part of the concept.</x:v>
       </x:c>
       <x:c r="F29" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G29" s="32" t="str">
-        <x:v>Kept additive and conceptual instead of rewiring older light-client mechanism leaves in the same slice.</x:v>
+        <x:v>Direct edge keeps the node connected to transaction-cost tradeoffs rather than only to wallet UX.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32" t="str">
-        <x:v>fundamentals.validation-sovereignty</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B30" s="32" t="str">
-        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
+        <x:v>protocol.change-outputs</x:v>
       </x:c>
       <x:c r="C30" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11431,21 +12025,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E30" s="32" t="str">
-        <x:v>The comparison only matters once the learner understands why self-validation is valuable in the first place.</x:v>
+        <x:v>Change is a specific kind of transaction output, so learners need the basic output and spendability model before the leftover-value pattern makes sense.</x:v>
       </x:c>
       <x:c r="F30" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G30" s="32" t="str">
-        <x:v>User-facing prerequisite edge for the wallet-mode decision.</x:v>
+        <x:v>Direct edge keeps the node between raw output structure and the later wallet-decision branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B31" s="32" t="str">
-        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
+        <x:v>dev.taproot-descriptors</x:v>
       </x:c>
       <x:c r="C31" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11454,21 +12048,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E31" s="32" t="str">
-        <x:v>Learners need the mechanism-level trust tradeoffs before comparing full-node wallets with lightweight clients.</x:v>
+        <x:v>Taproot descriptors extend the general descriptor grammar, so learners need the base descriptor model before the tr() specialization makes sense.</x:v>
       </x:c>
       <x:c r="F31" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G31" s="32" t="str">
-        <x:v>First downstream consumer for the light-client trust branch.</x:v>
+        <x:v>Direct edge keeps the node scoped to descriptor structure instead of wallet import behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B32" s="32" t="str">
-        <x:v>protocol.p2pk</x:v>
+        <x:v>dev.taproot-descriptors</x:v>
       </x:c>
       <x:c r="C32" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11477,21 +12071,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E32" s="32" t="str">
-        <x:v>P2PK is a concrete legacy script template, so learners first need the locking and unlocking model from Bitcoin Script.</x:v>
+        <x:v>The tr() descriptor exists specifically to encode P2TR outputs and optional Taproot script-path commitments, so learners need the Taproot output model first.</x:v>
       </x:c>
       <x:c r="F32" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G32" s="32" t="str">
-        <x:v>Chosen as the first script-history leaf from Decoding after dedupe and direct-edge review.</x:v>
+        <x:v>Direct edge keeps the node grounded in Taproot output semantics rather than in generic descriptor syntax alone.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="32" t="str">
-        <x:v>fundamentals.schnorr-signatures</x:v>
+        <x:v>protocol.transaction-pinning</x:v>
       </x:c>
       <x:c r="B33" s="32" t="str">
-        <x:v>security.nonce-reuse-attack</x:v>
+        <x:v>protocol.version-3-transaction-relay</x:v>
       </x:c>
       <x:c r="C33" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11500,21 +12094,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E33" s="32" t="str">
-        <x:v>The nonce-reuse failure only makes sense after the learner understands the Schnorr signing flow that produces the nonce and signature pair.</x:v>
+        <x:v>Version 3 relay is a targeted policy response to transaction pinning, so learners should understand the attack class before the mitigation.</x:v>
       </x:c>
       <x:c r="F33" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G33" s="32" t="str">
-        <x:v>Chosen as a narrow additive security slice without bundling it to custody-side defenses.</x:v>
+        <x:v>Direct edge chosen over package-relay because the pinning problem is the narrower immediate teaching need.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="32" t="str">
-        <x:v>protocol.p2pk</x:v>
+        <x:v>fundamentals.trustlessness</x:v>
       </x:c>
       <x:c r="B34" s="32" t="str">
-        <x:v>protocol.p2pkh</x:v>
+        <x:v>fundamentals.validation-sovereignty</x:v>
       </x:c>
       <x:c r="C34" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11523,21 +12117,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E34" s="32" t="str">
-        <x:v>P2PKH is easiest to understand as the hashed-public-key refinement of a direct public-key output.</x:v>
+        <x:v>Validation sovereignty is an applied consequence of trustlessness and verification culture.</x:v>
       </x:c>
       <x:c r="F34" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G34" s="32" t="str">
-        <x:v>Chosen to preserve the output-template ladder without repeating the broader Script prerequisite directly.</x:v>
+        <x:v>Bridge edge inferred from philosophy sequencing.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>ops.run-full-node</x:v>
       </x:c>
       <x:c r="B35" s="32" t="str">
-        <x:v>protocol.p2pkh</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="C35" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11546,21 +12140,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E35" s="32" t="str">
-        <x:v>Hash-based locking only makes sense once the learner understands what a hash commits to and why it can stand in for the public key until spend time.</x:v>
+        <x:v>Learners need the full-node baseline before they can understand which validation guarantees a light client gives up.</x:v>
       </x:c>
       <x:c r="F35" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G35" s="32" t="str">
-        <x:v>Required to keep the node about public-key hashing rather than just script syntax.</x:v>
+        <x:v>Bridge edge inferred from full-node versus lightweight-client contrast.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>protocol.compact-block-filters</x:v>
       </x:c>
       <x:c r="B36" s="32" t="str">
-        <x:v>protocol.op-checkmultisig</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="C36" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11569,21 +12163,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E36" s="32" t="str">
-        <x:v>OP_CHECKMULTISIG is an opcode-level script mechanic, so learners first need the general Script model and stack execution basics.</x:v>
+        <x:v>Compact block filters provide the modern filtered-client mechanism that anchors the trust-model comparison.</x:v>
       </x:c>
       <x:c r="F36" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G36" s="32" t="str">
-        <x:v>Chosen as the mechanism bridge before protocol.p2ms.</x:v>
+        <x:v>Kept additive and conceptual instead of rewiring older light-client mechanism leaves in the same slice.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="32" t="str">
-        <x:v>protocol.op-checkmultisig</x:v>
+        <x:v>fundamentals.validation-sovereignty</x:v>
       </x:c>
       <x:c r="B37" s="32" t="str">
-        <x:v>protocol.p2ms</x:v>
+        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
       </x:c>
       <x:c r="C37" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11592,21 +12186,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E37" s="32" t="str">
-        <x:v>Bare multisig is the concrete locking template built from OP_CHECKMULTISIG, so the opcode is the clean direct parent once introduced.</x:v>
+        <x:v>The comparison only matters once the learner understands why self-validation is valuable in the first place.</x:v>
       </x:c>
       <x:c r="F37" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G37" s="32" t="str">
-        <x:v>Replaces the earlier curricular and wallet-semantic parent candidates.</x:v>
+        <x:v>User-facing prerequisite edge for the wallet-mode decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="32" t="str">
-        <x:v>protocol.p2ms</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="B38" s="32" t="str">
-        <x:v>protocol.bare-multisig-standardness</x:v>
+        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
       </x:c>
       <x:c r="C38" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11615,21 +12209,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E38" s="32" t="str">
-        <x:v>The relay treatment only makes sense once the learner understands what a bare multisig output actually is on-chain.</x:v>
+        <x:v>Learners need the mechanism-level trust tradeoffs before comparing full-node wallets with lightweight clients.</x:v>
       </x:c>
       <x:c r="F38" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G38" s="32" t="str">
-        <x:v>Policy leaf anchored on the specific legacy script template it constrains.</x:v>
+        <x:v>First downstream consumer for the light-client trust branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="32" t="str">
-        <x:v>protocol.standardness-policy</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B39" s="32" t="str">
-        <x:v>protocol.bare-multisig-standardness</x:v>
+        <x:v>protocol.p2pk</x:v>
       </x:c>
       <x:c r="C39" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11638,21 +12232,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E39" s="32" t="str">
-        <x:v>This node is a concrete application of standard transaction policy, so the general standardness concept should come first.</x:v>
+        <x:v>P2PK is a concrete legacy script template, so learners first need the locking and unlocking model from Bitcoin Script.</x:v>
       </x:c>
       <x:c r="F39" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G39" s="32" t="str">
-        <x:v>Policy-boundary prerequisite inherited through the existing mempool-policy branch.</x:v>
+        <x:v>Chosen as the first script-history leaf from Decoding after dedupe and direct-edge review.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="B40" s="32" t="str">
-        <x:v>dev.scriptpubkeymanagers</x:v>
+        <x:v>security.nonce-reuse-attack</x:v>
       </x:c>
       <x:c r="C40" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11661,21 +12255,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E40" s="32" t="str">
-        <x:v>Modern descriptor wallets hand descriptor-backed script templates to dedicated managers, so learners need the descriptor model before the SPKM boundary makes sense.</x:v>
+        <x:v>The nonce-reuse failure only makes sense after the learner understands the Schnorr signing flow that produces the nonce and signature pair.</x:v>
       </x:c>
       <x:c r="F40" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-wallet</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G40" s="32" t="str">
-        <x:v>Direct edge distinguishes the Core wallet abstraction from descriptor syntax without collapsing the two concepts into one node.</x:v>
+        <x:v>Chosen as a narrow additive security slice without bundling it to custody-side defenses.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32" t="str">
-        <x:v>protocol.mempool</x:v>
+        <x:v>protocol.p2pk</x:v>
       </x:c>
       <x:c r="B41" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>protocol.p2pkh</x:v>
       </x:c>
       <x:c r="C41" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11684,21 +12278,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E41" s="32" t="str">
-        <x:v>The unbroadcast set is a mempool-owned data structure, so learners need the local unconfirmed transaction pool model before this narrower tracking mechanism makes sense.</x:v>
+        <x:v>P2PKH is easiest to understand as the hashed-public-key refinement of a direct public-key output.</x:v>
       </x:c>
       <x:c r="F41" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G41" s="32" t="str">
-        <x:v>Direct edge keeps the concept scoped to local transaction state rather than broader relay policy.</x:v>
+        <x:v>Chosen to preserve the output-template ladder without repeating the broader Script prerequisite directly.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="32" t="str">
-        <x:v>protocol.transaction-relay-inv-getdata</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B42" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>protocol.p2pkh</x:v>
       </x:c>
       <x:c r="C42" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11707,21 +12301,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E42" s="32" t="str">
-        <x:v>This set only matters because nodes need to distinguish locally submitted transactions from those later observed through the network relay path and may retry announcing them.</x:v>
+        <x:v>Hash-based locking only makes sense once the learner understands what a hash commits to and why it can stand in for the public key until spend time.</x:v>
       </x:c>
       <x:c r="F42" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G42" s="32" t="str">
-        <x:v>Direct edge ties the mechanism to network propagation confirmation and rebroadcast attempts.</x:v>
+        <x:v>Required to keep the node about public-key hashing rather than just script syntax.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="32" t="str">
-        <x:v>privacy.address-reuse</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B43" s="32" t="str">
-        <x:v>custody.human-readable-addresses</x:v>
+        <x:v>protocol.op-checkmultisig</x:v>
       </x:c>
       <x:c r="C43" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11730,21 +12324,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E43" s="32" t="str">
-        <x:v>A major design constraint is that reusable human-readable handles can worsen privacy unless they resolve to reusable payment mechanisms or rotate safely, so learners need the address-reuse problem first.</x:v>
+        <x:v>OP_CHECKMULTISIG is an opcode-level script mechanic, so learners first need the general Script model and stack execution basics.</x:v>
       </x:c>
       <x:c r="F43" s="32" t="str">
-        <x:v>source.bitcoin-design-payment-formats</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G43" s="32" t="str">
-        <x:v>Direct edge captures the main privacy tradeoff without forcing downstream protocol-specific address schemes into prerequisites.</x:v>
+        <x:v>Chosen as the mechanism bridge before protocol.p2ms.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="32" t="str">
-        <x:v>custody.output-labeling</x:v>
+        <x:v>protocol.op-checkmultisig</x:v>
       </x:c>
       <x:c r="B44" s="32" t="str">
-        <x:v>custody.transaction-metadata</x:v>
+        <x:v>protocol.p2ms</x:v>
       </x:c>
       <x:c r="C44" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11753,21 +12347,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E44" s="32" t="str">
-        <x:v>Output labeling already introduces the idea that wallets attach their own context to payments and spendable objects, making it the cleanest direct bridge into broader transaction-level notes, contacts, and portability concerns.</x:v>
+        <x:v>Bare multisig is the concrete locking template built from OP_CHECKMULTISIG, so the opcode is the clean direct parent once introduced.</x:v>
       </x:c>
       <x:c r="F44" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G44" s="32" t="str">
-        <x:v>Direct edge distinguishes wider payment-history context from narrower spend-control labels without treating them as unrelated.</x:v>
+        <x:v>Replaces the earlier curricular and wallet-semantic parent candidates.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>protocol.p2ms</x:v>
       </x:c>
       <x:c r="B45" s="32" t="str">
-        <x:v>custody.transaction-metadata</x:v>
+        <x:v>protocol.bare-multisig-standardness</x:v>
       </x:c>
       <x:c r="C45" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11776,21 +12370,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E45" s="32" t="str">
-        <x:v>Wallet-added names, notes, and contact links matter partly because transaction history is only pseudonymous and can reveal meaningful patterns when users or tools correlate activity over time.</x:v>
+        <x:v>The relay treatment only makes sense once the learner understands what a bare multisig output actually is on-chain.</x:v>
       </x:c>
       <x:c r="F45" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G45" s="32" t="str">
-        <x:v>Direct edge keeps the node tied to the privacy and identity meaning of payment history rather than only to generic lifecycle sequencing.</x:v>
+        <x:v>Policy leaf anchored on the specific legacy script template it constrains.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="32" t="str">
-        <x:v>custody.self-custody</x:v>
+        <x:v>protocol.standardness-policy</x:v>
       </x:c>
       <x:c r="B46" s="32" t="str">
-        <x:v>custody.multiple-wallets</x:v>
+        <x:v>protocol.bare-multisig-standardness</x:v>
       </x:c>
       <x:c r="C46" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11799,21 +12393,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E46" s="32" t="str">
-        <x:v>Deliberately separating funds across different wallet buckets is a custody decision, so learners need the base self-custody responsibility model before the organizational pattern makes sense.</x:v>
+        <x:v>This node is a concrete application of standard transaction policy, so the general standardness concept should come first.</x:v>
       </x:c>
       <x:c r="F46" s="32" t="str">
-        <x:v>source.bitcoin-design-multiple-wallets</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G46" s="32" t="str">
-        <x:v>Kept the direct parent at the responsibility-model layer; multisig, watch-only, and HD account structures remain examples or implementation details rather than prerequisites.</x:v>
+        <x:v>Policy-boundary prerequisite inherited through the existing mempool-policy branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="32" t="str">
-        <x:v>custody.hardware-wallets</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B47" s="32" t="str">
-        <x:v>custody.progressive-security</x:v>
+        <x:v>dev.scriptpubkeymanagers</x:v>
       </x:c>
       <x:c r="C47" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11822,21 +12416,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E47" s="32" t="str">
-        <x:v>One of the core upgrade steps in the reference design is moving from default low-friction storage to an external signing device, so learners need the hardware-signing model before the staged-upgrade pattern makes sense.</x:v>
+        <x:v>Modern descriptor wallets hand descriptor-backed script templates to dedicated managers, so learners need the descriptor model before the SPKM boundary makes sense.</x:v>
       </x:c>
       <x:c r="F47" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoin-core-academy-wallet</x:v>
       </x:c>
       <x:c r="G47" s="32" t="str">
-        <x:v>Direct edge captures the mid-tier upgrade target without treating cloud backup itself as the core concept.</x:v>
+        <x:v>Direct edge distinguishes the Core wallet abstraction from descriptor syntax without collapsing the two concepts into one node.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>protocol.mempool</x:v>
       </x:c>
       <x:c r="B48" s="32" t="str">
-        <x:v>custody.progressive-security</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="C48" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11845,21 +12439,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E48" s="32" t="str">
-        <x:v>The higher-security end of the progression moves into 2-of-3 and 3-of-5 multi-key schemes, so learners need the multisig model before they can reason about why and when a wallet should escalate there.</x:v>
+        <x:v>The unbroadcast set is a mempool-owned data structure, so learners need the local unconfirmed transaction pool model before this narrower tracking mechanism makes sense.</x:v>
       </x:c>
       <x:c r="F48" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G48" s="32" t="str">
-        <x:v>Direct edge captures the high-assurance destination of the progression rather than a specific product flow.</x:v>
+        <x:v>Direct edge keeps the concept scoped to local transaction state rather than broader relay policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="32" t="str">
+        <x:v>protocol.transaction-relay-inv-getdata</x:v>
+      </x:c>
+      <x:c r="B49" s="32" t="str">
         <x:v>protocol.mempool-unbroadcast-set</x:v>
-      </x:c>
-      <x:c r="B49" s="32" t="str">
-        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
       </x:c>
       <x:c r="C49" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11868,21 +12462,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E49" s="32" t="str">
-        <x:v>Rebroadcast privacy builds directly on the local-node distinction between transactions merely accepted into the mempool and transactions known to have propagated, which is exactly the gap the unbroadcast set tracks.</x:v>
+        <x:v>This set only matters because nodes need to distinguish locally submitted transactions from those later observed through the network relay path and may retry announcing them.</x:v>
       </x:c>
       <x:c r="F49" s="32" t="str">
         <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G49" s="32" t="str">
-        <x:v>Direct parent keeps the slice on the local tracking mechanism rather than reintroducing generic relay ancestors.</x:v>
+        <x:v>Direct edge ties the mechanism to network propagation confirmation and rebroadcast attempts.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>privacy.address-reuse</x:v>
       </x:c>
       <x:c r="B50" s="32" t="str">
-        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
+        <x:v>custody.human-readable-addresses</x:v>
       </x:c>
       <x:c r="C50" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11891,21 +12485,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E50" s="32" t="str">
-        <x:v>Different rebroadcast patterns matter because observers can correlate network behavior with public transaction history and infer likely origin, so learners need the pseudonymity and linkage problem first.</x:v>
+        <x:v>A major design constraint is that reusable human-readable handles can worsen privacy unless they resolve to reusable payment mechanisms or rotate safely, so learners need the address-reuse problem first.</x:v>
       </x:c>
       <x:c r="F50" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-payment-formats</x:v>
       </x:c>
       <x:c r="G50" s="32" t="str">
-        <x:v>Direct parent keeps the node focused on why relay-side origin leakage matters, not just how rebroadcast code works.</x:v>
+        <x:v>Direct edge captures the main privacy tradeoff without forcing downstream protocol-specific address schemes into prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="32" t="str">
-        <x:v>protocol.segregated-witness</x:v>
+        <x:v>custody.output-labeling</x:v>
       </x:c>
       <x:c r="B51" s="32" t="str">
-        <x:v>protocol.txid-vs-wtxid</x:v>
+        <x:v>custody.transaction-metadata</x:v>
       </x:c>
       <x:c r="C51" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11914,21 +12508,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E51" s="32" t="str">
-        <x:v>The identifier split only exists because SegWit introduces a witness-inclusive serialization alongside the legacy serialization, so learners need the SegWit structure change before the two IDs make sense.</x:v>
+        <x:v>Output labeling already introduces the idea that wallets attach their own context to payments and spendable objects, making it the cleanest direct bridge into broader transaction-level notes, contacts, and portability concerns.</x:v>
       </x:c>
       <x:c r="F51" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="G51" s="32" t="str">
-        <x:v>Direct parent keeps the bridge on the serialization distinction instead of reintroducing downstream relay consequences.</x:v>
+        <x:v>Direct edge distinguishes wider payment-history context from narrower spend-control labels without treating them as unrelated.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="32" t="str">
-        <x:v>protocol.txid-vs-wtxid</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B52" s="32" t="str">
-        <x:v>protocol.wtxid-relay-bip339</x:v>
+        <x:v>custody.transaction-metadata</x:v>
       </x:c>
       <x:c r="C52" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11937,21 +12531,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E52" s="32" t="str">
-        <x:v>WTXID relay is specifically the choice to announce and request witness-bearing transactions by wtxid instead of txid, so the learner should understand the two identifier forms before the relay mode change.</x:v>
+        <x:v>Wallet-added names, notes, and contact links matter partly because transaction history is only pseudonymous and can reveal meaningful patterns when users or tools correlate activity over time.</x:v>
       </x:c>
       <x:c r="F52" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="G52" s="32" t="str">
-        <x:v>Added as a graph bridge so the existing relay node no longer has to explain the identifier distinction internally.</x:v>
+        <x:v>Direct edge keeps the node tied to the privacy and identity meaning of payment history rather than only to generic lifecycle sequencing.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="32" t="str">
-        <x:v>fundamentals.schnorr-signatures</x:v>
+        <x:v>custody.self-custody</x:v>
       </x:c>
       <x:c r="B53" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>custody.multiple-wallets</x:v>
       </x:c>
       <x:c r="C53" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11960,21 +12554,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E53" s="32" t="str">
-        <x:v>MuSig is a Schnorr aggregation protocol, so learners need the underlying Schnorr key and signature model before the combined-key protocol makes sense.</x:v>
+        <x:v>Deliberately separating funds across different wallet buckets is a custody decision, so learners need the base self-custody responsibility model before the organizational pattern makes sense.</x:v>
       </x:c>
       <x:c r="F53" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-design-multiple-wallets</x:v>
       </x:c>
       <x:c r="G53" s="32" t="str">
-        <x:v>Direct parent kept narrow; wallet-level multisig and Taproot remain context rather than prerequisites.</x:v>
+        <x:v>Kept the direct parent at the responsibility-model layer; multisig, watch-only, and HD account structures remain examples or implementation details rather than prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>custody.hardware-wallets</x:v>
       </x:c>
       <x:c r="B54" s="32" t="str">
-        <x:v>dev.descriptor-wallet-policies</x:v>
+        <x:v>custody.progressive-security</x:v>
       </x:c>
       <x:c r="C54" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11983,21 +12577,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E54" s="32" t="str">
-        <x:v>Wallet policies are built as descriptor templates, so the base descriptor language and template structure must come first.</x:v>
+        <x:v>One of the core upgrade steps in the reference design is moving from default low-friction storage to an external signing device, so learners need the hardware-signing model before the staged-upgrade pattern makes sense.</x:v>
       </x:c>
       <x:c r="F54" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="G54" s="32" t="str">
-        <x:v>Direct parent kept above import or signer flows because the node is about the representation itself.</x:v>
+        <x:v>Direct edge captures the mid-tier upgrade target without treating cloud backup itself as the core concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="32" t="str">
-        <x:v>dev.bip32</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B55" s="32" t="str">
-        <x:v>dev.descriptor-wallet-policies</x:v>
+        <x:v>custody.progressive-security</x:v>
       </x:c>
       <x:c r="C55" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12006,21 +12600,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E55" s="32" t="str">
-        <x:v>BIP388 key information items package xpubs and derivation origins, so learners need the HD derivation model before the portable wallet-policy format makes sense.</x:v>
+        <x:v>The higher-security end of the progression moves into 2-of-3 and 3-of-5 multi-key schemes, so learners need the multisig model before they can reason about why and when a wallet should escalate there.</x:v>
       </x:c>
       <x:c r="F55" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="G55" s="32" t="str">
-        <x:v>Non-redundant alongside dev.descriptors because neither concept implies the other in the current graph.</x:v>
+        <x:v>Direct edge captures the high-assurance destination of the progression rather than a specific product flow.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="B56" s="32" t="str">
-        <x:v>dev.descriptors-in-psbt</x:v>
+        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
       </x:c>
       <x:c r="C56" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12029,21 +12623,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E56" s="32" t="str">
-        <x:v>The node is about carrying descriptor information during transaction coordination, so learners need the descriptor syntax and script-template model first.</x:v>
+        <x:v>Rebroadcast privacy builds directly on the local-node distinction between transactions merely accepted into the mempool and transactions known to have propagated, which is exactly the gap the unbroadcast set tracks.</x:v>
       </x:c>
       <x:c r="F56" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G56" s="32" t="str">
-        <x:v>Direct parent kept at the representation layer rather than the wallet-policy or taproot-specific refinements.</x:v>
+        <x:v>Direct parent keeps the slice on the local tracking mechanism rather than reintroducing generic relay ancestors.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="32" t="str">
-        <x:v>custody.psbt</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B57" s="32" t="str">
-        <x:v>dev.descriptors-in-psbt</x:v>
+        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
       </x:c>
       <x:c r="C57" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12052,21 +12646,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E57" s="32" t="str">
-        <x:v>Descriptor-aware exchange only makes sense after the learner understands the general PSBT coordination workflow that transports signing-related data between tools.</x:v>
+        <x:v>Different rebroadcast patterns matter because observers can correlate network behavior with public transaction history and infer likely origin, so learners need the pseudonymity and linkage problem first.</x:v>
       </x:c>
       <x:c r="F57" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G57" s="32" t="str">
-        <x:v>Direct parent kept at the base PSBT workflow level instead of requiring later version-specific extensions.</x:v>
+        <x:v>Direct parent keeps the node focused on why relay-side origin leakage matters, not just how rebroadcast code works.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>protocol.segregated-witness</x:v>
       </x:c>
       <x:c r="B58" s="32" t="str">
-        <x:v>custody.degrading-multisig</x:v>
+        <x:v>protocol.txid-vs-wtxid</x:v>
       </x:c>
       <x:c r="C58" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12075,21 +12669,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E58" s="32" t="str">
-        <x:v>The policy only makes sense once the learner understands ordinary multisig threshold custody and why signers can be split into live and backup sets.</x:v>
+        <x:v>The identifier split only exists because SegWit introduces a witness-inclusive serialization alongside the legacy serialization, so learners need the SegWit structure change before the two IDs make sense.</x:v>
       </x:c>
       <x:c r="F58" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G58" s="32" t="str">
-        <x:v>Direct custody parent for the signer-threshold side of the construction.</x:v>
+        <x:v>Direct parent keeps the bridge on the serialization distinction instead of reintroducing downstream relay consequences.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="32" t="str">
-        <x:v>protocol.timelocks</x:v>
+        <x:v>protocol.txid-vs-wtxid</x:v>
       </x:c>
       <x:c r="B59" s="32" t="str">
-        <x:v>custody.degrading-multisig</x:v>
+        <x:v>protocol.wtxid-relay-bip339</x:v>
       </x:c>
       <x:c r="C59" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12098,21 +12692,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E59" s="32" t="str">
-        <x:v>The degrading policy activates its weaker backup path only after a timeout, so timelock semantics are a direct part of the construction.</x:v>
+        <x:v>WTXID relay is specifically the choice to announce and request witness-bearing transactions by wtxid instead of txid, so the learner should understand the two identifier forms before the relay mode change.</x:v>
       </x:c>
       <x:c r="F59" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G59" s="32" t="str">
-        <x:v>Needed alongside custody.multisig because the learner must understand the temporal rule, not just the signer policy.</x:v>
+        <x:v>Added as a graph bridge so the existing relay node no longer has to explain the identifier distinction internally.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="32" t="str">
-        <x:v>protocol.block-weight-vbytes</x:v>
+        <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="B60" s="32" t="str">
-        <x:v>protocol.fee-calculation</x:v>
+        <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="C60" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12121,21 +12715,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E60" s="32" t="str">
-        <x:v>Understanding whether an absolute fee is high or low requires relating it to the blockspace pricing unit, so learners need weight and virtual bytes before fee calculation is fully meaningful in practice.</x:v>
+        <x:v>MuSig is a Schnorr aggregation protocol, so learners need the underlying Schnorr key and signature model before the combined-key protocol makes sense.</x:v>
       </x:c>
       <x:c r="F60" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G60" s="32" t="str">
-        <x:v>Direct parent keeps the node at the mechanism layer without drifting into broader fee-market competition.</x:v>
+        <x:v>Direct parent kept narrow; wallet-level multisig and Taproot remain context rather than prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B61" s="32" t="str">
-        <x:v>protocol.bech32m-addresses</x:v>
+        <x:v>dev.descriptor-wallet-policies</x:v>
       </x:c>
       <x:c r="C61" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12144,21 +12738,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E61" s="32" t="str">
-        <x:v>Bech32m is an address-encoding format, so learners need the general relationship between addresses, script templates, and spendability before the newer checksum format is meaningful.</x:v>
+        <x:v>Wallet policies are built as descriptor templates, so the base descriptor language and template structure must come first.</x:v>
       </x:c>
       <x:c r="F61" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G61" s="32" t="str">
-        <x:v>Direct parent keeps the node on encoding semantics rather than on raw string-format trivia.</x:v>
+        <x:v>Direct parent kept above import or signer flows because the node is about the representation itself.</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>dev.bip32</x:v>
       </x:c>
       <x:c r="B62" s="32" t="str">
-        <x:v>protocol.bech32m-addresses</x:v>
+        <x:v>dev.descriptor-wallet-policies</x:v>
       </x:c>
       <x:c r="C62" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12167,21 +12761,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E62" s="32" t="str">
-        <x:v>Bech32m became necessary for witness version 1 and higher, and Taproot is the first major deployed witness-v1 use case, so learners need that upgrade context before the format distinction makes sense.</x:v>
+        <x:v>BIP388 key information items package xpubs and derivation origins, so learners need the HD derivation model before the portable wallet-policy format makes sense.</x:v>
       </x:c>
       <x:c r="F62" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G62" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored on the practical protocol transition that exposed Bech32m to users.</x:v>
+        <x:v>Non-redundant alongside dev.descriptors because neither concept implies the other in the current graph.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B63" s="32" t="str">
-        <x:v>protocol.script-execution-stack</x:v>
+        <x:v>dev.descriptors-in-psbt</x:v>
       </x:c>
       <x:c r="C63" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12190,21 +12784,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E63" s="32" t="str">
-        <x:v>The stack execution model is the direct mechanism by which Bitcoin Script evaluates spending conditions, so learners need the umbrella Script concept before drilling into stack behavior.</x:v>
+        <x:v>The node is about carrying descriptor information during transaction coordination, so learners need the descriptor syntax and script-template model first.</x:v>
       </x:c>
       <x:c r="F63" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G63" s="32" t="str">
-        <x:v>Direct parent positions the node as the conceptual middle layer between Script and opcode-specific leaves.</x:v>
+        <x:v>Direct parent kept at the representation layer rather than the wallet-policy or taproot-specific refinements.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="32" t="str">
-        <x:v>lightning.commitment-transactions</x:v>
+        <x:v>custody.psbt</x:v>
       </x:c>
       <x:c r="B64" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>dev.descriptors-in-psbt</x:v>
       </x:c>
       <x:c r="C64" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12213,21 +12807,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E64" s="32" t="str">
-        <x:v>Per-commitment secrets are generated for each new commitment state, so learners need the commitment-transaction model before the secret-rotation mechanism makes sense.</x:v>
+        <x:v>Descriptor-aware exchange only makes sense after the learner understands the general PSBT coordination workflow that transports signing-related data between tools.</x:v>
       </x:c>
       <x:c r="F64" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G64" s="32" t="str">
-        <x:v>Direct parent keeps the node on state evolution rather than on later punishment or watchtower behavior.</x:v>
+        <x:v>Direct parent kept at the base PSBT workflow level instead of requiring later version-specific extensions.</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B65" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>custody.degrading-multisig</x:v>
       </x:c>
       <x:c r="C65" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12236,21 +12830,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E65" s="32" t="str">
-        <x:v>The to_local and to_remote scripts rely on per-state key derivation, revocation keys, and delayed-payment keys, so learners need the per-commitment secret machinery first.</x:v>
+        <x:v>The policy only makes sense once the learner understands ordinary multisig threshold custody and why signers can be split into live and backup sets.</x:v>
       </x:c>
       <x:c r="F65" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G65" s="32" t="str">
-        <x:v>Direct parent keeps the node at the commitment-key layer instead of collapsing back into the broader commitment-transaction overview.</x:v>
+        <x:v>Direct custody parent for the signer-threshold side of the construction.</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="32" t="str">
-        <x:v>protocol.csv-bip112</x:v>
+        <x:v>protocol.timelocks</x:v>
       </x:c>
       <x:c r="B66" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>custody.degrading-multisig</x:v>
       </x:c>
       <x:c r="C66" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12259,21 +12853,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E66" s="32" t="str">
-        <x:v>The delayed to_local branch is defined by a CSV-enforced waiting period, so learners need the relative-timelock opcode before the script template makes sense.</x:v>
+        <x:v>The degrading policy activates its weaker backup path only after a timeout, so timelock semantics are a direct part of the construction.</x:v>
       </x:c>
       <x:c r="F66" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G66" s="32" t="str">
-        <x:v>Direct parent captures the script-mechanism side of the concept without dragging in broader force-close or HTLC timing behavior.</x:v>
+        <x:v>Needed alongside custody.multisig because the learner must understand the temporal rule, not just the signer policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="32" t="str">
-        <x:v>protocol.difficulty-adjustment</x:v>
+        <x:v>protocol.block-weight-vbytes</x:v>
       </x:c>
       <x:c r="B67" s="32" t="str">
-        <x:v>protocol.time-warp-attack</x:v>
+        <x:v>protocol.fee-calculation</x:v>
       </x:c>
       <x:c r="C67" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12282,21 +12876,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E67" s="32" t="str">
-        <x:v>The attack only makes sense once learners understand how Bitcoin retargets mining difficulty over long block windows.</x:v>
+        <x:v>Understanding whether an absolute fee is high or low requires relating it to the blockspace pricing unit, so learners need weight and virtual bytes before fee calculation is fully meaningful in practice.</x:v>
       </x:c>
       <x:c r="F67" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G67" s="32" t="str">
-        <x:v>Direct parent keeps the exploit tied to the retarget mechanism instead of burying it under generic mining vocabulary.</x:v>
+        <x:v>Direct parent keeps the node at the mechanism layer without drifting into broader fee-market competition.</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="32" t="str">
-        <x:v>protocol.median-time-past</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B68" s="32" t="str">
-        <x:v>protocol.time-warp-attack</x:v>
+        <x:v>protocol.bech32m-addresses</x:v>
       </x:c>
       <x:c r="C68" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12305,21 +12899,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E68" s="32" t="str">
-        <x:v>Learners need the consensus timestamp constraints before they can reason about how miners manipulate time data and where the remaining attack surface lives.</x:v>
+        <x:v>Bech32m is an address-encoding format, so learners need the general relationship between addresses, script templates, and spendability before the newer checksum format is meaningful.</x:v>
       </x:c>
       <x:c r="F68" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G68" s="32" t="str">
-        <x:v>Direct parent captures the timestamp-boundary side of the exploit without overloading timelocks or block headers.</x:v>
+        <x:v>Direct parent keeps the node on encoding semantics rather than on raw string-format trivia.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="32" t="str">
-        <x:v>fundamentals.blind-signatures</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B69" s="32" t="str">
-        <x:v>history.chaumian-ecash</x:v>
+        <x:v>protocol.bech32m-addresses</x:v>
       </x:c>
       <x:c r="C69" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12328,21 +12922,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E69" s="32" t="str">
-        <x:v>Chaumian ecash is defined by using blind signatures to let a mint issue private bearer tokens without seeing the final token contents.</x:v>
+        <x:v>Bech32m became necessary for witness version 1 and higher, and Taproot is the first major deployed witness-v1 use case, so learners need that upgrade context before the format distinction makes sense.</x:v>
       </x:c>
       <x:c r="F69" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G69" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the specific cryptographic mechanism rather than treating it as generic digital-money history.</x:v>
+        <x:v>Direct parent keeps the node anchored on the practical protocol transition that exposed Bech32m to users.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="32" t="str">
-        <x:v>history.double-spend-problem</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B70" s="32" t="str">
-        <x:v>history.chaumian-ecash</x:v>
+        <x:v>protocol.script-execution-stack</x:v>
       </x:c>
       <x:c r="C70" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12351,21 +12945,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E70" s="32" t="str">
-        <x:v>Learners need the unsolved scarcity problem in digital cash before the trusted-mint tradeoff in Chaumian designs becomes meaningful.</x:v>
+        <x:v>The stack execution model is the direct mechanism by which Bitcoin Script evaluates spending conditions, so learners need the umbrella Script concept before drilling into stack behavior.</x:v>
       </x:c>
       <x:c r="F70" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G70" s="32" t="str">
-        <x:v>Direct parent frames why the system still needed a central operator even though it improved privacy.</x:v>
+        <x:v>Direct parent positions the node as the conceptual middle layer between Script and opcode-specific leaves.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="32" t="str">
-        <x:v>economics.history-of-money</x:v>
+        <x:v>lightning.commitment-transactions</x:v>
       </x:c>
       <x:c r="B71" s="32" t="str">
-        <x:v>privacy.secret-right-to-cash</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="C71" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12374,21 +12968,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E71" s="32" t="str">
-        <x:v>The concept depends on understanding how money moved from bearer cash toward mediated account systems, so learners need the long-run monetary history first.</x:v>
+        <x:v>Per-commitment secrets are generated for each new commitment state, so learners need the commitment-transaction model before the secret-rotation mechanism makes sense.</x:v>
       </x:c>
       <x:c r="F71" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G71" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the bearer-versus-intermediated payment shift rather than drifting into generic civil-liberties framing.</x:v>
+        <x:v>Direct parent keeps the node on state evolution rather than on later punishment or watchtower behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="32" t="str">
-        <x:v>fundamentals.censorship-resistance</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="B72" s="32" t="str">
-        <x:v>privacy.secret-right-to-cash</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="C72" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12397,21 +12991,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E72" s="32" t="str">
-        <x:v>Learners need the general idea that payment systems can exclude or block participants before the loss of private cash as a payment right becomes fully meaningful.</x:v>
+        <x:v>The to_local and to_remote scripts rely on per-state key derivation, revocation keys, and delayed-payment keys, so learners need the per-commitment secret machinery first.</x:v>
       </x:c>
       <x:c r="F72" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G72" s="32" t="str">
-        <x:v>Direct parent captures the exclusion-risk side of the argument without reopening broader compliance or surveillance wrappers.</x:v>
+        <x:v>Direct parent keeps the node at the commitment-key layer instead of collapsing back into the broader commitment-transaction overview.</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="32" t="str">
-        <x:v>fundamentals.inflation</x:v>
+        <x:v>protocol.csv-bip112</x:v>
       </x:c>
       <x:c r="B73" s="32" t="str">
-        <x:v>economics.ideal-money</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="C73" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12420,21 +13014,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E73" s="32" t="str">
-        <x:v>The concept is about minimizing monetary distortion, so learners need to understand how inflation changes purchasing power and price signals first.</x:v>
+        <x:v>The delayed to_local branch is defined by a CSV-enforced waiting period, so learners need the relative-timelock opcode before the script template makes sense.</x:v>
       </x:c>
       <x:c r="F73" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G73" s="32" t="str">
-        <x:v>Direct parent captures the measurement-distortion problem that ideal money is trying to avoid.</x:v>
+        <x:v>Direct parent captures the script-mechanism side of the concept without dragging in broader force-close or HTLC timing behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>protocol.difficulty-adjustment</x:v>
       </x:c>
       <x:c r="B74" s="32" t="str">
-        <x:v>protocol.bitcoin-uri-bip21</x:v>
+        <x:v>protocol.time-warp-attack</x:v>
       </x:c>
       <x:c r="C74" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12443,21 +13037,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E74" s="32" t="str">
-        <x:v>The URI is a wrapper around a payment destination and amount, so learners need the underlying address and output model first.</x:v>
+        <x:v>The attack only makes sense once learners understand how Bitcoin retargets mining difficulty over long block windows.</x:v>
       </x:c>
       <x:c r="F74" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G74" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the standard request format rather than collapsing it into higher-level wallet UX systems.</x:v>
+        <x:v>Direct parent keeps the exploit tied to the retarget mechanism instead of burying it under generic mining vocabulary.</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="32" t="str">
-        <x:v>dev.bip32</x:v>
+        <x:v>protocol.median-time-past</x:v>
       </x:c>
       <x:c r="B75" s="32" t="str">
-        <x:v>dev.extended-keys</x:v>
+        <x:v>protocol.time-warp-attack</x:v>
       </x:c>
       <x:c r="C75" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12466,21 +13060,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E75" s="32" t="str">
-        <x:v>Extended keys are one specific export and branch-derivation surface inside the broader BIP32 HD tree model, so learners need the base tree-derivation mechanics first.</x:v>
+        <x:v>Learners need the consensus timestamp constraints before they can reason about how miners manipulate time data and where the remaining attack surface lives.</x:v>
       </x:c>
       <x:c r="F75" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G75" s="32" t="str">
-        <x:v>Direct parent keeps the node inside the HD derivation branch instead of treating xpub or xprv behavior as only a privacy or operational-wallet concept.</x:v>
+        <x:v>Direct parent captures the timestamp-boundary side of the exploit without overloading timelocks or block headers.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="32" t="str">
-        <x:v>dev.extended-keys</x:v>
+        <x:v>fundamentals.blind-signatures</x:v>
       </x:c>
       <x:c r="B76" s="32" t="str">
-        <x:v>dev.hardened-keys</x:v>
+        <x:v>history.chaumian-ecash</x:v>
       </x:c>
       <x:c r="C76" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12489,21 +13083,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E76" s="32" t="str">
-        <x:v>Hardened derivation is a constraint on what an extended public key can derive and on how extended private and public key boundaries behave, so learners need the base xpub/xprv model first.</x:v>
+        <x:v>Chaumian ecash is defined by using blind signatures to let a mint issue private bearer tokens without seeing the final token contents.</x:v>
       </x:c>
       <x:c r="F76" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G76" s="32" t="str">
-        <x:v>Direct parent closes the previously missing branch-level bridge between BIP32 generally and hardened derivation specifically.</x:v>
+        <x:v>Direct parent keeps the node tied to the specific cryptographic mechanism rather than treating it as generic digital-money history.</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>history.double-spend-problem</x:v>
       </x:c>
       <x:c r="B77" s="32" t="str">
-        <x:v>protocol.escrow-and-arbitration</x:v>
+        <x:v>history.chaumian-ecash</x:v>
       </x:c>
       <x:c r="C77" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12512,21 +13106,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E77" s="32" t="str">
-        <x:v>The escrow flow depends on understanding how multiple signers can authorize one spend and why a 2-of-3 threshold changes trust assumptions between buyer, seller, and arbitrator.</x:v>
+        <x:v>Learners need the unsolved scarcity problem in digital cash before the trusted-mint tradeoff in Chaumian designs becomes meaningful.</x:v>
       </x:c>
       <x:c r="F77" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G77" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the threshold-signing contract pattern instead of treating it as generic dispute-resolution theory.</x:v>
+        <x:v>Direct parent frames why the system still needed a central operator even though it improved privacy.</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="32" t="str">
-        <x:v>protocol.pay-to-script-hash</x:v>
+        <x:v>economics.history-of-money</x:v>
       </x:c>
       <x:c r="B78" s="32" t="str">
-        <x:v>protocol.escrow-and-arbitration</x:v>
+        <x:v>privacy.secret-right-to-cash</x:v>
       </x:c>
       <x:c r="C78" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12535,21 +13129,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E78" s="32" t="str">
-        <x:v>The contract uses a P2SH redeem script to hide the multisig spending conditions until spend time, so learners need the P2SH wrapper first.</x:v>
+        <x:v>The concept depends on understanding how money moved from bearer cash toward mediated account systems, so learners need the long-run monetary history first.</x:v>
       </x:c>
       <x:c r="F78" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G78" s="32" t="str">
-        <x:v>Direct parent captures the on-chain contract packaging layer that makes the escrow pattern practical.</x:v>
+        <x:v>Direct parent keeps the node tied to the bearer-versus-intermediated payment shift rather than drifting into generic civil-liberties framing.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>fundamentals.censorship-resistance</x:v>
       </x:c>
       <x:c r="B79" s="32" t="str">
-        <x:v>dev.wallet-import-format-wif</x:v>
+        <x:v>privacy.secret-right-to-cash</x:v>
       </x:c>
       <x:c r="C79" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12558,21 +13152,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E79" s="32" t="str">
-        <x:v>WIF is a serialization format for one private key, so learners need the underlying asymmetric-key concept before the network prefix, checksum, and compression flag details make sense.</x:v>
+        <x:v>Learners need the general idea that payment systems can exclude or block participants before the loss of private cash as a payment right becomes fully meaningful.</x:v>
       </x:c>
       <x:c r="F79" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G79" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored on key material itself instead of overfitting it to address formats or HD wallet hierarchies.</x:v>
+        <x:v>Direct parent captures the exclusion-risk side of the argument without reopening broader compliance or surveillance wrappers.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>fundamentals.inflation</x:v>
       </x:c>
       <x:c r="B80" s="32" t="str">
-        <x:v>mining.pool-shares</x:v>
+        <x:v>economics.ideal-money</x:v>
       </x:c>
       <x:c r="C80" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12581,21 +13175,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E80" s="32" t="str">
-        <x:v>Pool shares only make sense after learners understand why pooled mining exists and why miners need a lower-variance way to prove contributed work before an actual block is found.</x:v>
+        <x:v>The concept is about minimizing monetary distortion, so learners need to understand how inflation changes purchasing power and price signals first.</x:v>
       </x:c>
       <x:c r="F80" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G80" s="32" t="str">
-        <x:v>Direct parent keeps the node at the pooled-mining accounting layer without adding redundant proof-of-work or difficulty edges.</x:v>
+        <x:v>Direct parent captures the measurement-distortion problem that ideal money is trying to avoid.</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B81" s="32" t="str">
-        <x:v>lightning.obscured-commitment-number</x:v>
+        <x:v>protocol.bitcoin-uri-bip21</x:v>
       </x:c>
       <x:c r="C81" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12604,21 +13198,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E81" s="32" t="str">
-        <x:v>The obscured commitment number is part of the same commitment-state machinery as the per-state secret chain, so learners need that state-derivation context before the field-level encoding scheme makes sense.</x:v>
+        <x:v>The URI is a wrapper around a payment destination and amount, so learners need the underlying address and output model first.</x:v>
       </x:c>
       <x:c r="F81" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G81" s="32" t="str">
-        <x:v>Direct parent keeps the node in the narrow commitment-state branch instead of pulling in broader closure or HTLC behavior.</x:v>
+        <x:v>Direct parent keeps the node tied to the standard request format rather than collapsing it into higher-level wallet UX systems.</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="32" t="str">
-        <x:v>lightning.htlc</x:v>
+        <x:v>dev.bip32</x:v>
       </x:c>
       <x:c r="B82" s="32" t="str">
-        <x:v>lightning.htlc-output-scripts</x:v>
+        <x:v>dev.extended-keys</x:v>
       </x:c>
       <x:c r="C82" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12627,21 +13221,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E82" s="32" t="str">
-        <x:v>Learners need the base HTLC idea before the offered and received witness-script branches, timeout paths, and preimage-claim paths become meaningful.</x:v>
+        <x:v>Extended keys are one specific export and branch-derivation surface inside the broader BIP32 HD tree model, so learners need the base tree-derivation mechanics first.</x:v>
       </x:c>
       <x:c r="F82" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G82" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the payment-contract primitive instead of treating it as generic script trivia.</x:v>
+        <x:v>Direct parent keeps the node inside the HD derivation branch instead of treating xpub or xprv behavior as only a privacy or operational-wallet concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>dev.extended-keys</x:v>
       </x:c>
       <x:c r="B83" s="32" t="str">
-        <x:v>lightning.htlc-output-scripts</x:v>
+        <x:v>dev.hardened-keys</x:v>
       </x:c>
       <x:c r="C83" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12650,21 +13244,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E83" s="32" t="str">
-        <x:v>HTLC output scripts are additional commitment-transaction outputs layered on top of the same to_local and to_remote commitment-script structure, so learners need that earlier script layer first.</x:v>
+        <x:v>Hardened derivation is a constraint on what an extended public key can derive and on how extended private and public key boundaries behave, so learners need the base xpub/xprv model first.</x:v>
       </x:c>
       <x:c r="F83" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G83" s="32" t="str">
-        <x:v>Direct parent places the node at the next script layer above commitment outputs without dragging in later close-handling or watchtower flows.</x:v>
+        <x:v>Direct parent closes the previously missing branch-level bridge between BIP32 generally and hardened derivation specifically.</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="32" t="str">
-        <x:v>protocol.coinbase-transaction</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B84" s="32" t="str">
-        <x:v>protocol.duplicate-transaction-bug</x:v>
+        <x:v>protocol.escrow-and-arbitration</x:v>
       </x:c>
       <x:c r="C84" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12673,21 +13267,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E84" s="32" t="str">
-        <x:v>The bug is historically tied to duplicated coinbase transactions, so learners need the special structure and validation role of coinbase transactions before the replay vector makes sense.</x:v>
+        <x:v>The escrow flow depends on understanding how multiple signers can authorize one spend and why a 2-of-3 threshold changes trust assumptions between buyer, seller, and arbitrator.</x:v>
       </x:c>
       <x:c r="F84" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G84" s="32" t="str">
-        <x:v>Direct parent keeps the bug tied to the early-coinbase uniqueness failure instead of burying it under general mining history.</x:v>
+        <x:v>Direct parent keeps the node tied to the threshold-signing contract pattern instead of treating it as generic dispute-resolution theory.</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="32" t="str">
-        <x:v>protocol.utxo-model</x:v>
+        <x:v>protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="B85" s="32" t="str">
-        <x:v>protocol.duplicate-transaction-bug</x:v>
+        <x:v>protocol.escrow-and-arbitration</x:v>
       </x:c>
       <x:c r="C85" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12696,21 +13290,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E85" s="32" t="str">
-        <x:v>Learners need the txid-plus-output-index reference model to understand why identical transaction ids could confuse later spends and overwrite assumptions in the UTXO set.</x:v>
+        <x:v>The contract uses a P2SH redeem script to hide the multisig spending conditions until spend time, so learners need the P2SH wrapper first.</x:v>
       </x:c>
       <x:c r="F85" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G85" s="32" t="str">
-        <x:v>Direct parent captures the reference-model side of the bug without conflating it with double-spend history or malleability.</x:v>
+        <x:v>Direct parent captures the on-chain contract packaging layer that makes the escrow pattern practical.</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="32" t="str">
-        <x:v>protocol.block-structure</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B86" s="32" t="str">
-        <x:v>protocol.64-byte-transaction-bug</x:v>
+        <x:v>dev.wallet-import-format-wif</x:v>
       </x:c>
       <x:c r="C86" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12719,21 +13313,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E86" s="32" t="str">
-        <x:v>The bug only makes sense once learners understand how transaction hashes sit inside the block merkle tree and why internal-node preimages matter for block commitments.</x:v>
+        <x:v>WIF is a serialization format for one private key, so learners need the underlying asymmetric-key concept before the network prefix, checksum, and compression flag details make sense.</x:v>
       </x:c>
       <x:c r="F86" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G86" s="32" t="str">
-        <x:v>One direct parent keeps the node at the block-commitment layer instead of reopening broader hashing or SPV overview branches.</x:v>
+        <x:v>Direct parent keeps the node anchored on key material itself instead of overfitting it to address formats or HD wallet hierarchies.</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="32" t="str">
-        <x:v>fundamentals.digital-signatures</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B87" s="32" t="str">
-        <x:v>fundamentals.lamport-signatures</x:v>
+        <x:v>mining.pool-shares</x:v>
       </x:c>
       <x:c r="C87" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12742,21 +13336,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E87" s="32" t="str">
-        <x:v>Learners need the general signing-and-verification mental model before the one-time Lamport construction and its tradeoffs become meaningful.</x:v>
+        <x:v>Pool shares only make sense after learners understand why pooled mining exists and why miners need a lower-variance way to prove contributed work before an actual block is found.</x:v>
       </x:c>
       <x:c r="F87" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G87" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to signature semantics instead of treating it as only a post-quantum curiosity.</x:v>
+        <x:v>Direct parent keeps the node at the pooled-mining accounting layer without adding redundant proof-of-work or difficulty edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="B88" s="32" t="str">
-        <x:v>fundamentals.lamport-signatures</x:v>
+        <x:v>lightning.obscured-commitment-number</x:v>
       </x:c>
       <x:c r="C88" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12765,21 +13359,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E88" s="32" t="str">
-        <x:v>Lamport signatures replace elliptic-curve arithmetic with one-way hash preimages and comparisons, so learners need the hash primitive first.</x:v>
+        <x:v>The obscured commitment number is part of the same commitment-state machinery as the per-state secret chain, so learners need that state-derivation context before the field-level encoding scheme makes sense.</x:v>
       </x:c>
       <x:c r="F88" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G88" s="32" t="str">
-        <x:v>Direct parent captures the actual cryptographic mechanism rather than forcing learners through unrelated elliptic-curve details.</x:v>
+        <x:v>Direct parent keeps the node in the narrow commitment-state branch instead of pulling in broader closure or HTLC behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="32" t="str">
-        <x:v>custody.backups-recovery</x:v>
+        <x:v>lightning.htlc</x:v>
       </x:c>
       <x:c r="B89" s="32" t="str">
-        <x:v>custody.shamirs-secret-sharing</x:v>
+        <x:v>lightning.htlc-output-scripts</x:v>
       </x:c>
       <x:c r="C89" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12788,21 +13382,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E89" s="32" t="str">
-        <x:v>In Bitcoin practice the scheme is used as one backup-and-recovery method, so learners need the broader custody problem before the threshold-share design choice becomes meaningful.</x:v>
+        <x:v>Learners need the base HTLC idea before the offered and received witness-script branches, timeout paths, and preimage-claim paths become meaningful.</x:v>
       </x:c>
       <x:c r="F89" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G89" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored in practical custody use instead of drifting into a purely abstract cryptography topic.</x:v>
+        <x:v>Direct parent keeps the node tied to the payment-contract primitive instead of treating it as generic script trivia.</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="32" t="str">
-        <x:v>protocol.segregated-witness</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="B90" s="32" t="str">
-        <x:v>protocol.witness-structure</x:v>
+        <x:v>lightning.htlc-output-scripts</x:v>
       </x:c>
       <x:c r="C90" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12811,21 +13405,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E90" s="32" t="str">
-        <x:v>The transaction witness layout only makes sense after the learner understands that SegWit separates witness data from the legacy transaction serialization.</x:v>
+        <x:v>HTLC output scripts are additional commitment-transaction outputs layered on top of the same to_local and to_remote commitment-script structure, so learners need that earlier script layer first.</x:v>
       </x:c>
       <x:c r="F90" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G90" s="32" t="str">
-        <x:v>Direct edge keeps the node at the transaction-format layer; TXID/WTXID and witness-commitment consequences remain downstream concepts.</x:v>
+        <x:v>Direct parent places the node at the next script layer above commitment outputs without dragging in later close-handling or watchtower flows.</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="32" t="str">
-        <x:v>protocol.block-structure</x:v>
+        <x:v>protocol.coinbase-transaction</x:v>
       </x:c>
       <x:c r="B91" s="32" t="str">
-        <x:v>protocol.partial-merkle-proofs</x:v>
+        <x:v>protocol.duplicate-transaction-bug</x:v>
       </x:c>
       <x:c r="C91" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12834,21 +13428,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E91" s="32" t="str">
-        <x:v>Partial Merkle proofs reconstruct a transaction's inclusion path against the Merkle root carried by a block, so learners need block composition and root placement first.</x:v>
+        <x:v>The bug is historically tied to duplicated coinbase transactions, so learners need the special structure and validation role of coinbase transactions before the replay vector makes sense.</x:v>
       </x:c>
       <x:c r="F91" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G91" s="32" t="str">
-        <x:v>The block-structure parent already inherits fundamentals.merkle-trees, avoiding a redundant direct edge.</x:v>
+        <x:v>Direct parent keeps the bug tied to the early-coinbase uniqueness failure instead of burying it under general mining history.</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="32" t="str">
-        <x:v>dev.bips-process</x:v>
+        <x:v>protocol.utxo-model</x:v>
       </x:c>
       <x:c r="B92" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>protocol.duplicate-transaction-bug</x:v>
       </x:c>
       <x:c r="C92" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12857,21 +13451,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E92" s="32" t="str">
-        <x:v>Review culture is applied throughout the proposal and implementation lifecycle, so learners need to understand the process in which Bitcoin changes are proposed and evaluated.</x:v>
+        <x:v>Learners need the txid-plus-output-index reference model to understand why identical transaction ids could confuse later spends and overwrite assumptions in the UTXO set.</x:v>
       </x:c>
       <x:c r="F92" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G92" s="32" t="str">
-        <x:v>Direct edge supplies the development-lifecycle context without adding downstream release or deployment details.</x:v>
+        <x:v>Direct parent captures the reference-model side of the bug without conflating it with double-spend history or malleability.</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="32" t="str">
-        <x:v>security.adversarial-thinking</x:v>
+        <x:v>protocol.block-structure</x:v>
       </x:c>
       <x:c r="B93" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>protocol.64-byte-transaction-bug</x:v>
       </x:c>
       <x:c r="C93" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12880,21 +13474,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E93" s="32" t="str">
-        <x:v>Independent review in Bitcoin is deliberately adversarial: reviewers look for correctness failures, attack paths, and compatibility hazards before changes are merged.</x:v>
+        <x:v>The bug only makes sense once learners understand how transaction hashes sit inside the block merkle tree and why internal-node preimages matter for block commitments.</x:v>
       </x:c>
       <x:c r="F93" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G93" s="32" t="str">
-        <x:v>Direct edge keeps review distinct from responsible disclosure and reproducible-build verification, which are specialized downstream safeguards.</x:v>
+        <x:v>One direct parent keeps the node at the block-commitment layer instead of reopening broader hashing or SPV overview branches.</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="32" t="str">
-        <x:v>lightning.gossip-protocol</x:v>
+        <x:v>fundamentals.digital-signatures</x:v>
       </x:c>
       <x:c r="B94" s="32" t="str">
-        <x:v>lightning.feature-flags</x:v>
+        <x:v>fundamentals.lamport-signatures</x:v>
       </x:c>
       <x:c r="C94" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12903,21 +13497,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E94" s="32" t="str">
-        <x:v>Feature negotiation is used to advertise and interpret capabilities across Lightning peers and network announcements, so learners need the surrounding gossip and announcement context first.</x:v>
+        <x:v>Learners need the general signing-and-verification mental model before the one-time Lamport construction and its tradeoffs become meaningful.</x:v>
       </x:c>
       <x:c r="F94" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G94" s="32" t="str">
-        <x:v>Direct edge keeps the feature-bit mechanism distinct from the lower-level message transport and downstream routing protocols.</x:v>
+        <x:v>Direct parent keeps the node tied to signature semantics instead of treating it as only a post-quantum curiosity.</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="32" t="str">
-        <x:v>lightning.feature-flags</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B95" s="32" t="str">
-        <x:v>lightning.onion-messages</x:v>
+        <x:v>fundamentals.lamport-signatures</x:v>
       </x:c>
       <x:c r="C95" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12926,21 +13520,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E95" s="32" t="str">
-        <x:v>Peers use a negotiated feature bit to advertise whether they can send and forward onion messages, so learners need the capability-negotiation model first.</x:v>
+        <x:v>Lamport signatures replace elliptic-curve arithmetic with one-way hash preimages and comparisons, so learners need the hash primitive first.</x:v>
       </x:c>
       <x:c r="F95" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G95" s="32" t="str">
-        <x:v>Direct edge keeps the feature gate separate from the message forwarding mechanism.</x:v>
+        <x:v>Direct parent captures the actual cryptographic mechanism rather than forcing learners through unrelated elliptic-curve details.</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="32" t="str">
-        <x:v>lightning.route-blinding</x:v>
+        <x:v>custody.backups-recovery</x:v>
       </x:c>
       <x:c r="B96" s="32" t="str">
-        <x:v>lightning.onion-messages</x:v>
+        <x:v>custody.shamirs-secret-sharing</x:v>
       </x:c>
       <x:c r="C96" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12949,21 +13543,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E96" s="32" t="str">
-        <x:v>Onion messages use blinded paths to forward channel-independent payloads without exposing the final destination topology, so the route-blinding model must come first.</x:v>
+        <x:v>In Bitcoin practice the scheme is used as one backup-and-recovery method, so learners need the broader custody problem before the threshold-share design choice becomes meaningful.</x:v>
       </x:c>
       <x:c r="F96" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G96" s="32" t="str">
-        <x:v>Payment onion routing and BOLT12 offers remain related sibling or downstream concepts rather than direct prerequisites.</x:v>
+        <x:v>Direct parent keeps the node anchored in practical custody use instead of drifting into a purely abstract cryptography topic.</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>protocol.segregated-witness</x:v>
       </x:c>
       <x:c r="B97" s="32" t="str">
-        <x:v>lightning.encrypted-authenticated-transport</x:v>
+        <x:v>protocol.witness-structure</x:v>
       </x:c>
       <x:c r="C97" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12972,21 +13566,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E97" s="32" t="str">
-        <x:v>The Noise_XK handshake authenticates long-term Lightning node identities with public/private key material, so learners need that identity model first.</x:v>
+        <x:v>The transaction witness layout only makes sense after the learner understands that SegWit separates witness data from the legacy transaction serialization.</x:v>
       </x:c>
       <x:c r="F97" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G97" s="32" t="str">
-        <x:v>Direct edge keeps identity foundations separate from the session-key derivation mechanism.</x:v>
+        <x:v>Direct edge keeps the node at the transaction-format layer; TXID/WTXID and witness-commitment consequences remain downstream concepts.</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="32" t="str">
-        <x:v>fundamentals.diffie-hellman-key-exchange</x:v>
+        <x:v>protocol.block-structure</x:v>
       </x:c>
       <x:c r="B98" s="32" t="str">
-        <x:v>lightning.encrypted-authenticated-transport</x:v>
+        <x:v>protocol.partial-merkle-proofs</x:v>
       </x:c>
       <x:c r="C98" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12995,21 +13589,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E98" s="32" t="str">
-        <x:v>BOLT 08 uses elliptic-curve Diffie-Hellman operations to derive shared session secrets, so the key-exchange primitive must be understood first.</x:v>
+        <x:v>Partial Merkle proofs reconstruct a transaction's inclusion path against the Merkle root carried by a block, so learners need block composition and root placement first.</x:v>
       </x:c>
       <x:c r="F98" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G98" s="32" t="str">
-        <x:v>Bitcoin P2P v2 transport remains a related sibling rather than a direct prerequisite because it is a different protocol context.</x:v>
+        <x:v>The block-structure parent already inherits fundamentals.merkle-trees, avoiding a redundant direct edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>dev.bips-process</x:v>
       </x:c>
       <x:c r="B99" s="32" t="str">
-        <x:v>protocol.strict-der-signatures</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="C99" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13018,21 +13612,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E99" s="32" t="str">
-        <x:v>Strict DER enforcement occurs while Script validates an ECDSA signature, so learners need the spending-condition and interpreter context first.</x:v>
+        <x:v>Review culture is applied throughout the proposal and implementation lifecycle, so learners need to understand the process in which Bitcoin changes are proposed and evaluated.</x:v>
       </x:c>
       <x:c r="F99" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G99" s="32" t="str">
-        <x:v>Direct edge keeps the rule at the script-validation layer rather than treating BIP 66 as a broad historical upgrade topic.</x:v>
+        <x:v>Direct edge supplies the development-lifecycle context without adding downstream release or deployment details.</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>security.adversarial-thinking</x:v>
       </x:c>
       <x:c r="B100" s="32" t="str">
-        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="C100" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13041,21 +13635,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E100" s="32" t="str">
-        <x:v>The node builds on the wallet-level threshold signer policy before specifying a deterministic ordering convention for the signer keys.</x:v>
+        <x:v>Independent review in Bitcoin is deliberately adversarial: reviewers look for correctness failures, attack paths, and compatibility hazards before changes are merged.</x:v>
       </x:c>
       <x:c r="F100" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G100" s="32" t="str">
-        <x:v>Direct edge preserves the distinction between multisig policy and the BIP 67 interoperability rule.</x:v>
+        <x:v>Direct edge keeps review distinct from responsible disclosure and reproducible-build verification, which are specialized downstream safeguards.</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="32" t="str">
-        <x:v>protocol.pay-to-script-hash</x:v>
+        <x:v>lightning.gossip-protocol</x:v>
       </x:c>
       <x:c r="B101" s="32" t="str">
-        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+        <x:v>lightning.feature-flags</x:v>
       </x:c>
       <x:c r="C101" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13064,21 +13658,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E101" s="32" t="str">
-        <x:v>BIP 67 is commonly applied when constructing the redeem script whose hash is committed by P2SH, so the script-hash wrapper provides the output context.</x:v>
+        <x:v>Feature negotiation is used to advertise and interpret capabilities across Lightning peers and network announcements, so learners need the surrounding gossip and announcement context first.</x:v>
       </x:c>
       <x:c r="F101" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G101" s="32" t="str">
-        <x:v>The shared protocol.script ancestor remains inherited rather than a redundant direct edge.</x:v>
+        <x:v>Direct edge keeps the feature-bit mechanism distinct from the lower-level message transport and downstream routing protocols.</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="32" t="str">
-        <x:v>ops.mempool-policy</x:v>
+        <x:v>lightning.feature-flags</x:v>
       </x:c>
       <x:c r="B102" s="32" t="str">
-        <x:v>ops.mempool-purging</x:v>
+        <x:v>lightning.onion-messages</x:v>
       </x:c>
       <x:c r="C102" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13087,21 +13681,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E102" s="32" t="str">
-        <x:v>Rolling minimum fee escalation and transaction eviction are local consequences of the node's mempool relay policy, so learners need that policy boundary first.</x:v>
+        <x:v>Peers use a negotiated feature bit to advertise whether they can send and forward onion messages, so learners need the capability-negotiation model first.</x:v>
       </x:c>
       <x:c r="F102" s="32" t="str">
-        <x:v>source.mempool-space-docs</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G102" s="32" t="str">
-        <x:v>The generic mempool, fee-market, and consensus-policy branches remain inherited or adjacent rather than direct prerequisites.</x:v>
+        <x:v>Direct edge keeps the feature gate separate from the message forwarding mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>lightning.route-blinding</x:v>
       </x:c>
       <x:c r="B103" s="32" t="str">
-        <x:v>protocol.generic-signed-messages</x:v>
+        <x:v>lightning.onion-messages</x:v>
       </x:c>
       <x:c r="C103" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13110,21 +13704,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E103" s="32" t="str">
-        <x:v>BIP 322 proves message authorization by constructing virtual transactions that satisfy a Bitcoin output script, so learners need the Script spending-condition model first.</x:v>
+        <x:v>Onion messages use blinded paths to forward channel-independent payloads without exposing the final destination topology, so the route-blinding model must come first.</x:v>
       </x:c>
       <x:c r="F103" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G103" s="32" t="str">
-        <x:v>The digital-signature path is inherited through Script; PSBT, Schnorr, and Taproot remain related variants rather than redundant direct edges.</x:v>
+        <x:v>Payment onion routing and BOLT12 offers remain related sibling or downstream concepts rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="32" t="str">
-        <x:v>dev.bitcoin-core-rpc</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B104" s="32" t="str">
-        <x:v>security.bitcoin-core-rpc-access</x:v>
+        <x:v>lightning.encrypted-authenticated-transport</x:v>
       </x:c>
       <x:c r="C104" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13133,21 +13727,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E104" s="32" t="str">
-        <x:v>RPC access security is the control boundary around Bitcoin Core's programmatic interface, so learners need to understand the interface and its authority before securing exposure to it.</x:v>
+        <x:v>The Noise_XK handshake authenticates long-term Lightning node identities with public/private key material, so learners need that identity model first.</x:v>
       </x:c>
       <x:c r="F104" s="32" t="str">
-        <x:v>source.bitcoin-core-operator-docs</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G104" s="32" t="str">
-        <x:v>Full-node operation is inherited through dev.bitcoin-core-rpc; wallet RPC and transaction-preflight nodes remain downstream use cases rather than direct parents.</x:v>
+        <x:v>Direct edge keeps identity foundations separate from the session-key derivation mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="32" t="str">
-        <x:v>dev.testmempoolaccept-rpc</x:v>
+        <x:v>fundamentals.diffie-hellman-key-exchange</x:v>
       </x:c>
       <x:c r="B105" s="32" t="str">
-        <x:v>dev.submitpackage-rpc</x:v>
+        <x:v>lightning.encrypted-authenticated-transport</x:v>
       </x:c>
       <x:c r="C105" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13156,21 +13750,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E105" s="32" t="str">
-        <x:v>submitpackage is the admission counterpart to the existing testmempoolaccept preflight workflow, so learners need to understand local package checks before attempting submission and interpreting package results.</x:v>
+        <x:v>BOLT 08 uses elliptic-curve Diffie-Hellman operations to derive shared session secrets, so the key-exchange primitive must be understood first.</x:v>
       </x:c>
       <x:c r="F105" s="32" t="str">
-        <x:v>source.bitcoin-core-package-policy</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G105" s="32" t="str">
-        <x:v>Package relay and cluster mempool remain neighboring concepts rather than direct prerequisites because this node focuses on one local RPC operation.</x:v>
+        <x:v>Bitcoin P2P v2 transport remains a related sibling rather than a direct prerequisite because it is a different protocol context.</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="32" t="str">
-        <x:v>protocol.rbf</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B106" s="32" t="str">
-        <x:v>protocol.package-rbf</x:v>
+        <x:v>protocol.strict-der-signatures</x:v>
       </x:c>
       <x:c r="C106" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13179,21 +13773,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E106" s="32" t="str">
-        <x:v>Package RBF extends the ordinary replacement-policy model with package-level fee and cluster conditions, so learners need base RBF semantics first.</x:v>
+        <x:v>Strict DER enforcement occurs while Script validates an ECDSA signature, so learners need the spending-condition and interpreter context first.</x:v>
       </x:c>
       <x:c r="F106" s="32" t="str">
-        <x:v>source.bitcoin-core-package-policy</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G106" s="32" t="str">
-        <x:v>Package relay, cluster mempool, submitpackage, and pinning remain adjacent concepts rather than redundant direct edges.</x:v>
+        <x:v>Direct edge keeps the rule at the script-validation layer rather than treating BIP 66 as a broad historical upgrade topic.</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="32" t="str">
-        <x:v>protocol.cluster-mempool</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B107" s="32" t="str">
-        <x:v>ops.mempool-cluster-limits</x:v>
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
       </x:c>
       <x:c r="C107" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13202,21 +13796,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E107" s="32" t="str">
-        <x:v>Cluster limits bound connected transaction sets, so learners need the cluster-mempool model before understanding why count and aggregate virtual-size limits replace legacy ancestor/descendant limits.</x:v>
+        <x:v>The node builds on the wallet-level threshold signer policy before specifying a deterministic ordering convention for the signer keys.</x:v>
       </x:c>
       <x:c r="F107" s="32" t="str">
-        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G107" s="32" t="str">
-        <x:v>Package relay, Package RBF, CPFP, and version 3 relay remain affected workflows or neighboring policy mechanisms rather than direct prerequisites.</x:v>
+        <x:v>Direct edge preserves the distinction between multisig policy and the BIP 67 interoperability rule.</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="32" t="str">
-        <x:v>ops.dns-seeds</x:v>
+        <x:v>protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="B108" s="32" t="str">
-        <x:v>lightning.dns-seeds</x:v>
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
       </x:c>
       <x:c r="C108" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13225,21 +13819,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E108" s="32" t="str">
-        <x:v>Lightning DNS seeds specialize the general DNS bootstrap pattern with Lightning-specific query filters and known-peer lookup, so learners need the base DNS-seed model first.</x:v>
+        <x:v>BIP 67 is commonly applied when constructing the redeem script whose hash is committed by P2SH, so the script-hash wrapper provides the output context.</x:v>
       </x:c>
       <x:c r="F108" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G108" s="32" t="str">
-        <x:v>Peer discovery is inherited through ops.dns-seeds; generic Bitcoin P2P bootstrapping remains a parent concept rather than a duplicated edge.</x:v>
+        <x:v>The shared protocol.script ancestor remains inherited rather than a redundant direct edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="32" t="str">
-        <x:v>lightning.gossip-protocol</x:v>
+        <x:v>ops.mempool-policy</x:v>
       </x:c>
       <x:c r="B109" s="32" t="str">
-        <x:v>lightning.dns-seeds</x:v>
+        <x:v>ops.mempool-purging</x:v>
       </x:c>
       <x:c r="C109" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13248,21 +13842,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E109" s="32" t="str">
-        <x:v>BOLT 10 locates Lightning peers and filters results by Lightning address information, so learners need Lightning's node-discovery and gossip context before understanding the assisted-location mechanism.</x:v>
+        <x:v>Rolling minimum fee escalation and transaction eviction are local consequences of the node's mempool relay policy, so learners need that policy boundary first.</x:v>
       </x:c>
       <x:c r="F109" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.mempool-space-docs</x:v>
       </x:c>
       <x:c r="G109" s="32" t="str">
-        <x:v>Lightning routing and generic P2P messages are inherited through gossip rather than added as transitive prerequisites.</x:v>
+        <x:v>The generic mempool, fee-market, and consensus-policy branches remain inherited or adjacent rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="32" t="str">
-        <x:v>lightning.payment-channels</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B110" s="32" t="str">
-        <x:v>lightning.short-channel-id</x:v>
+        <x:v>protocol.generic-signed-messages</x:v>
       </x:c>
       <x:c r="C110" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13271,21 +13865,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E110" s="32" t="str">
-        <x:v>The identifier names a Lightning channel's on-chain funding output, so learners need the channel and funding relationship first.</x:v>
+        <x:v>BIP 322 proves message authorization by constructing virtual transactions that satisfy a Bitcoin output script, so learners need the Script spending-condition model first.</x:v>
       </x:c>
       <x:c r="F110" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G110" s="32" t="str">
-        <x:v>Direct channel context; the gossip protocol is a downstream consumer rather than a prerequisite.</x:v>
+        <x:v>The digital-signature path is inherited through Script; PSBT, Schnorr, and Taproot remain related variants rather than redundant direct edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="32" t="str">
-        <x:v>protocol.block-height</x:v>
+        <x:v>dev.bitcoin-core-rpc</x:v>
       </x:c>
       <x:c r="B111" s="32" t="str">
-        <x:v>lightning.short-channel-id</x:v>
+        <x:v>security.bitcoin-core-rpc-access</x:v>
       </x:c>
       <x:c r="C111" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13294,21 +13888,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E111" s="32" t="str">
-        <x:v>Short Channel IDs encode block height as their first component, so learners need the block-height concept before decoding the identifier.</x:v>
+        <x:v>RPC access security is the control boundary around Bitcoin Core's programmatic interface, so learners need to understand the interface and its authority before securing exposure to it.</x:v>
       </x:c>
       <x:c r="F111" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-core-operator-docs</x:v>
       </x:c>
       <x:c r="G111" s="32" t="str">
-        <x:v>The transaction-index and output-index components remain part of the identifier's own outcome rather than extra transitive edges.</x:v>
+        <x:v>Full-node operation is inherited through dev.bitcoin-core-rpc; wallet RPC and transaction-preflight nodes remain downstream use cases rather than direct parents.</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="32" t="str">
-        <x:v>protocol.nodes-vs-miners</x:v>
+        <x:v>dev.testmempoolaccept-rpc</x:v>
       </x:c>
       <x:c r="B112" s="32" t="str">
-        <x:v>mining.miner-decentralization</x:v>
+        <x:v>dev.submitpackage-rpc</x:v>
       </x:c>
       <x:c r="C112" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13317,21 +13911,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E112" s="32" t="str">
-        <x:v>Miner decentralization only makes sense once learners distinguish miners' transaction-ordering role from full nodes' independent enforcement of consensus validity.</x:v>
+        <x:v>submitpackage is the admission counterpart to the existing testmempoolaccept preflight workflow, so learners need to understand local package checks before attempting submission and interpreting package results.</x:v>
       </x:c>
       <x:c r="F112" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-core-package-policy</x:v>
       </x:c>
       <x:c r="G112" s="32" t="str">
-        <x:v>The edge keeps censorship power separate from authority to change consensus rules.</x:v>
+        <x:v>Package relay and cluster mempool remain neighboring concepts rather than direct prerequisites because this node focuses on one local RPC operation.</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>protocol.rbf</x:v>
       </x:c>
       <x:c r="B113" s="32" t="str">
-        <x:v>mining.miner-decentralization</x:v>
+        <x:v>protocol.package-rbf</x:v>
       </x:c>
       <x:c r="C113" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13340,21 +13934,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E113" s="32" t="str">
-        <x:v>Pool and solo mining explain the participant and coordination structure whose concentration or dispersion determines practical control over transaction ordering.</x:v>
+        <x:v>Package RBF extends the ordinary replacement-policy model with package-level fee and cluster conditions, so learners need base RBF semantics first.</x:v>
       </x:c>
       <x:c r="F113" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-core-package-policy</x:v>
       </x:c>
       <x:c r="G113" s="32" t="str">
-        <x:v>Stratum V2 remains optional implementation context, not a direct prerequisite.</x:v>
+        <x:v>Package relay, cluster mempool, submitpackage, and pinning remain adjacent concepts rather than redundant direct edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>protocol.cluster-mempool</x:v>
       </x:c>
       <x:c r="B114" s="32" t="str">
-        <x:v>dev.selection-cryptography</x:v>
+        <x:v>ops.mempool-cluster-limits</x:v>
       </x:c>
       <x:c r="C114" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13363,21 +13957,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E114" s="32" t="str">
-        <x:v>Selection cryptography evaluates cryptographic tools and dependencies through evidence, testing, authorship, and review quality, so learners need the broader Bitcoin review discipline first.</x:v>
+        <x:v>Cluster limits bound connected transaction sets, so learners need the cluster-mempool model before understanding why count and aggregate virtual-size limits replace legacy ancestor/descendant limits.</x:v>
       </x:c>
       <x:c r="F114" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
       </x:c>
       <x:c r="G114" s="32" t="str">
-        <x:v>Adversarial thinking is inherited through dev.review-culture; reproducible builds are a downstream verification practice rather than a prerequisite.</x:v>
+        <x:v>Package relay, Package RBF, CPFP, and version 3 relay remain affected workflows or neighboring policy mechanisms rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="32" t="str">
-        <x:v>mining.pool-shares</x:v>
+        <x:v>ops.dns-seeds</x:v>
       </x:c>
       <x:c r="B115" s="32" t="str">
-        <x:v>mining.block-withholding</x:v>
+        <x:v>lightning.dns-seeds</x:v>
       </x:c>
       <x:c r="C115" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13386,21 +13980,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E115" s="32" t="str">
-        <x:v>Block withholding exploits the difference between a pool-paid share and a share that also meets the network target, so learners must understand share accounting before the attack model makes sense.</x:v>
+        <x:v>Lightning DNS seeds specialize the general DNS bootstrap pattern with Lightning-specific query filters and known-peer lookup, so learners need the base DNS-seed model first.</x:v>
       </x:c>
       <x:c r="F115" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G115" s="32" t="str">
-        <x:v>Pool-versus-solo and mining economics are inherited through mining.pool-shares; do not add a redundant majority-attack edge.</x:v>
+        <x:v>Peer discovery is inherited through ops.dns-seeds; generic Bitcoin P2P bootstrapping remains a parent concept rather than a duplicated edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>lightning.gossip-protocol</x:v>
       </x:c>
       <x:c r="B116" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>lightning.dns-seeds</x:v>
       </x:c>
       <x:c r="C116" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13409,21 +14003,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E116" s="32" t="str">
-        <x:v>P2C tweaks a public key to commit to contract data, so learners need the public/private key model.</x:v>
+        <x:v>BOLT 10 locates Lightning peers and filters results by Lightning address information, so learners need Lightning's node-discovery and gossip context before understanding the assisted-location mechanism.</x:v>
       </x:c>
       <x:c r="F116" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G116" s="32" t="str">
-        <x:v>Taproot is adjacent, not a direct requirement.</x:v>
+        <x:v>Lightning routing and generic P2P messages are inherited through gossip rather than added as transitive prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>lightning.payment-channels</x:v>
       </x:c>
       <x:c r="B117" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>lightning.short-channel-id</x:v>
       </x:c>
       <x:c r="C117" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13432,21 +14026,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E117" s="32" t="str">
-        <x:v>P2C derives a commitment tweak from contract data using a hash, so learners need hash commitments first.</x:v>
+        <x:v>The identifier names a Lightning channel's on-chain funding output, so learners need the channel and funding relationship first.</x:v>
       </x:c>
       <x:c r="F117" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G117" s="32" t="str">
-        <x:v>The hash is part of the construction rather than generic background.</x:v>
+        <x:v>Direct channel context; the gossip protocol is a downstream consumer rather than a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="32" t="str">
-        <x:v>protocol.utxo-model</x:v>
+        <x:v>protocol.block-height</x:v>
       </x:c>
       <x:c r="B118" s="32" t="str">
-        <x:v>extension.single-use-seals</x:v>
+        <x:v>lightning.short-channel-id</x:v>
       </x:c>
       <x:c r="C118" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13455,21 +14049,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E118" s="32" t="str">
-        <x:v>Single-use seals rely on a UTXO's one-time spend property.</x:v>
+        <x:v>Short Channel IDs encode block height as their first component, so learners need the block-height concept before decoding the identifier.</x:v>
       </x:c>
       <x:c r="F118" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G118" s="32" t="str">
-        <x:v>This explicit bridge prevents hiding the seal invariant inside generic UTXO semantics.</x:v>
+        <x:v>The transaction-index and output-index components remain part of the identifier's own outcome rather than extra transitive edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="32" t="str">
-        <x:v>extension.single-use-seals</x:v>
+        <x:v>protocol.nodes-vs-miners</x:v>
       </x:c>
       <x:c r="B119" s="32" t="str">
-        <x:v>extension.client-side-validation</x:v>
+        <x:v>mining.miner-decentralization</x:v>
       </x:c>
       <x:c r="C119" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13478,21 +14072,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E119" s="32" t="str">
-        <x:v>Client-side validation relies on seals to prevent an offchain transition from being valid twice.</x:v>
+        <x:v>Miner decentralization only makes sense once learners distinguish miners' transaction-ordering role from full nodes' independent enforcement of consensus validity.</x:v>
       </x:c>
       <x:c r="F119" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G119" s="32" t="str">
-        <x:v>The UTXO parent is inherited through the seal and is intentionally not duplicated.</x:v>
+        <x:v>The edge keeps censorship power separate from authority to change consensus rules.</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B120" s="32" t="str">
-        <x:v>extension.client-side-validation</x:v>
+        <x:v>mining.miner-decentralization</x:v>
       </x:c>
       <x:c r="C120" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13501,21 +14095,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E120" s="32" t="str">
-        <x:v>Client-side validation uses cryptographic commitments to bind offchain asset rules and transitions, so P2C supplies the contract-anchoring mechanism.</x:v>
+        <x:v>Pool and solo mining explain the participant and coordination structure whose concentration or dispersion determines practical control over transaction ordering.</x:v>
       </x:c>
       <x:c r="F120" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G120" s="32" t="str">
-        <x:v>Keep this direct edge: it prevents treating client-side validation as a vague UTXO-only extension.</x:v>
+        <x:v>Stratum V2 remains optional implementation context, not a direct prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="32" t="str">
-        <x:v>protocol.rbf</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="B121" s="32" t="str">
-        <x:v>protocol.replacement-cycling</x:v>
+        <x:v>dev.selection-cryptography</x:v>
       </x:c>
       <x:c r="C121" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13524,21 +14118,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E121" s="32" t="str">
-        <x:v>Replacement cycling repeatedly uses transaction replacement, so learners need the RBF policy mechanism first.</x:v>
+        <x:v>Selection cryptography evaluates cryptographic tools and dependencies through evidence, testing, authorship, and review quality, so learners need the broader Bitcoin review discipline first.</x:v>
       </x:c>
       <x:c r="F121" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G121" s="32" t="str">
-        <x:v>Package RBF is related but not required for the core attack sequence.</x:v>
+        <x:v>Adversarial thinking is inherited through dev.review-culture; reproducible builds are a downstream verification practice rather than a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="32" t="str">
-        <x:v>protocol.cpfp</x:v>
+        <x:v>mining.pool-shares</x:v>
       </x:c>
       <x:c r="B122" s="32" t="str">
-        <x:v>protocol.replacement-cycling</x:v>
+        <x:v>mining.block-withholding</x:v>
       </x:c>
       <x:c r="C122" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13547,21 +14141,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E122" s="32" t="str">
-        <x:v>The attack cycles child-fee relationships to evict a target, so learners need CPFP mechanics first.</x:v>
+        <x:v>Block withholding exploits the difference between a pool-paid share and a share that also meets the network target, so learners must understand share accounting before the attack model makes sense.</x:v>
       </x:c>
       <x:c r="F122" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G122" s="32" t="str">
-        <x:v>Transaction pinning is the broader downstream risk class, not a prerequisite.</x:v>
+        <x:v>Pool-versus-solo and mining economics are inherited through mining.pool-shares; do not add a redundant majority-attack edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="32" t="str">
-        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B123" s="32" t="str">
-        <x:v>protocol.taproot-control-blocks</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="C123" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13570,21 +14164,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E123" s="32" t="str">
-        <x:v>Control blocks extend the tapleaf proof path with internal-key and parity data.</x:v>
+        <x:v>P2C tweaks a public key to commit to contract data, so learners need the public/private key model.</x:v>
       </x:c>
       <x:c r="F123" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G123" s="32" t="str">
-        <x:v>Generic Merkle trees are inherited through the proof node.</x:v>
+        <x:v>Taproot is adjacent, not a direct requirement.</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B124" s="32" t="str">
-        <x:v>dev.pseudonymous-development</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="C124" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13593,21 +14187,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E124" s="32" t="str">
-        <x:v>Pseudonymous development relies on public technical evidence and independent peer review to preserve accountability without requiring legal-identity disclosure.</x:v>
+        <x:v>P2C derives a commitment tweak from contract data using a hash, so learners need hash commitments first.</x:v>
       </x:c>
       <x:c r="F124" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G124" s="32" t="str">
-        <x:v>Privacy pseudonymity is related context, not a direct prerequisite, because this node concerns contributor identity and governance rather than transaction linkage.</x:v>
+        <x:v>The hash is part of the construction rather than generic background.</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="32" t="str">
-        <x:v>fundamentals.merkle-trees</x:v>
+        <x:v>protocol.utxo-model</x:v>
       </x:c>
       <x:c r="B125" s="32" t="str">
-        <x:v>protocol.mast</x:v>
+        <x:v>extension.single-use-seals</x:v>
       </x:c>
       <x:c r="C125" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13616,21 +14210,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E125" s="32" t="str">
-        <x:v>MAST uses a Merkle tree to commit to multiple alternative script branches while revealing only one branch during spending.</x:v>
+        <x:v>Single-use seals rely on a UTXO's one-time spend property.</x:v>
       </x:c>
       <x:c r="F125" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G125" s="32" t="str">
-        <x:v>Direct cryptographic structure; TapTree remains a downstream Taproot-specific realization.</x:v>
+        <x:v>This explicit bridge prevents hiding the seal invariant inside generic UTXO semantics.</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>extension.single-use-seals</x:v>
       </x:c>
       <x:c r="B126" s="32" t="str">
-        <x:v>protocol.mast</x:v>
+        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="C126" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13639,21 +14233,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E126" s="32" t="str">
-        <x:v>MAST commits to alternative Bitcoin Script branches, so learners need the locking and spending language before the tree commitment is meaningful.</x:v>
+        <x:v>Client-side validation relies on seals to prevent an offchain transition from being valid twice.</x:v>
       </x:c>
       <x:c r="F126" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G126" s="32" t="str">
-        <x:v>Keep Script direct; the node is not only a generic Merkle-tree concept.</x:v>
+        <x:v>The UTXO parent is inherited through the seal and is intentionally not duplicated.</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="32" t="str">
-        <x:v>protocol.sighash-flags</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="B127" s="32" t="str">
-        <x:v>protocol.sighash-quadratic-hashing</x:v>
+        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="C127" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13662,21 +14256,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E127" s="32" t="str">
-        <x:v>The quadratic hashing problem is a performance consequence of how legacy signature digests are constructed under SIGHASH semantics.</x:v>
+        <x:v>Client-side validation uses cryptographic commitments to bind offchain asset rules and transitions, so P2C supplies the contract-anchoring mechanism.</x:v>
       </x:c>
       <x:c r="F127" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G127" s="32" t="str">
-        <x:v>BIP 143 is a supporting mitigation source, not a prerequisite edge.</x:v>
+        <x:v>Keep this direct edge: it prevents treating client-side validation as a vague UTXO-only extension.</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>protocol.rbf</x:v>
       </x:c>
       <x:c r="B128" s="32" t="str">
-        <x:v>security.rogue-key-attack</x:v>
+        <x:v>protocol.replacement-cycling</x:v>
       </x:c>
       <x:c r="C128" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13685,21 +14279,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E128" s="32" t="str">
-        <x:v>The rogue-key attack occurs in naive public-key aggregation, so learners need the MuSig aggregation setting before the failure mode.</x:v>
+        <x:v>Replacement cycling repeatedly uses transaction replacement, so learners need the RBF policy mechanism first.</x:v>
       </x:c>
       <x:c r="F128" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G128" s="32" t="str">
-        <x:v>Schnorr is inherited through MuSig; avoid a redundant direct Schnorr edge.</x:v>
+        <x:v>Package RBF is related but not required for the core attack sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>protocol.cpfp</x:v>
       </x:c>
       <x:c r="B129" s="32" t="str">
-        <x:v>mining.selfish-mining</x:v>
+        <x:v>protocol.replacement-cycling</x:v>
       </x:c>
       <x:c r="C129" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13708,21 +14302,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E129" s="32" t="str">
-        <x:v>Selfish mining is an incentive strategy by miners and pools, so learners need the pooled-versus-solo mining context first.</x:v>
+        <x:v>The attack cycles child-fee relationships to evict a target, so learners need CPFP mechanics first.</x:v>
       </x:c>
       <x:c r="F129" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G129" s="32" t="str">
-        <x:v>Pool economics is one direct parent; chain selection is supplied by the finality parent below.</x:v>
+        <x:v>Transaction pinning is the broader downstream risk class, not a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="32" t="str">
-        <x:v>protocol.reorgs-finality</x:v>
+        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
       </x:c>
       <x:c r="B130" s="32" t="str">
-        <x:v>mining.selfish-mining</x:v>
+        <x:v>protocol.taproot-control-blocks</x:v>
       </x:c>
       <x:c r="C130" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13731,21 +14325,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E130" s="32" t="str">
-        <x:v>Selfish mining relies on strategic withholding and release of competing branches, which requires the chain-reorganization and finality model.</x:v>
+        <x:v>Control blocks extend the tapleaf proof path with internal-key and parity data.</x:v>
       </x:c>
       <x:c r="F130" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G130" s="32" t="str">
-        <x:v>Keep the reorganization model direct rather than adding generic proof-of-work as a redundant ancestor.</x:v>
+        <x:v>Generic Merkle trees are inherited through the proof node.</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="B131" s="32" t="str">
-        <x:v>protocol.commit-delay-reveal</x:v>
+        <x:v>dev.pseudonymous-development</x:v>
       </x:c>
       <x:c r="C131" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13754,21 +14348,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E131" s="32" t="str">
-        <x:v>Commit-delay-reveal composes a cryptographic commitment with a timed reveal, so the learner first needs the hiding and binding commitment model.</x:v>
+        <x:v>Pseudonymous development relies on public technical evidence and independent peer review to preserve accountability without requiring legal-identity disclosure.</x:v>
       </x:c>
       <x:c r="F131" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G131" s="32" t="str">
-        <x:v>The delay/reveal composition is the node's distinct outcome.</x:v>
+        <x:v>Privacy pseudonymity is related context, not a direct prerequisite, because this node concerns contributor identity and governance rather than transaction linkage.</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="32" t="str">
-        <x:v>protocol.dust-policy</x:v>
+        <x:v>fundamentals.merkle-trees</x:v>
       </x:c>
       <x:c r="B132" s="32" t="str">
-        <x:v>security.dust-attack</x:v>
+        <x:v>protocol.mast</x:v>
       </x:c>
       <x:c r="C132" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13777,21 +14371,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E132" s="32" t="str">
-        <x:v>Dust attacks exploit the distinction between tiny-output relay policy and the ability to place trace-value UTXOs in a wallet.</x:v>
+        <x:v>MAST uses a Merkle tree to commit to multiple alternative script branches while revealing only one branch during spending.</x:v>
       </x:c>
       <x:c r="F132" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
       </x:c>
       <x:c r="G132" s="32" t="str">
-        <x:v>Policy threshold is direct context for the attack mechanism.</x:v>
+        <x:v>Direct cryptographic structure; TapTree remains a downstream Taproot-specific realization.</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B133" s="32" t="str">
-        <x:v>security.dust-attack</x:v>
+        <x:v>protocol.mast</x:v>
       </x:c>
       <x:c r="C133" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13800,21 +14394,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E133" s="32" t="str">
-        <x:v>The privacy harm of dusting comes from linking future spends and wallet activity, so learners need the pseudonymity and linkage model.</x:v>
+        <x:v>MAST commits to alternative Bitcoin Script branches, so learners need the locking and spending language before the tree commitment is meaningful.</x:v>
       </x:c>
       <x:c r="F133" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
       </x:c>
       <x:c r="G133" s="32" t="str">
-        <x:v>Keep privacy linkage direct; it is not inherited through dust policy.</x:v>
+        <x:v>Keep Script direct; the node is not only a generic Merkle-tree concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="32" t="str">
-        <x:v>fundamentals.neutrality</x:v>
+        <x:v>protocol.sighash-flags</x:v>
       </x:c>
       <x:c r="B134" s="32" t="str">
-        <x:v>dev.permissionless-development</x:v>
+        <x:v>protocol.sighash-quadratic-hashing</x:v>
       </x:c>
       <x:c r="C134" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13823,21 +14417,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E134" s="32" t="str">
-        <x:v>Permissionless development depends on a neutral protocol that does not select which users or applications may participate.</x:v>
+        <x:v>The quadratic hashing problem is a performance consequence of how legacy signature digests are constructed under SIGHASH semantics.</x:v>
       </x:c>
       <x:c r="F134" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
       </x:c>
       <x:c r="G134" s="32" t="str">
-        <x:v>Neutrality supplies the protocol property; the BIPs process supplies the change/proposal lifecycle below.</x:v>
+        <x:v>BIP 143 is a supporting mitigation source, not a prerequisite edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="32" t="str">
-        <x:v>dev.bips-process</x:v>
+        <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="B135" s="32" t="str">
-        <x:v>dev.permissionless-development</x:v>
+        <x:v>security.rogue-key-attack</x:v>
       </x:c>
       <x:c r="C135" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13846,21 +14440,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E135" s="32" t="str">
-        <x:v>Learners need the proposal and deployment process to distinguish building permissionlessly from changing Bitcoin's consensus rules without broad adoption.</x:v>
+        <x:v>The rogue-key attack occurs in naive public-key aggregation, so learners need the MuSig aggregation setting before the failure mode.</x:v>
       </x:c>
       <x:c r="F135" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
       </x:c>
       <x:c r="G135" s="32" t="str">
-        <x:v>Review culture remains related but is not a direct prerequisite for permissionless access.</x:v>
+        <x:v>Schnorr is inherited through MuSig; avoid a redundant direct Schnorr edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="32" t="str">
-        <x:v>dev.reproducible-builds</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B136" s="32" t="str">
-        <x:v>dev.bootstrappable-builds</x:v>
+        <x:v>mining.selfish-mining</x:v>
       </x:c>
       <x:c r="C136" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13869,21 +14463,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E136" s="32" t="str">
-        <x:v>Bootstrappable builds extend reproducible builds by reducing trust in the compiler and build-tool binaries used to produce the reproducible output.</x:v>
+        <x:v>Selfish mining is an incentive strategy by miners and pools, so learners need the pooled-versus-solo mining context first.</x:v>
       </x:c>
       <x:c r="F136" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
       </x:c>
       <x:c r="G136" s="32" t="str">
-        <x:v>Keep this as a direct downstream edge; the node is not a duplicate alias for reproducible builds.</x:v>
+        <x:v>Pool economics is one direct parent; chain selection is supplied by the finality parent below.</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="32" t="str">
-        <x:v>protocol.transaction-lifecycle</x:v>
+        <x:v>protocol.reorgs-finality</x:v>
       </x:c>
       <x:c r="B137" s="32" t="str">
-        <x:v>protocol.proof-of-payment</x:v>
+        <x:v>mining.selfish-mining</x:v>
       </x:c>
       <x:c r="C137" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13892,21 +14486,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E137" s="32" t="str">
-        <x:v>Proof of Payment refers to a prior payment and reconstructs a transaction-shaped proof, so learners need the transaction lifecycle first.</x:v>
+        <x:v>Selfish mining relies on strategic withholding and release of competing branches, which requires the chain-reorganization and finality model.</x:v>
       </x:c>
       <x:c r="F137" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
       </x:c>
       <x:c r="G137" s="32" t="str">
-        <x:v>Direct payment context; wallet UX and URI transport remain downstream or optional details.</x:v>
+        <x:v>Keep the reorganization model direct rather than adding generic proof-of-work as a redundant ancestor.</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="32" t="str">
-        <x:v>protocol.ephemeral-anchors</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="B138" s="32" t="str">
-        <x:v>protocol.pay-to-anchor</x:v>
+        <x:v>protocol.commit-delay-reveal</x:v>
       </x:c>
       <x:c r="C138" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13915,12 +14509,173 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E138" s="32" t="str">
+        <x:v>Commit-delay-reveal composes a cryptographic commitment with a timed reveal, so the learner first needs the hiding and binding commitment model.</x:v>
+      </x:c>
+      <x:c r="F138" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
+      </x:c>
+      <x:c r="G138" s="32" t="str">
+        <x:v>The delay/reveal composition is the node's distinct outcome.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" s="32" t="str">
+        <x:v>protocol.dust-policy</x:v>
+      </x:c>
+      <x:c r="B139" s="32" t="str">
+        <x:v>security.dust-attack</x:v>
+      </x:c>
+      <x:c r="C139" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D139" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E139" s="32" t="str">
+        <x:v>Dust attacks exploit the distinction between tiny-output relay policy and the ability to place trace-value UTXOs in a wallet.</x:v>
+      </x:c>
+      <x:c r="F139" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+      </x:c>
+      <x:c r="G139" s="32" t="str">
+        <x:v>Policy threshold is direct context for the attack mechanism.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" s="32" t="str">
+        <x:v>privacy.pseudonymity</x:v>
+      </x:c>
+      <x:c r="B140" s="32" t="str">
+        <x:v>security.dust-attack</x:v>
+      </x:c>
+      <x:c r="C140" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D140" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E140" s="32" t="str">
+        <x:v>The privacy harm of dusting comes from linking future spends and wallet activity, so learners need the pseudonymity and linkage model.</x:v>
+      </x:c>
+      <x:c r="F140" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+      </x:c>
+      <x:c r="G140" s="32" t="str">
+        <x:v>Keep privacy linkage direct; it is not inherited through dust policy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" s="32" t="str">
+        <x:v>fundamentals.neutrality</x:v>
+      </x:c>
+      <x:c r="B141" s="32" t="str">
+        <x:v>dev.permissionless-development</x:v>
+      </x:c>
+      <x:c r="C141" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D141" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E141" s="32" t="str">
+        <x:v>Permissionless development depends on a neutral protocol that does not select which users or applications may participate.</x:v>
+      </x:c>
+      <x:c r="F141" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G141" s="32" t="str">
+        <x:v>Neutrality supplies the protocol property; the BIPs process supplies the change/proposal lifecycle below.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="32" t="str">
+        <x:v>dev.bips-process</x:v>
+      </x:c>
+      <x:c r="B142" s="32" t="str">
+        <x:v>dev.permissionless-development</x:v>
+      </x:c>
+      <x:c r="C142" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D142" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E142" s="32" t="str">
+        <x:v>Learners need the proposal and deployment process to distinguish building permissionlessly from changing Bitcoin's consensus rules without broad adoption.</x:v>
+      </x:c>
+      <x:c r="F142" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G142" s="32" t="str">
+        <x:v>Review culture remains related but is not a direct prerequisite for permissionless access.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="32" t="str">
+        <x:v>dev.reproducible-builds</x:v>
+      </x:c>
+      <x:c r="B143" s="32" t="str">
+        <x:v>dev.bootstrappable-builds</x:v>
+      </x:c>
+      <x:c r="C143" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D143" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E143" s="32" t="str">
+        <x:v>Bootstrappable builds extend reproducible builds by reducing trust in the compiler and build-tool binaries used to produce the reproducible output.</x:v>
+      </x:c>
+      <x:c r="F143" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G143" s="32" t="str">
+        <x:v>Keep this as a direct downstream edge; the node is not a duplicate alias for reproducible builds.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" s="32" t="str">
+        <x:v>protocol.transaction-lifecycle</x:v>
+      </x:c>
+      <x:c r="B144" s="32" t="str">
+        <x:v>protocol.proof-of-payment</x:v>
+      </x:c>
+      <x:c r="C144" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D144" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E144" s="32" t="str">
+        <x:v>Proof of Payment refers to a prior payment and reconstructs a transaction-shaped proof, so learners need the transaction lifecycle first.</x:v>
+      </x:c>
+      <x:c r="F144" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="G144" s="32" t="str">
+        <x:v>Direct payment context; wallet UX and URI transport remain downstream or optional details.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" s="32" t="str">
+        <x:v>protocol.ephemeral-anchors</x:v>
+      </x:c>
+      <x:c r="B145" s="32" t="str">
+        <x:v>protocol.pay-to-anchor</x:v>
+      </x:c>
+      <x:c r="C145" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D145" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E145" s="32" t="str">
         <x:v>Pay to Anchor is a keyless refinement of the anchor-output and package-relay fee-bumping pattern, so learners need that broader context first.</x:v>
       </x:c>
-      <x:c r="F138" s="32" t="str">
+      <x:c r="F145" s="32" t="str">
         <x:v>source.bitcoin-bips</x:v>
       </x:c>
-      <x:c r="G138" s="32" t="str">
+      <x:c r="G145" s="32" t="str">
         <x:v>BIP 431/TRUC is related anti-pinning context, not an inherent prerequisite.</x:v>
       </x:c>
     </x:row>
@@ -13930,10 +14685,10 @@
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C138">
+    <x:dataValidation type="list" sqref="C12:C145">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D138">
+    <x:dataValidation type="list" sqref="D12:D145">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -16783,16 +17538,222 @@
         <x:v>Keep these as audit candidates and source references, but do not mint product/API wrapper nodes.</x:v>
       </x:c>
     </x:row>
+    <x:row r="119">
+      <x:c r="A119" s="32" t="str">
+        <x:v>decision.101-perguntas-bitcoin-1ed-inventory</x:v>
+      </x:c>
+      <x:c r="B119" s="32" t="str">
+        <x:v>inventory</x:v>
+      </x:c>
+      <x:c r="C119" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="D119" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E119" s="32" t="str">
+        <x:v>The completed first edition contains 101 numbered Markdown chapters and was reviewed as a full source family. The unfinished second edition was excluded from this pass.</x:v>
+      </x:c>
+      <x:c r="F119" s="32" t="str"/>
+      <x:c r="G119" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="H119" s="32" t="str">
+        <x:v>All 101 chapter files have a normalized disposition; no claim is made about the incomplete second edition.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" s="32" t="str">
+        <x:v>decision.101-satoshi-nakamoto-slice</x:v>
+      </x:c>
+      <x:c r="B120" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C120" s="32" t="str">
+        <x:v>history.satoshi-nakamoto</x:v>
+      </x:c>
+      <x:c r="D120" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E120" s="32" t="str">
+        <x:v>The creator pseudonym and disappearance are a distinct historical/governance learning outcome not represented by the generic whitepaper and early-history nodes.</x:v>
+      </x:c>
+      <x:c r="F120" s="32" t="str">
+        <x:v>history.satoshi-nakamoto, history.cypherpunk-roots-bitcoin-origin, history.bitcoin-whitepaper</x:v>
+      </x:c>
+      <x:c r="G120" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="H120" s="32" t="str">
+        <x:v>Keep speculative identity claims out of the node; focus on the pseudonym, launch authorship, and founder independence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" s="32" t="str">
+        <x:v>decision.101-bitcoin-denominations-slice</x:v>
+      </x:c>
+      <x:c r="B121" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C121" s="32" t="str">
+        <x:v>economics.bitcoin-denominations</x:v>
+      </x:c>
+      <x:c r="D121" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E121" s="32" t="str">
+        <x:v>BTC and satoshis are concrete units learners must recognize and use; they are not redundant with scarcity or monetary properties.</x:v>
+      </x:c>
+      <x:c r="F121" s="32" t="str">
+        <x:v>economics.bitcoin-denominations, fundamentals.money-properties, fundamentals.digital-scarcity</x:v>
+      </x:c>
+      <x:c r="G121" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="H121" s="32" t="str">
+        <x:v>Do not create separate nodes for capitalization, protocol/software naming, BTC, and satoshi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" s="32" t="str">
+        <x:v>decision.101-block-subsidy-slice</x:v>
+      </x:c>
+      <x:c r="B122" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C122" s="32" t="str">
+        <x:v>economics.block-subsidy</x:v>
+      </x:c>
+      <x:c r="D122" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E122" s="32" t="str">
+        <x:v>The newly issued component of miner revenue is a distinct issuance concept even though coinbase transactions and halvings already exist.</x:v>
+      </x:c>
+      <x:c r="F122" s="32" t="str">
+        <x:v>economics.block-subsidy, protocol.coinbase-transaction, protocol.halving, economics.miner-revenue-composition</x:v>
+      </x:c>
+      <x:c r="G122" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="H122" s="32" t="str">
+        <x:v>Keep transaction fees separate from subsidy and avoid a redundant direct edge to halving.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" s="32" t="str">
+        <x:v>decision.101-quantum-threat-slice</x:v>
+      </x:c>
+      <x:c r="B123" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C123" s="32" t="str">
+        <x:v>security.quantum-computing-threat</x:v>
+      </x:c>
+      <x:c r="D123" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E123" s="32" t="str">
+        <x:v>The quantum threat model spans signature authorization and proof-of-work and is not replaced by adding one post-quantum primitive such as Lamport signatures.</x:v>
+      </x:c>
+      <x:c r="F123" s="32" t="str">
+        <x:v>security.quantum-computing-threat, fundamentals.digital-signatures, protocol.proof-of-work, fundamentals.lamport-signatures</x:v>
+      </x:c>
+      <x:c r="G123" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="H123" s="32" t="str">
+        <x:v>Keep proof-of-work as threat-model context and mitigation primitives as resources or neighboring nodes; do not add a redundant direct proof-of-work edge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" s="32" t="str">
+        <x:v>decision.101-ordinals-inscriptions-slice</x:v>
+      </x:c>
+      <x:c r="B124" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C124" s="32" t="str">
+        <x:v>extension.ordinals-inscriptions</x:v>
+      </x:c>
+      <x:c r="D124" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E124" s="32" t="str">
+        <x:v>Ordinals and inscriptions are a distinct Bitcoin application family with a real learner outcome around satoshi numbering, witness data, and block-space tradeoffs.</x:v>
+      </x:c>
+      <x:c r="F124" s="32" t="str">
+        <x:v>extension.ordinals-inscriptions, protocol.taproot, protocol.witness-structure, protocol.op-return</x:v>
+      </x:c>
+      <x:c r="G124" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="H124" s="32" t="str">
+        <x:v>Do not expand individual collections, marketplaces, or inscription formats into separate nodes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" s="32" t="str">
+        <x:v>decision.101-proof-of-existence-slice</x:v>
+      </x:c>
+      <x:c r="B125" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C125" s="32" t="str">
+        <x:v>extension.proof-of-existence</x:v>
+      </x:c>
+      <x:c r="D125" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E125" s="32" t="str">
+        <x:v>Bitcoin-anchored timestamping is a reusable application concept illustrated by the Genesis Block and OpenTimestamps, not merely an OP_RETURN implementation detail.</x:v>
+      </x:c>
+      <x:c r="F125" s="32" t="str">
+        <x:v>extension.proof-of-existence, fundamentals.commitment-schemes, protocol.op-return, history.genesis-block</x:v>
+      </x:c>
+      <x:c r="G125" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="H125" s="32" t="str">
+        <x:v>Use commitments and off-chain aggregation as the conceptual center; keep OpenTimestamps as a resource.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" s="32" t="str">
+        <x:v>decision.101-contextual-exclusions</x:v>
+      </x:c>
+      <x:c r="B126" s="32" t="str">
+        <x:v>exclusion</x:v>
+      </x:c>
+      <x:c r="C126" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="D126" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E126" s="32" t="str">
+        <x:v>Stablecoins, altcoins, exchanges, HODL, and named offline transport products are comparative, cultural, legal, or product context rather than missing Bitcoin graph concepts.</x:v>
+      </x:c>
+      <x:c r="F126" s="32" t="str">
+        <x:v>economics.stablecoins, economics.altcoins, ops.exchange-custody, ops.offline-bitcoin-transport, economics.hodling, extension.sidechains, fundamentals.bitcoin-layers</x:v>
+      </x:c>
+      <x:c r="G126" s="32" t="str">
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+      </x:c>
+      <x:c r="H126" s="32" t="str">
+        <x:v>Offline transport examples merge into ops.mesh-networks; the other candidates remain source context without learner-facing nodes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B118">
+    <x:dataValidation type="list" sqref="B12:B126">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D118">
+    <x:dataValidation type="list" sqref="D12:D126">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -16845,7 +17806,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.71990200232</x:v>
+        <x:v>46214.757944282406</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -16853,7 +17814,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>58</x:v>
+        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -16861,7 +17822,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>58</x:v>
+        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -16869,7 +17830,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>147</x:v>
+        <x:v>158</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -16877,7 +17838,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>127</x:v>
+        <x:v>134</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -16901,7 +17862,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>93</x:v>
+        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add Spark protocol concept
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R9c284e7c62df4b80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R715056b261ee4006"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R0fdaba2da65a40dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R88475d6a5d104e02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R0ec50bb3c72c41dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Re8f80b25478343de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rcd89c3d133654fb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rdc1578168c024e74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R2d3ac541ebbc4270"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R62086872aaee405b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rf53e320eac4f4bb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R4638edeb17084cf3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3313,22 +3313,69 @@
         <x:v>Complete first-edition pass over all 101 chapter files. Six concepts were added, six candidates were merged or excluded: Satoshi Nakamoto, Bitcoin denominations and satoshis, block subsidy, quantum-computing threats, Ordinals and inscriptions, and proof of existence/timestamping. Stablecoins, altcoins, exchanges, satellites, and named products remain contextual or implementation/product scope. The unfinished second edition was intentionally excluded.</x:v>
       </x:c>
     </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="32" t="str">
+        <x:v>source.spark-protocol</x:v>
+      </x:c>
+      <x:c r="B71" s="32" t="str">
+        <x:v>Spark Bitcoin Layer 2 Protocol</x:v>
+      </x:c>
+      <x:c r="C71" s="32" t="str">
+        <x:v>https://docs.spark.money/start/overview</x:v>
+      </x:c>
+      <x:c r="D71" s="32" t="str">
+        <x:v>protocol-documentation-repository</x:v>
+      </x:c>
+      <x:c r="E71" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F71" s="32" t="str">
+        <x:v>Spark's statechain-based Bitcoin Layer 2 protocol, operator model, off-chain asset transfers, Lightning interoperability, and developer implementation.</x:v>
+      </x:c>
+      <x:c r="G71" s="32" t="str">
+        <x:v>Track the official overview and open-source repository as one protocol cluster. Separate the learner-facing Spark architecture from generic statechains, threshold-signature internals, and product-specific wallet workflows.</x:v>
+      </x:c>
+      <x:c r="H71" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I71" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J71" s="32" t="str">
+        <x:v>Normalized</x:v>
+      </x:c>
+      <x:c r="K71" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L71" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M71" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N71" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O71" s="32" t="str">
+        <x:v>Added Spark as a distinct implementation/protocol node downstream of Statechains; operator coordination and Lightning interoperability remain inside the Spark concept rather than becoming separate nodes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H70">
+    <x:dataValidation type="list" sqref="H12:H71">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I70">
+    <x:dataValidation type="list" sqref="I12:I71">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J70">
+    <x:dataValidation type="list" sqref="J12:J71">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K70">
+    <x:dataValidation type="list" sqref="K12:K71">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11522,16 +11569,67 @@
         <x:v>Skip as culture/behavior; volatility and savings concepts remain the relevant learner outcomes.</x:v>
       </x:c>
     </x:row>
+    <x:row r="170">
+      <x:c r="A170" s="32" t="str">
+        <x:v>extension.spark</x:v>
+      </x:c>
+      <x:c r="B170" s="32" t="str">
+        <x:v>Spark Protocol</x:v>
+      </x:c>
+      <x:c r="C170" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D170" s="32" t="str">
+        <x:v>source.spark-protocol</x:v>
+      </x:c>
+      <x:c r="E170" s="32" t="str">
+        <x:v>https://docs.spark.money/start/overview</x:v>
+      </x:c>
+      <x:c r="F170" s="32" t="str">
+        <x:v>Official Spark overview and open-source protocol repository</x:v>
+      </x:c>
+      <x:c r="G170" s="32" t="str"/>
+      <x:c r="H170" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I170" s="32" t="str">
+        <x:v>Spark is a concrete Bitcoin Layer 2 protocol with a distinct operator, transfer, and interoperability model built on statechain ideas; it is not merely an alias for the generic Statechains concept.</x:v>
+      </x:c>
+      <x:c r="J170" s="32" t="str">
+        <x:v>extension.statechains</x:v>
+      </x:c>
+      <x:c r="K170" s="32" t="str">
+        <x:v>extension.statechains</x:v>
+      </x:c>
+      <x:c r="L170" s="32" t="str">
+        <x:v>Statechains provide the architecture needed to understand Spark's off-chain ownership-transfer model; threshold-signature coordination is kept inside the node description rather than minted as an unreviewed implementation node.</x:v>
+      </x:c>
+      <x:c r="M170" s="32" t="str">
+        <x:v>Spark Bitcoin L2, Spark statechain protocol</x:v>
+      </x:c>
+      <x:c r="N170" s="32" t="str">
+        <x:v>bitcoin-l2, statechains, off-chain, lightning</x:v>
+      </x:c>
+      <x:c r="O170" s="32" t="str">
+        <x:v>60m</x:v>
+      </x:c>
+      <x:c r="P170" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q170" s="32" t="str">
+        <x:v>Added at the user's request after confirming the official protocol documentation and repository.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H169">
+    <x:dataValidation type="list" sqref="H12:H170">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P169">
+    <x:dataValidation type="list" sqref="P12:P170">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11599,10 +11697,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="32" t="str">
-        <x:v>history.cypherpunk-roots-bitcoin-origin</x:v>
+        <x:v>extension.statechains</x:v>
       </x:c>
       <x:c r="B12" s="32" t="str">
-        <x:v>history.satoshi-nakamoto</x:v>
+        <x:v>extension.spark</x:v>
       </x:c>
       <x:c r="C12" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11611,10 +11709,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E12" s="32" t="str">
-        <x:v>Satoshi's pseudonym and founder independence are best understood in the context of Bitcoin's cypherpunk roots and origin story.</x:v>
+        <x:v>Spark's architecture extends statechain-style off-chain ownership transfer with a distributed operator set and Lightning interoperability.</x:v>
       </x:c>
       <x:c r="F12" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.spark-protocol</x:v>
       </x:c>
       <x:c r="G12" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11622,10 +11720,10 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="32" t="str">
-        <x:v>fundamentals.money-properties</x:v>
+        <x:v>history.cypherpunk-roots-bitcoin-origin</x:v>
       </x:c>
       <x:c r="B13" s="32" t="str">
-        <x:v>economics.bitcoin-denominations</x:v>
+        <x:v>history.satoshi-nakamoto</x:v>
       </x:c>
       <x:c r="C13" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11634,7 +11732,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E13" s="32" t="str">
-        <x:v>The learner needs a basic monetary-unit model before BTC and satoshis are meaningful denominations.</x:v>
+        <x:v>Satoshi's pseudonym and founder independence are best understood in the context of Bitcoin's cypherpunk roots and origin story.</x:v>
       </x:c>
       <x:c r="F13" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
@@ -11645,10 +11743,10 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="32" t="str">
-        <x:v>protocol.coinbase-transaction</x:v>
+        <x:v>fundamentals.money-properties</x:v>
       </x:c>
       <x:c r="B14" s="32" t="str">
-        <x:v>economics.block-subsidy</x:v>
+        <x:v>economics.bitcoin-denominations</x:v>
       </x:c>
       <x:c r="C14" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11657,21 +11755,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E14" s="32" t="str">
-        <x:v>The block subsidy is the newly issued component claimed by a coinbase transaction.</x:v>
+        <x:v>The learner needs a basic monetary-unit model before BTC and satoshis are meaningful denominations.</x:v>
       </x:c>
       <x:c r="F14" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G14" s="32" t="str">
-        <x:v>The coinbase node already carries the halving prerequisite, so no redundant direct halving edge is added.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="32" t="str">
-        <x:v>fundamentals.digital-signatures</x:v>
+        <x:v>protocol.coinbase-transaction</x:v>
       </x:c>
       <x:c r="B15" s="32" t="str">
-        <x:v>security.quantum-computing-threat</x:v>
+        <x:v>economics.block-subsidy</x:v>
       </x:c>
       <x:c r="C15" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11680,21 +11778,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E15" s="32" t="str">
-        <x:v>Quantum attacks on public-key authorization require understanding ordinary Bitcoin signature security first.</x:v>
+        <x:v>The block subsidy is the newly issued component claimed by a coinbase transaction.</x:v>
       </x:c>
       <x:c r="F15" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G15" s="32" t="str">
-        <x:v>Source-driven bridge edge.</x:v>
+        <x:v>The coinbase node already carries the halving prerequisite, so no redundant direct halving edge is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>fundamentals.digital-signatures</x:v>
       </x:c>
       <x:c r="B16" s="32" t="str">
-        <x:v>extension.ordinals-inscriptions</x:v>
+        <x:v>security.quantum-computing-threat</x:v>
       </x:c>
       <x:c r="C16" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11703,7 +11801,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E16" s="32" t="str">
-        <x:v>The source explains inscriptions as a Taproot-era witness-data application.</x:v>
+        <x:v>Quantum attacks on public-key authorization require understanding ordinary Bitcoin signature security first.</x:v>
       </x:c>
       <x:c r="F16" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
@@ -11714,7 +11812,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="32" t="str">
-        <x:v>protocol.witness-structure</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B17" s="32" t="str">
         <x:v>extension.ordinals-inscriptions</x:v>
@@ -11726,7 +11824,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E17" s="32" t="str">
-        <x:v>Witness structure is needed to understand where inscription data is carried and how it affects block space.</x:v>
+        <x:v>The source explains inscriptions as a Taproot-era witness-data application.</x:v>
       </x:c>
       <x:c r="F17" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
@@ -11737,10 +11835,10 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>protocol.witness-structure</x:v>
       </x:c>
       <x:c r="B18" s="32" t="str">
-        <x:v>extension.proof-of-existence</x:v>
+        <x:v>extension.ordinals-inscriptions</x:v>
       </x:c>
       <x:c r="C18" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11749,7 +11847,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E18" s="32" t="str">
-        <x:v>Timestamp proofs commit evidence without requiring the complete document to be stored on-chain.</x:v>
+        <x:v>Witness structure is needed to understand where inscription data is carried and how it affects block space.</x:v>
       </x:c>
       <x:c r="F18" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
@@ -11760,10 +11858,10 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="32" t="str">
-        <x:v>protocol.tagged-hashes</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="B19" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>extension.proof-of-existence</x:v>
       </x:c>
       <x:c r="C19" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11772,10 +11870,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E19" s="32" t="str">
-        <x:v>TapTweak is defined using tagged hashes directly in Taproot key tweaking.</x:v>
+        <x:v>Timestamp proofs commit evidence without requiring the complete document to be stored on-chain.</x:v>
       </x:c>
       <x:c r="F19" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G19" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11783,7 +11881,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="32" t="str">
-        <x:v>protocol.x-only-public-keys</x:v>
+        <x:v>protocol.tagged-hashes</x:v>
       </x:c>
       <x:c r="B20" s="32" t="str">
         <x:v>protocol.taptweak</x:v>
@@ -11795,7 +11893,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E20" s="32" t="str">
-        <x:v>TapTweak operates on x-only public keys in the Taproot construction.</x:v>
+        <x:v>TapTweak is defined using tagged hashes directly in Taproot key tweaking.</x:v>
       </x:c>
       <x:c r="F20" s="32" t="str">
         <x:v>source.optech-schnorr-taproot-workshop</x:v>
@@ -11806,10 +11904,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="str">
+        <x:v>protocol.x-only-public-keys</x:v>
+      </x:c>
+      <x:c r="B21" s="32" t="str">
         <x:v>protocol.taptweak</x:v>
-      </x:c>
-      <x:c r="B21" s="32" t="str">
-        <x:v>protocol.taproot-key-path-spends</x:v>
       </x:c>
       <x:c r="C21" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11818,21 +11916,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E21" s="32" t="str">
-        <x:v>A key-path spend verifies against the tweaked Taproot output key, so learners need the tweak mechanism before the spending mode makes sense.</x:v>
+        <x:v>TapTweak operates on x-only public keys in the Taproot construction.</x:v>
       </x:c>
       <x:c r="F21" s="32" t="str">
         <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G21" s="32" t="str">
-        <x:v>Direct parent keeps the node focused on the spend mode rather than on broad Taproot overview material.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32" t="str">
-        <x:v>protocol.taptree</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="B22" s="32" t="str">
-        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
+        <x:v>protocol.taproot-key-path-spends</x:v>
       </x:c>
       <x:c r="C22" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11841,13 +11939,13 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E22" s="32" t="str">
-        <x:v>The inclusion proof only makes sense after the learner understands the TapTree structure.</x:v>
+        <x:v>A key-path spend verifies against the tweaked Taproot output key, so learners need the tweak mechanism before the spending mode makes sense.</x:v>
       </x:c>
       <x:c r="F22" s="32" t="str">
         <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G22" s="32" t="str">
-        <x:v>Source-driven bridge edge.</x:v>
+        <x:v>Direct parent keeps the node focused on the spend mode rather than on broad Taproot overview material.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -11855,7 +11953,7 @@
         <x:v>protocol.taptree</x:v>
       </x:c>
       <x:c r="B23" s="32" t="str">
-        <x:v>protocol.huffman-optimized-taptrees</x:v>
+        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
       </x:c>
       <x:c r="C23" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11864,7 +11962,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E23" s="32" t="str">
-        <x:v>Huffman optimization is a refinement of how TapTree leaves are arranged.</x:v>
+        <x:v>The inclusion proof only makes sense after the learner understands the TapTree structure.</x:v>
       </x:c>
       <x:c r="F23" s="32" t="str">
         <x:v>source.optech-schnorr-taproot-workshop</x:v>
@@ -11875,10 +11973,10 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="str">
-        <x:v>protocol.softfork-hardfork</x:v>
+        <x:v>protocol.taptree</x:v>
       </x:c>
       <x:c r="B24" s="32" t="str">
-        <x:v>protocol.chain-split-risk</x:v>
+        <x:v>protocol.huffman-optimized-taptrees</x:v>
       </x:c>
       <x:c r="C24" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11887,21 +11985,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E24" s="32" t="str">
-        <x:v>Split risk is a downstream consequence of incompatible upgrade paths, so learners should understand the compatibility boundary first.</x:v>
+        <x:v>Huffman optimization is a refinement of how TapTree leaves are arranged.</x:v>
       </x:c>
       <x:c r="F24" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G24" s="32" t="str">
-        <x:v>Direct edge chosen over activation-history case studies because those are downstream examples, not prerequisites.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.softfork-hardfork</x:v>
       </x:c>
       <x:c r="B25" s="32" t="str">
-        <x:v>protocol.tapscript</x:v>
+        <x:v>protocol.chain-split-risk</x:v>
       </x:c>
       <x:c r="C25" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11910,21 +12008,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E25" s="32" t="str">
-        <x:v>Tapscript is a Taproot-specific script version, so learners need the Taproot spend context before its rule changes make sense.</x:v>
+        <x:v>Split risk is a downstream consequence of incompatible upgrade paths, so learners should understand the compatibility boundary first.</x:v>
       </x:c>
       <x:c r="F25" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G25" s="32" t="str">
-        <x:v>Direct edge keeps the node scoped to the Taproot family without collapsing it into a generic script refresher.</x:v>
+        <x:v>Direct edge chosen over activation-history case studies because those are downstream examples, not prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="str">
-        <x:v>custody.psbt</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B26" s="32" t="str">
-        <x:v>dev.taproot-psbt-fields</x:v>
+        <x:v>protocol.tapscript</x:v>
       </x:c>
       <x:c r="C26" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11933,18 +12031,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E26" s="32" t="str">
-        <x:v>Taproot PSBT fields extend the base PSBT container, so learners need the general workflow and field model before the Taproot additions make sense.</x:v>
+        <x:v>Tapscript is a Taproot-specific script version, so learners need the Taproot spend context before its rule changes make sense.</x:v>
       </x:c>
       <x:c r="F26" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G26" s="32" t="str">
-        <x:v>Direct edge keeps the slice anchored on the generic PSBT exchange model rather than on a narrower implementation variant.</x:v>
+        <x:v>Direct edge keeps the node scoped to the Taproot family without collapsing it into a generic script refresher.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>custody.psbt</x:v>
       </x:c>
       <x:c r="B27" s="32" t="str">
         <x:v>dev.taproot-psbt-fields</x:v>
@@ -11956,21 +12054,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E27" s="32" t="str">
-        <x:v>These fields carry Taproot-specific keys, scripts, and Merkle-path data, so learners need the Taproot spend model before the PSBT extensions are meaningful.</x:v>
+        <x:v>Taproot PSBT fields extend the base PSBT container, so learners need the general workflow and field model before the Taproot additions make sense.</x:v>
       </x:c>
       <x:c r="F27" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G27" s="32" t="str">
-        <x:v>The direct dev.psbt-v2 edge was intentionally dropped because BIP371 applies to PSBTv0 and PSBTv2.</x:v>
+        <x:v>Direct edge keeps the slice anchored on the generic PSBT exchange model rather than on a narrower implementation variant.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32" t="str">
-        <x:v>protocol.softfork-hardfork</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B28" s="32" t="str">
-        <x:v>protocol.accidental-confiscation</x:v>
+        <x:v>dev.taproot-psbt-fields</x:v>
       </x:c>
       <x:c r="C28" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11979,21 +12077,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E28" s="32" t="str">
-        <x:v>Accidental confiscation is a failure mode caused by new soft-fork restrictions, so learners need the soft-fork compatibility model before the risk is intelligible.</x:v>
+        <x:v>These fields carry Taproot-specific keys, scripts, and Merkle-path data, so learners need the Taproot spend model before the PSBT extensions are meaningful.</x:v>
       </x:c>
       <x:c r="F28" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G28" s="32" t="str">
-        <x:v>Direct edge chosen over chain-split-risk and standardness-policy because those branches add context but are not required for the core failure mode.</x:v>
+        <x:v>The direct dev.psbt-v2 edge was intentionally dropped because BIP371 applies to PSBTv0 and PSBTv2.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="32" t="str">
-        <x:v>protocol.fee-market</x:v>
+        <x:v>protocol.softfork-hardfork</x:v>
       </x:c>
       <x:c r="B29" s="32" t="str">
-        <x:v>custody.coin-selection</x:v>
+        <x:v>protocol.accidental-confiscation</x:v>
       </x:c>
       <x:c r="C29" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12002,21 +12100,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E29" s="32" t="str">
-        <x:v>Wallets choose different UTXO sets partly to minimize transaction size and fee cost, so fee pressure is a direct part of the concept.</x:v>
+        <x:v>Accidental confiscation is a failure mode caused by new soft-fork restrictions, so learners need the soft-fork compatibility model before the risk is intelligible.</x:v>
       </x:c>
       <x:c r="F29" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G29" s="32" t="str">
-        <x:v>Direct edge keeps the node connected to transaction-cost tradeoffs rather than only to wallet UX.</x:v>
+        <x:v>Direct edge chosen over chain-split-risk and standardness-policy because those branches add context but are not required for the core failure mode.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>protocol.fee-market</x:v>
       </x:c>
       <x:c r="B30" s="32" t="str">
-        <x:v>protocol.change-outputs</x:v>
+        <x:v>custody.coin-selection</x:v>
       </x:c>
       <x:c r="C30" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12025,21 +12123,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E30" s="32" t="str">
-        <x:v>Change is a specific kind of transaction output, so learners need the basic output and spendability model before the leftover-value pattern makes sense.</x:v>
+        <x:v>Wallets choose different UTXO sets partly to minimize transaction size and fee cost, so fee pressure is a direct part of the concept.</x:v>
       </x:c>
       <x:c r="F30" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G30" s="32" t="str">
-        <x:v>Direct edge keeps the node between raw output structure and the later wallet-decision branch.</x:v>
+        <x:v>Direct edge keeps the node connected to transaction-cost tradeoffs rather than only to wallet UX.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B31" s="32" t="str">
-        <x:v>dev.taproot-descriptors</x:v>
+        <x:v>protocol.change-outputs</x:v>
       </x:c>
       <x:c r="C31" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12048,18 +12146,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E31" s="32" t="str">
-        <x:v>Taproot descriptors extend the general descriptor grammar, so learners need the base descriptor model before the tr() specialization makes sense.</x:v>
+        <x:v>Change is a specific kind of transaction output, so learners need the basic output and spendability model before the leftover-value pattern makes sense.</x:v>
       </x:c>
       <x:c r="F31" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G31" s="32" t="str">
-        <x:v>Direct edge keeps the node scoped to descriptor structure instead of wallet import behavior.</x:v>
+        <x:v>Direct edge keeps the node between raw output structure and the later wallet-decision branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B32" s="32" t="str">
         <x:v>dev.taproot-descriptors</x:v>
@@ -12071,21 +12169,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E32" s="32" t="str">
-        <x:v>The tr() descriptor exists specifically to encode P2TR outputs and optional Taproot script-path commitments, so learners need the Taproot output model first.</x:v>
+        <x:v>Taproot descriptors extend the general descriptor grammar, so learners need the base descriptor model before the tr() specialization makes sense.</x:v>
       </x:c>
       <x:c r="F32" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G32" s="32" t="str">
-        <x:v>Direct edge keeps the node grounded in Taproot output semantics rather than in generic descriptor syntax alone.</x:v>
+        <x:v>Direct edge keeps the node scoped to descriptor structure instead of wallet import behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="32" t="str">
-        <x:v>protocol.transaction-pinning</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B33" s="32" t="str">
-        <x:v>protocol.version-3-transaction-relay</x:v>
+        <x:v>dev.taproot-descriptors</x:v>
       </x:c>
       <x:c r="C33" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12094,21 +12192,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E33" s="32" t="str">
-        <x:v>Version 3 relay is a targeted policy response to transaction pinning, so learners should understand the attack class before the mitigation.</x:v>
+        <x:v>The tr() descriptor exists specifically to encode P2TR outputs and optional Taproot script-path commitments, so learners need the Taproot output model first.</x:v>
       </x:c>
       <x:c r="F33" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G33" s="32" t="str">
-        <x:v>Direct edge chosen over package-relay because the pinning problem is the narrower immediate teaching need.</x:v>
+        <x:v>Direct edge keeps the node grounded in Taproot output semantics rather than in generic descriptor syntax alone.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="32" t="str">
-        <x:v>fundamentals.trustlessness</x:v>
+        <x:v>protocol.transaction-pinning</x:v>
       </x:c>
       <x:c r="B34" s="32" t="str">
-        <x:v>fundamentals.validation-sovereignty</x:v>
+        <x:v>protocol.version-3-transaction-relay</x:v>
       </x:c>
       <x:c r="C34" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12117,21 +12215,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E34" s="32" t="str">
-        <x:v>Validation sovereignty is an applied consequence of trustlessness and verification culture.</x:v>
+        <x:v>Version 3 relay is a targeted policy response to transaction pinning, so learners should understand the attack class before the mitigation.</x:v>
       </x:c>
       <x:c r="F34" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G34" s="32" t="str">
-        <x:v>Bridge edge inferred from philosophy sequencing.</x:v>
+        <x:v>Direct edge chosen over package-relay because the pinning problem is the narrower immediate teaching need.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="32" t="str">
-        <x:v>ops.run-full-node</x:v>
+        <x:v>fundamentals.trustlessness</x:v>
       </x:c>
       <x:c r="B35" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>fundamentals.validation-sovereignty</x:v>
       </x:c>
       <x:c r="C35" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12140,18 +12238,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E35" s="32" t="str">
-        <x:v>Learners need the full-node baseline before they can understand which validation guarantees a light client gives up.</x:v>
+        <x:v>Validation sovereignty is an applied consequence of trustlessness and verification culture.</x:v>
       </x:c>
       <x:c r="F35" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G35" s="32" t="str">
-        <x:v>Bridge edge inferred from full-node versus lightweight-client contrast.</x:v>
+        <x:v>Bridge edge inferred from philosophy sequencing.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="32" t="str">
-        <x:v>protocol.compact-block-filters</x:v>
+        <x:v>ops.run-full-node</x:v>
       </x:c>
       <x:c r="B36" s="32" t="str">
         <x:v>protocol.light-client-trust-model</x:v>
@@ -12163,21 +12261,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E36" s="32" t="str">
-        <x:v>Compact block filters provide the modern filtered-client mechanism that anchors the trust-model comparison.</x:v>
+        <x:v>Learners need the full-node baseline before they can understand which validation guarantees a light client gives up.</x:v>
       </x:c>
       <x:c r="F36" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G36" s="32" t="str">
-        <x:v>Kept additive and conceptual instead of rewiring older light-client mechanism leaves in the same slice.</x:v>
+        <x:v>Bridge edge inferred from full-node versus lightweight-client contrast.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="32" t="str">
-        <x:v>fundamentals.validation-sovereignty</x:v>
+        <x:v>protocol.compact-block-filters</x:v>
       </x:c>
       <x:c r="B37" s="32" t="str">
-        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="C37" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12186,18 +12284,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E37" s="32" t="str">
-        <x:v>The comparison only matters once the learner understands why self-validation is valuable in the first place.</x:v>
+        <x:v>Compact block filters provide the modern filtered-client mechanism that anchors the trust-model comparison.</x:v>
       </x:c>
       <x:c r="F37" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G37" s="32" t="str">
-        <x:v>User-facing prerequisite edge for the wallet-mode decision.</x:v>
+        <x:v>Kept additive and conceptual instead of rewiring older light-client mechanism leaves in the same slice.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>fundamentals.validation-sovereignty</x:v>
       </x:c>
       <x:c r="B38" s="32" t="str">
         <x:v>ops.full-node-vs-lightweight-wallet</x:v>
@@ -12209,21 +12307,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E38" s="32" t="str">
-        <x:v>Learners need the mechanism-level trust tradeoffs before comparing full-node wallets with lightweight clients.</x:v>
+        <x:v>The comparison only matters once the learner understands why self-validation is valuable in the first place.</x:v>
       </x:c>
       <x:c r="F38" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G38" s="32" t="str">
-        <x:v>First downstream consumer for the light-client trust branch.</x:v>
+        <x:v>User-facing prerequisite edge for the wallet-mode decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="B39" s="32" t="str">
-        <x:v>protocol.p2pk</x:v>
+        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
       </x:c>
       <x:c r="C39" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12232,21 +12330,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E39" s="32" t="str">
-        <x:v>P2PK is a concrete legacy script template, so learners first need the locking and unlocking model from Bitcoin Script.</x:v>
+        <x:v>Learners need the mechanism-level trust tradeoffs before comparing full-node wallets with lightweight clients.</x:v>
       </x:c>
       <x:c r="F39" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G39" s="32" t="str">
-        <x:v>Chosen as the first script-history leaf from Decoding after dedupe and direct-edge review.</x:v>
+        <x:v>First downstream consumer for the light-client trust branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="32" t="str">
-        <x:v>fundamentals.schnorr-signatures</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B40" s="32" t="str">
-        <x:v>security.nonce-reuse-attack</x:v>
+        <x:v>protocol.p2pk</x:v>
       </x:c>
       <x:c r="C40" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12255,21 +12353,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E40" s="32" t="str">
-        <x:v>The nonce-reuse failure only makes sense after the learner understands the Schnorr signing flow that produces the nonce and signature pair.</x:v>
+        <x:v>P2PK is a concrete legacy script template, so learners first need the locking and unlocking model from Bitcoin Script.</x:v>
       </x:c>
       <x:c r="F40" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G40" s="32" t="str">
-        <x:v>Chosen as a narrow additive security slice without bundling it to custody-side defenses.</x:v>
+        <x:v>Chosen as the first script-history leaf from Decoding after dedupe and direct-edge review.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32" t="str">
-        <x:v>protocol.p2pk</x:v>
+        <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="B41" s="32" t="str">
-        <x:v>protocol.p2pkh</x:v>
+        <x:v>security.nonce-reuse-attack</x:v>
       </x:c>
       <x:c r="C41" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12278,18 +12376,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E41" s="32" t="str">
-        <x:v>P2PKH is easiest to understand as the hashed-public-key refinement of a direct public-key output.</x:v>
+        <x:v>The nonce-reuse failure only makes sense after the learner understands the Schnorr signing flow that produces the nonce and signature pair.</x:v>
       </x:c>
       <x:c r="F41" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G41" s="32" t="str">
-        <x:v>Chosen to preserve the output-template ladder without repeating the broader Script prerequisite directly.</x:v>
+        <x:v>Chosen as a narrow additive security slice without bundling it to custody-side defenses.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>protocol.p2pk</x:v>
       </x:c>
       <x:c r="B42" s="32" t="str">
         <x:v>protocol.p2pkh</x:v>
@@ -12301,21 +12399,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E42" s="32" t="str">
-        <x:v>Hash-based locking only makes sense once the learner understands what a hash commits to and why it can stand in for the public key until spend time.</x:v>
+        <x:v>P2PKH is easiest to understand as the hashed-public-key refinement of a direct public-key output.</x:v>
       </x:c>
       <x:c r="F42" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G42" s="32" t="str">
-        <x:v>Required to keep the node about public-key hashing rather than just script syntax.</x:v>
+        <x:v>Chosen to preserve the output-template ladder without repeating the broader Script prerequisite directly.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B43" s="32" t="str">
-        <x:v>protocol.op-checkmultisig</x:v>
+        <x:v>protocol.p2pkh</x:v>
       </x:c>
       <x:c r="C43" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12324,21 +12422,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E43" s="32" t="str">
-        <x:v>OP_CHECKMULTISIG is an opcode-level script mechanic, so learners first need the general Script model and stack execution basics.</x:v>
+        <x:v>Hash-based locking only makes sense once the learner understands what a hash commits to and why it can stand in for the public key until spend time.</x:v>
       </x:c>
       <x:c r="F43" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G43" s="32" t="str">
-        <x:v>Chosen as the mechanism bridge before protocol.p2ms.</x:v>
+        <x:v>Required to keep the node about public-key hashing rather than just script syntax.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="32" t="str">
+        <x:v>protocol.script</x:v>
+      </x:c>
+      <x:c r="B44" s="32" t="str">
         <x:v>protocol.op-checkmultisig</x:v>
-      </x:c>
-      <x:c r="B44" s="32" t="str">
-        <x:v>protocol.p2ms</x:v>
       </x:c>
       <x:c r="C44" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12347,21 +12445,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E44" s="32" t="str">
-        <x:v>Bare multisig is the concrete locking template built from OP_CHECKMULTISIG, so the opcode is the clean direct parent once introduced.</x:v>
+        <x:v>OP_CHECKMULTISIG is an opcode-level script mechanic, so learners first need the general Script model and stack execution basics.</x:v>
       </x:c>
       <x:c r="F44" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G44" s="32" t="str">
-        <x:v>Replaces the earlier curricular and wallet-semantic parent candidates.</x:v>
+        <x:v>Chosen as the mechanism bridge before protocol.p2ms.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="32" t="str">
+        <x:v>protocol.op-checkmultisig</x:v>
+      </x:c>
+      <x:c r="B45" s="32" t="str">
         <x:v>protocol.p2ms</x:v>
-      </x:c>
-      <x:c r="B45" s="32" t="str">
-        <x:v>protocol.bare-multisig-standardness</x:v>
       </x:c>
       <x:c r="C45" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12370,18 +12468,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E45" s="32" t="str">
-        <x:v>The relay treatment only makes sense once the learner understands what a bare multisig output actually is on-chain.</x:v>
+        <x:v>Bare multisig is the concrete locking template built from OP_CHECKMULTISIG, so the opcode is the clean direct parent once introduced.</x:v>
       </x:c>
       <x:c r="F45" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G45" s="32" t="str">
-        <x:v>Policy leaf anchored on the specific legacy script template it constrains.</x:v>
+        <x:v>Replaces the earlier curricular and wallet-semantic parent candidates.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="32" t="str">
-        <x:v>protocol.standardness-policy</x:v>
+        <x:v>protocol.p2ms</x:v>
       </x:c>
       <x:c r="B46" s="32" t="str">
         <x:v>protocol.bare-multisig-standardness</x:v>
@@ -12393,21 +12491,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E46" s="32" t="str">
-        <x:v>This node is a concrete application of standard transaction policy, so the general standardness concept should come first.</x:v>
+        <x:v>The relay treatment only makes sense once the learner understands what a bare multisig output actually is on-chain.</x:v>
       </x:c>
       <x:c r="F46" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G46" s="32" t="str">
-        <x:v>Policy-boundary prerequisite inherited through the existing mempool-policy branch.</x:v>
+        <x:v>Policy leaf anchored on the specific legacy script template it constrains.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>protocol.standardness-policy</x:v>
       </x:c>
       <x:c r="B47" s="32" t="str">
-        <x:v>dev.scriptpubkeymanagers</x:v>
+        <x:v>protocol.bare-multisig-standardness</x:v>
       </x:c>
       <x:c r="C47" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12416,21 +12514,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E47" s="32" t="str">
-        <x:v>Modern descriptor wallets hand descriptor-backed script templates to dedicated managers, so learners need the descriptor model before the SPKM boundary makes sense.</x:v>
+        <x:v>This node is a concrete application of standard transaction policy, so the general standardness concept should come first.</x:v>
       </x:c>
       <x:c r="F47" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-wallet</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G47" s="32" t="str">
-        <x:v>Direct edge distinguishes the Core wallet abstraction from descriptor syntax without collapsing the two concepts into one node.</x:v>
+        <x:v>Policy-boundary prerequisite inherited through the existing mempool-policy branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="32" t="str">
-        <x:v>protocol.mempool</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B48" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>dev.scriptpubkeymanagers</x:v>
       </x:c>
       <x:c r="C48" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12439,18 +12537,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E48" s="32" t="str">
-        <x:v>The unbroadcast set is a mempool-owned data structure, so learners need the local unconfirmed transaction pool model before this narrower tracking mechanism makes sense.</x:v>
+        <x:v>Modern descriptor wallets hand descriptor-backed script templates to dedicated managers, so learners need the descriptor model before the SPKM boundary makes sense.</x:v>
       </x:c>
       <x:c r="F48" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-core-academy-wallet</x:v>
       </x:c>
       <x:c r="G48" s="32" t="str">
-        <x:v>Direct edge keeps the concept scoped to local transaction state rather than broader relay policy.</x:v>
+        <x:v>Direct edge distinguishes the Core wallet abstraction from descriptor syntax without collapsing the two concepts into one node.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="32" t="str">
-        <x:v>protocol.transaction-relay-inv-getdata</x:v>
+        <x:v>protocol.mempool</x:v>
       </x:c>
       <x:c r="B49" s="32" t="str">
         <x:v>protocol.mempool-unbroadcast-set</x:v>
@@ -12462,21 +12560,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E49" s="32" t="str">
-        <x:v>This set only matters because nodes need to distinguish locally submitted transactions from those later observed through the network relay path and may retry announcing them.</x:v>
+        <x:v>The unbroadcast set is a mempool-owned data structure, so learners need the local unconfirmed transaction pool model before this narrower tracking mechanism makes sense.</x:v>
       </x:c>
       <x:c r="F49" s="32" t="str">
         <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G49" s="32" t="str">
-        <x:v>Direct edge ties the mechanism to network propagation confirmation and rebroadcast attempts.</x:v>
+        <x:v>Direct edge keeps the concept scoped to local transaction state rather than broader relay policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="32" t="str">
-        <x:v>privacy.address-reuse</x:v>
+        <x:v>protocol.transaction-relay-inv-getdata</x:v>
       </x:c>
       <x:c r="B50" s="32" t="str">
-        <x:v>custody.human-readable-addresses</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="C50" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12485,21 +12583,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E50" s="32" t="str">
-        <x:v>A major design constraint is that reusable human-readable handles can worsen privacy unless they resolve to reusable payment mechanisms or rotate safely, so learners need the address-reuse problem first.</x:v>
+        <x:v>This set only matters because nodes need to distinguish locally submitted transactions from those later observed through the network relay path and may retry announcing them.</x:v>
       </x:c>
       <x:c r="F50" s="32" t="str">
-        <x:v>source.bitcoin-design-payment-formats</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G50" s="32" t="str">
-        <x:v>Direct edge captures the main privacy tradeoff without forcing downstream protocol-specific address schemes into prerequisites.</x:v>
+        <x:v>Direct edge ties the mechanism to network propagation confirmation and rebroadcast attempts.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="32" t="str">
-        <x:v>custody.output-labeling</x:v>
+        <x:v>privacy.address-reuse</x:v>
       </x:c>
       <x:c r="B51" s="32" t="str">
-        <x:v>custody.transaction-metadata</x:v>
+        <x:v>custody.human-readable-addresses</x:v>
       </x:c>
       <x:c r="C51" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12508,18 +12606,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E51" s="32" t="str">
-        <x:v>Output labeling already introduces the idea that wallets attach their own context to payments and spendable objects, making it the cleanest direct bridge into broader transaction-level notes, contacts, and portability concerns.</x:v>
+        <x:v>A major design constraint is that reusable human-readable handles can worsen privacy unless they resolve to reusable payment mechanisms or rotate safely, so learners need the address-reuse problem first.</x:v>
       </x:c>
       <x:c r="F51" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoin-design-payment-formats</x:v>
       </x:c>
       <x:c r="G51" s="32" t="str">
-        <x:v>Direct edge distinguishes wider payment-history context from narrower spend-control labels without treating them as unrelated.</x:v>
+        <x:v>Direct edge captures the main privacy tradeoff without forcing downstream protocol-specific address schemes into prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>custody.output-labeling</x:v>
       </x:c>
       <x:c r="B52" s="32" t="str">
         <x:v>custody.transaction-metadata</x:v>
@@ -12531,21 +12629,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E52" s="32" t="str">
-        <x:v>Wallet-added names, notes, and contact links matter partly because transaction history is only pseudonymous and can reveal meaningful patterns when users or tools correlate activity over time.</x:v>
+        <x:v>Output labeling already introduces the idea that wallets attach their own context to payments and spendable objects, making it the cleanest direct bridge into broader transaction-level notes, contacts, and portability concerns.</x:v>
       </x:c>
       <x:c r="F52" s="32" t="str">
         <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="G52" s="32" t="str">
-        <x:v>Direct edge keeps the node tied to the privacy and identity meaning of payment history rather than only to generic lifecycle sequencing.</x:v>
+        <x:v>Direct edge distinguishes wider payment-history context from narrower spend-control labels without treating them as unrelated.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="32" t="str">
-        <x:v>custody.self-custody</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B53" s="32" t="str">
-        <x:v>custody.multiple-wallets</x:v>
+        <x:v>custody.transaction-metadata</x:v>
       </x:c>
       <x:c r="C53" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12554,21 +12652,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E53" s="32" t="str">
-        <x:v>Deliberately separating funds across different wallet buckets is a custody decision, so learners need the base self-custody responsibility model before the organizational pattern makes sense.</x:v>
+        <x:v>Wallet-added names, notes, and contact links matter partly because transaction history is only pseudonymous and can reveal meaningful patterns when users or tools correlate activity over time.</x:v>
       </x:c>
       <x:c r="F53" s="32" t="str">
-        <x:v>source.bitcoin-design-multiple-wallets</x:v>
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="G53" s="32" t="str">
-        <x:v>Kept the direct parent at the responsibility-model layer; multisig, watch-only, and HD account structures remain examples or implementation details rather than prerequisites.</x:v>
+        <x:v>Direct edge keeps the node tied to the privacy and identity meaning of payment history rather than only to generic lifecycle sequencing.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="32" t="str">
-        <x:v>custody.hardware-wallets</x:v>
+        <x:v>custody.self-custody</x:v>
       </x:c>
       <x:c r="B54" s="32" t="str">
-        <x:v>custody.progressive-security</x:v>
+        <x:v>custody.multiple-wallets</x:v>
       </x:c>
       <x:c r="C54" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12577,18 +12675,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E54" s="32" t="str">
-        <x:v>One of the core upgrade steps in the reference design is moving from default low-friction storage to an external signing device, so learners need the hardware-signing model before the staged-upgrade pattern makes sense.</x:v>
+        <x:v>Deliberately separating funds across different wallet buckets is a custody decision, so learners need the base self-custody responsibility model before the organizational pattern makes sense.</x:v>
       </x:c>
       <x:c r="F54" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoin-design-multiple-wallets</x:v>
       </x:c>
       <x:c r="G54" s="32" t="str">
-        <x:v>Direct edge captures the mid-tier upgrade target without treating cloud backup itself as the core concept.</x:v>
+        <x:v>Kept the direct parent at the responsibility-model layer; multisig, watch-only, and HD account structures remain examples or implementation details rather than prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>custody.hardware-wallets</x:v>
       </x:c>
       <x:c r="B55" s="32" t="str">
         <x:v>custody.progressive-security</x:v>
@@ -12600,21 +12698,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E55" s="32" t="str">
-        <x:v>The higher-security end of the progression moves into 2-of-3 and 3-of-5 multi-key schemes, so learners need the multisig model before they can reason about why and when a wallet should escalate there.</x:v>
+        <x:v>One of the core upgrade steps in the reference design is moving from default low-friction storage to an external signing device, so learners need the hardware-signing model before the staged-upgrade pattern makes sense.</x:v>
       </x:c>
       <x:c r="F55" s="32" t="str">
         <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="G55" s="32" t="str">
-        <x:v>Direct edge captures the high-assurance destination of the progression rather than a specific product flow.</x:v>
+        <x:v>Direct edge captures the mid-tier upgrade target without treating cloud backup itself as the core concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B56" s="32" t="str">
-        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
+        <x:v>custody.progressive-security</x:v>
       </x:c>
       <x:c r="C56" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12623,18 +12721,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E56" s="32" t="str">
-        <x:v>Rebroadcast privacy builds directly on the local-node distinction between transactions merely accepted into the mempool and transactions known to have propagated, which is exactly the gap the unbroadcast set tracks.</x:v>
+        <x:v>The higher-security end of the progression moves into 2-of-3 and 3-of-5 multi-key schemes, so learners need the multisig model before they can reason about why and when a wallet should escalate there.</x:v>
       </x:c>
       <x:c r="F56" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="G56" s="32" t="str">
-        <x:v>Direct parent keeps the slice on the local tracking mechanism rather than reintroducing generic relay ancestors.</x:v>
+        <x:v>Direct edge captures the high-assurance destination of the progression rather than a specific product flow.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="B57" s="32" t="str">
         <x:v>protocol.transaction-rebroadcast-privacy</x:v>
@@ -12646,21 +12744,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E57" s="32" t="str">
-        <x:v>Different rebroadcast patterns matter because observers can correlate network behavior with public transaction history and infer likely origin, so learners need the pseudonymity and linkage problem first.</x:v>
+        <x:v>Rebroadcast privacy builds directly on the local-node distinction between transactions merely accepted into the mempool and transactions known to have propagated, which is exactly the gap the unbroadcast set tracks.</x:v>
       </x:c>
       <x:c r="F57" s="32" t="str">
         <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G57" s="32" t="str">
-        <x:v>Direct parent keeps the node focused on why relay-side origin leakage matters, not just how rebroadcast code works.</x:v>
+        <x:v>Direct parent keeps the slice on the local tracking mechanism rather than reintroducing generic relay ancestors.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="32" t="str">
-        <x:v>protocol.segregated-witness</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B58" s="32" t="str">
-        <x:v>protocol.txid-vs-wtxid</x:v>
+        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
       </x:c>
       <x:c r="C58" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12669,21 +12767,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E58" s="32" t="str">
-        <x:v>The identifier split only exists because SegWit introduces a witness-inclusive serialization alongside the legacy serialization, so learners need the SegWit structure change before the two IDs make sense.</x:v>
+        <x:v>Different rebroadcast patterns matter because observers can correlate network behavior with public transaction history and infer likely origin, so learners need the pseudonymity and linkage problem first.</x:v>
       </x:c>
       <x:c r="F58" s="32" t="str">
         <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G58" s="32" t="str">
-        <x:v>Direct parent keeps the bridge on the serialization distinction instead of reintroducing downstream relay consequences.</x:v>
+        <x:v>Direct parent keeps the node focused on why relay-side origin leakage matters, not just how rebroadcast code works.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="32" t="str">
+        <x:v>protocol.segregated-witness</x:v>
+      </x:c>
+      <x:c r="B59" s="32" t="str">
         <x:v>protocol.txid-vs-wtxid</x:v>
-      </x:c>
-      <x:c r="B59" s="32" t="str">
-        <x:v>protocol.wtxid-relay-bip339</x:v>
       </x:c>
       <x:c r="C59" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12692,21 +12790,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E59" s="32" t="str">
-        <x:v>WTXID relay is specifically the choice to announce and request witness-bearing transactions by wtxid instead of txid, so the learner should understand the two identifier forms before the relay mode change.</x:v>
+        <x:v>The identifier split only exists because SegWit introduces a witness-inclusive serialization alongside the legacy serialization, so learners need the SegWit structure change before the two IDs make sense.</x:v>
       </x:c>
       <x:c r="F59" s="32" t="str">
         <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G59" s="32" t="str">
-        <x:v>Added as a graph bridge so the existing relay node no longer has to explain the identifier distinction internally.</x:v>
+        <x:v>Direct parent keeps the bridge on the serialization distinction instead of reintroducing downstream relay consequences.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="32" t="str">
-        <x:v>fundamentals.schnorr-signatures</x:v>
+        <x:v>protocol.txid-vs-wtxid</x:v>
       </x:c>
       <x:c r="B60" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>protocol.wtxid-relay-bip339</x:v>
       </x:c>
       <x:c r="C60" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12715,21 +12813,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E60" s="32" t="str">
-        <x:v>MuSig is a Schnorr aggregation protocol, so learners need the underlying Schnorr key and signature model before the combined-key protocol makes sense.</x:v>
+        <x:v>WTXID relay is specifically the choice to announce and request witness-bearing transactions by wtxid instead of txid, so the learner should understand the two identifier forms before the relay mode change.</x:v>
       </x:c>
       <x:c r="F60" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G60" s="32" t="str">
-        <x:v>Direct parent kept narrow; wallet-level multisig and Taproot remain context rather than prerequisites.</x:v>
+        <x:v>Added as a graph bridge so the existing relay node no longer has to explain the identifier distinction internally.</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="B61" s="32" t="str">
-        <x:v>dev.descriptor-wallet-policies</x:v>
+        <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="C61" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12738,18 +12836,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E61" s="32" t="str">
-        <x:v>Wallet policies are built as descriptor templates, so the base descriptor language and template structure must come first.</x:v>
+        <x:v>MuSig is a Schnorr aggregation protocol, so learners need the underlying Schnorr key and signature model before the combined-key protocol makes sense.</x:v>
       </x:c>
       <x:c r="F61" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G61" s="32" t="str">
-        <x:v>Direct parent kept above import or signer flows because the node is about the representation itself.</x:v>
+        <x:v>Direct parent kept narrow; wallet-level multisig and Taproot remain context rather than prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="32" t="str">
-        <x:v>dev.bip32</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B62" s="32" t="str">
         <x:v>dev.descriptor-wallet-policies</x:v>
@@ -12761,21 +12859,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E62" s="32" t="str">
-        <x:v>BIP388 key information items package xpubs and derivation origins, so learners need the HD derivation model before the portable wallet-policy format makes sense.</x:v>
+        <x:v>Wallet policies are built as descriptor templates, so the base descriptor language and template structure must come first.</x:v>
       </x:c>
       <x:c r="F62" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G62" s="32" t="str">
-        <x:v>Non-redundant alongside dev.descriptors because neither concept implies the other in the current graph.</x:v>
+        <x:v>Direct parent kept above import or signer flows because the node is about the representation itself.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>dev.bip32</x:v>
       </x:c>
       <x:c r="B63" s="32" t="str">
-        <x:v>dev.descriptors-in-psbt</x:v>
+        <x:v>dev.descriptor-wallet-policies</x:v>
       </x:c>
       <x:c r="C63" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12784,18 +12882,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E63" s="32" t="str">
-        <x:v>The node is about carrying descriptor information during transaction coordination, so learners need the descriptor syntax and script-template model first.</x:v>
+        <x:v>BIP388 key information items package xpubs and derivation origins, so learners need the HD derivation model before the portable wallet-policy format makes sense.</x:v>
       </x:c>
       <x:c r="F63" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G63" s="32" t="str">
-        <x:v>Direct parent kept at the representation layer rather than the wallet-policy or taproot-specific refinements.</x:v>
+        <x:v>Non-redundant alongside dev.descriptors because neither concept implies the other in the current graph.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="32" t="str">
-        <x:v>custody.psbt</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B64" s="32" t="str">
         <x:v>dev.descriptors-in-psbt</x:v>
@@ -12807,21 +12905,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E64" s="32" t="str">
-        <x:v>Descriptor-aware exchange only makes sense after the learner understands the general PSBT coordination workflow that transports signing-related data between tools.</x:v>
+        <x:v>The node is about carrying descriptor information during transaction coordination, so learners need the descriptor syntax and script-template model first.</x:v>
       </x:c>
       <x:c r="F64" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G64" s="32" t="str">
-        <x:v>Direct parent kept at the base PSBT workflow level instead of requiring later version-specific extensions.</x:v>
+        <x:v>Direct parent kept at the representation layer rather than the wallet-policy or taproot-specific refinements.</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>custody.psbt</x:v>
       </x:c>
       <x:c r="B65" s="32" t="str">
-        <x:v>custody.degrading-multisig</x:v>
+        <x:v>dev.descriptors-in-psbt</x:v>
       </x:c>
       <x:c r="C65" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12830,18 +12928,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E65" s="32" t="str">
-        <x:v>The policy only makes sense once the learner understands ordinary multisig threshold custody and why signers can be split into live and backup sets.</x:v>
+        <x:v>Descriptor-aware exchange only makes sense after the learner understands the general PSBT coordination workflow that transports signing-related data between tools.</x:v>
       </x:c>
       <x:c r="F65" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G65" s="32" t="str">
-        <x:v>Direct custody parent for the signer-threshold side of the construction.</x:v>
+        <x:v>Direct parent kept at the base PSBT workflow level instead of requiring later version-specific extensions.</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="32" t="str">
-        <x:v>protocol.timelocks</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B66" s="32" t="str">
         <x:v>custody.degrading-multisig</x:v>
@@ -12853,21 +12951,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E66" s="32" t="str">
-        <x:v>The degrading policy activates its weaker backup path only after a timeout, so timelock semantics are a direct part of the construction.</x:v>
+        <x:v>The policy only makes sense once the learner understands ordinary multisig threshold custody and why signers can be split into live and backup sets.</x:v>
       </x:c>
       <x:c r="F66" s="32" t="str">
         <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G66" s="32" t="str">
-        <x:v>Needed alongside custody.multisig because the learner must understand the temporal rule, not just the signer policy.</x:v>
+        <x:v>Direct custody parent for the signer-threshold side of the construction.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="32" t="str">
-        <x:v>protocol.block-weight-vbytes</x:v>
+        <x:v>protocol.timelocks</x:v>
       </x:c>
       <x:c r="B67" s="32" t="str">
-        <x:v>protocol.fee-calculation</x:v>
+        <x:v>custody.degrading-multisig</x:v>
       </x:c>
       <x:c r="C67" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12876,21 +12974,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E67" s="32" t="str">
-        <x:v>Understanding whether an absolute fee is high or low requires relating it to the blockspace pricing unit, so learners need weight and virtual bytes before fee calculation is fully meaningful in practice.</x:v>
+        <x:v>The degrading policy activates its weaker backup path only after a timeout, so timelock semantics are a direct part of the construction.</x:v>
       </x:c>
       <x:c r="F67" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G67" s="32" t="str">
-        <x:v>Direct parent keeps the node at the mechanism layer without drifting into broader fee-market competition.</x:v>
+        <x:v>Needed alongside custody.multisig because the learner must understand the temporal rule, not just the signer policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>protocol.block-weight-vbytes</x:v>
       </x:c>
       <x:c r="B68" s="32" t="str">
-        <x:v>protocol.bech32m-addresses</x:v>
+        <x:v>protocol.fee-calculation</x:v>
       </x:c>
       <x:c r="C68" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12899,18 +12997,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E68" s="32" t="str">
-        <x:v>Bech32m is an address-encoding format, so learners need the general relationship between addresses, script templates, and spendability before the newer checksum format is meaningful.</x:v>
+        <x:v>Understanding whether an absolute fee is high or low requires relating it to the blockspace pricing unit, so learners need weight and virtual bytes before fee calculation is fully meaningful in practice.</x:v>
       </x:c>
       <x:c r="F68" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G68" s="32" t="str">
-        <x:v>Direct parent keeps the node on encoding semantics rather than on raw string-format trivia.</x:v>
+        <x:v>Direct parent keeps the node at the mechanism layer without drifting into broader fee-market competition.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B69" s="32" t="str">
         <x:v>protocol.bech32m-addresses</x:v>
@@ -12922,21 +13020,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E69" s="32" t="str">
-        <x:v>Bech32m became necessary for witness version 1 and higher, and Taproot is the first major deployed witness-v1 use case, so learners need that upgrade context before the format distinction makes sense.</x:v>
+        <x:v>Bech32m is an address-encoding format, so learners need the general relationship between addresses, script templates, and spendability before the newer checksum format is meaningful.</x:v>
       </x:c>
       <x:c r="F69" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G69" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored on the practical protocol transition that exposed Bech32m to users.</x:v>
+        <x:v>Direct parent keeps the node on encoding semantics rather than on raw string-format trivia.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B70" s="32" t="str">
-        <x:v>protocol.script-execution-stack</x:v>
+        <x:v>protocol.bech32m-addresses</x:v>
       </x:c>
       <x:c r="C70" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12945,21 +13043,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E70" s="32" t="str">
-        <x:v>The stack execution model is the direct mechanism by which Bitcoin Script evaluates spending conditions, so learners need the umbrella Script concept before drilling into stack behavior.</x:v>
+        <x:v>Bech32m became necessary for witness version 1 and higher, and Taproot is the first major deployed witness-v1 use case, so learners need that upgrade context before the format distinction makes sense.</x:v>
       </x:c>
       <x:c r="F70" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G70" s="32" t="str">
-        <x:v>Direct parent positions the node as the conceptual middle layer between Script and opcode-specific leaves.</x:v>
+        <x:v>Direct parent keeps the node anchored on the practical protocol transition that exposed Bech32m to users.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="32" t="str">
-        <x:v>lightning.commitment-transactions</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B71" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>protocol.script-execution-stack</x:v>
       </x:c>
       <x:c r="C71" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12968,21 +13066,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E71" s="32" t="str">
-        <x:v>Per-commitment secrets are generated for each new commitment state, so learners need the commitment-transaction model before the secret-rotation mechanism makes sense.</x:v>
+        <x:v>The stack execution model is the direct mechanism by which Bitcoin Script evaluates spending conditions, so learners need the umbrella Script concept before drilling into stack behavior.</x:v>
       </x:c>
       <x:c r="F71" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G71" s="32" t="str">
-        <x:v>Direct parent keeps the node on state evolution rather than on later punishment or watchtower behavior.</x:v>
+        <x:v>Direct parent positions the node as the conceptual middle layer between Script and opcode-specific leaves.</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="32" t="str">
+        <x:v>lightning.commitment-transactions</x:v>
+      </x:c>
+      <x:c r="B72" s="32" t="str">
         <x:v>lightning.per-commitment-secrets</x:v>
-      </x:c>
-      <x:c r="B72" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="C72" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12991,18 +13089,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E72" s="32" t="str">
-        <x:v>The to_local and to_remote scripts rely on per-state key derivation, revocation keys, and delayed-payment keys, so learners need the per-commitment secret machinery first.</x:v>
+        <x:v>Per-commitment secrets are generated for each new commitment state, so learners need the commitment-transaction model before the secret-rotation mechanism makes sense.</x:v>
       </x:c>
       <x:c r="F72" s="32" t="str">
         <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G72" s="32" t="str">
-        <x:v>Direct parent keeps the node at the commitment-key layer instead of collapsing back into the broader commitment-transaction overview.</x:v>
+        <x:v>Direct parent keeps the node on state evolution rather than on later punishment or watchtower behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="32" t="str">
-        <x:v>protocol.csv-bip112</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="B73" s="32" t="str">
         <x:v>lightning.commitment-output-scripts</x:v>
@@ -13014,21 +13112,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E73" s="32" t="str">
-        <x:v>The delayed to_local branch is defined by a CSV-enforced waiting period, so learners need the relative-timelock opcode before the script template makes sense.</x:v>
+        <x:v>The to_local and to_remote scripts rely on per-state key derivation, revocation keys, and delayed-payment keys, so learners need the per-commitment secret machinery first.</x:v>
       </x:c>
       <x:c r="F73" s="32" t="str">
         <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G73" s="32" t="str">
-        <x:v>Direct parent captures the script-mechanism side of the concept without dragging in broader force-close or HTLC timing behavior.</x:v>
+        <x:v>Direct parent keeps the node at the commitment-key layer instead of collapsing back into the broader commitment-transaction overview.</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="32" t="str">
-        <x:v>protocol.difficulty-adjustment</x:v>
+        <x:v>protocol.csv-bip112</x:v>
       </x:c>
       <x:c r="B74" s="32" t="str">
-        <x:v>protocol.time-warp-attack</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="C74" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13037,18 +13135,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E74" s="32" t="str">
-        <x:v>The attack only makes sense once learners understand how Bitcoin retargets mining difficulty over long block windows.</x:v>
+        <x:v>The delayed to_local branch is defined by a CSV-enforced waiting period, so learners need the relative-timelock opcode before the script template makes sense.</x:v>
       </x:c>
       <x:c r="F74" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G74" s="32" t="str">
-        <x:v>Direct parent keeps the exploit tied to the retarget mechanism instead of burying it under generic mining vocabulary.</x:v>
+        <x:v>Direct parent captures the script-mechanism side of the concept without dragging in broader force-close or HTLC timing behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="32" t="str">
-        <x:v>protocol.median-time-past</x:v>
+        <x:v>protocol.difficulty-adjustment</x:v>
       </x:c>
       <x:c r="B75" s="32" t="str">
         <x:v>protocol.time-warp-attack</x:v>
@@ -13060,21 +13158,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E75" s="32" t="str">
-        <x:v>Learners need the consensus timestamp constraints before they can reason about how miners manipulate time data and where the remaining attack surface lives.</x:v>
+        <x:v>The attack only makes sense once learners understand how Bitcoin retargets mining difficulty over long block windows.</x:v>
       </x:c>
       <x:c r="F75" s="32" t="str">
         <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G75" s="32" t="str">
-        <x:v>Direct parent captures the timestamp-boundary side of the exploit without overloading timelocks or block headers.</x:v>
+        <x:v>Direct parent keeps the exploit tied to the retarget mechanism instead of burying it under generic mining vocabulary.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="32" t="str">
-        <x:v>fundamentals.blind-signatures</x:v>
+        <x:v>protocol.median-time-past</x:v>
       </x:c>
       <x:c r="B76" s="32" t="str">
-        <x:v>history.chaumian-ecash</x:v>
+        <x:v>protocol.time-warp-attack</x:v>
       </x:c>
       <x:c r="C76" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13083,18 +13181,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E76" s="32" t="str">
-        <x:v>Chaumian ecash is defined by using blind signatures to let a mint issue private bearer tokens without seeing the final token contents.</x:v>
+        <x:v>Learners need the consensus timestamp constraints before they can reason about how miners manipulate time data and where the remaining attack surface lives.</x:v>
       </x:c>
       <x:c r="F76" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G76" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the specific cryptographic mechanism rather than treating it as generic digital-money history.</x:v>
+        <x:v>Direct parent captures the timestamp-boundary side of the exploit without overloading timelocks or block headers.</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="32" t="str">
-        <x:v>history.double-spend-problem</x:v>
+        <x:v>fundamentals.blind-signatures</x:v>
       </x:c>
       <x:c r="B77" s="32" t="str">
         <x:v>history.chaumian-ecash</x:v>
@@ -13106,21 +13204,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E77" s="32" t="str">
-        <x:v>Learners need the unsolved scarcity problem in digital cash before the trusted-mint tradeoff in Chaumian designs becomes meaningful.</x:v>
+        <x:v>Chaumian ecash is defined by using blind signatures to let a mint issue private bearer tokens without seeing the final token contents.</x:v>
       </x:c>
       <x:c r="F77" s="32" t="str">
         <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G77" s="32" t="str">
-        <x:v>Direct parent frames why the system still needed a central operator even though it improved privacy.</x:v>
+        <x:v>Direct parent keeps the node tied to the specific cryptographic mechanism rather than treating it as generic digital-money history.</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="32" t="str">
-        <x:v>economics.history-of-money</x:v>
+        <x:v>history.double-spend-problem</x:v>
       </x:c>
       <x:c r="B78" s="32" t="str">
-        <x:v>privacy.secret-right-to-cash</x:v>
+        <x:v>history.chaumian-ecash</x:v>
       </x:c>
       <x:c r="C78" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13129,18 +13227,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E78" s="32" t="str">
-        <x:v>The concept depends on understanding how money moved from bearer cash toward mediated account systems, so learners need the long-run monetary history first.</x:v>
+        <x:v>Learners need the unsolved scarcity problem in digital cash before the trusted-mint tradeoff in Chaumian designs becomes meaningful.</x:v>
       </x:c>
       <x:c r="F78" s="32" t="str">
         <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G78" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the bearer-versus-intermediated payment shift rather than drifting into generic civil-liberties framing.</x:v>
+        <x:v>Direct parent frames why the system still needed a central operator even though it improved privacy.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="32" t="str">
-        <x:v>fundamentals.censorship-resistance</x:v>
+        <x:v>economics.history-of-money</x:v>
       </x:c>
       <x:c r="B79" s="32" t="str">
         <x:v>privacy.secret-right-to-cash</x:v>
@@ -13152,21 +13250,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E79" s="32" t="str">
-        <x:v>Learners need the general idea that payment systems can exclude or block participants before the loss of private cash as a payment right becomes fully meaningful.</x:v>
+        <x:v>The concept depends on understanding how money moved from bearer cash toward mediated account systems, so learners need the long-run monetary history first.</x:v>
       </x:c>
       <x:c r="F79" s="32" t="str">
         <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G79" s="32" t="str">
-        <x:v>Direct parent captures the exclusion-risk side of the argument without reopening broader compliance or surveillance wrappers.</x:v>
+        <x:v>Direct parent keeps the node tied to the bearer-versus-intermediated payment shift rather than drifting into generic civil-liberties framing.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="32" t="str">
-        <x:v>fundamentals.inflation</x:v>
+        <x:v>fundamentals.censorship-resistance</x:v>
       </x:c>
       <x:c r="B80" s="32" t="str">
-        <x:v>economics.ideal-money</x:v>
+        <x:v>privacy.secret-right-to-cash</x:v>
       </x:c>
       <x:c r="C80" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13175,21 +13273,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E80" s="32" t="str">
-        <x:v>The concept is about minimizing monetary distortion, so learners need to understand how inflation changes purchasing power and price signals first.</x:v>
+        <x:v>Learners need the general idea that payment systems can exclude or block participants before the loss of private cash as a payment right becomes fully meaningful.</x:v>
       </x:c>
       <x:c r="F80" s="32" t="str">
         <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G80" s="32" t="str">
-        <x:v>Direct parent captures the measurement-distortion problem that ideal money is trying to avoid.</x:v>
+        <x:v>Direct parent captures the exclusion-risk side of the argument without reopening broader compliance or surveillance wrappers.</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>fundamentals.inflation</x:v>
       </x:c>
       <x:c r="B81" s="32" t="str">
-        <x:v>protocol.bitcoin-uri-bip21</x:v>
+        <x:v>economics.ideal-money</x:v>
       </x:c>
       <x:c r="C81" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13198,21 +13296,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E81" s="32" t="str">
-        <x:v>The URI is a wrapper around a payment destination and amount, so learners need the underlying address and output model first.</x:v>
+        <x:v>The concept is about minimizing monetary distortion, so learners need to understand how inflation changes purchasing power and price signals first.</x:v>
       </x:c>
       <x:c r="F81" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G81" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the standard request format rather than collapsing it into higher-level wallet UX systems.</x:v>
+        <x:v>Direct parent captures the measurement-distortion problem that ideal money is trying to avoid.</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="32" t="str">
-        <x:v>dev.bip32</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B82" s="32" t="str">
-        <x:v>dev.extended-keys</x:v>
+        <x:v>protocol.bitcoin-uri-bip21</x:v>
       </x:c>
       <x:c r="C82" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13221,21 +13319,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E82" s="32" t="str">
-        <x:v>Extended keys are one specific export and branch-derivation surface inside the broader BIP32 HD tree model, so learners need the base tree-derivation mechanics first.</x:v>
+        <x:v>The URI is a wrapper around a payment destination and amount, so learners need the underlying address and output model first.</x:v>
       </x:c>
       <x:c r="F82" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G82" s="32" t="str">
-        <x:v>Direct parent keeps the node inside the HD derivation branch instead of treating xpub or xprv behavior as only a privacy or operational-wallet concept.</x:v>
+        <x:v>Direct parent keeps the node tied to the standard request format rather than collapsing it into higher-level wallet UX systems.</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="32" t="str">
+        <x:v>dev.bip32</x:v>
+      </x:c>
+      <x:c r="B83" s="32" t="str">
         <x:v>dev.extended-keys</x:v>
-      </x:c>
-      <x:c r="B83" s="32" t="str">
-        <x:v>dev.hardened-keys</x:v>
       </x:c>
       <x:c r="C83" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13244,21 +13342,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E83" s="32" t="str">
-        <x:v>Hardened derivation is a constraint on what an extended public key can derive and on how extended private and public key boundaries behave, so learners need the base xpub/xprv model first.</x:v>
+        <x:v>Extended keys are one specific export and branch-derivation surface inside the broader BIP32 HD tree model, so learners need the base tree-derivation mechanics first.</x:v>
       </x:c>
       <x:c r="F83" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G83" s="32" t="str">
-        <x:v>Direct parent closes the previously missing branch-level bridge between BIP32 generally and hardened derivation specifically.</x:v>
+        <x:v>Direct parent keeps the node inside the HD derivation branch instead of treating xpub or xprv behavior as only a privacy or operational-wallet concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>dev.extended-keys</x:v>
       </x:c>
       <x:c r="B84" s="32" t="str">
-        <x:v>protocol.escrow-and-arbitration</x:v>
+        <x:v>dev.hardened-keys</x:v>
       </x:c>
       <x:c r="C84" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13267,18 +13365,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E84" s="32" t="str">
-        <x:v>The escrow flow depends on understanding how multiple signers can authorize one spend and why a 2-of-3 threshold changes trust assumptions between buyer, seller, and arbitrator.</x:v>
+        <x:v>Hardened derivation is a constraint on what an extended public key can derive and on how extended private and public key boundaries behave, so learners need the base xpub/xprv model first.</x:v>
       </x:c>
       <x:c r="F84" s="32" t="str">
         <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G84" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the threshold-signing contract pattern instead of treating it as generic dispute-resolution theory.</x:v>
+        <x:v>Direct parent closes the previously missing branch-level bridge between BIP32 generally and hardened derivation specifically.</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="32" t="str">
-        <x:v>protocol.pay-to-script-hash</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B85" s="32" t="str">
         <x:v>protocol.escrow-and-arbitration</x:v>
@@ -13290,21 +13388,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E85" s="32" t="str">
-        <x:v>The contract uses a P2SH redeem script to hide the multisig spending conditions until spend time, so learners need the P2SH wrapper first.</x:v>
+        <x:v>The escrow flow depends on understanding how multiple signers can authorize one spend and why a 2-of-3 threshold changes trust assumptions between buyer, seller, and arbitrator.</x:v>
       </x:c>
       <x:c r="F85" s="32" t="str">
         <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G85" s="32" t="str">
-        <x:v>Direct parent captures the on-chain contract packaging layer that makes the escrow pattern practical.</x:v>
+        <x:v>Direct parent keeps the node tied to the threshold-signing contract pattern instead of treating it as generic dispute-resolution theory.</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="B86" s="32" t="str">
-        <x:v>dev.wallet-import-format-wif</x:v>
+        <x:v>protocol.escrow-and-arbitration</x:v>
       </x:c>
       <x:c r="C86" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13313,21 +13411,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E86" s="32" t="str">
-        <x:v>WIF is a serialization format for one private key, so learners need the underlying asymmetric-key concept before the network prefix, checksum, and compression flag details make sense.</x:v>
+        <x:v>The contract uses a P2SH redeem script to hide the multisig spending conditions until spend time, so learners need the P2SH wrapper first.</x:v>
       </x:c>
       <x:c r="F86" s="32" t="str">
         <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G86" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored on key material itself instead of overfitting it to address formats or HD wallet hierarchies.</x:v>
+        <x:v>Direct parent captures the on-chain contract packaging layer that makes the escrow pattern practical.</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B87" s="32" t="str">
-        <x:v>mining.pool-shares</x:v>
+        <x:v>dev.wallet-import-format-wif</x:v>
       </x:c>
       <x:c r="C87" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13336,21 +13434,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E87" s="32" t="str">
-        <x:v>Pool shares only make sense after learners understand why pooled mining exists and why miners need a lower-variance way to prove contributed work before an actual block is found.</x:v>
+        <x:v>WIF is a serialization format for one private key, so learners need the underlying asymmetric-key concept before the network prefix, checksum, and compression flag details make sense.</x:v>
       </x:c>
       <x:c r="F87" s="32" t="str">
         <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G87" s="32" t="str">
-        <x:v>Direct parent keeps the node at the pooled-mining accounting layer without adding redundant proof-of-work or difficulty edges.</x:v>
+        <x:v>Direct parent keeps the node anchored on key material itself instead of overfitting it to address formats or HD wallet hierarchies.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B88" s="32" t="str">
-        <x:v>lightning.obscured-commitment-number</x:v>
+        <x:v>mining.pool-shares</x:v>
       </x:c>
       <x:c r="C88" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13359,21 +13457,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E88" s="32" t="str">
-        <x:v>The obscured commitment number is part of the same commitment-state machinery as the per-state secret chain, so learners need that state-derivation context before the field-level encoding scheme makes sense.</x:v>
+        <x:v>Pool shares only make sense after learners understand why pooled mining exists and why miners need a lower-variance way to prove contributed work before an actual block is found.</x:v>
       </x:c>
       <x:c r="F88" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G88" s="32" t="str">
-        <x:v>Direct parent keeps the node in the narrow commitment-state branch instead of pulling in broader closure or HTLC behavior.</x:v>
+        <x:v>Direct parent keeps the node at the pooled-mining accounting layer without adding redundant proof-of-work or difficulty edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="32" t="str">
-        <x:v>lightning.htlc</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="B89" s="32" t="str">
-        <x:v>lightning.htlc-output-scripts</x:v>
+        <x:v>lightning.obscured-commitment-number</x:v>
       </x:c>
       <x:c r="C89" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13382,18 +13480,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E89" s="32" t="str">
-        <x:v>Learners need the base HTLC idea before the offered and received witness-script branches, timeout paths, and preimage-claim paths become meaningful.</x:v>
+        <x:v>The obscured commitment number is part of the same commitment-state machinery as the per-state secret chain, so learners need that state-derivation context before the field-level encoding scheme makes sense.</x:v>
       </x:c>
       <x:c r="F89" s="32" t="str">
         <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G89" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the payment-contract primitive instead of treating it as generic script trivia.</x:v>
+        <x:v>Direct parent keeps the node in the narrow commitment-state branch instead of pulling in broader closure or HTLC behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>lightning.htlc</x:v>
       </x:c>
       <x:c r="B90" s="32" t="str">
         <x:v>lightning.htlc-output-scripts</x:v>
@@ -13405,21 +13503,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E90" s="32" t="str">
-        <x:v>HTLC output scripts are additional commitment-transaction outputs layered on top of the same to_local and to_remote commitment-script structure, so learners need that earlier script layer first.</x:v>
+        <x:v>Learners need the base HTLC idea before the offered and received witness-script branches, timeout paths, and preimage-claim paths become meaningful.</x:v>
       </x:c>
       <x:c r="F90" s="32" t="str">
         <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G90" s="32" t="str">
-        <x:v>Direct parent places the node at the next script layer above commitment outputs without dragging in later close-handling or watchtower flows.</x:v>
+        <x:v>Direct parent keeps the node tied to the payment-contract primitive instead of treating it as generic script trivia.</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="32" t="str">
-        <x:v>protocol.coinbase-transaction</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="B91" s="32" t="str">
-        <x:v>protocol.duplicate-transaction-bug</x:v>
+        <x:v>lightning.htlc-output-scripts</x:v>
       </x:c>
       <x:c r="C91" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13428,18 +13526,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E91" s="32" t="str">
-        <x:v>The bug is historically tied to duplicated coinbase transactions, so learners need the special structure and validation role of coinbase transactions before the replay vector makes sense.</x:v>
+        <x:v>HTLC output scripts are additional commitment-transaction outputs layered on top of the same to_local and to_remote commitment-script structure, so learners need that earlier script layer first.</x:v>
       </x:c>
       <x:c r="F91" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G91" s="32" t="str">
-        <x:v>Direct parent keeps the bug tied to the early-coinbase uniqueness failure instead of burying it under general mining history.</x:v>
+        <x:v>Direct parent places the node at the next script layer above commitment outputs without dragging in later close-handling or watchtower flows.</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="32" t="str">
-        <x:v>protocol.utxo-model</x:v>
+        <x:v>protocol.coinbase-transaction</x:v>
       </x:c>
       <x:c r="B92" s="32" t="str">
         <x:v>protocol.duplicate-transaction-bug</x:v>
@@ -13451,21 +13549,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E92" s="32" t="str">
-        <x:v>Learners need the txid-plus-output-index reference model to understand why identical transaction ids could confuse later spends and overwrite assumptions in the UTXO set.</x:v>
+        <x:v>The bug is historically tied to duplicated coinbase transactions, so learners need the special structure and validation role of coinbase transactions before the replay vector makes sense.</x:v>
       </x:c>
       <x:c r="F92" s="32" t="str">
         <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G92" s="32" t="str">
-        <x:v>Direct parent captures the reference-model side of the bug without conflating it with double-spend history or malleability.</x:v>
+        <x:v>Direct parent keeps the bug tied to the early-coinbase uniqueness failure instead of burying it under general mining history.</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="32" t="str">
-        <x:v>protocol.block-structure</x:v>
+        <x:v>protocol.utxo-model</x:v>
       </x:c>
       <x:c r="B93" s="32" t="str">
-        <x:v>protocol.64-byte-transaction-bug</x:v>
+        <x:v>protocol.duplicate-transaction-bug</x:v>
       </x:c>
       <x:c r="C93" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13474,21 +13572,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E93" s="32" t="str">
-        <x:v>The bug only makes sense once learners understand how transaction hashes sit inside the block merkle tree and why internal-node preimages matter for block commitments.</x:v>
+        <x:v>Learners need the txid-plus-output-index reference model to understand why identical transaction ids could confuse later spends and overwrite assumptions in the UTXO set.</x:v>
       </x:c>
       <x:c r="F93" s="32" t="str">
         <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G93" s="32" t="str">
-        <x:v>One direct parent keeps the node at the block-commitment layer instead of reopening broader hashing or SPV overview branches.</x:v>
+        <x:v>Direct parent captures the reference-model side of the bug without conflating it with double-spend history or malleability.</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="32" t="str">
-        <x:v>fundamentals.digital-signatures</x:v>
+        <x:v>protocol.block-structure</x:v>
       </x:c>
       <x:c r="B94" s="32" t="str">
-        <x:v>fundamentals.lamport-signatures</x:v>
+        <x:v>protocol.64-byte-transaction-bug</x:v>
       </x:c>
       <x:c r="C94" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13497,18 +13595,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E94" s="32" t="str">
-        <x:v>Learners need the general signing-and-verification mental model before the one-time Lamport construction and its tradeoffs become meaningful.</x:v>
+        <x:v>The bug only makes sense once learners understand how transaction hashes sit inside the block merkle tree and why internal-node preimages matter for block commitments.</x:v>
       </x:c>
       <x:c r="F94" s="32" t="str">
         <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G94" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to signature semantics instead of treating it as only a post-quantum curiosity.</x:v>
+        <x:v>One direct parent keeps the node at the block-commitment layer instead of reopening broader hashing or SPV overview branches.</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>fundamentals.digital-signatures</x:v>
       </x:c>
       <x:c r="B95" s="32" t="str">
         <x:v>fundamentals.lamport-signatures</x:v>
@@ -13520,21 +13618,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E95" s="32" t="str">
-        <x:v>Lamport signatures replace elliptic-curve arithmetic with one-way hash preimages and comparisons, so learners need the hash primitive first.</x:v>
+        <x:v>Learners need the general signing-and-verification mental model before the one-time Lamport construction and its tradeoffs become meaningful.</x:v>
       </x:c>
       <x:c r="F95" s="32" t="str">
         <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G95" s="32" t="str">
-        <x:v>Direct parent captures the actual cryptographic mechanism rather than forcing learners through unrelated elliptic-curve details.</x:v>
+        <x:v>Direct parent keeps the node tied to signature semantics instead of treating it as only a post-quantum curiosity.</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="32" t="str">
-        <x:v>custody.backups-recovery</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B96" s="32" t="str">
-        <x:v>custody.shamirs-secret-sharing</x:v>
+        <x:v>fundamentals.lamport-signatures</x:v>
       </x:c>
       <x:c r="C96" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13543,21 +13641,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E96" s="32" t="str">
-        <x:v>In Bitcoin practice the scheme is used as one backup-and-recovery method, so learners need the broader custody problem before the threshold-share design choice becomes meaningful.</x:v>
+        <x:v>Lamport signatures replace elliptic-curve arithmetic with one-way hash preimages and comparisons, so learners need the hash primitive first.</x:v>
       </x:c>
       <x:c r="F96" s="32" t="str">
         <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G96" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored in practical custody use instead of drifting into a purely abstract cryptography topic.</x:v>
+        <x:v>Direct parent captures the actual cryptographic mechanism rather than forcing learners through unrelated elliptic-curve details.</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="32" t="str">
-        <x:v>protocol.segregated-witness</x:v>
+        <x:v>custody.backups-recovery</x:v>
       </x:c>
       <x:c r="B97" s="32" t="str">
-        <x:v>protocol.witness-structure</x:v>
+        <x:v>custody.shamirs-secret-sharing</x:v>
       </x:c>
       <x:c r="C97" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13566,21 +13664,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E97" s="32" t="str">
-        <x:v>The transaction witness layout only makes sense after the learner understands that SegWit separates witness data from the legacy transaction serialization.</x:v>
+        <x:v>In Bitcoin practice the scheme is used as one backup-and-recovery method, so learners need the broader custody problem before the threshold-share design choice becomes meaningful.</x:v>
       </x:c>
       <x:c r="F97" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G97" s="32" t="str">
-        <x:v>Direct edge keeps the node at the transaction-format layer; TXID/WTXID and witness-commitment consequences remain downstream concepts.</x:v>
+        <x:v>Direct parent keeps the node anchored in practical custody use instead of drifting into a purely abstract cryptography topic.</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="32" t="str">
-        <x:v>protocol.block-structure</x:v>
+        <x:v>protocol.segregated-witness</x:v>
       </x:c>
       <x:c r="B98" s="32" t="str">
-        <x:v>protocol.partial-merkle-proofs</x:v>
+        <x:v>protocol.witness-structure</x:v>
       </x:c>
       <x:c r="C98" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13589,21 +13687,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E98" s="32" t="str">
-        <x:v>Partial Merkle proofs reconstruct a transaction's inclusion path against the Merkle root carried by a block, so learners need block composition and root placement first.</x:v>
+        <x:v>The transaction witness layout only makes sense after the learner understands that SegWit separates witness data from the legacy transaction serialization.</x:v>
       </x:c>
       <x:c r="F98" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G98" s="32" t="str">
-        <x:v>The block-structure parent already inherits fundamentals.merkle-trees, avoiding a redundant direct edge.</x:v>
+        <x:v>Direct edge keeps the node at the transaction-format layer; TXID/WTXID and witness-commitment consequences remain downstream concepts.</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="32" t="str">
-        <x:v>dev.bips-process</x:v>
+        <x:v>protocol.block-structure</x:v>
       </x:c>
       <x:c r="B99" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>protocol.partial-merkle-proofs</x:v>
       </x:c>
       <x:c r="C99" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13612,18 +13710,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E99" s="32" t="str">
-        <x:v>Review culture is applied throughout the proposal and implementation lifecycle, so learners need to understand the process in which Bitcoin changes are proposed and evaluated.</x:v>
+        <x:v>Partial Merkle proofs reconstruct a transaction's inclusion path against the Merkle root carried by a block, so learners need block composition and root placement first.</x:v>
       </x:c>
       <x:c r="F99" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G99" s="32" t="str">
-        <x:v>Direct edge supplies the development-lifecycle context without adding downstream release or deployment details.</x:v>
+        <x:v>The block-structure parent already inherits fundamentals.merkle-trees, avoiding a redundant direct edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="32" t="str">
-        <x:v>security.adversarial-thinking</x:v>
+        <x:v>dev.bips-process</x:v>
       </x:c>
       <x:c r="B100" s="32" t="str">
         <x:v>dev.review-culture</x:v>
@@ -13635,21 +13733,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E100" s="32" t="str">
-        <x:v>Independent review in Bitcoin is deliberately adversarial: reviewers look for correctness failures, attack paths, and compatibility hazards before changes are merged.</x:v>
+        <x:v>Review culture is applied throughout the proposal and implementation lifecycle, so learners need to understand the process in which Bitcoin changes are proposed and evaluated.</x:v>
       </x:c>
       <x:c r="F100" s="32" t="str">
         <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G100" s="32" t="str">
-        <x:v>Direct edge keeps review distinct from responsible disclosure and reproducible-build verification, which are specialized downstream safeguards.</x:v>
+        <x:v>Direct edge supplies the development-lifecycle context without adding downstream release or deployment details.</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="32" t="str">
-        <x:v>lightning.gossip-protocol</x:v>
+        <x:v>security.adversarial-thinking</x:v>
       </x:c>
       <x:c r="B101" s="32" t="str">
-        <x:v>lightning.feature-flags</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="C101" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13658,21 +13756,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E101" s="32" t="str">
-        <x:v>Feature negotiation is used to advertise and interpret capabilities across Lightning peers and network announcements, so learners need the surrounding gossip and announcement context first.</x:v>
+        <x:v>Independent review in Bitcoin is deliberately adversarial: reviewers look for correctness failures, attack paths, and compatibility hazards before changes are merged.</x:v>
       </x:c>
       <x:c r="F101" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G101" s="32" t="str">
-        <x:v>Direct edge keeps the feature-bit mechanism distinct from the lower-level message transport and downstream routing protocols.</x:v>
+        <x:v>Direct edge keeps review distinct from responsible disclosure and reproducible-build verification, which are specialized downstream safeguards.</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="32" t="str">
+        <x:v>lightning.gossip-protocol</x:v>
+      </x:c>
+      <x:c r="B102" s="32" t="str">
         <x:v>lightning.feature-flags</x:v>
-      </x:c>
-      <x:c r="B102" s="32" t="str">
-        <x:v>lightning.onion-messages</x:v>
       </x:c>
       <x:c r="C102" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13681,18 +13779,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E102" s="32" t="str">
-        <x:v>Peers use a negotiated feature bit to advertise whether they can send and forward onion messages, so learners need the capability-negotiation model first.</x:v>
+        <x:v>Feature negotiation is used to advertise and interpret capabilities across Lightning peers and network announcements, so learners need the surrounding gossip and announcement context first.</x:v>
       </x:c>
       <x:c r="F102" s="32" t="str">
         <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G102" s="32" t="str">
-        <x:v>Direct edge keeps the feature gate separate from the message forwarding mechanism.</x:v>
+        <x:v>Direct edge keeps the feature-bit mechanism distinct from the lower-level message transport and downstream routing protocols.</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="32" t="str">
-        <x:v>lightning.route-blinding</x:v>
+        <x:v>lightning.feature-flags</x:v>
       </x:c>
       <x:c r="B103" s="32" t="str">
         <x:v>lightning.onion-messages</x:v>
@@ -13704,21 +13802,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E103" s="32" t="str">
-        <x:v>Onion messages use blinded paths to forward channel-independent payloads without exposing the final destination topology, so the route-blinding model must come first.</x:v>
+        <x:v>Peers use a negotiated feature bit to advertise whether they can send and forward onion messages, so learners need the capability-negotiation model first.</x:v>
       </x:c>
       <x:c r="F103" s="32" t="str">
         <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G103" s="32" t="str">
-        <x:v>Payment onion routing and BOLT12 offers remain related sibling or downstream concepts rather than direct prerequisites.</x:v>
+        <x:v>Direct edge keeps the feature gate separate from the message forwarding mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>lightning.route-blinding</x:v>
       </x:c>
       <x:c r="B104" s="32" t="str">
-        <x:v>lightning.encrypted-authenticated-transport</x:v>
+        <x:v>lightning.onion-messages</x:v>
       </x:c>
       <x:c r="C104" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13727,18 +13825,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E104" s="32" t="str">
-        <x:v>The Noise_XK handshake authenticates long-term Lightning node identities with public/private key material, so learners need that identity model first.</x:v>
+        <x:v>Onion messages use blinded paths to forward channel-independent payloads without exposing the final destination topology, so the route-blinding model must come first.</x:v>
       </x:c>
       <x:c r="F104" s="32" t="str">
         <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G104" s="32" t="str">
-        <x:v>Direct edge keeps identity foundations separate from the session-key derivation mechanism.</x:v>
+        <x:v>Payment onion routing and BOLT12 offers remain related sibling or downstream concepts rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="32" t="str">
-        <x:v>fundamentals.diffie-hellman-key-exchange</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B105" s="32" t="str">
         <x:v>lightning.encrypted-authenticated-transport</x:v>
@@ -13750,21 +13848,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E105" s="32" t="str">
-        <x:v>BOLT 08 uses elliptic-curve Diffie-Hellman operations to derive shared session secrets, so the key-exchange primitive must be understood first.</x:v>
+        <x:v>The Noise_XK handshake authenticates long-term Lightning node identities with public/private key material, so learners need that identity model first.</x:v>
       </x:c>
       <x:c r="F105" s="32" t="str">
         <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G105" s="32" t="str">
-        <x:v>Bitcoin P2P v2 transport remains a related sibling rather than a direct prerequisite because it is a different protocol context.</x:v>
+        <x:v>Direct edge keeps identity foundations separate from the session-key derivation mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>fundamentals.diffie-hellman-key-exchange</x:v>
       </x:c>
       <x:c r="B106" s="32" t="str">
-        <x:v>protocol.strict-der-signatures</x:v>
+        <x:v>lightning.encrypted-authenticated-transport</x:v>
       </x:c>
       <x:c r="C106" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13773,21 +13871,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E106" s="32" t="str">
-        <x:v>Strict DER enforcement occurs while Script validates an ECDSA signature, so learners need the spending-condition and interpreter context first.</x:v>
+        <x:v>BOLT 08 uses elliptic-curve Diffie-Hellman operations to derive shared session secrets, so the key-exchange primitive must be understood first.</x:v>
       </x:c>
       <x:c r="F106" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G106" s="32" t="str">
-        <x:v>Direct edge keeps the rule at the script-validation layer rather than treating BIP 66 as a broad historical upgrade topic.</x:v>
+        <x:v>Bitcoin P2P v2 transport remains a related sibling rather than a direct prerequisite because it is a different protocol context.</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B107" s="32" t="str">
-        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+        <x:v>protocol.strict-der-signatures</x:v>
       </x:c>
       <x:c r="C107" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13796,18 +13894,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E107" s="32" t="str">
-        <x:v>The node builds on the wallet-level threshold signer policy before specifying a deterministic ordering convention for the signer keys.</x:v>
+        <x:v>Strict DER enforcement occurs while Script validates an ECDSA signature, so learners need the spending-condition and interpreter context first.</x:v>
       </x:c>
       <x:c r="F107" s="32" t="str">
         <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G107" s="32" t="str">
-        <x:v>Direct edge preserves the distinction between multisig policy and the BIP 67 interoperability rule.</x:v>
+        <x:v>Direct edge keeps the rule at the script-validation layer rather than treating BIP 66 as a broad historical upgrade topic.</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="32" t="str">
-        <x:v>protocol.pay-to-script-hash</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B108" s="32" t="str">
         <x:v>custody.deterministic-multisig-key-sorting</x:v>
@@ -13819,21 +13917,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E108" s="32" t="str">
-        <x:v>BIP 67 is commonly applied when constructing the redeem script whose hash is committed by P2SH, so the script-hash wrapper provides the output context.</x:v>
+        <x:v>The node builds on the wallet-level threshold signer policy before specifying a deterministic ordering convention for the signer keys.</x:v>
       </x:c>
       <x:c r="F108" s="32" t="str">
         <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G108" s="32" t="str">
-        <x:v>The shared protocol.script ancestor remains inherited rather than a redundant direct edge.</x:v>
+        <x:v>Direct edge preserves the distinction between multisig policy and the BIP 67 interoperability rule.</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="32" t="str">
-        <x:v>ops.mempool-policy</x:v>
+        <x:v>protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="B109" s="32" t="str">
-        <x:v>ops.mempool-purging</x:v>
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
       </x:c>
       <x:c r="C109" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13842,21 +13940,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E109" s="32" t="str">
-        <x:v>Rolling minimum fee escalation and transaction eviction are local consequences of the node's mempool relay policy, so learners need that policy boundary first.</x:v>
+        <x:v>BIP 67 is commonly applied when constructing the redeem script whose hash is committed by P2SH, so the script-hash wrapper provides the output context.</x:v>
       </x:c>
       <x:c r="F109" s="32" t="str">
-        <x:v>source.mempool-space-docs</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G109" s="32" t="str">
-        <x:v>The generic mempool, fee-market, and consensus-policy branches remain inherited or adjacent rather than direct prerequisites.</x:v>
+        <x:v>The shared protocol.script ancestor remains inherited rather than a redundant direct edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>ops.mempool-policy</x:v>
       </x:c>
       <x:c r="B110" s="32" t="str">
-        <x:v>protocol.generic-signed-messages</x:v>
+        <x:v>ops.mempool-purging</x:v>
       </x:c>
       <x:c r="C110" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13865,21 +13963,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E110" s="32" t="str">
-        <x:v>BIP 322 proves message authorization by constructing virtual transactions that satisfy a Bitcoin output script, so learners need the Script spending-condition model first.</x:v>
+        <x:v>Rolling minimum fee escalation and transaction eviction are local consequences of the node's mempool relay policy, so learners need that policy boundary first.</x:v>
       </x:c>
       <x:c r="F110" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.mempool-space-docs</x:v>
       </x:c>
       <x:c r="G110" s="32" t="str">
-        <x:v>The digital-signature path is inherited through Script; PSBT, Schnorr, and Taproot remain related variants rather than redundant direct edges.</x:v>
+        <x:v>The generic mempool, fee-market, and consensus-policy branches remain inherited or adjacent rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="32" t="str">
-        <x:v>dev.bitcoin-core-rpc</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B111" s="32" t="str">
-        <x:v>security.bitcoin-core-rpc-access</x:v>
+        <x:v>protocol.generic-signed-messages</x:v>
       </x:c>
       <x:c r="C111" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13888,21 +13986,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E111" s="32" t="str">
-        <x:v>RPC access security is the control boundary around Bitcoin Core's programmatic interface, so learners need to understand the interface and its authority before securing exposure to it.</x:v>
+        <x:v>BIP 322 proves message authorization by constructing virtual transactions that satisfy a Bitcoin output script, so learners need the Script spending-condition model first.</x:v>
       </x:c>
       <x:c r="F111" s="32" t="str">
-        <x:v>source.bitcoin-core-operator-docs</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G111" s="32" t="str">
-        <x:v>Full-node operation is inherited through dev.bitcoin-core-rpc; wallet RPC and transaction-preflight nodes remain downstream use cases rather than direct parents.</x:v>
+        <x:v>The digital-signature path is inherited through Script; PSBT, Schnorr, and Taproot remain related variants rather than redundant direct edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="32" t="str">
-        <x:v>dev.testmempoolaccept-rpc</x:v>
+        <x:v>dev.bitcoin-core-rpc</x:v>
       </x:c>
       <x:c r="B112" s="32" t="str">
-        <x:v>dev.submitpackage-rpc</x:v>
+        <x:v>security.bitcoin-core-rpc-access</x:v>
       </x:c>
       <x:c r="C112" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13911,21 +14009,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E112" s="32" t="str">
-        <x:v>submitpackage is the admission counterpart to the existing testmempoolaccept preflight workflow, so learners need to understand local package checks before attempting submission and interpreting package results.</x:v>
+        <x:v>RPC access security is the control boundary around Bitcoin Core's programmatic interface, so learners need to understand the interface and its authority before securing exposure to it.</x:v>
       </x:c>
       <x:c r="F112" s="32" t="str">
-        <x:v>source.bitcoin-core-package-policy</x:v>
+        <x:v>source.bitcoin-core-operator-docs</x:v>
       </x:c>
       <x:c r="G112" s="32" t="str">
-        <x:v>Package relay and cluster mempool remain neighboring concepts rather than direct prerequisites because this node focuses on one local RPC operation.</x:v>
+        <x:v>Full-node operation is inherited through dev.bitcoin-core-rpc; wallet RPC and transaction-preflight nodes remain downstream use cases rather than direct parents.</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="32" t="str">
-        <x:v>protocol.rbf</x:v>
+        <x:v>dev.testmempoolaccept-rpc</x:v>
       </x:c>
       <x:c r="B113" s="32" t="str">
-        <x:v>protocol.package-rbf</x:v>
+        <x:v>dev.submitpackage-rpc</x:v>
       </x:c>
       <x:c r="C113" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13934,21 +14032,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E113" s="32" t="str">
-        <x:v>Package RBF extends the ordinary replacement-policy model with package-level fee and cluster conditions, so learners need base RBF semantics first.</x:v>
+        <x:v>submitpackage is the admission counterpart to the existing testmempoolaccept preflight workflow, so learners need to understand local package checks before attempting submission and interpreting package results.</x:v>
       </x:c>
       <x:c r="F113" s="32" t="str">
         <x:v>source.bitcoin-core-package-policy</x:v>
       </x:c>
       <x:c r="G113" s="32" t="str">
-        <x:v>Package relay, cluster mempool, submitpackage, and pinning remain adjacent concepts rather than redundant direct edges.</x:v>
+        <x:v>Package relay and cluster mempool remain neighboring concepts rather than direct prerequisites because this node focuses on one local RPC operation.</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="32" t="str">
-        <x:v>protocol.cluster-mempool</x:v>
+        <x:v>protocol.rbf</x:v>
       </x:c>
       <x:c r="B114" s="32" t="str">
-        <x:v>ops.mempool-cluster-limits</x:v>
+        <x:v>protocol.package-rbf</x:v>
       </x:c>
       <x:c r="C114" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13957,21 +14055,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E114" s="32" t="str">
-        <x:v>Cluster limits bound connected transaction sets, so learners need the cluster-mempool model before understanding why count and aggregate virtual-size limits replace legacy ancestor/descendant limits.</x:v>
+        <x:v>Package RBF extends the ordinary replacement-policy model with package-level fee and cluster conditions, so learners need base RBF semantics first.</x:v>
       </x:c>
       <x:c r="F114" s="32" t="str">
-        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+        <x:v>source.bitcoin-core-package-policy</x:v>
       </x:c>
       <x:c r="G114" s="32" t="str">
-        <x:v>Package relay, Package RBF, CPFP, and version 3 relay remain affected workflows or neighboring policy mechanisms rather than direct prerequisites.</x:v>
+        <x:v>Package relay, cluster mempool, submitpackage, and pinning remain adjacent concepts rather than redundant direct edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="32" t="str">
-        <x:v>ops.dns-seeds</x:v>
+        <x:v>protocol.cluster-mempool</x:v>
       </x:c>
       <x:c r="B115" s="32" t="str">
-        <x:v>lightning.dns-seeds</x:v>
+        <x:v>ops.mempool-cluster-limits</x:v>
       </x:c>
       <x:c r="C115" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13980,18 +14078,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E115" s="32" t="str">
-        <x:v>Lightning DNS seeds specialize the general DNS bootstrap pattern with Lightning-specific query filters and known-peer lookup, so learners need the base DNS-seed model first.</x:v>
+        <x:v>Cluster limits bound connected transaction sets, so learners need the cluster-mempool model before understanding why count and aggregate virtual-size limits replace legacy ancestor/descendant limits.</x:v>
       </x:c>
       <x:c r="F115" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
       </x:c>
       <x:c r="G115" s="32" t="str">
-        <x:v>Peer discovery is inherited through ops.dns-seeds; generic Bitcoin P2P bootstrapping remains a parent concept rather than a duplicated edge.</x:v>
+        <x:v>Package relay, Package RBF, CPFP, and version 3 relay remain affected workflows or neighboring policy mechanisms rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="32" t="str">
-        <x:v>lightning.gossip-protocol</x:v>
+        <x:v>ops.dns-seeds</x:v>
       </x:c>
       <x:c r="B116" s="32" t="str">
         <x:v>lightning.dns-seeds</x:v>
@@ -14003,21 +14101,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E116" s="32" t="str">
-        <x:v>BOLT 10 locates Lightning peers and filters results by Lightning address information, so learners need Lightning's node-discovery and gossip context before understanding the assisted-location mechanism.</x:v>
+        <x:v>Lightning DNS seeds specialize the general DNS bootstrap pattern with Lightning-specific query filters and known-peer lookup, so learners need the base DNS-seed model first.</x:v>
       </x:c>
       <x:c r="F116" s="32" t="str">
         <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G116" s="32" t="str">
-        <x:v>Lightning routing and generic P2P messages are inherited through gossip rather than added as transitive prerequisites.</x:v>
+        <x:v>Peer discovery is inherited through ops.dns-seeds; generic Bitcoin P2P bootstrapping remains a parent concept rather than a duplicated edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="32" t="str">
-        <x:v>lightning.payment-channels</x:v>
+        <x:v>lightning.gossip-protocol</x:v>
       </x:c>
       <x:c r="B117" s="32" t="str">
-        <x:v>lightning.short-channel-id</x:v>
+        <x:v>lightning.dns-seeds</x:v>
       </x:c>
       <x:c r="C117" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14026,18 +14124,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E117" s="32" t="str">
-        <x:v>The identifier names a Lightning channel's on-chain funding output, so learners need the channel and funding relationship first.</x:v>
+        <x:v>BOLT 10 locates Lightning peers and filters results by Lightning address information, so learners need Lightning's node-discovery and gossip context before understanding the assisted-location mechanism.</x:v>
       </x:c>
       <x:c r="F117" s="32" t="str">
         <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G117" s="32" t="str">
-        <x:v>Direct channel context; the gossip protocol is a downstream consumer rather than a prerequisite.</x:v>
+        <x:v>Lightning routing and generic P2P messages are inherited through gossip rather than added as transitive prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="32" t="str">
-        <x:v>protocol.block-height</x:v>
+        <x:v>lightning.payment-channels</x:v>
       </x:c>
       <x:c r="B118" s="32" t="str">
         <x:v>lightning.short-channel-id</x:v>
@@ -14049,21 +14147,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E118" s="32" t="str">
-        <x:v>Short Channel IDs encode block height as their first component, so learners need the block-height concept before decoding the identifier.</x:v>
+        <x:v>The identifier names a Lightning channel's on-chain funding output, so learners need the channel and funding relationship first.</x:v>
       </x:c>
       <x:c r="F118" s="32" t="str">
         <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G118" s="32" t="str">
-        <x:v>The transaction-index and output-index components remain part of the identifier's own outcome rather than extra transitive edges.</x:v>
+        <x:v>Direct channel context; the gossip protocol is a downstream consumer rather than a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="32" t="str">
-        <x:v>protocol.nodes-vs-miners</x:v>
+        <x:v>protocol.block-height</x:v>
       </x:c>
       <x:c r="B119" s="32" t="str">
-        <x:v>mining.miner-decentralization</x:v>
+        <x:v>lightning.short-channel-id</x:v>
       </x:c>
       <x:c r="C119" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14072,18 +14170,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E119" s="32" t="str">
-        <x:v>Miner decentralization only makes sense once learners distinguish miners' transaction-ordering role from full nodes' independent enforcement of consensus validity.</x:v>
+        <x:v>Short Channel IDs encode block height as their first component, so learners need the block-height concept before decoding the identifier.</x:v>
       </x:c>
       <x:c r="F119" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G119" s="32" t="str">
-        <x:v>The edge keeps censorship power separate from authority to change consensus rules.</x:v>
+        <x:v>The transaction-index and output-index components remain part of the identifier's own outcome rather than extra transitive edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>protocol.nodes-vs-miners</x:v>
       </x:c>
       <x:c r="B120" s="32" t="str">
         <x:v>mining.miner-decentralization</x:v>
@@ -14095,21 +14193,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E120" s="32" t="str">
-        <x:v>Pool and solo mining explain the participant and coordination structure whose concentration or dispersion determines practical control over transaction ordering.</x:v>
+        <x:v>Miner decentralization only makes sense once learners distinguish miners' transaction-ordering role from full nodes' independent enforcement of consensus validity.</x:v>
       </x:c>
       <x:c r="F120" s="32" t="str">
         <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G120" s="32" t="str">
-        <x:v>Stratum V2 remains optional implementation context, not a direct prerequisite.</x:v>
+        <x:v>The edge keeps censorship power separate from authority to change consensus rules.</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B121" s="32" t="str">
-        <x:v>dev.selection-cryptography</x:v>
+        <x:v>mining.miner-decentralization</x:v>
       </x:c>
       <x:c r="C121" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14118,21 +14216,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E121" s="32" t="str">
-        <x:v>Selection cryptography evaluates cryptographic tools and dependencies through evidence, testing, authorship, and review quality, so learners need the broader Bitcoin review discipline first.</x:v>
+        <x:v>Pool and solo mining explain the participant and coordination structure whose concentration or dispersion determines practical control over transaction ordering.</x:v>
       </x:c>
       <x:c r="F121" s="32" t="str">
         <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G121" s="32" t="str">
-        <x:v>Adversarial thinking is inherited through dev.review-culture; reproducible builds are a downstream verification practice rather than a prerequisite.</x:v>
+        <x:v>Stratum V2 remains optional implementation context, not a direct prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="32" t="str">
-        <x:v>mining.pool-shares</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="B122" s="32" t="str">
-        <x:v>mining.block-withholding</x:v>
+        <x:v>dev.selection-cryptography</x:v>
       </x:c>
       <x:c r="C122" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14141,21 +14239,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E122" s="32" t="str">
-        <x:v>Block withholding exploits the difference between a pool-paid share and a share that also meets the network target, so learners must understand share accounting before the attack model makes sense.</x:v>
+        <x:v>Selection cryptography evaluates cryptographic tools and dependencies through evidence, testing, authorship, and review quality, so learners need the broader Bitcoin review discipline first.</x:v>
       </x:c>
       <x:c r="F122" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G122" s="32" t="str">
-        <x:v>Pool-versus-solo and mining economics are inherited through mining.pool-shares; do not add a redundant majority-attack edge.</x:v>
+        <x:v>Adversarial thinking is inherited through dev.review-culture; reproducible builds are a downstream verification practice rather than a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>mining.pool-shares</x:v>
       </x:c>
       <x:c r="B123" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>mining.block-withholding</x:v>
       </x:c>
       <x:c r="C123" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14164,18 +14262,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E123" s="32" t="str">
-        <x:v>P2C tweaks a public key to commit to contract data, so learners need the public/private key model.</x:v>
+        <x:v>Block withholding exploits the difference between a pool-paid share and a share that also meets the network target, so learners must understand share accounting before the attack model makes sense.</x:v>
       </x:c>
       <x:c r="F123" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G123" s="32" t="str">
-        <x:v>Taproot is adjacent, not a direct requirement.</x:v>
+        <x:v>Pool-versus-solo and mining economics are inherited through mining.pool-shares; do not add a redundant majority-attack edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B124" s="32" t="str">
         <x:v>protocol.pay-to-contract</x:v>
@@ -14187,21 +14285,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E124" s="32" t="str">
-        <x:v>P2C derives a commitment tweak from contract data using a hash, so learners need hash commitments first.</x:v>
+        <x:v>P2C tweaks a public key to commit to contract data, so learners need the public/private key model.</x:v>
       </x:c>
       <x:c r="F124" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G124" s="32" t="str">
-        <x:v>The hash is part of the construction rather than generic background.</x:v>
+        <x:v>Taproot is adjacent, not a direct requirement.</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="32" t="str">
-        <x:v>protocol.utxo-model</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B125" s="32" t="str">
-        <x:v>extension.single-use-seals</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="C125" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14210,21 +14308,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E125" s="32" t="str">
-        <x:v>Single-use seals rely on a UTXO's one-time spend property.</x:v>
+        <x:v>P2C derives a commitment tweak from contract data using a hash, so learners need hash commitments first.</x:v>
       </x:c>
       <x:c r="F125" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G125" s="32" t="str">
-        <x:v>This explicit bridge prevents hiding the seal invariant inside generic UTXO semantics.</x:v>
+        <x:v>The hash is part of the construction rather than generic background.</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="32" t="str">
+        <x:v>protocol.utxo-model</x:v>
+      </x:c>
+      <x:c r="B126" s="32" t="str">
         <x:v>extension.single-use-seals</x:v>
-      </x:c>
-      <x:c r="B126" s="32" t="str">
-        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="C126" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14233,18 +14331,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E126" s="32" t="str">
-        <x:v>Client-side validation relies on seals to prevent an offchain transition from being valid twice.</x:v>
+        <x:v>Single-use seals rely on a UTXO's one-time spend property.</x:v>
       </x:c>
       <x:c r="F126" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G126" s="32" t="str">
-        <x:v>The UTXO parent is inherited through the seal and is intentionally not duplicated.</x:v>
+        <x:v>This explicit bridge prevents hiding the seal invariant inside generic UTXO semantics.</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>extension.single-use-seals</x:v>
       </x:c>
       <x:c r="B127" s="32" t="str">
         <x:v>extension.client-side-validation</x:v>
@@ -14256,21 +14354,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E127" s="32" t="str">
-        <x:v>Client-side validation uses cryptographic commitments to bind offchain asset rules and transitions, so P2C supplies the contract-anchoring mechanism.</x:v>
+        <x:v>Client-side validation relies on seals to prevent an offchain transition from being valid twice.</x:v>
       </x:c>
       <x:c r="F127" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G127" s="32" t="str">
-        <x:v>Keep this direct edge: it prevents treating client-side validation as a vague UTXO-only extension.</x:v>
+        <x:v>The UTXO parent is inherited through the seal and is intentionally not duplicated.</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="32" t="str">
-        <x:v>protocol.rbf</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="B128" s="32" t="str">
-        <x:v>protocol.replacement-cycling</x:v>
+        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="C128" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14279,18 +14377,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E128" s="32" t="str">
-        <x:v>Replacement cycling repeatedly uses transaction replacement, so learners need the RBF policy mechanism first.</x:v>
+        <x:v>Client-side validation uses cryptographic commitments to bind offchain asset rules and transitions, so P2C supplies the contract-anchoring mechanism.</x:v>
       </x:c>
       <x:c r="F128" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G128" s="32" t="str">
-        <x:v>Package RBF is related but not required for the core attack sequence.</x:v>
+        <x:v>Keep this direct edge: it prevents treating client-side validation as a vague UTXO-only extension.</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="32" t="str">
-        <x:v>protocol.cpfp</x:v>
+        <x:v>protocol.rbf</x:v>
       </x:c>
       <x:c r="B129" s="32" t="str">
         <x:v>protocol.replacement-cycling</x:v>
@@ -14302,21 +14400,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E129" s="32" t="str">
-        <x:v>The attack cycles child-fee relationships to evict a target, so learners need CPFP mechanics first.</x:v>
+        <x:v>Replacement cycling repeatedly uses transaction replacement, so learners need the RBF policy mechanism first.</x:v>
       </x:c>
       <x:c r="F129" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G129" s="32" t="str">
-        <x:v>Transaction pinning is the broader downstream risk class, not a prerequisite.</x:v>
+        <x:v>Package RBF is related but not required for the core attack sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="32" t="str">
-        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
+        <x:v>protocol.cpfp</x:v>
       </x:c>
       <x:c r="B130" s="32" t="str">
-        <x:v>protocol.taproot-control-blocks</x:v>
+        <x:v>protocol.replacement-cycling</x:v>
       </x:c>
       <x:c r="C130" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14325,21 +14423,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E130" s="32" t="str">
-        <x:v>Control blocks extend the tapleaf proof path with internal-key and parity data.</x:v>
+        <x:v>The attack cycles child-fee relationships to evict a target, so learners need CPFP mechanics first.</x:v>
       </x:c>
       <x:c r="F130" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G130" s="32" t="str">
-        <x:v>Generic Merkle trees are inherited through the proof node.</x:v>
+        <x:v>Transaction pinning is the broader downstream risk class, not a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
       </x:c>
       <x:c r="B131" s="32" t="str">
-        <x:v>dev.pseudonymous-development</x:v>
+        <x:v>protocol.taproot-control-blocks</x:v>
       </x:c>
       <x:c r="C131" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14348,21 +14446,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E131" s="32" t="str">
-        <x:v>Pseudonymous development relies on public technical evidence and independent peer review to preserve accountability without requiring legal-identity disclosure.</x:v>
+        <x:v>Control blocks extend the tapleaf proof path with internal-key and parity data.</x:v>
       </x:c>
       <x:c r="F131" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G131" s="32" t="str">
-        <x:v>Privacy pseudonymity is related context, not a direct prerequisite, because this node concerns contributor identity and governance rather than transaction linkage.</x:v>
+        <x:v>Generic Merkle trees are inherited through the proof node.</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="32" t="str">
-        <x:v>fundamentals.merkle-trees</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="B132" s="32" t="str">
-        <x:v>protocol.mast</x:v>
+        <x:v>dev.pseudonymous-development</x:v>
       </x:c>
       <x:c r="C132" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14371,18 +14469,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E132" s="32" t="str">
-        <x:v>MAST uses a Merkle tree to commit to multiple alternative script branches while revealing only one branch during spending.</x:v>
+        <x:v>Pseudonymous development relies on public technical evidence and independent peer review to preserve accountability without requiring legal-identity disclosure.</x:v>
       </x:c>
       <x:c r="F132" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G132" s="32" t="str">
-        <x:v>Direct cryptographic structure; TapTree remains a downstream Taproot-specific realization.</x:v>
+        <x:v>Privacy pseudonymity is related context, not a direct prerequisite, because this node concerns contributor identity and governance rather than transaction linkage.</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>fundamentals.merkle-trees</x:v>
       </x:c>
       <x:c r="B133" s="32" t="str">
         <x:v>protocol.mast</x:v>
@@ -14394,21 +14492,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E133" s="32" t="str">
-        <x:v>MAST commits to alternative Bitcoin Script branches, so learners need the locking and spending language before the tree commitment is meaningful.</x:v>
+        <x:v>MAST uses a Merkle tree to commit to multiple alternative script branches while revealing only one branch during spending.</x:v>
       </x:c>
       <x:c r="F133" s="32" t="str">
         <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
       </x:c>
       <x:c r="G133" s="32" t="str">
-        <x:v>Keep Script direct; the node is not only a generic Merkle-tree concept.</x:v>
+        <x:v>Direct cryptographic structure; TapTree remains a downstream Taproot-specific realization.</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="32" t="str">
-        <x:v>protocol.sighash-flags</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B134" s="32" t="str">
-        <x:v>protocol.sighash-quadratic-hashing</x:v>
+        <x:v>protocol.mast</x:v>
       </x:c>
       <x:c r="C134" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14417,21 +14515,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E134" s="32" t="str">
-        <x:v>The quadratic hashing problem is a performance consequence of how legacy signature digests are constructed under SIGHASH semantics.</x:v>
+        <x:v>MAST commits to alternative Bitcoin Script branches, so learners need the locking and spending language before the tree commitment is meaningful.</x:v>
       </x:c>
       <x:c r="F134" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
       </x:c>
       <x:c r="G134" s="32" t="str">
-        <x:v>BIP 143 is a supporting mitigation source, not a prerequisite edge.</x:v>
+        <x:v>Keep Script direct; the node is not only a generic Merkle-tree concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>protocol.sighash-flags</x:v>
       </x:c>
       <x:c r="B135" s="32" t="str">
-        <x:v>security.rogue-key-attack</x:v>
+        <x:v>protocol.sighash-quadratic-hashing</x:v>
       </x:c>
       <x:c r="C135" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14440,21 +14538,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E135" s="32" t="str">
-        <x:v>The rogue-key attack occurs in naive public-key aggregation, so learners need the MuSig aggregation setting before the failure mode.</x:v>
+        <x:v>The quadratic hashing problem is a performance consequence of how legacy signature digests are constructed under SIGHASH semantics.</x:v>
       </x:c>
       <x:c r="F135" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
+        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
       </x:c>
       <x:c r="G135" s="32" t="str">
-        <x:v>Schnorr is inherited through MuSig; avoid a redundant direct Schnorr edge.</x:v>
+        <x:v>BIP 143 is a supporting mitigation source, not a prerequisite edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="B136" s="32" t="str">
-        <x:v>mining.selfish-mining</x:v>
+        <x:v>security.rogue-key-attack</x:v>
       </x:c>
       <x:c r="C136" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14463,18 +14561,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E136" s="32" t="str">
-        <x:v>Selfish mining is an incentive strategy by miners and pools, so learners need the pooled-versus-solo mining context first.</x:v>
+        <x:v>The rogue-key attack occurs in naive public-key aggregation, so learners need the MuSig aggregation setting before the failure mode.</x:v>
       </x:c>
       <x:c r="F136" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
       </x:c>
       <x:c r="G136" s="32" t="str">
-        <x:v>Pool economics is one direct parent; chain selection is supplied by the finality parent below.</x:v>
+        <x:v>Schnorr is inherited through MuSig; avoid a redundant direct Schnorr edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="32" t="str">
-        <x:v>protocol.reorgs-finality</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B137" s="32" t="str">
         <x:v>mining.selfish-mining</x:v>
@@ -14486,21 +14584,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E137" s="32" t="str">
-        <x:v>Selfish mining relies on strategic withholding and release of competing branches, which requires the chain-reorganization and finality model.</x:v>
+        <x:v>Selfish mining is an incentive strategy by miners and pools, so learners need the pooled-versus-solo mining context first.</x:v>
       </x:c>
       <x:c r="F137" s="32" t="str">
         <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
       </x:c>
       <x:c r="G137" s="32" t="str">
-        <x:v>Keep the reorganization model direct rather than adding generic proof-of-work as a redundant ancestor.</x:v>
+        <x:v>Pool economics is one direct parent; chain selection is supplied by the finality parent below.</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>protocol.reorgs-finality</x:v>
       </x:c>
       <x:c r="B138" s="32" t="str">
-        <x:v>protocol.commit-delay-reveal</x:v>
+        <x:v>mining.selfish-mining</x:v>
       </x:c>
       <x:c r="C138" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14509,21 +14607,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E138" s="32" t="str">
-        <x:v>Commit-delay-reveal composes a cryptographic commitment with a timed reveal, so the learner first needs the hiding and binding commitment model.</x:v>
+        <x:v>Selfish mining relies on strategic withholding and release of competing branches, which requires the chain-reorganization and finality model.</x:v>
       </x:c>
       <x:c r="F138" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
       </x:c>
       <x:c r="G138" s="32" t="str">
-        <x:v>The delay/reveal composition is the node's distinct outcome.</x:v>
+        <x:v>Keep the reorganization model direct rather than adding generic proof-of-work as a redundant ancestor.</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="32" t="str">
-        <x:v>protocol.dust-policy</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="B139" s="32" t="str">
-        <x:v>security.dust-attack</x:v>
+        <x:v>protocol.commit-delay-reveal</x:v>
       </x:c>
       <x:c r="C139" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14532,18 +14630,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E139" s="32" t="str">
-        <x:v>Dust attacks exploit the distinction between tiny-output relay policy and the ability to place trace-value UTXOs in a wallet.</x:v>
+        <x:v>Commit-delay-reveal composes a cryptographic commitment with a timed reveal, so the learner first needs the hiding and binding commitment model.</x:v>
       </x:c>
       <x:c r="F139" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
       </x:c>
       <x:c r="G139" s="32" t="str">
-        <x:v>Policy threshold is direct context for the attack mechanism.</x:v>
+        <x:v>The delay/reveal composition is the node's distinct outcome.</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>protocol.dust-policy</x:v>
       </x:c>
       <x:c r="B140" s="32" t="str">
         <x:v>security.dust-attack</x:v>
@@ -14555,21 +14653,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E140" s="32" t="str">
-        <x:v>The privacy harm of dusting comes from linking future spends and wallet activity, so learners need the pseudonymity and linkage model.</x:v>
+        <x:v>Dust attacks exploit the distinction between tiny-output relay policy and the ability to place trace-value UTXOs in a wallet.</x:v>
       </x:c>
       <x:c r="F140" s="32" t="str">
         <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
       </x:c>
       <x:c r="G140" s="32" t="str">
-        <x:v>Keep privacy linkage direct; it is not inherited through dust policy.</x:v>
+        <x:v>Policy threshold is direct context for the attack mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="32" t="str">
-        <x:v>fundamentals.neutrality</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B141" s="32" t="str">
-        <x:v>dev.permissionless-development</x:v>
+        <x:v>security.dust-attack</x:v>
       </x:c>
       <x:c r="C141" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14578,18 +14676,18 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E141" s="32" t="str">
-        <x:v>Permissionless development depends on a neutral protocol that does not select which users or applications may participate.</x:v>
+        <x:v>The privacy harm of dusting comes from linking future spends and wallet activity, so learners need the pseudonymity and linkage model.</x:v>
       </x:c>
       <x:c r="F141" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
       </x:c>
       <x:c r="G141" s="32" t="str">
-        <x:v>Neutrality supplies the protocol property; the BIPs process supplies the change/proposal lifecycle below.</x:v>
+        <x:v>Keep privacy linkage direct; it is not inherited through dust policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="32" t="str">
-        <x:v>dev.bips-process</x:v>
+        <x:v>fundamentals.neutrality</x:v>
       </x:c>
       <x:c r="B142" s="32" t="str">
         <x:v>dev.permissionless-development</x:v>
@@ -14601,21 +14699,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E142" s="32" t="str">
-        <x:v>Learners need the proposal and deployment process to distinguish building permissionlessly from changing Bitcoin's consensus rules without broad adoption.</x:v>
+        <x:v>Permissionless development depends on a neutral protocol that does not select which users or applications may participate.</x:v>
       </x:c>
       <x:c r="F142" s="32" t="str">
         <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G142" s="32" t="str">
-        <x:v>Review culture remains related but is not a direct prerequisite for permissionless access.</x:v>
+        <x:v>Neutrality supplies the protocol property; the BIPs process supplies the change/proposal lifecycle below.</x:v>
       </x:c>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="32" t="str">
-        <x:v>dev.reproducible-builds</x:v>
+        <x:v>dev.bips-process</x:v>
       </x:c>
       <x:c r="B143" s="32" t="str">
-        <x:v>dev.bootstrappable-builds</x:v>
+        <x:v>dev.permissionless-development</x:v>
       </x:c>
       <x:c r="C143" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14624,21 +14722,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E143" s="32" t="str">
-        <x:v>Bootstrappable builds extend reproducible builds by reducing trust in the compiler and build-tool binaries used to produce the reproducible output.</x:v>
+        <x:v>Learners need the proposal and deployment process to distinguish building permissionlessly from changing Bitcoin's consensus rules without broad adoption.</x:v>
       </x:c>
       <x:c r="F143" s="32" t="str">
         <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G143" s="32" t="str">
-        <x:v>Keep this as a direct downstream edge; the node is not a duplicate alias for reproducible builds.</x:v>
+        <x:v>Review culture remains related but is not a direct prerequisite for permissionless access.</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="32" t="str">
-        <x:v>protocol.transaction-lifecycle</x:v>
+        <x:v>dev.reproducible-builds</x:v>
       </x:c>
       <x:c r="B144" s="32" t="str">
-        <x:v>protocol.proof-of-payment</x:v>
+        <x:v>dev.bootstrappable-builds</x:v>
       </x:c>
       <x:c r="C144" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14647,21 +14745,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E144" s="32" t="str">
-        <x:v>Proof of Payment refers to a prior payment and reconstructs a transaction-shaped proof, so learners need the transaction lifecycle first.</x:v>
+        <x:v>Bootstrappable builds extend reproducible builds by reducing trust in the compiler and build-tool binaries used to produce the reproducible output.</x:v>
       </x:c>
       <x:c r="F144" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G144" s="32" t="str">
-        <x:v>Direct payment context; wallet UX and URI transport remain downstream or optional details.</x:v>
+        <x:v>Keep this as a direct downstream edge; the node is not a duplicate alias for reproducible builds.</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="32" t="str">
-        <x:v>protocol.ephemeral-anchors</x:v>
+        <x:v>protocol.transaction-lifecycle</x:v>
       </x:c>
       <x:c r="B145" s="32" t="str">
-        <x:v>protocol.pay-to-anchor</x:v>
+        <x:v>protocol.proof-of-payment</x:v>
       </x:c>
       <x:c r="C145" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14670,12 +14768,35 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E145" s="32" t="str">
-        <x:v>Pay to Anchor is a keyless refinement of the anchor-output and package-relay fee-bumping pattern, so learners need that broader context first.</x:v>
+        <x:v>Proof of Payment refers to a prior payment and reconstructs a transaction-shaped proof, so learners need the transaction lifecycle first.</x:v>
       </x:c>
       <x:c r="F145" s="32" t="str">
         <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G145" s="32" t="str">
+        <x:v>Direct payment context; wallet UX and URI transport remain downstream or optional details.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" s="32" t="str">
+        <x:v>protocol.ephemeral-anchors</x:v>
+      </x:c>
+      <x:c r="B146" s="32" t="str">
+        <x:v>protocol.pay-to-anchor</x:v>
+      </x:c>
+      <x:c r="C146" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D146" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E146" s="32" t="str">
+        <x:v>Pay to Anchor is a keyless refinement of the anchor-output and package-relay fee-bumping pattern, so learners need that broader context first.</x:v>
+      </x:c>
+      <x:c r="F146" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="G146" s="32" t="str">
         <x:v>BIP 431/TRUC is related anti-pinning context, not an inherent prerequisite.</x:v>
       </x:c>
     </x:row>
@@ -14685,10 +14806,10 @@
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C145">
+    <x:dataValidation type="list" sqref="C12:C146">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D145">
+    <x:dataValidation type="list" sqref="D12:D146">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -17744,16 +17865,42 @@
         <x:v>Offline transport examples merge into ops.mesh-networks; the other candidates remain source context without learner-facing nodes.</x:v>
       </x:c>
     </x:row>
+    <x:row r="127">
+      <x:c r="A127" s="32" t="str">
+        <x:v>decision.spark-protocol-slice</x:v>
+      </x:c>
+      <x:c r="B127" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C127" s="32" t="str">
+        <x:v>extension.spark</x:v>
+      </x:c>
+      <x:c r="D127" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E127" s="32" t="str">
+        <x:v>Spark has a distinct learner outcome from generic Statechains: understanding a concrete Bitcoin Layer 2 protocol with distributed operator coordination, off-chain transfers, offline receiving, and Lightning interoperability.</x:v>
+      </x:c>
+      <x:c r="F127" s="32" t="str">
+        <x:v>extension.spark, extension.statechains, lightning.payment-channels</x:v>
+      </x:c>
+      <x:c r="G127" s="32" t="str">
+        <x:v>source.spark-protocol</x:v>
+      </x:c>
+      <x:c r="H127" s="32" t="str">
+        <x:v>Keep Spark-specific operator internals, SDK APIs, and wallet products inside the node resources rather than creating implementation-shaped children.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B126">
+    <x:dataValidation type="list" sqref="B12:B127">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D126">
+    <x:dataValidation type="list" sqref="D12:D127">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -17806,7 +17953,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.757944282406</x:v>
+        <x:v>46214.77399011574</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -17814,7 +17961,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -17822,7 +17969,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -17830,7 +17977,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>158</x:v>
+        <x:v>159</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -17838,7 +17985,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>134</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -17862,7 +18009,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>99</x:v>
+        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add Cube learning concepts
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rcd89c3d133654fb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Rdc1578168c024e74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R2d3ac541ebbc4270"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R62086872aaee405b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rf53e320eac4f4bb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R4638edeb17084cf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R82332111d56a47a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R6863410656d446c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R9e05f0fb7cc8447b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R6c5f3171318842f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rf8400f2beddf4fb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rc13a9796e51f41e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3360,22 +3360,69 @@
         <x:v>Added Spark as a distinct implementation/protocol node downstream of Statechains; operator coordination and Lightning interoperability remain inside the Spark concept rather than becoming separate nodes.</x:v>
       </x:c>
     </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="32" t="str">
+        <x:v>source.cube-introducing</x:v>
+      </x:c>
+      <x:c r="B72" s="32" t="str">
+        <x:v>Introducing Cube</x:v>
+      </x:c>
+      <x:c r="C72" s="32" t="str">
+        <x:v>https://medium.com/cube-bitcoin/introducing-cube-8b3702e470a5</x:v>
+      </x:c>
+      <x:c r="D72" s="32" t="str">
+        <x:v>protocol-proposal-article</x:v>
+      </x:c>
+      <x:c r="E72" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F72" s="32" t="str">
+        <x:v>Cube's Bitcoin-native Layer 2, CubeVM, ZKTLCs, timeout-tree ownership virtualization, unilateral exits, Shadowing, Projector, lifting, and data-availability encoding.</x:v>
+      </x:c>
+      <x:c r="G72" s="32" t="str">
+        <x:v>Track the article's named sections as one source cluster, separating reusable learner-facing primitives from Cube-specific implementation mechanisms and speculative research directions.</x:v>
+      </x:c>
+      <x:c r="H72" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I72" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J72" s="32" t="str">
+        <x:v>Normalized</x:v>
+      </x:c>
+      <x:c r="K72" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L72" s="32" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="M72" s="32" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="N72" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O72" s="32" t="str">
+        <x:v>Added Cube, Timeout Trees, and ZKTLCs. Shadowing, Shadow Space, Projector, Hosted/Black Box Projection, Lifting, exit-ladder internals, and APE/bit-level encoding remain inside Cube or source context because they are implementation-specific mechanisms rather than independent Bitcoin learning prerequisites.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H71">
+    <x:dataValidation type="list" sqref="H12:H72">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I71">
+    <x:dataValidation type="list" sqref="I12:I72">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J71">
+    <x:dataValidation type="list" sqref="J12:J72">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K71">
+    <x:dataValidation type="list" sqref="K12:K72">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11620,16 +11667,169 @@
         <x:v>Added at the user's request after confirming the official protocol documentation and repository.</x:v>
       </x:c>
     </x:row>
+    <x:row r="171">
+      <x:c r="A171" s="32" t="str">
+        <x:v>extension.timeout-trees</x:v>
+      </x:c>
+      <x:c r="B171" s="32" t="str">
+        <x:v>Timeout Trees</x:v>
+      </x:c>
+      <x:c r="C171" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D171" s="32" t="str">
+        <x:v>source.cube-introducing</x:v>
+      </x:c>
+      <x:c r="E171" s="32" t="str">
+        <x:v>https://medium.com/cube-bitcoin/introducing-cube-8b3702e470a5</x:v>
+      </x:c>
+      <x:c r="F171" s="32" t="str">
+        <x:v>Timeout Trees section and ownership-virtualization architecture</x:v>
+      </x:c>
+      <x:c r="G171" s="32" t="str"/>
+      <x:c r="H171" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I171" s="32" t="str">
+        <x:v>Timeout Trees are a reusable settlement primitive that virtualizes many ownership outputs under a pre-signed transaction tree while preserving unilateral timeout redemption; they are broader than Cube itself.</x:v>
+      </x:c>
+      <x:c r="J171" s="32" t="str">
+        <x:v>protocol.timelocks</x:v>
+      </x:c>
+      <x:c r="K171" s="32" t="str">
+        <x:v>protocol.timelocks</x:v>
+      </x:c>
+      <x:c r="L171" s="32" t="str">
+        <x:v>Timelocks are the direct Bitcoin primitive that makes the delayed unilateral redemption path intelligible; transaction-tree details remain inside the concept.</x:v>
+      </x:c>
+      <x:c r="M171" s="32" t="str">
+        <x:v>timeout trees, transaction timeout trees</x:v>
+      </x:c>
+      <x:c r="N171" s="32" t="str">
+        <x:v>bitcoin-l2, timelocks, off-chain, settlement</x:v>
+      </x:c>
+      <x:c r="O171" s="32" t="str">
+        <x:v>50m</x:v>
+      </x:c>
+      <x:c r="P171" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q171" s="32" t="str">
+        <x:v>Add as a distinct reusable primitive rather than hiding it under Ark or Cube.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" s="32" t="str">
+        <x:v>extension.zktlcs</x:v>
+      </x:c>
+      <x:c r="B172" s="32" t="str">
+        <x:v>Zero-Knowledge Time-Locked Contracts</x:v>
+      </x:c>
+      <x:c r="C172" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D172" s="32" t="str">
+        <x:v>source.cube-introducing</x:v>
+      </x:c>
+      <x:c r="E172" s="32" t="str">
+        <x:v>https://medium.com/cube-bitcoin/introducing-cube-8b3702e470a5</x:v>
+      </x:c>
+      <x:c r="F172" s="32" t="str">
+        <x:v>ZKTLCs section and virtualized computation ownership architecture</x:v>
+      </x:c>
+      <x:c r="G172" s="32" t="str"/>
+      <x:c r="H172" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I172" s="32" t="str">
+        <x:v>ZKTLCs compose timeout-tree ownership virtualization with BitVM-style disprovable computation and unilateral timeout exits; the composition has a distinct learning outcome.</x:v>
+      </x:c>
+      <x:c r="J172" s="32" t="str">
+        <x:v>extension.timeout-trees, extension.bitvm</x:v>
+      </x:c>
+      <x:c r="K172" s="32" t="str">
+        <x:v>extension.timeout-trees, extension.bitvm</x:v>
+      </x:c>
+      <x:c r="L172" s="32" t="str">
+        <x:v>The two components are the explicit architectural halves of the primitive: delayed ownership redemption and challengeable computation.</x:v>
+      </x:c>
+      <x:c r="M172" s="32" t="str">
+        <x:v>ZKTLCs, ZK time-locked contracts, zero-knowledge time-locked contracts</x:v>
+      </x:c>
+      <x:c r="N172" s="32" t="str">
+        <x:v>bitcoin-l2, bitvm, contracts, zk</x:v>
+      </x:c>
+      <x:c r="O172" s="32" t="str">
+        <x:v>75m</x:v>
+      </x:c>
+      <x:c r="P172" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q172" s="32" t="str">
+        <x:v>Treat as a named composition, not as a duplicate of generic zero-knowledge proofs or BitVM.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" s="32" t="str">
+        <x:v>extension.cube</x:v>
+      </x:c>
+      <x:c r="B173" s="32" t="str">
+        <x:v>Cube</x:v>
+      </x:c>
+      <x:c r="C173" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D173" s="32" t="str">
+        <x:v>source.cube-introducing</x:v>
+      </x:c>
+      <x:c r="E173" s="32" t="str">
+        <x:v>https://medium.com/cube-bitcoin/introducing-cube-8b3702e470a5</x:v>
+      </x:c>
+      <x:c r="F173" s="32" t="str">
+        <x:v>Cube, CubeVM, and trustless Bitcoin-native Layer 2 architecture</x:v>
+      </x:c>
+      <x:c r="G173" s="32" t="str"/>
+      <x:c r="H173" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I173" s="32" t="str">
+        <x:v>Cube is a concrete Bitcoin-native Layer 2 and virtual machine with a distinct trust, execution, and unilateral-exit model; it is not interchangeable with generic BitVM, Ark, or smart-contract concepts.</x:v>
+      </x:c>
+      <x:c r="J173" s="32" t="str">
+        <x:v>extension.zktlcs</x:v>
+      </x:c>
+      <x:c r="K173" s="32" t="str">
+        <x:v>extension.zktlcs</x:v>
+      </x:c>
+      <x:c r="L173" s="32" t="str">
+        <x:v>ZKTLCs are the central execution-and-ownership primitive described by the article; CubeVM and data-availability details are downstream architecture.</x:v>
+      </x:c>
+      <x:c r="M173" s="32" t="str">
+        <x:v>Cube Bitcoin, CubeVM</x:v>
+      </x:c>
+      <x:c r="N173" s="32" t="str">
+        <x:v>bitcoin-l2, smart-contracts, virtual-machine, self-custody</x:v>
+      </x:c>
+      <x:c r="O173" s="32" t="str">
+        <x:v>90m</x:v>
+      </x:c>
+      <x:c r="P173" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q173" s="32" t="str">
+        <x:v>Keep Shadowing, Projector, lifting, exit-ladder internals, and DA encoding as Cube mechanisms and resources rather than separate nodes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H170">
+    <x:dataValidation type="list" sqref="H12:H173">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P170">
+    <x:dataValidation type="list" sqref="P12:P173">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11697,10 +11897,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="32" t="str">
-        <x:v>extension.statechains</x:v>
+        <x:v>protocol.timelocks</x:v>
       </x:c>
       <x:c r="B12" s="32" t="str">
-        <x:v>extension.spark</x:v>
+        <x:v>extension.timeout-trees</x:v>
       </x:c>
       <x:c r="C12" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11709,10 +11909,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E12" s="32" t="str">
-        <x:v>Spark's architecture extends statechain-style off-chain ownership transfer with a distributed operator set and Lightning interoperability.</x:v>
+        <x:v>Timeout Trees use delayed transaction branches to preserve unilateral redemption, so learners need Bitcoin timelocks first.</x:v>
       </x:c>
       <x:c r="F12" s="32" t="str">
-        <x:v>source.spark-protocol</x:v>
+        <x:v>source.cube-introducing</x:v>
       </x:c>
       <x:c r="G12" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11720,10 +11920,10 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="32" t="str">
-        <x:v>history.cypherpunk-roots-bitcoin-origin</x:v>
+        <x:v>extension.timeout-trees</x:v>
       </x:c>
       <x:c r="B13" s="32" t="str">
-        <x:v>history.satoshi-nakamoto</x:v>
+        <x:v>extension.zktlcs</x:v>
       </x:c>
       <x:c r="C13" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11732,10 +11932,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E13" s="32" t="str">
-        <x:v>Satoshi's pseudonym and founder independence are best understood in the context of Bitcoin's cypherpunk roots and origin story.</x:v>
+        <x:v>ZKTLCs use timeout-tree ownership virtualization as one half of their unified primitive.</x:v>
       </x:c>
       <x:c r="F13" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.cube-introducing</x:v>
       </x:c>
       <x:c r="G13" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11743,10 +11943,10 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="32" t="str">
-        <x:v>fundamentals.money-properties</x:v>
+        <x:v>extension.bitvm</x:v>
       </x:c>
       <x:c r="B14" s="32" t="str">
-        <x:v>economics.bitcoin-denominations</x:v>
+        <x:v>extension.zktlcs</x:v>
       </x:c>
       <x:c r="C14" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11755,10 +11955,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E14" s="32" t="str">
-        <x:v>The learner needs a basic monetary-unit model before BTC and satoshis are meaningful denominations.</x:v>
+        <x:v>ZKTLCs use BitVM-style challenge and disproof to enforce computation without trusting the executor.</x:v>
       </x:c>
       <x:c r="F14" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.cube-introducing</x:v>
       </x:c>
       <x:c r="G14" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11766,10 +11966,10 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="32" t="str">
-        <x:v>protocol.coinbase-transaction</x:v>
+        <x:v>extension.zktlcs</x:v>
       </x:c>
       <x:c r="B15" s="32" t="str">
-        <x:v>economics.block-subsidy</x:v>
+        <x:v>extension.cube</x:v>
       </x:c>
       <x:c r="C15" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11778,21 +11978,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E15" s="32" t="str">
-        <x:v>The block subsidy is the newly issued component claimed by a coinbase transaction.</x:v>
+        <x:v>Cube's architecture is built around ZKTLCs for programmable execution, ownership, and unilateral exit.</x:v>
       </x:c>
       <x:c r="F15" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.cube-introducing</x:v>
       </x:c>
       <x:c r="G15" s="32" t="str">
-        <x:v>The coinbase node already carries the halving prerequisite, so no redundant direct halving edge is added.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="32" t="str">
-        <x:v>fundamentals.digital-signatures</x:v>
+        <x:v>extension.statechains</x:v>
       </x:c>
       <x:c r="B16" s="32" t="str">
-        <x:v>security.quantum-computing-threat</x:v>
+        <x:v>extension.spark</x:v>
       </x:c>
       <x:c r="C16" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11801,10 +12001,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E16" s="32" t="str">
-        <x:v>Quantum attacks on public-key authorization require understanding ordinary Bitcoin signature security first.</x:v>
+        <x:v>Spark's architecture extends statechain-style off-chain ownership transfer with a distributed operator set and Lightning interoperability.</x:v>
       </x:c>
       <x:c r="F16" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.spark-protocol</x:v>
       </x:c>
       <x:c r="G16" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11812,10 +12012,10 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>history.cypherpunk-roots-bitcoin-origin</x:v>
       </x:c>
       <x:c r="B17" s="32" t="str">
-        <x:v>extension.ordinals-inscriptions</x:v>
+        <x:v>history.satoshi-nakamoto</x:v>
       </x:c>
       <x:c r="C17" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11824,7 +12024,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E17" s="32" t="str">
-        <x:v>The source explains inscriptions as a Taproot-era witness-data application.</x:v>
+        <x:v>Satoshi's pseudonym and founder independence are best understood in the context of Bitcoin's cypherpunk roots and origin story.</x:v>
       </x:c>
       <x:c r="F17" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
@@ -11835,10 +12035,10 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="32" t="str">
-        <x:v>protocol.witness-structure</x:v>
+        <x:v>fundamentals.money-properties</x:v>
       </x:c>
       <x:c r="B18" s="32" t="str">
-        <x:v>extension.ordinals-inscriptions</x:v>
+        <x:v>economics.bitcoin-denominations</x:v>
       </x:c>
       <x:c r="C18" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11847,7 +12047,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E18" s="32" t="str">
-        <x:v>Witness structure is needed to understand where inscription data is carried and how it affects block space.</x:v>
+        <x:v>The learner needs a basic monetary-unit model before BTC and satoshis are meaningful denominations.</x:v>
       </x:c>
       <x:c r="F18" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
@@ -11858,10 +12058,10 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>protocol.coinbase-transaction</x:v>
       </x:c>
       <x:c r="B19" s="32" t="str">
-        <x:v>extension.proof-of-existence</x:v>
+        <x:v>economics.block-subsidy</x:v>
       </x:c>
       <x:c r="C19" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11870,21 +12070,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E19" s="32" t="str">
-        <x:v>Timestamp proofs commit evidence without requiring the complete document to be stored on-chain.</x:v>
+        <x:v>The block subsidy is the newly issued component claimed by a coinbase transaction.</x:v>
       </x:c>
       <x:c r="F19" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G19" s="32" t="str">
-        <x:v>Source-driven bridge edge.</x:v>
+        <x:v>The coinbase node already carries the halving prerequisite, so no redundant direct halving edge is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="32" t="str">
-        <x:v>protocol.tagged-hashes</x:v>
+        <x:v>fundamentals.digital-signatures</x:v>
       </x:c>
       <x:c r="B20" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>security.quantum-computing-threat</x:v>
       </x:c>
       <x:c r="C20" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11893,10 +12093,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E20" s="32" t="str">
-        <x:v>TapTweak is defined using tagged hashes directly in Taproot key tweaking.</x:v>
+        <x:v>Quantum attacks on public-key authorization require understanding ordinary Bitcoin signature security first.</x:v>
       </x:c>
       <x:c r="F20" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G20" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11904,10 +12104,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="str">
-        <x:v>protocol.x-only-public-keys</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B21" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>extension.ordinals-inscriptions</x:v>
       </x:c>
       <x:c r="C21" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11916,10 +12116,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E21" s="32" t="str">
-        <x:v>TapTweak operates on x-only public keys in the Taproot construction.</x:v>
+        <x:v>The source explains inscriptions as a Taproot-era witness-data application.</x:v>
       </x:c>
       <x:c r="F21" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G21" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11927,10 +12127,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>protocol.witness-structure</x:v>
       </x:c>
       <x:c r="B22" s="32" t="str">
-        <x:v>protocol.taproot-key-path-spends</x:v>
+        <x:v>extension.ordinals-inscriptions</x:v>
       </x:c>
       <x:c r="C22" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11939,21 +12139,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E22" s="32" t="str">
-        <x:v>A key-path spend verifies against the tweaked Taproot output key, so learners need the tweak mechanism before the spending mode makes sense.</x:v>
+        <x:v>Witness structure is needed to understand where inscription data is carried and how it affects block space.</x:v>
       </x:c>
       <x:c r="F22" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G22" s="32" t="str">
-        <x:v>Direct parent keeps the node focused on the spend mode rather than on broad Taproot overview material.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32" t="str">
-        <x:v>protocol.taptree</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="B23" s="32" t="str">
-        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
+        <x:v>extension.proof-of-existence</x:v>
       </x:c>
       <x:c r="C23" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11962,10 +12162,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E23" s="32" t="str">
-        <x:v>The inclusion proof only makes sense after the learner understands the TapTree structure.</x:v>
+        <x:v>Timestamp proofs commit evidence without requiring the complete document to be stored on-chain.</x:v>
       </x:c>
       <x:c r="F23" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G23" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11973,10 +12173,10 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="str">
-        <x:v>protocol.taptree</x:v>
+        <x:v>protocol.tagged-hashes</x:v>
       </x:c>
       <x:c r="B24" s="32" t="str">
-        <x:v>protocol.huffman-optimized-taptrees</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="C24" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11985,7 +12185,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E24" s="32" t="str">
-        <x:v>Huffman optimization is a refinement of how TapTree leaves are arranged.</x:v>
+        <x:v>TapTweak is defined using tagged hashes directly in Taproot key tweaking.</x:v>
       </x:c>
       <x:c r="F24" s="32" t="str">
         <x:v>source.optech-schnorr-taproot-workshop</x:v>
@@ -11996,10 +12196,10 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="str">
-        <x:v>protocol.softfork-hardfork</x:v>
+        <x:v>protocol.x-only-public-keys</x:v>
       </x:c>
       <x:c r="B25" s="32" t="str">
-        <x:v>protocol.chain-split-risk</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="C25" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12008,21 +12208,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E25" s="32" t="str">
-        <x:v>Split risk is a downstream consequence of incompatible upgrade paths, so learners should understand the compatibility boundary first.</x:v>
+        <x:v>TapTweak operates on x-only public keys in the Taproot construction.</x:v>
       </x:c>
       <x:c r="F25" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G25" s="32" t="str">
-        <x:v>Direct edge chosen over activation-history case studies because those are downstream examples, not prerequisites.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="B26" s="32" t="str">
-        <x:v>protocol.tapscript</x:v>
+        <x:v>protocol.taproot-key-path-spends</x:v>
       </x:c>
       <x:c r="C26" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12031,21 +12231,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E26" s="32" t="str">
-        <x:v>Tapscript is a Taproot-specific script version, so learners need the Taproot spend context before its rule changes make sense.</x:v>
+        <x:v>A key-path spend verifies against the tweaked Taproot output key, so learners need the tweak mechanism before the spending mode makes sense.</x:v>
       </x:c>
       <x:c r="F26" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G26" s="32" t="str">
-        <x:v>Direct edge keeps the node scoped to the Taproot family without collapsing it into a generic script refresher.</x:v>
+        <x:v>Direct parent keeps the node focused on the spend mode rather than on broad Taproot overview material.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="str">
-        <x:v>custody.psbt</x:v>
+        <x:v>protocol.taptree</x:v>
       </x:c>
       <x:c r="B27" s="32" t="str">
-        <x:v>dev.taproot-psbt-fields</x:v>
+        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
       </x:c>
       <x:c r="C27" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12054,21 +12254,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E27" s="32" t="str">
-        <x:v>Taproot PSBT fields extend the base PSBT container, so learners need the general workflow and field model before the Taproot additions make sense.</x:v>
+        <x:v>The inclusion proof only makes sense after the learner understands the TapTree structure.</x:v>
       </x:c>
       <x:c r="F27" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G27" s="32" t="str">
-        <x:v>Direct edge keeps the slice anchored on the generic PSBT exchange model rather than on a narrower implementation variant.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.taptree</x:v>
       </x:c>
       <x:c r="B28" s="32" t="str">
-        <x:v>dev.taproot-psbt-fields</x:v>
+        <x:v>protocol.huffman-optimized-taptrees</x:v>
       </x:c>
       <x:c r="C28" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12077,13 +12277,13 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E28" s="32" t="str">
-        <x:v>These fields carry Taproot-specific keys, scripts, and Merkle-path data, so learners need the Taproot spend model before the PSBT extensions are meaningful.</x:v>
+        <x:v>Huffman optimization is a refinement of how TapTree leaves are arranged.</x:v>
       </x:c>
       <x:c r="F28" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G28" s="32" t="str">
-        <x:v>The direct dev.psbt-v2 edge was intentionally dropped because BIP371 applies to PSBTv0 and PSBTv2.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -12091,7 +12291,7 @@
         <x:v>protocol.softfork-hardfork</x:v>
       </x:c>
       <x:c r="B29" s="32" t="str">
-        <x:v>protocol.accidental-confiscation</x:v>
+        <x:v>protocol.chain-split-risk</x:v>
       </x:c>
       <x:c r="C29" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12100,21 +12300,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E29" s="32" t="str">
-        <x:v>Accidental confiscation is a failure mode caused by new soft-fork restrictions, so learners need the soft-fork compatibility model before the risk is intelligible.</x:v>
+        <x:v>Split risk is a downstream consequence of incompatible upgrade paths, so learners should understand the compatibility boundary first.</x:v>
       </x:c>
       <x:c r="F29" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G29" s="32" t="str">
-        <x:v>Direct edge chosen over chain-split-risk and standardness-policy because those branches add context but are not required for the core failure mode.</x:v>
+        <x:v>Direct edge chosen over activation-history case studies because those are downstream examples, not prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32" t="str">
-        <x:v>protocol.fee-market</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B30" s="32" t="str">
-        <x:v>custody.coin-selection</x:v>
+        <x:v>protocol.tapscript</x:v>
       </x:c>
       <x:c r="C30" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12123,21 +12323,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E30" s="32" t="str">
-        <x:v>Wallets choose different UTXO sets partly to minimize transaction size and fee cost, so fee pressure is a direct part of the concept.</x:v>
+        <x:v>Tapscript is a Taproot-specific script version, so learners need the Taproot spend context before its rule changes make sense.</x:v>
       </x:c>
       <x:c r="F30" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G30" s="32" t="str">
-        <x:v>Direct edge keeps the node connected to transaction-cost tradeoffs rather than only to wallet UX.</x:v>
+        <x:v>Direct edge keeps the node scoped to the Taproot family without collapsing it into a generic script refresher.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>custody.psbt</x:v>
       </x:c>
       <x:c r="B31" s="32" t="str">
-        <x:v>protocol.change-outputs</x:v>
+        <x:v>dev.taproot-psbt-fields</x:v>
       </x:c>
       <x:c r="C31" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12146,21 +12346,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E31" s="32" t="str">
-        <x:v>Change is a specific kind of transaction output, so learners need the basic output and spendability model before the leftover-value pattern makes sense.</x:v>
+        <x:v>Taproot PSBT fields extend the base PSBT container, so learners need the general workflow and field model before the Taproot additions make sense.</x:v>
       </x:c>
       <x:c r="F31" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G31" s="32" t="str">
-        <x:v>Direct edge keeps the node between raw output structure and the later wallet-decision branch.</x:v>
+        <x:v>Direct edge keeps the slice anchored on the generic PSBT exchange model rather than on a narrower implementation variant.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B32" s="32" t="str">
-        <x:v>dev.taproot-descriptors</x:v>
+        <x:v>dev.taproot-psbt-fields</x:v>
       </x:c>
       <x:c r="C32" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12169,21 +12369,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E32" s="32" t="str">
-        <x:v>Taproot descriptors extend the general descriptor grammar, so learners need the base descriptor model before the tr() specialization makes sense.</x:v>
+        <x:v>These fields carry Taproot-specific keys, scripts, and Merkle-path data, so learners need the Taproot spend model before the PSBT extensions are meaningful.</x:v>
       </x:c>
       <x:c r="F32" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G32" s="32" t="str">
-        <x:v>Direct edge keeps the node scoped to descriptor structure instead of wallet import behavior.</x:v>
+        <x:v>The direct dev.psbt-v2 edge was intentionally dropped because BIP371 applies to PSBTv0 and PSBTv2.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.softfork-hardfork</x:v>
       </x:c>
       <x:c r="B33" s="32" t="str">
-        <x:v>dev.taproot-descriptors</x:v>
+        <x:v>protocol.accidental-confiscation</x:v>
       </x:c>
       <x:c r="C33" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12192,21 +12392,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E33" s="32" t="str">
-        <x:v>The tr() descriptor exists specifically to encode P2TR outputs and optional Taproot script-path commitments, so learners need the Taproot output model first.</x:v>
+        <x:v>Accidental confiscation is a failure mode caused by new soft-fork restrictions, so learners need the soft-fork compatibility model before the risk is intelligible.</x:v>
       </x:c>
       <x:c r="F33" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G33" s="32" t="str">
-        <x:v>Direct edge keeps the node grounded in Taproot output semantics rather than in generic descriptor syntax alone.</x:v>
+        <x:v>Direct edge chosen over chain-split-risk and standardness-policy because those branches add context but are not required for the core failure mode.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="32" t="str">
-        <x:v>protocol.transaction-pinning</x:v>
+        <x:v>protocol.fee-market</x:v>
       </x:c>
       <x:c r="B34" s="32" t="str">
-        <x:v>protocol.version-3-transaction-relay</x:v>
+        <x:v>custody.coin-selection</x:v>
       </x:c>
       <x:c r="C34" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12215,21 +12415,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E34" s="32" t="str">
-        <x:v>Version 3 relay is a targeted policy response to transaction pinning, so learners should understand the attack class before the mitigation.</x:v>
+        <x:v>Wallets choose different UTXO sets partly to minimize transaction size and fee cost, so fee pressure is a direct part of the concept.</x:v>
       </x:c>
       <x:c r="F34" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G34" s="32" t="str">
-        <x:v>Direct edge chosen over package-relay because the pinning problem is the narrower immediate teaching need.</x:v>
+        <x:v>Direct edge keeps the node connected to transaction-cost tradeoffs rather than only to wallet UX.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="32" t="str">
-        <x:v>fundamentals.trustlessness</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B35" s="32" t="str">
-        <x:v>fundamentals.validation-sovereignty</x:v>
+        <x:v>protocol.change-outputs</x:v>
       </x:c>
       <x:c r="C35" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12238,21 +12438,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E35" s="32" t="str">
-        <x:v>Validation sovereignty is an applied consequence of trustlessness and verification culture.</x:v>
+        <x:v>Change is a specific kind of transaction output, so learners need the basic output and spendability model before the leftover-value pattern makes sense.</x:v>
       </x:c>
       <x:c r="F35" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G35" s="32" t="str">
-        <x:v>Bridge edge inferred from philosophy sequencing.</x:v>
+        <x:v>Direct edge keeps the node between raw output structure and the later wallet-decision branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="32" t="str">
-        <x:v>ops.run-full-node</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B36" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>dev.taproot-descriptors</x:v>
       </x:c>
       <x:c r="C36" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12261,21 +12461,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E36" s="32" t="str">
-        <x:v>Learners need the full-node baseline before they can understand which validation guarantees a light client gives up.</x:v>
+        <x:v>Taproot descriptors extend the general descriptor grammar, so learners need the base descriptor model before the tr() specialization makes sense.</x:v>
       </x:c>
       <x:c r="F36" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G36" s="32" t="str">
-        <x:v>Bridge edge inferred from full-node versus lightweight-client contrast.</x:v>
+        <x:v>Direct edge keeps the node scoped to descriptor structure instead of wallet import behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="32" t="str">
-        <x:v>protocol.compact-block-filters</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B37" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>dev.taproot-descriptors</x:v>
       </x:c>
       <x:c r="C37" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12284,21 +12484,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E37" s="32" t="str">
-        <x:v>Compact block filters provide the modern filtered-client mechanism that anchors the trust-model comparison.</x:v>
+        <x:v>The tr() descriptor exists specifically to encode P2TR outputs and optional Taproot script-path commitments, so learners need the Taproot output model first.</x:v>
       </x:c>
       <x:c r="F37" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G37" s="32" t="str">
-        <x:v>Kept additive and conceptual instead of rewiring older light-client mechanism leaves in the same slice.</x:v>
+        <x:v>Direct edge keeps the node grounded in Taproot output semantics rather than in generic descriptor syntax alone.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="32" t="str">
-        <x:v>fundamentals.validation-sovereignty</x:v>
+        <x:v>protocol.transaction-pinning</x:v>
       </x:c>
       <x:c r="B38" s="32" t="str">
-        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
+        <x:v>protocol.version-3-transaction-relay</x:v>
       </x:c>
       <x:c r="C38" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12307,21 +12507,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E38" s="32" t="str">
-        <x:v>The comparison only matters once the learner understands why self-validation is valuable in the first place.</x:v>
+        <x:v>Version 3 relay is a targeted policy response to transaction pinning, so learners should understand the attack class before the mitigation.</x:v>
       </x:c>
       <x:c r="F38" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G38" s="32" t="str">
-        <x:v>User-facing prerequisite edge for the wallet-mode decision.</x:v>
+        <x:v>Direct edge chosen over package-relay because the pinning problem is the narrower immediate teaching need.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>fundamentals.trustlessness</x:v>
       </x:c>
       <x:c r="B39" s="32" t="str">
-        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
+        <x:v>fundamentals.validation-sovereignty</x:v>
       </x:c>
       <x:c r="C39" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12330,21 +12530,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E39" s="32" t="str">
-        <x:v>Learners need the mechanism-level trust tradeoffs before comparing full-node wallets with lightweight clients.</x:v>
+        <x:v>Validation sovereignty is an applied consequence of trustlessness and verification culture.</x:v>
       </x:c>
       <x:c r="F39" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G39" s="32" t="str">
-        <x:v>First downstream consumer for the light-client trust branch.</x:v>
+        <x:v>Bridge edge inferred from philosophy sequencing.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>ops.run-full-node</x:v>
       </x:c>
       <x:c r="B40" s="32" t="str">
-        <x:v>protocol.p2pk</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="C40" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12353,21 +12553,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E40" s="32" t="str">
-        <x:v>P2PK is a concrete legacy script template, so learners first need the locking and unlocking model from Bitcoin Script.</x:v>
+        <x:v>Learners need the full-node baseline before they can understand which validation guarantees a light client gives up.</x:v>
       </x:c>
       <x:c r="F40" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G40" s="32" t="str">
-        <x:v>Chosen as the first script-history leaf from Decoding after dedupe and direct-edge review.</x:v>
+        <x:v>Bridge edge inferred from full-node versus lightweight-client contrast.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32" t="str">
-        <x:v>fundamentals.schnorr-signatures</x:v>
+        <x:v>protocol.compact-block-filters</x:v>
       </x:c>
       <x:c r="B41" s="32" t="str">
-        <x:v>security.nonce-reuse-attack</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="C41" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12376,21 +12576,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E41" s="32" t="str">
-        <x:v>The nonce-reuse failure only makes sense after the learner understands the Schnorr signing flow that produces the nonce and signature pair.</x:v>
+        <x:v>Compact block filters provide the modern filtered-client mechanism that anchors the trust-model comparison.</x:v>
       </x:c>
       <x:c r="F41" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G41" s="32" t="str">
-        <x:v>Chosen as a narrow additive security slice without bundling it to custody-side defenses.</x:v>
+        <x:v>Kept additive and conceptual instead of rewiring older light-client mechanism leaves in the same slice.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="32" t="str">
-        <x:v>protocol.p2pk</x:v>
+        <x:v>fundamentals.validation-sovereignty</x:v>
       </x:c>
       <x:c r="B42" s="32" t="str">
-        <x:v>protocol.p2pkh</x:v>
+        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
       </x:c>
       <x:c r="C42" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12399,21 +12599,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E42" s="32" t="str">
-        <x:v>P2PKH is easiest to understand as the hashed-public-key refinement of a direct public-key output.</x:v>
+        <x:v>The comparison only matters once the learner understands why self-validation is valuable in the first place.</x:v>
       </x:c>
       <x:c r="F42" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G42" s="32" t="str">
-        <x:v>Chosen to preserve the output-template ladder without repeating the broader Script prerequisite directly.</x:v>
+        <x:v>User-facing prerequisite edge for the wallet-mode decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="B43" s="32" t="str">
-        <x:v>protocol.p2pkh</x:v>
+        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
       </x:c>
       <x:c r="C43" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12422,13 +12622,13 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E43" s="32" t="str">
-        <x:v>Hash-based locking only makes sense once the learner understands what a hash commits to and why it can stand in for the public key until spend time.</x:v>
+        <x:v>Learners need the mechanism-level trust tradeoffs before comparing full-node wallets with lightweight clients.</x:v>
       </x:c>
       <x:c r="F43" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G43" s="32" t="str">
-        <x:v>Required to keep the node about public-key hashing rather than just script syntax.</x:v>
+        <x:v>First downstream consumer for the light-client trust branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -12436,7 +12636,7 @@
         <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B44" s="32" t="str">
-        <x:v>protocol.op-checkmultisig</x:v>
+        <x:v>protocol.p2pk</x:v>
       </x:c>
       <x:c r="C44" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12445,21 +12645,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E44" s="32" t="str">
-        <x:v>OP_CHECKMULTISIG is an opcode-level script mechanic, so learners first need the general Script model and stack execution basics.</x:v>
+        <x:v>P2PK is a concrete legacy script template, so learners first need the locking and unlocking model from Bitcoin Script.</x:v>
       </x:c>
       <x:c r="F44" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G44" s="32" t="str">
-        <x:v>Chosen as the mechanism bridge before protocol.p2ms.</x:v>
+        <x:v>Chosen as the first script-history leaf from Decoding after dedupe and direct-edge review.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="32" t="str">
-        <x:v>protocol.op-checkmultisig</x:v>
+        <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="B45" s="32" t="str">
-        <x:v>protocol.p2ms</x:v>
+        <x:v>security.nonce-reuse-attack</x:v>
       </x:c>
       <x:c r="C45" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12468,21 +12668,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E45" s="32" t="str">
-        <x:v>Bare multisig is the concrete locking template built from OP_CHECKMULTISIG, so the opcode is the clean direct parent once introduced.</x:v>
+        <x:v>The nonce-reuse failure only makes sense after the learner understands the Schnorr signing flow that produces the nonce and signature pair.</x:v>
       </x:c>
       <x:c r="F45" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G45" s="32" t="str">
-        <x:v>Replaces the earlier curricular and wallet-semantic parent candidates.</x:v>
+        <x:v>Chosen as a narrow additive security slice without bundling it to custody-side defenses.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="32" t="str">
-        <x:v>protocol.p2ms</x:v>
+        <x:v>protocol.p2pk</x:v>
       </x:c>
       <x:c r="B46" s="32" t="str">
-        <x:v>protocol.bare-multisig-standardness</x:v>
+        <x:v>protocol.p2pkh</x:v>
       </x:c>
       <x:c r="C46" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12491,21 +12691,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E46" s="32" t="str">
-        <x:v>The relay treatment only makes sense once the learner understands what a bare multisig output actually is on-chain.</x:v>
+        <x:v>P2PKH is easiest to understand as the hashed-public-key refinement of a direct public-key output.</x:v>
       </x:c>
       <x:c r="F46" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G46" s="32" t="str">
-        <x:v>Policy leaf anchored on the specific legacy script template it constrains.</x:v>
+        <x:v>Chosen to preserve the output-template ladder without repeating the broader Script prerequisite directly.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="32" t="str">
-        <x:v>protocol.standardness-policy</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B47" s="32" t="str">
-        <x:v>protocol.bare-multisig-standardness</x:v>
+        <x:v>protocol.p2pkh</x:v>
       </x:c>
       <x:c r="C47" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12514,21 +12714,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E47" s="32" t="str">
-        <x:v>This node is a concrete application of standard transaction policy, so the general standardness concept should come first.</x:v>
+        <x:v>Hash-based locking only makes sense once the learner understands what a hash commits to and why it can stand in for the public key until spend time.</x:v>
       </x:c>
       <x:c r="F47" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G47" s="32" t="str">
-        <x:v>Policy-boundary prerequisite inherited through the existing mempool-policy branch.</x:v>
+        <x:v>Required to keep the node about public-key hashing rather than just script syntax.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B48" s="32" t="str">
-        <x:v>dev.scriptpubkeymanagers</x:v>
+        <x:v>protocol.op-checkmultisig</x:v>
       </x:c>
       <x:c r="C48" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12537,21 +12737,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E48" s="32" t="str">
-        <x:v>Modern descriptor wallets hand descriptor-backed script templates to dedicated managers, so learners need the descriptor model before the SPKM boundary makes sense.</x:v>
+        <x:v>OP_CHECKMULTISIG is an opcode-level script mechanic, so learners first need the general Script model and stack execution basics.</x:v>
       </x:c>
       <x:c r="F48" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-wallet</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G48" s="32" t="str">
-        <x:v>Direct edge distinguishes the Core wallet abstraction from descriptor syntax without collapsing the two concepts into one node.</x:v>
+        <x:v>Chosen as the mechanism bridge before protocol.p2ms.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="32" t="str">
-        <x:v>protocol.mempool</x:v>
+        <x:v>protocol.op-checkmultisig</x:v>
       </x:c>
       <x:c r="B49" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>protocol.p2ms</x:v>
       </x:c>
       <x:c r="C49" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12560,21 +12760,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E49" s="32" t="str">
-        <x:v>The unbroadcast set is a mempool-owned data structure, so learners need the local unconfirmed transaction pool model before this narrower tracking mechanism makes sense.</x:v>
+        <x:v>Bare multisig is the concrete locking template built from OP_CHECKMULTISIG, so the opcode is the clean direct parent once introduced.</x:v>
       </x:c>
       <x:c r="F49" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G49" s="32" t="str">
-        <x:v>Direct edge keeps the concept scoped to local transaction state rather than broader relay policy.</x:v>
+        <x:v>Replaces the earlier curricular and wallet-semantic parent candidates.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="32" t="str">
-        <x:v>protocol.transaction-relay-inv-getdata</x:v>
+        <x:v>protocol.p2ms</x:v>
       </x:c>
       <x:c r="B50" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>protocol.bare-multisig-standardness</x:v>
       </x:c>
       <x:c r="C50" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12583,21 +12783,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E50" s="32" t="str">
-        <x:v>This set only matters because nodes need to distinguish locally submitted transactions from those later observed through the network relay path and may retry announcing them.</x:v>
+        <x:v>The relay treatment only makes sense once the learner understands what a bare multisig output actually is on-chain.</x:v>
       </x:c>
       <x:c r="F50" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G50" s="32" t="str">
-        <x:v>Direct edge ties the mechanism to network propagation confirmation and rebroadcast attempts.</x:v>
+        <x:v>Policy leaf anchored on the specific legacy script template it constrains.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="32" t="str">
-        <x:v>privacy.address-reuse</x:v>
+        <x:v>protocol.standardness-policy</x:v>
       </x:c>
       <x:c r="B51" s="32" t="str">
-        <x:v>custody.human-readable-addresses</x:v>
+        <x:v>protocol.bare-multisig-standardness</x:v>
       </x:c>
       <x:c r="C51" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12606,21 +12806,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E51" s="32" t="str">
-        <x:v>A major design constraint is that reusable human-readable handles can worsen privacy unless they resolve to reusable payment mechanisms or rotate safely, so learners need the address-reuse problem first.</x:v>
+        <x:v>This node is a concrete application of standard transaction policy, so the general standardness concept should come first.</x:v>
       </x:c>
       <x:c r="F51" s="32" t="str">
-        <x:v>source.bitcoin-design-payment-formats</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G51" s="32" t="str">
-        <x:v>Direct edge captures the main privacy tradeoff without forcing downstream protocol-specific address schemes into prerequisites.</x:v>
+        <x:v>Policy-boundary prerequisite inherited through the existing mempool-policy branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="32" t="str">
-        <x:v>custody.output-labeling</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B52" s="32" t="str">
-        <x:v>custody.transaction-metadata</x:v>
+        <x:v>dev.scriptpubkeymanagers</x:v>
       </x:c>
       <x:c r="C52" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12629,21 +12829,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E52" s="32" t="str">
-        <x:v>Output labeling already introduces the idea that wallets attach their own context to payments and spendable objects, making it the cleanest direct bridge into broader transaction-level notes, contacts, and portability concerns.</x:v>
+        <x:v>Modern descriptor wallets hand descriptor-backed script templates to dedicated managers, so learners need the descriptor model before the SPKM boundary makes sense.</x:v>
       </x:c>
       <x:c r="F52" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoin-core-academy-wallet</x:v>
       </x:c>
       <x:c r="G52" s="32" t="str">
-        <x:v>Direct edge distinguishes wider payment-history context from narrower spend-control labels without treating them as unrelated.</x:v>
+        <x:v>Direct edge distinguishes the Core wallet abstraction from descriptor syntax without collapsing the two concepts into one node.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>protocol.mempool</x:v>
       </x:c>
       <x:c r="B53" s="32" t="str">
-        <x:v>custody.transaction-metadata</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="C53" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12652,21 +12852,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E53" s="32" t="str">
-        <x:v>Wallet-added names, notes, and contact links matter partly because transaction history is only pseudonymous and can reveal meaningful patterns when users or tools correlate activity over time.</x:v>
+        <x:v>The unbroadcast set is a mempool-owned data structure, so learners need the local unconfirmed transaction pool model before this narrower tracking mechanism makes sense.</x:v>
       </x:c>
       <x:c r="F53" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G53" s="32" t="str">
-        <x:v>Direct edge keeps the node tied to the privacy and identity meaning of payment history rather than only to generic lifecycle sequencing.</x:v>
+        <x:v>Direct edge keeps the concept scoped to local transaction state rather than broader relay policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="32" t="str">
-        <x:v>custody.self-custody</x:v>
+        <x:v>protocol.transaction-relay-inv-getdata</x:v>
       </x:c>
       <x:c r="B54" s="32" t="str">
-        <x:v>custody.multiple-wallets</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="C54" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12675,21 +12875,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E54" s="32" t="str">
-        <x:v>Deliberately separating funds across different wallet buckets is a custody decision, so learners need the base self-custody responsibility model before the organizational pattern makes sense.</x:v>
+        <x:v>This set only matters because nodes need to distinguish locally submitted transactions from those later observed through the network relay path and may retry announcing them.</x:v>
       </x:c>
       <x:c r="F54" s="32" t="str">
-        <x:v>source.bitcoin-design-multiple-wallets</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G54" s="32" t="str">
-        <x:v>Kept the direct parent at the responsibility-model layer; multisig, watch-only, and HD account structures remain examples or implementation details rather than prerequisites.</x:v>
+        <x:v>Direct edge ties the mechanism to network propagation confirmation and rebroadcast attempts.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="32" t="str">
-        <x:v>custody.hardware-wallets</x:v>
+        <x:v>privacy.address-reuse</x:v>
       </x:c>
       <x:c r="B55" s="32" t="str">
-        <x:v>custody.progressive-security</x:v>
+        <x:v>custody.human-readable-addresses</x:v>
       </x:c>
       <x:c r="C55" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12698,21 +12898,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E55" s="32" t="str">
-        <x:v>One of the core upgrade steps in the reference design is moving from default low-friction storage to an external signing device, so learners need the hardware-signing model before the staged-upgrade pattern makes sense.</x:v>
+        <x:v>A major design constraint is that reusable human-readable handles can worsen privacy unless they resolve to reusable payment mechanisms or rotate safely, so learners need the address-reuse problem first.</x:v>
       </x:c>
       <x:c r="F55" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoin-design-payment-formats</x:v>
       </x:c>
       <x:c r="G55" s="32" t="str">
-        <x:v>Direct edge captures the mid-tier upgrade target without treating cloud backup itself as the core concept.</x:v>
+        <x:v>Direct edge captures the main privacy tradeoff without forcing downstream protocol-specific address schemes into prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>custody.output-labeling</x:v>
       </x:c>
       <x:c r="B56" s="32" t="str">
-        <x:v>custody.progressive-security</x:v>
+        <x:v>custody.transaction-metadata</x:v>
       </x:c>
       <x:c r="C56" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12721,21 +12921,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E56" s="32" t="str">
-        <x:v>The higher-security end of the progression moves into 2-of-3 and 3-of-5 multi-key schemes, so learners need the multisig model before they can reason about why and when a wallet should escalate there.</x:v>
+        <x:v>Output labeling already introduces the idea that wallets attach their own context to payments and spendable objects, making it the cleanest direct bridge into broader transaction-level notes, contacts, and portability concerns.</x:v>
       </x:c>
       <x:c r="F56" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="G56" s="32" t="str">
-        <x:v>Direct edge captures the high-assurance destination of the progression rather than a specific product flow.</x:v>
+        <x:v>Direct edge distinguishes wider payment-history context from narrower spend-control labels without treating them as unrelated.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B57" s="32" t="str">
-        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
+        <x:v>custody.transaction-metadata</x:v>
       </x:c>
       <x:c r="C57" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12744,21 +12944,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E57" s="32" t="str">
-        <x:v>Rebroadcast privacy builds directly on the local-node distinction between transactions merely accepted into the mempool and transactions known to have propagated, which is exactly the gap the unbroadcast set tracks.</x:v>
+        <x:v>Wallet-added names, notes, and contact links matter partly because transaction history is only pseudonymous and can reveal meaningful patterns when users or tools correlate activity over time.</x:v>
       </x:c>
       <x:c r="F57" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="G57" s="32" t="str">
-        <x:v>Direct parent keeps the slice on the local tracking mechanism rather than reintroducing generic relay ancestors.</x:v>
+        <x:v>Direct edge keeps the node tied to the privacy and identity meaning of payment history rather than only to generic lifecycle sequencing.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>custody.self-custody</x:v>
       </x:c>
       <x:c r="B58" s="32" t="str">
-        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
+        <x:v>custody.multiple-wallets</x:v>
       </x:c>
       <x:c r="C58" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12767,21 +12967,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E58" s="32" t="str">
-        <x:v>Different rebroadcast patterns matter because observers can correlate network behavior with public transaction history and infer likely origin, so learners need the pseudonymity and linkage problem first.</x:v>
+        <x:v>Deliberately separating funds across different wallet buckets is a custody decision, so learners need the base self-custody responsibility model before the organizational pattern makes sense.</x:v>
       </x:c>
       <x:c r="F58" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-multiple-wallets</x:v>
       </x:c>
       <x:c r="G58" s="32" t="str">
-        <x:v>Direct parent keeps the node focused on why relay-side origin leakage matters, not just how rebroadcast code works.</x:v>
+        <x:v>Kept the direct parent at the responsibility-model layer; multisig, watch-only, and HD account structures remain examples or implementation details rather than prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="32" t="str">
-        <x:v>protocol.segregated-witness</x:v>
+        <x:v>custody.hardware-wallets</x:v>
       </x:c>
       <x:c r="B59" s="32" t="str">
-        <x:v>protocol.txid-vs-wtxid</x:v>
+        <x:v>custody.progressive-security</x:v>
       </x:c>
       <x:c r="C59" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12790,21 +12990,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E59" s="32" t="str">
-        <x:v>The identifier split only exists because SegWit introduces a witness-inclusive serialization alongside the legacy serialization, so learners need the SegWit structure change before the two IDs make sense.</x:v>
+        <x:v>One of the core upgrade steps in the reference design is moving from default low-friction storage to an external signing device, so learners need the hardware-signing model before the staged-upgrade pattern makes sense.</x:v>
       </x:c>
       <x:c r="F59" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="G59" s="32" t="str">
-        <x:v>Direct parent keeps the bridge on the serialization distinction instead of reintroducing downstream relay consequences.</x:v>
+        <x:v>Direct edge captures the mid-tier upgrade target without treating cloud backup itself as the core concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="32" t="str">
-        <x:v>protocol.txid-vs-wtxid</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B60" s="32" t="str">
-        <x:v>protocol.wtxid-relay-bip339</x:v>
+        <x:v>custody.progressive-security</x:v>
       </x:c>
       <x:c r="C60" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12813,21 +13013,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E60" s="32" t="str">
-        <x:v>WTXID relay is specifically the choice to announce and request witness-bearing transactions by wtxid instead of txid, so the learner should understand the two identifier forms before the relay mode change.</x:v>
+        <x:v>The higher-security end of the progression moves into 2-of-3 and 3-of-5 multi-key schemes, so learners need the multisig model before they can reason about why and when a wallet should escalate there.</x:v>
       </x:c>
       <x:c r="F60" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="G60" s="32" t="str">
-        <x:v>Added as a graph bridge so the existing relay node no longer has to explain the identifier distinction internally.</x:v>
+        <x:v>Direct edge captures the high-assurance destination of the progression rather than a specific product flow.</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="32" t="str">
-        <x:v>fundamentals.schnorr-signatures</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="B61" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
       </x:c>
       <x:c r="C61" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12836,21 +13036,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E61" s="32" t="str">
-        <x:v>MuSig is a Schnorr aggregation protocol, so learners need the underlying Schnorr key and signature model before the combined-key protocol makes sense.</x:v>
+        <x:v>Rebroadcast privacy builds directly on the local-node distinction between transactions merely accepted into the mempool and transactions known to have propagated, which is exactly the gap the unbroadcast set tracks.</x:v>
       </x:c>
       <x:c r="F61" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G61" s="32" t="str">
-        <x:v>Direct parent kept narrow; wallet-level multisig and Taproot remain context rather than prerequisites.</x:v>
+        <x:v>Direct parent keeps the slice on the local tracking mechanism rather than reintroducing generic relay ancestors.</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B62" s="32" t="str">
-        <x:v>dev.descriptor-wallet-policies</x:v>
+        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
       </x:c>
       <x:c r="C62" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12859,21 +13059,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E62" s="32" t="str">
-        <x:v>Wallet policies are built as descriptor templates, so the base descriptor language and template structure must come first.</x:v>
+        <x:v>Different rebroadcast patterns matter because observers can correlate network behavior with public transaction history and infer likely origin, so learners need the pseudonymity and linkage problem first.</x:v>
       </x:c>
       <x:c r="F62" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G62" s="32" t="str">
-        <x:v>Direct parent kept above import or signer flows because the node is about the representation itself.</x:v>
+        <x:v>Direct parent keeps the node focused on why relay-side origin leakage matters, not just how rebroadcast code works.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="32" t="str">
-        <x:v>dev.bip32</x:v>
+        <x:v>protocol.segregated-witness</x:v>
       </x:c>
       <x:c r="B63" s="32" t="str">
-        <x:v>dev.descriptor-wallet-policies</x:v>
+        <x:v>protocol.txid-vs-wtxid</x:v>
       </x:c>
       <x:c r="C63" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12882,21 +13082,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E63" s="32" t="str">
-        <x:v>BIP388 key information items package xpubs and derivation origins, so learners need the HD derivation model before the portable wallet-policy format makes sense.</x:v>
+        <x:v>The identifier split only exists because SegWit introduces a witness-inclusive serialization alongside the legacy serialization, so learners need the SegWit structure change before the two IDs make sense.</x:v>
       </x:c>
       <x:c r="F63" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G63" s="32" t="str">
-        <x:v>Non-redundant alongside dev.descriptors because neither concept implies the other in the current graph.</x:v>
+        <x:v>Direct parent keeps the bridge on the serialization distinction instead of reintroducing downstream relay consequences.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>protocol.txid-vs-wtxid</x:v>
       </x:c>
       <x:c r="B64" s="32" t="str">
-        <x:v>dev.descriptors-in-psbt</x:v>
+        <x:v>protocol.wtxid-relay-bip339</x:v>
       </x:c>
       <x:c r="C64" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12905,21 +13105,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E64" s="32" t="str">
-        <x:v>The node is about carrying descriptor information during transaction coordination, so learners need the descriptor syntax and script-template model first.</x:v>
+        <x:v>WTXID relay is specifically the choice to announce and request witness-bearing transactions by wtxid instead of txid, so the learner should understand the two identifier forms before the relay mode change.</x:v>
       </x:c>
       <x:c r="F64" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G64" s="32" t="str">
-        <x:v>Direct parent kept at the representation layer rather than the wallet-policy or taproot-specific refinements.</x:v>
+        <x:v>Added as a graph bridge so the existing relay node no longer has to explain the identifier distinction internally.</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="32" t="str">
-        <x:v>custody.psbt</x:v>
+        <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="B65" s="32" t="str">
-        <x:v>dev.descriptors-in-psbt</x:v>
+        <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="C65" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12928,21 +13128,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E65" s="32" t="str">
-        <x:v>Descriptor-aware exchange only makes sense after the learner understands the general PSBT coordination workflow that transports signing-related data between tools.</x:v>
+        <x:v>MuSig is a Schnorr aggregation protocol, so learners need the underlying Schnorr key and signature model before the combined-key protocol makes sense.</x:v>
       </x:c>
       <x:c r="F65" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G65" s="32" t="str">
-        <x:v>Direct parent kept at the base PSBT workflow level instead of requiring later version-specific extensions.</x:v>
+        <x:v>Direct parent kept narrow; wallet-level multisig and Taproot remain context rather than prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B66" s="32" t="str">
-        <x:v>custody.degrading-multisig</x:v>
+        <x:v>dev.descriptor-wallet-policies</x:v>
       </x:c>
       <x:c r="C66" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12951,21 +13151,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E66" s="32" t="str">
-        <x:v>The policy only makes sense once the learner understands ordinary multisig threshold custody and why signers can be split into live and backup sets.</x:v>
+        <x:v>Wallet policies are built as descriptor templates, so the base descriptor language and template structure must come first.</x:v>
       </x:c>
       <x:c r="F66" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G66" s="32" t="str">
-        <x:v>Direct custody parent for the signer-threshold side of the construction.</x:v>
+        <x:v>Direct parent kept above import or signer flows because the node is about the representation itself.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="32" t="str">
-        <x:v>protocol.timelocks</x:v>
+        <x:v>dev.bip32</x:v>
       </x:c>
       <x:c r="B67" s="32" t="str">
-        <x:v>custody.degrading-multisig</x:v>
+        <x:v>dev.descriptor-wallet-policies</x:v>
       </x:c>
       <x:c r="C67" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12974,21 +13174,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E67" s="32" t="str">
-        <x:v>The degrading policy activates its weaker backup path only after a timeout, so timelock semantics are a direct part of the construction.</x:v>
+        <x:v>BIP388 key information items package xpubs and derivation origins, so learners need the HD derivation model before the portable wallet-policy format makes sense.</x:v>
       </x:c>
       <x:c r="F67" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G67" s="32" t="str">
-        <x:v>Needed alongside custody.multisig because the learner must understand the temporal rule, not just the signer policy.</x:v>
+        <x:v>Non-redundant alongside dev.descriptors because neither concept implies the other in the current graph.</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="32" t="str">
-        <x:v>protocol.block-weight-vbytes</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B68" s="32" t="str">
-        <x:v>protocol.fee-calculation</x:v>
+        <x:v>dev.descriptors-in-psbt</x:v>
       </x:c>
       <x:c r="C68" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12997,21 +13197,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E68" s="32" t="str">
-        <x:v>Understanding whether an absolute fee is high or low requires relating it to the blockspace pricing unit, so learners need weight and virtual bytes before fee calculation is fully meaningful in practice.</x:v>
+        <x:v>The node is about carrying descriptor information during transaction coordination, so learners need the descriptor syntax and script-template model first.</x:v>
       </x:c>
       <x:c r="F68" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G68" s="32" t="str">
-        <x:v>Direct parent keeps the node at the mechanism layer without drifting into broader fee-market competition.</x:v>
+        <x:v>Direct parent kept at the representation layer rather than the wallet-policy or taproot-specific refinements.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>custody.psbt</x:v>
       </x:c>
       <x:c r="B69" s="32" t="str">
-        <x:v>protocol.bech32m-addresses</x:v>
+        <x:v>dev.descriptors-in-psbt</x:v>
       </x:c>
       <x:c r="C69" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13020,21 +13220,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E69" s="32" t="str">
-        <x:v>Bech32m is an address-encoding format, so learners need the general relationship between addresses, script templates, and spendability before the newer checksum format is meaningful.</x:v>
+        <x:v>Descriptor-aware exchange only makes sense after the learner understands the general PSBT coordination workflow that transports signing-related data between tools.</x:v>
       </x:c>
       <x:c r="F69" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G69" s="32" t="str">
-        <x:v>Direct parent keeps the node on encoding semantics rather than on raw string-format trivia.</x:v>
+        <x:v>Direct parent kept at the base PSBT workflow level instead of requiring later version-specific extensions.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B70" s="32" t="str">
-        <x:v>protocol.bech32m-addresses</x:v>
+        <x:v>custody.degrading-multisig</x:v>
       </x:c>
       <x:c r="C70" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13043,21 +13243,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E70" s="32" t="str">
-        <x:v>Bech32m became necessary for witness version 1 and higher, and Taproot is the first major deployed witness-v1 use case, so learners need that upgrade context before the format distinction makes sense.</x:v>
+        <x:v>The policy only makes sense once the learner understands ordinary multisig threshold custody and why signers can be split into live and backup sets.</x:v>
       </x:c>
       <x:c r="F70" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G70" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored on the practical protocol transition that exposed Bech32m to users.</x:v>
+        <x:v>Direct custody parent for the signer-threshold side of the construction.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>protocol.timelocks</x:v>
       </x:c>
       <x:c r="B71" s="32" t="str">
-        <x:v>protocol.script-execution-stack</x:v>
+        <x:v>custody.degrading-multisig</x:v>
       </x:c>
       <x:c r="C71" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13066,21 +13266,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E71" s="32" t="str">
-        <x:v>The stack execution model is the direct mechanism by which Bitcoin Script evaluates spending conditions, so learners need the umbrella Script concept before drilling into stack behavior.</x:v>
+        <x:v>The degrading policy activates its weaker backup path only after a timeout, so timelock semantics are a direct part of the construction.</x:v>
       </x:c>
       <x:c r="F71" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G71" s="32" t="str">
-        <x:v>Direct parent positions the node as the conceptual middle layer between Script and opcode-specific leaves.</x:v>
+        <x:v>Needed alongside custody.multisig because the learner must understand the temporal rule, not just the signer policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="32" t="str">
-        <x:v>lightning.commitment-transactions</x:v>
+        <x:v>protocol.block-weight-vbytes</x:v>
       </x:c>
       <x:c r="B72" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>protocol.fee-calculation</x:v>
       </x:c>
       <x:c r="C72" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13089,21 +13289,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E72" s="32" t="str">
-        <x:v>Per-commitment secrets are generated for each new commitment state, so learners need the commitment-transaction model before the secret-rotation mechanism makes sense.</x:v>
+        <x:v>Understanding whether an absolute fee is high or low requires relating it to the blockspace pricing unit, so learners need weight and virtual bytes before fee calculation is fully meaningful in practice.</x:v>
       </x:c>
       <x:c r="F72" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G72" s="32" t="str">
-        <x:v>Direct parent keeps the node on state evolution rather than on later punishment or watchtower behavior.</x:v>
+        <x:v>Direct parent keeps the node at the mechanism layer without drifting into broader fee-market competition.</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B73" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>protocol.bech32m-addresses</x:v>
       </x:c>
       <x:c r="C73" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13112,21 +13312,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E73" s="32" t="str">
-        <x:v>The to_local and to_remote scripts rely on per-state key derivation, revocation keys, and delayed-payment keys, so learners need the per-commitment secret machinery first.</x:v>
+        <x:v>Bech32m is an address-encoding format, so learners need the general relationship between addresses, script templates, and spendability before the newer checksum format is meaningful.</x:v>
       </x:c>
       <x:c r="F73" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G73" s="32" t="str">
-        <x:v>Direct parent keeps the node at the commitment-key layer instead of collapsing back into the broader commitment-transaction overview.</x:v>
+        <x:v>Direct parent keeps the node on encoding semantics rather than on raw string-format trivia.</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="32" t="str">
-        <x:v>protocol.csv-bip112</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B74" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>protocol.bech32m-addresses</x:v>
       </x:c>
       <x:c r="C74" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13135,21 +13335,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E74" s="32" t="str">
-        <x:v>The delayed to_local branch is defined by a CSV-enforced waiting period, so learners need the relative-timelock opcode before the script template makes sense.</x:v>
+        <x:v>Bech32m became necessary for witness version 1 and higher, and Taproot is the first major deployed witness-v1 use case, so learners need that upgrade context before the format distinction makes sense.</x:v>
       </x:c>
       <x:c r="F74" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G74" s="32" t="str">
-        <x:v>Direct parent captures the script-mechanism side of the concept without dragging in broader force-close or HTLC timing behavior.</x:v>
+        <x:v>Direct parent keeps the node anchored on the practical protocol transition that exposed Bech32m to users.</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="32" t="str">
-        <x:v>protocol.difficulty-adjustment</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B75" s="32" t="str">
-        <x:v>protocol.time-warp-attack</x:v>
+        <x:v>protocol.script-execution-stack</x:v>
       </x:c>
       <x:c r="C75" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13158,21 +13358,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E75" s="32" t="str">
-        <x:v>The attack only makes sense once learners understand how Bitcoin retargets mining difficulty over long block windows.</x:v>
+        <x:v>The stack execution model is the direct mechanism by which Bitcoin Script evaluates spending conditions, so learners need the umbrella Script concept before drilling into stack behavior.</x:v>
       </x:c>
       <x:c r="F75" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G75" s="32" t="str">
-        <x:v>Direct parent keeps the exploit tied to the retarget mechanism instead of burying it under generic mining vocabulary.</x:v>
+        <x:v>Direct parent positions the node as the conceptual middle layer between Script and opcode-specific leaves.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="32" t="str">
-        <x:v>protocol.median-time-past</x:v>
+        <x:v>lightning.commitment-transactions</x:v>
       </x:c>
       <x:c r="B76" s="32" t="str">
-        <x:v>protocol.time-warp-attack</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="C76" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13181,21 +13381,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E76" s="32" t="str">
-        <x:v>Learners need the consensus timestamp constraints before they can reason about how miners manipulate time data and where the remaining attack surface lives.</x:v>
+        <x:v>Per-commitment secrets are generated for each new commitment state, so learners need the commitment-transaction model before the secret-rotation mechanism makes sense.</x:v>
       </x:c>
       <x:c r="F76" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G76" s="32" t="str">
-        <x:v>Direct parent captures the timestamp-boundary side of the exploit without overloading timelocks or block headers.</x:v>
+        <x:v>Direct parent keeps the node on state evolution rather than on later punishment or watchtower behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="32" t="str">
-        <x:v>fundamentals.blind-signatures</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="B77" s="32" t="str">
-        <x:v>history.chaumian-ecash</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="C77" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13204,21 +13404,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E77" s="32" t="str">
-        <x:v>Chaumian ecash is defined by using blind signatures to let a mint issue private bearer tokens without seeing the final token contents.</x:v>
+        <x:v>The to_local and to_remote scripts rely on per-state key derivation, revocation keys, and delayed-payment keys, so learners need the per-commitment secret machinery first.</x:v>
       </x:c>
       <x:c r="F77" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G77" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the specific cryptographic mechanism rather than treating it as generic digital-money history.</x:v>
+        <x:v>Direct parent keeps the node at the commitment-key layer instead of collapsing back into the broader commitment-transaction overview.</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="32" t="str">
-        <x:v>history.double-spend-problem</x:v>
+        <x:v>protocol.csv-bip112</x:v>
       </x:c>
       <x:c r="B78" s="32" t="str">
-        <x:v>history.chaumian-ecash</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="C78" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13227,21 +13427,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E78" s="32" t="str">
-        <x:v>Learners need the unsolved scarcity problem in digital cash before the trusted-mint tradeoff in Chaumian designs becomes meaningful.</x:v>
+        <x:v>The delayed to_local branch is defined by a CSV-enforced waiting period, so learners need the relative-timelock opcode before the script template makes sense.</x:v>
       </x:c>
       <x:c r="F78" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G78" s="32" t="str">
-        <x:v>Direct parent frames why the system still needed a central operator even though it improved privacy.</x:v>
+        <x:v>Direct parent captures the script-mechanism side of the concept without dragging in broader force-close or HTLC timing behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="32" t="str">
-        <x:v>economics.history-of-money</x:v>
+        <x:v>protocol.difficulty-adjustment</x:v>
       </x:c>
       <x:c r="B79" s="32" t="str">
-        <x:v>privacy.secret-right-to-cash</x:v>
+        <x:v>protocol.time-warp-attack</x:v>
       </x:c>
       <x:c r="C79" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13250,21 +13450,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E79" s="32" t="str">
-        <x:v>The concept depends on understanding how money moved from bearer cash toward mediated account systems, so learners need the long-run monetary history first.</x:v>
+        <x:v>The attack only makes sense once learners understand how Bitcoin retargets mining difficulty over long block windows.</x:v>
       </x:c>
       <x:c r="F79" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G79" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the bearer-versus-intermediated payment shift rather than drifting into generic civil-liberties framing.</x:v>
+        <x:v>Direct parent keeps the exploit tied to the retarget mechanism instead of burying it under generic mining vocabulary.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="32" t="str">
-        <x:v>fundamentals.censorship-resistance</x:v>
+        <x:v>protocol.median-time-past</x:v>
       </x:c>
       <x:c r="B80" s="32" t="str">
-        <x:v>privacy.secret-right-to-cash</x:v>
+        <x:v>protocol.time-warp-attack</x:v>
       </x:c>
       <x:c r="C80" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13273,21 +13473,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E80" s="32" t="str">
-        <x:v>Learners need the general idea that payment systems can exclude or block participants before the loss of private cash as a payment right becomes fully meaningful.</x:v>
+        <x:v>Learners need the consensus timestamp constraints before they can reason about how miners manipulate time data and where the remaining attack surface lives.</x:v>
       </x:c>
       <x:c r="F80" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G80" s="32" t="str">
-        <x:v>Direct parent captures the exclusion-risk side of the argument without reopening broader compliance or surveillance wrappers.</x:v>
+        <x:v>Direct parent captures the timestamp-boundary side of the exploit without overloading timelocks or block headers.</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="32" t="str">
-        <x:v>fundamentals.inflation</x:v>
+        <x:v>fundamentals.blind-signatures</x:v>
       </x:c>
       <x:c r="B81" s="32" t="str">
-        <x:v>economics.ideal-money</x:v>
+        <x:v>history.chaumian-ecash</x:v>
       </x:c>
       <x:c r="C81" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13296,21 +13496,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E81" s="32" t="str">
-        <x:v>The concept is about minimizing monetary distortion, so learners need to understand how inflation changes purchasing power and price signals first.</x:v>
+        <x:v>Chaumian ecash is defined by using blind signatures to let a mint issue private bearer tokens without seeing the final token contents.</x:v>
       </x:c>
       <x:c r="F81" s="32" t="str">
         <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G81" s="32" t="str">
-        <x:v>Direct parent captures the measurement-distortion problem that ideal money is trying to avoid.</x:v>
+        <x:v>Direct parent keeps the node tied to the specific cryptographic mechanism rather than treating it as generic digital-money history.</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>history.double-spend-problem</x:v>
       </x:c>
       <x:c r="B82" s="32" t="str">
-        <x:v>protocol.bitcoin-uri-bip21</x:v>
+        <x:v>history.chaumian-ecash</x:v>
       </x:c>
       <x:c r="C82" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13319,21 +13519,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E82" s="32" t="str">
-        <x:v>The URI is a wrapper around a payment destination and amount, so learners need the underlying address and output model first.</x:v>
+        <x:v>Learners need the unsolved scarcity problem in digital cash before the trusted-mint tradeoff in Chaumian designs becomes meaningful.</x:v>
       </x:c>
       <x:c r="F82" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G82" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the standard request format rather than collapsing it into higher-level wallet UX systems.</x:v>
+        <x:v>Direct parent frames why the system still needed a central operator even though it improved privacy.</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="32" t="str">
-        <x:v>dev.bip32</x:v>
+        <x:v>economics.history-of-money</x:v>
       </x:c>
       <x:c r="B83" s="32" t="str">
-        <x:v>dev.extended-keys</x:v>
+        <x:v>privacy.secret-right-to-cash</x:v>
       </x:c>
       <x:c r="C83" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13342,21 +13542,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E83" s="32" t="str">
-        <x:v>Extended keys are one specific export and branch-derivation surface inside the broader BIP32 HD tree model, so learners need the base tree-derivation mechanics first.</x:v>
+        <x:v>The concept depends on understanding how money moved from bearer cash toward mediated account systems, so learners need the long-run monetary history first.</x:v>
       </x:c>
       <x:c r="F83" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G83" s="32" t="str">
-        <x:v>Direct parent keeps the node inside the HD derivation branch instead of treating xpub or xprv behavior as only a privacy or operational-wallet concept.</x:v>
+        <x:v>Direct parent keeps the node tied to the bearer-versus-intermediated payment shift rather than drifting into generic civil-liberties framing.</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="32" t="str">
-        <x:v>dev.extended-keys</x:v>
+        <x:v>fundamentals.censorship-resistance</x:v>
       </x:c>
       <x:c r="B84" s="32" t="str">
-        <x:v>dev.hardened-keys</x:v>
+        <x:v>privacy.secret-right-to-cash</x:v>
       </x:c>
       <x:c r="C84" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13365,21 +13565,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E84" s="32" t="str">
-        <x:v>Hardened derivation is a constraint on what an extended public key can derive and on how extended private and public key boundaries behave, so learners need the base xpub/xprv model first.</x:v>
+        <x:v>Learners need the general idea that payment systems can exclude or block participants before the loss of private cash as a payment right becomes fully meaningful.</x:v>
       </x:c>
       <x:c r="F84" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G84" s="32" t="str">
-        <x:v>Direct parent closes the previously missing branch-level bridge between BIP32 generally and hardened derivation specifically.</x:v>
+        <x:v>Direct parent captures the exclusion-risk side of the argument without reopening broader compliance or surveillance wrappers.</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>fundamentals.inflation</x:v>
       </x:c>
       <x:c r="B85" s="32" t="str">
-        <x:v>protocol.escrow-and-arbitration</x:v>
+        <x:v>economics.ideal-money</x:v>
       </x:c>
       <x:c r="C85" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13388,21 +13588,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E85" s="32" t="str">
-        <x:v>The escrow flow depends on understanding how multiple signers can authorize one spend and why a 2-of-3 threshold changes trust assumptions between buyer, seller, and arbitrator.</x:v>
+        <x:v>The concept is about minimizing monetary distortion, so learners need to understand how inflation changes purchasing power and price signals first.</x:v>
       </x:c>
       <x:c r="F85" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G85" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the threshold-signing contract pattern instead of treating it as generic dispute-resolution theory.</x:v>
+        <x:v>Direct parent captures the measurement-distortion problem that ideal money is trying to avoid.</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="32" t="str">
-        <x:v>protocol.pay-to-script-hash</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B86" s="32" t="str">
-        <x:v>protocol.escrow-and-arbitration</x:v>
+        <x:v>protocol.bitcoin-uri-bip21</x:v>
       </x:c>
       <x:c r="C86" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13411,21 +13611,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E86" s="32" t="str">
-        <x:v>The contract uses a P2SH redeem script to hide the multisig spending conditions until spend time, so learners need the P2SH wrapper first.</x:v>
+        <x:v>The URI is a wrapper around a payment destination and amount, so learners need the underlying address and output model first.</x:v>
       </x:c>
       <x:c r="F86" s="32" t="str">
         <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G86" s="32" t="str">
-        <x:v>Direct parent captures the on-chain contract packaging layer that makes the escrow pattern practical.</x:v>
+        <x:v>Direct parent keeps the node tied to the standard request format rather than collapsing it into higher-level wallet UX systems.</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>dev.bip32</x:v>
       </x:c>
       <x:c r="B87" s="32" t="str">
-        <x:v>dev.wallet-import-format-wif</x:v>
+        <x:v>dev.extended-keys</x:v>
       </x:c>
       <x:c r="C87" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13434,21 +13634,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E87" s="32" t="str">
-        <x:v>WIF is a serialization format for one private key, so learners need the underlying asymmetric-key concept before the network prefix, checksum, and compression flag details make sense.</x:v>
+        <x:v>Extended keys are one specific export and branch-derivation surface inside the broader BIP32 HD tree model, so learners need the base tree-derivation mechanics first.</x:v>
       </x:c>
       <x:c r="F87" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G87" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored on key material itself instead of overfitting it to address formats or HD wallet hierarchies.</x:v>
+        <x:v>Direct parent keeps the node inside the HD derivation branch instead of treating xpub or xprv behavior as only a privacy or operational-wallet concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>dev.extended-keys</x:v>
       </x:c>
       <x:c r="B88" s="32" t="str">
-        <x:v>mining.pool-shares</x:v>
+        <x:v>dev.hardened-keys</x:v>
       </x:c>
       <x:c r="C88" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13457,21 +13657,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E88" s="32" t="str">
-        <x:v>Pool shares only make sense after learners understand why pooled mining exists and why miners need a lower-variance way to prove contributed work before an actual block is found.</x:v>
+        <x:v>Hardened derivation is a constraint on what an extended public key can derive and on how extended private and public key boundaries behave, so learners need the base xpub/xprv model first.</x:v>
       </x:c>
       <x:c r="F88" s="32" t="str">
         <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G88" s="32" t="str">
-        <x:v>Direct parent keeps the node at the pooled-mining accounting layer without adding redundant proof-of-work or difficulty edges.</x:v>
+        <x:v>Direct parent closes the previously missing branch-level bridge between BIP32 generally and hardened derivation specifically.</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B89" s="32" t="str">
-        <x:v>lightning.obscured-commitment-number</x:v>
+        <x:v>protocol.escrow-and-arbitration</x:v>
       </x:c>
       <x:c r="C89" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13480,21 +13680,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E89" s="32" t="str">
-        <x:v>The obscured commitment number is part of the same commitment-state machinery as the per-state secret chain, so learners need that state-derivation context before the field-level encoding scheme makes sense.</x:v>
+        <x:v>The escrow flow depends on understanding how multiple signers can authorize one spend and why a 2-of-3 threshold changes trust assumptions between buyer, seller, and arbitrator.</x:v>
       </x:c>
       <x:c r="F89" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G89" s="32" t="str">
-        <x:v>Direct parent keeps the node in the narrow commitment-state branch instead of pulling in broader closure or HTLC behavior.</x:v>
+        <x:v>Direct parent keeps the node tied to the threshold-signing contract pattern instead of treating it as generic dispute-resolution theory.</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="32" t="str">
-        <x:v>lightning.htlc</x:v>
+        <x:v>protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="B90" s="32" t="str">
-        <x:v>lightning.htlc-output-scripts</x:v>
+        <x:v>protocol.escrow-and-arbitration</x:v>
       </x:c>
       <x:c r="C90" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13503,21 +13703,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E90" s="32" t="str">
-        <x:v>Learners need the base HTLC idea before the offered and received witness-script branches, timeout paths, and preimage-claim paths become meaningful.</x:v>
+        <x:v>The contract uses a P2SH redeem script to hide the multisig spending conditions until spend time, so learners need the P2SH wrapper first.</x:v>
       </x:c>
       <x:c r="F90" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G90" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the payment-contract primitive instead of treating it as generic script trivia.</x:v>
+        <x:v>Direct parent captures the on-chain contract packaging layer that makes the escrow pattern practical.</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B91" s="32" t="str">
-        <x:v>lightning.htlc-output-scripts</x:v>
+        <x:v>dev.wallet-import-format-wif</x:v>
       </x:c>
       <x:c r="C91" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13526,21 +13726,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E91" s="32" t="str">
-        <x:v>HTLC output scripts are additional commitment-transaction outputs layered on top of the same to_local and to_remote commitment-script structure, so learners need that earlier script layer first.</x:v>
+        <x:v>WIF is a serialization format for one private key, so learners need the underlying asymmetric-key concept before the network prefix, checksum, and compression flag details make sense.</x:v>
       </x:c>
       <x:c r="F91" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G91" s="32" t="str">
-        <x:v>Direct parent places the node at the next script layer above commitment outputs without dragging in later close-handling or watchtower flows.</x:v>
+        <x:v>Direct parent keeps the node anchored on key material itself instead of overfitting it to address formats or HD wallet hierarchies.</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="32" t="str">
-        <x:v>protocol.coinbase-transaction</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B92" s="32" t="str">
-        <x:v>protocol.duplicate-transaction-bug</x:v>
+        <x:v>mining.pool-shares</x:v>
       </x:c>
       <x:c r="C92" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13549,21 +13749,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E92" s="32" t="str">
-        <x:v>The bug is historically tied to duplicated coinbase transactions, so learners need the special structure and validation role of coinbase transactions before the replay vector makes sense.</x:v>
+        <x:v>Pool shares only make sense after learners understand why pooled mining exists and why miners need a lower-variance way to prove contributed work before an actual block is found.</x:v>
       </x:c>
       <x:c r="F92" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G92" s="32" t="str">
-        <x:v>Direct parent keeps the bug tied to the early-coinbase uniqueness failure instead of burying it under general mining history.</x:v>
+        <x:v>Direct parent keeps the node at the pooled-mining accounting layer without adding redundant proof-of-work or difficulty edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="32" t="str">
-        <x:v>protocol.utxo-model</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="B93" s="32" t="str">
-        <x:v>protocol.duplicate-transaction-bug</x:v>
+        <x:v>lightning.obscured-commitment-number</x:v>
       </x:c>
       <x:c r="C93" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13572,21 +13772,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E93" s="32" t="str">
-        <x:v>Learners need the txid-plus-output-index reference model to understand why identical transaction ids could confuse later spends and overwrite assumptions in the UTXO set.</x:v>
+        <x:v>The obscured commitment number is part of the same commitment-state machinery as the per-state secret chain, so learners need that state-derivation context before the field-level encoding scheme makes sense.</x:v>
       </x:c>
       <x:c r="F93" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G93" s="32" t="str">
-        <x:v>Direct parent captures the reference-model side of the bug without conflating it with double-spend history or malleability.</x:v>
+        <x:v>Direct parent keeps the node in the narrow commitment-state branch instead of pulling in broader closure or HTLC behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="32" t="str">
-        <x:v>protocol.block-structure</x:v>
+        <x:v>lightning.htlc</x:v>
       </x:c>
       <x:c r="B94" s="32" t="str">
-        <x:v>protocol.64-byte-transaction-bug</x:v>
+        <x:v>lightning.htlc-output-scripts</x:v>
       </x:c>
       <x:c r="C94" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13595,21 +13795,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E94" s="32" t="str">
-        <x:v>The bug only makes sense once learners understand how transaction hashes sit inside the block merkle tree and why internal-node preimages matter for block commitments.</x:v>
+        <x:v>Learners need the base HTLC idea before the offered and received witness-script branches, timeout paths, and preimage-claim paths become meaningful.</x:v>
       </x:c>
       <x:c r="F94" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G94" s="32" t="str">
-        <x:v>One direct parent keeps the node at the block-commitment layer instead of reopening broader hashing or SPV overview branches.</x:v>
+        <x:v>Direct parent keeps the node tied to the payment-contract primitive instead of treating it as generic script trivia.</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="32" t="str">
-        <x:v>fundamentals.digital-signatures</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="B95" s="32" t="str">
-        <x:v>fundamentals.lamport-signatures</x:v>
+        <x:v>lightning.htlc-output-scripts</x:v>
       </x:c>
       <x:c r="C95" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13618,21 +13818,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E95" s="32" t="str">
-        <x:v>Learners need the general signing-and-verification mental model before the one-time Lamport construction and its tradeoffs become meaningful.</x:v>
+        <x:v>HTLC output scripts are additional commitment-transaction outputs layered on top of the same to_local and to_remote commitment-script structure, so learners need that earlier script layer first.</x:v>
       </x:c>
       <x:c r="F95" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G95" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to signature semantics instead of treating it as only a post-quantum curiosity.</x:v>
+        <x:v>Direct parent places the node at the next script layer above commitment outputs without dragging in later close-handling or watchtower flows.</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>protocol.coinbase-transaction</x:v>
       </x:c>
       <x:c r="B96" s="32" t="str">
-        <x:v>fundamentals.lamport-signatures</x:v>
+        <x:v>protocol.duplicate-transaction-bug</x:v>
       </x:c>
       <x:c r="C96" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13641,21 +13841,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E96" s="32" t="str">
-        <x:v>Lamport signatures replace elliptic-curve arithmetic with one-way hash preimages and comparisons, so learners need the hash primitive first.</x:v>
+        <x:v>The bug is historically tied to duplicated coinbase transactions, so learners need the special structure and validation role of coinbase transactions before the replay vector makes sense.</x:v>
       </x:c>
       <x:c r="F96" s="32" t="str">
         <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G96" s="32" t="str">
-        <x:v>Direct parent captures the actual cryptographic mechanism rather than forcing learners through unrelated elliptic-curve details.</x:v>
+        <x:v>Direct parent keeps the bug tied to the early-coinbase uniqueness failure instead of burying it under general mining history.</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="32" t="str">
-        <x:v>custody.backups-recovery</x:v>
+        <x:v>protocol.utxo-model</x:v>
       </x:c>
       <x:c r="B97" s="32" t="str">
-        <x:v>custody.shamirs-secret-sharing</x:v>
+        <x:v>protocol.duplicate-transaction-bug</x:v>
       </x:c>
       <x:c r="C97" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13664,21 +13864,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E97" s="32" t="str">
-        <x:v>In Bitcoin practice the scheme is used as one backup-and-recovery method, so learners need the broader custody problem before the threshold-share design choice becomes meaningful.</x:v>
+        <x:v>Learners need the txid-plus-output-index reference model to understand why identical transaction ids could confuse later spends and overwrite assumptions in the UTXO set.</x:v>
       </x:c>
       <x:c r="F97" s="32" t="str">
         <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G97" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored in practical custody use instead of drifting into a purely abstract cryptography topic.</x:v>
+        <x:v>Direct parent captures the reference-model side of the bug without conflating it with double-spend history or malleability.</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="32" t="str">
-        <x:v>protocol.segregated-witness</x:v>
+        <x:v>protocol.block-structure</x:v>
       </x:c>
       <x:c r="B98" s="32" t="str">
-        <x:v>protocol.witness-structure</x:v>
+        <x:v>protocol.64-byte-transaction-bug</x:v>
       </x:c>
       <x:c r="C98" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13687,21 +13887,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E98" s="32" t="str">
-        <x:v>The transaction witness layout only makes sense after the learner understands that SegWit separates witness data from the legacy transaction serialization.</x:v>
+        <x:v>The bug only makes sense once learners understand how transaction hashes sit inside the block merkle tree and why internal-node preimages matter for block commitments.</x:v>
       </x:c>
       <x:c r="F98" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G98" s="32" t="str">
-        <x:v>Direct edge keeps the node at the transaction-format layer; TXID/WTXID and witness-commitment consequences remain downstream concepts.</x:v>
+        <x:v>One direct parent keeps the node at the block-commitment layer instead of reopening broader hashing or SPV overview branches.</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="32" t="str">
-        <x:v>protocol.block-structure</x:v>
+        <x:v>fundamentals.digital-signatures</x:v>
       </x:c>
       <x:c r="B99" s="32" t="str">
-        <x:v>protocol.partial-merkle-proofs</x:v>
+        <x:v>fundamentals.lamport-signatures</x:v>
       </x:c>
       <x:c r="C99" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13710,21 +13910,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E99" s="32" t="str">
-        <x:v>Partial Merkle proofs reconstruct a transaction's inclusion path against the Merkle root carried by a block, so learners need block composition and root placement first.</x:v>
+        <x:v>Learners need the general signing-and-verification mental model before the one-time Lamport construction and its tradeoffs become meaningful.</x:v>
       </x:c>
       <x:c r="F99" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G99" s="32" t="str">
-        <x:v>The block-structure parent already inherits fundamentals.merkle-trees, avoiding a redundant direct edge.</x:v>
+        <x:v>Direct parent keeps the node tied to signature semantics instead of treating it as only a post-quantum curiosity.</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="32" t="str">
-        <x:v>dev.bips-process</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B100" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>fundamentals.lamport-signatures</x:v>
       </x:c>
       <x:c r="C100" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13733,21 +13933,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E100" s="32" t="str">
-        <x:v>Review culture is applied throughout the proposal and implementation lifecycle, so learners need to understand the process in which Bitcoin changes are proposed and evaluated.</x:v>
+        <x:v>Lamport signatures replace elliptic-curve arithmetic with one-way hash preimages and comparisons, so learners need the hash primitive first.</x:v>
       </x:c>
       <x:c r="F100" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G100" s="32" t="str">
-        <x:v>Direct edge supplies the development-lifecycle context without adding downstream release or deployment details.</x:v>
+        <x:v>Direct parent captures the actual cryptographic mechanism rather than forcing learners through unrelated elliptic-curve details.</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="32" t="str">
-        <x:v>security.adversarial-thinking</x:v>
+        <x:v>custody.backups-recovery</x:v>
       </x:c>
       <x:c r="B101" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>custody.shamirs-secret-sharing</x:v>
       </x:c>
       <x:c r="C101" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13756,21 +13956,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E101" s="32" t="str">
-        <x:v>Independent review in Bitcoin is deliberately adversarial: reviewers look for correctness failures, attack paths, and compatibility hazards before changes are merged.</x:v>
+        <x:v>In Bitcoin practice the scheme is used as one backup-and-recovery method, so learners need the broader custody problem before the threshold-share design choice becomes meaningful.</x:v>
       </x:c>
       <x:c r="F101" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G101" s="32" t="str">
-        <x:v>Direct edge keeps review distinct from responsible disclosure and reproducible-build verification, which are specialized downstream safeguards.</x:v>
+        <x:v>Direct parent keeps the node anchored in practical custody use instead of drifting into a purely abstract cryptography topic.</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="32" t="str">
-        <x:v>lightning.gossip-protocol</x:v>
+        <x:v>protocol.segregated-witness</x:v>
       </x:c>
       <x:c r="B102" s="32" t="str">
-        <x:v>lightning.feature-flags</x:v>
+        <x:v>protocol.witness-structure</x:v>
       </x:c>
       <x:c r="C102" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13779,21 +13979,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E102" s="32" t="str">
-        <x:v>Feature negotiation is used to advertise and interpret capabilities across Lightning peers and network announcements, so learners need the surrounding gossip and announcement context first.</x:v>
+        <x:v>The transaction witness layout only makes sense after the learner understands that SegWit separates witness data from the legacy transaction serialization.</x:v>
       </x:c>
       <x:c r="F102" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G102" s="32" t="str">
-        <x:v>Direct edge keeps the feature-bit mechanism distinct from the lower-level message transport and downstream routing protocols.</x:v>
+        <x:v>Direct edge keeps the node at the transaction-format layer; TXID/WTXID and witness-commitment consequences remain downstream concepts.</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="32" t="str">
-        <x:v>lightning.feature-flags</x:v>
+        <x:v>protocol.block-structure</x:v>
       </x:c>
       <x:c r="B103" s="32" t="str">
-        <x:v>lightning.onion-messages</x:v>
+        <x:v>protocol.partial-merkle-proofs</x:v>
       </x:c>
       <x:c r="C103" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13802,21 +14002,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E103" s="32" t="str">
-        <x:v>Peers use a negotiated feature bit to advertise whether they can send and forward onion messages, so learners need the capability-negotiation model first.</x:v>
+        <x:v>Partial Merkle proofs reconstruct a transaction's inclusion path against the Merkle root carried by a block, so learners need block composition and root placement first.</x:v>
       </x:c>
       <x:c r="F103" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G103" s="32" t="str">
-        <x:v>Direct edge keeps the feature gate separate from the message forwarding mechanism.</x:v>
+        <x:v>The block-structure parent already inherits fundamentals.merkle-trees, avoiding a redundant direct edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="32" t="str">
-        <x:v>lightning.route-blinding</x:v>
+        <x:v>dev.bips-process</x:v>
       </x:c>
       <x:c r="B104" s="32" t="str">
-        <x:v>lightning.onion-messages</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="C104" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13825,21 +14025,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E104" s="32" t="str">
-        <x:v>Onion messages use blinded paths to forward channel-independent payloads without exposing the final destination topology, so the route-blinding model must come first.</x:v>
+        <x:v>Review culture is applied throughout the proposal and implementation lifecycle, so learners need to understand the process in which Bitcoin changes are proposed and evaluated.</x:v>
       </x:c>
       <x:c r="F104" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G104" s="32" t="str">
-        <x:v>Payment onion routing and BOLT12 offers remain related sibling or downstream concepts rather than direct prerequisites.</x:v>
+        <x:v>Direct edge supplies the development-lifecycle context without adding downstream release or deployment details.</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>security.adversarial-thinking</x:v>
       </x:c>
       <x:c r="B105" s="32" t="str">
-        <x:v>lightning.encrypted-authenticated-transport</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="C105" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13848,21 +14048,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E105" s="32" t="str">
-        <x:v>The Noise_XK handshake authenticates long-term Lightning node identities with public/private key material, so learners need that identity model first.</x:v>
+        <x:v>Independent review in Bitcoin is deliberately adversarial: reviewers look for correctness failures, attack paths, and compatibility hazards before changes are merged.</x:v>
       </x:c>
       <x:c r="F105" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G105" s="32" t="str">
-        <x:v>Direct edge keeps identity foundations separate from the session-key derivation mechanism.</x:v>
+        <x:v>Direct edge keeps review distinct from responsible disclosure and reproducible-build verification, which are specialized downstream safeguards.</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="32" t="str">
-        <x:v>fundamentals.diffie-hellman-key-exchange</x:v>
+        <x:v>lightning.gossip-protocol</x:v>
       </x:c>
       <x:c r="B106" s="32" t="str">
-        <x:v>lightning.encrypted-authenticated-transport</x:v>
+        <x:v>lightning.feature-flags</x:v>
       </x:c>
       <x:c r="C106" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13871,21 +14071,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E106" s="32" t="str">
-        <x:v>BOLT 08 uses elliptic-curve Diffie-Hellman operations to derive shared session secrets, so the key-exchange primitive must be understood first.</x:v>
+        <x:v>Feature negotiation is used to advertise and interpret capabilities across Lightning peers and network announcements, so learners need the surrounding gossip and announcement context first.</x:v>
       </x:c>
       <x:c r="F106" s="32" t="str">
         <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G106" s="32" t="str">
-        <x:v>Bitcoin P2P v2 transport remains a related sibling rather than a direct prerequisite because it is a different protocol context.</x:v>
+        <x:v>Direct edge keeps the feature-bit mechanism distinct from the lower-level message transport and downstream routing protocols.</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>lightning.feature-flags</x:v>
       </x:c>
       <x:c r="B107" s="32" t="str">
-        <x:v>protocol.strict-der-signatures</x:v>
+        <x:v>lightning.onion-messages</x:v>
       </x:c>
       <x:c r="C107" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13894,21 +14094,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E107" s="32" t="str">
-        <x:v>Strict DER enforcement occurs while Script validates an ECDSA signature, so learners need the spending-condition and interpreter context first.</x:v>
+        <x:v>Peers use a negotiated feature bit to advertise whether they can send and forward onion messages, so learners need the capability-negotiation model first.</x:v>
       </x:c>
       <x:c r="F107" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G107" s="32" t="str">
-        <x:v>Direct edge keeps the rule at the script-validation layer rather than treating BIP 66 as a broad historical upgrade topic.</x:v>
+        <x:v>Direct edge keeps the feature gate separate from the message forwarding mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>lightning.route-blinding</x:v>
       </x:c>
       <x:c r="B108" s="32" t="str">
-        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+        <x:v>lightning.onion-messages</x:v>
       </x:c>
       <x:c r="C108" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13917,21 +14117,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E108" s="32" t="str">
-        <x:v>The node builds on the wallet-level threshold signer policy before specifying a deterministic ordering convention for the signer keys.</x:v>
+        <x:v>Onion messages use blinded paths to forward channel-independent payloads without exposing the final destination topology, so the route-blinding model must come first.</x:v>
       </x:c>
       <x:c r="F108" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G108" s="32" t="str">
-        <x:v>Direct edge preserves the distinction between multisig policy and the BIP 67 interoperability rule.</x:v>
+        <x:v>Payment onion routing and BOLT12 offers remain related sibling or downstream concepts rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="32" t="str">
-        <x:v>protocol.pay-to-script-hash</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B109" s="32" t="str">
-        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+        <x:v>lightning.encrypted-authenticated-transport</x:v>
       </x:c>
       <x:c r="C109" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13940,21 +14140,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E109" s="32" t="str">
-        <x:v>BIP 67 is commonly applied when constructing the redeem script whose hash is committed by P2SH, so the script-hash wrapper provides the output context.</x:v>
+        <x:v>The Noise_XK handshake authenticates long-term Lightning node identities with public/private key material, so learners need that identity model first.</x:v>
       </x:c>
       <x:c r="F109" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G109" s="32" t="str">
-        <x:v>The shared protocol.script ancestor remains inherited rather than a redundant direct edge.</x:v>
+        <x:v>Direct edge keeps identity foundations separate from the session-key derivation mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="32" t="str">
-        <x:v>ops.mempool-policy</x:v>
+        <x:v>fundamentals.diffie-hellman-key-exchange</x:v>
       </x:c>
       <x:c r="B110" s="32" t="str">
-        <x:v>ops.mempool-purging</x:v>
+        <x:v>lightning.encrypted-authenticated-transport</x:v>
       </x:c>
       <x:c r="C110" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13963,13 +14163,13 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E110" s="32" t="str">
-        <x:v>Rolling minimum fee escalation and transaction eviction are local consequences of the node's mempool relay policy, so learners need that policy boundary first.</x:v>
+        <x:v>BOLT 08 uses elliptic-curve Diffie-Hellman operations to derive shared session secrets, so the key-exchange primitive must be understood first.</x:v>
       </x:c>
       <x:c r="F110" s="32" t="str">
-        <x:v>source.mempool-space-docs</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G110" s="32" t="str">
-        <x:v>The generic mempool, fee-market, and consensus-policy branches remain inherited or adjacent rather than direct prerequisites.</x:v>
+        <x:v>Bitcoin P2P v2 transport remains a related sibling rather than a direct prerequisite because it is a different protocol context.</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
@@ -13977,7 +14177,7 @@
         <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B111" s="32" t="str">
-        <x:v>protocol.generic-signed-messages</x:v>
+        <x:v>protocol.strict-der-signatures</x:v>
       </x:c>
       <x:c r="C111" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13986,21 +14186,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E111" s="32" t="str">
-        <x:v>BIP 322 proves message authorization by constructing virtual transactions that satisfy a Bitcoin output script, so learners need the Script spending-condition model first.</x:v>
+        <x:v>Strict DER enforcement occurs while Script validates an ECDSA signature, so learners need the spending-condition and interpreter context first.</x:v>
       </x:c>
       <x:c r="F111" s="32" t="str">
         <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G111" s="32" t="str">
-        <x:v>The digital-signature path is inherited through Script; PSBT, Schnorr, and Taproot remain related variants rather than redundant direct edges.</x:v>
+        <x:v>Direct edge keeps the rule at the script-validation layer rather than treating BIP 66 as a broad historical upgrade topic.</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="32" t="str">
-        <x:v>dev.bitcoin-core-rpc</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B112" s="32" t="str">
-        <x:v>security.bitcoin-core-rpc-access</x:v>
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
       </x:c>
       <x:c r="C112" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14009,21 +14209,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E112" s="32" t="str">
-        <x:v>RPC access security is the control boundary around Bitcoin Core's programmatic interface, so learners need to understand the interface and its authority before securing exposure to it.</x:v>
+        <x:v>The node builds on the wallet-level threshold signer policy before specifying a deterministic ordering convention for the signer keys.</x:v>
       </x:c>
       <x:c r="F112" s="32" t="str">
-        <x:v>source.bitcoin-core-operator-docs</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G112" s="32" t="str">
-        <x:v>Full-node operation is inherited through dev.bitcoin-core-rpc; wallet RPC and transaction-preflight nodes remain downstream use cases rather than direct parents.</x:v>
+        <x:v>Direct edge preserves the distinction between multisig policy and the BIP 67 interoperability rule.</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="32" t="str">
-        <x:v>dev.testmempoolaccept-rpc</x:v>
+        <x:v>protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="B113" s="32" t="str">
-        <x:v>dev.submitpackage-rpc</x:v>
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
       </x:c>
       <x:c r="C113" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14032,21 +14232,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E113" s="32" t="str">
-        <x:v>submitpackage is the admission counterpart to the existing testmempoolaccept preflight workflow, so learners need to understand local package checks before attempting submission and interpreting package results.</x:v>
+        <x:v>BIP 67 is commonly applied when constructing the redeem script whose hash is committed by P2SH, so the script-hash wrapper provides the output context.</x:v>
       </x:c>
       <x:c r="F113" s="32" t="str">
-        <x:v>source.bitcoin-core-package-policy</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G113" s="32" t="str">
-        <x:v>Package relay and cluster mempool remain neighboring concepts rather than direct prerequisites because this node focuses on one local RPC operation.</x:v>
+        <x:v>The shared protocol.script ancestor remains inherited rather than a redundant direct edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="32" t="str">
-        <x:v>protocol.rbf</x:v>
+        <x:v>ops.mempool-policy</x:v>
       </x:c>
       <x:c r="B114" s="32" t="str">
-        <x:v>protocol.package-rbf</x:v>
+        <x:v>ops.mempool-purging</x:v>
       </x:c>
       <x:c r="C114" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14055,21 +14255,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E114" s="32" t="str">
-        <x:v>Package RBF extends the ordinary replacement-policy model with package-level fee and cluster conditions, so learners need base RBF semantics first.</x:v>
+        <x:v>Rolling minimum fee escalation and transaction eviction are local consequences of the node's mempool relay policy, so learners need that policy boundary first.</x:v>
       </x:c>
       <x:c r="F114" s="32" t="str">
-        <x:v>source.bitcoin-core-package-policy</x:v>
+        <x:v>source.mempool-space-docs</x:v>
       </x:c>
       <x:c r="G114" s="32" t="str">
-        <x:v>Package relay, cluster mempool, submitpackage, and pinning remain adjacent concepts rather than redundant direct edges.</x:v>
+        <x:v>The generic mempool, fee-market, and consensus-policy branches remain inherited or adjacent rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="32" t="str">
-        <x:v>protocol.cluster-mempool</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B115" s="32" t="str">
-        <x:v>ops.mempool-cluster-limits</x:v>
+        <x:v>protocol.generic-signed-messages</x:v>
       </x:c>
       <x:c r="C115" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14078,21 +14278,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E115" s="32" t="str">
-        <x:v>Cluster limits bound connected transaction sets, so learners need the cluster-mempool model before understanding why count and aggregate virtual-size limits replace legacy ancestor/descendant limits.</x:v>
+        <x:v>BIP 322 proves message authorization by constructing virtual transactions that satisfy a Bitcoin output script, so learners need the Script spending-condition model first.</x:v>
       </x:c>
       <x:c r="F115" s="32" t="str">
-        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G115" s="32" t="str">
-        <x:v>Package relay, Package RBF, CPFP, and version 3 relay remain affected workflows or neighboring policy mechanisms rather than direct prerequisites.</x:v>
+        <x:v>The digital-signature path is inherited through Script; PSBT, Schnorr, and Taproot remain related variants rather than redundant direct edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="32" t="str">
-        <x:v>ops.dns-seeds</x:v>
+        <x:v>dev.bitcoin-core-rpc</x:v>
       </x:c>
       <x:c r="B116" s="32" t="str">
-        <x:v>lightning.dns-seeds</x:v>
+        <x:v>security.bitcoin-core-rpc-access</x:v>
       </x:c>
       <x:c r="C116" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14101,21 +14301,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E116" s="32" t="str">
-        <x:v>Lightning DNS seeds specialize the general DNS bootstrap pattern with Lightning-specific query filters and known-peer lookup, so learners need the base DNS-seed model first.</x:v>
+        <x:v>RPC access security is the control boundary around Bitcoin Core's programmatic interface, so learners need to understand the interface and its authority before securing exposure to it.</x:v>
       </x:c>
       <x:c r="F116" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-core-operator-docs</x:v>
       </x:c>
       <x:c r="G116" s="32" t="str">
-        <x:v>Peer discovery is inherited through ops.dns-seeds; generic Bitcoin P2P bootstrapping remains a parent concept rather than a duplicated edge.</x:v>
+        <x:v>Full-node operation is inherited through dev.bitcoin-core-rpc; wallet RPC and transaction-preflight nodes remain downstream use cases rather than direct parents.</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="32" t="str">
-        <x:v>lightning.gossip-protocol</x:v>
+        <x:v>dev.testmempoolaccept-rpc</x:v>
       </x:c>
       <x:c r="B117" s="32" t="str">
-        <x:v>lightning.dns-seeds</x:v>
+        <x:v>dev.submitpackage-rpc</x:v>
       </x:c>
       <x:c r="C117" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14124,21 +14324,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E117" s="32" t="str">
-        <x:v>BOLT 10 locates Lightning peers and filters results by Lightning address information, so learners need Lightning's node-discovery and gossip context before understanding the assisted-location mechanism.</x:v>
+        <x:v>submitpackage is the admission counterpart to the existing testmempoolaccept preflight workflow, so learners need to understand local package checks before attempting submission and interpreting package results.</x:v>
       </x:c>
       <x:c r="F117" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-core-package-policy</x:v>
       </x:c>
       <x:c r="G117" s="32" t="str">
-        <x:v>Lightning routing and generic P2P messages are inherited through gossip rather than added as transitive prerequisites.</x:v>
+        <x:v>Package relay and cluster mempool remain neighboring concepts rather than direct prerequisites because this node focuses on one local RPC operation.</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="32" t="str">
-        <x:v>lightning.payment-channels</x:v>
+        <x:v>protocol.rbf</x:v>
       </x:c>
       <x:c r="B118" s="32" t="str">
-        <x:v>lightning.short-channel-id</x:v>
+        <x:v>protocol.package-rbf</x:v>
       </x:c>
       <x:c r="C118" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14147,21 +14347,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E118" s="32" t="str">
-        <x:v>The identifier names a Lightning channel's on-chain funding output, so learners need the channel and funding relationship first.</x:v>
+        <x:v>Package RBF extends the ordinary replacement-policy model with package-level fee and cluster conditions, so learners need base RBF semantics first.</x:v>
       </x:c>
       <x:c r="F118" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-core-package-policy</x:v>
       </x:c>
       <x:c r="G118" s="32" t="str">
-        <x:v>Direct channel context; the gossip protocol is a downstream consumer rather than a prerequisite.</x:v>
+        <x:v>Package relay, cluster mempool, submitpackage, and pinning remain adjacent concepts rather than redundant direct edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="32" t="str">
-        <x:v>protocol.block-height</x:v>
+        <x:v>protocol.cluster-mempool</x:v>
       </x:c>
       <x:c r="B119" s="32" t="str">
-        <x:v>lightning.short-channel-id</x:v>
+        <x:v>ops.mempool-cluster-limits</x:v>
       </x:c>
       <x:c r="C119" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14170,21 +14370,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E119" s="32" t="str">
-        <x:v>Short Channel IDs encode block height as their first component, so learners need the block-height concept before decoding the identifier.</x:v>
+        <x:v>Cluster limits bound connected transaction sets, so learners need the cluster-mempool model before understanding why count and aggregate virtual-size limits replace legacy ancestor/descendant limits.</x:v>
       </x:c>
       <x:c r="F119" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
       </x:c>
       <x:c r="G119" s="32" t="str">
-        <x:v>The transaction-index and output-index components remain part of the identifier's own outcome rather than extra transitive edges.</x:v>
+        <x:v>Package relay, Package RBF, CPFP, and version 3 relay remain affected workflows or neighboring policy mechanisms rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="32" t="str">
-        <x:v>protocol.nodes-vs-miners</x:v>
+        <x:v>ops.dns-seeds</x:v>
       </x:c>
       <x:c r="B120" s="32" t="str">
-        <x:v>mining.miner-decentralization</x:v>
+        <x:v>lightning.dns-seeds</x:v>
       </x:c>
       <x:c r="C120" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14193,21 +14393,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E120" s="32" t="str">
-        <x:v>Miner decentralization only makes sense once learners distinguish miners' transaction-ordering role from full nodes' independent enforcement of consensus validity.</x:v>
+        <x:v>Lightning DNS seeds specialize the general DNS bootstrap pattern with Lightning-specific query filters and known-peer lookup, so learners need the base DNS-seed model first.</x:v>
       </x:c>
       <x:c r="F120" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G120" s="32" t="str">
-        <x:v>The edge keeps censorship power separate from authority to change consensus rules.</x:v>
+        <x:v>Peer discovery is inherited through ops.dns-seeds; generic Bitcoin P2P bootstrapping remains a parent concept rather than a duplicated edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>lightning.gossip-protocol</x:v>
       </x:c>
       <x:c r="B121" s="32" t="str">
-        <x:v>mining.miner-decentralization</x:v>
+        <x:v>lightning.dns-seeds</x:v>
       </x:c>
       <x:c r="C121" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14216,21 +14416,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E121" s="32" t="str">
-        <x:v>Pool and solo mining explain the participant and coordination structure whose concentration or dispersion determines practical control over transaction ordering.</x:v>
+        <x:v>BOLT 10 locates Lightning peers and filters results by Lightning address information, so learners need Lightning's node-discovery and gossip context before understanding the assisted-location mechanism.</x:v>
       </x:c>
       <x:c r="F121" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G121" s="32" t="str">
-        <x:v>Stratum V2 remains optional implementation context, not a direct prerequisite.</x:v>
+        <x:v>Lightning routing and generic P2P messages are inherited through gossip rather than added as transitive prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>lightning.payment-channels</x:v>
       </x:c>
       <x:c r="B122" s="32" t="str">
-        <x:v>dev.selection-cryptography</x:v>
+        <x:v>lightning.short-channel-id</x:v>
       </x:c>
       <x:c r="C122" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14239,21 +14439,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E122" s="32" t="str">
-        <x:v>Selection cryptography evaluates cryptographic tools and dependencies through evidence, testing, authorship, and review quality, so learners need the broader Bitcoin review discipline first.</x:v>
+        <x:v>The identifier names a Lightning channel's on-chain funding output, so learners need the channel and funding relationship first.</x:v>
       </x:c>
       <x:c r="F122" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G122" s="32" t="str">
-        <x:v>Adversarial thinking is inherited through dev.review-culture; reproducible builds are a downstream verification practice rather than a prerequisite.</x:v>
+        <x:v>Direct channel context; the gossip protocol is a downstream consumer rather than a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="32" t="str">
-        <x:v>mining.pool-shares</x:v>
+        <x:v>protocol.block-height</x:v>
       </x:c>
       <x:c r="B123" s="32" t="str">
-        <x:v>mining.block-withholding</x:v>
+        <x:v>lightning.short-channel-id</x:v>
       </x:c>
       <x:c r="C123" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14262,21 +14462,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E123" s="32" t="str">
-        <x:v>Block withholding exploits the difference between a pool-paid share and a share that also meets the network target, so learners must understand share accounting before the attack model makes sense.</x:v>
+        <x:v>Short Channel IDs encode block height as their first component, so learners need the block-height concept before decoding the identifier.</x:v>
       </x:c>
       <x:c r="F123" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G123" s="32" t="str">
-        <x:v>Pool-versus-solo and mining economics are inherited through mining.pool-shares; do not add a redundant majority-attack edge.</x:v>
+        <x:v>The transaction-index and output-index components remain part of the identifier's own outcome rather than extra transitive edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>protocol.nodes-vs-miners</x:v>
       </x:c>
       <x:c r="B124" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>mining.miner-decentralization</x:v>
       </x:c>
       <x:c r="C124" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14285,21 +14485,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E124" s="32" t="str">
-        <x:v>P2C tweaks a public key to commit to contract data, so learners need the public/private key model.</x:v>
+        <x:v>Miner decentralization only makes sense once learners distinguish miners' transaction-ordering role from full nodes' independent enforcement of consensus validity.</x:v>
       </x:c>
       <x:c r="F124" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G124" s="32" t="str">
-        <x:v>Taproot is adjacent, not a direct requirement.</x:v>
+        <x:v>The edge keeps censorship power separate from authority to change consensus rules.</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B125" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>mining.miner-decentralization</x:v>
       </x:c>
       <x:c r="C125" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14308,21 +14508,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E125" s="32" t="str">
-        <x:v>P2C derives a commitment tweak from contract data using a hash, so learners need hash commitments first.</x:v>
+        <x:v>Pool and solo mining explain the participant and coordination structure whose concentration or dispersion determines practical control over transaction ordering.</x:v>
       </x:c>
       <x:c r="F125" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G125" s="32" t="str">
-        <x:v>The hash is part of the construction rather than generic background.</x:v>
+        <x:v>Stratum V2 remains optional implementation context, not a direct prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="32" t="str">
-        <x:v>protocol.utxo-model</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="B126" s="32" t="str">
-        <x:v>extension.single-use-seals</x:v>
+        <x:v>dev.selection-cryptography</x:v>
       </x:c>
       <x:c r="C126" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14331,21 +14531,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E126" s="32" t="str">
-        <x:v>Single-use seals rely on a UTXO's one-time spend property.</x:v>
+        <x:v>Selection cryptography evaluates cryptographic tools and dependencies through evidence, testing, authorship, and review quality, so learners need the broader Bitcoin review discipline first.</x:v>
       </x:c>
       <x:c r="F126" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G126" s="32" t="str">
-        <x:v>This explicit bridge prevents hiding the seal invariant inside generic UTXO semantics.</x:v>
+        <x:v>Adversarial thinking is inherited through dev.review-culture; reproducible builds are a downstream verification practice rather than a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="32" t="str">
-        <x:v>extension.single-use-seals</x:v>
+        <x:v>mining.pool-shares</x:v>
       </x:c>
       <x:c r="B127" s="32" t="str">
-        <x:v>extension.client-side-validation</x:v>
+        <x:v>mining.block-withholding</x:v>
       </x:c>
       <x:c r="C127" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14354,21 +14554,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E127" s="32" t="str">
-        <x:v>Client-side validation relies on seals to prevent an offchain transition from being valid twice.</x:v>
+        <x:v>Block withholding exploits the difference between a pool-paid share and a share that also meets the network target, so learners must understand share accounting before the attack model makes sense.</x:v>
       </x:c>
       <x:c r="F127" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G127" s="32" t="str">
-        <x:v>The UTXO parent is inherited through the seal and is intentionally not duplicated.</x:v>
+        <x:v>Pool-versus-solo and mining economics are inherited through mining.pool-shares; do not add a redundant majority-attack edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="32" t="str">
+        <x:v>fundamentals.public-private-keys</x:v>
+      </x:c>
+      <x:c r="B128" s="32" t="str">
         <x:v>protocol.pay-to-contract</x:v>
-      </x:c>
-      <x:c r="B128" s="32" t="str">
-        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="C128" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14377,21 +14577,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E128" s="32" t="str">
-        <x:v>Client-side validation uses cryptographic commitments to bind offchain asset rules and transitions, so P2C supplies the contract-anchoring mechanism.</x:v>
+        <x:v>P2C tweaks a public key to commit to contract data, so learners need the public/private key model.</x:v>
       </x:c>
       <x:c r="F128" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G128" s="32" t="str">
-        <x:v>Keep this direct edge: it prevents treating client-side validation as a vague UTXO-only extension.</x:v>
+        <x:v>Taproot is adjacent, not a direct requirement.</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="32" t="str">
-        <x:v>protocol.rbf</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B129" s="32" t="str">
-        <x:v>protocol.replacement-cycling</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="C129" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14400,21 +14600,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E129" s="32" t="str">
-        <x:v>Replacement cycling repeatedly uses transaction replacement, so learners need the RBF policy mechanism first.</x:v>
+        <x:v>P2C derives a commitment tweak from contract data using a hash, so learners need hash commitments first.</x:v>
       </x:c>
       <x:c r="F129" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G129" s="32" t="str">
-        <x:v>Package RBF is related but not required for the core attack sequence.</x:v>
+        <x:v>The hash is part of the construction rather than generic background.</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="32" t="str">
-        <x:v>protocol.cpfp</x:v>
+        <x:v>protocol.utxo-model</x:v>
       </x:c>
       <x:c r="B130" s="32" t="str">
-        <x:v>protocol.replacement-cycling</x:v>
+        <x:v>extension.single-use-seals</x:v>
       </x:c>
       <x:c r="C130" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14423,21 +14623,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E130" s="32" t="str">
-        <x:v>The attack cycles child-fee relationships to evict a target, so learners need CPFP mechanics first.</x:v>
+        <x:v>Single-use seals rely on a UTXO's one-time spend property.</x:v>
       </x:c>
       <x:c r="F130" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G130" s="32" t="str">
-        <x:v>Transaction pinning is the broader downstream risk class, not a prerequisite.</x:v>
+        <x:v>This explicit bridge prevents hiding the seal invariant inside generic UTXO semantics.</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="32" t="str">
-        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
+        <x:v>extension.single-use-seals</x:v>
       </x:c>
       <x:c r="B131" s="32" t="str">
-        <x:v>protocol.taproot-control-blocks</x:v>
+        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="C131" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14446,21 +14646,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E131" s="32" t="str">
-        <x:v>Control blocks extend the tapleaf proof path with internal-key and parity data.</x:v>
+        <x:v>Client-side validation relies on seals to prevent an offchain transition from being valid twice.</x:v>
       </x:c>
       <x:c r="F131" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G131" s="32" t="str">
-        <x:v>Generic Merkle trees are inherited through the proof node.</x:v>
+        <x:v>The UTXO parent is inherited through the seal and is intentionally not duplicated.</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="B132" s="32" t="str">
-        <x:v>dev.pseudonymous-development</x:v>
+        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="C132" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14469,21 +14669,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E132" s="32" t="str">
-        <x:v>Pseudonymous development relies on public technical evidence and independent peer review to preserve accountability without requiring legal-identity disclosure.</x:v>
+        <x:v>Client-side validation uses cryptographic commitments to bind offchain asset rules and transitions, so P2C supplies the contract-anchoring mechanism.</x:v>
       </x:c>
       <x:c r="F132" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G132" s="32" t="str">
-        <x:v>Privacy pseudonymity is related context, not a direct prerequisite, because this node concerns contributor identity and governance rather than transaction linkage.</x:v>
+        <x:v>Keep this direct edge: it prevents treating client-side validation as a vague UTXO-only extension.</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="32" t="str">
-        <x:v>fundamentals.merkle-trees</x:v>
+        <x:v>protocol.rbf</x:v>
       </x:c>
       <x:c r="B133" s="32" t="str">
-        <x:v>protocol.mast</x:v>
+        <x:v>protocol.replacement-cycling</x:v>
       </x:c>
       <x:c r="C133" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14492,21 +14692,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E133" s="32" t="str">
-        <x:v>MAST uses a Merkle tree to commit to multiple alternative script branches while revealing only one branch during spending.</x:v>
+        <x:v>Replacement cycling repeatedly uses transaction replacement, so learners need the RBF policy mechanism first.</x:v>
       </x:c>
       <x:c r="F133" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G133" s="32" t="str">
-        <x:v>Direct cryptographic structure; TapTree remains a downstream Taproot-specific realization.</x:v>
+        <x:v>Package RBF is related but not required for the core attack sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>protocol.cpfp</x:v>
       </x:c>
       <x:c r="B134" s="32" t="str">
-        <x:v>protocol.mast</x:v>
+        <x:v>protocol.replacement-cycling</x:v>
       </x:c>
       <x:c r="C134" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14515,21 +14715,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E134" s="32" t="str">
-        <x:v>MAST commits to alternative Bitcoin Script branches, so learners need the locking and spending language before the tree commitment is meaningful.</x:v>
+        <x:v>The attack cycles child-fee relationships to evict a target, so learners need CPFP mechanics first.</x:v>
       </x:c>
       <x:c r="F134" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G134" s="32" t="str">
-        <x:v>Keep Script direct; the node is not only a generic Merkle-tree concept.</x:v>
+        <x:v>Transaction pinning is the broader downstream risk class, not a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="32" t="str">
-        <x:v>protocol.sighash-flags</x:v>
+        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
       </x:c>
       <x:c r="B135" s="32" t="str">
-        <x:v>protocol.sighash-quadratic-hashing</x:v>
+        <x:v>protocol.taproot-control-blocks</x:v>
       </x:c>
       <x:c r="C135" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14538,21 +14738,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E135" s="32" t="str">
-        <x:v>The quadratic hashing problem is a performance consequence of how legacy signature digests are constructed under SIGHASH semantics.</x:v>
+        <x:v>Control blocks extend the tapleaf proof path with internal-key and parity data.</x:v>
       </x:c>
       <x:c r="F135" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G135" s="32" t="str">
-        <x:v>BIP 143 is a supporting mitigation source, not a prerequisite edge.</x:v>
+        <x:v>Generic Merkle trees are inherited through the proof node.</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="B136" s="32" t="str">
-        <x:v>security.rogue-key-attack</x:v>
+        <x:v>dev.pseudonymous-development</x:v>
       </x:c>
       <x:c r="C136" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14561,21 +14761,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E136" s="32" t="str">
-        <x:v>The rogue-key attack occurs in naive public-key aggregation, so learners need the MuSig aggregation setting before the failure mode.</x:v>
+        <x:v>Pseudonymous development relies on public technical evidence and independent peer review to preserve accountability without requiring legal-identity disclosure.</x:v>
       </x:c>
       <x:c r="F136" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G136" s="32" t="str">
-        <x:v>Schnorr is inherited through MuSig; avoid a redundant direct Schnorr edge.</x:v>
+        <x:v>Privacy pseudonymity is related context, not a direct prerequisite, because this node concerns contributor identity and governance rather than transaction linkage.</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>fundamentals.merkle-trees</x:v>
       </x:c>
       <x:c r="B137" s="32" t="str">
-        <x:v>mining.selfish-mining</x:v>
+        <x:v>protocol.mast</x:v>
       </x:c>
       <x:c r="C137" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14584,21 +14784,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E137" s="32" t="str">
-        <x:v>Selfish mining is an incentive strategy by miners and pools, so learners need the pooled-versus-solo mining context first.</x:v>
+        <x:v>MAST uses a Merkle tree to commit to multiple alternative script branches while revealing only one branch during spending.</x:v>
       </x:c>
       <x:c r="F137" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
       </x:c>
       <x:c r="G137" s="32" t="str">
-        <x:v>Pool economics is one direct parent; chain selection is supplied by the finality parent below.</x:v>
+        <x:v>Direct cryptographic structure; TapTree remains a downstream Taproot-specific realization.</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="32" t="str">
-        <x:v>protocol.reorgs-finality</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B138" s="32" t="str">
-        <x:v>mining.selfish-mining</x:v>
+        <x:v>protocol.mast</x:v>
       </x:c>
       <x:c r="C138" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14607,21 +14807,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E138" s="32" t="str">
-        <x:v>Selfish mining relies on strategic withholding and release of competing branches, which requires the chain-reorganization and finality model.</x:v>
+        <x:v>MAST commits to alternative Bitcoin Script branches, so learners need the locking and spending language before the tree commitment is meaningful.</x:v>
       </x:c>
       <x:c r="F138" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
       </x:c>
       <x:c r="G138" s="32" t="str">
-        <x:v>Keep the reorganization model direct rather than adding generic proof-of-work as a redundant ancestor.</x:v>
+        <x:v>Keep Script direct; the node is not only a generic Merkle-tree concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>protocol.sighash-flags</x:v>
       </x:c>
       <x:c r="B139" s="32" t="str">
-        <x:v>protocol.commit-delay-reveal</x:v>
+        <x:v>protocol.sighash-quadratic-hashing</x:v>
       </x:c>
       <x:c r="C139" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14630,21 +14830,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E139" s="32" t="str">
-        <x:v>Commit-delay-reveal composes a cryptographic commitment with a timed reveal, so the learner first needs the hiding and binding commitment model.</x:v>
+        <x:v>The quadratic hashing problem is a performance consequence of how legacy signature digests are constructed under SIGHASH semantics.</x:v>
       </x:c>
       <x:c r="F139" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
+        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
       </x:c>
       <x:c r="G139" s="32" t="str">
-        <x:v>The delay/reveal composition is the node's distinct outcome.</x:v>
+        <x:v>BIP 143 is a supporting mitigation source, not a prerequisite edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="32" t="str">
-        <x:v>protocol.dust-policy</x:v>
+        <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="B140" s="32" t="str">
-        <x:v>security.dust-attack</x:v>
+        <x:v>security.rogue-key-attack</x:v>
       </x:c>
       <x:c r="C140" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14653,21 +14853,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E140" s="32" t="str">
-        <x:v>Dust attacks exploit the distinction between tiny-output relay policy and the ability to place trace-value UTXOs in a wallet.</x:v>
+        <x:v>The rogue-key attack occurs in naive public-key aggregation, so learners need the MuSig aggregation setting before the failure mode.</x:v>
       </x:c>
       <x:c r="F140" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
       </x:c>
       <x:c r="G140" s="32" t="str">
-        <x:v>Policy threshold is direct context for the attack mechanism.</x:v>
+        <x:v>Schnorr is inherited through MuSig; avoid a redundant direct Schnorr edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B141" s="32" t="str">
-        <x:v>security.dust-attack</x:v>
+        <x:v>mining.selfish-mining</x:v>
       </x:c>
       <x:c r="C141" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14676,21 +14876,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E141" s="32" t="str">
-        <x:v>The privacy harm of dusting comes from linking future spends and wallet activity, so learners need the pseudonymity and linkage model.</x:v>
+        <x:v>Selfish mining is an incentive strategy by miners and pools, so learners need the pooled-versus-solo mining context first.</x:v>
       </x:c>
       <x:c r="F141" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
       </x:c>
       <x:c r="G141" s="32" t="str">
-        <x:v>Keep privacy linkage direct; it is not inherited through dust policy.</x:v>
+        <x:v>Pool economics is one direct parent; chain selection is supplied by the finality parent below.</x:v>
       </x:c>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="32" t="str">
-        <x:v>fundamentals.neutrality</x:v>
+        <x:v>protocol.reorgs-finality</x:v>
       </x:c>
       <x:c r="B142" s="32" t="str">
-        <x:v>dev.permissionless-development</x:v>
+        <x:v>mining.selfish-mining</x:v>
       </x:c>
       <x:c r="C142" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14699,21 +14899,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E142" s="32" t="str">
-        <x:v>Permissionless development depends on a neutral protocol that does not select which users or applications may participate.</x:v>
+        <x:v>Selfish mining relies on strategic withholding and release of competing branches, which requires the chain-reorganization and finality model.</x:v>
       </x:c>
       <x:c r="F142" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
       </x:c>
       <x:c r="G142" s="32" t="str">
-        <x:v>Neutrality supplies the protocol property; the BIPs process supplies the change/proposal lifecycle below.</x:v>
+        <x:v>Keep the reorganization model direct rather than adding generic proof-of-work as a redundant ancestor.</x:v>
       </x:c>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="32" t="str">
-        <x:v>dev.bips-process</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="B143" s="32" t="str">
-        <x:v>dev.permissionless-development</x:v>
+        <x:v>protocol.commit-delay-reveal</x:v>
       </x:c>
       <x:c r="C143" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14722,21 +14922,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E143" s="32" t="str">
-        <x:v>Learners need the proposal and deployment process to distinguish building permissionlessly from changing Bitcoin's consensus rules without broad adoption.</x:v>
+        <x:v>Commit-delay-reveal composes a cryptographic commitment with a timed reveal, so the learner first needs the hiding and binding commitment model.</x:v>
       </x:c>
       <x:c r="F143" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
       </x:c>
       <x:c r="G143" s="32" t="str">
-        <x:v>Review culture remains related but is not a direct prerequisite for permissionless access.</x:v>
+        <x:v>The delay/reveal composition is the node's distinct outcome.</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="32" t="str">
-        <x:v>dev.reproducible-builds</x:v>
+        <x:v>protocol.dust-policy</x:v>
       </x:c>
       <x:c r="B144" s="32" t="str">
-        <x:v>dev.bootstrappable-builds</x:v>
+        <x:v>security.dust-attack</x:v>
       </x:c>
       <x:c r="C144" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14745,21 +14945,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E144" s="32" t="str">
-        <x:v>Bootstrappable builds extend reproducible builds by reducing trust in the compiler and build-tool binaries used to produce the reproducible output.</x:v>
+        <x:v>Dust attacks exploit the distinction between tiny-output relay policy and the ability to place trace-value UTXOs in a wallet.</x:v>
       </x:c>
       <x:c r="F144" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
       </x:c>
       <x:c r="G144" s="32" t="str">
-        <x:v>Keep this as a direct downstream edge; the node is not a duplicate alias for reproducible builds.</x:v>
+        <x:v>Policy threshold is direct context for the attack mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="32" t="str">
-        <x:v>protocol.transaction-lifecycle</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B145" s="32" t="str">
-        <x:v>protocol.proof-of-payment</x:v>
+        <x:v>security.dust-attack</x:v>
       </x:c>
       <x:c r="C145" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14768,21 +14968,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E145" s="32" t="str">
-        <x:v>Proof of Payment refers to a prior payment and reconstructs a transaction-shaped proof, so learners need the transaction lifecycle first.</x:v>
+        <x:v>The privacy harm of dusting comes from linking future spends and wallet activity, so learners need the pseudonymity and linkage model.</x:v>
       </x:c>
       <x:c r="F145" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
       </x:c>
       <x:c r="G145" s="32" t="str">
-        <x:v>Direct payment context; wallet UX and URI transport remain downstream or optional details.</x:v>
+        <x:v>Keep privacy linkage direct; it is not inherited through dust policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="32" t="str">
-        <x:v>protocol.ephemeral-anchors</x:v>
+        <x:v>fundamentals.neutrality</x:v>
       </x:c>
       <x:c r="B146" s="32" t="str">
-        <x:v>protocol.pay-to-anchor</x:v>
+        <x:v>dev.permissionless-development</x:v>
       </x:c>
       <x:c r="C146" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14791,12 +14991,104 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E146" s="32" t="str">
+        <x:v>Permissionless development depends on a neutral protocol that does not select which users or applications may participate.</x:v>
+      </x:c>
+      <x:c r="F146" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G146" s="32" t="str">
+        <x:v>Neutrality supplies the protocol property; the BIPs process supplies the change/proposal lifecycle below.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" s="32" t="str">
+        <x:v>dev.bips-process</x:v>
+      </x:c>
+      <x:c r="B147" s="32" t="str">
+        <x:v>dev.permissionless-development</x:v>
+      </x:c>
+      <x:c r="C147" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D147" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E147" s="32" t="str">
+        <x:v>Learners need the proposal and deployment process to distinguish building permissionlessly from changing Bitcoin's consensus rules without broad adoption.</x:v>
+      </x:c>
+      <x:c r="F147" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G147" s="32" t="str">
+        <x:v>Review culture remains related but is not a direct prerequisite for permissionless access.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" s="32" t="str">
+        <x:v>dev.reproducible-builds</x:v>
+      </x:c>
+      <x:c r="B148" s="32" t="str">
+        <x:v>dev.bootstrappable-builds</x:v>
+      </x:c>
+      <x:c r="C148" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D148" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E148" s="32" t="str">
+        <x:v>Bootstrappable builds extend reproducible builds by reducing trust in the compiler and build-tool binaries used to produce the reproducible output.</x:v>
+      </x:c>
+      <x:c r="F148" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G148" s="32" t="str">
+        <x:v>Keep this as a direct downstream edge; the node is not a duplicate alias for reproducible builds.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" s="32" t="str">
+        <x:v>protocol.transaction-lifecycle</x:v>
+      </x:c>
+      <x:c r="B149" s="32" t="str">
+        <x:v>protocol.proof-of-payment</x:v>
+      </x:c>
+      <x:c r="C149" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D149" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E149" s="32" t="str">
+        <x:v>Proof of Payment refers to a prior payment and reconstructs a transaction-shaped proof, so learners need the transaction lifecycle first.</x:v>
+      </x:c>
+      <x:c r="F149" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="G149" s="32" t="str">
+        <x:v>Direct payment context; wallet UX and URI transport remain downstream or optional details.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" s="32" t="str">
+        <x:v>protocol.ephemeral-anchors</x:v>
+      </x:c>
+      <x:c r="B150" s="32" t="str">
+        <x:v>protocol.pay-to-anchor</x:v>
+      </x:c>
+      <x:c r="C150" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D150" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E150" s="32" t="str">
         <x:v>Pay to Anchor is a keyless refinement of the anchor-output and package-relay fee-bumping pattern, so learners need that broader context first.</x:v>
       </x:c>
-      <x:c r="F146" s="32" t="str">
+      <x:c r="F150" s="32" t="str">
         <x:v>source.bitcoin-bips</x:v>
       </x:c>
-      <x:c r="G146" s="32" t="str">
+      <x:c r="G150" s="32" t="str">
         <x:v>BIP 431/TRUC is related anti-pinning context, not an inherent prerequisite.</x:v>
       </x:c>
     </x:row>
@@ -14806,10 +15098,10 @@
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C146">
+    <x:dataValidation type="list" sqref="C12:C150">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D146">
+    <x:dataValidation type="list" sqref="D12:D150">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -17891,16 +18183,42 @@
         <x:v>Keep Spark-specific operator internals, SDK APIs, and wallet products inside the node resources rather than creating implementation-shaped children.</x:v>
       </x:c>
     </x:row>
+    <x:row r="128">
+      <x:c r="A128" s="32" t="str">
+        <x:v>decision.cube-scope-slice</x:v>
+      </x:c>
+      <x:c r="B128" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C128" s="32" t="str">
+        <x:v>source.cube-introducing</x:v>
+      </x:c>
+      <x:c r="D128" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E128" s="32" t="str">
+        <x:v>The article contains both reusable protocol primitives and Cube-specific mechanisms; only concepts with an independent learner outcome and prerequisite chain should become graph nodes.</x:v>
+      </x:c>
+      <x:c r="F128" s="32" t="str">
+        <x:v>extension.cube, extension.timeout-trees, extension.zktlcs, extension.bitvm, protocol.timelocks</x:v>
+      </x:c>
+      <x:c r="G128" s="32" t="str">
+        <x:v>source.cube-introducing</x:v>
+      </x:c>
+      <x:c r="H128" s="32" t="str">
+        <x:v>Add Cube, Timeout Trees, and ZKTLCs. Keep Shadowing, Shadow Space, Projector, Hosted/Black Box Projection, Lifting, exit-ladder internals, and APE/bit-level encoding inside Cube/source context.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B127">
+    <x:dataValidation type="list" sqref="B12:B128">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D127">
+    <x:dataValidation type="list" sqref="D12:D128">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -17953,7 +18271,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.77399011574</x:v>
+        <x:v>46214.77654195602</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -17961,7 +18279,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -17969,7 +18287,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -17977,7 +18295,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>159</x:v>
+        <x:v>162</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -17985,7 +18303,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>135</x:v>
+        <x:v>139</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -18009,7 +18327,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>100</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add RGB and Liquid concepts
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R82332111d56a47a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R6863410656d446c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R9e05f0fb7cc8447b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R6c5f3171318842f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rf8400f2beddf4fb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rc13a9796e51f41e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rcade66270f8544f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R649bbcab81eb41ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rd304d81d6c984638"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R01f6aca1234345a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rd610340fcbc84d59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rad365721cefc4641"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3407,22 +3407,116 @@
         <x:v>Added Cube, Timeout Trees, and ZKTLCs. Shadowing, Shadow Space, Projector, Hosted/Black Box Projection, Lifting, exit-ladder internals, and APE/bit-level encoding remain inside Cube or source context because they are implementation-specific mechanisms rather than independent Bitcoin learning prerequisites.</x:v>
       </x:c>
     </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="32" t="str">
+        <x:v>source.rgb-protocol</x:v>
+      </x:c>
+      <x:c r="B73" s="32" t="str">
+        <x:v>RGB Protocol Documentation and Repository</x:v>
+      </x:c>
+      <x:c r="C73" s="32" t="str">
+        <x:v>https://rgb.tech/docs/</x:v>
+      </x:c>
+      <x:c r="D73" s="32" t="str">
+        <x:v>protocol-documentation-repository</x:v>
+      </x:c>
+      <x:c r="E73" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F73" s="32" t="str">
+        <x:v>RGB client-side-validated smart contracts for Bitcoin and Lightning, including commitments, contract state, asset history, and integration surfaces.</x:v>
+      </x:c>
+      <x:c r="G73" s="32" t="str">
+        <x:v>Track the official RGB documentation, blueprint, standards index, and reference repository as one protocol cluster. Separate the RGB protocol outcome from already-covered client-side validation, single-use seals, and implementation APIs.</x:v>
+      </x:c>
+      <x:c r="H73" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I73" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J73" s="32" t="str">
+        <x:v>Normalized</x:v>
+      </x:c>
+      <x:c r="K73" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L73" s="32" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="M73" s="32" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N73" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O73" s="32" t="str">
+        <x:v>Added RGB as the protocol-level concept. Client-side validation, single-use seals, pay-to-contract, consignments, and library/API details remain prerequisites or implementation context rather than duplicate nodes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="32" t="str">
+        <x:v>source.liquid-elements</x:v>
+      </x:c>
+      <x:c r="B74" s="32" t="str">
+        <x:v>Liquid Network and Elements Documentation</x:v>
+      </x:c>
+      <x:c r="C74" s="32" t="str">
+        <x:v>https://docs.liquid.net/docs/welcome-to-liquid-developer-documentation-portal</x:v>
+      </x:c>
+      <x:c r="D74" s="32" t="str">
+        <x:v>protocol-documentation-cluster</x:v>
+      </x:c>
+      <x:c r="E74" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F74" s="32" t="str">
+        <x:v>Elements as a Bitcoin-derived sidechain platform and Liquid as its production federated network, including confidential transactions, issued assets, two-way peg flows, and Lightning interoperability.</x:v>
+      </x:c>
+      <x:c r="G74" s="32" t="str">
+        <x:v>Track official Liquid documentation, Liquid technical/how-it-works pages, Elements project documentation, and the reference repository as one cluster. Keep the platform, production network, and reusable confidential-transaction primitive distinct; keep RPCs, wallet products, and individual assets inside resources.</x:v>
+      </x:c>
+      <x:c r="H74" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I74" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J74" s="32" t="str">
+        <x:v>Normalized</x:v>
+      </x:c>
+      <x:c r="K74" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L74" s="32" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="M74" s="32" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="N74" s="32" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O74" s="32" t="str">
+        <x:v>Added Elements, Liquid Network, and Confidential Transactions. Generic sidechains remains the direct context for Elements; Liquid-specific peg, federation, L-BTC, and issued-asset workflows remain inside the protocol node.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H72">
+    <x:dataValidation type="list" sqref="H12:H74">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I72">
+    <x:dataValidation type="list" sqref="I12:I74">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J72">
+    <x:dataValidation type="list" sqref="J12:J74">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K72">
+    <x:dataValidation type="list" sqref="K12:K74">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11820,16 +11914,220 @@
         <x:v>Keep Shadowing, Projector, lifting, exit-ladder internals, and DA encoding as Cube mechanisms and resources rather than separate nodes.</x:v>
       </x:c>
     </x:row>
+    <x:row r="174">
+      <x:c r="A174" s="32" t="str">
+        <x:v>extension.rgb</x:v>
+      </x:c>
+      <x:c r="B174" s="32" t="str">
+        <x:v>RGB Protocol</x:v>
+      </x:c>
+      <x:c r="C174" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D174" s="32" t="str">
+        <x:v>source.rgb-protocol</x:v>
+      </x:c>
+      <x:c r="E174" s="32" t="str">
+        <x:v>https://rgb.tech/docs/</x:v>
+      </x:c>
+      <x:c r="F174" s="32" t="str">
+        <x:v>Official RGB documentation, blueprint, standards, and reference repository</x:v>
+      </x:c>
+      <x:c r="G174" s="32" t="str"/>
+      <x:c r="H174" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I174" s="32" t="str">
+        <x:v>RGB is a concrete client-side-validated smart-contract protocol for Bitcoin and Lightning with its own contract-state, asset-history, and commitment model; it is not merely an alias for client-side validation or token basics.</x:v>
+      </x:c>
+      <x:c r="J174" s="32" t="str">
+        <x:v>extension.client-side-validation</x:v>
+      </x:c>
+      <x:c r="K174" s="32" t="str">
+        <x:v>extension.client-side-validation</x:v>
+      </x:c>
+      <x:c r="L174" s="32" t="str">
+        <x:v>Client-side validation supplies the core model of participant-validated off-chain state; single-use seals and pay-to-contract are already inherited through that node's prerequisite path.</x:v>
+      </x:c>
+      <x:c r="M174" s="32" t="str">
+        <x:v>RGB smart contracts, RGB protocol</x:v>
+      </x:c>
+      <x:c r="N174" s="32" t="str">
+        <x:v>rgb, client-side-validation, smart-contracts, assets, lightning</x:v>
+      </x:c>
+      <x:c r="O174" s="32" t="str">
+        <x:v>75m</x:v>
+      </x:c>
+      <x:c r="P174" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q174" s="32" t="str">
+        <x:v>Add RGB as a protocol-level node; consignments, schemas, RGB20/RGB21 interfaces, and library APIs remain internal protocol details or resources.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175">
+      <x:c r="A175" s="32" t="str">
+        <x:v>protocol.confidential-transactions</x:v>
+      </x:c>
+      <x:c r="B175" s="32" t="str">
+        <x:v>Confidential Transactions</x:v>
+      </x:c>
+      <x:c r="C175" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D175" s="32" t="str">
+        <x:v>source.liquid-elements</x:v>
+      </x:c>
+      <x:c r="E175" s="32" t="str">
+        <x:v>https://docs.liquid.net/docs/technical-overview</x:v>
+      </x:c>
+      <x:c r="F175" s="32" t="str">
+        <x:v>Liquid technical overview and Elements confidential-transaction model</x:v>
+      </x:c>
+      <x:c r="G175" s="32" t="str"/>
+      <x:c r="H175" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I175" s="32" t="str">
+        <x:v>Confidential Transactions are a reusable cryptographic transaction model that hides amounts and selected asset information while preserving validation; they are a distinct learner outcome from generic privacy, commitments, or Liquid itself.</x:v>
+      </x:c>
+      <x:c r="J175" s="32" t="str">
+        <x:v>fundamentals.commitment-schemes</x:v>
+      </x:c>
+      <x:c r="K175" s="32" t="str">
+        <x:v>fundamentals.commitment-schemes</x:v>
+      </x:c>
+      <x:c r="L175" s="32" t="str">
+        <x:v>Commitments provide the core hiding-and-binding model needed before confidential amounts and proof-based validation make sense.</x:v>
+      </x:c>
+      <x:c r="M175" s="32" t="str">
+        <x:v>confidential transactions, confidential assets, CT</x:v>
+      </x:c>
+      <x:c r="N175" s="32" t="str">
+        <x:v>privacy, commitments, range-proofs, liquid, elements</x:v>
+      </x:c>
+      <x:c r="O175" s="32" t="str">
+        <x:v>60m</x:v>
+      </x:c>
+      <x:c r="P175" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q175" s="32" t="str">
+        <x:v>Add as the reusable primitive behind Liquid and Elements; range proofs and asset blinding remain supporting mechanisms rather than separate nodes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" s="32" t="str">
+        <x:v>extension.elements</x:v>
+      </x:c>
+      <x:c r="B176" s="32" t="str">
+        <x:v>Elements Platform</x:v>
+      </x:c>
+      <x:c r="C176" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D176" s="32" t="str">
+        <x:v>source.liquid-elements</x:v>
+      </x:c>
+      <x:c r="E176" s="32" t="str">
+        <x:v>https://elementsproject.org/</x:v>
+      </x:c>
+      <x:c r="F176" s="32" t="str">
+        <x:v>Elements platform overview, documentation, and reference repository</x:v>
+      </x:c>
+      <x:c r="G176" s="32" t="str"/>
+      <x:c r="H176" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I176" s="32" t="str">
+        <x:v>Elements is a concrete Bitcoin-derived platform for building sidechains and application-specific networks, distinct from the generic sidechain design space and from Liquid's production network instance.</x:v>
+      </x:c>
+      <x:c r="J176" s="32" t="str">
+        <x:v>extension.sidechains</x:v>
+      </x:c>
+      <x:c r="K176" s="32" t="str">
+        <x:v>extension.sidechains</x:v>
+      </x:c>
+      <x:c r="L176" s="32" t="str">
+        <x:v>Sidechains provide the architecture and security-model context needed to understand what Elements extends and deploys.</x:v>
+      </x:c>
+      <x:c r="M176" s="32" t="str">
+        <x:v>Elements blockchain platform, Elements Core</x:v>
+      </x:c>
+      <x:c r="N176" s="32" t="str">
+        <x:v>elements, sidechains, confidential-transactions, assets</x:v>
+      </x:c>
+      <x:c r="O176" s="32" t="str">
+        <x:v>60m</x:v>
+      </x:c>
+      <x:c r="P176" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q176" s="32" t="str">
+        <x:v>Keep Elements RPCs, opcodes, and local regtest workflows as implementation resources rather than standalone nodes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177">
+      <x:c r="A177" s="32" t="str">
+        <x:v>extension.liquid</x:v>
+      </x:c>
+      <x:c r="B177" s="32" t="str">
+        <x:v>Liquid Network</x:v>
+      </x:c>
+      <x:c r="C177" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D177" s="32" t="str">
+        <x:v>source.liquid-elements</x:v>
+      </x:c>
+      <x:c r="E177" s="32" t="str">
+        <x:v>https://docs.liquid.net/docs/welcome-to-liquid-developer-documentation-portal</x:v>
+      </x:c>
+      <x:c r="F177" s="32" t="str">
+        <x:v>Liquid developer portal and How Liquid Works</x:v>
+      </x:c>
+      <x:c r="G177" s="32" t="str"/>
+      <x:c r="H177" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I177" s="32" t="str">
+        <x:v>Liquid is a production federated Bitcoin sidechain with a distinct peg, settlement, privacy, and asset-issuance model; it is not interchangeable with generic sidechains or the Elements platform.</x:v>
+      </x:c>
+      <x:c r="J177" s="32" t="str">
+        <x:v>extension.elements, protocol.confidential-transactions</x:v>
+      </x:c>
+      <x:c r="K177" s="32" t="str">
+        <x:v>extension.elements, protocol.confidential-transactions</x:v>
+      </x:c>
+      <x:c r="L177" s="32" t="str">
+        <x:v>Elements explains the implementation platform, while Confidential Transactions explains Liquid's defining privacy and asset-transfer primitive.</x:v>
+      </x:c>
+      <x:c r="M177" s="32" t="str">
+        <x:v>Liquid Network, Liquid sidechain, L-BTC</x:v>
+      </x:c>
+      <x:c r="N177" s="32" t="str">
+        <x:v>liquid, sidechains, elements, assets, confidential-transactions, lightning</x:v>
+      </x:c>
+      <x:c r="O177" s="32" t="str">
+        <x:v>75m</x:v>
+      </x:c>
+      <x:c r="P177" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q177" s="32" t="str">
+        <x:v>Keep peg-in/peg-out, federation operations, L-BTC, and individual issued assets inside the Liquid protocol node.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H173">
+    <x:dataValidation type="list" sqref="H12:H177">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P173">
+    <x:dataValidation type="list" sqref="P12:P177">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -11897,10 +12195,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="32" t="str">
-        <x:v>protocol.timelocks</x:v>
+        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="B12" s="32" t="str">
-        <x:v>extension.timeout-trees</x:v>
+        <x:v>extension.rgb</x:v>
       </x:c>
       <x:c r="C12" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11909,10 +12207,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E12" s="32" t="str">
-        <x:v>Timeout Trees use delayed transaction branches to preserve unilateral redemption, so learners need Bitcoin timelocks first.</x:v>
+        <x:v>RGB builds its contract and asset model on client-side validation of off-chain state anchored to Bitcoin outputs.</x:v>
       </x:c>
       <x:c r="F12" s="32" t="str">
-        <x:v>source.cube-introducing</x:v>
+        <x:v>source.rgb-protocol</x:v>
       </x:c>
       <x:c r="G12" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11920,10 +12218,10 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="32" t="str">
-        <x:v>extension.timeout-trees</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="B13" s="32" t="str">
-        <x:v>extension.zktlcs</x:v>
+        <x:v>protocol.confidential-transactions</x:v>
       </x:c>
       <x:c r="C13" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11932,10 +12230,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E13" s="32" t="str">
-        <x:v>ZKTLCs use timeout-tree ownership virtualization as one half of their unified primitive.</x:v>
+        <x:v>Confidential Transactions use cryptographic commitments to hide values while preserving verifiability.</x:v>
       </x:c>
       <x:c r="F13" s="32" t="str">
-        <x:v>source.cube-introducing</x:v>
+        <x:v>source.liquid-elements</x:v>
       </x:c>
       <x:c r="G13" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11943,10 +12241,10 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="32" t="str">
-        <x:v>extension.bitvm</x:v>
+        <x:v>extension.sidechains</x:v>
       </x:c>
       <x:c r="B14" s="32" t="str">
-        <x:v>extension.zktlcs</x:v>
+        <x:v>extension.elements</x:v>
       </x:c>
       <x:c r="C14" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11955,10 +12253,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E14" s="32" t="str">
-        <x:v>ZKTLCs use BitVM-style challenge and disproof to enforce computation without trusting the executor.</x:v>
+        <x:v>Elements is a concrete platform for constructing Bitcoin-derived sidechains and application-specific networks.</x:v>
       </x:c>
       <x:c r="F14" s="32" t="str">
-        <x:v>source.cube-introducing</x:v>
+        <x:v>source.liquid-elements</x:v>
       </x:c>
       <x:c r="G14" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11966,10 +12264,10 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="32" t="str">
-        <x:v>extension.zktlcs</x:v>
+        <x:v>extension.elements</x:v>
       </x:c>
       <x:c r="B15" s="32" t="str">
-        <x:v>extension.cube</x:v>
+        <x:v>extension.liquid</x:v>
       </x:c>
       <x:c r="C15" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -11978,10 +12276,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E15" s="32" t="str">
-        <x:v>Cube's architecture is built around ZKTLCs for programmable execution, ownership, and unilateral exit.</x:v>
+        <x:v>Liquid is a production network built on the Elements platform, with its own federation, peg, and asset policies.</x:v>
       </x:c>
       <x:c r="F15" s="32" t="str">
-        <x:v>source.cube-introducing</x:v>
+        <x:v>source.liquid-elements</x:v>
       </x:c>
       <x:c r="G15" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -11989,10 +12287,10 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="32" t="str">
-        <x:v>extension.statechains</x:v>
+        <x:v>protocol.confidential-transactions</x:v>
       </x:c>
       <x:c r="B16" s="32" t="str">
-        <x:v>extension.spark</x:v>
+        <x:v>extension.liquid</x:v>
       </x:c>
       <x:c r="C16" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12001,10 +12299,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E16" s="32" t="str">
-        <x:v>Spark's architecture extends statechain-style off-chain ownership transfer with a distributed operator set and Lightning interoperability.</x:v>
+        <x:v>Liquid's privacy and issued-asset behavior depends on Confidential Transactions as a core transaction primitive.</x:v>
       </x:c>
       <x:c r="F16" s="32" t="str">
-        <x:v>source.spark-protocol</x:v>
+        <x:v>source.liquid-elements</x:v>
       </x:c>
       <x:c r="G16" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12012,10 +12310,10 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="32" t="str">
-        <x:v>history.cypherpunk-roots-bitcoin-origin</x:v>
+        <x:v>protocol.timelocks</x:v>
       </x:c>
       <x:c r="B17" s="32" t="str">
-        <x:v>history.satoshi-nakamoto</x:v>
+        <x:v>extension.timeout-trees</x:v>
       </x:c>
       <x:c r="C17" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12024,10 +12322,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E17" s="32" t="str">
-        <x:v>Satoshi's pseudonym and founder independence are best understood in the context of Bitcoin's cypherpunk roots and origin story.</x:v>
+        <x:v>Timeout Trees use delayed transaction branches to preserve unilateral redemption, so learners need Bitcoin timelocks first.</x:v>
       </x:c>
       <x:c r="F17" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.cube-introducing</x:v>
       </x:c>
       <x:c r="G17" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12035,10 +12333,10 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="32" t="str">
-        <x:v>fundamentals.money-properties</x:v>
+        <x:v>extension.timeout-trees</x:v>
       </x:c>
       <x:c r="B18" s="32" t="str">
-        <x:v>economics.bitcoin-denominations</x:v>
+        <x:v>extension.zktlcs</x:v>
       </x:c>
       <x:c r="C18" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12047,10 +12345,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E18" s="32" t="str">
-        <x:v>The learner needs a basic monetary-unit model before BTC and satoshis are meaningful denominations.</x:v>
+        <x:v>ZKTLCs use timeout-tree ownership virtualization as one half of their unified primitive.</x:v>
       </x:c>
       <x:c r="F18" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.cube-introducing</x:v>
       </x:c>
       <x:c r="G18" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12058,10 +12356,10 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="32" t="str">
-        <x:v>protocol.coinbase-transaction</x:v>
+        <x:v>extension.bitvm</x:v>
       </x:c>
       <x:c r="B19" s="32" t="str">
-        <x:v>economics.block-subsidy</x:v>
+        <x:v>extension.zktlcs</x:v>
       </x:c>
       <x:c r="C19" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12070,21 +12368,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E19" s="32" t="str">
-        <x:v>The block subsidy is the newly issued component claimed by a coinbase transaction.</x:v>
+        <x:v>ZKTLCs use BitVM-style challenge and disproof to enforce computation without trusting the executor.</x:v>
       </x:c>
       <x:c r="F19" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.cube-introducing</x:v>
       </x:c>
       <x:c r="G19" s="32" t="str">
-        <x:v>The coinbase node already carries the halving prerequisite, so no redundant direct halving edge is added.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="32" t="str">
-        <x:v>fundamentals.digital-signatures</x:v>
+        <x:v>extension.zktlcs</x:v>
       </x:c>
       <x:c r="B20" s="32" t="str">
-        <x:v>security.quantum-computing-threat</x:v>
+        <x:v>extension.cube</x:v>
       </x:c>
       <x:c r="C20" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12093,10 +12391,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E20" s="32" t="str">
-        <x:v>Quantum attacks on public-key authorization require understanding ordinary Bitcoin signature security first.</x:v>
+        <x:v>Cube's architecture is built around ZKTLCs for programmable execution, ownership, and unilateral exit.</x:v>
       </x:c>
       <x:c r="F20" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.cube-introducing</x:v>
       </x:c>
       <x:c r="G20" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12104,10 +12402,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>extension.statechains</x:v>
       </x:c>
       <x:c r="B21" s="32" t="str">
-        <x:v>extension.ordinals-inscriptions</x:v>
+        <x:v>extension.spark</x:v>
       </x:c>
       <x:c r="C21" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12116,10 +12414,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E21" s="32" t="str">
-        <x:v>The source explains inscriptions as a Taproot-era witness-data application.</x:v>
+        <x:v>Spark's architecture extends statechain-style off-chain ownership transfer with a distributed operator set and Lightning interoperability.</x:v>
       </x:c>
       <x:c r="F21" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.spark-protocol</x:v>
       </x:c>
       <x:c r="G21" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12127,10 +12425,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32" t="str">
-        <x:v>protocol.witness-structure</x:v>
+        <x:v>history.cypherpunk-roots-bitcoin-origin</x:v>
       </x:c>
       <x:c r="B22" s="32" t="str">
-        <x:v>extension.ordinals-inscriptions</x:v>
+        <x:v>history.satoshi-nakamoto</x:v>
       </x:c>
       <x:c r="C22" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12139,7 +12437,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E22" s="32" t="str">
-        <x:v>Witness structure is needed to understand where inscription data is carried and how it affects block space.</x:v>
+        <x:v>Satoshi's pseudonym and founder independence are best understood in the context of Bitcoin's cypherpunk roots and origin story.</x:v>
       </x:c>
       <x:c r="F22" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
@@ -12150,10 +12448,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>fundamentals.money-properties</x:v>
       </x:c>
       <x:c r="B23" s="32" t="str">
-        <x:v>extension.proof-of-existence</x:v>
+        <x:v>economics.bitcoin-denominations</x:v>
       </x:c>
       <x:c r="C23" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12162,7 +12460,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E23" s="32" t="str">
-        <x:v>Timestamp proofs commit evidence without requiring the complete document to be stored on-chain.</x:v>
+        <x:v>The learner needs a basic monetary-unit model before BTC and satoshis are meaningful denominations.</x:v>
       </x:c>
       <x:c r="F23" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
@@ -12173,10 +12471,10 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="str">
-        <x:v>protocol.tagged-hashes</x:v>
+        <x:v>protocol.coinbase-transaction</x:v>
       </x:c>
       <x:c r="B24" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>economics.block-subsidy</x:v>
       </x:c>
       <x:c r="C24" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12185,21 +12483,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E24" s="32" t="str">
-        <x:v>TapTweak is defined using tagged hashes directly in Taproot key tweaking.</x:v>
+        <x:v>The block subsidy is the newly issued component claimed by a coinbase transaction.</x:v>
       </x:c>
       <x:c r="F24" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G24" s="32" t="str">
-        <x:v>Source-driven bridge edge.</x:v>
+        <x:v>The coinbase node already carries the halving prerequisite, so no redundant direct halving edge is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="str">
-        <x:v>protocol.x-only-public-keys</x:v>
+        <x:v>fundamentals.digital-signatures</x:v>
       </x:c>
       <x:c r="B25" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>security.quantum-computing-threat</x:v>
       </x:c>
       <x:c r="C25" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12208,10 +12506,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E25" s="32" t="str">
-        <x:v>TapTweak operates on x-only public keys in the Taproot construction.</x:v>
+        <x:v>Quantum attacks on public-key authorization require understanding ordinary Bitcoin signature security first.</x:v>
       </x:c>
       <x:c r="F25" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G25" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12219,10 +12517,10 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B26" s="32" t="str">
-        <x:v>protocol.taproot-key-path-spends</x:v>
+        <x:v>extension.ordinals-inscriptions</x:v>
       </x:c>
       <x:c r="C26" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12231,21 +12529,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E26" s="32" t="str">
-        <x:v>A key-path spend verifies against the tweaked Taproot output key, so learners need the tweak mechanism before the spending mode makes sense.</x:v>
+        <x:v>The source explains inscriptions as a Taproot-era witness-data application.</x:v>
       </x:c>
       <x:c r="F26" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G26" s="32" t="str">
-        <x:v>Direct parent keeps the node focused on the spend mode rather than on broad Taproot overview material.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="str">
-        <x:v>protocol.taptree</x:v>
+        <x:v>protocol.witness-structure</x:v>
       </x:c>
       <x:c r="B27" s="32" t="str">
-        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
+        <x:v>extension.ordinals-inscriptions</x:v>
       </x:c>
       <x:c r="C27" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12254,10 +12552,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E27" s="32" t="str">
-        <x:v>The inclusion proof only makes sense after the learner understands the TapTree structure.</x:v>
+        <x:v>Witness structure is needed to understand where inscription data is carried and how it affects block space.</x:v>
       </x:c>
       <x:c r="F27" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G27" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12265,10 +12563,10 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32" t="str">
-        <x:v>protocol.taptree</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="B28" s="32" t="str">
-        <x:v>protocol.huffman-optimized-taptrees</x:v>
+        <x:v>extension.proof-of-existence</x:v>
       </x:c>
       <x:c r="C28" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12277,10 +12575,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E28" s="32" t="str">
-        <x:v>Huffman optimization is a refinement of how TapTree leaves are arranged.</x:v>
+        <x:v>Timestamp proofs commit evidence without requiring the complete document to be stored on-chain.</x:v>
       </x:c>
       <x:c r="F28" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G28" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12288,10 +12586,10 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="32" t="str">
-        <x:v>protocol.softfork-hardfork</x:v>
+        <x:v>protocol.tagged-hashes</x:v>
       </x:c>
       <x:c r="B29" s="32" t="str">
-        <x:v>protocol.chain-split-risk</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="C29" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12300,21 +12598,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E29" s="32" t="str">
-        <x:v>Split risk is a downstream consequence of incompatible upgrade paths, so learners should understand the compatibility boundary first.</x:v>
+        <x:v>TapTweak is defined using tagged hashes directly in Taproot key tweaking.</x:v>
       </x:c>
       <x:c r="F29" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G29" s="32" t="str">
-        <x:v>Direct edge chosen over activation-history case studies because those are downstream examples, not prerequisites.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.x-only-public-keys</x:v>
       </x:c>
       <x:c r="B30" s="32" t="str">
-        <x:v>protocol.tapscript</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="C30" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12323,21 +12621,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E30" s="32" t="str">
-        <x:v>Tapscript is a Taproot-specific script version, so learners need the Taproot spend context before its rule changes make sense.</x:v>
+        <x:v>TapTweak operates on x-only public keys in the Taproot construction.</x:v>
       </x:c>
       <x:c r="F30" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G30" s="32" t="str">
-        <x:v>Direct edge keeps the node scoped to the Taproot family without collapsing it into a generic script refresher.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="str">
-        <x:v>custody.psbt</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="B31" s="32" t="str">
-        <x:v>dev.taproot-psbt-fields</x:v>
+        <x:v>protocol.taproot-key-path-spends</x:v>
       </x:c>
       <x:c r="C31" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12346,21 +12644,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E31" s="32" t="str">
-        <x:v>Taproot PSBT fields extend the base PSBT container, so learners need the general workflow and field model before the Taproot additions make sense.</x:v>
+        <x:v>A key-path spend verifies against the tweaked Taproot output key, so learners need the tweak mechanism before the spending mode makes sense.</x:v>
       </x:c>
       <x:c r="F31" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G31" s="32" t="str">
-        <x:v>Direct edge keeps the slice anchored on the generic PSBT exchange model rather than on a narrower implementation variant.</x:v>
+        <x:v>Direct parent keeps the node focused on the spend mode rather than on broad Taproot overview material.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.taptree</x:v>
       </x:c>
       <x:c r="B32" s="32" t="str">
-        <x:v>dev.taproot-psbt-fields</x:v>
+        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
       </x:c>
       <x:c r="C32" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12369,21 +12667,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E32" s="32" t="str">
-        <x:v>These fields carry Taproot-specific keys, scripts, and Merkle-path data, so learners need the Taproot spend model before the PSBT extensions are meaningful.</x:v>
+        <x:v>The inclusion proof only makes sense after the learner understands the TapTree structure.</x:v>
       </x:c>
       <x:c r="F32" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G32" s="32" t="str">
-        <x:v>The direct dev.psbt-v2 edge was intentionally dropped because BIP371 applies to PSBTv0 and PSBTv2.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="32" t="str">
-        <x:v>protocol.softfork-hardfork</x:v>
+        <x:v>protocol.taptree</x:v>
       </x:c>
       <x:c r="B33" s="32" t="str">
-        <x:v>protocol.accidental-confiscation</x:v>
+        <x:v>protocol.huffman-optimized-taptrees</x:v>
       </x:c>
       <x:c r="C33" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12392,21 +12690,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E33" s="32" t="str">
-        <x:v>Accidental confiscation is a failure mode caused by new soft-fork restrictions, so learners need the soft-fork compatibility model before the risk is intelligible.</x:v>
+        <x:v>Huffman optimization is a refinement of how TapTree leaves are arranged.</x:v>
       </x:c>
       <x:c r="F33" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G33" s="32" t="str">
-        <x:v>Direct edge chosen over chain-split-risk and standardness-policy because those branches add context but are not required for the core failure mode.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="32" t="str">
-        <x:v>protocol.fee-market</x:v>
+        <x:v>protocol.softfork-hardfork</x:v>
       </x:c>
       <x:c r="B34" s="32" t="str">
-        <x:v>custody.coin-selection</x:v>
+        <x:v>protocol.chain-split-risk</x:v>
       </x:c>
       <x:c r="C34" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12415,21 +12713,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E34" s="32" t="str">
-        <x:v>Wallets choose different UTXO sets partly to minimize transaction size and fee cost, so fee pressure is a direct part of the concept.</x:v>
+        <x:v>Split risk is a downstream consequence of incompatible upgrade paths, so learners should understand the compatibility boundary first.</x:v>
       </x:c>
       <x:c r="F34" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G34" s="32" t="str">
-        <x:v>Direct edge keeps the node connected to transaction-cost tradeoffs rather than only to wallet UX.</x:v>
+        <x:v>Direct edge chosen over activation-history case studies because those are downstream examples, not prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B35" s="32" t="str">
-        <x:v>protocol.change-outputs</x:v>
+        <x:v>protocol.tapscript</x:v>
       </x:c>
       <x:c r="C35" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12438,21 +12736,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E35" s="32" t="str">
-        <x:v>Change is a specific kind of transaction output, so learners need the basic output and spendability model before the leftover-value pattern makes sense.</x:v>
+        <x:v>Tapscript is a Taproot-specific script version, so learners need the Taproot spend context before its rule changes make sense.</x:v>
       </x:c>
       <x:c r="F35" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G35" s="32" t="str">
-        <x:v>Direct edge keeps the node between raw output structure and the later wallet-decision branch.</x:v>
+        <x:v>Direct edge keeps the node scoped to the Taproot family without collapsing it into a generic script refresher.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>custody.psbt</x:v>
       </x:c>
       <x:c r="B36" s="32" t="str">
-        <x:v>dev.taproot-descriptors</x:v>
+        <x:v>dev.taproot-psbt-fields</x:v>
       </x:c>
       <x:c r="C36" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12461,13 +12759,13 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E36" s="32" t="str">
-        <x:v>Taproot descriptors extend the general descriptor grammar, so learners need the base descriptor model before the tr() specialization makes sense.</x:v>
+        <x:v>Taproot PSBT fields extend the base PSBT container, so learners need the general workflow and field model before the Taproot additions make sense.</x:v>
       </x:c>
       <x:c r="F36" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G36" s="32" t="str">
-        <x:v>Direct edge keeps the node scoped to descriptor structure instead of wallet import behavior.</x:v>
+        <x:v>Direct edge keeps the slice anchored on the generic PSBT exchange model rather than on a narrower implementation variant.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -12475,7 +12773,7 @@
         <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B37" s="32" t="str">
-        <x:v>dev.taproot-descriptors</x:v>
+        <x:v>dev.taproot-psbt-fields</x:v>
       </x:c>
       <x:c r="C37" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12484,21 +12782,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E37" s="32" t="str">
-        <x:v>The tr() descriptor exists specifically to encode P2TR outputs and optional Taproot script-path commitments, so learners need the Taproot output model first.</x:v>
+        <x:v>These fields carry Taproot-specific keys, scripts, and Merkle-path data, so learners need the Taproot spend model before the PSBT extensions are meaningful.</x:v>
       </x:c>
       <x:c r="F37" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G37" s="32" t="str">
-        <x:v>Direct edge keeps the node grounded in Taproot output semantics rather than in generic descriptor syntax alone.</x:v>
+        <x:v>The direct dev.psbt-v2 edge was intentionally dropped because BIP371 applies to PSBTv0 and PSBTv2.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="32" t="str">
-        <x:v>protocol.transaction-pinning</x:v>
+        <x:v>protocol.softfork-hardfork</x:v>
       </x:c>
       <x:c r="B38" s="32" t="str">
-        <x:v>protocol.version-3-transaction-relay</x:v>
+        <x:v>protocol.accidental-confiscation</x:v>
       </x:c>
       <x:c r="C38" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12507,21 +12805,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E38" s="32" t="str">
-        <x:v>Version 3 relay is a targeted policy response to transaction pinning, so learners should understand the attack class before the mitigation.</x:v>
+        <x:v>Accidental confiscation is a failure mode caused by new soft-fork restrictions, so learners need the soft-fork compatibility model before the risk is intelligible.</x:v>
       </x:c>
       <x:c r="F38" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G38" s="32" t="str">
-        <x:v>Direct edge chosen over package-relay because the pinning problem is the narrower immediate teaching need.</x:v>
+        <x:v>Direct edge chosen over chain-split-risk and standardness-policy because those branches add context but are not required for the core failure mode.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="32" t="str">
-        <x:v>fundamentals.trustlessness</x:v>
+        <x:v>protocol.fee-market</x:v>
       </x:c>
       <x:c r="B39" s="32" t="str">
-        <x:v>fundamentals.validation-sovereignty</x:v>
+        <x:v>custody.coin-selection</x:v>
       </x:c>
       <x:c r="C39" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12530,21 +12828,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E39" s="32" t="str">
-        <x:v>Validation sovereignty is an applied consequence of trustlessness and verification culture.</x:v>
+        <x:v>Wallets choose different UTXO sets partly to minimize transaction size and fee cost, so fee pressure is a direct part of the concept.</x:v>
       </x:c>
       <x:c r="F39" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G39" s="32" t="str">
-        <x:v>Bridge edge inferred from philosophy sequencing.</x:v>
+        <x:v>Direct edge keeps the node connected to transaction-cost tradeoffs rather than only to wallet UX.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="32" t="str">
-        <x:v>ops.run-full-node</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B40" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>protocol.change-outputs</x:v>
       </x:c>
       <x:c r="C40" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12553,21 +12851,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E40" s="32" t="str">
-        <x:v>Learners need the full-node baseline before they can understand which validation guarantees a light client gives up.</x:v>
+        <x:v>Change is a specific kind of transaction output, so learners need the basic output and spendability model before the leftover-value pattern makes sense.</x:v>
       </x:c>
       <x:c r="F40" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G40" s="32" t="str">
-        <x:v>Bridge edge inferred from full-node versus lightweight-client contrast.</x:v>
+        <x:v>Direct edge keeps the node between raw output structure and the later wallet-decision branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32" t="str">
-        <x:v>protocol.compact-block-filters</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B41" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>dev.taproot-descriptors</x:v>
       </x:c>
       <x:c r="C41" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12576,21 +12874,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E41" s="32" t="str">
-        <x:v>Compact block filters provide the modern filtered-client mechanism that anchors the trust-model comparison.</x:v>
+        <x:v>Taproot descriptors extend the general descriptor grammar, so learners need the base descriptor model before the tr() specialization makes sense.</x:v>
       </x:c>
       <x:c r="F41" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G41" s="32" t="str">
-        <x:v>Kept additive and conceptual instead of rewiring older light-client mechanism leaves in the same slice.</x:v>
+        <x:v>Direct edge keeps the node scoped to descriptor structure instead of wallet import behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="32" t="str">
-        <x:v>fundamentals.validation-sovereignty</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B42" s="32" t="str">
-        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
+        <x:v>dev.taproot-descriptors</x:v>
       </x:c>
       <x:c r="C42" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12599,21 +12897,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E42" s="32" t="str">
-        <x:v>The comparison only matters once the learner understands why self-validation is valuable in the first place.</x:v>
+        <x:v>The tr() descriptor exists specifically to encode P2TR outputs and optional Taproot script-path commitments, so learners need the Taproot output model first.</x:v>
       </x:c>
       <x:c r="F42" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G42" s="32" t="str">
-        <x:v>User-facing prerequisite edge for the wallet-mode decision.</x:v>
+        <x:v>Direct edge keeps the node grounded in Taproot output semantics rather than in generic descriptor syntax alone.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>protocol.transaction-pinning</x:v>
       </x:c>
       <x:c r="B43" s="32" t="str">
-        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
+        <x:v>protocol.version-3-transaction-relay</x:v>
       </x:c>
       <x:c r="C43" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12622,21 +12920,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E43" s="32" t="str">
-        <x:v>Learners need the mechanism-level trust tradeoffs before comparing full-node wallets with lightweight clients.</x:v>
+        <x:v>Version 3 relay is a targeted policy response to transaction pinning, so learners should understand the attack class before the mitigation.</x:v>
       </x:c>
       <x:c r="F43" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G43" s="32" t="str">
-        <x:v>First downstream consumer for the light-client trust branch.</x:v>
+        <x:v>Direct edge chosen over package-relay because the pinning problem is the narrower immediate teaching need.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>fundamentals.trustlessness</x:v>
       </x:c>
       <x:c r="B44" s="32" t="str">
-        <x:v>protocol.p2pk</x:v>
+        <x:v>fundamentals.validation-sovereignty</x:v>
       </x:c>
       <x:c r="C44" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12645,21 +12943,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E44" s="32" t="str">
-        <x:v>P2PK is a concrete legacy script template, so learners first need the locking and unlocking model from Bitcoin Script.</x:v>
+        <x:v>Validation sovereignty is an applied consequence of trustlessness and verification culture.</x:v>
       </x:c>
       <x:c r="F44" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G44" s="32" t="str">
-        <x:v>Chosen as the first script-history leaf from Decoding after dedupe and direct-edge review.</x:v>
+        <x:v>Bridge edge inferred from philosophy sequencing.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="32" t="str">
-        <x:v>fundamentals.schnorr-signatures</x:v>
+        <x:v>ops.run-full-node</x:v>
       </x:c>
       <x:c r="B45" s="32" t="str">
-        <x:v>security.nonce-reuse-attack</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="C45" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12668,21 +12966,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E45" s="32" t="str">
-        <x:v>The nonce-reuse failure only makes sense after the learner understands the Schnorr signing flow that produces the nonce and signature pair.</x:v>
+        <x:v>Learners need the full-node baseline before they can understand which validation guarantees a light client gives up.</x:v>
       </x:c>
       <x:c r="F45" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G45" s="32" t="str">
-        <x:v>Chosen as a narrow additive security slice without bundling it to custody-side defenses.</x:v>
+        <x:v>Bridge edge inferred from full-node versus lightweight-client contrast.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="32" t="str">
-        <x:v>protocol.p2pk</x:v>
+        <x:v>protocol.compact-block-filters</x:v>
       </x:c>
       <x:c r="B46" s="32" t="str">
-        <x:v>protocol.p2pkh</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="C46" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12691,21 +12989,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E46" s="32" t="str">
-        <x:v>P2PKH is easiest to understand as the hashed-public-key refinement of a direct public-key output.</x:v>
+        <x:v>Compact block filters provide the modern filtered-client mechanism that anchors the trust-model comparison.</x:v>
       </x:c>
       <x:c r="F46" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G46" s="32" t="str">
-        <x:v>Chosen to preserve the output-template ladder without repeating the broader Script prerequisite directly.</x:v>
+        <x:v>Kept additive and conceptual instead of rewiring older light-client mechanism leaves in the same slice.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>fundamentals.validation-sovereignty</x:v>
       </x:c>
       <x:c r="B47" s="32" t="str">
-        <x:v>protocol.p2pkh</x:v>
+        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
       </x:c>
       <x:c r="C47" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12714,21 +13012,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E47" s="32" t="str">
-        <x:v>Hash-based locking only makes sense once the learner understands what a hash commits to and why it can stand in for the public key until spend time.</x:v>
+        <x:v>The comparison only matters once the learner understands why self-validation is valuable in the first place.</x:v>
       </x:c>
       <x:c r="F47" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G47" s="32" t="str">
-        <x:v>Required to keep the node about public-key hashing rather than just script syntax.</x:v>
+        <x:v>User-facing prerequisite edge for the wallet-mode decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="B48" s="32" t="str">
-        <x:v>protocol.op-checkmultisig</x:v>
+        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
       </x:c>
       <x:c r="C48" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12737,21 +13035,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E48" s="32" t="str">
-        <x:v>OP_CHECKMULTISIG is an opcode-level script mechanic, so learners first need the general Script model and stack execution basics.</x:v>
+        <x:v>Learners need the mechanism-level trust tradeoffs before comparing full-node wallets with lightweight clients.</x:v>
       </x:c>
       <x:c r="F48" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G48" s="32" t="str">
-        <x:v>Chosen as the mechanism bridge before protocol.p2ms.</x:v>
+        <x:v>First downstream consumer for the light-client trust branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="32" t="str">
-        <x:v>protocol.op-checkmultisig</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B49" s="32" t="str">
-        <x:v>protocol.p2ms</x:v>
+        <x:v>protocol.p2pk</x:v>
       </x:c>
       <x:c r="C49" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12760,21 +13058,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E49" s="32" t="str">
-        <x:v>Bare multisig is the concrete locking template built from OP_CHECKMULTISIG, so the opcode is the clean direct parent once introduced.</x:v>
+        <x:v>P2PK is a concrete legacy script template, so learners first need the locking and unlocking model from Bitcoin Script.</x:v>
       </x:c>
       <x:c r="F49" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G49" s="32" t="str">
-        <x:v>Replaces the earlier curricular and wallet-semantic parent candidates.</x:v>
+        <x:v>Chosen as the first script-history leaf from Decoding after dedupe and direct-edge review.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="32" t="str">
-        <x:v>protocol.p2ms</x:v>
+        <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="B50" s="32" t="str">
-        <x:v>protocol.bare-multisig-standardness</x:v>
+        <x:v>security.nonce-reuse-attack</x:v>
       </x:c>
       <x:c r="C50" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12783,21 +13081,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E50" s="32" t="str">
-        <x:v>The relay treatment only makes sense once the learner understands what a bare multisig output actually is on-chain.</x:v>
+        <x:v>The nonce-reuse failure only makes sense after the learner understands the Schnorr signing flow that produces the nonce and signature pair.</x:v>
       </x:c>
       <x:c r="F50" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G50" s="32" t="str">
-        <x:v>Policy leaf anchored on the specific legacy script template it constrains.</x:v>
+        <x:v>Chosen as a narrow additive security slice without bundling it to custody-side defenses.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="32" t="str">
-        <x:v>protocol.standardness-policy</x:v>
+        <x:v>protocol.p2pk</x:v>
       </x:c>
       <x:c r="B51" s="32" t="str">
-        <x:v>protocol.bare-multisig-standardness</x:v>
+        <x:v>protocol.p2pkh</x:v>
       </x:c>
       <x:c r="C51" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12806,21 +13104,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E51" s="32" t="str">
-        <x:v>This node is a concrete application of standard transaction policy, so the general standardness concept should come first.</x:v>
+        <x:v>P2PKH is easiest to understand as the hashed-public-key refinement of a direct public-key output.</x:v>
       </x:c>
       <x:c r="F51" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G51" s="32" t="str">
-        <x:v>Policy-boundary prerequisite inherited through the existing mempool-policy branch.</x:v>
+        <x:v>Chosen to preserve the output-template ladder without repeating the broader Script prerequisite directly.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B52" s="32" t="str">
-        <x:v>dev.scriptpubkeymanagers</x:v>
+        <x:v>protocol.p2pkh</x:v>
       </x:c>
       <x:c r="C52" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12829,21 +13127,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E52" s="32" t="str">
-        <x:v>Modern descriptor wallets hand descriptor-backed script templates to dedicated managers, so learners need the descriptor model before the SPKM boundary makes sense.</x:v>
+        <x:v>Hash-based locking only makes sense once the learner understands what a hash commits to and why it can stand in for the public key until spend time.</x:v>
       </x:c>
       <x:c r="F52" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-wallet</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G52" s="32" t="str">
-        <x:v>Direct edge distinguishes the Core wallet abstraction from descriptor syntax without collapsing the two concepts into one node.</x:v>
+        <x:v>Required to keep the node about public-key hashing rather than just script syntax.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="32" t="str">
-        <x:v>protocol.mempool</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B53" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>protocol.op-checkmultisig</x:v>
       </x:c>
       <x:c r="C53" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12852,21 +13150,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E53" s="32" t="str">
-        <x:v>The unbroadcast set is a mempool-owned data structure, so learners need the local unconfirmed transaction pool model before this narrower tracking mechanism makes sense.</x:v>
+        <x:v>OP_CHECKMULTISIG is an opcode-level script mechanic, so learners first need the general Script model and stack execution basics.</x:v>
       </x:c>
       <x:c r="F53" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G53" s="32" t="str">
-        <x:v>Direct edge keeps the concept scoped to local transaction state rather than broader relay policy.</x:v>
+        <x:v>Chosen as the mechanism bridge before protocol.p2ms.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="32" t="str">
-        <x:v>protocol.transaction-relay-inv-getdata</x:v>
+        <x:v>protocol.op-checkmultisig</x:v>
       </x:c>
       <x:c r="B54" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>protocol.p2ms</x:v>
       </x:c>
       <x:c r="C54" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12875,21 +13173,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E54" s="32" t="str">
-        <x:v>This set only matters because nodes need to distinguish locally submitted transactions from those later observed through the network relay path and may retry announcing them.</x:v>
+        <x:v>Bare multisig is the concrete locking template built from OP_CHECKMULTISIG, so the opcode is the clean direct parent once introduced.</x:v>
       </x:c>
       <x:c r="F54" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G54" s="32" t="str">
-        <x:v>Direct edge ties the mechanism to network propagation confirmation and rebroadcast attempts.</x:v>
+        <x:v>Replaces the earlier curricular and wallet-semantic parent candidates.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="32" t="str">
-        <x:v>privacy.address-reuse</x:v>
+        <x:v>protocol.p2ms</x:v>
       </x:c>
       <x:c r="B55" s="32" t="str">
-        <x:v>custody.human-readable-addresses</x:v>
+        <x:v>protocol.bare-multisig-standardness</x:v>
       </x:c>
       <x:c r="C55" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12898,21 +13196,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E55" s="32" t="str">
-        <x:v>A major design constraint is that reusable human-readable handles can worsen privacy unless they resolve to reusable payment mechanisms or rotate safely, so learners need the address-reuse problem first.</x:v>
+        <x:v>The relay treatment only makes sense once the learner understands what a bare multisig output actually is on-chain.</x:v>
       </x:c>
       <x:c r="F55" s="32" t="str">
-        <x:v>source.bitcoin-design-payment-formats</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G55" s="32" t="str">
-        <x:v>Direct edge captures the main privacy tradeoff without forcing downstream protocol-specific address schemes into prerequisites.</x:v>
+        <x:v>Policy leaf anchored on the specific legacy script template it constrains.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="32" t="str">
-        <x:v>custody.output-labeling</x:v>
+        <x:v>protocol.standardness-policy</x:v>
       </x:c>
       <x:c r="B56" s="32" t="str">
-        <x:v>custody.transaction-metadata</x:v>
+        <x:v>protocol.bare-multisig-standardness</x:v>
       </x:c>
       <x:c r="C56" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12921,21 +13219,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E56" s="32" t="str">
-        <x:v>Output labeling already introduces the idea that wallets attach their own context to payments and spendable objects, making it the cleanest direct bridge into broader transaction-level notes, contacts, and portability concerns.</x:v>
+        <x:v>This node is a concrete application of standard transaction policy, so the general standardness concept should come first.</x:v>
       </x:c>
       <x:c r="F56" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G56" s="32" t="str">
-        <x:v>Direct edge distinguishes wider payment-history context from narrower spend-control labels without treating them as unrelated.</x:v>
+        <x:v>Policy-boundary prerequisite inherited through the existing mempool-policy branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B57" s="32" t="str">
-        <x:v>custody.transaction-metadata</x:v>
+        <x:v>dev.scriptpubkeymanagers</x:v>
       </x:c>
       <x:c r="C57" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12944,21 +13242,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E57" s="32" t="str">
-        <x:v>Wallet-added names, notes, and contact links matter partly because transaction history is only pseudonymous and can reveal meaningful patterns when users or tools correlate activity over time.</x:v>
+        <x:v>Modern descriptor wallets hand descriptor-backed script templates to dedicated managers, so learners need the descriptor model before the SPKM boundary makes sense.</x:v>
       </x:c>
       <x:c r="F57" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoin-core-academy-wallet</x:v>
       </x:c>
       <x:c r="G57" s="32" t="str">
-        <x:v>Direct edge keeps the node tied to the privacy and identity meaning of payment history rather than only to generic lifecycle sequencing.</x:v>
+        <x:v>Direct edge distinguishes the Core wallet abstraction from descriptor syntax without collapsing the two concepts into one node.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="32" t="str">
-        <x:v>custody.self-custody</x:v>
+        <x:v>protocol.mempool</x:v>
       </x:c>
       <x:c r="B58" s="32" t="str">
-        <x:v>custody.multiple-wallets</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="C58" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12967,21 +13265,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E58" s="32" t="str">
-        <x:v>Deliberately separating funds across different wallet buckets is a custody decision, so learners need the base self-custody responsibility model before the organizational pattern makes sense.</x:v>
+        <x:v>The unbroadcast set is a mempool-owned data structure, so learners need the local unconfirmed transaction pool model before this narrower tracking mechanism makes sense.</x:v>
       </x:c>
       <x:c r="F58" s="32" t="str">
-        <x:v>source.bitcoin-design-multiple-wallets</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G58" s="32" t="str">
-        <x:v>Kept the direct parent at the responsibility-model layer; multisig, watch-only, and HD account structures remain examples or implementation details rather than prerequisites.</x:v>
+        <x:v>Direct edge keeps the concept scoped to local transaction state rather than broader relay policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="32" t="str">
-        <x:v>custody.hardware-wallets</x:v>
+        <x:v>protocol.transaction-relay-inv-getdata</x:v>
       </x:c>
       <x:c r="B59" s="32" t="str">
-        <x:v>custody.progressive-security</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="C59" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12990,21 +13288,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E59" s="32" t="str">
-        <x:v>One of the core upgrade steps in the reference design is moving from default low-friction storage to an external signing device, so learners need the hardware-signing model before the staged-upgrade pattern makes sense.</x:v>
+        <x:v>This set only matters because nodes need to distinguish locally submitted transactions from those later observed through the network relay path and may retry announcing them.</x:v>
       </x:c>
       <x:c r="F59" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G59" s="32" t="str">
-        <x:v>Direct edge captures the mid-tier upgrade target without treating cloud backup itself as the core concept.</x:v>
+        <x:v>Direct edge ties the mechanism to network propagation confirmation and rebroadcast attempts.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>privacy.address-reuse</x:v>
       </x:c>
       <x:c r="B60" s="32" t="str">
-        <x:v>custody.progressive-security</x:v>
+        <x:v>custody.human-readable-addresses</x:v>
       </x:c>
       <x:c r="C60" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13013,21 +13311,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E60" s="32" t="str">
-        <x:v>The higher-security end of the progression moves into 2-of-3 and 3-of-5 multi-key schemes, so learners need the multisig model before they can reason about why and when a wallet should escalate there.</x:v>
+        <x:v>A major design constraint is that reusable human-readable handles can worsen privacy unless they resolve to reusable payment mechanisms or rotate safely, so learners need the address-reuse problem first.</x:v>
       </x:c>
       <x:c r="F60" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoin-design-payment-formats</x:v>
       </x:c>
       <x:c r="G60" s="32" t="str">
-        <x:v>Direct edge captures the high-assurance destination of the progression rather than a specific product flow.</x:v>
+        <x:v>Direct edge captures the main privacy tradeoff without forcing downstream protocol-specific address schemes into prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>custody.output-labeling</x:v>
       </x:c>
       <x:c r="B61" s="32" t="str">
-        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
+        <x:v>custody.transaction-metadata</x:v>
       </x:c>
       <x:c r="C61" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13036,13 +13334,13 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E61" s="32" t="str">
-        <x:v>Rebroadcast privacy builds directly on the local-node distinction between transactions merely accepted into the mempool and transactions known to have propagated, which is exactly the gap the unbroadcast set tracks.</x:v>
+        <x:v>Output labeling already introduces the idea that wallets attach their own context to payments and spendable objects, making it the cleanest direct bridge into broader transaction-level notes, contacts, and portability concerns.</x:v>
       </x:c>
       <x:c r="F61" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="G61" s="32" t="str">
-        <x:v>Direct parent keeps the slice on the local tracking mechanism rather than reintroducing generic relay ancestors.</x:v>
+        <x:v>Direct edge distinguishes wider payment-history context from narrower spend-control labels without treating them as unrelated.</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -13050,7 +13348,7 @@
         <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B62" s="32" t="str">
-        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
+        <x:v>custody.transaction-metadata</x:v>
       </x:c>
       <x:c r="C62" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13059,21 +13357,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E62" s="32" t="str">
-        <x:v>Different rebroadcast patterns matter because observers can correlate network behavior with public transaction history and infer likely origin, so learners need the pseudonymity and linkage problem first.</x:v>
+        <x:v>Wallet-added names, notes, and contact links matter partly because transaction history is only pseudonymous and can reveal meaningful patterns when users or tools correlate activity over time.</x:v>
       </x:c>
       <x:c r="F62" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="G62" s="32" t="str">
-        <x:v>Direct parent keeps the node focused on why relay-side origin leakage matters, not just how rebroadcast code works.</x:v>
+        <x:v>Direct edge keeps the node tied to the privacy and identity meaning of payment history rather than only to generic lifecycle sequencing.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="32" t="str">
-        <x:v>protocol.segregated-witness</x:v>
+        <x:v>custody.self-custody</x:v>
       </x:c>
       <x:c r="B63" s="32" t="str">
-        <x:v>protocol.txid-vs-wtxid</x:v>
+        <x:v>custody.multiple-wallets</x:v>
       </x:c>
       <x:c r="C63" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13082,21 +13380,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E63" s="32" t="str">
-        <x:v>The identifier split only exists because SegWit introduces a witness-inclusive serialization alongside the legacy serialization, so learners need the SegWit structure change before the two IDs make sense.</x:v>
+        <x:v>Deliberately separating funds across different wallet buckets is a custody decision, so learners need the base self-custody responsibility model before the organizational pattern makes sense.</x:v>
       </x:c>
       <x:c r="F63" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-multiple-wallets</x:v>
       </x:c>
       <x:c r="G63" s="32" t="str">
-        <x:v>Direct parent keeps the bridge on the serialization distinction instead of reintroducing downstream relay consequences.</x:v>
+        <x:v>Kept the direct parent at the responsibility-model layer; multisig, watch-only, and HD account structures remain examples or implementation details rather than prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="32" t="str">
-        <x:v>protocol.txid-vs-wtxid</x:v>
+        <x:v>custody.hardware-wallets</x:v>
       </x:c>
       <x:c r="B64" s="32" t="str">
-        <x:v>protocol.wtxid-relay-bip339</x:v>
+        <x:v>custody.progressive-security</x:v>
       </x:c>
       <x:c r="C64" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13105,21 +13403,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E64" s="32" t="str">
-        <x:v>WTXID relay is specifically the choice to announce and request witness-bearing transactions by wtxid instead of txid, so the learner should understand the two identifier forms before the relay mode change.</x:v>
+        <x:v>One of the core upgrade steps in the reference design is moving from default low-friction storage to an external signing device, so learners need the hardware-signing model before the staged-upgrade pattern makes sense.</x:v>
       </x:c>
       <x:c r="F64" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="G64" s="32" t="str">
-        <x:v>Added as a graph bridge so the existing relay node no longer has to explain the identifier distinction internally.</x:v>
+        <x:v>Direct edge captures the mid-tier upgrade target without treating cloud backup itself as the core concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="32" t="str">
-        <x:v>fundamentals.schnorr-signatures</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B65" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>custody.progressive-security</x:v>
       </x:c>
       <x:c r="C65" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13128,21 +13426,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E65" s="32" t="str">
-        <x:v>MuSig is a Schnorr aggregation protocol, so learners need the underlying Schnorr key and signature model before the combined-key protocol makes sense.</x:v>
+        <x:v>The higher-security end of the progression moves into 2-of-3 and 3-of-5 multi-key schemes, so learners need the multisig model before they can reason about why and when a wallet should escalate there.</x:v>
       </x:c>
       <x:c r="F65" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="G65" s="32" t="str">
-        <x:v>Direct parent kept narrow; wallet-level multisig and Taproot remain context rather than prerequisites.</x:v>
+        <x:v>Direct edge captures the high-assurance destination of the progression rather than a specific product flow.</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="B66" s="32" t="str">
-        <x:v>dev.descriptor-wallet-policies</x:v>
+        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
       </x:c>
       <x:c r="C66" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13151,21 +13449,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E66" s="32" t="str">
-        <x:v>Wallet policies are built as descriptor templates, so the base descriptor language and template structure must come first.</x:v>
+        <x:v>Rebroadcast privacy builds directly on the local-node distinction between transactions merely accepted into the mempool and transactions known to have propagated, which is exactly the gap the unbroadcast set tracks.</x:v>
       </x:c>
       <x:c r="F66" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G66" s="32" t="str">
-        <x:v>Direct parent kept above import or signer flows because the node is about the representation itself.</x:v>
+        <x:v>Direct parent keeps the slice on the local tracking mechanism rather than reintroducing generic relay ancestors.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="32" t="str">
-        <x:v>dev.bip32</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B67" s="32" t="str">
-        <x:v>dev.descriptor-wallet-policies</x:v>
+        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
       </x:c>
       <x:c r="C67" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13174,21 +13472,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E67" s="32" t="str">
-        <x:v>BIP388 key information items package xpubs and derivation origins, so learners need the HD derivation model before the portable wallet-policy format makes sense.</x:v>
+        <x:v>Different rebroadcast patterns matter because observers can correlate network behavior with public transaction history and infer likely origin, so learners need the pseudonymity and linkage problem first.</x:v>
       </x:c>
       <x:c r="F67" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G67" s="32" t="str">
-        <x:v>Non-redundant alongside dev.descriptors because neither concept implies the other in the current graph.</x:v>
+        <x:v>Direct parent keeps the node focused on why relay-side origin leakage matters, not just how rebroadcast code works.</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>protocol.segregated-witness</x:v>
       </x:c>
       <x:c r="B68" s="32" t="str">
-        <x:v>dev.descriptors-in-psbt</x:v>
+        <x:v>protocol.txid-vs-wtxid</x:v>
       </x:c>
       <x:c r="C68" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13197,21 +13495,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E68" s="32" t="str">
-        <x:v>The node is about carrying descriptor information during transaction coordination, so learners need the descriptor syntax and script-template model first.</x:v>
+        <x:v>The identifier split only exists because SegWit introduces a witness-inclusive serialization alongside the legacy serialization, so learners need the SegWit structure change before the two IDs make sense.</x:v>
       </x:c>
       <x:c r="F68" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G68" s="32" t="str">
-        <x:v>Direct parent kept at the representation layer rather than the wallet-policy or taproot-specific refinements.</x:v>
+        <x:v>Direct parent keeps the bridge on the serialization distinction instead of reintroducing downstream relay consequences.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="32" t="str">
-        <x:v>custody.psbt</x:v>
+        <x:v>protocol.txid-vs-wtxid</x:v>
       </x:c>
       <x:c r="B69" s="32" t="str">
-        <x:v>dev.descriptors-in-psbt</x:v>
+        <x:v>protocol.wtxid-relay-bip339</x:v>
       </x:c>
       <x:c r="C69" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13220,21 +13518,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E69" s="32" t="str">
-        <x:v>Descriptor-aware exchange only makes sense after the learner understands the general PSBT coordination workflow that transports signing-related data between tools.</x:v>
+        <x:v>WTXID relay is specifically the choice to announce and request witness-bearing transactions by wtxid instead of txid, so the learner should understand the two identifier forms before the relay mode change.</x:v>
       </x:c>
       <x:c r="F69" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G69" s="32" t="str">
-        <x:v>Direct parent kept at the base PSBT workflow level instead of requiring later version-specific extensions.</x:v>
+        <x:v>Added as a graph bridge so the existing relay node no longer has to explain the identifier distinction internally.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="B70" s="32" t="str">
-        <x:v>custody.degrading-multisig</x:v>
+        <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="C70" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13243,21 +13541,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E70" s="32" t="str">
-        <x:v>The policy only makes sense once the learner understands ordinary multisig threshold custody and why signers can be split into live and backup sets.</x:v>
+        <x:v>MuSig is a Schnorr aggregation protocol, so learners need the underlying Schnorr key and signature model before the combined-key protocol makes sense.</x:v>
       </x:c>
       <x:c r="F70" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G70" s="32" t="str">
-        <x:v>Direct custody parent for the signer-threshold side of the construction.</x:v>
+        <x:v>Direct parent kept narrow; wallet-level multisig and Taproot remain context rather than prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="32" t="str">
-        <x:v>protocol.timelocks</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B71" s="32" t="str">
-        <x:v>custody.degrading-multisig</x:v>
+        <x:v>dev.descriptor-wallet-policies</x:v>
       </x:c>
       <x:c r="C71" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13266,21 +13564,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E71" s="32" t="str">
-        <x:v>The degrading policy activates its weaker backup path only after a timeout, so timelock semantics are a direct part of the construction.</x:v>
+        <x:v>Wallet policies are built as descriptor templates, so the base descriptor language and template structure must come first.</x:v>
       </x:c>
       <x:c r="F71" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G71" s="32" t="str">
-        <x:v>Needed alongside custody.multisig because the learner must understand the temporal rule, not just the signer policy.</x:v>
+        <x:v>Direct parent kept above import or signer flows because the node is about the representation itself.</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="32" t="str">
-        <x:v>protocol.block-weight-vbytes</x:v>
+        <x:v>dev.bip32</x:v>
       </x:c>
       <x:c r="B72" s="32" t="str">
-        <x:v>protocol.fee-calculation</x:v>
+        <x:v>dev.descriptor-wallet-policies</x:v>
       </x:c>
       <x:c r="C72" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13289,21 +13587,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E72" s="32" t="str">
-        <x:v>Understanding whether an absolute fee is high or low requires relating it to the blockspace pricing unit, so learners need weight and virtual bytes before fee calculation is fully meaningful in practice.</x:v>
+        <x:v>BIP388 key information items package xpubs and derivation origins, so learners need the HD derivation model before the portable wallet-policy format makes sense.</x:v>
       </x:c>
       <x:c r="F72" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G72" s="32" t="str">
-        <x:v>Direct parent keeps the node at the mechanism layer without drifting into broader fee-market competition.</x:v>
+        <x:v>Non-redundant alongside dev.descriptors because neither concept implies the other in the current graph.</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B73" s="32" t="str">
-        <x:v>protocol.bech32m-addresses</x:v>
+        <x:v>dev.descriptors-in-psbt</x:v>
       </x:c>
       <x:c r="C73" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13312,21 +13610,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E73" s="32" t="str">
-        <x:v>Bech32m is an address-encoding format, so learners need the general relationship between addresses, script templates, and spendability before the newer checksum format is meaningful.</x:v>
+        <x:v>The node is about carrying descriptor information during transaction coordination, so learners need the descriptor syntax and script-template model first.</x:v>
       </x:c>
       <x:c r="F73" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G73" s="32" t="str">
-        <x:v>Direct parent keeps the node on encoding semantics rather than on raw string-format trivia.</x:v>
+        <x:v>Direct parent kept at the representation layer rather than the wallet-policy or taproot-specific refinements.</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>custody.psbt</x:v>
       </x:c>
       <x:c r="B74" s="32" t="str">
-        <x:v>protocol.bech32m-addresses</x:v>
+        <x:v>dev.descriptors-in-psbt</x:v>
       </x:c>
       <x:c r="C74" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13335,21 +13633,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E74" s="32" t="str">
-        <x:v>Bech32m became necessary for witness version 1 and higher, and Taproot is the first major deployed witness-v1 use case, so learners need that upgrade context before the format distinction makes sense.</x:v>
+        <x:v>Descriptor-aware exchange only makes sense after the learner understands the general PSBT coordination workflow that transports signing-related data between tools.</x:v>
       </x:c>
       <x:c r="F74" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G74" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored on the practical protocol transition that exposed Bech32m to users.</x:v>
+        <x:v>Direct parent kept at the base PSBT workflow level instead of requiring later version-specific extensions.</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B75" s="32" t="str">
-        <x:v>protocol.script-execution-stack</x:v>
+        <x:v>custody.degrading-multisig</x:v>
       </x:c>
       <x:c r="C75" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13358,21 +13656,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E75" s="32" t="str">
-        <x:v>The stack execution model is the direct mechanism by which Bitcoin Script evaluates spending conditions, so learners need the umbrella Script concept before drilling into stack behavior.</x:v>
+        <x:v>The policy only makes sense once the learner understands ordinary multisig threshold custody and why signers can be split into live and backup sets.</x:v>
       </x:c>
       <x:c r="F75" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G75" s="32" t="str">
-        <x:v>Direct parent positions the node as the conceptual middle layer between Script and opcode-specific leaves.</x:v>
+        <x:v>Direct custody parent for the signer-threshold side of the construction.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="32" t="str">
-        <x:v>lightning.commitment-transactions</x:v>
+        <x:v>protocol.timelocks</x:v>
       </x:c>
       <x:c r="B76" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>custody.degrading-multisig</x:v>
       </x:c>
       <x:c r="C76" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13381,21 +13679,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E76" s="32" t="str">
-        <x:v>Per-commitment secrets are generated for each new commitment state, so learners need the commitment-transaction model before the secret-rotation mechanism makes sense.</x:v>
+        <x:v>The degrading policy activates its weaker backup path only after a timeout, so timelock semantics are a direct part of the construction.</x:v>
       </x:c>
       <x:c r="F76" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G76" s="32" t="str">
-        <x:v>Direct parent keeps the node on state evolution rather than on later punishment or watchtower behavior.</x:v>
+        <x:v>Needed alongside custody.multisig because the learner must understand the temporal rule, not just the signer policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>protocol.block-weight-vbytes</x:v>
       </x:c>
       <x:c r="B77" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>protocol.fee-calculation</x:v>
       </x:c>
       <x:c r="C77" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13404,21 +13702,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E77" s="32" t="str">
-        <x:v>The to_local and to_remote scripts rely on per-state key derivation, revocation keys, and delayed-payment keys, so learners need the per-commitment secret machinery first.</x:v>
+        <x:v>Understanding whether an absolute fee is high or low requires relating it to the blockspace pricing unit, so learners need weight and virtual bytes before fee calculation is fully meaningful in practice.</x:v>
       </x:c>
       <x:c r="F77" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G77" s="32" t="str">
-        <x:v>Direct parent keeps the node at the commitment-key layer instead of collapsing back into the broader commitment-transaction overview.</x:v>
+        <x:v>Direct parent keeps the node at the mechanism layer without drifting into broader fee-market competition.</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="32" t="str">
-        <x:v>protocol.csv-bip112</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B78" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>protocol.bech32m-addresses</x:v>
       </x:c>
       <x:c r="C78" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13427,21 +13725,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E78" s="32" t="str">
-        <x:v>The delayed to_local branch is defined by a CSV-enforced waiting period, so learners need the relative-timelock opcode before the script template makes sense.</x:v>
+        <x:v>Bech32m is an address-encoding format, so learners need the general relationship between addresses, script templates, and spendability before the newer checksum format is meaningful.</x:v>
       </x:c>
       <x:c r="F78" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G78" s="32" t="str">
-        <x:v>Direct parent captures the script-mechanism side of the concept without dragging in broader force-close or HTLC timing behavior.</x:v>
+        <x:v>Direct parent keeps the node on encoding semantics rather than on raw string-format trivia.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="32" t="str">
-        <x:v>protocol.difficulty-adjustment</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B79" s="32" t="str">
-        <x:v>protocol.time-warp-attack</x:v>
+        <x:v>protocol.bech32m-addresses</x:v>
       </x:c>
       <x:c r="C79" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13450,21 +13748,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E79" s="32" t="str">
-        <x:v>The attack only makes sense once learners understand how Bitcoin retargets mining difficulty over long block windows.</x:v>
+        <x:v>Bech32m became necessary for witness version 1 and higher, and Taproot is the first major deployed witness-v1 use case, so learners need that upgrade context before the format distinction makes sense.</x:v>
       </x:c>
       <x:c r="F79" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G79" s="32" t="str">
-        <x:v>Direct parent keeps the exploit tied to the retarget mechanism instead of burying it under generic mining vocabulary.</x:v>
+        <x:v>Direct parent keeps the node anchored on the practical protocol transition that exposed Bech32m to users.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="32" t="str">
-        <x:v>protocol.median-time-past</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B80" s="32" t="str">
-        <x:v>protocol.time-warp-attack</x:v>
+        <x:v>protocol.script-execution-stack</x:v>
       </x:c>
       <x:c r="C80" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13473,21 +13771,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E80" s="32" t="str">
-        <x:v>Learners need the consensus timestamp constraints before they can reason about how miners manipulate time data and where the remaining attack surface lives.</x:v>
+        <x:v>The stack execution model is the direct mechanism by which Bitcoin Script evaluates spending conditions, so learners need the umbrella Script concept before drilling into stack behavior.</x:v>
       </x:c>
       <x:c r="F80" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G80" s="32" t="str">
-        <x:v>Direct parent captures the timestamp-boundary side of the exploit without overloading timelocks or block headers.</x:v>
+        <x:v>Direct parent positions the node as the conceptual middle layer between Script and opcode-specific leaves.</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="32" t="str">
-        <x:v>fundamentals.blind-signatures</x:v>
+        <x:v>lightning.commitment-transactions</x:v>
       </x:c>
       <x:c r="B81" s="32" t="str">
-        <x:v>history.chaumian-ecash</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="C81" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13496,21 +13794,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E81" s="32" t="str">
-        <x:v>Chaumian ecash is defined by using blind signatures to let a mint issue private bearer tokens without seeing the final token contents.</x:v>
+        <x:v>Per-commitment secrets are generated for each new commitment state, so learners need the commitment-transaction model before the secret-rotation mechanism makes sense.</x:v>
       </x:c>
       <x:c r="F81" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G81" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the specific cryptographic mechanism rather than treating it as generic digital-money history.</x:v>
+        <x:v>Direct parent keeps the node on state evolution rather than on later punishment or watchtower behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="32" t="str">
-        <x:v>history.double-spend-problem</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="B82" s="32" t="str">
-        <x:v>history.chaumian-ecash</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="C82" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13519,21 +13817,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E82" s="32" t="str">
-        <x:v>Learners need the unsolved scarcity problem in digital cash before the trusted-mint tradeoff in Chaumian designs becomes meaningful.</x:v>
+        <x:v>The to_local and to_remote scripts rely on per-state key derivation, revocation keys, and delayed-payment keys, so learners need the per-commitment secret machinery first.</x:v>
       </x:c>
       <x:c r="F82" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G82" s="32" t="str">
-        <x:v>Direct parent frames why the system still needed a central operator even though it improved privacy.</x:v>
+        <x:v>Direct parent keeps the node at the commitment-key layer instead of collapsing back into the broader commitment-transaction overview.</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="32" t="str">
-        <x:v>economics.history-of-money</x:v>
+        <x:v>protocol.csv-bip112</x:v>
       </x:c>
       <x:c r="B83" s="32" t="str">
-        <x:v>privacy.secret-right-to-cash</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="C83" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13542,21 +13840,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E83" s="32" t="str">
-        <x:v>The concept depends on understanding how money moved from bearer cash toward mediated account systems, so learners need the long-run monetary history first.</x:v>
+        <x:v>The delayed to_local branch is defined by a CSV-enforced waiting period, so learners need the relative-timelock opcode before the script template makes sense.</x:v>
       </x:c>
       <x:c r="F83" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G83" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the bearer-versus-intermediated payment shift rather than drifting into generic civil-liberties framing.</x:v>
+        <x:v>Direct parent captures the script-mechanism side of the concept without dragging in broader force-close or HTLC timing behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="32" t="str">
-        <x:v>fundamentals.censorship-resistance</x:v>
+        <x:v>protocol.difficulty-adjustment</x:v>
       </x:c>
       <x:c r="B84" s="32" t="str">
-        <x:v>privacy.secret-right-to-cash</x:v>
+        <x:v>protocol.time-warp-attack</x:v>
       </x:c>
       <x:c r="C84" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13565,21 +13863,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E84" s="32" t="str">
-        <x:v>Learners need the general idea that payment systems can exclude or block participants before the loss of private cash as a payment right becomes fully meaningful.</x:v>
+        <x:v>The attack only makes sense once learners understand how Bitcoin retargets mining difficulty over long block windows.</x:v>
       </x:c>
       <x:c r="F84" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G84" s="32" t="str">
-        <x:v>Direct parent captures the exclusion-risk side of the argument without reopening broader compliance or surveillance wrappers.</x:v>
+        <x:v>Direct parent keeps the exploit tied to the retarget mechanism instead of burying it under generic mining vocabulary.</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="32" t="str">
-        <x:v>fundamentals.inflation</x:v>
+        <x:v>protocol.median-time-past</x:v>
       </x:c>
       <x:c r="B85" s="32" t="str">
-        <x:v>economics.ideal-money</x:v>
+        <x:v>protocol.time-warp-attack</x:v>
       </x:c>
       <x:c r="C85" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13588,21 +13886,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E85" s="32" t="str">
-        <x:v>The concept is about minimizing monetary distortion, so learners need to understand how inflation changes purchasing power and price signals first.</x:v>
+        <x:v>Learners need the consensus timestamp constraints before they can reason about how miners manipulate time data and where the remaining attack surface lives.</x:v>
       </x:c>
       <x:c r="F85" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G85" s="32" t="str">
-        <x:v>Direct parent captures the measurement-distortion problem that ideal money is trying to avoid.</x:v>
+        <x:v>Direct parent captures the timestamp-boundary side of the exploit without overloading timelocks or block headers.</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>fundamentals.blind-signatures</x:v>
       </x:c>
       <x:c r="B86" s="32" t="str">
-        <x:v>protocol.bitcoin-uri-bip21</x:v>
+        <x:v>history.chaumian-ecash</x:v>
       </x:c>
       <x:c r="C86" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13611,21 +13909,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E86" s="32" t="str">
-        <x:v>The URI is a wrapper around a payment destination and amount, so learners need the underlying address and output model first.</x:v>
+        <x:v>Chaumian ecash is defined by using blind signatures to let a mint issue private bearer tokens without seeing the final token contents.</x:v>
       </x:c>
       <x:c r="F86" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G86" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the standard request format rather than collapsing it into higher-level wallet UX systems.</x:v>
+        <x:v>Direct parent keeps the node tied to the specific cryptographic mechanism rather than treating it as generic digital-money history.</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="32" t="str">
-        <x:v>dev.bip32</x:v>
+        <x:v>history.double-spend-problem</x:v>
       </x:c>
       <x:c r="B87" s="32" t="str">
-        <x:v>dev.extended-keys</x:v>
+        <x:v>history.chaumian-ecash</x:v>
       </x:c>
       <x:c r="C87" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13634,21 +13932,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E87" s="32" t="str">
-        <x:v>Extended keys are one specific export and branch-derivation surface inside the broader BIP32 HD tree model, so learners need the base tree-derivation mechanics first.</x:v>
+        <x:v>Learners need the unsolved scarcity problem in digital cash before the trusted-mint tradeoff in Chaumian designs becomes meaningful.</x:v>
       </x:c>
       <x:c r="F87" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G87" s="32" t="str">
-        <x:v>Direct parent keeps the node inside the HD derivation branch instead of treating xpub or xprv behavior as only a privacy or operational-wallet concept.</x:v>
+        <x:v>Direct parent frames why the system still needed a central operator even though it improved privacy.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="32" t="str">
-        <x:v>dev.extended-keys</x:v>
+        <x:v>economics.history-of-money</x:v>
       </x:c>
       <x:c r="B88" s="32" t="str">
-        <x:v>dev.hardened-keys</x:v>
+        <x:v>privacy.secret-right-to-cash</x:v>
       </x:c>
       <x:c r="C88" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13657,21 +13955,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E88" s="32" t="str">
-        <x:v>Hardened derivation is a constraint on what an extended public key can derive and on how extended private and public key boundaries behave, so learners need the base xpub/xprv model first.</x:v>
+        <x:v>The concept depends on understanding how money moved from bearer cash toward mediated account systems, so learners need the long-run monetary history first.</x:v>
       </x:c>
       <x:c r="F88" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G88" s="32" t="str">
-        <x:v>Direct parent closes the previously missing branch-level bridge between BIP32 generally and hardened derivation specifically.</x:v>
+        <x:v>Direct parent keeps the node tied to the bearer-versus-intermediated payment shift rather than drifting into generic civil-liberties framing.</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>fundamentals.censorship-resistance</x:v>
       </x:c>
       <x:c r="B89" s="32" t="str">
-        <x:v>protocol.escrow-and-arbitration</x:v>
+        <x:v>privacy.secret-right-to-cash</x:v>
       </x:c>
       <x:c r="C89" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13680,21 +13978,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E89" s="32" t="str">
-        <x:v>The escrow flow depends on understanding how multiple signers can authorize one spend and why a 2-of-3 threshold changes trust assumptions between buyer, seller, and arbitrator.</x:v>
+        <x:v>Learners need the general idea that payment systems can exclude or block participants before the loss of private cash as a payment right becomes fully meaningful.</x:v>
       </x:c>
       <x:c r="F89" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G89" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the threshold-signing contract pattern instead of treating it as generic dispute-resolution theory.</x:v>
+        <x:v>Direct parent captures the exclusion-risk side of the argument without reopening broader compliance or surveillance wrappers.</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="32" t="str">
-        <x:v>protocol.pay-to-script-hash</x:v>
+        <x:v>fundamentals.inflation</x:v>
       </x:c>
       <x:c r="B90" s="32" t="str">
-        <x:v>protocol.escrow-and-arbitration</x:v>
+        <x:v>economics.ideal-money</x:v>
       </x:c>
       <x:c r="C90" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13703,21 +14001,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E90" s="32" t="str">
-        <x:v>The contract uses a P2SH redeem script to hide the multisig spending conditions until spend time, so learners need the P2SH wrapper first.</x:v>
+        <x:v>The concept is about minimizing monetary distortion, so learners need to understand how inflation changes purchasing power and price signals first.</x:v>
       </x:c>
       <x:c r="F90" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G90" s="32" t="str">
-        <x:v>Direct parent captures the on-chain contract packaging layer that makes the escrow pattern practical.</x:v>
+        <x:v>Direct parent captures the measurement-distortion problem that ideal money is trying to avoid.</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B91" s="32" t="str">
-        <x:v>dev.wallet-import-format-wif</x:v>
+        <x:v>protocol.bitcoin-uri-bip21</x:v>
       </x:c>
       <x:c r="C91" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13726,21 +14024,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E91" s="32" t="str">
-        <x:v>WIF is a serialization format for one private key, so learners need the underlying asymmetric-key concept before the network prefix, checksum, and compression flag details make sense.</x:v>
+        <x:v>The URI is a wrapper around a payment destination and amount, so learners need the underlying address and output model first.</x:v>
       </x:c>
       <x:c r="F91" s="32" t="str">
         <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G91" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored on key material itself instead of overfitting it to address formats or HD wallet hierarchies.</x:v>
+        <x:v>Direct parent keeps the node tied to the standard request format rather than collapsing it into higher-level wallet UX systems.</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>dev.bip32</x:v>
       </x:c>
       <x:c r="B92" s="32" t="str">
-        <x:v>mining.pool-shares</x:v>
+        <x:v>dev.extended-keys</x:v>
       </x:c>
       <x:c r="C92" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13749,21 +14047,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E92" s="32" t="str">
-        <x:v>Pool shares only make sense after learners understand why pooled mining exists and why miners need a lower-variance way to prove contributed work before an actual block is found.</x:v>
+        <x:v>Extended keys are one specific export and branch-derivation surface inside the broader BIP32 HD tree model, so learners need the base tree-derivation mechanics first.</x:v>
       </x:c>
       <x:c r="F92" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G92" s="32" t="str">
-        <x:v>Direct parent keeps the node at the pooled-mining accounting layer without adding redundant proof-of-work or difficulty edges.</x:v>
+        <x:v>Direct parent keeps the node inside the HD derivation branch instead of treating xpub or xprv behavior as only a privacy or operational-wallet concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>dev.extended-keys</x:v>
       </x:c>
       <x:c r="B93" s="32" t="str">
-        <x:v>lightning.obscured-commitment-number</x:v>
+        <x:v>dev.hardened-keys</x:v>
       </x:c>
       <x:c r="C93" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13772,21 +14070,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E93" s="32" t="str">
-        <x:v>The obscured commitment number is part of the same commitment-state machinery as the per-state secret chain, so learners need that state-derivation context before the field-level encoding scheme makes sense.</x:v>
+        <x:v>Hardened derivation is a constraint on what an extended public key can derive and on how extended private and public key boundaries behave, so learners need the base xpub/xprv model first.</x:v>
       </x:c>
       <x:c r="F93" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G93" s="32" t="str">
-        <x:v>Direct parent keeps the node in the narrow commitment-state branch instead of pulling in broader closure or HTLC behavior.</x:v>
+        <x:v>Direct parent closes the previously missing branch-level bridge between BIP32 generally and hardened derivation specifically.</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="32" t="str">
-        <x:v>lightning.htlc</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B94" s="32" t="str">
-        <x:v>lightning.htlc-output-scripts</x:v>
+        <x:v>protocol.escrow-and-arbitration</x:v>
       </x:c>
       <x:c r="C94" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13795,21 +14093,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E94" s="32" t="str">
-        <x:v>Learners need the base HTLC idea before the offered and received witness-script branches, timeout paths, and preimage-claim paths become meaningful.</x:v>
+        <x:v>The escrow flow depends on understanding how multiple signers can authorize one spend and why a 2-of-3 threshold changes trust assumptions between buyer, seller, and arbitrator.</x:v>
       </x:c>
       <x:c r="F94" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G94" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the payment-contract primitive instead of treating it as generic script trivia.</x:v>
+        <x:v>Direct parent keeps the node tied to the threshold-signing contract pattern instead of treating it as generic dispute-resolution theory.</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="B95" s="32" t="str">
-        <x:v>lightning.htlc-output-scripts</x:v>
+        <x:v>protocol.escrow-and-arbitration</x:v>
       </x:c>
       <x:c r="C95" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13818,21 +14116,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E95" s="32" t="str">
-        <x:v>HTLC output scripts are additional commitment-transaction outputs layered on top of the same to_local and to_remote commitment-script structure, so learners need that earlier script layer first.</x:v>
+        <x:v>The contract uses a P2SH redeem script to hide the multisig spending conditions until spend time, so learners need the P2SH wrapper first.</x:v>
       </x:c>
       <x:c r="F95" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G95" s="32" t="str">
-        <x:v>Direct parent places the node at the next script layer above commitment outputs without dragging in later close-handling or watchtower flows.</x:v>
+        <x:v>Direct parent captures the on-chain contract packaging layer that makes the escrow pattern practical.</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="32" t="str">
-        <x:v>protocol.coinbase-transaction</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B96" s="32" t="str">
-        <x:v>protocol.duplicate-transaction-bug</x:v>
+        <x:v>dev.wallet-import-format-wif</x:v>
       </x:c>
       <x:c r="C96" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13841,21 +14139,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E96" s="32" t="str">
-        <x:v>The bug is historically tied to duplicated coinbase transactions, so learners need the special structure and validation role of coinbase transactions before the replay vector makes sense.</x:v>
+        <x:v>WIF is a serialization format for one private key, so learners need the underlying asymmetric-key concept before the network prefix, checksum, and compression flag details make sense.</x:v>
       </x:c>
       <x:c r="F96" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G96" s="32" t="str">
-        <x:v>Direct parent keeps the bug tied to the early-coinbase uniqueness failure instead of burying it under general mining history.</x:v>
+        <x:v>Direct parent keeps the node anchored on key material itself instead of overfitting it to address formats or HD wallet hierarchies.</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="32" t="str">
-        <x:v>protocol.utxo-model</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B97" s="32" t="str">
-        <x:v>protocol.duplicate-transaction-bug</x:v>
+        <x:v>mining.pool-shares</x:v>
       </x:c>
       <x:c r="C97" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13864,21 +14162,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E97" s="32" t="str">
-        <x:v>Learners need the txid-plus-output-index reference model to understand why identical transaction ids could confuse later spends and overwrite assumptions in the UTXO set.</x:v>
+        <x:v>Pool shares only make sense after learners understand why pooled mining exists and why miners need a lower-variance way to prove contributed work before an actual block is found.</x:v>
       </x:c>
       <x:c r="F97" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G97" s="32" t="str">
-        <x:v>Direct parent captures the reference-model side of the bug without conflating it with double-spend history or malleability.</x:v>
+        <x:v>Direct parent keeps the node at the pooled-mining accounting layer without adding redundant proof-of-work or difficulty edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="32" t="str">
-        <x:v>protocol.block-structure</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="B98" s="32" t="str">
-        <x:v>protocol.64-byte-transaction-bug</x:v>
+        <x:v>lightning.obscured-commitment-number</x:v>
       </x:c>
       <x:c r="C98" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13887,21 +14185,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E98" s="32" t="str">
-        <x:v>The bug only makes sense once learners understand how transaction hashes sit inside the block merkle tree and why internal-node preimages matter for block commitments.</x:v>
+        <x:v>The obscured commitment number is part of the same commitment-state machinery as the per-state secret chain, so learners need that state-derivation context before the field-level encoding scheme makes sense.</x:v>
       </x:c>
       <x:c r="F98" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G98" s="32" t="str">
-        <x:v>One direct parent keeps the node at the block-commitment layer instead of reopening broader hashing or SPV overview branches.</x:v>
+        <x:v>Direct parent keeps the node in the narrow commitment-state branch instead of pulling in broader closure or HTLC behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="32" t="str">
-        <x:v>fundamentals.digital-signatures</x:v>
+        <x:v>lightning.htlc</x:v>
       </x:c>
       <x:c r="B99" s="32" t="str">
-        <x:v>fundamentals.lamport-signatures</x:v>
+        <x:v>lightning.htlc-output-scripts</x:v>
       </x:c>
       <x:c r="C99" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13910,21 +14208,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E99" s="32" t="str">
-        <x:v>Learners need the general signing-and-verification mental model before the one-time Lamport construction and its tradeoffs become meaningful.</x:v>
+        <x:v>Learners need the base HTLC idea before the offered and received witness-script branches, timeout paths, and preimage-claim paths become meaningful.</x:v>
       </x:c>
       <x:c r="F99" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G99" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to signature semantics instead of treating it as only a post-quantum curiosity.</x:v>
+        <x:v>Direct parent keeps the node tied to the payment-contract primitive instead of treating it as generic script trivia.</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="B100" s="32" t="str">
-        <x:v>fundamentals.lamport-signatures</x:v>
+        <x:v>lightning.htlc-output-scripts</x:v>
       </x:c>
       <x:c r="C100" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13933,21 +14231,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E100" s="32" t="str">
-        <x:v>Lamport signatures replace elliptic-curve arithmetic with one-way hash preimages and comparisons, so learners need the hash primitive first.</x:v>
+        <x:v>HTLC output scripts are additional commitment-transaction outputs layered on top of the same to_local and to_remote commitment-script structure, so learners need that earlier script layer first.</x:v>
       </x:c>
       <x:c r="F100" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G100" s="32" t="str">
-        <x:v>Direct parent captures the actual cryptographic mechanism rather than forcing learners through unrelated elliptic-curve details.</x:v>
+        <x:v>Direct parent places the node at the next script layer above commitment outputs without dragging in later close-handling or watchtower flows.</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="32" t="str">
-        <x:v>custody.backups-recovery</x:v>
+        <x:v>protocol.coinbase-transaction</x:v>
       </x:c>
       <x:c r="B101" s="32" t="str">
-        <x:v>custody.shamirs-secret-sharing</x:v>
+        <x:v>protocol.duplicate-transaction-bug</x:v>
       </x:c>
       <x:c r="C101" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13956,21 +14254,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E101" s="32" t="str">
-        <x:v>In Bitcoin practice the scheme is used as one backup-and-recovery method, so learners need the broader custody problem before the threshold-share design choice becomes meaningful.</x:v>
+        <x:v>The bug is historically tied to duplicated coinbase transactions, so learners need the special structure and validation role of coinbase transactions before the replay vector makes sense.</x:v>
       </x:c>
       <x:c r="F101" s="32" t="str">
         <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G101" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored in practical custody use instead of drifting into a purely abstract cryptography topic.</x:v>
+        <x:v>Direct parent keeps the bug tied to the early-coinbase uniqueness failure instead of burying it under general mining history.</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="32" t="str">
-        <x:v>protocol.segregated-witness</x:v>
+        <x:v>protocol.utxo-model</x:v>
       </x:c>
       <x:c r="B102" s="32" t="str">
-        <x:v>protocol.witness-structure</x:v>
+        <x:v>protocol.duplicate-transaction-bug</x:v>
       </x:c>
       <x:c r="C102" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13979,13 +14277,13 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E102" s="32" t="str">
-        <x:v>The transaction witness layout only makes sense after the learner understands that SegWit separates witness data from the legacy transaction serialization.</x:v>
+        <x:v>Learners need the txid-plus-output-index reference model to understand why identical transaction ids could confuse later spends and overwrite assumptions in the UTXO set.</x:v>
       </x:c>
       <x:c r="F102" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G102" s="32" t="str">
-        <x:v>Direct edge keeps the node at the transaction-format layer; TXID/WTXID and witness-commitment consequences remain downstream concepts.</x:v>
+        <x:v>Direct parent captures the reference-model side of the bug without conflating it with double-spend history or malleability.</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
@@ -13993,7 +14291,7 @@
         <x:v>protocol.block-structure</x:v>
       </x:c>
       <x:c r="B103" s="32" t="str">
-        <x:v>protocol.partial-merkle-proofs</x:v>
+        <x:v>protocol.64-byte-transaction-bug</x:v>
       </x:c>
       <x:c r="C103" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14002,21 +14300,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E103" s="32" t="str">
-        <x:v>Partial Merkle proofs reconstruct a transaction's inclusion path against the Merkle root carried by a block, so learners need block composition and root placement first.</x:v>
+        <x:v>The bug only makes sense once learners understand how transaction hashes sit inside the block merkle tree and why internal-node preimages matter for block commitments.</x:v>
       </x:c>
       <x:c r="F103" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G103" s="32" t="str">
-        <x:v>The block-structure parent already inherits fundamentals.merkle-trees, avoiding a redundant direct edge.</x:v>
+        <x:v>One direct parent keeps the node at the block-commitment layer instead of reopening broader hashing or SPV overview branches.</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="32" t="str">
-        <x:v>dev.bips-process</x:v>
+        <x:v>fundamentals.digital-signatures</x:v>
       </x:c>
       <x:c r="B104" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>fundamentals.lamport-signatures</x:v>
       </x:c>
       <x:c r="C104" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14025,21 +14323,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E104" s="32" t="str">
-        <x:v>Review culture is applied throughout the proposal and implementation lifecycle, so learners need to understand the process in which Bitcoin changes are proposed and evaluated.</x:v>
+        <x:v>Learners need the general signing-and-verification mental model before the one-time Lamport construction and its tradeoffs become meaningful.</x:v>
       </x:c>
       <x:c r="F104" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G104" s="32" t="str">
-        <x:v>Direct edge supplies the development-lifecycle context without adding downstream release or deployment details.</x:v>
+        <x:v>Direct parent keeps the node tied to signature semantics instead of treating it as only a post-quantum curiosity.</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="32" t="str">
-        <x:v>security.adversarial-thinking</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B105" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>fundamentals.lamport-signatures</x:v>
       </x:c>
       <x:c r="C105" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14048,21 +14346,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E105" s="32" t="str">
-        <x:v>Independent review in Bitcoin is deliberately adversarial: reviewers look for correctness failures, attack paths, and compatibility hazards before changes are merged.</x:v>
+        <x:v>Lamport signatures replace elliptic-curve arithmetic with one-way hash preimages and comparisons, so learners need the hash primitive first.</x:v>
       </x:c>
       <x:c r="F105" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G105" s="32" t="str">
-        <x:v>Direct edge keeps review distinct from responsible disclosure and reproducible-build verification, which are specialized downstream safeguards.</x:v>
+        <x:v>Direct parent captures the actual cryptographic mechanism rather than forcing learners through unrelated elliptic-curve details.</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="32" t="str">
-        <x:v>lightning.gossip-protocol</x:v>
+        <x:v>custody.backups-recovery</x:v>
       </x:c>
       <x:c r="B106" s="32" t="str">
-        <x:v>lightning.feature-flags</x:v>
+        <x:v>custody.shamirs-secret-sharing</x:v>
       </x:c>
       <x:c r="C106" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14071,21 +14369,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E106" s="32" t="str">
-        <x:v>Feature negotiation is used to advertise and interpret capabilities across Lightning peers and network announcements, so learners need the surrounding gossip and announcement context first.</x:v>
+        <x:v>In Bitcoin practice the scheme is used as one backup-and-recovery method, so learners need the broader custody problem before the threshold-share design choice becomes meaningful.</x:v>
       </x:c>
       <x:c r="F106" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G106" s="32" t="str">
-        <x:v>Direct edge keeps the feature-bit mechanism distinct from the lower-level message transport and downstream routing protocols.</x:v>
+        <x:v>Direct parent keeps the node anchored in practical custody use instead of drifting into a purely abstract cryptography topic.</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="32" t="str">
-        <x:v>lightning.feature-flags</x:v>
+        <x:v>protocol.segregated-witness</x:v>
       </x:c>
       <x:c r="B107" s="32" t="str">
-        <x:v>lightning.onion-messages</x:v>
+        <x:v>protocol.witness-structure</x:v>
       </x:c>
       <x:c r="C107" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14094,21 +14392,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E107" s="32" t="str">
-        <x:v>Peers use a negotiated feature bit to advertise whether they can send and forward onion messages, so learners need the capability-negotiation model first.</x:v>
+        <x:v>The transaction witness layout only makes sense after the learner understands that SegWit separates witness data from the legacy transaction serialization.</x:v>
       </x:c>
       <x:c r="F107" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G107" s="32" t="str">
-        <x:v>Direct edge keeps the feature gate separate from the message forwarding mechanism.</x:v>
+        <x:v>Direct edge keeps the node at the transaction-format layer; TXID/WTXID and witness-commitment consequences remain downstream concepts.</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="32" t="str">
-        <x:v>lightning.route-blinding</x:v>
+        <x:v>protocol.block-structure</x:v>
       </x:c>
       <x:c r="B108" s="32" t="str">
-        <x:v>lightning.onion-messages</x:v>
+        <x:v>protocol.partial-merkle-proofs</x:v>
       </x:c>
       <x:c r="C108" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14117,21 +14415,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E108" s="32" t="str">
-        <x:v>Onion messages use blinded paths to forward channel-independent payloads without exposing the final destination topology, so the route-blinding model must come first.</x:v>
+        <x:v>Partial Merkle proofs reconstruct a transaction's inclusion path against the Merkle root carried by a block, so learners need block composition and root placement first.</x:v>
       </x:c>
       <x:c r="F108" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G108" s="32" t="str">
-        <x:v>Payment onion routing and BOLT12 offers remain related sibling or downstream concepts rather than direct prerequisites.</x:v>
+        <x:v>The block-structure parent already inherits fundamentals.merkle-trees, avoiding a redundant direct edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>dev.bips-process</x:v>
       </x:c>
       <x:c r="B109" s="32" t="str">
-        <x:v>lightning.encrypted-authenticated-transport</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="C109" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14140,21 +14438,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E109" s="32" t="str">
-        <x:v>The Noise_XK handshake authenticates long-term Lightning node identities with public/private key material, so learners need that identity model first.</x:v>
+        <x:v>Review culture is applied throughout the proposal and implementation lifecycle, so learners need to understand the process in which Bitcoin changes are proposed and evaluated.</x:v>
       </x:c>
       <x:c r="F109" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G109" s="32" t="str">
-        <x:v>Direct edge keeps identity foundations separate from the session-key derivation mechanism.</x:v>
+        <x:v>Direct edge supplies the development-lifecycle context without adding downstream release or deployment details.</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="32" t="str">
-        <x:v>fundamentals.diffie-hellman-key-exchange</x:v>
+        <x:v>security.adversarial-thinking</x:v>
       </x:c>
       <x:c r="B110" s="32" t="str">
-        <x:v>lightning.encrypted-authenticated-transport</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="C110" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14163,21 +14461,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E110" s="32" t="str">
-        <x:v>BOLT 08 uses elliptic-curve Diffie-Hellman operations to derive shared session secrets, so the key-exchange primitive must be understood first.</x:v>
+        <x:v>Independent review in Bitcoin is deliberately adversarial: reviewers look for correctness failures, attack paths, and compatibility hazards before changes are merged.</x:v>
       </x:c>
       <x:c r="F110" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G110" s="32" t="str">
-        <x:v>Bitcoin P2P v2 transport remains a related sibling rather than a direct prerequisite because it is a different protocol context.</x:v>
+        <x:v>Direct edge keeps review distinct from responsible disclosure and reproducible-build verification, which are specialized downstream safeguards.</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>lightning.gossip-protocol</x:v>
       </x:c>
       <x:c r="B111" s="32" t="str">
-        <x:v>protocol.strict-der-signatures</x:v>
+        <x:v>lightning.feature-flags</x:v>
       </x:c>
       <x:c r="C111" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14186,21 +14484,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E111" s="32" t="str">
-        <x:v>Strict DER enforcement occurs while Script validates an ECDSA signature, so learners need the spending-condition and interpreter context first.</x:v>
+        <x:v>Feature negotiation is used to advertise and interpret capabilities across Lightning peers and network announcements, so learners need the surrounding gossip and announcement context first.</x:v>
       </x:c>
       <x:c r="F111" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G111" s="32" t="str">
-        <x:v>Direct edge keeps the rule at the script-validation layer rather than treating BIP 66 as a broad historical upgrade topic.</x:v>
+        <x:v>Direct edge keeps the feature-bit mechanism distinct from the lower-level message transport and downstream routing protocols.</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>lightning.feature-flags</x:v>
       </x:c>
       <x:c r="B112" s="32" t="str">
-        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+        <x:v>lightning.onion-messages</x:v>
       </x:c>
       <x:c r="C112" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14209,21 +14507,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E112" s="32" t="str">
-        <x:v>The node builds on the wallet-level threshold signer policy before specifying a deterministic ordering convention for the signer keys.</x:v>
+        <x:v>Peers use a negotiated feature bit to advertise whether they can send and forward onion messages, so learners need the capability-negotiation model first.</x:v>
       </x:c>
       <x:c r="F112" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G112" s="32" t="str">
-        <x:v>Direct edge preserves the distinction between multisig policy and the BIP 67 interoperability rule.</x:v>
+        <x:v>Direct edge keeps the feature gate separate from the message forwarding mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="32" t="str">
-        <x:v>protocol.pay-to-script-hash</x:v>
+        <x:v>lightning.route-blinding</x:v>
       </x:c>
       <x:c r="B113" s="32" t="str">
-        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+        <x:v>lightning.onion-messages</x:v>
       </x:c>
       <x:c r="C113" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14232,21 +14530,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E113" s="32" t="str">
-        <x:v>BIP 67 is commonly applied when constructing the redeem script whose hash is committed by P2SH, so the script-hash wrapper provides the output context.</x:v>
+        <x:v>Onion messages use blinded paths to forward channel-independent payloads without exposing the final destination topology, so the route-blinding model must come first.</x:v>
       </x:c>
       <x:c r="F113" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G113" s="32" t="str">
-        <x:v>The shared protocol.script ancestor remains inherited rather than a redundant direct edge.</x:v>
+        <x:v>Payment onion routing and BOLT12 offers remain related sibling or downstream concepts rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="32" t="str">
-        <x:v>ops.mempool-policy</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B114" s="32" t="str">
-        <x:v>ops.mempool-purging</x:v>
+        <x:v>lightning.encrypted-authenticated-transport</x:v>
       </x:c>
       <x:c r="C114" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14255,21 +14553,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E114" s="32" t="str">
-        <x:v>Rolling minimum fee escalation and transaction eviction are local consequences of the node's mempool relay policy, so learners need that policy boundary first.</x:v>
+        <x:v>The Noise_XK handshake authenticates long-term Lightning node identities with public/private key material, so learners need that identity model first.</x:v>
       </x:c>
       <x:c r="F114" s="32" t="str">
-        <x:v>source.mempool-space-docs</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G114" s="32" t="str">
-        <x:v>The generic mempool, fee-market, and consensus-policy branches remain inherited or adjacent rather than direct prerequisites.</x:v>
+        <x:v>Direct edge keeps identity foundations separate from the session-key derivation mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>fundamentals.diffie-hellman-key-exchange</x:v>
       </x:c>
       <x:c r="B115" s="32" t="str">
-        <x:v>protocol.generic-signed-messages</x:v>
+        <x:v>lightning.encrypted-authenticated-transport</x:v>
       </x:c>
       <x:c r="C115" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14278,21 +14576,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E115" s="32" t="str">
-        <x:v>BIP 322 proves message authorization by constructing virtual transactions that satisfy a Bitcoin output script, so learners need the Script spending-condition model first.</x:v>
+        <x:v>BOLT 08 uses elliptic-curve Diffie-Hellman operations to derive shared session secrets, so the key-exchange primitive must be understood first.</x:v>
       </x:c>
       <x:c r="F115" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G115" s="32" t="str">
-        <x:v>The digital-signature path is inherited through Script; PSBT, Schnorr, and Taproot remain related variants rather than redundant direct edges.</x:v>
+        <x:v>Bitcoin P2P v2 transport remains a related sibling rather than a direct prerequisite because it is a different protocol context.</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="32" t="str">
-        <x:v>dev.bitcoin-core-rpc</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B116" s="32" t="str">
-        <x:v>security.bitcoin-core-rpc-access</x:v>
+        <x:v>protocol.strict-der-signatures</x:v>
       </x:c>
       <x:c r="C116" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14301,21 +14599,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E116" s="32" t="str">
-        <x:v>RPC access security is the control boundary around Bitcoin Core's programmatic interface, so learners need to understand the interface and its authority before securing exposure to it.</x:v>
+        <x:v>Strict DER enforcement occurs while Script validates an ECDSA signature, so learners need the spending-condition and interpreter context first.</x:v>
       </x:c>
       <x:c r="F116" s="32" t="str">
-        <x:v>source.bitcoin-core-operator-docs</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G116" s="32" t="str">
-        <x:v>Full-node operation is inherited through dev.bitcoin-core-rpc; wallet RPC and transaction-preflight nodes remain downstream use cases rather than direct parents.</x:v>
+        <x:v>Direct edge keeps the rule at the script-validation layer rather than treating BIP 66 as a broad historical upgrade topic.</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="32" t="str">
-        <x:v>dev.testmempoolaccept-rpc</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B117" s="32" t="str">
-        <x:v>dev.submitpackage-rpc</x:v>
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
       </x:c>
       <x:c r="C117" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14324,21 +14622,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E117" s="32" t="str">
-        <x:v>submitpackage is the admission counterpart to the existing testmempoolaccept preflight workflow, so learners need to understand local package checks before attempting submission and interpreting package results.</x:v>
+        <x:v>The node builds on the wallet-level threshold signer policy before specifying a deterministic ordering convention for the signer keys.</x:v>
       </x:c>
       <x:c r="F117" s="32" t="str">
-        <x:v>source.bitcoin-core-package-policy</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G117" s="32" t="str">
-        <x:v>Package relay and cluster mempool remain neighboring concepts rather than direct prerequisites because this node focuses on one local RPC operation.</x:v>
+        <x:v>Direct edge preserves the distinction between multisig policy and the BIP 67 interoperability rule.</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="32" t="str">
-        <x:v>protocol.rbf</x:v>
+        <x:v>protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="B118" s="32" t="str">
-        <x:v>protocol.package-rbf</x:v>
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
       </x:c>
       <x:c r="C118" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14347,21 +14645,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E118" s="32" t="str">
-        <x:v>Package RBF extends the ordinary replacement-policy model with package-level fee and cluster conditions, so learners need base RBF semantics first.</x:v>
+        <x:v>BIP 67 is commonly applied when constructing the redeem script whose hash is committed by P2SH, so the script-hash wrapper provides the output context.</x:v>
       </x:c>
       <x:c r="F118" s="32" t="str">
-        <x:v>source.bitcoin-core-package-policy</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G118" s="32" t="str">
-        <x:v>Package relay, cluster mempool, submitpackage, and pinning remain adjacent concepts rather than redundant direct edges.</x:v>
+        <x:v>The shared protocol.script ancestor remains inherited rather than a redundant direct edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="32" t="str">
-        <x:v>protocol.cluster-mempool</x:v>
+        <x:v>ops.mempool-policy</x:v>
       </x:c>
       <x:c r="B119" s="32" t="str">
-        <x:v>ops.mempool-cluster-limits</x:v>
+        <x:v>ops.mempool-purging</x:v>
       </x:c>
       <x:c r="C119" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14370,21 +14668,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E119" s="32" t="str">
-        <x:v>Cluster limits bound connected transaction sets, so learners need the cluster-mempool model before understanding why count and aggregate virtual-size limits replace legacy ancestor/descendant limits.</x:v>
+        <x:v>Rolling minimum fee escalation and transaction eviction are local consequences of the node's mempool relay policy, so learners need that policy boundary first.</x:v>
       </x:c>
       <x:c r="F119" s="32" t="str">
-        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+        <x:v>source.mempool-space-docs</x:v>
       </x:c>
       <x:c r="G119" s="32" t="str">
-        <x:v>Package relay, Package RBF, CPFP, and version 3 relay remain affected workflows or neighboring policy mechanisms rather than direct prerequisites.</x:v>
+        <x:v>The generic mempool, fee-market, and consensus-policy branches remain inherited or adjacent rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="32" t="str">
-        <x:v>ops.dns-seeds</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B120" s="32" t="str">
-        <x:v>lightning.dns-seeds</x:v>
+        <x:v>protocol.generic-signed-messages</x:v>
       </x:c>
       <x:c r="C120" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14393,21 +14691,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E120" s="32" t="str">
-        <x:v>Lightning DNS seeds specialize the general DNS bootstrap pattern with Lightning-specific query filters and known-peer lookup, so learners need the base DNS-seed model first.</x:v>
+        <x:v>BIP 322 proves message authorization by constructing virtual transactions that satisfy a Bitcoin output script, so learners need the Script spending-condition model first.</x:v>
       </x:c>
       <x:c r="F120" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G120" s="32" t="str">
-        <x:v>Peer discovery is inherited through ops.dns-seeds; generic Bitcoin P2P bootstrapping remains a parent concept rather than a duplicated edge.</x:v>
+        <x:v>The digital-signature path is inherited through Script; PSBT, Schnorr, and Taproot remain related variants rather than redundant direct edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="32" t="str">
-        <x:v>lightning.gossip-protocol</x:v>
+        <x:v>dev.bitcoin-core-rpc</x:v>
       </x:c>
       <x:c r="B121" s="32" t="str">
-        <x:v>lightning.dns-seeds</x:v>
+        <x:v>security.bitcoin-core-rpc-access</x:v>
       </x:c>
       <x:c r="C121" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14416,21 +14714,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E121" s="32" t="str">
-        <x:v>BOLT 10 locates Lightning peers and filters results by Lightning address information, so learners need Lightning's node-discovery and gossip context before understanding the assisted-location mechanism.</x:v>
+        <x:v>RPC access security is the control boundary around Bitcoin Core's programmatic interface, so learners need to understand the interface and its authority before securing exposure to it.</x:v>
       </x:c>
       <x:c r="F121" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-core-operator-docs</x:v>
       </x:c>
       <x:c r="G121" s="32" t="str">
-        <x:v>Lightning routing and generic P2P messages are inherited through gossip rather than added as transitive prerequisites.</x:v>
+        <x:v>Full-node operation is inherited through dev.bitcoin-core-rpc; wallet RPC and transaction-preflight nodes remain downstream use cases rather than direct parents.</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="32" t="str">
-        <x:v>lightning.payment-channels</x:v>
+        <x:v>dev.testmempoolaccept-rpc</x:v>
       </x:c>
       <x:c r="B122" s="32" t="str">
-        <x:v>lightning.short-channel-id</x:v>
+        <x:v>dev.submitpackage-rpc</x:v>
       </x:c>
       <x:c r="C122" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14439,21 +14737,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E122" s="32" t="str">
-        <x:v>The identifier names a Lightning channel's on-chain funding output, so learners need the channel and funding relationship first.</x:v>
+        <x:v>submitpackage is the admission counterpart to the existing testmempoolaccept preflight workflow, so learners need to understand local package checks before attempting submission and interpreting package results.</x:v>
       </x:c>
       <x:c r="F122" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-core-package-policy</x:v>
       </x:c>
       <x:c r="G122" s="32" t="str">
-        <x:v>Direct channel context; the gossip protocol is a downstream consumer rather than a prerequisite.</x:v>
+        <x:v>Package relay and cluster mempool remain neighboring concepts rather than direct prerequisites because this node focuses on one local RPC operation.</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="32" t="str">
-        <x:v>protocol.block-height</x:v>
+        <x:v>protocol.rbf</x:v>
       </x:c>
       <x:c r="B123" s="32" t="str">
-        <x:v>lightning.short-channel-id</x:v>
+        <x:v>protocol.package-rbf</x:v>
       </x:c>
       <x:c r="C123" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14462,21 +14760,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E123" s="32" t="str">
-        <x:v>Short Channel IDs encode block height as their first component, so learners need the block-height concept before decoding the identifier.</x:v>
+        <x:v>Package RBF extends the ordinary replacement-policy model with package-level fee and cluster conditions, so learners need base RBF semantics first.</x:v>
       </x:c>
       <x:c r="F123" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-core-package-policy</x:v>
       </x:c>
       <x:c r="G123" s="32" t="str">
-        <x:v>The transaction-index and output-index components remain part of the identifier's own outcome rather than extra transitive edges.</x:v>
+        <x:v>Package relay, cluster mempool, submitpackage, and pinning remain adjacent concepts rather than redundant direct edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="32" t="str">
-        <x:v>protocol.nodes-vs-miners</x:v>
+        <x:v>protocol.cluster-mempool</x:v>
       </x:c>
       <x:c r="B124" s="32" t="str">
-        <x:v>mining.miner-decentralization</x:v>
+        <x:v>ops.mempool-cluster-limits</x:v>
       </x:c>
       <x:c r="C124" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14485,21 +14783,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E124" s="32" t="str">
-        <x:v>Miner decentralization only makes sense once learners distinguish miners' transaction-ordering role from full nodes' independent enforcement of consensus validity.</x:v>
+        <x:v>Cluster limits bound connected transaction sets, so learners need the cluster-mempool model before understanding why count and aggregate virtual-size limits replace legacy ancestor/descendant limits.</x:v>
       </x:c>
       <x:c r="F124" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
       </x:c>
       <x:c r="G124" s="32" t="str">
-        <x:v>The edge keeps censorship power separate from authority to change consensus rules.</x:v>
+        <x:v>Package relay, Package RBF, CPFP, and version 3 relay remain affected workflows or neighboring policy mechanisms rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>ops.dns-seeds</x:v>
       </x:c>
       <x:c r="B125" s="32" t="str">
-        <x:v>mining.miner-decentralization</x:v>
+        <x:v>lightning.dns-seeds</x:v>
       </x:c>
       <x:c r="C125" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14508,21 +14806,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E125" s="32" t="str">
-        <x:v>Pool and solo mining explain the participant and coordination structure whose concentration or dispersion determines practical control over transaction ordering.</x:v>
+        <x:v>Lightning DNS seeds specialize the general DNS bootstrap pattern with Lightning-specific query filters and known-peer lookup, so learners need the base DNS-seed model first.</x:v>
       </x:c>
       <x:c r="F125" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G125" s="32" t="str">
-        <x:v>Stratum V2 remains optional implementation context, not a direct prerequisite.</x:v>
+        <x:v>Peer discovery is inherited through ops.dns-seeds; generic Bitcoin P2P bootstrapping remains a parent concept rather than a duplicated edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>lightning.gossip-protocol</x:v>
       </x:c>
       <x:c r="B126" s="32" t="str">
-        <x:v>dev.selection-cryptography</x:v>
+        <x:v>lightning.dns-seeds</x:v>
       </x:c>
       <x:c r="C126" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14531,21 +14829,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E126" s="32" t="str">
-        <x:v>Selection cryptography evaluates cryptographic tools and dependencies through evidence, testing, authorship, and review quality, so learners need the broader Bitcoin review discipline first.</x:v>
+        <x:v>BOLT 10 locates Lightning peers and filters results by Lightning address information, so learners need Lightning's node-discovery and gossip context before understanding the assisted-location mechanism.</x:v>
       </x:c>
       <x:c r="F126" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G126" s="32" t="str">
-        <x:v>Adversarial thinking is inherited through dev.review-culture; reproducible builds are a downstream verification practice rather than a prerequisite.</x:v>
+        <x:v>Lightning routing and generic P2P messages are inherited through gossip rather than added as transitive prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="32" t="str">
-        <x:v>mining.pool-shares</x:v>
+        <x:v>lightning.payment-channels</x:v>
       </x:c>
       <x:c r="B127" s="32" t="str">
-        <x:v>mining.block-withholding</x:v>
+        <x:v>lightning.short-channel-id</x:v>
       </x:c>
       <x:c r="C127" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14554,21 +14852,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E127" s="32" t="str">
-        <x:v>Block withholding exploits the difference between a pool-paid share and a share that also meets the network target, so learners must understand share accounting before the attack model makes sense.</x:v>
+        <x:v>The identifier names a Lightning channel's on-chain funding output, so learners need the channel and funding relationship first.</x:v>
       </x:c>
       <x:c r="F127" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G127" s="32" t="str">
-        <x:v>Pool-versus-solo and mining economics are inherited through mining.pool-shares; do not add a redundant majority-attack edge.</x:v>
+        <x:v>Direct channel context; the gossip protocol is a downstream consumer rather than a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>protocol.block-height</x:v>
       </x:c>
       <x:c r="B128" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>lightning.short-channel-id</x:v>
       </x:c>
       <x:c r="C128" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14577,21 +14875,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E128" s="32" t="str">
-        <x:v>P2C tweaks a public key to commit to contract data, so learners need the public/private key model.</x:v>
+        <x:v>Short Channel IDs encode block height as their first component, so learners need the block-height concept before decoding the identifier.</x:v>
       </x:c>
       <x:c r="F128" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G128" s="32" t="str">
-        <x:v>Taproot is adjacent, not a direct requirement.</x:v>
+        <x:v>The transaction-index and output-index components remain part of the identifier's own outcome rather than extra transitive edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>protocol.nodes-vs-miners</x:v>
       </x:c>
       <x:c r="B129" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>mining.miner-decentralization</x:v>
       </x:c>
       <x:c r="C129" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14600,21 +14898,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E129" s="32" t="str">
-        <x:v>P2C derives a commitment tweak from contract data using a hash, so learners need hash commitments first.</x:v>
+        <x:v>Miner decentralization only makes sense once learners distinguish miners' transaction-ordering role from full nodes' independent enforcement of consensus validity.</x:v>
       </x:c>
       <x:c r="F129" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G129" s="32" t="str">
-        <x:v>The hash is part of the construction rather than generic background.</x:v>
+        <x:v>The edge keeps censorship power separate from authority to change consensus rules.</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="32" t="str">
-        <x:v>protocol.utxo-model</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B130" s="32" t="str">
-        <x:v>extension.single-use-seals</x:v>
+        <x:v>mining.miner-decentralization</x:v>
       </x:c>
       <x:c r="C130" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14623,21 +14921,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E130" s="32" t="str">
-        <x:v>Single-use seals rely on a UTXO's one-time spend property.</x:v>
+        <x:v>Pool and solo mining explain the participant and coordination structure whose concentration or dispersion determines practical control over transaction ordering.</x:v>
       </x:c>
       <x:c r="F130" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G130" s="32" t="str">
-        <x:v>This explicit bridge prevents hiding the seal invariant inside generic UTXO semantics.</x:v>
+        <x:v>Stratum V2 remains optional implementation context, not a direct prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="32" t="str">
-        <x:v>extension.single-use-seals</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="B131" s="32" t="str">
-        <x:v>extension.client-side-validation</x:v>
+        <x:v>dev.selection-cryptography</x:v>
       </x:c>
       <x:c r="C131" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14646,21 +14944,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E131" s="32" t="str">
-        <x:v>Client-side validation relies on seals to prevent an offchain transition from being valid twice.</x:v>
+        <x:v>Selection cryptography evaluates cryptographic tools and dependencies through evidence, testing, authorship, and review quality, so learners need the broader Bitcoin review discipline first.</x:v>
       </x:c>
       <x:c r="F131" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G131" s="32" t="str">
-        <x:v>The UTXO parent is inherited through the seal and is intentionally not duplicated.</x:v>
+        <x:v>Adversarial thinking is inherited through dev.review-culture; reproducible builds are a downstream verification practice rather than a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>mining.pool-shares</x:v>
       </x:c>
       <x:c r="B132" s="32" t="str">
-        <x:v>extension.client-side-validation</x:v>
+        <x:v>mining.block-withholding</x:v>
       </x:c>
       <x:c r="C132" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14669,21 +14967,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E132" s="32" t="str">
-        <x:v>Client-side validation uses cryptographic commitments to bind offchain asset rules and transitions, so P2C supplies the contract-anchoring mechanism.</x:v>
+        <x:v>Block withholding exploits the difference between a pool-paid share and a share that also meets the network target, so learners must understand share accounting before the attack model makes sense.</x:v>
       </x:c>
       <x:c r="F132" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G132" s="32" t="str">
-        <x:v>Keep this direct edge: it prevents treating client-side validation as a vague UTXO-only extension.</x:v>
+        <x:v>Pool-versus-solo and mining economics are inherited through mining.pool-shares; do not add a redundant majority-attack edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="32" t="str">
-        <x:v>protocol.rbf</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B133" s="32" t="str">
-        <x:v>protocol.replacement-cycling</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="C133" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14692,21 +14990,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E133" s="32" t="str">
-        <x:v>Replacement cycling repeatedly uses transaction replacement, so learners need the RBF policy mechanism first.</x:v>
+        <x:v>P2C tweaks a public key to commit to contract data, so learners need the public/private key model.</x:v>
       </x:c>
       <x:c r="F133" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G133" s="32" t="str">
-        <x:v>Package RBF is related but not required for the core attack sequence.</x:v>
+        <x:v>Taproot is adjacent, not a direct requirement.</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="32" t="str">
-        <x:v>protocol.cpfp</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B134" s="32" t="str">
-        <x:v>protocol.replacement-cycling</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="C134" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14715,21 +15013,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E134" s="32" t="str">
-        <x:v>The attack cycles child-fee relationships to evict a target, so learners need CPFP mechanics first.</x:v>
+        <x:v>P2C derives a commitment tweak from contract data using a hash, so learners need hash commitments first.</x:v>
       </x:c>
       <x:c r="F134" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G134" s="32" t="str">
-        <x:v>Transaction pinning is the broader downstream risk class, not a prerequisite.</x:v>
+        <x:v>The hash is part of the construction rather than generic background.</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="32" t="str">
-        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
+        <x:v>protocol.utxo-model</x:v>
       </x:c>
       <x:c r="B135" s="32" t="str">
-        <x:v>protocol.taproot-control-blocks</x:v>
+        <x:v>extension.single-use-seals</x:v>
       </x:c>
       <x:c r="C135" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14738,21 +15036,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E135" s="32" t="str">
-        <x:v>Control blocks extend the tapleaf proof path with internal-key and parity data.</x:v>
+        <x:v>Single-use seals rely on a UTXO's one-time spend property.</x:v>
       </x:c>
       <x:c r="F135" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G135" s="32" t="str">
-        <x:v>Generic Merkle trees are inherited through the proof node.</x:v>
+        <x:v>This explicit bridge prevents hiding the seal invariant inside generic UTXO semantics.</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>extension.single-use-seals</x:v>
       </x:c>
       <x:c r="B136" s="32" t="str">
-        <x:v>dev.pseudonymous-development</x:v>
+        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="C136" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14761,21 +15059,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E136" s="32" t="str">
-        <x:v>Pseudonymous development relies on public technical evidence and independent peer review to preserve accountability without requiring legal-identity disclosure.</x:v>
+        <x:v>Client-side validation relies on seals to prevent an offchain transition from being valid twice.</x:v>
       </x:c>
       <x:c r="F136" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G136" s="32" t="str">
-        <x:v>Privacy pseudonymity is related context, not a direct prerequisite, because this node concerns contributor identity and governance rather than transaction linkage.</x:v>
+        <x:v>The UTXO parent is inherited through the seal and is intentionally not duplicated.</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="32" t="str">
-        <x:v>fundamentals.merkle-trees</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="B137" s="32" t="str">
-        <x:v>protocol.mast</x:v>
+        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="C137" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14784,21 +15082,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E137" s="32" t="str">
-        <x:v>MAST uses a Merkle tree to commit to multiple alternative script branches while revealing only one branch during spending.</x:v>
+        <x:v>Client-side validation uses cryptographic commitments to bind offchain asset rules and transitions, so P2C supplies the contract-anchoring mechanism.</x:v>
       </x:c>
       <x:c r="F137" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G137" s="32" t="str">
-        <x:v>Direct cryptographic structure; TapTree remains a downstream Taproot-specific realization.</x:v>
+        <x:v>Keep this direct edge: it prevents treating client-side validation as a vague UTXO-only extension.</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>protocol.rbf</x:v>
       </x:c>
       <x:c r="B138" s="32" t="str">
-        <x:v>protocol.mast</x:v>
+        <x:v>protocol.replacement-cycling</x:v>
       </x:c>
       <x:c r="C138" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14807,21 +15105,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E138" s="32" t="str">
-        <x:v>MAST commits to alternative Bitcoin Script branches, so learners need the locking and spending language before the tree commitment is meaningful.</x:v>
+        <x:v>Replacement cycling repeatedly uses transaction replacement, so learners need the RBF policy mechanism first.</x:v>
       </x:c>
       <x:c r="F138" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G138" s="32" t="str">
-        <x:v>Keep Script direct; the node is not only a generic Merkle-tree concept.</x:v>
+        <x:v>Package RBF is related but not required for the core attack sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="32" t="str">
-        <x:v>protocol.sighash-flags</x:v>
+        <x:v>protocol.cpfp</x:v>
       </x:c>
       <x:c r="B139" s="32" t="str">
-        <x:v>protocol.sighash-quadratic-hashing</x:v>
+        <x:v>protocol.replacement-cycling</x:v>
       </x:c>
       <x:c r="C139" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14830,21 +15128,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E139" s="32" t="str">
-        <x:v>The quadratic hashing problem is a performance consequence of how legacy signature digests are constructed under SIGHASH semantics.</x:v>
+        <x:v>The attack cycles child-fee relationships to evict a target, so learners need CPFP mechanics first.</x:v>
       </x:c>
       <x:c r="F139" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G139" s="32" t="str">
-        <x:v>BIP 143 is a supporting mitigation source, not a prerequisite edge.</x:v>
+        <x:v>Transaction pinning is the broader downstream risk class, not a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
       </x:c>
       <x:c r="B140" s="32" t="str">
-        <x:v>security.rogue-key-attack</x:v>
+        <x:v>protocol.taproot-control-blocks</x:v>
       </x:c>
       <x:c r="C140" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14853,21 +15151,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E140" s="32" t="str">
-        <x:v>The rogue-key attack occurs in naive public-key aggregation, so learners need the MuSig aggregation setting before the failure mode.</x:v>
+        <x:v>Control blocks extend the tapleaf proof path with internal-key and parity data.</x:v>
       </x:c>
       <x:c r="F140" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G140" s="32" t="str">
-        <x:v>Schnorr is inherited through MuSig; avoid a redundant direct Schnorr edge.</x:v>
+        <x:v>Generic Merkle trees are inherited through the proof node.</x:v>
       </x:c>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="B141" s="32" t="str">
-        <x:v>mining.selfish-mining</x:v>
+        <x:v>dev.pseudonymous-development</x:v>
       </x:c>
       <x:c r="C141" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14876,21 +15174,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E141" s="32" t="str">
-        <x:v>Selfish mining is an incentive strategy by miners and pools, so learners need the pooled-versus-solo mining context first.</x:v>
+        <x:v>Pseudonymous development relies on public technical evidence and independent peer review to preserve accountability without requiring legal-identity disclosure.</x:v>
       </x:c>
       <x:c r="F141" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G141" s="32" t="str">
-        <x:v>Pool economics is one direct parent; chain selection is supplied by the finality parent below.</x:v>
+        <x:v>Privacy pseudonymity is related context, not a direct prerequisite, because this node concerns contributor identity and governance rather than transaction linkage.</x:v>
       </x:c>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="32" t="str">
-        <x:v>protocol.reorgs-finality</x:v>
+        <x:v>fundamentals.merkle-trees</x:v>
       </x:c>
       <x:c r="B142" s="32" t="str">
-        <x:v>mining.selfish-mining</x:v>
+        <x:v>protocol.mast</x:v>
       </x:c>
       <x:c r="C142" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14899,21 +15197,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E142" s="32" t="str">
-        <x:v>Selfish mining relies on strategic withholding and release of competing branches, which requires the chain-reorganization and finality model.</x:v>
+        <x:v>MAST uses a Merkle tree to commit to multiple alternative script branches while revealing only one branch during spending.</x:v>
       </x:c>
       <x:c r="F142" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
       </x:c>
       <x:c r="G142" s="32" t="str">
-        <x:v>Keep the reorganization model direct rather than adding generic proof-of-work as a redundant ancestor.</x:v>
+        <x:v>Direct cryptographic structure; TapTree remains a downstream Taproot-specific realization.</x:v>
       </x:c>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B143" s="32" t="str">
-        <x:v>protocol.commit-delay-reveal</x:v>
+        <x:v>protocol.mast</x:v>
       </x:c>
       <x:c r="C143" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14922,21 +15220,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E143" s="32" t="str">
-        <x:v>Commit-delay-reveal composes a cryptographic commitment with a timed reveal, so the learner first needs the hiding and binding commitment model.</x:v>
+        <x:v>MAST commits to alternative Bitcoin Script branches, so learners need the locking and spending language before the tree commitment is meaningful.</x:v>
       </x:c>
       <x:c r="F143" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
       </x:c>
       <x:c r="G143" s="32" t="str">
-        <x:v>The delay/reveal composition is the node's distinct outcome.</x:v>
+        <x:v>Keep Script direct; the node is not only a generic Merkle-tree concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="32" t="str">
-        <x:v>protocol.dust-policy</x:v>
+        <x:v>protocol.sighash-flags</x:v>
       </x:c>
       <x:c r="B144" s="32" t="str">
-        <x:v>security.dust-attack</x:v>
+        <x:v>protocol.sighash-quadratic-hashing</x:v>
       </x:c>
       <x:c r="C144" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14945,21 +15243,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E144" s="32" t="str">
-        <x:v>Dust attacks exploit the distinction between tiny-output relay policy and the ability to place trace-value UTXOs in a wallet.</x:v>
+        <x:v>The quadratic hashing problem is a performance consequence of how legacy signature digests are constructed under SIGHASH semantics.</x:v>
       </x:c>
       <x:c r="F144" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
       </x:c>
       <x:c r="G144" s="32" t="str">
-        <x:v>Policy threshold is direct context for the attack mechanism.</x:v>
+        <x:v>BIP 143 is a supporting mitigation source, not a prerequisite edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="B145" s="32" t="str">
-        <x:v>security.dust-attack</x:v>
+        <x:v>security.rogue-key-attack</x:v>
       </x:c>
       <x:c r="C145" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14968,21 +15266,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E145" s="32" t="str">
-        <x:v>The privacy harm of dusting comes from linking future spends and wallet activity, so learners need the pseudonymity and linkage model.</x:v>
+        <x:v>The rogue-key attack occurs in naive public-key aggregation, so learners need the MuSig aggregation setting before the failure mode.</x:v>
       </x:c>
       <x:c r="F145" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
       </x:c>
       <x:c r="G145" s="32" t="str">
-        <x:v>Keep privacy linkage direct; it is not inherited through dust policy.</x:v>
+        <x:v>Schnorr is inherited through MuSig; avoid a redundant direct Schnorr edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="32" t="str">
-        <x:v>fundamentals.neutrality</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B146" s="32" t="str">
-        <x:v>dev.permissionless-development</x:v>
+        <x:v>mining.selfish-mining</x:v>
       </x:c>
       <x:c r="C146" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14991,21 +15289,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E146" s="32" t="str">
-        <x:v>Permissionless development depends on a neutral protocol that does not select which users or applications may participate.</x:v>
+        <x:v>Selfish mining is an incentive strategy by miners and pools, so learners need the pooled-versus-solo mining context first.</x:v>
       </x:c>
       <x:c r="F146" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
       </x:c>
       <x:c r="G146" s="32" t="str">
-        <x:v>Neutrality supplies the protocol property; the BIPs process supplies the change/proposal lifecycle below.</x:v>
+        <x:v>Pool economics is one direct parent; chain selection is supplied by the finality parent below.</x:v>
       </x:c>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="32" t="str">
-        <x:v>dev.bips-process</x:v>
+        <x:v>protocol.reorgs-finality</x:v>
       </x:c>
       <x:c r="B147" s="32" t="str">
-        <x:v>dev.permissionless-development</x:v>
+        <x:v>mining.selfish-mining</x:v>
       </x:c>
       <x:c r="C147" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15014,21 +15312,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E147" s="32" t="str">
-        <x:v>Learners need the proposal and deployment process to distinguish building permissionlessly from changing Bitcoin's consensus rules without broad adoption.</x:v>
+        <x:v>Selfish mining relies on strategic withholding and release of competing branches, which requires the chain-reorganization and finality model.</x:v>
       </x:c>
       <x:c r="F147" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
       </x:c>
       <x:c r="G147" s="32" t="str">
-        <x:v>Review culture remains related but is not a direct prerequisite for permissionless access.</x:v>
+        <x:v>Keep the reorganization model direct rather than adding generic proof-of-work as a redundant ancestor.</x:v>
       </x:c>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="32" t="str">
-        <x:v>dev.reproducible-builds</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="B148" s="32" t="str">
-        <x:v>dev.bootstrappable-builds</x:v>
+        <x:v>protocol.commit-delay-reveal</x:v>
       </x:c>
       <x:c r="C148" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15037,21 +15335,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E148" s="32" t="str">
-        <x:v>Bootstrappable builds extend reproducible builds by reducing trust in the compiler and build-tool binaries used to produce the reproducible output.</x:v>
+        <x:v>Commit-delay-reveal composes a cryptographic commitment with a timed reveal, so the learner first needs the hiding and binding commitment model.</x:v>
       </x:c>
       <x:c r="F148" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
       </x:c>
       <x:c r="G148" s="32" t="str">
-        <x:v>Keep this as a direct downstream edge; the node is not a duplicate alias for reproducible builds.</x:v>
+        <x:v>The delay/reveal composition is the node's distinct outcome.</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="32" t="str">
-        <x:v>protocol.transaction-lifecycle</x:v>
+        <x:v>protocol.dust-policy</x:v>
       </x:c>
       <x:c r="B149" s="32" t="str">
-        <x:v>protocol.proof-of-payment</x:v>
+        <x:v>security.dust-attack</x:v>
       </x:c>
       <x:c r="C149" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15060,21 +15358,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E149" s="32" t="str">
-        <x:v>Proof of Payment refers to a prior payment and reconstructs a transaction-shaped proof, so learners need the transaction lifecycle first.</x:v>
+        <x:v>Dust attacks exploit the distinction between tiny-output relay policy and the ability to place trace-value UTXOs in a wallet.</x:v>
       </x:c>
       <x:c r="F149" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
       </x:c>
       <x:c r="G149" s="32" t="str">
-        <x:v>Direct payment context; wallet UX and URI transport remain downstream or optional details.</x:v>
+        <x:v>Policy threshold is direct context for the attack mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="32" t="str">
-        <x:v>protocol.ephemeral-anchors</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B150" s="32" t="str">
-        <x:v>protocol.pay-to-anchor</x:v>
+        <x:v>security.dust-attack</x:v>
       </x:c>
       <x:c r="C150" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15083,12 +15381,127 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E150" s="32" t="str">
+        <x:v>The privacy harm of dusting comes from linking future spends and wallet activity, so learners need the pseudonymity and linkage model.</x:v>
+      </x:c>
+      <x:c r="F150" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+      </x:c>
+      <x:c r="G150" s="32" t="str">
+        <x:v>Keep privacy linkage direct; it is not inherited through dust policy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" s="32" t="str">
+        <x:v>fundamentals.neutrality</x:v>
+      </x:c>
+      <x:c r="B151" s="32" t="str">
+        <x:v>dev.permissionless-development</x:v>
+      </x:c>
+      <x:c r="C151" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D151" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E151" s="32" t="str">
+        <x:v>Permissionless development depends on a neutral protocol that does not select which users or applications may participate.</x:v>
+      </x:c>
+      <x:c r="F151" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G151" s="32" t="str">
+        <x:v>Neutrality supplies the protocol property; the BIPs process supplies the change/proposal lifecycle below.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" s="32" t="str">
+        <x:v>dev.bips-process</x:v>
+      </x:c>
+      <x:c r="B152" s="32" t="str">
+        <x:v>dev.permissionless-development</x:v>
+      </x:c>
+      <x:c r="C152" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D152" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E152" s="32" t="str">
+        <x:v>Learners need the proposal and deployment process to distinguish building permissionlessly from changing Bitcoin's consensus rules without broad adoption.</x:v>
+      </x:c>
+      <x:c r="F152" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G152" s="32" t="str">
+        <x:v>Review culture remains related but is not a direct prerequisite for permissionless access.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" s="32" t="str">
+        <x:v>dev.reproducible-builds</x:v>
+      </x:c>
+      <x:c r="B153" s="32" t="str">
+        <x:v>dev.bootstrappable-builds</x:v>
+      </x:c>
+      <x:c r="C153" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D153" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E153" s="32" t="str">
+        <x:v>Bootstrappable builds extend reproducible builds by reducing trust in the compiler and build-tool binaries used to produce the reproducible output.</x:v>
+      </x:c>
+      <x:c r="F153" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G153" s="32" t="str">
+        <x:v>Keep this as a direct downstream edge; the node is not a duplicate alias for reproducible builds.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" s="32" t="str">
+        <x:v>protocol.transaction-lifecycle</x:v>
+      </x:c>
+      <x:c r="B154" s="32" t="str">
+        <x:v>protocol.proof-of-payment</x:v>
+      </x:c>
+      <x:c r="C154" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D154" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E154" s="32" t="str">
+        <x:v>Proof of Payment refers to a prior payment and reconstructs a transaction-shaped proof, so learners need the transaction lifecycle first.</x:v>
+      </x:c>
+      <x:c r="F154" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="G154" s="32" t="str">
+        <x:v>Direct payment context; wallet UX and URI transport remain downstream or optional details.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" s="32" t="str">
+        <x:v>protocol.ephemeral-anchors</x:v>
+      </x:c>
+      <x:c r="B155" s="32" t="str">
+        <x:v>protocol.pay-to-anchor</x:v>
+      </x:c>
+      <x:c r="C155" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D155" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E155" s="32" t="str">
         <x:v>Pay to Anchor is a keyless refinement of the anchor-output and package-relay fee-bumping pattern, so learners need that broader context first.</x:v>
       </x:c>
-      <x:c r="F150" s="32" t="str">
+      <x:c r="F155" s="32" t="str">
         <x:v>source.bitcoin-bips</x:v>
       </x:c>
-      <x:c r="G150" s="32" t="str">
+      <x:c r="G155" s="32" t="str">
         <x:v>BIP 431/TRUC is related anti-pinning context, not an inherent prerequisite.</x:v>
       </x:c>
     </x:row>
@@ -15098,10 +15511,10 @@
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C150">
+    <x:dataValidation type="list" sqref="C12:C155">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D150">
+    <x:dataValidation type="list" sqref="D12:D155">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -18209,16 +18622,42 @@
         <x:v>Add Cube, Timeout Trees, and ZKTLCs. Keep Shadowing, Shadow Space, Projector, Hosted/Black Box Projection, Lifting, exit-ladder internals, and APE/bit-level encoding inside Cube/source context.</x:v>
       </x:c>
     </x:row>
+    <x:row r="129">
+      <x:c r="A129" s="32" t="str">
+        <x:v>decision.rgb-liquid-elements-scope</x:v>
+      </x:c>
+      <x:c r="B129" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C129" s="32" t="str">
+        <x:v>source.rgb-protocol</x:v>
+      </x:c>
+      <x:c r="D129" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E129" s="32" t="str">
+        <x:v>RGB and Liquid/Elements are protocol families with distinct architecture and learner outcomes, while several named mechanisms are already represented or are implementation details.</x:v>
+      </x:c>
+      <x:c r="F129" s="32" t="str">
+        <x:v>extension.rgb, extension.client-side-validation, extension.elements, extension.liquid, protocol.confidential-transactions, extension.sidechains</x:v>
+      </x:c>
+      <x:c r="G129" s="32" t="str">
+        <x:v>source.rgb-protocol, source.liquid-elements</x:v>
+      </x:c>
+      <x:c r="H129" s="32" t="str">
+        <x:v>Add RGB, Elements, Liquid, and Confidential Transactions. Keep RGB consignments/schemas/APIs and Liquid peg, federation, L-BTC, and individual assets inside the protocol nodes and resources.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B128">
+    <x:dataValidation type="list" sqref="B12:B129">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D128">
+    <x:dataValidation type="list" sqref="D12:D129">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -18271,7 +18710,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.77654195602</x:v>
+        <x:v>46214.7851172338</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -18279,7 +18718,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>61</x:v>
+        <x:v>63</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -18287,7 +18726,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>61</x:v>
+        <x:v>63</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -18295,7 +18734,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>162</x:v>
+        <x:v>166</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -18303,7 +18742,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>139</x:v>
+        <x:v>144</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -18327,7 +18766,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>103</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
docs: audit Bitcoin history resources
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rcade66270f8544f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R649bbcab81eb41ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rd304d81d6c984638"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R01f6aca1234345a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rd610340fcbc84d59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rad365721cefc4641"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R2cdf5bafa8db4849"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R05556d81d07c4f04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R90574371a5cd4ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Re719b4588f5444e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R7631f8b1a04e4836"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R738c0d9ea5ab4d3f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3501,22 +3501,69 @@
         <x:v>Added Elements, Liquid Network, and Confidential Transactions. Generic sidechains remains the direct context for Elements; Liquid-specific peg, federation, L-BTC, and issued-asset workflows remain inside the protocol node.</x:v>
       </x:c>
     </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="32" t="str">
+        <x:v>source.lopp-bitcoin-history</x:v>
+      </x:c>
+      <x:c r="B75" s="32" t="str">
+        <x:v>Jameson Lopp Bitcoin History Resource Index</x:v>
+      </x:c>
+      <x:c r="C75" s="32" t="str">
+        <x:v>https://www.lopp.net/bitcoin-information/history.html</x:v>
+      </x:c>
+      <x:c r="D75" s="32" t="str">
+        <x:v>history-resource-index</x:v>
+      </x:c>
+      <x:c r="E75" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F75" s="32" t="str">
+        <x:v>Historical readings, timelines, development logs, Satoshi archives, security incidents, books, and scaling-debate resources related to Bitcoin's prehistory and evolution.</x:v>
+      </x:c>
+      <x:c r="G75" s="32" t="str">
+        <x:v>Review the index by historical theme rather than importing every linked article: prehistory and cypherpunk roots, Satoshi and early Bitcoin, consensus forks and scaling, development process, security incidents, and custody incidents.</x:v>
+      </x:c>
+      <x:c r="H75" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I75" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J75" s="32" t="str">
+        <x:v>Normalized</x:v>
+      </x:c>
+      <x:c r="K75" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L75" s="32" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="M75" s="32" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="N75" s="32" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="O75" s="32" t="str">
+        <x:v>No new learner-facing node was required. High-signal history is already represented by pre-Bitcoin digital cash, cypherpunk roots, Satoshi Nakamoto, Early Bitcoin History, Genesis Block, Soft Forks vs Hard Forks, SegWit/UASF/Taproot activation, Block Size War, Chain Split Risk, historical consensus bugs, Reorgs and Finality, and Bitcoin Narrative Cycles. Exchange hacks, Silk Road, obituaries, memes, private-key challenges, and individual biographies remain context or product-specific material. Hardware-wallet incident links are tracked as input to issue #26 rather than as a new historical node.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H74">
+    <x:dataValidation type="list" sqref="H12:H75">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I74">
+    <x:dataValidation type="list" sqref="I12:I75">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J74">
+    <x:dataValidation type="list" sqref="J12:J75">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K74">
+    <x:dataValidation type="list" sqref="K12:K75">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -18648,16 +18695,42 @@
         <x:v>Add RGB, Elements, Liquid, and Confidential Transactions. Keep RGB consignments/schemas/APIs and Liquid peg, federation, L-BTC, and individual assets inside the protocol nodes and resources.</x:v>
       </x:c>
     </x:row>
+    <x:row r="130">
+      <x:c r="A130" s="32" t="str">
+        <x:v>decision.lopp-bitcoin-history-inventory</x:v>
+      </x:c>
+      <x:c r="B130" s="32" t="str">
+        <x:v>inventory</x:v>
+      </x:c>
+      <x:c r="C130" s="32" t="str">
+        <x:v>source.lopp-bitcoin-history</x:v>
+      </x:c>
+      <x:c r="D130" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E130" s="32" t="str">
+        <x:v>The Lopp page is a curated index of historical resources. Its main learning outcomes are already represented across the graph, while importing every linked event, person, book, hack, or cultural artifact would create non-atomic and product-specific nodes.</x:v>
+      </x:c>
+      <x:c r="F130" s="32" t="str">
+        <x:v>history.pre-bitcoin-digital-cash, history.cypherpunk-roots-bitcoin-origin, history.satoshi-nakamoto, history.early-bitcoin, history.genesis-block, protocol.softfork-hardfork, history.segwit-activation, history.user-activated-soft-fork, history.taproot-activation, history.block-size-war, protocol.chain-split-risk, protocol.64-byte-transaction-bug, protocol.duplicate-transaction-bug, protocol.reorgs-finality, history.bitcoin-narrative-cycles, dev.review-culture, security.responsible-disclosure</x:v>
+      </x:c>
+      <x:c r="G130" s="32" t="str">
+        <x:v>source.lopp-bitcoin-history</x:v>
+      </x:c>
+      <x:c r="H130" s="32" t="str">
+        <x:v>No new node added. Keep the index as a source hub; use its hardware-wallet-hack links to inform the separate hardware-wallet coverage review in issue #26.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B129">
+    <x:dataValidation type="list" sqref="B12:B130">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D129">
+    <x:dataValidation type="list" sqref="D12:D130">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -18710,7 +18783,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.7851172338</x:v>
+        <x:v>46214.79017565972</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -18718,7 +18791,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -18726,7 +18799,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="8">

</xml_diff>

<commit_message>
docs: audit Bitcoin governance resources
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R2cdf5bafa8db4849"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R05556d81d07c4f04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R90574371a5cd4ca1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Re719b4588f5444e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R7631f8b1a04e4836"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R738c0d9ea5ab4d3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R3191cbfd08cc406d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R34b38aa566e64d84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rb00bddeebfa84a35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R5964f9c0333a4c1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R07f820ba714746ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R754f24ca3da64735"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3548,22 +3548,69 @@
         <x:v>No new learner-facing node was required. High-signal history is already represented by pre-Bitcoin digital cash, cypherpunk roots, Satoshi Nakamoto, Early Bitcoin History, Genesis Block, Soft Forks vs Hard Forks, SegWit/UASF/Taproot activation, Block Size War, Chain Split Risk, historical consensus bugs, Reorgs and Finality, and Bitcoin Narrative Cycles. Exchange hacks, Silk Road, obituaries, memes, private-key challenges, and individual biographies remain context or product-specific material. Hardware-wallet incident links are tracked as input to issue #26 rather than as a new historical node.</x:v>
       </x:c>
     </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="32" t="str">
+        <x:v>source.lopp-bitcoin-governance</x:v>
+      </x:c>
+      <x:c r="B76" s="32" t="str">
+        <x:v>Jameson Lopp Bitcoin Governance Resource Index</x:v>
+      </x:c>
+      <x:c r="C76" s="32" t="str">
+        <x:v>https://www.lopp.net/bitcoin-information/governance.html</x:v>
+      </x:c>
+      <x:c r="D76" s="32" t="str">
+        <x:v>governance-resource-index</x:v>
+      </x:c>
+      <x:c r="E76" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F76" s="32" t="str">
+        <x:v>Curated essays and talks about Bitcoin's informal and inverted governance model, consensus upgrades, social contract, control distribution, invalid blocks, and regulation.</x:v>
+      </x:c>
+      <x:c r="G76" s="32" t="str">
+        <x:v>Review the linked resources by governance mechanism: consensus and upgrade risks, social consensus, developer and miner power, invalid-block rejection, and permissionless participation. Deduplicate against existing governance, development, decentralization, and fork nodes.</x:v>
+      </x:c>
+      <x:c r="H76" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I76" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J76" s="32" t="str">
+        <x:v>Normalized</x:v>
+      </x:c>
+      <x:c r="K76" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L76" s="32" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M76" s="32" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N76" s="32" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="O76" s="32" t="str">
+        <x:v>No new node was required. The page's central governance model is already represented by Bitcoin as Social Technology, Consensus Rules, Protocol Neutrality, BIPs Process, Review Culture, Permissionless Development, Miner Decentralization, and Chain Split Risk. Do not add a broad Bitcoin Governance umbrella node; retain the linked essays as contextual resources.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H75">
+    <x:dataValidation type="list" sqref="H12:H76">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I75">
+    <x:dataValidation type="list" sqref="I12:I76">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J75">
+    <x:dataValidation type="list" sqref="J12:J76">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K75">
+    <x:dataValidation type="list" sqref="K12:K76">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -18721,16 +18768,42 @@
         <x:v>No new node added. Keep the index as a source hub; use its hardware-wallet-hack links to inform the separate hardware-wallet coverage review in issue #26.</x:v>
       </x:c>
     </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="32" t="str">
+        <x:v>decision.lopp-bitcoin-governance-inventory</x:v>
+      </x:c>
+      <x:c r="B131" s="32" t="str">
+        <x:v>inventory</x:v>
+      </x:c>
+      <x:c r="C131" s="32" t="str">
+        <x:v>source.lopp-bitcoin-governance</x:v>
+      </x:c>
+      <x:c r="D131" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E131" s="32" t="str">
+        <x:v>The governance page is a curated index of essays and talks whose main claims are already decomposed into narrower concepts in the graph. A broad governance node would obscure the different mechanisms of social consensus, rule enforcement, proposal process, and power distribution.</x:v>
+      </x:c>
+      <x:c r="F131" s="32" t="str">
+        <x:v>history.social-consensus-technology, protocol.consensus-rules, fundamentals.neutrality, dev.bips-process, dev.review-culture, dev.permissionless-development, mining.miner-decentralization, protocol.chain-split-risk</x:v>
+      </x:c>
+      <x:c r="G131" s="32" t="str">
+        <x:v>source.lopp-bitcoin-governance</x:v>
+      </x:c>
+      <x:c r="H131" s="32" t="str">
+        <x:v>No new node added. Keep the resource index available for context and future source-level research.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B130">
+    <x:dataValidation type="list" sqref="B12:B131">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D130">
+    <x:dataValidation type="list" sqref="D12:D131">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -18783,7 +18856,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.79017565972</x:v>
+        <x:v>46214.793565381944</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -18791,7 +18864,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -18799,7 +18872,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="8">

</xml_diff>

<commit_message>
docs: audit Bitcoin investment resources
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R3191cbfd08cc406d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R34b38aa566e64d84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rb00bddeebfa84a35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R5964f9c0333a4c1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R07f820ba714746ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R754f24ca3da64735"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Re4edeeecf0b34893"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R36359f7617ad459d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R905660e10fd64ba4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R2b0b9073b46843e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rf3a37faf1bb74367"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R0a0c3d94f7604b9c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3595,22 +3595,69 @@
         <x:v>No new node was required. The page's central governance model is already represented by Bitcoin as Social Technology, Consensus Rules, Protocol Neutrality, BIPs Process, Review Culture, Permissionless Development, Miner Decentralization, and Chain Split Risk. Do not add a broad Bitcoin Governance umbrella node; retain the linked essays as contextual resources.</x:v>
       </x:c>
     </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="32" t="str">
+        <x:v>source.lopp-bitcoin-investment-theses</x:v>
+      </x:c>
+      <x:c r="B77" s="32" t="str">
+        <x:v>Jameson Lopp Bitcoin Investment Theses Resource Index</x:v>
+      </x:c>
+      <x:c r="C77" s="32" t="str">
+        <x:v>https://www.lopp.net/bitcoin-information/investment-theses.html</x:v>
+      </x:c>
+      <x:c r="D77" s="32" t="str">
+        <x:v>investment-resource-index</x:v>
+      </x:c>
+      <x:c r="E77" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F77" s="32" t="str">
+        <x:v>Curated investment theses, corporate treasury materials, Bitcoin value models, monetary arguments, and comparative altcoin investment resources.</x:v>
+      </x:c>
+      <x:c r="G77" s="32" t="str">
+        <x:v>Review the index by economic concept rather than importing every report or forecast: money and monetary premium, scarcity and issuance, monetization and adoption, risk and volatility, corporate reserves, valuation models, and altcoin comparisons.</x:v>
+      </x:c>
+      <x:c r="H77" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I77" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J77" s="32" t="str">
+        <x:v>Normalized</x:v>
+      </x:c>
+      <x:c r="K77" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L77" s="32" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="M77" s="32" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N77" s="32" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="O77" s="32" t="str">
+        <x:v>No new learner-facing node was required. Existing coverage includes Properties of Money, Scarcity and Sound Money, Monetary Premium, Monetization Process, Bitcoin Supply and Demand, Block Subsidy, Halving Cycle, Volatility Psychology and Risk Sizing, Savings vs Investment, and Token/Altcoin context. Price targets, stock-to-flow and Metcalfe-style forecasts, corporate treasury case studies, and individual portfolio recommendations remain models or context rather than stable Bitcoin prerequisites.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H76">
+    <x:dataValidation type="list" sqref="H12:H77">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I76">
+    <x:dataValidation type="list" sqref="I12:I77">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J76">
+    <x:dataValidation type="list" sqref="J12:J77">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K76">
+    <x:dataValidation type="list" sqref="K12:K77">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -18794,16 +18841,42 @@
         <x:v>No new node added. Keep the resource index available for context and future source-level research.</x:v>
       </x:c>
     </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="32" t="str">
+        <x:v>decision.lopp-bitcoin-investment-theses-inventory</x:v>
+      </x:c>
+      <x:c r="B132" s="32" t="str">
+        <x:v>inventory</x:v>
+      </x:c>
+      <x:c r="C132" s="32" t="str">
+        <x:v>source.lopp-bitcoin-investment-theses</x:v>
+      </x:c>
+      <x:c r="D132" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E132" s="32" t="str">
+        <x:v>Investment theses are arguments and models that reuse monetary, economic, and risk concepts; they are not themselves atomic Bitcoin prerequisites. Importing price forecasts, corporate examples, or portfolio recommendations would make the graph time-sensitive and advisory rather than educational.</x:v>
+      </x:c>
+      <x:c r="F132" s="32" t="str">
+        <x:v>fundamentals.money-properties, economics.scarcity, economics.monetary-premium, economics.monetization-process, economics.bitcoin-supply-demand, economics.block-subsidy, protocol.halving, economics.volatility-psychology-risk-sizing, economics.savings-vs-investment, economics.token-basics</x:v>
+      </x:c>
+      <x:c r="G132" s="32" t="str">
+        <x:v>source.lopp-bitcoin-investment-theses</x:v>
+      </x:c>
+      <x:c r="H132" s="32" t="str">
+        <x:v>No new node added. Keep the index as a curated source hub for economic context; do not treat it as financial advice or a source of canonical price predictions.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B131">
+    <x:dataValidation type="list" sqref="B12:B132">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D131">
+    <x:dataValidation type="list" sqref="D12:D132">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -18856,7 +18929,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.793565381944</x:v>
+        <x:v>46214.79455947917</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -18864,7 +18937,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -18872,7 +18945,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="8">

</xml_diff>

<commit_message>
feat: add merged mining concept
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Re4edeeecf0b34893"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R36359f7617ad459d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R905660e10fd64ba4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R2b0b9073b46843e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rf3a37faf1bb74367"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R0a0c3d94f7604b9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Ra4e3ca3834b44fc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Re95844196c46405c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Ra778732ec1314968"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Ra49a519a43c34549"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R6e3e3b87f9804649"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R23430160e27a402f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3642,22 +3642,69 @@
         <x:v>No new learner-facing node was required. Existing coverage includes Properties of Money, Scarcity and Sound Money, Monetary Premium, Monetization Process, Bitcoin Supply and Demand, Block Subsidy, Halving Cycle, Volatility Psychology and Risk Sizing, Savings vs Investment, and Token/Altcoin context. Price targets, stock-to-flow and Metcalfe-style forecasts, corporate treasury case studies, and individual portfolio recommendations remain models or context rather than stable Bitcoin prerequisites.</x:v>
       </x:c>
     </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="32" t="str">
+        <x:v>source.lopp-bitcoin-mining</x:v>
+      </x:c>
+      <x:c r="B78" s="32" t="str">
+        <x:v>Jameson Lopp Bitcoin Mining Resource Index</x:v>
+      </x:c>
+      <x:c r="C78" s="32" t="str">
+        <x:v>https://www.lopp.net/bitcoin-information/mining.html</x:v>
+      </x:c>
+      <x:c r="D78" s="32" t="str">
+        <x:v>mining-resource-index</x:v>
+      </x:c>
+      <x:c r="E78" s="32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F78" s="32" t="str">
+        <x:v>Curated Bitcoin mining explainers, mining hardware and pool resources, profitability tools, energy research, security analysis, timestamping, and merged-mining references.</x:v>
+      </x:c>
+      <x:c r="G78" s="32" t="str">
+        <x:v>Review the index by mining concept: proof-of-work and security, hardware and pool operations, mining economics, energy and externalities, attacks, and auxiliary proof-of-work. Keep calculators, dashboards, vendors, and hosted-mining services as resources rather than nodes.</x:v>
+      </x:c>
+      <x:c r="H78" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I78" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J78" s="32" t="str">
+        <x:v>Normalized</x:v>
+      </x:c>
+      <x:c r="K78" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L78" s="32" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="M78" s="32" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="N78" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O78" s="32" t="str">
+        <x:v>Added Merged Mining as the only new learner-facing concept. Proof of Work, 51% attacks, ASICs, pool/solo mining, mining economics, energy accounting, environmental tradeoffs, miner decentralization, block timestamping, and long-term security budget already exist. Hashprice, calculators, pool monitors, cloud-mining providers, and company research remain operational resources.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H77">
+    <x:dataValidation type="list" sqref="H12:H78">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I77">
+    <x:dataValidation type="list" sqref="I12:I78">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J77">
+    <x:dataValidation type="list" sqref="J12:J78">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K77">
+    <x:dataValidation type="list" sqref="K12:K78">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -18867,16 +18914,42 @@
         <x:v>No new node added. Keep the index as a curated source hub for economic context; do not treat it as financial advice or a source of canonical price predictions.</x:v>
       </x:c>
     </x:row>
+    <x:row r="133">
+      <x:c r="A133" s="32" t="str">
+        <x:v>decision.lopp-bitcoin-mining-slice</x:v>
+      </x:c>
+      <x:c r="B133" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C133" s="32" t="str">
+        <x:v>mining.merge-mining</x:v>
+      </x:c>
+      <x:c r="D133" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E133" s="32" t="str">
+        <x:v>Merged mining is a distinct mining and security mechanism: one proof-of-work process can secure multiple compatible chains. It has an independent learning outcome and is not represented by generic proof-of-work, pool mining, or sidechains alone.</x:v>
+      </x:c>
+      <x:c r="F133" s="32" t="str">
+        <x:v>mining.merge-mining, protocol.proof-of-work, mining.pool-vs-solo, extension.sidechains, mining.51-percent-attack</x:v>
+      </x:c>
+      <x:c r="G133" s="32" t="str">
+        <x:v>source.lopp-bitcoin-mining</x:v>
+      </x:c>
+      <x:c r="H133" s="32" t="str">
+        <x:v>Add Merged Mining. Keep hashprice, difficulty estimators, profitability calculators, monitors, hosted-mining companies, and energy datasets as resources or operational context.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B132">
+    <x:dataValidation type="list" sqref="B12:B133">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D132">
+    <x:dataValidation type="list" sqref="D12:D133">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -18929,7 +19002,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.79455947917</x:v>
+        <x:v>46214.795559212966</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -18937,7 +19010,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -18945,7 +19018,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="8">

</xml_diff>

<commit_message>
feat: add layer architecture concepts
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Ra4e3ca3834b44fc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Re95844196c46405c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Ra778732ec1314968"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Ra49a519a43c34549"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R6e3e3b87f9804649"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R23430160e27a402f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rf0e2a5ba15f54f22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Raf1d774e401e49a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R3cbb145a9f964051"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rc006879e0b3e49db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rdef7987bcef6459d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rd06385608df0405e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3689,22 +3689,116 @@
         <x:v>Added Merged Mining as the only new learner-facing concept. Proof of Work, 51% attacks, ASICs, pool/solo mining, mining economics, energy accounting, environmental tradeoffs, miner decentralization, block timestamping, and long-term security budget already exist. Hashprice, calculators, pool monitors, cloud-mining providers, and company research remain operational resources.</x:v>
       </x:c>
     </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="32" t="str">
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
+      </x:c>
+      <x:c r="B79" s="32" t="str">
+        <x:v>Jameson Lopp Bitcoin Layer Two Resource Index</x:v>
+      </x:c>
+      <x:c r="C79" s="32" t="str">
+        <x:v>https://www.lopp.net/bitcoin-information/other-layers.html</x:v>
+      </x:c>
+      <x:c r="D79" s="32" t="str">
+        <x:v>layer-resource-index</x:v>
+      </x:c>
+      <x:c r="E79" s="32" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F79" s="32" t="str">
+        <x:v>Curated Bitcoin layer-two and anchored-protocol resources spanning Lightning, sidechains, statechains, softchains, spacechains, spiderchains, BitVM, DLCs, ecash, rollups, identity protocols, smart-contract systems, and cross-chain bridges.</x:v>
+      </x:c>
+      <x:c r="G79" s="32" t="str">
+        <x:v>Review the index by architecture rather than importing every named project: payment channels, sidechains and platforms, alternative peg designs, statechains, validity rollups, bridge security, identity protocols, and application-specific protocols. Deduplicate against existing protocol nodes and keep project directories, vendors, playgrounds, and individual products as resources.</x:v>
+      </x:c>
+      <x:c r="H79" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I79" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J79" s="32" t="str">
+        <x:v>Normalized</x:v>
+      </x:c>
+      <x:c r="K79" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L79" s="32" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="M79" s="32" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="N79" s="32" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O79" s="32" t="str">
+        <x:v>Added Drivechains, Softchains, Spiderchains, Bitcoin Rollups, and Cross-Chain Bridges. Lightning, Liquid, Elements, Statechains, Spark, Spacechains, BitVM, DLCs, Cashu, Fedimint, Ark, Cube, RGB, Nostr, and Covenants already exist. Rootstock, Stacks, Citrea, Mainstay, Counterparty, Revault, Sapio, Tachi, TradeLayer, ION, and Spaces remain named projects or specialized protocols for future source-specific review rather than automatic nodes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="32" t="str">
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
+      </x:c>
+      <x:c r="B80" s="32" t="str">
+        <x:v>Jameson Lopp Bitcoin Layer Two Resource Index</x:v>
+      </x:c>
+      <x:c r="C80" s="32" t="str">
+        <x:v>https://www.lopp.net/bitcoin-information/other-layers.html</x:v>
+      </x:c>
+      <x:c r="D80" s="32" t="str">
+        <x:v>layer-resource-index</x:v>
+      </x:c>
+      <x:c r="E80" s="32" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F80" s="32" t="str">
+        <x:v>Curated Bitcoin layer-two and anchored-protocol resources spanning Lightning, sidechains, statechains, softchains, spacechains, spiderchains, BitVM, DLCs, ecash, rollups, identity protocols, smart-contract systems, and cross-chain bridges.</x:v>
+      </x:c>
+      <x:c r="G80" s="32" t="str">
+        <x:v>Review the index by architecture rather than importing every named project: payment channels, sidechains and platforms, alternative peg designs, statechains, validity rollups, bridge security, identity protocols, and application-specific protocols. Deduplicate against existing protocol nodes and keep project directories, vendors, playgrounds, and individual products as resources.</x:v>
+      </x:c>
+      <x:c r="H80" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I80" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J80" s="32" t="str">
+        <x:v>Normalized</x:v>
+      </x:c>
+      <x:c r="K80" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L80" s="32" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="M80" s="32" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="N80" s="32" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O80" s="32" t="str">
+        <x:v>Added Drivechains, Softchains, Spiderchains, Bitcoin Rollups, and Cross-Chain Bridges. Lightning, Liquid, Elements, Statechains, Spark, Spacechains, BitVM, DLCs, Cashu, Fedimint, Ark, Cube, RGB, Nostr, and Covenants already exist. Rootstock, Stacks, Citrea, Mainstay, Counterparty, Revault, Sapio, Tachi, TradeLayer, ION, and Spaces remain named projects or specialized protocols for future source-specific review rather than automatic nodes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H78">
+    <x:dataValidation type="list" sqref="H12:H80">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I78">
+    <x:dataValidation type="list" sqref="I12:I80">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J78">
+    <x:dataValidation type="list" sqref="J12:J80">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K78">
+    <x:dataValidation type="list" sqref="K12:K80">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -12306,16 +12400,271 @@
         <x:v>Keep peg-in/peg-out, federation operations, L-BTC, and individual issued assets inside the Liquid protocol node.</x:v>
       </x:c>
     </x:row>
+    <x:row r="178">
+      <x:c r="A178" s="32" t="str">
+        <x:v>extension.drivechains</x:v>
+      </x:c>
+      <x:c r="B178" s="32" t="str">
+        <x:v>Drivechains</x:v>
+      </x:c>
+      <x:c r="C178" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D178" s="32" t="str">
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
+      </x:c>
+      <x:c r="E178" s="32" t="str">
+        <x:v>https://www.lopp.net/bitcoin-information/other-layers.html</x:v>
+      </x:c>
+      <x:c r="F178" s="32" t="str">
+        <x:v>Drivechains section and drivechain.info resource</x:v>
+      </x:c>
+      <x:c r="G178" s="32" t="str"/>
+      <x:c r="H178" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I178" s="32" t="str">
+        <x:v>Drivechains are a distinct sidechain and miner-mediated peg design that combines auxiliary proof-of-work with withdrawal governance; generic sidechains and merged mining do not explain the combined mechanism.</x:v>
+      </x:c>
+      <x:c r="J178" s="32" t="str">
+        <x:v>extension.sidechains, mining.merge-mining</x:v>
+      </x:c>
+      <x:c r="K178" s="32" t="str">
+        <x:v>extension.sidechains, mining.merge-mining</x:v>
+      </x:c>
+      <x:c r="L178" s="32" t="str">
+        <x:v>The concept combines sidechain settlement with merged-mining and miner-mediated withdrawal assumptions.</x:v>
+      </x:c>
+      <x:c r="M178" s="32" t="str">
+        <x:v>drivechain, drivechains</x:v>
+      </x:c>
+      <x:c r="N178" s="32" t="str">
+        <x:v>bitcoin-l2, sidechains, merged-mining, peg</x:v>
+      </x:c>
+      <x:c r="O178" s="32" t="str">
+        <x:v>50m</x:v>
+      </x:c>
+      <x:c r="P178" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q178" s="32" t="str">
+        <x:v>Add as a design concept; BIP-specific implementation and policy debates remain resources.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179">
+      <x:c r="A179" s="32" t="str">
+        <x:v>extension.softchains</x:v>
+      </x:c>
+      <x:c r="B179" s="32" t="str">
+        <x:v>Softchains</x:v>
+      </x:c>
+      <x:c r="C179" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D179" s="32" t="str">
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
+      </x:c>
+      <x:c r="E179" s="32" t="str">
+        <x:v>https://www.lopp.net/bitcoin-information/other-layers.html</x:v>
+      </x:c>
+      <x:c r="F179" s="32" t="str">
+        <x:v>Softchains section and softchain proposal resource</x:v>
+      </x:c>
+      <x:c r="G179" s="32" t="str"/>
+      <x:c r="H179" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I179" s="32" t="str">
+        <x:v>Softchains are a distinct proposed Bitcoin layer architecture exploring soft-fork-compatible enforcement for auxiliary execution environments.</x:v>
+      </x:c>
+      <x:c r="J179" s="32" t="str">
+        <x:v>extension.sidechains</x:v>
+      </x:c>
+      <x:c r="K179" s="32" t="str">
+        <x:v>extension.sidechains</x:v>
+      </x:c>
+      <x:c r="L179" s="32" t="str">
+        <x:v>Sidechains supplies the layer and anchoring model; its inherited consensus context already covers soft-fork distinctions.</x:v>
+      </x:c>
+      <x:c r="M179" s="32" t="str">
+        <x:v>softchain, softchains</x:v>
+      </x:c>
+      <x:c r="N179" s="32" t="str">
+        <x:v>bitcoin-l2, sidechains, soft-forks, covenants</x:v>
+      </x:c>
+      <x:c r="O179" s="32" t="str">
+        <x:v>45m</x:v>
+      </x:c>
+      <x:c r="P179" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q179" s="32" t="str">
+        <x:v>Add as an architecture-level proposal, not as a specific implementation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180">
+      <x:c r="A180" s="32" t="str">
+        <x:v>extension.spiderchains</x:v>
+      </x:c>
+      <x:c r="B180" s="32" t="str">
+        <x:v>Spiderchains</x:v>
+      </x:c>
+      <x:c r="C180" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D180" s="32" t="str">
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
+      </x:c>
+      <x:c r="E180" s="32" t="str">
+        <x:v>https://www.lopp.net/bitcoin-information/other-layers.html</x:v>
+      </x:c>
+      <x:c r="F180" s="32" t="str">
+        <x:v>Spiderchains section and Botanix whitepaper</x:v>
+      </x:c>
+      <x:c r="G180" s="32" t="str"/>
+      <x:c r="H180" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I180" s="32" t="str">
+        <x:v>Spiderchains are a distinct sidechain architecture using collateralized multisig operators and Bitcoin transactions to coordinate peg operations.</x:v>
+      </x:c>
+      <x:c r="J180" s="32" t="str">
+        <x:v>extension.sidechains, custody.multisig</x:v>
+      </x:c>
+      <x:c r="K180" s="32" t="str">
+        <x:v>extension.sidechains, custody.multisig</x:v>
+      </x:c>
+      <x:c r="L180" s="32" t="str">
+        <x:v>The design combines a sidechain with multisig-based operator custody and peg coordination.</x:v>
+      </x:c>
+      <x:c r="M180" s="32" t="str">
+        <x:v>spiderchain, spiderchains</x:v>
+      </x:c>
+      <x:c r="N180" s="32" t="str">
+        <x:v>bitcoin-l2, sidechains, multisig, peg</x:v>
+      </x:c>
+      <x:c r="O180" s="32" t="str">
+        <x:v>50m</x:v>
+      </x:c>
+      <x:c r="P180" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q180" s="32" t="str">
+        <x:v>Add as a design concept; Botanix-specific EVM and operational details remain resources.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181">
+      <x:c r="A181" s="32" t="str">
+        <x:v>extension.rollups</x:v>
+      </x:c>
+      <x:c r="B181" s="32" t="str">
+        <x:v>Bitcoin Rollups</x:v>
+      </x:c>
+      <x:c r="C181" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D181" s="32" t="str">
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
+      </x:c>
+      <x:c r="E181" s="32" t="str">
+        <x:v>https://www.lopp.net/bitcoin-information/other-layers.html</x:v>
+      </x:c>
+      <x:c r="F181" s="32" t="str">
+        <x:v>Rollups section and Bitcoin rollups resource</x:v>
+      </x:c>
+      <x:c r="G181" s="32" t="str"/>
+      <x:c r="H181" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I181" s="32" t="str">
+        <x:v>Bitcoin rollups are an execution-scaling architecture that commits compressed state or validity evidence to Bitcoin; they are distinct from generic sidechains and zero-knowledge proofs.</x:v>
+      </x:c>
+      <x:c r="J181" s="32" t="str">
+        <x:v>fundamentals.zero-knowledge-proofs, extension.sidechains</x:v>
+      </x:c>
+      <x:c r="K181" s="32" t="str">
+        <x:v>fundamentals.zero-knowledge-proofs, extension.sidechains</x:v>
+      </x:c>
+      <x:c r="L181" s="32" t="str">
+        <x:v>The learner needs both proof-based off-chain computation and the broader anchored-layer model.</x:v>
+      </x:c>
+      <x:c r="M181" s="32" t="str">
+        <x:v>Bitcoin rollup, validity rollups</x:v>
+      </x:c>
+      <x:c r="N181" s="32" t="str">
+        <x:v>bitcoin-l2, rollups, zero-knowledge, scaling</x:v>
+      </x:c>
+      <x:c r="O181" s="32" t="str">
+        <x:v>60m</x:v>
+      </x:c>
+      <x:c r="P181" s="32" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="Q181" s="32" t="str">
+        <x:v>Keep individual projects such as Citrea as separate source-specific audits.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182">
+      <x:c r="A182" s="32" t="str">
+        <x:v>extension.cross-chain-bridges</x:v>
+      </x:c>
+      <x:c r="B182" s="32" t="str">
+        <x:v>Cross-Chain Bridges</x:v>
+      </x:c>
+      <x:c r="C182" s="32" t="str">
+        <x:v>Extension Systems</x:v>
+      </x:c>
+      <x:c r="D182" s="32" t="str">
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
+      </x:c>
+      <x:c r="E182" s="32" t="str">
+        <x:v>https://www.lopp.net/bitcoin-information/other-layers.html</x:v>
+      </x:c>
+      <x:c r="F182" s="32" t="str">
+        <x:v>Cross-Chain Bridges section and Interlay/Threshold/Wrapped Bitcoin resources</x:v>
+      </x:c>
+      <x:c r="G182" s="32" t="str"/>
+      <x:c r="H182" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I182" s="32" t="str">
+        <x:v>Cross-chain bridges have a distinct security outcome around representing or moving assets across independent consensus systems; their trust assumptions are not captured by generic sidechains alone.</x:v>
+      </x:c>
+      <x:c r="J182" s="32" t="str">
+        <x:v>extension.sidechains</x:v>
+      </x:c>
+      <x:c r="K182" s="32" t="str">
+        <x:v>extension.sidechains</x:v>
+      </x:c>
+      <x:c r="L182" s="32" t="str">
+        <x:v>Sidechains provides the minimal model for anchored secondary systems; bridge mechanism variants remain inside the node.</x:v>
+      </x:c>
+      <x:c r="M182" s="32" t="str">
+        <x:v>Bitcoin bridges, cross-chain bridge security</x:v>
+      </x:c>
+      <x:c r="N182" s="32" t="str">
+        <x:v>bridges, cross-chain, sidechains, custody</x:v>
+      </x:c>
+      <x:c r="O182" s="32" t="str">
+        <x:v>55m</x:v>
+      </x:c>
+      <x:c r="P182" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q182" s="32" t="str">
+        <x:v>Keep custodial, federated, light-client, and cryptographic bridge variants as comparative mechanisms rather than separate nodes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H177">
+    <x:dataValidation type="list" sqref="H12:H182">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P177">
+    <x:dataValidation type="list" sqref="P12:P182">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -12383,10 +12732,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="32" t="str">
-        <x:v>extension.client-side-validation</x:v>
+        <x:v>extension.sidechains</x:v>
       </x:c>
       <x:c r="B12" s="32" t="str">
-        <x:v>extension.rgb</x:v>
+        <x:v>extension.drivechains</x:v>
       </x:c>
       <x:c r="C12" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12395,10 +12744,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E12" s="32" t="str">
-        <x:v>RGB builds its contract and asset model on client-side validation of off-chain state anchored to Bitcoin outputs.</x:v>
+        <x:v>Drivechains are a concrete sidechain design with additional miner-mediated peg assumptions.</x:v>
       </x:c>
       <x:c r="F12" s="32" t="str">
-        <x:v>source.rgb-protocol</x:v>
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
       </x:c>
       <x:c r="G12" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12406,10 +12755,10 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>mining.merge-mining</x:v>
       </x:c>
       <x:c r="B13" s="32" t="str">
-        <x:v>protocol.confidential-transactions</x:v>
+        <x:v>extension.drivechains</x:v>
       </x:c>
       <x:c r="C13" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12418,10 +12767,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E13" s="32" t="str">
-        <x:v>Confidential Transactions use cryptographic commitments to hide values while preserving verifiability.</x:v>
+        <x:v>Drivechains use auxiliary proof-of-work and miner participation as part of their withdrawal model.</x:v>
       </x:c>
       <x:c r="F13" s="32" t="str">
-        <x:v>source.liquid-elements</x:v>
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
       </x:c>
       <x:c r="G13" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12432,7 +12781,7 @@
         <x:v>extension.sidechains</x:v>
       </x:c>
       <x:c r="B14" s="32" t="str">
-        <x:v>extension.elements</x:v>
+        <x:v>extension.softchains</x:v>
       </x:c>
       <x:c r="C14" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12441,10 +12790,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E14" s="32" t="str">
-        <x:v>Elements is a concrete platform for constructing Bitcoin-derived sidechains and application-specific networks.</x:v>
+        <x:v>Softchains are a proposed sidechain architecture with Bitcoin-enforced anchoring assumptions.</x:v>
       </x:c>
       <x:c r="F14" s="32" t="str">
-        <x:v>source.liquid-elements</x:v>
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
       </x:c>
       <x:c r="G14" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12452,10 +12801,10 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="32" t="str">
-        <x:v>extension.elements</x:v>
+        <x:v>extension.sidechains</x:v>
       </x:c>
       <x:c r="B15" s="32" t="str">
-        <x:v>extension.liquid</x:v>
+        <x:v>extension.spiderchains</x:v>
       </x:c>
       <x:c r="C15" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12464,10 +12813,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E15" s="32" t="str">
-        <x:v>Liquid is a production network built on the Elements platform, with its own federation, peg, and asset policies.</x:v>
+        <x:v>Spiderchains are a concrete sidechain design using operator multisig for peg coordination.</x:v>
       </x:c>
       <x:c r="F15" s="32" t="str">
-        <x:v>source.liquid-elements</x:v>
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
       </x:c>
       <x:c r="G15" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12475,10 +12824,10 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="32" t="str">
-        <x:v>protocol.confidential-transactions</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B16" s="32" t="str">
-        <x:v>extension.liquid</x:v>
+        <x:v>extension.spiderchains</x:v>
       </x:c>
       <x:c r="C16" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12487,10 +12836,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E16" s="32" t="str">
-        <x:v>Liquid's privacy and issued-asset behavior depends on Confidential Transactions as a core transaction primitive.</x:v>
+        <x:v>Spiderchains use collateralized multisig operators as a core coordination mechanism.</x:v>
       </x:c>
       <x:c r="F16" s="32" t="str">
-        <x:v>source.liquid-elements</x:v>
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
       </x:c>
       <x:c r="G16" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12498,10 +12847,10 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="32" t="str">
-        <x:v>protocol.timelocks</x:v>
+        <x:v>fundamentals.zero-knowledge-proofs</x:v>
       </x:c>
       <x:c r="B17" s="32" t="str">
-        <x:v>extension.timeout-trees</x:v>
+        <x:v>extension.rollups</x:v>
       </x:c>
       <x:c r="C17" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12510,10 +12859,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E17" s="32" t="str">
-        <x:v>Timeout Trees use delayed transaction branches to preserve unilateral redemption, so learners need Bitcoin timelocks first.</x:v>
+        <x:v>Validity-rollup designs use proof-based verification for off-chain execution claims.</x:v>
       </x:c>
       <x:c r="F17" s="32" t="str">
-        <x:v>source.cube-introducing</x:v>
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
       </x:c>
       <x:c r="G17" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12521,10 +12870,10 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="32" t="str">
-        <x:v>extension.timeout-trees</x:v>
+        <x:v>extension.sidechains</x:v>
       </x:c>
       <x:c r="B18" s="32" t="str">
-        <x:v>extension.zktlcs</x:v>
+        <x:v>extension.rollups</x:v>
       </x:c>
       <x:c r="C18" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12533,10 +12882,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E18" s="32" t="str">
-        <x:v>ZKTLCs use timeout-tree ownership virtualization as one half of their unified primitive.</x:v>
+        <x:v>Rollups are an anchored secondary execution layer and require the broader layer/settlement model.</x:v>
       </x:c>
       <x:c r="F18" s="32" t="str">
-        <x:v>source.cube-introducing</x:v>
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
       </x:c>
       <x:c r="G18" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12544,10 +12893,10 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="32" t="str">
-        <x:v>extension.bitvm</x:v>
+        <x:v>extension.sidechains</x:v>
       </x:c>
       <x:c r="B19" s="32" t="str">
-        <x:v>extension.zktlcs</x:v>
+        <x:v>extension.cross-chain-bridges</x:v>
       </x:c>
       <x:c r="C19" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12556,10 +12905,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E19" s="32" t="str">
-        <x:v>ZKTLCs use BitVM-style challenge and disproof to enforce computation without trusting the executor.</x:v>
+        <x:v>Bridge security is easiest to understand after the learner knows how anchored secondary chains differ from Bitcoin's base layer.</x:v>
       </x:c>
       <x:c r="F19" s="32" t="str">
-        <x:v>source.cube-introducing</x:v>
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
       </x:c>
       <x:c r="G19" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12567,10 +12916,10 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="32" t="str">
-        <x:v>extension.zktlcs</x:v>
+        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="B20" s="32" t="str">
-        <x:v>extension.cube</x:v>
+        <x:v>extension.rgb</x:v>
       </x:c>
       <x:c r="C20" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12579,10 +12928,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E20" s="32" t="str">
-        <x:v>Cube's architecture is built around ZKTLCs for programmable execution, ownership, and unilateral exit.</x:v>
+        <x:v>RGB builds its contract and asset model on client-side validation of off-chain state anchored to Bitcoin outputs.</x:v>
       </x:c>
       <x:c r="F20" s="32" t="str">
-        <x:v>source.cube-introducing</x:v>
+        <x:v>source.rgb-protocol</x:v>
       </x:c>
       <x:c r="G20" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12590,10 +12939,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="str">
-        <x:v>extension.statechains</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="B21" s="32" t="str">
-        <x:v>extension.spark</x:v>
+        <x:v>protocol.confidential-transactions</x:v>
       </x:c>
       <x:c r="C21" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12602,10 +12951,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E21" s="32" t="str">
-        <x:v>Spark's architecture extends statechain-style off-chain ownership transfer with a distributed operator set and Lightning interoperability.</x:v>
+        <x:v>Confidential Transactions use cryptographic commitments to hide values while preserving verifiability.</x:v>
       </x:c>
       <x:c r="F21" s="32" t="str">
-        <x:v>source.spark-protocol</x:v>
+        <x:v>source.liquid-elements</x:v>
       </x:c>
       <x:c r="G21" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12613,10 +12962,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32" t="str">
-        <x:v>history.cypherpunk-roots-bitcoin-origin</x:v>
+        <x:v>extension.sidechains</x:v>
       </x:c>
       <x:c r="B22" s="32" t="str">
-        <x:v>history.satoshi-nakamoto</x:v>
+        <x:v>extension.elements</x:v>
       </x:c>
       <x:c r="C22" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12625,10 +12974,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E22" s="32" t="str">
-        <x:v>Satoshi's pseudonym and founder independence are best understood in the context of Bitcoin's cypherpunk roots and origin story.</x:v>
+        <x:v>Elements is a concrete platform for constructing Bitcoin-derived sidechains and application-specific networks.</x:v>
       </x:c>
       <x:c r="F22" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.liquid-elements</x:v>
       </x:c>
       <x:c r="G22" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12636,10 +12985,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32" t="str">
-        <x:v>fundamentals.money-properties</x:v>
+        <x:v>extension.elements</x:v>
       </x:c>
       <x:c r="B23" s="32" t="str">
-        <x:v>economics.bitcoin-denominations</x:v>
+        <x:v>extension.liquid</x:v>
       </x:c>
       <x:c r="C23" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12648,10 +12997,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E23" s="32" t="str">
-        <x:v>The learner needs a basic monetary-unit model before BTC and satoshis are meaningful denominations.</x:v>
+        <x:v>Liquid is a production network built on the Elements platform, with its own federation, peg, and asset policies.</x:v>
       </x:c>
       <x:c r="F23" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.liquid-elements</x:v>
       </x:c>
       <x:c r="G23" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12659,10 +13008,10 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="str">
-        <x:v>protocol.coinbase-transaction</x:v>
+        <x:v>protocol.confidential-transactions</x:v>
       </x:c>
       <x:c r="B24" s="32" t="str">
-        <x:v>economics.block-subsidy</x:v>
+        <x:v>extension.liquid</x:v>
       </x:c>
       <x:c r="C24" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12671,21 +13020,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E24" s="32" t="str">
-        <x:v>The block subsidy is the newly issued component claimed by a coinbase transaction.</x:v>
+        <x:v>Liquid's privacy and issued-asset behavior depends on Confidential Transactions as a core transaction primitive.</x:v>
       </x:c>
       <x:c r="F24" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.liquid-elements</x:v>
       </x:c>
       <x:c r="G24" s="32" t="str">
-        <x:v>The coinbase node already carries the halving prerequisite, so no redundant direct halving edge is added.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="str">
-        <x:v>fundamentals.digital-signatures</x:v>
+        <x:v>protocol.timelocks</x:v>
       </x:c>
       <x:c r="B25" s="32" t="str">
-        <x:v>security.quantum-computing-threat</x:v>
+        <x:v>extension.timeout-trees</x:v>
       </x:c>
       <x:c r="C25" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12694,10 +13043,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E25" s="32" t="str">
-        <x:v>Quantum attacks on public-key authorization require understanding ordinary Bitcoin signature security first.</x:v>
+        <x:v>Timeout Trees use delayed transaction branches to preserve unilateral redemption, so learners need Bitcoin timelocks first.</x:v>
       </x:c>
       <x:c r="F25" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.cube-introducing</x:v>
       </x:c>
       <x:c r="G25" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12705,10 +13054,10 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>extension.timeout-trees</x:v>
       </x:c>
       <x:c r="B26" s="32" t="str">
-        <x:v>extension.ordinals-inscriptions</x:v>
+        <x:v>extension.zktlcs</x:v>
       </x:c>
       <x:c r="C26" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12717,10 +13066,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E26" s="32" t="str">
-        <x:v>The source explains inscriptions as a Taproot-era witness-data application.</x:v>
+        <x:v>ZKTLCs use timeout-tree ownership virtualization as one half of their unified primitive.</x:v>
       </x:c>
       <x:c r="F26" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.cube-introducing</x:v>
       </x:c>
       <x:c r="G26" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12728,10 +13077,10 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="str">
-        <x:v>protocol.witness-structure</x:v>
+        <x:v>extension.bitvm</x:v>
       </x:c>
       <x:c r="B27" s="32" t="str">
-        <x:v>extension.ordinals-inscriptions</x:v>
+        <x:v>extension.zktlcs</x:v>
       </x:c>
       <x:c r="C27" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12740,10 +13089,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E27" s="32" t="str">
-        <x:v>Witness structure is needed to understand where inscription data is carried and how it affects block space.</x:v>
+        <x:v>ZKTLCs use BitVM-style challenge and disproof to enforce computation without trusting the executor.</x:v>
       </x:c>
       <x:c r="F27" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.cube-introducing</x:v>
       </x:c>
       <x:c r="G27" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12751,10 +13100,10 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>extension.zktlcs</x:v>
       </x:c>
       <x:c r="B28" s="32" t="str">
-        <x:v>extension.proof-of-existence</x:v>
+        <x:v>extension.cube</x:v>
       </x:c>
       <x:c r="C28" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12763,10 +13112,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E28" s="32" t="str">
-        <x:v>Timestamp proofs commit evidence without requiring the complete document to be stored on-chain.</x:v>
+        <x:v>Cube's architecture is built around ZKTLCs for programmable execution, ownership, and unilateral exit.</x:v>
       </x:c>
       <x:c r="F28" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.cube-introducing</x:v>
       </x:c>
       <x:c r="G28" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12774,10 +13123,10 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="32" t="str">
-        <x:v>protocol.tagged-hashes</x:v>
+        <x:v>extension.statechains</x:v>
       </x:c>
       <x:c r="B29" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>extension.spark</x:v>
       </x:c>
       <x:c r="C29" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12786,10 +13135,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E29" s="32" t="str">
-        <x:v>TapTweak is defined using tagged hashes directly in Taproot key tweaking.</x:v>
+        <x:v>Spark's architecture extends statechain-style off-chain ownership transfer with a distributed operator set and Lightning interoperability.</x:v>
       </x:c>
       <x:c r="F29" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.spark-protocol</x:v>
       </x:c>
       <x:c r="G29" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12797,10 +13146,10 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32" t="str">
-        <x:v>protocol.x-only-public-keys</x:v>
+        <x:v>history.cypherpunk-roots-bitcoin-origin</x:v>
       </x:c>
       <x:c r="B30" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>history.satoshi-nakamoto</x:v>
       </x:c>
       <x:c r="C30" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12809,10 +13158,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E30" s="32" t="str">
-        <x:v>TapTweak operates on x-only public keys in the Taproot construction.</x:v>
+        <x:v>Satoshi's pseudonym and founder independence are best understood in the context of Bitcoin's cypherpunk roots and origin story.</x:v>
       </x:c>
       <x:c r="F30" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G30" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12820,10 +13169,10 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>fundamentals.money-properties</x:v>
       </x:c>
       <x:c r="B31" s="32" t="str">
-        <x:v>protocol.taproot-key-path-spends</x:v>
+        <x:v>economics.bitcoin-denominations</x:v>
       </x:c>
       <x:c r="C31" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12832,21 +13181,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E31" s="32" t="str">
-        <x:v>A key-path spend verifies against the tweaked Taproot output key, so learners need the tweak mechanism before the spending mode makes sense.</x:v>
+        <x:v>The learner needs a basic monetary-unit model before BTC and satoshis are meaningful denominations.</x:v>
       </x:c>
       <x:c r="F31" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G31" s="32" t="str">
-        <x:v>Direct parent keeps the node focused on the spend mode rather than on broad Taproot overview material.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="32" t="str">
-        <x:v>protocol.taptree</x:v>
+        <x:v>protocol.coinbase-transaction</x:v>
       </x:c>
       <x:c r="B32" s="32" t="str">
-        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
+        <x:v>economics.block-subsidy</x:v>
       </x:c>
       <x:c r="C32" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12855,21 +13204,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E32" s="32" t="str">
-        <x:v>The inclusion proof only makes sense after the learner understands the TapTree structure.</x:v>
+        <x:v>The block subsidy is the newly issued component claimed by a coinbase transaction.</x:v>
       </x:c>
       <x:c r="F32" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G32" s="32" t="str">
-        <x:v>Source-driven bridge edge.</x:v>
+        <x:v>The coinbase node already carries the halving prerequisite, so no redundant direct halving edge is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="32" t="str">
-        <x:v>protocol.taptree</x:v>
+        <x:v>fundamentals.digital-signatures</x:v>
       </x:c>
       <x:c r="B33" s="32" t="str">
-        <x:v>protocol.huffman-optimized-taptrees</x:v>
+        <x:v>security.quantum-computing-threat</x:v>
       </x:c>
       <x:c r="C33" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12878,10 +13227,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E33" s="32" t="str">
-        <x:v>Huffman optimization is a refinement of how TapTree leaves are arranged.</x:v>
+        <x:v>Quantum attacks on public-key authorization require understanding ordinary Bitcoin signature security first.</x:v>
       </x:c>
       <x:c r="F33" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G33" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12889,10 +13238,10 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="32" t="str">
-        <x:v>protocol.softfork-hardfork</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B34" s="32" t="str">
-        <x:v>protocol.chain-split-risk</x:v>
+        <x:v>extension.ordinals-inscriptions</x:v>
       </x:c>
       <x:c r="C34" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12901,21 +13250,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E34" s="32" t="str">
-        <x:v>Split risk is a downstream consequence of incompatible upgrade paths, so learners should understand the compatibility boundary first.</x:v>
+        <x:v>The source explains inscriptions as a Taproot-era witness-data application.</x:v>
       </x:c>
       <x:c r="F34" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G34" s="32" t="str">
-        <x:v>Direct edge chosen over activation-history case studies because those are downstream examples, not prerequisites.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.witness-structure</x:v>
       </x:c>
       <x:c r="B35" s="32" t="str">
-        <x:v>protocol.tapscript</x:v>
+        <x:v>extension.ordinals-inscriptions</x:v>
       </x:c>
       <x:c r="C35" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12924,21 +13273,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E35" s="32" t="str">
-        <x:v>Tapscript is a Taproot-specific script version, so learners need the Taproot spend context before its rule changes make sense.</x:v>
+        <x:v>Witness structure is needed to understand where inscription data is carried and how it affects block space.</x:v>
       </x:c>
       <x:c r="F35" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G35" s="32" t="str">
-        <x:v>Direct edge keeps the node scoped to the Taproot family without collapsing it into a generic script refresher.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="32" t="str">
-        <x:v>custody.psbt</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="B36" s="32" t="str">
-        <x:v>dev.taproot-psbt-fields</x:v>
+        <x:v>extension.proof-of-existence</x:v>
       </x:c>
       <x:c r="C36" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12947,21 +13296,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E36" s="32" t="str">
-        <x:v>Taproot PSBT fields extend the base PSBT container, so learners need the general workflow and field model before the Taproot additions make sense.</x:v>
+        <x:v>Timestamp proofs commit evidence without requiring the complete document to be stored on-chain.</x:v>
       </x:c>
       <x:c r="F36" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G36" s="32" t="str">
-        <x:v>Direct edge keeps the slice anchored on the generic PSBT exchange model rather than on a narrower implementation variant.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.tagged-hashes</x:v>
       </x:c>
       <x:c r="B37" s="32" t="str">
-        <x:v>dev.taproot-psbt-fields</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="C37" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12970,21 +13319,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E37" s="32" t="str">
-        <x:v>These fields carry Taproot-specific keys, scripts, and Merkle-path data, so learners need the Taproot spend model before the PSBT extensions are meaningful.</x:v>
+        <x:v>TapTweak is defined using tagged hashes directly in Taproot key tweaking.</x:v>
       </x:c>
       <x:c r="F37" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G37" s="32" t="str">
-        <x:v>The direct dev.psbt-v2 edge was intentionally dropped because BIP371 applies to PSBTv0 and PSBTv2.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="32" t="str">
-        <x:v>protocol.softfork-hardfork</x:v>
+        <x:v>protocol.x-only-public-keys</x:v>
       </x:c>
       <x:c r="B38" s="32" t="str">
-        <x:v>protocol.accidental-confiscation</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="C38" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12993,21 +13342,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E38" s="32" t="str">
-        <x:v>Accidental confiscation is a failure mode caused by new soft-fork restrictions, so learners need the soft-fork compatibility model before the risk is intelligible.</x:v>
+        <x:v>TapTweak operates on x-only public keys in the Taproot construction.</x:v>
       </x:c>
       <x:c r="F38" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G38" s="32" t="str">
-        <x:v>Direct edge chosen over chain-split-risk and standardness-policy because those branches add context but are not required for the core failure mode.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="32" t="str">
-        <x:v>protocol.fee-market</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="B39" s="32" t="str">
-        <x:v>custody.coin-selection</x:v>
+        <x:v>protocol.taproot-key-path-spends</x:v>
       </x:c>
       <x:c r="C39" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13016,21 +13365,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E39" s="32" t="str">
-        <x:v>Wallets choose different UTXO sets partly to minimize transaction size and fee cost, so fee pressure is a direct part of the concept.</x:v>
+        <x:v>A key-path spend verifies against the tweaked Taproot output key, so learners need the tweak mechanism before the spending mode makes sense.</x:v>
       </x:c>
       <x:c r="F39" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G39" s="32" t="str">
-        <x:v>Direct edge keeps the node connected to transaction-cost tradeoffs rather than only to wallet UX.</x:v>
+        <x:v>Direct parent keeps the node focused on the spend mode rather than on broad Taproot overview material.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>protocol.taptree</x:v>
       </x:c>
       <x:c r="B40" s="32" t="str">
-        <x:v>protocol.change-outputs</x:v>
+        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
       </x:c>
       <x:c r="C40" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13039,21 +13388,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E40" s="32" t="str">
-        <x:v>Change is a specific kind of transaction output, so learners need the basic output and spendability model before the leftover-value pattern makes sense.</x:v>
+        <x:v>The inclusion proof only makes sense after the learner understands the TapTree structure.</x:v>
       </x:c>
       <x:c r="F40" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G40" s="32" t="str">
-        <x:v>Direct edge keeps the node between raw output structure and the later wallet-decision branch.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>protocol.taptree</x:v>
       </x:c>
       <x:c r="B41" s="32" t="str">
-        <x:v>dev.taproot-descriptors</x:v>
+        <x:v>protocol.huffman-optimized-taptrees</x:v>
       </x:c>
       <x:c r="C41" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13062,21 +13411,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E41" s="32" t="str">
-        <x:v>Taproot descriptors extend the general descriptor grammar, so learners need the base descriptor model before the tr() specialization makes sense.</x:v>
+        <x:v>Huffman optimization is a refinement of how TapTree leaves are arranged.</x:v>
       </x:c>
       <x:c r="F41" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G41" s="32" t="str">
-        <x:v>Direct edge keeps the node scoped to descriptor structure instead of wallet import behavior.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.softfork-hardfork</x:v>
       </x:c>
       <x:c r="B42" s="32" t="str">
-        <x:v>dev.taproot-descriptors</x:v>
+        <x:v>protocol.chain-split-risk</x:v>
       </x:c>
       <x:c r="C42" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13085,21 +13434,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E42" s="32" t="str">
-        <x:v>The tr() descriptor exists specifically to encode P2TR outputs and optional Taproot script-path commitments, so learners need the Taproot output model first.</x:v>
+        <x:v>Split risk is a downstream consequence of incompatible upgrade paths, so learners should understand the compatibility boundary first.</x:v>
       </x:c>
       <x:c r="F42" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G42" s="32" t="str">
-        <x:v>Direct edge keeps the node grounded in Taproot output semantics rather than in generic descriptor syntax alone.</x:v>
+        <x:v>Direct edge chosen over activation-history case studies because those are downstream examples, not prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="32" t="str">
-        <x:v>protocol.transaction-pinning</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B43" s="32" t="str">
-        <x:v>protocol.version-3-transaction-relay</x:v>
+        <x:v>protocol.tapscript</x:v>
       </x:c>
       <x:c r="C43" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13108,21 +13457,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E43" s="32" t="str">
-        <x:v>Version 3 relay is a targeted policy response to transaction pinning, so learners should understand the attack class before the mitigation.</x:v>
+        <x:v>Tapscript is a Taproot-specific script version, so learners need the Taproot spend context before its rule changes make sense.</x:v>
       </x:c>
       <x:c r="F43" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G43" s="32" t="str">
-        <x:v>Direct edge chosen over package-relay because the pinning problem is the narrower immediate teaching need.</x:v>
+        <x:v>Direct edge keeps the node scoped to the Taproot family without collapsing it into a generic script refresher.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="32" t="str">
-        <x:v>fundamentals.trustlessness</x:v>
+        <x:v>custody.psbt</x:v>
       </x:c>
       <x:c r="B44" s="32" t="str">
-        <x:v>fundamentals.validation-sovereignty</x:v>
+        <x:v>dev.taproot-psbt-fields</x:v>
       </x:c>
       <x:c r="C44" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13131,21 +13480,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E44" s="32" t="str">
-        <x:v>Validation sovereignty is an applied consequence of trustlessness and verification culture.</x:v>
+        <x:v>Taproot PSBT fields extend the base PSBT container, so learners need the general workflow and field model before the Taproot additions make sense.</x:v>
       </x:c>
       <x:c r="F44" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G44" s="32" t="str">
-        <x:v>Bridge edge inferred from philosophy sequencing.</x:v>
+        <x:v>Direct edge keeps the slice anchored on the generic PSBT exchange model rather than on a narrower implementation variant.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="32" t="str">
-        <x:v>ops.run-full-node</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B45" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>dev.taproot-psbt-fields</x:v>
       </x:c>
       <x:c r="C45" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13154,21 +13503,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E45" s="32" t="str">
-        <x:v>Learners need the full-node baseline before they can understand which validation guarantees a light client gives up.</x:v>
+        <x:v>These fields carry Taproot-specific keys, scripts, and Merkle-path data, so learners need the Taproot spend model before the PSBT extensions are meaningful.</x:v>
       </x:c>
       <x:c r="F45" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G45" s="32" t="str">
-        <x:v>Bridge edge inferred from full-node versus lightweight-client contrast.</x:v>
+        <x:v>The direct dev.psbt-v2 edge was intentionally dropped because BIP371 applies to PSBTv0 and PSBTv2.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="32" t="str">
-        <x:v>protocol.compact-block-filters</x:v>
+        <x:v>protocol.softfork-hardfork</x:v>
       </x:c>
       <x:c r="B46" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>protocol.accidental-confiscation</x:v>
       </x:c>
       <x:c r="C46" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13177,21 +13526,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E46" s="32" t="str">
-        <x:v>Compact block filters provide the modern filtered-client mechanism that anchors the trust-model comparison.</x:v>
+        <x:v>Accidental confiscation is a failure mode caused by new soft-fork restrictions, so learners need the soft-fork compatibility model before the risk is intelligible.</x:v>
       </x:c>
       <x:c r="F46" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G46" s="32" t="str">
-        <x:v>Kept additive and conceptual instead of rewiring older light-client mechanism leaves in the same slice.</x:v>
+        <x:v>Direct edge chosen over chain-split-risk and standardness-policy because those branches add context but are not required for the core failure mode.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="32" t="str">
-        <x:v>fundamentals.validation-sovereignty</x:v>
+        <x:v>protocol.fee-market</x:v>
       </x:c>
       <x:c r="B47" s="32" t="str">
-        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
+        <x:v>custody.coin-selection</x:v>
       </x:c>
       <x:c r="C47" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13200,21 +13549,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E47" s="32" t="str">
-        <x:v>The comparison only matters once the learner understands why self-validation is valuable in the first place.</x:v>
+        <x:v>Wallets choose different UTXO sets partly to minimize transaction size and fee cost, so fee pressure is a direct part of the concept.</x:v>
       </x:c>
       <x:c r="F47" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G47" s="32" t="str">
-        <x:v>User-facing prerequisite edge for the wallet-mode decision.</x:v>
+        <x:v>Direct edge keeps the node connected to transaction-cost tradeoffs rather than only to wallet UX.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B48" s="32" t="str">
-        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
+        <x:v>protocol.change-outputs</x:v>
       </x:c>
       <x:c r="C48" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13223,21 +13572,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E48" s="32" t="str">
-        <x:v>Learners need the mechanism-level trust tradeoffs before comparing full-node wallets with lightweight clients.</x:v>
+        <x:v>Change is a specific kind of transaction output, so learners need the basic output and spendability model before the leftover-value pattern makes sense.</x:v>
       </x:c>
       <x:c r="F48" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G48" s="32" t="str">
-        <x:v>First downstream consumer for the light-client trust branch.</x:v>
+        <x:v>Direct edge keeps the node between raw output structure and the later wallet-decision branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B49" s="32" t="str">
-        <x:v>protocol.p2pk</x:v>
+        <x:v>dev.taproot-descriptors</x:v>
       </x:c>
       <x:c r="C49" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13246,21 +13595,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E49" s="32" t="str">
-        <x:v>P2PK is a concrete legacy script template, so learners first need the locking and unlocking model from Bitcoin Script.</x:v>
+        <x:v>Taproot descriptors extend the general descriptor grammar, so learners need the base descriptor model before the tr() specialization makes sense.</x:v>
       </x:c>
       <x:c r="F49" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G49" s="32" t="str">
-        <x:v>Chosen as the first script-history leaf from Decoding after dedupe and direct-edge review.</x:v>
+        <x:v>Direct edge keeps the node scoped to descriptor structure instead of wallet import behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="32" t="str">
-        <x:v>fundamentals.schnorr-signatures</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B50" s="32" t="str">
-        <x:v>security.nonce-reuse-attack</x:v>
+        <x:v>dev.taproot-descriptors</x:v>
       </x:c>
       <x:c r="C50" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13269,21 +13618,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E50" s="32" t="str">
-        <x:v>The nonce-reuse failure only makes sense after the learner understands the Schnorr signing flow that produces the nonce and signature pair.</x:v>
+        <x:v>The tr() descriptor exists specifically to encode P2TR outputs and optional Taproot script-path commitments, so learners need the Taproot output model first.</x:v>
       </x:c>
       <x:c r="F50" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G50" s="32" t="str">
-        <x:v>Chosen as a narrow additive security slice without bundling it to custody-side defenses.</x:v>
+        <x:v>Direct edge keeps the node grounded in Taproot output semantics rather than in generic descriptor syntax alone.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="32" t="str">
-        <x:v>protocol.p2pk</x:v>
+        <x:v>protocol.transaction-pinning</x:v>
       </x:c>
       <x:c r="B51" s="32" t="str">
-        <x:v>protocol.p2pkh</x:v>
+        <x:v>protocol.version-3-transaction-relay</x:v>
       </x:c>
       <x:c r="C51" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13292,21 +13641,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E51" s="32" t="str">
-        <x:v>P2PKH is easiest to understand as the hashed-public-key refinement of a direct public-key output.</x:v>
+        <x:v>Version 3 relay is a targeted policy response to transaction pinning, so learners should understand the attack class before the mitigation.</x:v>
       </x:c>
       <x:c r="F51" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G51" s="32" t="str">
-        <x:v>Chosen to preserve the output-template ladder without repeating the broader Script prerequisite directly.</x:v>
+        <x:v>Direct edge chosen over package-relay because the pinning problem is the narrower immediate teaching need.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>fundamentals.trustlessness</x:v>
       </x:c>
       <x:c r="B52" s="32" t="str">
-        <x:v>protocol.p2pkh</x:v>
+        <x:v>fundamentals.validation-sovereignty</x:v>
       </x:c>
       <x:c r="C52" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13315,21 +13664,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E52" s="32" t="str">
-        <x:v>Hash-based locking only makes sense once the learner understands what a hash commits to and why it can stand in for the public key until spend time.</x:v>
+        <x:v>Validation sovereignty is an applied consequence of trustlessness and verification culture.</x:v>
       </x:c>
       <x:c r="F52" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G52" s="32" t="str">
-        <x:v>Required to keep the node about public-key hashing rather than just script syntax.</x:v>
+        <x:v>Bridge edge inferred from philosophy sequencing.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>ops.run-full-node</x:v>
       </x:c>
       <x:c r="B53" s="32" t="str">
-        <x:v>protocol.op-checkmultisig</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="C53" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13338,21 +13687,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E53" s="32" t="str">
-        <x:v>OP_CHECKMULTISIG is an opcode-level script mechanic, so learners first need the general Script model and stack execution basics.</x:v>
+        <x:v>Learners need the full-node baseline before they can understand which validation guarantees a light client gives up.</x:v>
       </x:c>
       <x:c r="F53" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G53" s="32" t="str">
-        <x:v>Chosen as the mechanism bridge before protocol.p2ms.</x:v>
+        <x:v>Bridge edge inferred from full-node versus lightweight-client contrast.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="32" t="str">
-        <x:v>protocol.op-checkmultisig</x:v>
+        <x:v>protocol.compact-block-filters</x:v>
       </x:c>
       <x:c r="B54" s="32" t="str">
-        <x:v>protocol.p2ms</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="C54" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13361,21 +13710,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E54" s="32" t="str">
-        <x:v>Bare multisig is the concrete locking template built from OP_CHECKMULTISIG, so the opcode is the clean direct parent once introduced.</x:v>
+        <x:v>Compact block filters provide the modern filtered-client mechanism that anchors the trust-model comparison.</x:v>
       </x:c>
       <x:c r="F54" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G54" s="32" t="str">
-        <x:v>Replaces the earlier curricular and wallet-semantic parent candidates.</x:v>
+        <x:v>Kept additive and conceptual instead of rewiring older light-client mechanism leaves in the same slice.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="32" t="str">
-        <x:v>protocol.p2ms</x:v>
+        <x:v>fundamentals.validation-sovereignty</x:v>
       </x:c>
       <x:c r="B55" s="32" t="str">
-        <x:v>protocol.bare-multisig-standardness</x:v>
+        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
       </x:c>
       <x:c r="C55" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13384,21 +13733,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E55" s="32" t="str">
-        <x:v>The relay treatment only makes sense once the learner understands what a bare multisig output actually is on-chain.</x:v>
+        <x:v>The comparison only matters once the learner understands why self-validation is valuable in the first place.</x:v>
       </x:c>
       <x:c r="F55" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G55" s="32" t="str">
-        <x:v>Policy leaf anchored on the specific legacy script template it constrains.</x:v>
+        <x:v>User-facing prerequisite edge for the wallet-mode decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="32" t="str">
-        <x:v>protocol.standardness-policy</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="B56" s="32" t="str">
-        <x:v>protocol.bare-multisig-standardness</x:v>
+        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
       </x:c>
       <x:c r="C56" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13407,21 +13756,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E56" s="32" t="str">
-        <x:v>This node is a concrete application of standard transaction policy, so the general standardness concept should come first.</x:v>
+        <x:v>Learners need the mechanism-level trust tradeoffs before comparing full-node wallets with lightweight clients.</x:v>
       </x:c>
       <x:c r="F56" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G56" s="32" t="str">
-        <x:v>Policy-boundary prerequisite inherited through the existing mempool-policy branch.</x:v>
+        <x:v>First downstream consumer for the light-client trust branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B57" s="32" t="str">
-        <x:v>dev.scriptpubkeymanagers</x:v>
+        <x:v>protocol.p2pk</x:v>
       </x:c>
       <x:c r="C57" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13430,21 +13779,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E57" s="32" t="str">
-        <x:v>Modern descriptor wallets hand descriptor-backed script templates to dedicated managers, so learners need the descriptor model before the SPKM boundary makes sense.</x:v>
+        <x:v>P2PK is a concrete legacy script template, so learners first need the locking and unlocking model from Bitcoin Script.</x:v>
       </x:c>
       <x:c r="F57" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-wallet</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G57" s="32" t="str">
-        <x:v>Direct edge distinguishes the Core wallet abstraction from descriptor syntax without collapsing the two concepts into one node.</x:v>
+        <x:v>Chosen as the first script-history leaf from Decoding after dedupe and direct-edge review.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="32" t="str">
-        <x:v>protocol.mempool</x:v>
+        <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="B58" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>security.nonce-reuse-attack</x:v>
       </x:c>
       <x:c r="C58" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13453,21 +13802,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E58" s="32" t="str">
-        <x:v>The unbroadcast set is a mempool-owned data structure, so learners need the local unconfirmed transaction pool model before this narrower tracking mechanism makes sense.</x:v>
+        <x:v>The nonce-reuse failure only makes sense after the learner understands the Schnorr signing flow that produces the nonce and signature pair.</x:v>
       </x:c>
       <x:c r="F58" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G58" s="32" t="str">
-        <x:v>Direct edge keeps the concept scoped to local transaction state rather than broader relay policy.</x:v>
+        <x:v>Chosen as a narrow additive security slice without bundling it to custody-side defenses.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="32" t="str">
-        <x:v>protocol.transaction-relay-inv-getdata</x:v>
+        <x:v>protocol.p2pk</x:v>
       </x:c>
       <x:c r="B59" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>protocol.p2pkh</x:v>
       </x:c>
       <x:c r="C59" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13476,21 +13825,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E59" s="32" t="str">
-        <x:v>This set only matters because nodes need to distinguish locally submitted transactions from those later observed through the network relay path and may retry announcing them.</x:v>
+        <x:v>P2PKH is easiest to understand as the hashed-public-key refinement of a direct public-key output.</x:v>
       </x:c>
       <x:c r="F59" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G59" s="32" t="str">
-        <x:v>Direct edge ties the mechanism to network propagation confirmation and rebroadcast attempts.</x:v>
+        <x:v>Chosen to preserve the output-template ladder without repeating the broader Script prerequisite directly.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="32" t="str">
-        <x:v>privacy.address-reuse</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B60" s="32" t="str">
-        <x:v>custody.human-readable-addresses</x:v>
+        <x:v>protocol.p2pkh</x:v>
       </x:c>
       <x:c r="C60" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13499,21 +13848,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E60" s="32" t="str">
-        <x:v>A major design constraint is that reusable human-readable handles can worsen privacy unless they resolve to reusable payment mechanisms or rotate safely, so learners need the address-reuse problem first.</x:v>
+        <x:v>Hash-based locking only makes sense once the learner understands what a hash commits to and why it can stand in for the public key until spend time.</x:v>
       </x:c>
       <x:c r="F60" s="32" t="str">
-        <x:v>source.bitcoin-design-payment-formats</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G60" s="32" t="str">
-        <x:v>Direct edge captures the main privacy tradeoff without forcing downstream protocol-specific address schemes into prerequisites.</x:v>
+        <x:v>Required to keep the node about public-key hashing rather than just script syntax.</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="32" t="str">
-        <x:v>custody.output-labeling</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B61" s="32" t="str">
-        <x:v>custody.transaction-metadata</x:v>
+        <x:v>protocol.op-checkmultisig</x:v>
       </x:c>
       <x:c r="C61" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13522,21 +13871,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E61" s="32" t="str">
-        <x:v>Output labeling already introduces the idea that wallets attach their own context to payments and spendable objects, making it the cleanest direct bridge into broader transaction-level notes, contacts, and portability concerns.</x:v>
+        <x:v>OP_CHECKMULTISIG is an opcode-level script mechanic, so learners first need the general Script model and stack execution basics.</x:v>
       </x:c>
       <x:c r="F61" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G61" s="32" t="str">
-        <x:v>Direct edge distinguishes wider payment-history context from narrower spend-control labels without treating them as unrelated.</x:v>
+        <x:v>Chosen as the mechanism bridge before protocol.p2ms.</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>protocol.op-checkmultisig</x:v>
       </x:c>
       <x:c r="B62" s="32" t="str">
-        <x:v>custody.transaction-metadata</x:v>
+        <x:v>protocol.p2ms</x:v>
       </x:c>
       <x:c r="C62" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13545,21 +13894,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E62" s="32" t="str">
-        <x:v>Wallet-added names, notes, and contact links matter partly because transaction history is only pseudonymous and can reveal meaningful patterns when users or tools correlate activity over time.</x:v>
+        <x:v>Bare multisig is the concrete locking template built from OP_CHECKMULTISIG, so the opcode is the clean direct parent once introduced.</x:v>
       </x:c>
       <x:c r="F62" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G62" s="32" t="str">
-        <x:v>Direct edge keeps the node tied to the privacy and identity meaning of payment history rather than only to generic lifecycle sequencing.</x:v>
+        <x:v>Replaces the earlier curricular and wallet-semantic parent candidates.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="32" t="str">
-        <x:v>custody.self-custody</x:v>
+        <x:v>protocol.p2ms</x:v>
       </x:c>
       <x:c r="B63" s="32" t="str">
-        <x:v>custody.multiple-wallets</x:v>
+        <x:v>protocol.bare-multisig-standardness</x:v>
       </x:c>
       <x:c r="C63" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13568,21 +13917,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E63" s="32" t="str">
-        <x:v>Deliberately separating funds across different wallet buckets is a custody decision, so learners need the base self-custody responsibility model before the organizational pattern makes sense.</x:v>
+        <x:v>The relay treatment only makes sense once the learner understands what a bare multisig output actually is on-chain.</x:v>
       </x:c>
       <x:c r="F63" s="32" t="str">
-        <x:v>source.bitcoin-design-multiple-wallets</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G63" s="32" t="str">
-        <x:v>Kept the direct parent at the responsibility-model layer; multisig, watch-only, and HD account structures remain examples or implementation details rather than prerequisites.</x:v>
+        <x:v>Policy leaf anchored on the specific legacy script template it constrains.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="32" t="str">
-        <x:v>custody.hardware-wallets</x:v>
+        <x:v>protocol.standardness-policy</x:v>
       </x:c>
       <x:c r="B64" s="32" t="str">
-        <x:v>custody.progressive-security</x:v>
+        <x:v>protocol.bare-multisig-standardness</x:v>
       </x:c>
       <x:c r="C64" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13591,21 +13940,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E64" s="32" t="str">
-        <x:v>One of the core upgrade steps in the reference design is moving from default low-friction storage to an external signing device, so learners need the hardware-signing model before the staged-upgrade pattern makes sense.</x:v>
+        <x:v>This node is a concrete application of standard transaction policy, so the general standardness concept should come first.</x:v>
       </x:c>
       <x:c r="F64" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G64" s="32" t="str">
-        <x:v>Direct edge captures the mid-tier upgrade target without treating cloud backup itself as the core concept.</x:v>
+        <x:v>Policy-boundary prerequisite inherited through the existing mempool-policy branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B65" s="32" t="str">
-        <x:v>custody.progressive-security</x:v>
+        <x:v>dev.scriptpubkeymanagers</x:v>
       </x:c>
       <x:c r="C65" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13614,21 +13963,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E65" s="32" t="str">
-        <x:v>The higher-security end of the progression moves into 2-of-3 and 3-of-5 multi-key schemes, so learners need the multisig model before they can reason about why and when a wallet should escalate there.</x:v>
+        <x:v>Modern descriptor wallets hand descriptor-backed script templates to dedicated managers, so learners need the descriptor model before the SPKM boundary makes sense.</x:v>
       </x:c>
       <x:c r="F65" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoin-core-academy-wallet</x:v>
       </x:c>
       <x:c r="G65" s="32" t="str">
-        <x:v>Direct edge captures the high-assurance destination of the progression rather than a specific product flow.</x:v>
+        <x:v>Direct edge distinguishes the Core wallet abstraction from descriptor syntax without collapsing the two concepts into one node.</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="32" t="str">
+        <x:v>protocol.mempool</x:v>
+      </x:c>
+      <x:c r="B66" s="32" t="str">
         <x:v>protocol.mempool-unbroadcast-set</x:v>
-      </x:c>
-      <x:c r="B66" s="32" t="str">
-        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
       </x:c>
       <x:c r="C66" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13637,21 +13986,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E66" s="32" t="str">
-        <x:v>Rebroadcast privacy builds directly on the local-node distinction between transactions merely accepted into the mempool and transactions known to have propagated, which is exactly the gap the unbroadcast set tracks.</x:v>
+        <x:v>The unbroadcast set is a mempool-owned data structure, so learners need the local unconfirmed transaction pool model before this narrower tracking mechanism makes sense.</x:v>
       </x:c>
       <x:c r="F66" s="32" t="str">
         <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G66" s="32" t="str">
-        <x:v>Direct parent keeps the slice on the local tracking mechanism rather than reintroducing generic relay ancestors.</x:v>
+        <x:v>Direct edge keeps the concept scoped to local transaction state rather than broader relay policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>protocol.transaction-relay-inv-getdata</x:v>
       </x:c>
       <x:c r="B67" s="32" t="str">
-        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="C67" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13660,21 +14009,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E67" s="32" t="str">
-        <x:v>Different rebroadcast patterns matter because observers can correlate network behavior with public transaction history and infer likely origin, so learners need the pseudonymity and linkage problem first.</x:v>
+        <x:v>This set only matters because nodes need to distinguish locally submitted transactions from those later observed through the network relay path and may retry announcing them.</x:v>
       </x:c>
       <x:c r="F67" s="32" t="str">
         <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G67" s="32" t="str">
-        <x:v>Direct parent keeps the node focused on why relay-side origin leakage matters, not just how rebroadcast code works.</x:v>
+        <x:v>Direct edge ties the mechanism to network propagation confirmation and rebroadcast attempts.</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="32" t="str">
-        <x:v>protocol.segregated-witness</x:v>
+        <x:v>privacy.address-reuse</x:v>
       </x:c>
       <x:c r="B68" s="32" t="str">
-        <x:v>protocol.txid-vs-wtxid</x:v>
+        <x:v>custody.human-readable-addresses</x:v>
       </x:c>
       <x:c r="C68" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13683,21 +14032,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E68" s="32" t="str">
-        <x:v>The identifier split only exists because SegWit introduces a witness-inclusive serialization alongside the legacy serialization, so learners need the SegWit structure change before the two IDs make sense.</x:v>
+        <x:v>A major design constraint is that reusable human-readable handles can worsen privacy unless they resolve to reusable payment mechanisms or rotate safely, so learners need the address-reuse problem first.</x:v>
       </x:c>
       <x:c r="F68" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-payment-formats</x:v>
       </x:c>
       <x:c r="G68" s="32" t="str">
-        <x:v>Direct parent keeps the bridge on the serialization distinction instead of reintroducing downstream relay consequences.</x:v>
+        <x:v>Direct edge captures the main privacy tradeoff without forcing downstream protocol-specific address schemes into prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="32" t="str">
-        <x:v>protocol.txid-vs-wtxid</x:v>
+        <x:v>custody.output-labeling</x:v>
       </x:c>
       <x:c r="B69" s="32" t="str">
-        <x:v>protocol.wtxid-relay-bip339</x:v>
+        <x:v>custody.transaction-metadata</x:v>
       </x:c>
       <x:c r="C69" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13706,21 +14055,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E69" s="32" t="str">
-        <x:v>WTXID relay is specifically the choice to announce and request witness-bearing transactions by wtxid instead of txid, so the learner should understand the two identifier forms before the relay mode change.</x:v>
+        <x:v>Output labeling already introduces the idea that wallets attach their own context to payments and spendable objects, making it the cleanest direct bridge into broader transaction-level notes, contacts, and portability concerns.</x:v>
       </x:c>
       <x:c r="F69" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="G69" s="32" t="str">
-        <x:v>Added as a graph bridge so the existing relay node no longer has to explain the identifier distinction internally.</x:v>
+        <x:v>Direct edge distinguishes wider payment-history context from narrower spend-control labels without treating them as unrelated.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="32" t="str">
-        <x:v>fundamentals.schnorr-signatures</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B70" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>custody.transaction-metadata</x:v>
       </x:c>
       <x:c r="C70" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13729,21 +14078,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E70" s="32" t="str">
-        <x:v>MuSig is a Schnorr aggregation protocol, so learners need the underlying Schnorr key and signature model before the combined-key protocol makes sense.</x:v>
+        <x:v>Wallet-added names, notes, and contact links matter partly because transaction history is only pseudonymous and can reveal meaningful patterns when users or tools correlate activity over time.</x:v>
       </x:c>
       <x:c r="F70" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="G70" s="32" t="str">
-        <x:v>Direct parent kept narrow; wallet-level multisig and Taproot remain context rather than prerequisites.</x:v>
+        <x:v>Direct edge keeps the node tied to the privacy and identity meaning of payment history rather than only to generic lifecycle sequencing.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>custody.self-custody</x:v>
       </x:c>
       <x:c r="B71" s="32" t="str">
-        <x:v>dev.descriptor-wallet-policies</x:v>
+        <x:v>custody.multiple-wallets</x:v>
       </x:c>
       <x:c r="C71" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13752,21 +14101,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E71" s="32" t="str">
-        <x:v>Wallet policies are built as descriptor templates, so the base descriptor language and template structure must come first.</x:v>
+        <x:v>Deliberately separating funds across different wallet buckets is a custody decision, so learners need the base self-custody responsibility model before the organizational pattern makes sense.</x:v>
       </x:c>
       <x:c r="F71" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-design-multiple-wallets</x:v>
       </x:c>
       <x:c r="G71" s="32" t="str">
-        <x:v>Direct parent kept above import or signer flows because the node is about the representation itself.</x:v>
+        <x:v>Kept the direct parent at the responsibility-model layer; multisig, watch-only, and HD account structures remain examples or implementation details rather than prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="32" t="str">
-        <x:v>dev.bip32</x:v>
+        <x:v>custody.hardware-wallets</x:v>
       </x:c>
       <x:c r="B72" s="32" t="str">
-        <x:v>dev.descriptor-wallet-policies</x:v>
+        <x:v>custody.progressive-security</x:v>
       </x:c>
       <x:c r="C72" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13775,21 +14124,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E72" s="32" t="str">
-        <x:v>BIP388 key information items package xpubs and derivation origins, so learners need the HD derivation model before the portable wallet-policy format makes sense.</x:v>
+        <x:v>One of the core upgrade steps in the reference design is moving from default low-friction storage to an external signing device, so learners need the hardware-signing model before the staged-upgrade pattern makes sense.</x:v>
       </x:c>
       <x:c r="F72" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="G72" s="32" t="str">
-        <x:v>Non-redundant alongside dev.descriptors because neither concept implies the other in the current graph.</x:v>
+        <x:v>Direct edge captures the mid-tier upgrade target without treating cloud backup itself as the core concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B73" s="32" t="str">
-        <x:v>dev.descriptors-in-psbt</x:v>
+        <x:v>custody.progressive-security</x:v>
       </x:c>
       <x:c r="C73" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13798,21 +14147,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E73" s="32" t="str">
-        <x:v>The node is about carrying descriptor information during transaction coordination, so learners need the descriptor syntax and script-template model first.</x:v>
+        <x:v>The higher-security end of the progression moves into 2-of-3 and 3-of-5 multi-key schemes, so learners need the multisig model before they can reason about why and when a wallet should escalate there.</x:v>
       </x:c>
       <x:c r="F73" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="G73" s="32" t="str">
-        <x:v>Direct parent kept at the representation layer rather than the wallet-policy or taproot-specific refinements.</x:v>
+        <x:v>Direct edge captures the high-assurance destination of the progression rather than a specific product flow.</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="32" t="str">
-        <x:v>custody.psbt</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="B74" s="32" t="str">
-        <x:v>dev.descriptors-in-psbt</x:v>
+        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
       </x:c>
       <x:c r="C74" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13821,21 +14170,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E74" s="32" t="str">
-        <x:v>Descriptor-aware exchange only makes sense after the learner understands the general PSBT coordination workflow that transports signing-related data between tools.</x:v>
+        <x:v>Rebroadcast privacy builds directly on the local-node distinction between transactions merely accepted into the mempool and transactions known to have propagated, which is exactly the gap the unbroadcast set tracks.</x:v>
       </x:c>
       <x:c r="F74" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G74" s="32" t="str">
-        <x:v>Direct parent kept at the base PSBT workflow level instead of requiring later version-specific extensions.</x:v>
+        <x:v>Direct parent keeps the slice on the local tracking mechanism rather than reintroducing generic relay ancestors.</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B75" s="32" t="str">
-        <x:v>custody.degrading-multisig</x:v>
+        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
       </x:c>
       <x:c r="C75" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13844,21 +14193,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E75" s="32" t="str">
-        <x:v>The policy only makes sense once the learner understands ordinary multisig threshold custody and why signers can be split into live and backup sets.</x:v>
+        <x:v>Different rebroadcast patterns matter because observers can correlate network behavior with public transaction history and infer likely origin, so learners need the pseudonymity and linkage problem first.</x:v>
       </x:c>
       <x:c r="F75" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G75" s="32" t="str">
-        <x:v>Direct custody parent for the signer-threshold side of the construction.</x:v>
+        <x:v>Direct parent keeps the node focused on why relay-side origin leakage matters, not just how rebroadcast code works.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="32" t="str">
-        <x:v>protocol.timelocks</x:v>
+        <x:v>protocol.segregated-witness</x:v>
       </x:c>
       <x:c r="B76" s="32" t="str">
-        <x:v>custody.degrading-multisig</x:v>
+        <x:v>protocol.txid-vs-wtxid</x:v>
       </x:c>
       <x:c r="C76" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13867,21 +14216,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E76" s="32" t="str">
-        <x:v>The degrading policy activates its weaker backup path only after a timeout, so timelock semantics are a direct part of the construction.</x:v>
+        <x:v>The identifier split only exists because SegWit introduces a witness-inclusive serialization alongside the legacy serialization, so learners need the SegWit structure change before the two IDs make sense.</x:v>
       </x:c>
       <x:c r="F76" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G76" s="32" t="str">
-        <x:v>Needed alongside custody.multisig because the learner must understand the temporal rule, not just the signer policy.</x:v>
+        <x:v>Direct parent keeps the bridge on the serialization distinction instead of reintroducing downstream relay consequences.</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="32" t="str">
-        <x:v>protocol.block-weight-vbytes</x:v>
+        <x:v>protocol.txid-vs-wtxid</x:v>
       </x:c>
       <x:c r="B77" s="32" t="str">
-        <x:v>protocol.fee-calculation</x:v>
+        <x:v>protocol.wtxid-relay-bip339</x:v>
       </x:c>
       <x:c r="C77" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13890,21 +14239,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E77" s="32" t="str">
-        <x:v>Understanding whether an absolute fee is high or low requires relating it to the blockspace pricing unit, so learners need weight and virtual bytes before fee calculation is fully meaningful in practice.</x:v>
+        <x:v>WTXID relay is specifically the choice to announce and request witness-bearing transactions by wtxid instead of txid, so the learner should understand the two identifier forms before the relay mode change.</x:v>
       </x:c>
       <x:c r="F77" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G77" s="32" t="str">
-        <x:v>Direct parent keeps the node at the mechanism layer without drifting into broader fee-market competition.</x:v>
+        <x:v>Added as a graph bridge so the existing relay node no longer has to explain the identifier distinction internally.</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="B78" s="32" t="str">
-        <x:v>protocol.bech32m-addresses</x:v>
+        <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="C78" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13913,21 +14262,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E78" s="32" t="str">
-        <x:v>Bech32m is an address-encoding format, so learners need the general relationship between addresses, script templates, and spendability before the newer checksum format is meaningful.</x:v>
+        <x:v>MuSig is a Schnorr aggregation protocol, so learners need the underlying Schnorr key and signature model before the combined-key protocol makes sense.</x:v>
       </x:c>
       <x:c r="F78" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G78" s="32" t="str">
-        <x:v>Direct parent keeps the node on encoding semantics rather than on raw string-format trivia.</x:v>
+        <x:v>Direct parent kept narrow; wallet-level multisig and Taproot remain context rather than prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B79" s="32" t="str">
-        <x:v>protocol.bech32m-addresses</x:v>
+        <x:v>dev.descriptor-wallet-policies</x:v>
       </x:c>
       <x:c r="C79" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13936,21 +14285,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E79" s="32" t="str">
-        <x:v>Bech32m became necessary for witness version 1 and higher, and Taproot is the first major deployed witness-v1 use case, so learners need that upgrade context before the format distinction makes sense.</x:v>
+        <x:v>Wallet policies are built as descriptor templates, so the base descriptor language and template structure must come first.</x:v>
       </x:c>
       <x:c r="F79" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G79" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored on the practical protocol transition that exposed Bech32m to users.</x:v>
+        <x:v>Direct parent kept above import or signer flows because the node is about the representation itself.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>dev.bip32</x:v>
       </x:c>
       <x:c r="B80" s="32" t="str">
-        <x:v>protocol.script-execution-stack</x:v>
+        <x:v>dev.descriptor-wallet-policies</x:v>
       </x:c>
       <x:c r="C80" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13959,21 +14308,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E80" s="32" t="str">
-        <x:v>The stack execution model is the direct mechanism by which Bitcoin Script evaluates spending conditions, so learners need the umbrella Script concept before drilling into stack behavior.</x:v>
+        <x:v>BIP388 key information items package xpubs and derivation origins, so learners need the HD derivation model before the portable wallet-policy format makes sense.</x:v>
       </x:c>
       <x:c r="F80" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G80" s="32" t="str">
-        <x:v>Direct parent positions the node as the conceptual middle layer between Script and opcode-specific leaves.</x:v>
+        <x:v>Non-redundant alongside dev.descriptors because neither concept implies the other in the current graph.</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="32" t="str">
-        <x:v>lightning.commitment-transactions</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B81" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>dev.descriptors-in-psbt</x:v>
       </x:c>
       <x:c r="C81" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13982,21 +14331,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E81" s="32" t="str">
-        <x:v>Per-commitment secrets are generated for each new commitment state, so learners need the commitment-transaction model before the secret-rotation mechanism makes sense.</x:v>
+        <x:v>The node is about carrying descriptor information during transaction coordination, so learners need the descriptor syntax and script-template model first.</x:v>
       </x:c>
       <x:c r="F81" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G81" s="32" t="str">
-        <x:v>Direct parent keeps the node on state evolution rather than on later punishment or watchtower behavior.</x:v>
+        <x:v>Direct parent kept at the representation layer rather than the wallet-policy or taproot-specific refinements.</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>custody.psbt</x:v>
       </x:c>
       <x:c r="B82" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>dev.descriptors-in-psbt</x:v>
       </x:c>
       <x:c r="C82" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14005,21 +14354,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E82" s="32" t="str">
-        <x:v>The to_local and to_remote scripts rely on per-state key derivation, revocation keys, and delayed-payment keys, so learners need the per-commitment secret machinery first.</x:v>
+        <x:v>Descriptor-aware exchange only makes sense after the learner understands the general PSBT coordination workflow that transports signing-related data between tools.</x:v>
       </x:c>
       <x:c r="F82" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G82" s="32" t="str">
-        <x:v>Direct parent keeps the node at the commitment-key layer instead of collapsing back into the broader commitment-transaction overview.</x:v>
+        <x:v>Direct parent kept at the base PSBT workflow level instead of requiring later version-specific extensions.</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="32" t="str">
-        <x:v>protocol.csv-bip112</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B83" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>custody.degrading-multisig</x:v>
       </x:c>
       <x:c r="C83" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14028,21 +14377,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E83" s="32" t="str">
-        <x:v>The delayed to_local branch is defined by a CSV-enforced waiting period, so learners need the relative-timelock opcode before the script template makes sense.</x:v>
+        <x:v>The policy only makes sense once the learner understands ordinary multisig threshold custody and why signers can be split into live and backup sets.</x:v>
       </x:c>
       <x:c r="F83" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G83" s="32" t="str">
-        <x:v>Direct parent captures the script-mechanism side of the concept without dragging in broader force-close or HTLC timing behavior.</x:v>
+        <x:v>Direct custody parent for the signer-threshold side of the construction.</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="32" t="str">
-        <x:v>protocol.difficulty-adjustment</x:v>
+        <x:v>protocol.timelocks</x:v>
       </x:c>
       <x:c r="B84" s="32" t="str">
-        <x:v>protocol.time-warp-attack</x:v>
+        <x:v>custody.degrading-multisig</x:v>
       </x:c>
       <x:c r="C84" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14051,21 +14400,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E84" s="32" t="str">
-        <x:v>The attack only makes sense once learners understand how Bitcoin retargets mining difficulty over long block windows.</x:v>
+        <x:v>The degrading policy activates its weaker backup path only after a timeout, so timelock semantics are a direct part of the construction.</x:v>
       </x:c>
       <x:c r="F84" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G84" s="32" t="str">
-        <x:v>Direct parent keeps the exploit tied to the retarget mechanism instead of burying it under generic mining vocabulary.</x:v>
+        <x:v>Needed alongside custody.multisig because the learner must understand the temporal rule, not just the signer policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="32" t="str">
-        <x:v>protocol.median-time-past</x:v>
+        <x:v>protocol.block-weight-vbytes</x:v>
       </x:c>
       <x:c r="B85" s="32" t="str">
-        <x:v>protocol.time-warp-attack</x:v>
+        <x:v>protocol.fee-calculation</x:v>
       </x:c>
       <x:c r="C85" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14074,21 +14423,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E85" s="32" t="str">
-        <x:v>Learners need the consensus timestamp constraints before they can reason about how miners manipulate time data and where the remaining attack surface lives.</x:v>
+        <x:v>Understanding whether an absolute fee is high or low requires relating it to the blockspace pricing unit, so learners need weight and virtual bytes before fee calculation is fully meaningful in practice.</x:v>
       </x:c>
       <x:c r="F85" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G85" s="32" t="str">
-        <x:v>Direct parent captures the timestamp-boundary side of the exploit without overloading timelocks or block headers.</x:v>
+        <x:v>Direct parent keeps the node at the mechanism layer without drifting into broader fee-market competition.</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="32" t="str">
-        <x:v>fundamentals.blind-signatures</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B86" s="32" t="str">
-        <x:v>history.chaumian-ecash</x:v>
+        <x:v>protocol.bech32m-addresses</x:v>
       </x:c>
       <x:c r="C86" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14097,21 +14446,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E86" s="32" t="str">
-        <x:v>Chaumian ecash is defined by using blind signatures to let a mint issue private bearer tokens without seeing the final token contents.</x:v>
+        <x:v>Bech32m is an address-encoding format, so learners need the general relationship between addresses, script templates, and spendability before the newer checksum format is meaningful.</x:v>
       </x:c>
       <x:c r="F86" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G86" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the specific cryptographic mechanism rather than treating it as generic digital-money history.</x:v>
+        <x:v>Direct parent keeps the node on encoding semantics rather than on raw string-format trivia.</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="32" t="str">
-        <x:v>history.double-spend-problem</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B87" s="32" t="str">
-        <x:v>history.chaumian-ecash</x:v>
+        <x:v>protocol.bech32m-addresses</x:v>
       </x:c>
       <x:c r="C87" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14120,21 +14469,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E87" s="32" t="str">
-        <x:v>Learners need the unsolved scarcity problem in digital cash before the trusted-mint tradeoff in Chaumian designs becomes meaningful.</x:v>
+        <x:v>Bech32m became necessary for witness version 1 and higher, and Taproot is the first major deployed witness-v1 use case, so learners need that upgrade context before the format distinction makes sense.</x:v>
       </x:c>
       <x:c r="F87" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G87" s="32" t="str">
-        <x:v>Direct parent frames why the system still needed a central operator even though it improved privacy.</x:v>
+        <x:v>Direct parent keeps the node anchored on the practical protocol transition that exposed Bech32m to users.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="32" t="str">
-        <x:v>economics.history-of-money</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B88" s="32" t="str">
-        <x:v>privacy.secret-right-to-cash</x:v>
+        <x:v>protocol.script-execution-stack</x:v>
       </x:c>
       <x:c r="C88" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14143,21 +14492,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E88" s="32" t="str">
-        <x:v>The concept depends on understanding how money moved from bearer cash toward mediated account systems, so learners need the long-run monetary history first.</x:v>
+        <x:v>The stack execution model is the direct mechanism by which Bitcoin Script evaluates spending conditions, so learners need the umbrella Script concept before drilling into stack behavior.</x:v>
       </x:c>
       <x:c r="F88" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G88" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the bearer-versus-intermediated payment shift rather than drifting into generic civil-liberties framing.</x:v>
+        <x:v>Direct parent positions the node as the conceptual middle layer between Script and opcode-specific leaves.</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="32" t="str">
-        <x:v>fundamentals.censorship-resistance</x:v>
+        <x:v>lightning.commitment-transactions</x:v>
       </x:c>
       <x:c r="B89" s="32" t="str">
-        <x:v>privacy.secret-right-to-cash</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="C89" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14166,21 +14515,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E89" s="32" t="str">
-        <x:v>Learners need the general idea that payment systems can exclude or block participants before the loss of private cash as a payment right becomes fully meaningful.</x:v>
+        <x:v>Per-commitment secrets are generated for each new commitment state, so learners need the commitment-transaction model before the secret-rotation mechanism makes sense.</x:v>
       </x:c>
       <x:c r="F89" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G89" s="32" t="str">
-        <x:v>Direct parent captures the exclusion-risk side of the argument without reopening broader compliance or surveillance wrappers.</x:v>
+        <x:v>Direct parent keeps the node on state evolution rather than on later punishment or watchtower behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="32" t="str">
-        <x:v>fundamentals.inflation</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="B90" s="32" t="str">
-        <x:v>economics.ideal-money</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="C90" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14189,21 +14538,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E90" s="32" t="str">
-        <x:v>The concept is about minimizing monetary distortion, so learners need to understand how inflation changes purchasing power and price signals first.</x:v>
+        <x:v>The to_local and to_remote scripts rely on per-state key derivation, revocation keys, and delayed-payment keys, so learners need the per-commitment secret machinery first.</x:v>
       </x:c>
       <x:c r="F90" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G90" s="32" t="str">
-        <x:v>Direct parent captures the measurement-distortion problem that ideal money is trying to avoid.</x:v>
+        <x:v>Direct parent keeps the node at the commitment-key layer instead of collapsing back into the broader commitment-transaction overview.</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>protocol.csv-bip112</x:v>
       </x:c>
       <x:c r="B91" s="32" t="str">
-        <x:v>protocol.bitcoin-uri-bip21</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="C91" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14212,21 +14561,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E91" s="32" t="str">
-        <x:v>The URI is a wrapper around a payment destination and amount, so learners need the underlying address and output model first.</x:v>
+        <x:v>The delayed to_local branch is defined by a CSV-enforced waiting period, so learners need the relative-timelock opcode before the script template makes sense.</x:v>
       </x:c>
       <x:c r="F91" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G91" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the standard request format rather than collapsing it into higher-level wallet UX systems.</x:v>
+        <x:v>Direct parent captures the script-mechanism side of the concept without dragging in broader force-close or HTLC timing behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="32" t="str">
-        <x:v>dev.bip32</x:v>
+        <x:v>protocol.difficulty-adjustment</x:v>
       </x:c>
       <x:c r="B92" s="32" t="str">
-        <x:v>dev.extended-keys</x:v>
+        <x:v>protocol.time-warp-attack</x:v>
       </x:c>
       <x:c r="C92" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14235,21 +14584,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E92" s="32" t="str">
-        <x:v>Extended keys are one specific export and branch-derivation surface inside the broader BIP32 HD tree model, so learners need the base tree-derivation mechanics first.</x:v>
+        <x:v>The attack only makes sense once learners understand how Bitcoin retargets mining difficulty over long block windows.</x:v>
       </x:c>
       <x:c r="F92" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G92" s="32" t="str">
-        <x:v>Direct parent keeps the node inside the HD derivation branch instead of treating xpub or xprv behavior as only a privacy or operational-wallet concept.</x:v>
+        <x:v>Direct parent keeps the exploit tied to the retarget mechanism instead of burying it under generic mining vocabulary.</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="32" t="str">
-        <x:v>dev.extended-keys</x:v>
+        <x:v>protocol.median-time-past</x:v>
       </x:c>
       <x:c r="B93" s="32" t="str">
-        <x:v>dev.hardened-keys</x:v>
+        <x:v>protocol.time-warp-attack</x:v>
       </x:c>
       <x:c r="C93" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14258,21 +14607,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E93" s="32" t="str">
-        <x:v>Hardened derivation is a constraint on what an extended public key can derive and on how extended private and public key boundaries behave, so learners need the base xpub/xprv model first.</x:v>
+        <x:v>Learners need the consensus timestamp constraints before they can reason about how miners manipulate time data and where the remaining attack surface lives.</x:v>
       </x:c>
       <x:c r="F93" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G93" s="32" t="str">
-        <x:v>Direct parent closes the previously missing branch-level bridge between BIP32 generally and hardened derivation specifically.</x:v>
+        <x:v>Direct parent captures the timestamp-boundary side of the exploit without overloading timelocks or block headers.</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>fundamentals.blind-signatures</x:v>
       </x:c>
       <x:c r="B94" s="32" t="str">
-        <x:v>protocol.escrow-and-arbitration</x:v>
+        <x:v>history.chaumian-ecash</x:v>
       </x:c>
       <x:c r="C94" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14281,21 +14630,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E94" s="32" t="str">
-        <x:v>The escrow flow depends on understanding how multiple signers can authorize one spend and why a 2-of-3 threshold changes trust assumptions between buyer, seller, and arbitrator.</x:v>
+        <x:v>Chaumian ecash is defined by using blind signatures to let a mint issue private bearer tokens without seeing the final token contents.</x:v>
       </x:c>
       <x:c r="F94" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G94" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the threshold-signing contract pattern instead of treating it as generic dispute-resolution theory.</x:v>
+        <x:v>Direct parent keeps the node tied to the specific cryptographic mechanism rather than treating it as generic digital-money history.</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="32" t="str">
-        <x:v>protocol.pay-to-script-hash</x:v>
+        <x:v>history.double-spend-problem</x:v>
       </x:c>
       <x:c r="B95" s="32" t="str">
-        <x:v>protocol.escrow-and-arbitration</x:v>
+        <x:v>history.chaumian-ecash</x:v>
       </x:c>
       <x:c r="C95" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14304,21 +14653,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E95" s="32" t="str">
-        <x:v>The contract uses a P2SH redeem script to hide the multisig spending conditions until spend time, so learners need the P2SH wrapper first.</x:v>
+        <x:v>Learners need the unsolved scarcity problem in digital cash before the trusted-mint tradeoff in Chaumian designs becomes meaningful.</x:v>
       </x:c>
       <x:c r="F95" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G95" s="32" t="str">
-        <x:v>Direct parent captures the on-chain contract packaging layer that makes the escrow pattern practical.</x:v>
+        <x:v>Direct parent frames why the system still needed a central operator even though it improved privacy.</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>economics.history-of-money</x:v>
       </x:c>
       <x:c r="B96" s="32" t="str">
-        <x:v>dev.wallet-import-format-wif</x:v>
+        <x:v>privacy.secret-right-to-cash</x:v>
       </x:c>
       <x:c r="C96" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14327,21 +14676,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E96" s="32" t="str">
-        <x:v>WIF is a serialization format for one private key, so learners need the underlying asymmetric-key concept before the network prefix, checksum, and compression flag details make sense.</x:v>
+        <x:v>The concept depends on understanding how money moved from bearer cash toward mediated account systems, so learners need the long-run monetary history first.</x:v>
       </x:c>
       <x:c r="F96" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G96" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored on key material itself instead of overfitting it to address formats or HD wallet hierarchies.</x:v>
+        <x:v>Direct parent keeps the node tied to the bearer-versus-intermediated payment shift rather than drifting into generic civil-liberties framing.</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>fundamentals.censorship-resistance</x:v>
       </x:c>
       <x:c r="B97" s="32" t="str">
-        <x:v>mining.pool-shares</x:v>
+        <x:v>privacy.secret-right-to-cash</x:v>
       </x:c>
       <x:c r="C97" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14350,21 +14699,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E97" s="32" t="str">
-        <x:v>Pool shares only make sense after learners understand why pooled mining exists and why miners need a lower-variance way to prove contributed work before an actual block is found.</x:v>
+        <x:v>Learners need the general idea that payment systems can exclude or block participants before the loss of private cash as a payment right becomes fully meaningful.</x:v>
       </x:c>
       <x:c r="F97" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G97" s="32" t="str">
-        <x:v>Direct parent keeps the node at the pooled-mining accounting layer without adding redundant proof-of-work or difficulty edges.</x:v>
+        <x:v>Direct parent captures the exclusion-risk side of the argument without reopening broader compliance or surveillance wrappers.</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>fundamentals.inflation</x:v>
       </x:c>
       <x:c r="B98" s="32" t="str">
-        <x:v>lightning.obscured-commitment-number</x:v>
+        <x:v>economics.ideal-money</x:v>
       </x:c>
       <x:c r="C98" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14373,21 +14722,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E98" s="32" t="str">
-        <x:v>The obscured commitment number is part of the same commitment-state machinery as the per-state secret chain, so learners need that state-derivation context before the field-level encoding scheme makes sense.</x:v>
+        <x:v>The concept is about minimizing monetary distortion, so learners need to understand how inflation changes purchasing power and price signals first.</x:v>
       </x:c>
       <x:c r="F98" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G98" s="32" t="str">
-        <x:v>Direct parent keeps the node in the narrow commitment-state branch instead of pulling in broader closure or HTLC behavior.</x:v>
+        <x:v>Direct parent captures the measurement-distortion problem that ideal money is trying to avoid.</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="32" t="str">
-        <x:v>lightning.htlc</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B99" s="32" t="str">
-        <x:v>lightning.htlc-output-scripts</x:v>
+        <x:v>protocol.bitcoin-uri-bip21</x:v>
       </x:c>
       <x:c r="C99" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14396,21 +14745,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E99" s="32" t="str">
-        <x:v>Learners need the base HTLC idea before the offered and received witness-script branches, timeout paths, and preimage-claim paths become meaningful.</x:v>
+        <x:v>The URI is a wrapper around a payment destination and amount, so learners need the underlying address and output model first.</x:v>
       </x:c>
       <x:c r="F99" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G99" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the payment-contract primitive instead of treating it as generic script trivia.</x:v>
+        <x:v>Direct parent keeps the node tied to the standard request format rather than collapsing it into higher-level wallet UX systems.</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>dev.bip32</x:v>
       </x:c>
       <x:c r="B100" s="32" t="str">
-        <x:v>lightning.htlc-output-scripts</x:v>
+        <x:v>dev.extended-keys</x:v>
       </x:c>
       <x:c r="C100" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14419,21 +14768,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E100" s="32" t="str">
-        <x:v>HTLC output scripts are additional commitment-transaction outputs layered on top of the same to_local and to_remote commitment-script structure, so learners need that earlier script layer first.</x:v>
+        <x:v>Extended keys are one specific export and branch-derivation surface inside the broader BIP32 HD tree model, so learners need the base tree-derivation mechanics first.</x:v>
       </x:c>
       <x:c r="F100" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G100" s="32" t="str">
-        <x:v>Direct parent places the node at the next script layer above commitment outputs without dragging in later close-handling or watchtower flows.</x:v>
+        <x:v>Direct parent keeps the node inside the HD derivation branch instead of treating xpub or xprv behavior as only a privacy or operational-wallet concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="32" t="str">
-        <x:v>protocol.coinbase-transaction</x:v>
+        <x:v>dev.extended-keys</x:v>
       </x:c>
       <x:c r="B101" s="32" t="str">
-        <x:v>protocol.duplicate-transaction-bug</x:v>
+        <x:v>dev.hardened-keys</x:v>
       </x:c>
       <x:c r="C101" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14442,21 +14791,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E101" s="32" t="str">
-        <x:v>The bug is historically tied to duplicated coinbase transactions, so learners need the special structure and validation role of coinbase transactions before the replay vector makes sense.</x:v>
+        <x:v>Hardened derivation is a constraint on what an extended public key can derive and on how extended private and public key boundaries behave, so learners need the base xpub/xprv model first.</x:v>
       </x:c>
       <x:c r="F101" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G101" s="32" t="str">
-        <x:v>Direct parent keeps the bug tied to the early-coinbase uniqueness failure instead of burying it under general mining history.</x:v>
+        <x:v>Direct parent closes the previously missing branch-level bridge between BIP32 generally and hardened derivation specifically.</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="32" t="str">
-        <x:v>protocol.utxo-model</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B102" s="32" t="str">
-        <x:v>protocol.duplicate-transaction-bug</x:v>
+        <x:v>protocol.escrow-and-arbitration</x:v>
       </x:c>
       <x:c r="C102" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14465,21 +14814,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E102" s="32" t="str">
-        <x:v>Learners need the txid-plus-output-index reference model to understand why identical transaction ids could confuse later spends and overwrite assumptions in the UTXO set.</x:v>
+        <x:v>The escrow flow depends on understanding how multiple signers can authorize one spend and why a 2-of-3 threshold changes trust assumptions between buyer, seller, and arbitrator.</x:v>
       </x:c>
       <x:c r="F102" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G102" s="32" t="str">
-        <x:v>Direct parent captures the reference-model side of the bug without conflating it with double-spend history or malleability.</x:v>
+        <x:v>Direct parent keeps the node tied to the threshold-signing contract pattern instead of treating it as generic dispute-resolution theory.</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="32" t="str">
-        <x:v>protocol.block-structure</x:v>
+        <x:v>protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="B103" s="32" t="str">
-        <x:v>protocol.64-byte-transaction-bug</x:v>
+        <x:v>protocol.escrow-and-arbitration</x:v>
       </x:c>
       <x:c r="C103" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14488,21 +14837,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E103" s="32" t="str">
-        <x:v>The bug only makes sense once learners understand how transaction hashes sit inside the block merkle tree and why internal-node preimages matter for block commitments.</x:v>
+        <x:v>The contract uses a P2SH redeem script to hide the multisig spending conditions until spend time, so learners need the P2SH wrapper first.</x:v>
       </x:c>
       <x:c r="F103" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G103" s="32" t="str">
-        <x:v>One direct parent keeps the node at the block-commitment layer instead of reopening broader hashing or SPV overview branches.</x:v>
+        <x:v>Direct parent captures the on-chain contract packaging layer that makes the escrow pattern practical.</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="32" t="str">
-        <x:v>fundamentals.digital-signatures</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B104" s="32" t="str">
-        <x:v>fundamentals.lamport-signatures</x:v>
+        <x:v>dev.wallet-import-format-wif</x:v>
       </x:c>
       <x:c r="C104" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14511,21 +14860,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E104" s="32" t="str">
-        <x:v>Learners need the general signing-and-verification mental model before the one-time Lamport construction and its tradeoffs become meaningful.</x:v>
+        <x:v>WIF is a serialization format for one private key, so learners need the underlying asymmetric-key concept before the network prefix, checksum, and compression flag details make sense.</x:v>
       </x:c>
       <x:c r="F104" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G104" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to signature semantics instead of treating it as only a post-quantum curiosity.</x:v>
+        <x:v>Direct parent keeps the node anchored on key material itself instead of overfitting it to address formats or HD wallet hierarchies.</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B105" s="32" t="str">
-        <x:v>fundamentals.lamport-signatures</x:v>
+        <x:v>mining.pool-shares</x:v>
       </x:c>
       <x:c r="C105" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14534,21 +14883,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E105" s="32" t="str">
-        <x:v>Lamport signatures replace elliptic-curve arithmetic with one-way hash preimages and comparisons, so learners need the hash primitive first.</x:v>
+        <x:v>Pool shares only make sense after learners understand why pooled mining exists and why miners need a lower-variance way to prove contributed work before an actual block is found.</x:v>
       </x:c>
       <x:c r="F105" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G105" s="32" t="str">
-        <x:v>Direct parent captures the actual cryptographic mechanism rather than forcing learners through unrelated elliptic-curve details.</x:v>
+        <x:v>Direct parent keeps the node at the pooled-mining accounting layer without adding redundant proof-of-work or difficulty edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="32" t="str">
-        <x:v>custody.backups-recovery</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="B106" s="32" t="str">
-        <x:v>custody.shamirs-secret-sharing</x:v>
+        <x:v>lightning.obscured-commitment-number</x:v>
       </x:c>
       <x:c r="C106" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14557,21 +14906,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E106" s="32" t="str">
-        <x:v>In Bitcoin practice the scheme is used as one backup-and-recovery method, so learners need the broader custody problem before the threshold-share design choice becomes meaningful.</x:v>
+        <x:v>The obscured commitment number is part of the same commitment-state machinery as the per-state secret chain, so learners need that state-derivation context before the field-level encoding scheme makes sense.</x:v>
       </x:c>
       <x:c r="F106" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G106" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored in practical custody use instead of drifting into a purely abstract cryptography topic.</x:v>
+        <x:v>Direct parent keeps the node in the narrow commitment-state branch instead of pulling in broader closure or HTLC behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="32" t="str">
-        <x:v>protocol.segregated-witness</x:v>
+        <x:v>lightning.htlc</x:v>
       </x:c>
       <x:c r="B107" s="32" t="str">
-        <x:v>protocol.witness-structure</x:v>
+        <x:v>lightning.htlc-output-scripts</x:v>
       </x:c>
       <x:c r="C107" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14580,21 +14929,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E107" s="32" t="str">
-        <x:v>The transaction witness layout only makes sense after the learner understands that SegWit separates witness data from the legacy transaction serialization.</x:v>
+        <x:v>Learners need the base HTLC idea before the offered and received witness-script branches, timeout paths, and preimage-claim paths become meaningful.</x:v>
       </x:c>
       <x:c r="F107" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G107" s="32" t="str">
-        <x:v>Direct edge keeps the node at the transaction-format layer; TXID/WTXID and witness-commitment consequences remain downstream concepts.</x:v>
+        <x:v>Direct parent keeps the node tied to the payment-contract primitive instead of treating it as generic script trivia.</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="32" t="str">
-        <x:v>protocol.block-structure</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="B108" s="32" t="str">
-        <x:v>protocol.partial-merkle-proofs</x:v>
+        <x:v>lightning.htlc-output-scripts</x:v>
       </x:c>
       <x:c r="C108" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14603,21 +14952,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E108" s="32" t="str">
-        <x:v>Partial Merkle proofs reconstruct a transaction's inclusion path against the Merkle root carried by a block, so learners need block composition and root placement first.</x:v>
+        <x:v>HTLC output scripts are additional commitment-transaction outputs layered on top of the same to_local and to_remote commitment-script structure, so learners need that earlier script layer first.</x:v>
       </x:c>
       <x:c r="F108" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G108" s="32" t="str">
-        <x:v>The block-structure parent already inherits fundamentals.merkle-trees, avoiding a redundant direct edge.</x:v>
+        <x:v>Direct parent places the node at the next script layer above commitment outputs without dragging in later close-handling or watchtower flows.</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="32" t="str">
-        <x:v>dev.bips-process</x:v>
+        <x:v>protocol.coinbase-transaction</x:v>
       </x:c>
       <x:c r="B109" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>protocol.duplicate-transaction-bug</x:v>
       </x:c>
       <x:c r="C109" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14626,21 +14975,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E109" s="32" t="str">
-        <x:v>Review culture is applied throughout the proposal and implementation lifecycle, so learners need to understand the process in which Bitcoin changes are proposed and evaluated.</x:v>
+        <x:v>The bug is historically tied to duplicated coinbase transactions, so learners need the special structure and validation role of coinbase transactions before the replay vector makes sense.</x:v>
       </x:c>
       <x:c r="F109" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G109" s="32" t="str">
-        <x:v>Direct edge supplies the development-lifecycle context without adding downstream release or deployment details.</x:v>
+        <x:v>Direct parent keeps the bug tied to the early-coinbase uniqueness failure instead of burying it under general mining history.</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="32" t="str">
-        <x:v>security.adversarial-thinking</x:v>
+        <x:v>protocol.utxo-model</x:v>
       </x:c>
       <x:c r="B110" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>protocol.duplicate-transaction-bug</x:v>
       </x:c>
       <x:c r="C110" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14649,21 +14998,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E110" s="32" t="str">
-        <x:v>Independent review in Bitcoin is deliberately adversarial: reviewers look for correctness failures, attack paths, and compatibility hazards before changes are merged.</x:v>
+        <x:v>Learners need the txid-plus-output-index reference model to understand why identical transaction ids could confuse later spends and overwrite assumptions in the UTXO set.</x:v>
       </x:c>
       <x:c r="F110" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G110" s="32" t="str">
-        <x:v>Direct edge keeps review distinct from responsible disclosure and reproducible-build verification, which are specialized downstream safeguards.</x:v>
+        <x:v>Direct parent captures the reference-model side of the bug without conflating it with double-spend history or malleability.</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="32" t="str">
-        <x:v>lightning.gossip-protocol</x:v>
+        <x:v>protocol.block-structure</x:v>
       </x:c>
       <x:c r="B111" s="32" t="str">
-        <x:v>lightning.feature-flags</x:v>
+        <x:v>protocol.64-byte-transaction-bug</x:v>
       </x:c>
       <x:c r="C111" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14672,21 +15021,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E111" s="32" t="str">
-        <x:v>Feature negotiation is used to advertise and interpret capabilities across Lightning peers and network announcements, so learners need the surrounding gossip and announcement context first.</x:v>
+        <x:v>The bug only makes sense once learners understand how transaction hashes sit inside the block merkle tree and why internal-node preimages matter for block commitments.</x:v>
       </x:c>
       <x:c r="F111" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G111" s="32" t="str">
-        <x:v>Direct edge keeps the feature-bit mechanism distinct from the lower-level message transport and downstream routing protocols.</x:v>
+        <x:v>One direct parent keeps the node at the block-commitment layer instead of reopening broader hashing or SPV overview branches.</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="32" t="str">
-        <x:v>lightning.feature-flags</x:v>
+        <x:v>fundamentals.digital-signatures</x:v>
       </x:c>
       <x:c r="B112" s="32" t="str">
-        <x:v>lightning.onion-messages</x:v>
+        <x:v>fundamentals.lamport-signatures</x:v>
       </x:c>
       <x:c r="C112" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14695,21 +15044,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E112" s="32" t="str">
-        <x:v>Peers use a negotiated feature bit to advertise whether they can send and forward onion messages, so learners need the capability-negotiation model first.</x:v>
+        <x:v>Learners need the general signing-and-verification mental model before the one-time Lamport construction and its tradeoffs become meaningful.</x:v>
       </x:c>
       <x:c r="F112" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G112" s="32" t="str">
-        <x:v>Direct edge keeps the feature gate separate from the message forwarding mechanism.</x:v>
+        <x:v>Direct parent keeps the node tied to signature semantics instead of treating it as only a post-quantum curiosity.</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="32" t="str">
-        <x:v>lightning.route-blinding</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B113" s="32" t="str">
-        <x:v>lightning.onion-messages</x:v>
+        <x:v>fundamentals.lamport-signatures</x:v>
       </x:c>
       <x:c r="C113" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14718,21 +15067,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E113" s="32" t="str">
-        <x:v>Onion messages use blinded paths to forward channel-independent payloads without exposing the final destination topology, so the route-blinding model must come first.</x:v>
+        <x:v>Lamport signatures replace elliptic-curve arithmetic with one-way hash preimages and comparisons, so learners need the hash primitive first.</x:v>
       </x:c>
       <x:c r="F113" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G113" s="32" t="str">
-        <x:v>Payment onion routing and BOLT12 offers remain related sibling or downstream concepts rather than direct prerequisites.</x:v>
+        <x:v>Direct parent captures the actual cryptographic mechanism rather than forcing learners through unrelated elliptic-curve details.</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>custody.backups-recovery</x:v>
       </x:c>
       <x:c r="B114" s="32" t="str">
-        <x:v>lightning.encrypted-authenticated-transport</x:v>
+        <x:v>custody.shamirs-secret-sharing</x:v>
       </x:c>
       <x:c r="C114" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14741,21 +15090,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E114" s="32" t="str">
-        <x:v>The Noise_XK handshake authenticates long-term Lightning node identities with public/private key material, so learners need that identity model first.</x:v>
+        <x:v>In Bitcoin practice the scheme is used as one backup-and-recovery method, so learners need the broader custody problem before the threshold-share design choice becomes meaningful.</x:v>
       </x:c>
       <x:c r="F114" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G114" s="32" t="str">
-        <x:v>Direct edge keeps identity foundations separate from the session-key derivation mechanism.</x:v>
+        <x:v>Direct parent keeps the node anchored in practical custody use instead of drifting into a purely abstract cryptography topic.</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="32" t="str">
-        <x:v>fundamentals.diffie-hellman-key-exchange</x:v>
+        <x:v>protocol.segregated-witness</x:v>
       </x:c>
       <x:c r="B115" s="32" t="str">
-        <x:v>lightning.encrypted-authenticated-transport</x:v>
+        <x:v>protocol.witness-structure</x:v>
       </x:c>
       <x:c r="C115" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14764,21 +15113,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E115" s="32" t="str">
-        <x:v>BOLT 08 uses elliptic-curve Diffie-Hellman operations to derive shared session secrets, so the key-exchange primitive must be understood first.</x:v>
+        <x:v>The transaction witness layout only makes sense after the learner understands that SegWit separates witness data from the legacy transaction serialization.</x:v>
       </x:c>
       <x:c r="F115" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G115" s="32" t="str">
-        <x:v>Bitcoin P2P v2 transport remains a related sibling rather than a direct prerequisite because it is a different protocol context.</x:v>
+        <x:v>Direct edge keeps the node at the transaction-format layer; TXID/WTXID and witness-commitment consequences remain downstream concepts.</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>protocol.block-structure</x:v>
       </x:c>
       <x:c r="B116" s="32" t="str">
-        <x:v>protocol.strict-der-signatures</x:v>
+        <x:v>protocol.partial-merkle-proofs</x:v>
       </x:c>
       <x:c r="C116" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14787,21 +15136,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E116" s="32" t="str">
-        <x:v>Strict DER enforcement occurs while Script validates an ECDSA signature, so learners need the spending-condition and interpreter context first.</x:v>
+        <x:v>Partial Merkle proofs reconstruct a transaction's inclusion path against the Merkle root carried by a block, so learners need block composition and root placement first.</x:v>
       </x:c>
       <x:c r="F116" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G116" s="32" t="str">
-        <x:v>Direct edge keeps the rule at the script-validation layer rather than treating BIP 66 as a broad historical upgrade topic.</x:v>
+        <x:v>The block-structure parent already inherits fundamentals.merkle-trees, avoiding a redundant direct edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>dev.bips-process</x:v>
       </x:c>
       <x:c r="B117" s="32" t="str">
-        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="C117" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14810,21 +15159,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E117" s="32" t="str">
-        <x:v>The node builds on the wallet-level threshold signer policy before specifying a deterministic ordering convention for the signer keys.</x:v>
+        <x:v>Review culture is applied throughout the proposal and implementation lifecycle, so learners need to understand the process in which Bitcoin changes are proposed and evaluated.</x:v>
       </x:c>
       <x:c r="F117" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G117" s="32" t="str">
-        <x:v>Direct edge preserves the distinction between multisig policy and the BIP 67 interoperability rule.</x:v>
+        <x:v>Direct edge supplies the development-lifecycle context without adding downstream release or deployment details.</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="32" t="str">
-        <x:v>protocol.pay-to-script-hash</x:v>
+        <x:v>security.adversarial-thinking</x:v>
       </x:c>
       <x:c r="B118" s="32" t="str">
-        <x:v>custody.deterministic-multisig-key-sorting</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="C118" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14833,21 +15182,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E118" s="32" t="str">
-        <x:v>BIP 67 is commonly applied when constructing the redeem script whose hash is committed by P2SH, so the script-hash wrapper provides the output context.</x:v>
+        <x:v>Independent review in Bitcoin is deliberately adversarial: reviewers look for correctness failures, attack paths, and compatibility hazards before changes are merged.</x:v>
       </x:c>
       <x:c r="F118" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G118" s="32" t="str">
-        <x:v>The shared protocol.script ancestor remains inherited rather than a redundant direct edge.</x:v>
+        <x:v>Direct edge keeps review distinct from responsible disclosure and reproducible-build verification, which are specialized downstream safeguards.</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="32" t="str">
-        <x:v>ops.mempool-policy</x:v>
+        <x:v>lightning.gossip-protocol</x:v>
       </x:c>
       <x:c r="B119" s="32" t="str">
-        <x:v>ops.mempool-purging</x:v>
+        <x:v>lightning.feature-flags</x:v>
       </x:c>
       <x:c r="C119" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14856,21 +15205,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E119" s="32" t="str">
-        <x:v>Rolling minimum fee escalation and transaction eviction are local consequences of the node's mempool relay policy, so learners need that policy boundary first.</x:v>
+        <x:v>Feature negotiation is used to advertise and interpret capabilities across Lightning peers and network announcements, so learners need the surrounding gossip and announcement context first.</x:v>
       </x:c>
       <x:c r="F119" s="32" t="str">
-        <x:v>source.mempool-space-docs</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G119" s="32" t="str">
-        <x:v>The generic mempool, fee-market, and consensus-policy branches remain inherited or adjacent rather than direct prerequisites.</x:v>
+        <x:v>Direct edge keeps the feature-bit mechanism distinct from the lower-level message transport and downstream routing protocols.</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>lightning.feature-flags</x:v>
       </x:c>
       <x:c r="B120" s="32" t="str">
-        <x:v>protocol.generic-signed-messages</x:v>
+        <x:v>lightning.onion-messages</x:v>
       </x:c>
       <x:c r="C120" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14879,21 +15228,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E120" s="32" t="str">
-        <x:v>BIP 322 proves message authorization by constructing virtual transactions that satisfy a Bitcoin output script, so learners need the Script spending-condition model first.</x:v>
+        <x:v>Peers use a negotiated feature bit to advertise whether they can send and forward onion messages, so learners need the capability-negotiation model first.</x:v>
       </x:c>
       <x:c r="F120" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G120" s="32" t="str">
-        <x:v>The digital-signature path is inherited through Script; PSBT, Schnorr, and Taproot remain related variants rather than redundant direct edges.</x:v>
+        <x:v>Direct edge keeps the feature gate separate from the message forwarding mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="32" t="str">
-        <x:v>dev.bitcoin-core-rpc</x:v>
+        <x:v>lightning.route-blinding</x:v>
       </x:c>
       <x:c r="B121" s="32" t="str">
-        <x:v>security.bitcoin-core-rpc-access</x:v>
+        <x:v>lightning.onion-messages</x:v>
       </x:c>
       <x:c r="C121" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14902,21 +15251,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E121" s="32" t="str">
-        <x:v>RPC access security is the control boundary around Bitcoin Core's programmatic interface, so learners need to understand the interface and its authority before securing exposure to it.</x:v>
+        <x:v>Onion messages use blinded paths to forward channel-independent payloads without exposing the final destination topology, so the route-blinding model must come first.</x:v>
       </x:c>
       <x:c r="F121" s="32" t="str">
-        <x:v>source.bitcoin-core-operator-docs</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G121" s="32" t="str">
-        <x:v>Full-node operation is inherited through dev.bitcoin-core-rpc; wallet RPC and transaction-preflight nodes remain downstream use cases rather than direct parents.</x:v>
+        <x:v>Payment onion routing and BOLT12 offers remain related sibling or downstream concepts rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="32" t="str">
-        <x:v>dev.testmempoolaccept-rpc</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B122" s="32" t="str">
-        <x:v>dev.submitpackage-rpc</x:v>
+        <x:v>lightning.encrypted-authenticated-transport</x:v>
       </x:c>
       <x:c r="C122" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14925,21 +15274,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E122" s="32" t="str">
-        <x:v>submitpackage is the admission counterpart to the existing testmempoolaccept preflight workflow, so learners need to understand local package checks before attempting submission and interpreting package results.</x:v>
+        <x:v>The Noise_XK handshake authenticates long-term Lightning node identities with public/private key material, so learners need that identity model first.</x:v>
       </x:c>
       <x:c r="F122" s="32" t="str">
-        <x:v>source.bitcoin-core-package-policy</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G122" s="32" t="str">
-        <x:v>Package relay and cluster mempool remain neighboring concepts rather than direct prerequisites because this node focuses on one local RPC operation.</x:v>
+        <x:v>Direct edge keeps identity foundations separate from the session-key derivation mechanism.</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="32" t="str">
-        <x:v>protocol.rbf</x:v>
+        <x:v>fundamentals.diffie-hellman-key-exchange</x:v>
       </x:c>
       <x:c r="B123" s="32" t="str">
-        <x:v>protocol.package-rbf</x:v>
+        <x:v>lightning.encrypted-authenticated-transport</x:v>
       </x:c>
       <x:c r="C123" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14948,21 +15297,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E123" s="32" t="str">
-        <x:v>Package RBF extends the ordinary replacement-policy model with package-level fee and cluster conditions, so learners need base RBF semantics first.</x:v>
+        <x:v>BOLT 08 uses elliptic-curve Diffie-Hellman operations to derive shared session secrets, so the key-exchange primitive must be understood first.</x:v>
       </x:c>
       <x:c r="F123" s="32" t="str">
-        <x:v>source.bitcoin-core-package-policy</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G123" s="32" t="str">
-        <x:v>Package relay, cluster mempool, submitpackage, and pinning remain adjacent concepts rather than redundant direct edges.</x:v>
+        <x:v>Bitcoin P2P v2 transport remains a related sibling rather than a direct prerequisite because it is a different protocol context.</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="32" t="str">
-        <x:v>protocol.cluster-mempool</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B124" s="32" t="str">
-        <x:v>ops.mempool-cluster-limits</x:v>
+        <x:v>protocol.strict-der-signatures</x:v>
       </x:c>
       <x:c r="C124" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14971,21 +15320,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E124" s="32" t="str">
-        <x:v>Cluster limits bound connected transaction sets, so learners need the cluster-mempool model before understanding why count and aggregate virtual-size limits replace legacy ancestor/descendant limits.</x:v>
+        <x:v>Strict DER enforcement occurs while Script validates an ECDSA signature, so learners need the spending-condition and interpreter context first.</x:v>
       </x:c>
       <x:c r="F124" s="32" t="str">
-        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G124" s="32" t="str">
-        <x:v>Package relay, Package RBF, CPFP, and version 3 relay remain affected workflows or neighboring policy mechanisms rather than direct prerequisites.</x:v>
+        <x:v>Direct edge keeps the rule at the script-validation layer rather than treating BIP 66 as a broad historical upgrade topic.</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="32" t="str">
-        <x:v>ops.dns-seeds</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B125" s="32" t="str">
-        <x:v>lightning.dns-seeds</x:v>
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
       </x:c>
       <x:c r="C125" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14994,21 +15343,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E125" s="32" t="str">
-        <x:v>Lightning DNS seeds specialize the general DNS bootstrap pattern with Lightning-specific query filters and known-peer lookup, so learners need the base DNS-seed model first.</x:v>
+        <x:v>The node builds on the wallet-level threshold signer policy before specifying a deterministic ordering convention for the signer keys.</x:v>
       </x:c>
       <x:c r="F125" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G125" s="32" t="str">
-        <x:v>Peer discovery is inherited through ops.dns-seeds; generic Bitcoin P2P bootstrapping remains a parent concept rather than a duplicated edge.</x:v>
+        <x:v>Direct edge preserves the distinction between multisig policy and the BIP 67 interoperability rule.</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="32" t="str">
-        <x:v>lightning.gossip-protocol</x:v>
+        <x:v>protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="B126" s="32" t="str">
-        <x:v>lightning.dns-seeds</x:v>
+        <x:v>custody.deterministic-multisig-key-sorting</x:v>
       </x:c>
       <x:c r="C126" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15017,21 +15366,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E126" s="32" t="str">
-        <x:v>BOLT 10 locates Lightning peers and filters results by Lightning address information, so learners need Lightning's node-discovery and gossip context before understanding the assisted-location mechanism.</x:v>
+        <x:v>BIP 67 is commonly applied when constructing the redeem script whose hash is committed by P2SH, so the script-hash wrapper provides the output context.</x:v>
       </x:c>
       <x:c r="F126" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G126" s="32" t="str">
-        <x:v>Lightning routing and generic P2P messages are inherited through gossip rather than added as transitive prerequisites.</x:v>
+        <x:v>The shared protocol.script ancestor remains inherited rather than a redundant direct edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="32" t="str">
-        <x:v>lightning.payment-channels</x:v>
+        <x:v>ops.mempool-policy</x:v>
       </x:c>
       <x:c r="B127" s="32" t="str">
-        <x:v>lightning.short-channel-id</x:v>
+        <x:v>ops.mempool-purging</x:v>
       </x:c>
       <x:c r="C127" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15040,21 +15389,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E127" s="32" t="str">
-        <x:v>The identifier names a Lightning channel's on-chain funding output, so learners need the channel and funding relationship first.</x:v>
+        <x:v>Rolling minimum fee escalation and transaction eviction are local consequences of the node's mempool relay policy, so learners need that policy boundary first.</x:v>
       </x:c>
       <x:c r="F127" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.mempool-space-docs</x:v>
       </x:c>
       <x:c r="G127" s="32" t="str">
-        <x:v>Direct channel context; the gossip protocol is a downstream consumer rather than a prerequisite.</x:v>
+        <x:v>The generic mempool, fee-market, and consensus-policy branches remain inherited or adjacent rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="32" t="str">
-        <x:v>protocol.block-height</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B128" s="32" t="str">
-        <x:v>lightning.short-channel-id</x:v>
+        <x:v>protocol.generic-signed-messages</x:v>
       </x:c>
       <x:c r="C128" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15063,21 +15412,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E128" s="32" t="str">
-        <x:v>Short Channel IDs encode block height as their first component, so learners need the block-height concept before decoding the identifier.</x:v>
+        <x:v>BIP 322 proves message authorization by constructing virtual transactions that satisfy a Bitcoin output script, so learners need the Script spending-condition model first.</x:v>
       </x:c>
       <x:c r="F128" s="32" t="str">
-        <x:v>source.lightning-bolts</x:v>
+        <x:v>source.bitcoin-bips</x:v>
       </x:c>
       <x:c r="G128" s="32" t="str">
-        <x:v>The transaction-index and output-index components remain part of the identifier's own outcome rather than extra transitive edges.</x:v>
+        <x:v>The digital-signature path is inherited through Script; PSBT, Schnorr, and Taproot remain related variants rather than redundant direct edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="32" t="str">
-        <x:v>protocol.nodes-vs-miners</x:v>
+        <x:v>dev.bitcoin-core-rpc</x:v>
       </x:c>
       <x:c r="B129" s="32" t="str">
-        <x:v>mining.miner-decentralization</x:v>
+        <x:v>security.bitcoin-core-rpc-access</x:v>
       </x:c>
       <x:c r="C129" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15086,21 +15435,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E129" s="32" t="str">
-        <x:v>Miner decentralization only makes sense once learners distinguish miners' transaction-ordering role from full nodes' independent enforcement of consensus validity.</x:v>
+        <x:v>RPC access security is the control boundary around Bitcoin Core's programmatic interface, so learners need to understand the interface and its authority before securing exposure to it.</x:v>
       </x:c>
       <x:c r="F129" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-core-operator-docs</x:v>
       </x:c>
       <x:c r="G129" s="32" t="str">
-        <x:v>The edge keeps censorship power separate from authority to change consensus rules.</x:v>
+        <x:v>Full-node operation is inherited through dev.bitcoin-core-rpc; wallet RPC and transaction-preflight nodes remain downstream use cases rather than direct parents.</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>dev.testmempoolaccept-rpc</x:v>
       </x:c>
       <x:c r="B130" s="32" t="str">
-        <x:v>mining.miner-decentralization</x:v>
+        <x:v>dev.submitpackage-rpc</x:v>
       </x:c>
       <x:c r="C130" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15109,21 +15458,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E130" s="32" t="str">
-        <x:v>Pool and solo mining explain the participant and coordination structure whose concentration or dispersion determines practical control over transaction ordering.</x:v>
+        <x:v>submitpackage is the admission counterpart to the existing testmempoolaccept preflight workflow, so learners need to understand local package checks before attempting submission and interpreting package results.</x:v>
       </x:c>
       <x:c r="F130" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-core-package-policy</x:v>
       </x:c>
       <x:c r="G130" s="32" t="str">
-        <x:v>Stratum V2 remains optional implementation context, not a direct prerequisite.</x:v>
+        <x:v>Package relay and cluster mempool remain neighboring concepts rather than direct prerequisites because this node focuses on one local RPC operation.</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>protocol.rbf</x:v>
       </x:c>
       <x:c r="B131" s="32" t="str">
-        <x:v>dev.selection-cryptography</x:v>
+        <x:v>protocol.package-rbf</x:v>
       </x:c>
       <x:c r="C131" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15132,21 +15481,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E131" s="32" t="str">
-        <x:v>Selection cryptography evaluates cryptographic tools and dependencies through evidence, testing, authorship, and review quality, so learners need the broader Bitcoin review discipline first.</x:v>
+        <x:v>Package RBF extends the ordinary replacement-policy model with package-level fee and cluster conditions, so learners need base RBF semantics first.</x:v>
       </x:c>
       <x:c r="F131" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-core-package-policy</x:v>
       </x:c>
       <x:c r="G131" s="32" t="str">
-        <x:v>Adversarial thinking is inherited through dev.review-culture; reproducible builds are a downstream verification practice rather than a prerequisite.</x:v>
+        <x:v>Package relay, cluster mempool, submitpackage, and pinning remain adjacent concepts rather than redundant direct edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="32" t="str">
-        <x:v>mining.pool-shares</x:v>
+        <x:v>protocol.cluster-mempool</x:v>
       </x:c>
       <x:c r="B132" s="32" t="str">
-        <x:v>mining.block-withholding</x:v>
+        <x:v>ops.mempool-cluster-limits</x:v>
       </x:c>
       <x:c r="C132" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15155,21 +15504,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E132" s="32" t="str">
-        <x:v>Block withholding exploits the difference between a pool-paid share and a share that also meets the network target, so learners must understand share accounting before the attack model makes sense.</x:v>
+        <x:v>Cluster limits bound connected transaction sets, so learners need the cluster-mempool model before understanding why count and aggregate virtual-size limits replace legacy ancestor/descendant limits.</x:v>
       </x:c>
       <x:c r="F132" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-core-cluster-mempool-rpc</x:v>
       </x:c>
       <x:c r="G132" s="32" t="str">
-        <x:v>Pool-versus-solo and mining economics are inherited through mining.pool-shares; do not add a redundant majority-attack edge.</x:v>
+        <x:v>Package relay, Package RBF, CPFP, and version 3 relay remain affected workflows or neighboring policy mechanisms rather than direct prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>ops.dns-seeds</x:v>
       </x:c>
       <x:c r="B133" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>lightning.dns-seeds</x:v>
       </x:c>
       <x:c r="C133" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15178,21 +15527,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E133" s="32" t="str">
-        <x:v>P2C tweaks a public key to commit to contract data, so learners need the public/private key model.</x:v>
+        <x:v>Lightning DNS seeds specialize the general DNS bootstrap pattern with Lightning-specific query filters and known-peer lookup, so learners need the base DNS-seed model first.</x:v>
       </x:c>
       <x:c r="F133" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G133" s="32" t="str">
-        <x:v>Taproot is adjacent, not a direct requirement.</x:v>
+        <x:v>Peer discovery is inherited through ops.dns-seeds; generic Bitcoin P2P bootstrapping remains a parent concept rather than a duplicated edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>lightning.gossip-protocol</x:v>
       </x:c>
       <x:c r="B134" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>lightning.dns-seeds</x:v>
       </x:c>
       <x:c r="C134" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15201,21 +15550,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E134" s="32" t="str">
-        <x:v>P2C derives a commitment tweak from contract data using a hash, so learners need hash commitments first.</x:v>
+        <x:v>BOLT 10 locates Lightning peers and filters results by Lightning address information, so learners need Lightning's node-discovery and gossip context before understanding the assisted-location mechanism.</x:v>
       </x:c>
       <x:c r="F134" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G134" s="32" t="str">
-        <x:v>The hash is part of the construction rather than generic background.</x:v>
+        <x:v>Lightning routing and generic P2P messages are inherited through gossip rather than added as transitive prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="32" t="str">
-        <x:v>protocol.utxo-model</x:v>
+        <x:v>lightning.payment-channels</x:v>
       </x:c>
       <x:c r="B135" s="32" t="str">
-        <x:v>extension.single-use-seals</x:v>
+        <x:v>lightning.short-channel-id</x:v>
       </x:c>
       <x:c r="C135" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15224,21 +15573,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E135" s="32" t="str">
-        <x:v>Single-use seals rely on a UTXO's one-time spend property.</x:v>
+        <x:v>The identifier names a Lightning channel's on-chain funding output, so learners need the channel and funding relationship first.</x:v>
       </x:c>
       <x:c r="F135" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G135" s="32" t="str">
-        <x:v>This explicit bridge prevents hiding the seal invariant inside generic UTXO semantics.</x:v>
+        <x:v>Direct channel context; the gossip protocol is a downstream consumer rather than a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="32" t="str">
-        <x:v>extension.single-use-seals</x:v>
+        <x:v>protocol.block-height</x:v>
       </x:c>
       <x:c r="B136" s="32" t="str">
-        <x:v>extension.client-side-validation</x:v>
+        <x:v>lightning.short-channel-id</x:v>
       </x:c>
       <x:c r="C136" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15247,21 +15596,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E136" s="32" t="str">
-        <x:v>Client-side validation relies on seals to prevent an offchain transition from being valid twice.</x:v>
+        <x:v>Short Channel IDs encode block height as their first component, so learners need the block-height concept before decoding the identifier.</x:v>
       </x:c>
       <x:c r="F136" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.lightning-bolts</x:v>
       </x:c>
       <x:c r="G136" s="32" t="str">
-        <x:v>The UTXO parent is inherited through the seal and is intentionally not duplicated.</x:v>
+        <x:v>The transaction-index and output-index components remain part of the identifier's own outcome rather than extra transitive edges.</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="32" t="str">
-        <x:v>protocol.pay-to-contract</x:v>
+        <x:v>protocol.nodes-vs-miners</x:v>
       </x:c>
       <x:c r="B137" s="32" t="str">
-        <x:v>extension.client-side-validation</x:v>
+        <x:v>mining.miner-decentralization</x:v>
       </x:c>
       <x:c r="C137" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15270,21 +15619,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E137" s="32" t="str">
-        <x:v>Client-side validation uses cryptographic commitments to bind offchain asset rules and transitions, so P2C supplies the contract-anchoring mechanism.</x:v>
+        <x:v>Miner decentralization only makes sense once learners distinguish miners' transaction-ordering role from full nodes' independent enforcement of consensus validity.</x:v>
       </x:c>
       <x:c r="F137" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G137" s="32" t="str">
-        <x:v>Keep this direct edge: it prevents treating client-side validation as a vague UTXO-only extension.</x:v>
+        <x:v>The edge keeps censorship power separate from authority to change consensus rules.</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="32" t="str">
-        <x:v>protocol.rbf</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B138" s="32" t="str">
-        <x:v>protocol.replacement-cycling</x:v>
+        <x:v>mining.miner-decentralization</x:v>
       </x:c>
       <x:c r="C138" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15293,21 +15642,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E138" s="32" t="str">
-        <x:v>Replacement cycling repeatedly uses transaction replacement, so learners need the RBF policy mechanism first.</x:v>
+        <x:v>Pool and solo mining explain the participant and coordination structure whose concentration or dispersion determines practical control over transaction ordering.</x:v>
       </x:c>
       <x:c r="F138" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G138" s="32" t="str">
-        <x:v>Package RBF is related but not required for the core attack sequence.</x:v>
+        <x:v>Stratum V2 remains optional implementation context, not a direct prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="32" t="str">
-        <x:v>protocol.cpfp</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="B139" s="32" t="str">
-        <x:v>protocol.replacement-cycling</x:v>
+        <x:v>dev.selection-cryptography</x:v>
       </x:c>
       <x:c r="C139" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15316,21 +15665,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E139" s="32" t="str">
-        <x:v>The attack cycles child-fee relationships to evict a target, so learners need CPFP mechanics first.</x:v>
+        <x:v>Selection cryptography evaluates cryptographic tools and dependencies through evidence, testing, authorship, and review quality, so learners need the broader Bitcoin review discipline first.</x:v>
       </x:c>
       <x:c r="F139" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G139" s="32" t="str">
-        <x:v>Transaction pinning is the broader downstream risk class, not a prerequisite.</x:v>
+        <x:v>Adversarial thinking is inherited through dev.review-culture; reproducible builds are a downstream verification practice rather than a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="32" t="str">
-        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
+        <x:v>mining.pool-shares</x:v>
       </x:c>
       <x:c r="B140" s="32" t="str">
-        <x:v>protocol.taproot-control-blocks</x:v>
+        <x:v>mining.block-withholding</x:v>
       </x:c>
       <x:c r="C140" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15339,21 +15688,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E140" s="32" t="str">
-        <x:v>Control blocks extend the tapleaf proof path with internal-key and parity data.</x:v>
+        <x:v>Block withholding exploits the difference between a pool-paid share and a share that also meets the network target, so learners must understand share accounting before the attack model makes sense.</x:v>
       </x:c>
       <x:c r="F140" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G140" s="32" t="str">
-        <x:v>Generic Merkle trees are inherited through the proof node.</x:v>
+        <x:v>Pool-versus-solo and mining economics are inherited through mining.pool-shares; do not add a redundant majority-attack edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="32" t="str">
-        <x:v>dev.review-culture</x:v>
+        <x:v>fundamentals.public-private-keys</x:v>
       </x:c>
       <x:c r="B141" s="32" t="str">
-        <x:v>dev.pseudonymous-development</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="C141" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15362,21 +15711,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E141" s="32" t="str">
-        <x:v>Pseudonymous development relies on public technical evidence and independent peer review to preserve accountability without requiring legal-identity disclosure.</x:v>
+        <x:v>P2C tweaks a public key to commit to contract data, so learners need the public/private key model.</x:v>
       </x:c>
       <x:c r="F141" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G141" s="32" t="str">
-        <x:v>Privacy pseudonymity is related context, not a direct prerequisite, because this node concerns contributor identity and governance rather than transaction linkage.</x:v>
+        <x:v>Taproot is adjacent, not a direct requirement.</x:v>
       </x:c>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="32" t="str">
-        <x:v>fundamentals.merkle-trees</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B142" s="32" t="str">
-        <x:v>protocol.mast</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="C142" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15385,21 +15734,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E142" s="32" t="str">
-        <x:v>MAST uses a Merkle tree to commit to multiple alternative script branches while revealing only one branch during spending.</x:v>
+        <x:v>P2C derives a commitment tweak from contract data using a hash, so learners need hash commitments first.</x:v>
       </x:c>
       <x:c r="F142" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G142" s="32" t="str">
-        <x:v>Direct cryptographic structure; TapTree remains a downstream Taproot-specific realization.</x:v>
+        <x:v>The hash is part of the construction rather than generic background.</x:v>
       </x:c>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>protocol.utxo-model</x:v>
       </x:c>
       <x:c r="B143" s="32" t="str">
-        <x:v>protocol.mast</x:v>
+        <x:v>extension.single-use-seals</x:v>
       </x:c>
       <x:c r="C143" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15408,21 +15757,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E143" s="32" t="str">
-        <x:v>MAST commits to alternative Bitcoin Script branches, so learners need the locking and spending language before the tree commitment is meaningful.</x:v>
+        <x:v>Single-use seals rely on a UTXO's one-time spend property.</x:v>
       </x:c>
       <x:c r="F143" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G143" s="32" t="str">
-        <x:v>Keep Script direct; the node is not only a generic Merkle-tree concept.</x:v>
+        <x:v>This explicit bridge prevents hiding the seal invariant inside generic UTXO semantics.</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="32" t="str">
-        <x:v>protocol.sighash-flags</x:v>
+        <x:v>extension.single-use-seals</x:v>
       </x:c>
       <x:c r="B144" s="32" t="str">
-        <x:v>protocol.sighash-quadratic-hashing</x:v>
+        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="C144" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15431,21 +15780,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E144" s="32" t="str">
-        <x:v>The quadratic hashing problem is a performance consequence of how legacy signature digests are constructed under SIGHASH semantics.</x:v>
+        <x:v>Client-side validation relies on seals to prevent an offchain transition from being valid twice.</x:v>
       </x:c>
       <x:c r="F144" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G144" s="32" t="str">
-        <x:v>BIP 143 is a supporting mitigation source, not a prerequisite edge.</x:v>
+        <x:v>The UTXO parent is inherited through the seal and is intentionally not duplicated.</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>protocol.pay-to-contract</x:v>
       </x:c>
       <x:c r="B145" s="32" t="str">
-        <x:v>security.rogue-key-attack</x:v>
+        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="C145" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15454,21 +15803,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E145" s="32" t="str">
-        <x:v>The rogue-key attack occurs in naive public-key aggregation, so learners need the MuSig aggregation setting before the failure mode.</x:v>
+        <x:v>Client-side validation uses cryptographic commitments to bind offchain asset rules and transitions, so P2C supplies the contract-anchoring mechanism.</x:v>
       </x:c>
       <x:c r="F145" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G145" s="32" t="str">
-        <x:v>Schnorr is inherited through MuSig; avoid a redundant direct Schnorr edge.</x:v>
+        <x:v>Keep this direct edge: it prevents treating client-side validation as a vague UTXO-only extension.</x:v>
       </x:c>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>protocol.rbf</x:v>
       </x:c>
       <x:c r="B146" s="32" t="str">
-        <x:v>mining.selfish-mining</x:v>
+        <x:v>protocol.replacement-cycling</x:v>
       </x:c>
       <x:c r="C146" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15477,21 +15826,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E146" s="32" t="str">
-        <x:v>Selfish mining is an incentive strategy by miners and pools, so learners need the pooled-versus-solo mining context first.</x:v>
+        <x:v>Replacement cycling repeatedly uses transaction replacement, so learners need the RBF policy mechanism first.</x:v>
       </x:c>
       <x:c r="F146" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G146" s="32" t="str">
-        <x:v>Pool economics is one direct parent; chain selection is supplied by the finality parent below.</x:v>
+        <x:v>Package RBF is related but not required for the core attack sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="32" t="str">
-        <x:v>protocol.reorgs-finality</x:v>
+        <x:v>protocol.cpfp</x:v>
       </x:c>
       <x:c r="B147" s="32" t="str">
-        <x:v>mining.selfish-mining</x:v>
+        <x:v>protocol.replacement-cycling</x:v>
       </x:c>
       <x:c r="C147" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15500,21 +15849,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E147" s="32" t="str">
-        <x:v>Selfish mining relies on strategic withholding and release of competing branches, which requires the chain-reorganization and finality model.</x:v>
+        <x:v>The attack cycles child-fee relationships to evict a target, so learners need CPFP mechanics first.</x:v>
       </x:c>
       <x:c r="F147" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G147" s="32" t="str">
-        <x:v>Keep the reorganization model direct rather than adding generic proof-of-work as a redundant ancestor.</x:v>
+        <x:v>Transaction pinning is the broader downstream risk class, not a prerequisite.</x:v>
       </x:c>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
       </x:c>
       <x:c r="B148" s="32" t="str">
-        <x:v>protocol.commit-delay-reveal</x:v>
+        <x:v>protocol.taproot-control-blocks</x:v>
       </x:c>
       <x:c r="C148" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15523,21 +15872,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E148" s="32" t="str">
-        <x:v>Commit-delay-reveal composes a cryptographic commitment with a timed reveal, so the learner first needs the hiding and binding commitment model.</x:v>
+        <x:v>Control blocks extend the tapleaf proof path with internal-key and parity data.</x:v>
       </x:c>
       <x:c r="F148" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G148" s="32" t="str">
-        <x:v>The delay/reveal composition is the node's distinct outcome.</x:v>
+        <x:v>Generic Merkle trees are inherited through the proof node.</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="32" t="str">
-        <x:v>protocol.dust-policy</x:v>
+        <x:v>dev.review-culture</x:v>
       </x:c>
       <x:c r="B149" s="32" t="str">
-        <x:v>security.dust-attack</x:v>
+        <x:v>dev.pseudonymous-development</x:v>
       </x:c>
       <x:c r="C149" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15546,21 +15895,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E149" s="32" t="str">
-        <x:v>Dust attacks exploit the distinction between tiny-output relay policy and the ability to place trace-value UTXOs in a wallet.</x:v>
+        <x:v>Pseudonymous development relies on public technical evidence and independent peer review to preserve accountability without requiring legal-identity disclosure.</x:v>
       </x:c>
       <x:c r="F149" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G149" s="32" t="str">
-        <x:v>Policy threshold is direct context for the attack mechanism.</x:v>
+        <x:v>Privacy pseudonymity is related context, not a direct prerequisite, because this node concerns contributor identity and governance rather than transaction linkage.</x:v>
       </x:c>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>fundamentals.merkle-trees</x:v>
       </x:c>
       <x:c r="B150" s="32" t="str">
-        <x:v>security.dust-attack</x:v>
+        <x:v>protocol.mast</x:v>
       </x:c>
       <x:c r="C150" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15569,21 +15918,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E150" s="32" t="str">
-        <x:v>The privacy harm of dusting comes from linking future spends and wallet activity, so learners need the pseudonymity and linkage model.</x:v>
+        <x:v>MAST uses a Merkle tree to commit to multiple alternative script branches while revealing only one branch during spending.</x:v>
       </x:c>
       <x:c r="F150" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
       </x:c>
       <x:c r="G150" s="32" t="str">
-        <x:v>Keep privacy linkage direct; it is not inherited through dust policy.</x:v>
+        <x:v>Direct cryptographic structure; TapTree remains a downstream Taproot-specific realization.</x:v>
       </x:c>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="32" t="str">
-        <x:v>fundamentals.neutrality</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B151" s="32" t="str">
-        <x:v>dev.permissionless-development</x:v>
+        <x:v>protocol.mast</x:v>
       </x:c>
       <x:c r="C151" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15592,21 +15941,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E151" s="32" t="str">
-        <x:v>Permissionless development depends on a neutral protocol that does not select which users or applications may participate.</x:v>
+        <x:v>MAST commits to alternative Bitcoin Script branches, so learners need the locking and spending language before the tree commitment is meaningful.</x:v>
       </x:c>
       <x:c r="F151" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1998431297333501989</x:v>
       </x:c>
       <x:c r="G151" s="32" t="str">
-        <x:v>Neutrality supplies the protocol property; the BIPs process supplies the change/proposal lifecycle below.</x:v>
+        <x:v>Keep Script direct; the node is not only a generic Merkle-tree concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="32" t="str">
-        <x:v>dev.bips-process</x:v>
+        <x:v>protocol.sighash-flags</x:v>
       </x:c>
       <x:c r="B152" s="32" t="str">
-        <x:v>dev.permissionless-development</x:v>
+        <x:v>protocol.sighash-quadratic-hashing</x:v>
       </x:c>
       <x:c r="C152" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15615,21 +15964,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E152" s="32" t="str">
-        <x:v>Learners need the proposal and deployment process to distinguish building permissionlessly from changing Bitcoin's consensus rules without broad adoption.</x:v>
+        <x:v>The quadratic hashing problem is a performance consequence of how legacy signature digests are constructed under SIGHASH semantics.</x:v>
       </x:c>
       <x:c r="F152" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1987562939109306699</x:v>
       </x:c>
       <x:c r="G152" s="32" t="str">
-        <x:v>Review culture remains related but is not a direct prerequisite for permissionless access.</x:v>
+        <x:v>BIP 143 is a supporting mitigation source, not a prerequisite edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="32" t="str">
-        <x:v>dev.reproducible-builds</x:v>
+        <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="B153" s="32" t="str">
-        <x:v>dev.bootstrappable-builds</x:v>
+        <x:v>security.rogue-key-attack</x:v>
       </x:c>
       <x:c r="C153" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15638,21 +15987,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E153" s="32" t="str">
-        <x:v>Bootstrappable builds extend reproducible builds by reducing trust in the compiler and build-tool binaries used to produce the reproducible output.</x:v>
+        <x:v>The rogue-key attack occurs in naive public-key aggregation, so learners need the MuSig aggregation setting before the failure mode.</x:v>
       </x:c>
       <x:c r="F153" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoin-dev-project-post-1976008010108678258</x:v>
       </x:c>
       <x:c r="G153" s="32" t="str">
-        <x:v>Keep this as a direct downstream edge; the node is not a duplicate alias for reproducible builds.</x:v>
+        <x:v>Schnorr is inherited through MuSig; avoid a redundant direct Schnorr edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="32" t="str">
-        <x:v>protocol.transaction-lifecycle</x:v>
+        <x:v>mining.pool-vs-solo</x:v>
       </x:c>
       <x:c r="B154" s="32" t="str">
-        <x:v>protocol.proof-of-payment</x:v>
+        <x:v>mining.selfish-mining</x:v>
       </x:c>
       <x:c r="C154" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15661,21 +16010,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E154" s="32" t="str">
-        <x:v>Proof of Payment refers to a prior payment and reconstructs a transaction-shaped proof, so learners need the transaction lifecycle first.</x:v>
+        <x:v>Selfish mining is an incentive strategy by miners and pools, so learners need the pooled-versus-solo mining context first.</x:v>
       </x:c>
       <x:c r="F154" s="32" t="str">
-        <x:v>source.bitcoin-bips</x:v>
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
       </x:c>
       <x:c r="G154" s="32" t="str">
-        <x:v>Direct payment context; wallet UX and URI transport remain downstream or optional details.</x:v>
+        <x:v>Pool economics is one direct parent; chain selection is supplied by the finality parent below.</x:v>
       </x:c>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="32" t="str">
-        <x:v>protocol.ephemeral-anchors</x:v>
+        <x:v>protocol.reorgs-finality</x:v>
       </x:c>
       <x:c r="B155" s="32" t="str">
-        <x:v>protocol.pay-to-anchor</x:v>
+        <x:v>mining.selfish-mining</x:v>
       </x:c>
       <x:c r="C155" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -15684,12 +16033,196 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E155" s="32" t="str">
+        <x:v>Selfish mining relies on strategic withholding and release of competing branches, which requires the chain-reorganization and finality model.</x:v>
+      </x:c>
+      <x:c r="F155" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1975289920634925475</x:v>
+      </x:c>
+      <x:c r="G155" s="32" t="str">
+        <x:v>Keep the reorganization model direct rather than adding generic proof-of-work as a redundant ancestor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" s="32" t="str">
+        <x:v>fundamentals.commitment-schemes</x:v>
+      </x:c>
+      <x:c r="B156" s="32" t="str">
+        <x:v>protocol.commit-delay-reveal</x:v>
+      </x:c>
+      <x:c r="C156" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D156" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E156" s="32" t="str">
+        <x:v>Commit-delay-reveal composes a cryptographic commitment with a timed reveal, so the learner first needs the hiding and binding commitment model.</x:v>
+      </x:c>
+      <x:c r="F156" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1931775486449103086</x:v>
+      </x:c>
+      <x:c r="G156" s="32" t="str">
+        <x:v>The delay/reveal composition is the node's distinct outcome.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" s="32" t="str">
+        <x:v>protocol.dust-policy</x:v>
+      </x:c>
+      <x:c r="B157" s="32" t="str">
+        <x:v>security.dust-attack</x:v>
+      </x:c>
+      <x:c r="C157" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D157" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E157" s="32" t="str">
+        <x:v>Dust attacks exploit the distinction between tiny-output relay policy and the ability to place trace-value UTXOs in a wallet.</x:v>
+      </x:c>
+      <x:c r="F157" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+      </x:c>
+      <x:c r="G157" s="32" t="str">
+        <x:v>Policy threshold is direct context for the attack mechanism.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" s="32" t="str">
+        <x:v>privacy.pseudonymity</x:v>
+      </x:c>
+      <x:c r="B158" s="32" t="str">
+        <x:v>security.dust-attack</x:v>
+      </x:c>
+      <x:c r="C158" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D158" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E158" s="32" t="str">
+        <x:v>The privacy harm of dusting comes from linking future spends and wallet activity, so learners need the pseudonymity and linkage model.</x:v>
+      </x:c>
+      <x:c r="F158" s="32" t="str">
+        <x:v>source.bitcoin-dev-project-post-1904946739603452376</x:v>
+      </x:c>
+      <x:c r="G158" s="32" t="str">
+        <x:v>Keep privacy linkage direct; it is not inherited through dust policy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" s="32" t="str">
+        <x:v>fundamentals.neutrality</x:v>
+      </x:c>
+      <x:c r="B159" s="32" t="str">
+        <x:v>dev.permissionless-development</x:v>
+      </x:c>
+      <x:c r="C159" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D159" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E159" s="32" t="str">
+        <x:v>Permissionless development depends on a neutral protocol that does not select which users or applications may participate.</x:v>
+      </x:c>
+      <x:c r="F159" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G159" s="32" t="str">
+        <x:v>Neutrality supplies the protocol property; the BIPs process supplies the change/proposal lifecycle below.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="A160" s="32" t="str">
+        <x:v>dev.bips-process</x:v>
+      </x:c>
+      <x:c r="B160" s="32" t="str">
+        <x:v>dev.permissionless-development</x:v>
+      </x:c>
+      <x:c r="C160" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D160" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E160" s="32" t="str">
+        <x:v>Learners need the proposal and deployment process to distinguish building permissionlessly from changing Bitcoin's consensus rules without broad adoption.</x:v>
+      </x:c>
+      <x:c r="F160" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G160" s="32" t="str">
+        <x:v>Review culture remains related but is not a direct prerequisite for permissionless access.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161">
+      <x:c r="A161" s="32" t="str">
+        <x:v>dev.reproducible-builds</x:v>
+      </x:c>
+      <x:c r="B161" s="32" t="str">
+        <x:v>dev.bootstrappable-builds</x:v>
+      </x:c>
+      <x:c r="C161" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D161" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E161" s="32" t="str">
+        <x:v>Bootstrappable builds extend reproducible builds by reducing trust in the compiler and build-tool binaries used to produce the reproducible output.</x:v>
+      </x:c>
+      <x:c r="F161" s="32" t="str">
+        <x:v>source.bitcoin-dev-philosophy</x:v>
+      </x:c>
+      <x:c r="G161" s="32" t="str">
+        <x:v>Keep this as a direct downstream edge; the node is not a duplicate alias for reproducible builds.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162">
+      <x:c r="A162" s="32" t="str">
+        <x:v>protocol.transaction-lifecycle</x:v>
+      </x:c>
+      <x:c r="B162" s="32" t="str">
+        <x:v>protocol.proof-of-payment</x:v>
+      </x:c>
+      <x:c r="C162" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D162" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E162" s="32" t="str">
+        <x:v>Proof of Payment refers to a prior payment and reconstructs a transaction-shaped proof, so learners need the transaction lifecycle first.</x:v>
+      </x:c>
+      <x:c r="F162" s="32" t="str">
+        <x:v>source.bitcoin-bips</x:v>
+      </x:c>
+      <x:c r="G162" s="32" t="str">
+        <x:v>Direct payment context; wallet UX and URI transport remain downstream or optional details.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" s="32" t="str">
+        <x:v>protocol.ephemeral-anchors</x:v>
+      </x:c>
+      <x:c r="B163" s="32" t="str">
+        <x:v>protocol.pay-to-anchor</x:v>
+      </x:c>
+      <x:c r="C163" s="32" t="str">
+        <x:v>prerequisite</x:v>
+      </x:c>
+      <x:c r="D163" s="32" t="str">
+        <x:v>proposed</x:v>
+      </x:c>
+      <x:c r="E163" s="32" t="str">
         <x:v>Pay to Anchor is a keyless refinement of the anchor-output and package-relay fee-bumping pattern, so learners need that broader context first.</x:v>
       </x:c>
-      <x:c r="F155" s="32" t="str">
+      <x:c r="F163" s="32" t="str">
         <x:v>source.bitcoin-bips</x:v>
       </x:c>
-      <x:c r="G155" s="32" t="str">
+      <x:c r="G163" s="32" t="str">
         <x:v>BIP 431/TRUC is related anti-pinning context, not an inherent prerequisite.</x:v>
       </x:c>
     </x:row>
@@ -15699,10 +16232,10 @@
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C12:C155">
+    <x:dataValidation type="list" sqref="C12:C163">
       <x:formula1>Lists!$G$2:$G$2</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D155">
+    <x:dataValidation type="list" sqref="D12:D163">
       <x:formula1>Lists!$H$2:$H$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -18940,16 +19473,42 @@
         <x:v>Add Merged Mining. Keep hashprice, difficulty estimators, profitability calculators, monitors, hosted-mining companies, and energy datasets as resources or operational context.</x:v>
       </x:c>
     </x:row>
+    <x:row r="134">
+      <x:c r="A134" s="32" t="str">
+        <x:v>decision.lopp-bitcoin-other-layers-slice</x:v>
+      </x:c>
+      <x:c r="B134" s="32" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="C134" s="32" t="str">
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
+      </x:c>
+      <x:c r="D134" s="32" t="str">
+        <x:v>resolved</x:v>
+      </x:c>
+      <x:c r="E134" s="32" t="str">
+        <x:v>The index contains both reusable layer architectures and a long tail of named projects. The graph should add architectures with independent learning outcomes while preserving concrete protocols and products as future source-specific candidates or resources.</x:v>
+      </x:c>
+      <x:c r="F134" s="32" t="str">
+        <x:v>extension.drivechains, extension.softchains, extension.spiderchains, extension.rollups, extension.cross-chain-bridges, extension.sidechains, extension.statechains, extension.spacechains, extension.bitvm, extension.cube, extension.rgb, extension.liquid</x:v>
+      </x:c>
+      <x:c r="G134" s="32" t="str">
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
+      </x:c>
+      <x:c r="H134" s="32" t="str">
+        <x:v>Add five architectural concepts. Softchains and Cross-Chain Bridges use Sidechains as their only direct prerequisite because Sidechains already carries the inherited consensus and Byzantine-system context. Keep Rootstock, Stacks, Citrea, Mainstay, Counterparty, Revault, Sapio, Tachi, TradeLayer, ION, Spaces, and individual bridge/ecash implementations for separate audits rather than creating project-wrapper nodes from a directory listing.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B12:B133">
+    <x:dataValidation type="list" sqref="B12:B134">
       <x:formula1>Lists!$I$2:$I$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D12:D133">
+    <x:dataValidation type="list" sqref="D12:D134">
       <x:formula1>Lists!$J$2:$J$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -19002,7 +19561,7 @@
         <x:v>Generated At</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46214.795559212966</x:v>
+        <x:v>46214.80091740741</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -19010,7 +19569,7 @@
         <x:v>Seed Sources</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>67</x:v>
+        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -19018,7 +19577,7 @@
         <x:v>Completed Sources</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>67</x:v>
+        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -19026,7 +19585,7 @@
         <x:v>Concept Candidates</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>166</x:v>
+        <x:v>171</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -19034,7 +19593,7 @@
         <x:v>Proposed Edges</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>144</x:v>
+        <x:v>152</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -19058,7 +19617,7 @@
         <x:v>New Concepts</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>107</x:v>
+        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
feat: add covenant taxonomy concepts
</commit_message>
<xml_diff>
--- a/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
+++ b/outputs/content-source-audit/btc-graph-content-source-audit.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Rf0e2a5ba15f54f22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="Raf1d774e401e49a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R3cbb145a9f964051"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rc006879e0b3e49db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="Rdef7987bcef6459d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rd06385608df0405e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="Re28a601049024ca2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concepts" sheetId="2" r:id="R2d3eb348bb224c38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rc41f3409543640a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R15392b3f681346d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R251e32c85cd64e98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R905ec96883b2408b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3783,22 +3783,69 @@
         <x:v>Added Drivechains, Softchains, Spiderchains, Bitcoin Rollups, and Cross-Chain Bridges. Lightning, Liquid, Elements, Statechains, Spark, Spacechains, BitVM, DLCs, Cashu, Fedimint, Ark, Cube, RGB, Nostr, and Covenants already exist. Rootstock, Stacks, Citrea, Mainstay, Counterparty, Revault, Sapio, Tachi, TradeLayer, ION, and Spaces remain named projects or specialized protocols for future source-specific review rather than automatic nodes.</x:v>
       </x:c>
     </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="32" t="str">
+        <x:v>source.bitcoin-covenants</x:v>
+      </x:c>
+      <x:c r="B81" s="32" t="str">
+        <x:v>Bitcoin Covenants Research Compilation</x:v>
+      </x:c>
+      <x:c r="C81" s="32" t="str">
+        <x:v>https://bitcoincovenants.com/</x:v>
+      </x:c>
+      <x:c r="D81" s="32" t="str">
+        <x:v>protocol-research-compilation</x:v>
+      </x:c>
+      <x:c r="E81" s="32" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F81" s="32" t="str">
+        <x:v>Covenant definitions, generalized and recursive covenant distinctions, opcode-based and signature-based constructions, current proposals, and covenant use cases.</x:v>
+      </x:c>
+      <x:c r="G81" s="32" t="str">
+        <x:v>Track the compilation's conceptual taxonomy and proposal references as one covenant research cluster. Deduplicate opcode-specific entries against existing CTV, ANYPREVOUT, OP_CHECKSIGFROMSTACK, OP_CAT, MATT/CCV, and vault nodes; add only reusable distinctions absent from the graph.</x:v>
+      </x:c>
+      <x:c r="H81" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I81" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J81" s="32" t="str">
+        <x:v>Normalized</x:v>
+      </x:c>
+      <x:c r="K81" s="32" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="L81" s="32" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="M81" s="32" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="N81" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O81" s="32" t="str">
+        <x:v>Added Generalized Covenants and Recursive Covenants. The base Covenants node and the major mechanisms surveyed by the site already exist; obsolete or superseded proposals remain historical research context.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H12:H80">
+    <x:dataValidation type="list" sqref="H12:H81">
       <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I12:I80">
+    <x:dataValidation type="list" sqref="I12:I81">
       <x:formula1>Lists!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J12:J80">
+    <x:dataValidation type="list" sqref="J12:J81">
       <x:formula1>Lists!$C$2:$C$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K12:K80">
+    <x:dataValidation type="list" sqref="K12:K81">
       <x:formula1>Lists!$D$2:$D$5</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -12655,16 +12702,118 @@
         <x:v>Keep custodial, federated, light-client, and cryptographic bridge variants as comparative mechanisms rather than separate nodes.</x:v>
       </x:c>
     </x:row>
+    <x:row r="183">
+      <x:c r="A183" s="32" t="str">
+        <x:v>protocol.generalized-covenants</x:v>
+      </x:c>
+      <x:c r="B183" s="32" t="str">
+        <x:v>Generalized Covenants</x:v>
+      </x:c>
+      <x:c r="C183" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D183" s="32" t="str">
+        <x:v>source.bitcoin-covenants</x:v>
+      </x:c>
+      <x:c r="E183" s="32" t="str">
+        <x:v>https://bitcoincovenants.com/</x:v>
+      </x:c>
+      <x:c r="F183" s="32" t="str">
+        <x:v>Covenant taxonomy and generalized-versus-restricted discussion</x:v>
+      </x:c>
+      <x:c r="G183" s="32" t="str"/>
+      <x:c r="H183" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I183" s="32" t="str">
+        <x:v>Generalized covenants describe a distinct design space for broad future-transaction constraints, unlike narrowly scoped proposals such as CTV or vault-specific constructions.</x:v>
+      </x:c>
+      <x:c r="J183" s="32" t="str">
+        <x:v>protocol.covenants</x:v>
+      </x:c>
+      <x:c r="K183" s="32" t="str">
+        <x:v>protocol.covenants</x:v>
+      </x:c>
+      <x:c r="L183" s="32" t="str">
+        <x:v>The learner needs the generic covenant model before comparing generalized and restricted expressiveness.</x:v>
+      </x:c>
+      <x:c r="M183" s="32" t="str">
+        <x:v>generalized covenant, general covenants</x:v>
+      </x:c>
+      <x:c r="N183" s="32" t="str">
+        <x:v>covenants, script, transaction-introspection, protocol-design</x:v>
+      </x:c>
+      <x:c r="O183" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P183" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q183" s="32" t="str">
+        <x:v>Add as a taxonomy concept; individual opcode proposals remain separate nodes or resources.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184">
+      <x:c r="A184" s="32" t="str">
+        <x:v>protocol.recursive-covenants</x:v>
+      </x:c>
+      <x:c r="B184" s="32" t="str">
+        <x:v>Recursive Covenants</x:v>
+      </x:c>
+      <x:c r="C184" s="32" t="str">
+        <x:v>Protocol &amp; Consensus</x:v>
+      </x:c>
+      <x:c r="D184" s="32" t="str">
+        <x:v>source.bitcoin-covenants</x:v>
+      </x:c>
+      <x:c r="E184" s="32" t="str">
+        <x:v>https://bitcoincovenants.com/</x:v>
+      </x:c>
+      <x:c r="F184" s="32" t="str">
+        <x:v>Definition of recursive covenants and repeated output constraints</x:v>
+      </x:c>
+      <x:c r="G184" s="32" t="str"/>
+      <x:c r="H184" s="32" t="str">
+        <x:v>new</x:v>
+      </x:c>
+      <x:c r="I184" s="32" t="str">
+        <x:v>Recursive covenants preserve or reproduce spending constraints across successive outputs, creating a distinct learning outcome around repeated enforcement, escape paths, and liveness tradeoffs.</x:v>
+      </x:c>
+      <x:c r="J184" s="32" t="str">
+        <x:v>protocol.covenants</x:v>
+      </x:c>
+      <x:c r="K184" s="32" t="str">
+        <x:v>protocol.covenants</x:v>
+      </x:c>
+      <x:c r="L184" s="32" t="str">
+        <x:v>The generic covenant model is required before recursion across transaction generations can be understood.</x:v>
+      </x:c>
+      <x:c r="M184" s="32" t="str">
+        <x:v>recursive covenant, covenant recursion</x:v>
+      </x:c>
+      <x:c r="N184" s="32" t="str">
+        <x:v>covenants, recursive, script, transaction-introspection</x:v>
+      </x:c>
+      <x:c r="O184" s="32" t="str">
+        <x:v>35m</x:v>
+      </x:c>
+      <x:c r="P184" s="32" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="Q184" s="32" t="str">
+        <x:v>Add as a reusable covenant property; application-specific recursive constructions remain resources.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="H12:H182">
+    <x:dataValidation type="list" sqref="H12:H184">
       <x:formula1>Lists!$E$2:$E$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P12:P182">
+    <x:dataValidation type="list" sqref="P12:P184">
       <x:formula1>Lists!$F$2:$F$4</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -12732,10 +12881,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="32" t="str">
-        <x:v>extension.sidechains</x:v>
+        <x:v>protocol.covenants</x:v>
       </x:c>
       <x:c r="B12" s="32" t="str">
-        <x:v>extension.drivechains</x:v>
+        <x:v>protocol.generalized-covenants</x:v>
       </x:c>
       <x:c r="C12" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12744,10 +12893,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E12" s="32" t="str">
-        <x:v>Drivechains are a concrete sidechain design with additional miner-mediated peg assumptions.</x:v>
+        <x:v>Generalized covenants are a broader expressiveness category within the covenant design space.</x:v>
       </x:c>
       <x:c r="F12" s="32" t="str">
-        <x:v>source.lopp-bitcoin-other-layers</x:v>
+        <x:v>source.bitcoin-covenants</x:v>
       </x:c>
       <x:c r="G12" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12755,10 +12904,10 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="32" t="str">
-        <x:v>mining.merge-mining</x:v>
+        <x:v>protocol.covenants</x:v>
       </x:c>
       <x:c r="B13" s="32" t="str">
-        <x:v>extension.drivechains</x:v>
+        <x:v>protocol.recursive-covenants</x:v>
       </x:c>
       <x:c r="C13" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12767,10 +12916,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E13" s="32" t="str">
-        <x:v>Drivechains use auxiliary proof-of-work and miner participation as part of their withdrawal model.</x:v>
+        <x:v>Recursive covenants are a property of covenant constraints that persist across successive outputs.</x:v>
       </x:c>
       <x:c r="F13" s="32" t="str">
-        <x:v>source.lopp-bitcoin-other-layers</x:v>
+        <x:v>source.bitcoin-covenants</x:v>
       </x:c>
       <x:c r="G13" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12781,7 +12930,7 @@
         <x:v>extension.sidechains</x:v>
       </x:c>
       <x:c r="B14" s="32" t="str">
-        <x:v>extension.softchains</x:v>
+        <x:v>extension.drivechains</x:v>
       </x:c>
       <x:c r="C14" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12790,7 +12939,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E14" s="32" t="str">
-        <x:v>Softchains are a proposed sidechain architecture with Bitcoin-enforced anchoring assumptions.</x:v>
+        <x:v>Drivechains are a concrete sidechain design with additional miner-mediated peg assumptions.</x:v>
       </x:c>
       <x:c r="F14" s="32" t="str">
         <x:v>source.lopp-bitcoin-other-layers</x:v>
@@ -12801,10 +12950,10 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="32" t="str">
-        <x:v>extension.sidechains</x:v>
+        <x:v>mining.merge-mining</x:v>
       </x:c>
       <x:c r="B15" s="32" t="str">
-        <x:v>extension.spiderchains</x:v>
+        <x:v>extension.drivechains</x:v>
       </x:c>
       <x:c r="C15" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12813,7 +12962,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E15" s="32" t="str">
-        <x:v>Spiderchains are a concrete sidechain design using operator multisig for peg coordination.</x:v>
+        <x:v>Drivechains use auxiliary proof-of-work and miner participation as part of their withdrawal model.</x:v>
       </x:c>
       <x:c r="F15" s="32" t="str">
         <x:v>source.lopp-bitcoin-other-layers</x:v>
@@ -12824,10 +12973,10 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>extension.sidechains</x:v>
       </x:c>
       <x:c r="B16" s="32" t="str">
-        <x:v>extension.spiderchains</x:v>
+        <x:v>extension.softchains</x:v>
       </x:c>
       <x:c r="C16" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12836,7 +12985,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E16" s="32" t="str">
-        <x:v>Spiderchains use collateralized multisig operators as a core coordination mechanism.</x:v>
+        <x:v>Softchains are a proposed sidechain architecture with Bitcoin-enforced anchoring assumptions.</x:v>
       </x:c>
       <x:c r="F16" s="32" t="str">
         <x:v>source.lopp-bitcoin-other-layers</x:v>
@@ -12847,10 +12996,10 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="32" t="str">
-        <x:v>fundamentals.zero-knowledge-proofs</x:v>
+        <x:v>extension.sidechains</x:v>
       </x:c>
       <x:c r="B17" s="32" t="str">
-        <x:v>extension.rollups</x:v>
+        <x:v>extension.spiderchains</x:v>
       </x:c>
       <x:c r="C17" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12859,7 +13008,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E17" s="32" t="str">
-        <x:v>Validity-rollup designs use proof-based verification for off-chain execution claims.</x:v>
+        <x:v>Spiderchains are a concrete sidechain design using operator multisig for peg coordination.</x:v>
       </x:c>
       <x:c r="F17" s="32" t="str">
         <x:v>source.lopp-bitcoin-other-layers</x:v>
@@ -12870,10 +13019,10 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="32" t="str">
-        <x:v>extension.sidechains</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B18" s="32" t="str">
-        <x:v>extension.rollups</x:v>
+        <x:v>extension.spiderchains</x:v>
       </x:c>
       <x:c r="C18" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12882,7 +13031,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E18" s="32" t="str">
-        <x:v>Rollups are an anchored secondary execution layer and require the broader layer/settlement model.</x:v>
+        <x:v>Spiderchains use collateralized multisig operators as a core coordination mechanism.</x:v>
       </x:c>
       <x:c r="F18" s="32" t="str">
         <x:v>source.lopp-bitcoin-other-layers</x:v>
@@ -12893,10 +13042,10 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="32" t="str">
-        <x:v>extension.sidechains</x:v>
+        <x:v>fundamentals.zero-knowledge-proofs</x:v>
       </x:c>
       <x:c r="B19" s="32" t="str">
-        <x:v>extension.cross-chain-bridges</x:v>
+        <x:v>extension.rollups</x:v>
       </x:c>
       <x:c r="C19" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12905,7 +13054,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E19" s="32" t="str">
-        <x:v>Bridge security is easiest to understand after the learner knows how anchored secondary chains differ from Bitcoin's base layer.</x:v>
+        <x:v>Validity-rollup designs use proof-based verification for off-chain execution claims.</x:v>
       </x:c>
       <x:c r="F19" s="32" t="str">
         <x:v>source.lopp-bitcoin-other-layers</x:v>
@@ -12916,10 +13065,10 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="32" t="str">
-        <x:v>extension.client-side-validation</x:v>
+        <x:v>extension.sidechains</x:v>
       </x:c>
       <x:c r="B20" s="32" t="str">
-        <x:v>extension.rgb</x:v>
+        <x:v>extension.rollups</x:v>
       </x:c>
       <x:c r="C20" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12928,10 +13077,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E20" s="32" t="str">
-        <x:v>RGB builds its contract and asset model on client-side validation of off-chain state anchored to Bitcoin outputs.</x:v>
+        <x:v>Rollups are an anchored secondary execution layer and require the broader layer/settlement model.</x:v>
       </x:c>
       <x:c r="F20" s="32" t="str">
-        <x:v>source.rgb-protocol</x:v>
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
       </x:c>
       <x:c r="G20" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12939,10 +13088,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>extension.sidechains</x:v>
       </x:c>
       <x:c r="B21" s="32" t="str">
-        <x:v>protocol.confidential-transactions</x:v>
+        <x:v>extension.cross-chain-bridges</x:v>
       </x:c>
       <x:c r="C21" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12951,10 +13100,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E21" s="32" t="str">
-        <x:v>Confidential Transactions use cryptographic commitments to hide values while preserving verifiability.</x:v>
+        <x:v>Bridge security is easiest to understand after the learner knows how anchored secondary chains differ from Bitcoin's base layer.</x:v>
       </x:c>
       <x:c r="F21" s="32" t="str">
-        <x:v>source.liquid-elements</x:v>
+        <x:v>source.lopp-bitcoin-other-layers</x:v>
       </x:c>
       <x:c r="G21" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12962,10 +13111,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32" t="str">
-        <x:v>extension.sidechains</x:v>
+        <x:v>extension.client-side-validation</x:v>
       </x:c>
       <x:c r="B22" s="32" t="str">
-        <x:v>extension.elements</x:v>
+        <x:v>extension.rgb</x:v>
       </x:c>
       <x:c r="C22" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12974,10 +13123,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E22" s="32" t="str">
-        <x:v>Elements is a concrete platform for constructing Bitcoin-derived sidechains and application-specific networks.</x:v>
+        <x:v>RGB builds its contract and asset model on client-side validation of off-chain state anchored to Bitcoin outputs.</x:v>
       </x:c>
       <x:c r="F22" s="32" t="str">
-        <x:v>source.liquid-elements</x:v>
+        <x:v>source.rgb-protocol</x:v>
       </x:c>
       <x:c r="G22" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -12985,10 +13134,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32" t="str">
-        <x:v>extension.elements</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="B23" s="32" t="str">
-        <x:v>extension.liquid</x:v>
+        <x:v>protocol.confidential-transactions</x:v>
       </x:c>
       <x:c r="C23" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -12997,7 +13146,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E23" s="32" t="str">
-        <x:v>Liquid is a production network built on the Elements platform, with its own federation, peg, and asset policies.</x:v>
+        <x:v>Confidential Transactions use cryptographic commitments to hide values while preserving verifiability.</x:v>
       </x:c>
       <x:c r="F23" s="32" t="str">
         <x:v>source.liquid-elements</x:v>
@@ -13008,10 +13157,10 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="str">
-        <x:v>protocol.confidential-transactions</x:v>
+        <x:v>extension.sidechains</x:v>
       </x:c>
       <x:c r="B24" s="32" t="str">
-        <x:v>extension.liquid</x:v>
+        <x:v>extension.elements</x:v>
       </x:c>
       <x:c r="C24" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13020,7 +13169,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E24" s="32" t="str">
-        <x:v>Liquid's privacy and issued-asset behavior depends on Confidential Transactions as a core transaction primitive.</x:v>
+        <x:v>Elements is a concrete platform for constructing Bitcoin-derived sidechains and application-specific networks.</x:v>
       </x:c>
       <x:c r="F24" s="32" t="str">
         <x:v>source.liquid-elements</x:v>
@@ -13031,10 +13180,10 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="str">
-        <x:v>protocol.timelocks</x:v>
+        <x:v>extension.elements</x:v>
       </x:c>
       <x:c r="B25" s="32" t="str">
-        <x:v>extension.timeout-trees</x:v>
+        <x:v>extension.liquid</x:v>
       </x:c>
       <x:c r="C25" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13043,10 +13192,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E25" s="32" t="str">
-        <x:v>Timeout Trees use delayed transaction branches to preserve unilateral redemption, so learners need Bitcoin timelocks first.</x:v>
+        <x:v>Liquid is a production network built on the Elements platform, with its own federation, peg, and asset policies.</x:v>
       </x:c>
       <x:c r="F25" s="32" t="str">
-        <x:v>source.cube-introducing</x:v>
+        <x:v>source.liquid-elements</x:v>
       </x:c>
       <x:c r="G25" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -13054,10 +13203,10 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="str">
-        <x:v>extension.timeout-trees</x:v>
+        <x:v>protocol.confidential-transactions</x:v>
       </x:c>
       <x:c r="B26" s="32" t="str">
-        <x:v>extension.zktlcs</x:v>
+        <x:v>extension.liquid</x:v>
       </x:c>
       <x:c r="C26" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13066,10 +13215,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E26" s="32" t="str">
-        <x:v>ZKTLCs use timeout-tree ownership virtualization as one half of their unified primitive.</x:v>
+        <x:v>Liquid's privacy and issued-asset behavior depends on Confidential Transactions as a core transaction primitive.</x:v>
       </x:c>
       <x:c r="F26" s="32" t="str">
-        <x:v>source.cube-introducing</x:v>
+        <x:v>source.liquid-elements</x:v>
       </x:c>
       <x:c r="G26" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -13077,10 +13226,10 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="str">
-        <x:v>extension.bitvm</x:v>
+        <x:v>protocol.timelocks</x:v>
       </x:c>
       <x:c r="B27" s="32" t="str">
-        <x:v>extension.zktlcs</x:v>
+        <x:v>extension.timeout-trees</x:v>
       </x:c>
       <x:c r="C27" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13089,7 +13238,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E27" s="32" t="str">
-        <x:v>ZKTLCs use BitVM-style challenge and disproof to enforce computation without trusting the executor.</x:v>
+        <x:v>Timeout Trees use delayed transaction branches to preserve unilateral redemption, so learners need Bitcoin timelocks first.</x:v>
       </x:c>
       <x:c r="F27" s="32" t="str">
         <x:v>source.cube-introducing</x:v>
@@ -13100,10 +13249,10 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32" t="str">
+        <x:v>extension.timeout-trees</x:v>
+      </x:c>
+      <x:c r="B28" s="32" t="str">
         <x:v>extension.zktlcs</x:v>
-      </x:c>
-      <x:c r="B28" s="32" t="str">
-        <x:v>extension.cube</x:v>
       </x:c>
       <x:c r="C28" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13112,7 +13261,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E28" s="32" t="str">
-        <x:v>Cube's architecture is built around ZKTLCs for programmable execution, ownership, and unilateral exit.</x:v>
+        <x:v>ZKTLCs use timeout-tree ownership virtualization as one half of their unified primitive.</x:v>
       </x:c>
       <x:c r="F28" s="32" t="str">
         <x:v>source.cube-introducing</x:v>
@@ -13123,10 +13272,10 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="32" t="str">
-        <x:v>extension.statechains</x:v>
+        <x:v>extension.bitvm</x:v>
       </x:c>
       <x:c r="B29" s="32" t="str">
-        <x:v>extension.spark</x:v>
+        <x:v>extension.zktlcs</x:v>
       </x:c>
       <x:c r="C29" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13135,10 +13284,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E29" s="32" t="str">
-        <x:v>Spark's architecture extends statechain-style off-chain ownership transfer with a distributed operator set and Lightning interoperability.</x:v>
+        <x:v>ZKTLCs use BitVM-style challenge and disproof to enforce computation without trusting the executor.</x:v>
       </x:c>
       <x:c r="F29" s="32" t="str">
-        <x:v>source.spark-protocol</x:v>
+        <x:v>source.cube-introducing</x:v>
       </x:c>
       <x:c r="G29" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -13146,10 +13295,10 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32" t="str">
-        <x:v>history.cypherpunk-roots-bitcoin-origin</x:v>
+        <x:v>extension.zktlcs</x:v>
       </x:c>
       <x:c r="B30" s="32" t="str">
-        <x:v>history.satoshi-nakamoto</x:v>
+        <x:v>extension.cube</x:v>
       </x:c>
       <x:c r="C30" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13158,10 +13307,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E30" s="32" t="str">
-        <x:v>Satoshi's pseudonym and founder independence are best understood in the context of Bitcoin's cypherpunk roots and origin story.</x:v>
+        <x:v>Cube's architecture is built around ZKTLCs for programmable execution, ownership, and unilateral exit.</x:v>
       </x:c>
       <x:c r="F30" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.cube-introducing</x:v>
       </x:c>
       <x:c r="G30" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -13169,10 +13318,10 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="str">
-        <x:v>fundamentals.money-properties</x:v>
+        <x:v>extension.statechains</x:v>
       </x:c>
       <x:c r="B31" s="32" t="str">
-        <x:v>economics.bitcoin-denominations</x:v>
+        <x:v>extension.spark</x:v>
       </x:c>
       <x:c r="C31" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13181,10 +13330,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E31" s="32" t="str">
-        <x:v>The learner needs a basic monetary-unit model before BTC and satoshis are meaningful denominations.</x:v>
+        <x:v>Spark's architecture extends statechain-style off-chain ownership transfer with a distributed operator set and Lightning interoperability.</x:v>
       </x:c>
       <x:c r="F31" s="32" t="str">
-        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
+        <x:v>source.spark-protocol</x:v>
       </x:c>
       <x:c r="G31" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -13192,10 +13341,10 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="32" t="str">
-        <x:v>protocol.coinbase-transaction</x:v>
+        <x:v>history.cypherpunk-roots-bitcoin-origin</x:v>
       </x:c>
       <x:c r="B32" s="32" t="str">
-        <x:v>economics.block-subsidy</x:v>
+        <x:v>history.satoshi-nakamoto</x:v>
       </x:c>
       <x:c r="C32" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13204,21 +13353,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E32" s="32" t="str">
-        <x:v>The block subsidy is the newly issued component claimed by a coinbase transaction.</x:v>
+        <x:v>Satoshi's pseudonym and founder independence are best understood in the context of Bitcoin's cypherpunk roots and origin story.</x:v>
       </x:c>
       <x:c r="F32" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G32" s="32" t="str">
-        <x:v>The coinbase node already carries the halving prerequisite, so no redundant direct halving edge is added.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="32" t="str">
-        <x:v>fundamentals.digital-signatures</x:v>
+        <x:v>fundamentals.money-properties</x:v>
       </x:c>
       <x:c r="B33" s="32" t="str">
-        <x:v>security.quantum-computing-threat</x:v>
+        <x:v>economics.bitcoin-denominations</x:v>
       </x:c>
       <x:c r="C33" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13227,7 +13376,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E33" s="32" t="str">
-        <x:v>Quantum attacks on public-key authorization require understanding ordinary Bitcoin signature security first.</x:v>
+        <x:v>The learner needs a basic monetary-unit model before BTC and satoshis are meaningful denominations.</x:v>
       </x:c>
       <x:c r="F33" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
@@ -13238,10 +13387,10 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.coinbase-transaction</x:v>
       </x:c>
       <x:c r="B34" s="32" t="str">
-        <x:v>extension.ordinals-inscriptions</x:v>
+        <x:v>economics.block-subsidy</x:v>
       </x:c>
       <x:c r="C34" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13250,21 +13399,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E34" s="32" t="str">
-        <x:v>The source explains inscriptions as a Taproot-era witness-data application.</x:v>
+        <x:v>The block subsidy is the newly issued component claimed by a coinbase transaction.</x:v>
       </x:c>
       <x:c r="F34" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G34" s="32" t="str">
-        <x:v>Source-driven bridge edge.</x:v>
+        <x:v>The coinbase node already carries the halving prerequisite, so no redundant direct halving edge is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="32" t="str">
-        <x:v>protocol.witness-structure</x:v>
+        <x:v>fundamentals.digital-signatures</x:v>
       </x:c>
       <x:c r="B35" s="32" t="str">
-        <x:v>extension.ordinals-inscriptions</x:v>
+        <x:v>security.quantum-computing-threat</x:v>
       </x:c>
       <x:c r="C35" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13273,7 +13422,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E35" s="32" t="str">
-        <x:v>Witness structure is needed to understand where inscription data is carried and how it affects block space.</x:v>
+        <x:v>Quantum attacks on public-key authorization require understanding ordinary Bitcoin signature security first.</x:v>
       </x:c>
       <x:c r="F35" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
@@ -13284,10 +13433,10 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="32" t="str">
-        <x:v>fundamentals.commitment-schemes</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B36" s="32" t="str">
-        <x:v>extension.proof-of-existence</x:v>
+        <x:v>extension.ordinals-inscriptions</x:v>
       </x:c>
       <x:c r="C36" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13296,7 +13445,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E36" s="32" t="str">
-        <x:v>Timestamp proofs commit evidence without requiring the complete document to be stored on-chain.</x:v>
+        <x:v>The source explains inscriptions as a Taproot-era witness-data application.</x:v>
       </x:c>
       <x:c r="F36" s="32" t="str">
         <x:v>source.101-perguntas-bitcoin-1ed</x:v>
@@ -13307,10 +13456,10 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="32" t="str">
-        <x:v>protocol.tagged-hashes</x:v>
+        <x:v>protocol.witness-structure</x:v>
       </x:c>
       <x:c r="B37" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>extension.ordinals-inscriptions</x:v>
       </x:c>
       <x:c r="C37" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13319,10 +13468,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E37" s="32" t="str">
-        <x:v>TapTweak is defined using tagged hashes directly in Taproot key tweaking.</x:v>
+        <x:v>Witness structure is needed to understand where inscription data is carried and how it affects block space.</x:v>
       </x:c>
       <x:c r="F37" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G37" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -13330,10 +13479,10 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="32" t="str">
-        <x:v>protocol.x-only-public-keys</x:v>
+        <x:v>fundamentals.commitment-schemes</x:v>
       </x:c>
       <x:c r="B38" s="32" t="str">
-        <x:v>protocol.taptweak</x:v>
+        <x:v>extension.proof-of-existence</x:v>
       </x:c>
       <x:c r="C38" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13342,10 +13491,10 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E38" s="32" t="str">
-        <x:v>TapTweak operates on x-only public keys in the Taproot construction.</x:v>
+        <x:v>Timestamp proofs commit evidence without requiring the complete document to be stored on-chain.</x:v>
       </x:c>
       <x:c r="F38" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.101-perguntas-bitcoin-1ed</x:v>
       </x:c>
       <x:c r="G38" s="32" t="str">
         <x:v>Source-driven bridge edge.</x:v>
@@ -13353,10 +13502,10 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="32" t="str">
+        <x:v>protocol.tagged-hashes</x:v>
+      </x:c>
+      <x:c r="B39" s="32" t="str">
         <x:v>protocol.taptweak</x:v>
-      </x:c>
-      <x:c r="B39" s="32" t="str">
-        <x:v>protocol.taproot-key-path-spends</x:v>
       </x:c>
       <x:c r="C39" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13365,21 +13514,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E39" s="32" t="str">
-        <x:v>A key-path spend verifies against the tweaked Taproot output key, so learners need the tweak mechanism before the spending mode makes sense.</x:v>
+        <x:v>TapTweak is defined using tagged hashes directly in Taproot key tweaking.</x:v>
       </x:c>
       <x:c r="F39" s="32" t="str">
         <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G39" s="32" t="str">
-        <x:v>Direct parent keeps the node focused on the spend mode rather than on broad Taproot overview material.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="32" t="str">
-        <x:v>protocol.taptree</x:v>
+        <x:v>protocol.x-only-public-keys</x:v>
       </x:c>
       <x:c r="B40" s="32" t="str">
-        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="C40" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13388,7 +13537,7 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E40" s="32" t="str">
-        <x:v>The inclusion proof only makes sense after the learner understands the TapTree structure.</x:v>
+        <x:v>TapTweak operates on x-only public keys in the Taproot construction.</x:v>
       </x:c>
       <x:c r="F40" s="32" t="str">
         <x:v>source.optech-schnorr-taproot-workshop</x:v>
@@ -13399,10 +13548,10 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32" t="str">
-        <x:v>protocol.taptree</x:v>
+        <x:v>protocol.taptweak</x:v>
       </x:c>
       <x:c r="B41" s="32" t="str">
-        <x:v>protocol.huffman-optimized-taptrees</x:v>
+        <x:v>protocol.taproot-key-path-spends</x:v>
       </x:c>
       <x:c r="C41" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13411,21 +13560,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E41" s="32" t="str">
-        <x:v>Huffman optimization is a refinement of how TapTree leaves are arranged.</x:v>
+        <x:v>A key-path spend verifies against the tweaked Taproot output key, so learners need the tweak mechanism before the spending mode makes sense.</x:v>
       </x:c>
       <x:c r="F41" s="32" t="str">
         <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G41" s="32" t="str">
-        <x:v>Source-driven bridge edge.</x:v>
+        <x:v>Direct parent keeps the node focused on the spend mode rather than on broad Taproot overview material.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="32" t="str">
-        <x:v>protocol.softfork-hardfork</x:v>
+        <x:v>protocol.taptree</x:v>
       </x:c>
       <x:c r="B42" s="32" t="str">
-        <x:v>protocol.chain-split-risk</x:v>
+        <x:v>protocol.tapleaf-inclusion-proofs</x:v>
       </x:c>
       <x:c r="C42" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13434,21 +13583,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E42" s="32" t="str">
-        <x:v>Split risk is a downstream consequence of incompatible upgrade paths, so learners should understand the compatibility boundary first.</x:v>
+        <x:v>The inclusion proof only makes sense after the learner understands the TapTree structure.</x:v>
       </x:c>
       <x:c r="F42" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G42" s="32" t="str">
-        <x:v>Direct edge chosen over activation-history case studies because those are downstream examples, not prerequisites.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.taptree</x:v>
       </x:c>
       <x:c r="B43" s="32" t="str">
-        <x:v>protocol.tapscript</x:v>
+        <x:v>protocol.huffman-optimized-taptrees</x:v>
       </x:c>
       <x:c r="C43" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13457,21 +13606,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E43" s="32" t="str">
-        <x:v>Tapscript is a Taproot-specific script version, so learners need the Taproot spend context before its rule changes make sense.</x:v>
+        <x:v>Huffman optimization is a refinement of how TapTree leaves are arranged.</x:v>
       </x:c>
       <x:c r="F43" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G43" s="32" t="str">
-        <x:v>Direct edge keeps the node scoped to the Taproot family without collapsing it into a generic script refresher.</x:v>
+        <x:v>Source-driven bridge edge.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="32" t="str">
-        <x:v>custody.psbt</x:v>
+        <x:v>protocol.softfork-hardfork</x:v>
       </x:c>
       <x:c r="B44" s="32" t="str">
-        <x:v>dev.taproot-psbt-fields</x:v>
+        <x:v>protocol.chain-split-risk</x:v>
       </x:c>
       <x:c r="C44" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13480,13 +13629,13 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E44" s="32" t="str">
-        <x:v>Taproot PSBT fields extend the base PSBT container, so learners need the general workflow and field model before the Taproot additions make sense.</x:v>
+        <x:v>Split risk is a downstream consequence of incompatible upgrade paths, so learners should understand the compatibility boundary first.</x:v>
       </x:c>
       <x:c r="F44" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G44" s="32" t="str">
-        <x:v>Direct edge keeps the slice anchored on the generic PSBT exchange model rather than on a narrower implementation variant.</x:v>
+        <x:v>Direct edge chosen over activation-history case studies because those are downstream examples, not prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -13494,7 +13643,7 @@
         <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B45" s="32" t="str">
-        <x:v>dev.taproot-psbt-fields</x:v>
+        <x:v>protocol.tapscript</x:v>
       </x:c>
       <x:c r="C45" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13503,21 +13652,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E45" s="32" t="str">
-        <x:v>These fields carry Taproot-specific keys, scripts, and Merkle-path data, so learners need the Taproot spend model before the PSBT extensions are meaningful.</x:v>
+        <x:v>Tapscript is a Taproot-specific script version, so learners need the Taproot spend context before its rule changes make sense.</x:v>
       </x:c>
       <x:c r="F45" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G45" s="32" t="str">
-        <x:v>The direct dev.psbt-v2 edge was intentionally dropped because BIP371 applies to PSBTv0 and PSBTv2.</x:v>
+        <x:v>Direct edge keeps the node scoped to the Taproot family without collapsing it into a generic script refresher.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="32" t="str">
-        <x:v>protocol.softfork-hardfork</x:v>
+        <x:v>custody.psbt</x:v>
       </x:c>
       <x:c r="B46" s="32" t="str">
-        <x:v>protocol.accidental-confiscation</x:v>
+        <x:v>dev.taproot-psbt-fields</x:v>
       </x:c>
       <x:c r="C46" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13526,21 +13675,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E46" s="32" t="str">
-        <x:v>Accidental confiscation is a failure mode caused by new soft-fork restrictions, so learners need the soft-fork compatibility model before the risk is intelligible.</x:v>
+        <x:v>Taproot PSBT fields extend the base PSBT container, so learners need the general workflow and field model before the Taproot additions make sense.</x:v>
       </x:c>
       <x:c r="F46" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G46" s="32" t="str">
-        <x:v>Direct edge chosen over chain-split-risk and standardness-policy because those branches add context but are not required for the core failure mode.</x:v>
+        <x:v>Direct edge keeps the slice anchored on the generic PSBT exchange model rather than on a narrower implementation variant.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="32" t="str">
-        <x:v>protocol.fee-market</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B47" s="32" t="str">
-        <x:v>custody.coin-selection</x:v>
+        <x:v>dev.taproot-psbt-fields</x:v>
       </x:c>
       <x:c r="C47" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13549,21 +13698,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E47" s="32" t="str">
-        <x:v>Wallets choose different UTXO sets partly to minimize transaction size and fee cost, so fee pressure is a direct part of the concept.</x:v>
+        <x:v>These fields carry Taproot-specific keys, scripts, and Merkle-path data, so learners need the Taproot spend model before the PSBT extensions are meaningful.</x:v>
       </x:c>
       <x:c r="F47" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G47" s="32" t="str">
-        <x:v>Direct edge keeps the node connected to transaction-cost tradeoffs rather than only to wallet UX.</x:v>
+        <x:v>The direct dev.psbt-v2 edge was intentionally dropped because BIP371 applies to PSBTv0 and PSBTv2.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>protocol.softfork-hardfork</x:v>
       </x:c>
       <x:c r="B48" s="32" t="str">
-        <x:v>protocol.change-outputs</x:v>
+        <x:v>protocol.accidental-confiscation</x:v>
       </x:c>
       <x:c r="C48" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13572,21 +13721,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E48" s="32" t="str">
-        <x:v>Change is a specific kind of transaction output, so learners need the basic output and spendability model before the leftover-value pattern makes sense.</x:v>
+        <x:v>Accidental confiscation is a failure mode caused by new soft-fork restrictions, so learners need the soft-fork compatibility model before the risk is intelligible.</x:v>
       </x:c>
       <x:c r="F48" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G48" s="32" t="str">
-        <x:v>Direct edge keeps the node between raw output structure and the later wallet-decision branch.</x:v>
+        <x:v>Direct edge chosen over chain-split-risk and standardness-policy because those branches add context but are not required for the core failure mode.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>protocol.fee-market</x:v>
       </x:c>
       <x:c r="B49" s="32" t="str">
-        <x:v>dev.taproot-descriptors</x:v>
+        <x:v>custody.coin-selection</x:v>
       </x:c>
       <x:c r="C49" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13595,21 +13744,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E49" s="32" t="str">
-        <x:v>Taproot descriptors extend the general descriptor grammar, so learners need the base descriptor model before the tr() specialization makes sense.</x:v>
+        <x:v>Wallets choose different UTXO sets partly to minimize transaction size and fee cost, so fee pressure is a direct part of the concept.</x:v>
       </x:c>
       <x:c r="F49" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G49" s="32" t="str">
-        <x:v>Direct edge keeps the node scoped to descriptor structure instead of wallet import behavior.</x:v>
+        <x:v>Direct edge keeps the node connected to transaction-cost tradeoffs rather than only to wallet UX.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B50" s="32" t="str">
-        <x:v>dev.taproot-descriptors</x:v>
+        <x:v>protocol.change-outputs</x:v>
       </x:c>
       <x:c r="C50" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13618,21 +13767,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E50" s="32" t="str">
-        <x:v>The tr() descriptor exists specifically to encode P2TR outputs and optional Taproot script-path commitments, so learners need the Taproot output model first.</x:v>
+        <x:v>Change is a specific kind of transaction output, so learners need the basic output and spendability model before the leftover-value pattern makes sense.</x:v>
       </x:c>
       <x:c r="F50" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G50" s="32" t="str">
-        <x:v>Direct edge keeps the node grounded in Taproot output semantics rather than in generic descriptor syntax alone.</x:v>
+        <x:v>Direct edge keeps the node between raw output structure and the later wallet-decision branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="32" t="str">
-        <x:v>protocol.transaction-pinning</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B51" s="32" t="str">
-        <x:v>protocol.version-3-transaction-relay</x:v>
+        <x:v>dev.taproot-descriptors</x:v>
       </x:c>
       <x:c r="C51" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13641,21 +13790,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E51" s="32" t="str">
-        <x:v>Version 3 relay is a targeted policy response to transaction pinning, so learners should understand the attack class before the mitigation.</x:v>
+        <x:v>Taproot descriptors extend the general descriptor grammar, so learners need the base descriptor model before the tr() specialization makes sense.</x:v>
       </x:c>
       <x:c r="F51" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G51" s="32" t="str">
-        <x:v>Direct edge chosen over package-relay because the pinning problem is the narrower immediate teaching need.</x:v>
+        <x:v>Direct edge keeps the node scoped to descriptor structure instead of wallet import behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="32" t="str">
-        <x:v>fundamentals.trustlessness</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B52" s="32" t="str">
-        <x:v>fundamentals.validation-sovereignty</x:v>
+        <x:v>dev.taproot-descriptors</x:v>
       </x:c>
       <x:c r="C52" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13664,21 +13813,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E52" s="32" t="str">
-        <x:v>Validation sovereignty is an applied consequence of trustlessness and verification culture.</x:v>
+        <x:v>The tr() descriptor exists specifically to encode P2TR outputs and optional Taproot script-path commitments, so learners need the Taproot output model first.</x:v>
       </x:c>
       <x:c r="F52" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G52" s="32" t="str">
-        <x:v>Bridge edge inferred from philosophy sequencing.</x:v>
+        <x:v>Direct edge keeps the node grounded in Taproot output semantics rather than in generic descriptor syntax alone.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="32" t="str">
-        <x:v>ops.run-full-node</x:v>
+        <x:v>protocol.transaction-pinning</x:v>
       </x:c>
       <x:c r="B53" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>protocol.version-3-transaction-relay</x:v>
       </x:c>
       <x:c r="C53" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13687,21 +13836,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E53" s="32" t="str">
-        <x:v>Learners need the full-node baseline before they can understand which validation guarantees a light client gives up.</x:v>
+        <x:v>Version 3 relay is a targeted policy response to transaction pinning, so learners should understand the attack class before the mitigation.</x:v>
       </x:c>
       <x:c r="F53" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G53" s="32" t="str">
-        <x:v>Bridge edge inferred from full-node versus lightweight-client contrast.</x:v>
+        <x:v>Direct edge chosen over package-relay because the pinning problem is the narrower immediate teaching need.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="32" t="str">
-        <x:v>protocol.compact-block-filters</x:v>
+        <x:v>fundamentals.trustlessness</x:v>
       </x:c>
       <x:c r="B54" s="32" t="str">
-        <x:v>protocol.light-client-trust-model</x:v>
+        <x:v>fundamentals.validation-sovereignty</x:v>
       </x:c>
       <x:c r="C54" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13710,21 +13859,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E54" s="32" t="str">
-        <x:v>Compact block filters provide the modern filtered-client mechanism that anchors the trust-model comparison.</x:v>
+        <x:v>Validation sovereignty is an applied consequence of trustlessness and verification culture.</x:v>
       </x:c>
       <x:c r="F54" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G54" s="32" t="str">
-        <x:v>Kept additive and conceptual instead of rewiring older light-client mechanism leaves in the same slice.</x:v>
+        <x:v>Bridge edge inferred from philosophy sequencing.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="32" t="str">
-        <x:v>fundamentals.validation-sovereignty</x:v>
+        <x:v>ops.run-full-node</x:v>
       </x:c>
       <x:c r="B55" s="32" t="str">
-        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="C55" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13733,21 +13882,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E55" s="32" t="str">
-        <x:v>The comparison only matters once the learner understands why self-validation is valuable in the first place.</x:v>
+        <x:v>Learners need the full-node baseline before they can understand which validation guarantees a light client gives up.</x:v>
       </x:c>
       <x:c r="F55" s="32" t="str">
-        <x:v>source.bitcoin-dev-philosophy</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G55" s="32" t="str">
-        <x:v>User-facing prerequisite edge for the wallet-mode decision.</x:v>
+        <x:v>Bridge edge inferred from full-node versus lightweight-client contrast.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="32" t="str">
+        <x:v>protocol.compact-block-filters</x:v>
+      </x:c>
+      <x:c r="B56" s="32" t="str">
         <x:v>protocol.light-client-trust-model</x:v>
-      </x:c>
-      <x:c r="B56" s="32" t="str">
-        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
       </x:c>
       <x:c r="C56" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13756,21 +13905,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E56" s="32" t="str">
-        <x:v>Learners need the mechanism-level trust tradeoffs before comparing full-node wallets with lightweight clients.</x:v>
+        <x:v>Compact block filters provide the modern filtered-client mechanism that anchors the trust-model comparison.</x:v>
       </x:c>
       <x:c r="F56" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G56" s="32" t="str">
-        <x:v>First downstream consumer for the light-client trust branch.</x:v>
+        <x:v>Kept additive and conceptual instead of rewiring older light-client mechanism leaves in the same slice.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>fundamentals.validation-sovereignty</x:v>
       </x:c>
       <x:c r="B57" s="32" t="str">
-        <x:v>protocol.p2pk</x:v>
+        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
       </x:c>
       <x:c r="C57" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13779,21 +13928,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E57" s="32" t="str">
-        <x:v>P2PK is a concrete legacy script template, so learners first need the locking and unlocking model from Bitcoin Script.</x:v>
+        <x:v>The comparison only matters once the learner understands why self-validation is valuable in the first place.</x:v>
       </x:c>
       <x:c r="F57" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-dev-philosophy</x:v>
       </x:c>
       <x:c r="G57" s="32" t="str">
-        <x:v>Chosen as the first script-history leaf from Decoding after dedupe and direct-edge review.</x:v>
+        <x:v>User-facing prerequisite edge for the wallet-mode decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="32" t="str">
-        <x:v>fundamentals.schnorr-signatures</x:v>
+        <x:v>protocol.light-client-trust-model</x:v>
       </x:c>
       <x:c r="B58" s="32" t="str">
-        <x:v>security.nonce-reuse-attack</x:v>
+        <x:v>ops.full-node-vs-lightweight-wallet</x:v>
       </x:c>
       <x:c r="C58" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13802,21 +13951,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E58" s="32" t="str">
-        <x:v>The nonce-reuse failure only makes sense after the learner understands the Schnorr signing flow that produces the nonce and signature pair.</x:v>
+        <x:v>Learners need the mechanism-level trust tradeoffs before comparing full-node wallets with lightweight clients.</x:v>
       </x:c>
       <x:c r="F58" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G58" s="32" t="str">
-        <x:v>Chosen as a narrow additive security slice without bundling it to custody-side defenses.</x:v>
+        <x:v>First downstream consumer for the light-client trust branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="32" t="str">
+        <x:v>protocol.script</x:v>
+      </x:c>
+      <x:c r="B59" s="32" t="str">
         <x:v>protocol.p2pk</x:v>
-      </x:c>
-      <x:c r="B59" s="32" t="str">
-        <x:v>protocol.p2pkh</x:v>
       </x:c>
       <x:c r="C59" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13825,21 +13974,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E59" s="32" t="str">
-        <x:v>P2PKH is easiest to understand as the hashed-public-key refinement of a direct public-key output.</x:v>
+        <x:v>P2PK is a concrete legacy script template, so learners first need the locking and unlocking model from Bitcoin Script.</x:v>
       </x:c>
       <x:c r="F59" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G59" s="32" t="str">
-        <x:v>Chosen to preserve the output-template ladder without repeating the broader Script prerequisite directly.</x:v>
+        <x:v>Chosen as the first script-history leaf from Decoding after dedupe and direct-edge review.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="32" t="str">
-        <x:v>fundamentals.hash-functions</x:v>
+        <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="B60" s="32" t="str">
-        <x:v>protocol.p2pkh</x:v>
+        <x:v>security.nonce-reuse-attack</x:v>
       </x:c>
       <x:c r="C60" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13848,21 +13997,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E60" s="32" t="str">
-        <x:v>Hash-based locking only makes sense once the learner understands what a hash commits to and why it can stand in for the public key until spend time.</x:v>
+        <x:v>The nonce-reuse failure only makes sense after the learner understands the Schnorr signing flow that produces the nonce and signature pair.</x:v>
       </x:c>
       <x:c r="F60" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G60" s="32" t="str">
-        <x:v>Required to keep the node about public-key hashing rather than just script syntax.</x:v>
+        <x:v>Chosen as a narrow additive security slice without bundling it to custody-side defenses.</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>protocol.p2pk</x:v>
       </x:c>
       <x:c r="B61" s="32" t="str">
-        <x:v>protocol.op-checkmultisig</x:v>
+        <x:v>protocol.p2pkh</x:v>
       </x:c>
       <x:c r="C61" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13871,21 +14020,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E61" s="32" t="str">
-        <x:v>OP_CHECKMULTISIG is an opcode-level script mechanic, so learners first need the general Script model and stack execution basics.</x:v>
+        <x:v>P2PKH is easiest to understand as the hashed-public-key refinement of a direct public-key output.</x:v>
       </x:c>
       <x:c r="F61" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G61" s="32" t="str">
-        <x:v>Chosen as the mechanism bridge before protocol.p2ms.</x:v>
+        <x:v>Chosen to preserve the output-template ladder without repeating the broader Script prerequisite directly.</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="32" t="str">
-        <x:v>protocol.op-checkmultisig</x:v>
+        <x:v>fundamentals.hash-functions</x:v>
       </x:c>
       <x:c r="B62" s="32" t="str">
-        <x:v>protocol.p2ms</x:v>
+        <x:v>protocol.p2pkh</x:v>
       </x:c>
       <x:c r="C62" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13894,21 +14043,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E62" s="32" t="str">
-        <x:v>Bare multisig is the concrete locking template built from OP_CHECKMULTISIG, so the opcode is the clean direct parent once introduced.</x:v>
+        <x:v>Hash-based locking only makes sense once the learner understands what a hash commits to and why it can stand in for the public key until spend time.</x:v>
       </x:c>
       <x:c r="F62" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G62" s="32" t="str">
-        <x:v>Replaces the earlier curricular and wallet-semantic parent candidates.</x:v>
+        <x:v>Required to keep the node about public-key hashing rather than just script syntax.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="32" t="str">
-        <x:v>protocol.p2ms</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B63" s="32" t="str">
-        <x:v>protocol.bare-multisig-standardness</x:v>
+        <x:v>protocol.op-checkmultisig</x:v>
       </x:c>
       <x:c r="C63" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13917,21 +14066,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E63" s="32" t="str">
-        <x:v>The relay treatment only makes sense once the learner understands what a bare multisig output actually is on-chain.</x:v>
+        <x:v>OP_CHECKMULTISIG is an opcode-level script mechanic, so learners first need the general Script model and stack execution basics.</x:v>
       </x:c>
       <x:c r="F63" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G63" s="32" t="str">
-        <x:v>Policy leaf anchored on the specific legacy script template it constrains.</x:v>
+        <x:v>Chosen as the mechanism bridge before protocol.p2ms.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="32" t="str">
-        <x:v>protocol.standardness-policy</x:v>
+        <x:v>protocol.op-checkmultisig</x:v>
       </x:c>
       <x:c r="B64" s="32" t="str">
-        <x:v>protocol.bare-multisig-standardness</x:v>
+        <x:v>protocol.p2ms</x:v>
       </x:c>
       <x:c r="C64" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13940,21 +14089,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E64" s="32" t="str">
-        <x:v>This node is a concrete application of standard transaction policy, so the general standardness concept should come first.</x:v>
+        <x:v>Bare multisig is the concrete locking template built from OP_CHECKMULTISIG, so the opcode is the clean direct parent once introduced.</x:v>
       </x:c>
       <x:c r="F64" s="32" t="str">
         <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G64" s="32" t="str">
-        <x:v>Policy-boundary prerequisite inherited through the existing mempool-policy branch.</x:v>
+        <x:v>Replaces the earlier curricular and wallet-semantic parent candidates.</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>protocol.p2ms</x:v>
       </x:c>
       <x:c r="B65" s="32" t="str">
-        <x:v>dev.scriptpubkeymanagers</x:v>
+        <x:v>protocol.bare-multisig-standardness</x:v>
       </x:c>
       <x:c r="C65" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13963,21 +14112,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E65" s="32" t="str">
-        <x:v>Modern descriptor wallets hand descriptor-backed script templates to dedicated managers, so learners need the descriptor model before the SPKM boundary makes sense.</x:v>
+        <x:v>The relay treatment only makes sense once the learner understands what a bare multisig output actually is on-chain.</x:v>
       </x:c>
       <x:c r="F65" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-wallet</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G65" s="32" t="str">
-        <x:v>Direct edge distinguishes the Core wallet abstraction from descriptor syntax without collapsing the two concepts into one node.</x:v>
+        <x:v>Policy leaf anchored on the specific legacy script template it constrains.</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="32" t="str">
-        <x:v>protocol.mempool</x:v>
+        <x:v>protocol.standardness-policy</x:v>
       </x:c>
       <x:c r="B66" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>protocol.bare-multisig-standardness</x:v>
       </x:c>
       <x:c r="C66" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -13986,21 +14135,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E66" s="32" t="str">
-        <x:v>The unbroadcast set is a mempool-owned data structure, so learners need the local unconfirmed transaction pool model before this narrower tracking mechanism makes sense.</x:v>
+        <x:v>This node is a concrete application of standard transaction policy, so the general standardness concept should come first.</x:v>
       </x:c>
       <x:c r="F66" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G66" s="32" t="str">
-        <x:v>Direct edge keeps the concept scoped to local transaction state rather than broader relay policy.</x:v>
+        <x:v>Policy-boundary prerequisite inherited through the existing mempool-policy branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="32" t="str">
-        <x:v>protocol.transaction-relay-inv-getdata</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B67" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>dev.scriptpubkeymanagers</x:v>
       </x:c>
       <x:c r="C67" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14009,21 +14158,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E67" s="32" t="str">
-        <x:v>This set only matters because nodes need to distinguish locally submitted transactions from those later observed through the network relay path and may retry announcing them.</x:v>
+        <x:v>Modern descriptor wallets hand descriptor-backed script templates to dedicated managers, so learners need the descriptor model before the SPKM boundary makes sense.</x:v>
       </x:c>
       <x:c r="F67" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-core-academy-wallet</x:v>
       </x:c>
       <x:c r="G67" s="32" t="str">
-        <x:v>Direct edge ties the mechanism to network propagation confirmation and rebroadcast attempts.</x:v>
+        <x:v>Direct edge distinguishes the Core wallet abstraction from descriptor syntax without collapsing the two concepts into one node.</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="32" t="str">
-        <x:v>privacy.address-reuse</x:v>
+        <x:v>protocol.mempool</x:v>
       </x:c>
       <x:c r="B68" s="32" t="str">
-        <x:v>custody.human-readable-addresses</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="C68" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14032,21 +14181,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E68" s="32" t="str">
-        <x:v>A major design constraint is that reusable human-readable handles can worsen privacy unless they resolve to reusable payment mechanisms or rotate safely, so learners need the address-reuse problem first.</x:v>
+        <x:v>The unbroadcast set is a mempool-owned data structure, so learners need the local unconfirmed transaction pool model before this narrower tracking mechanism makes sense.</x:v>
       </x:c>
       <x:c r="F68" s="32" t="str">
-        <x:v>source.bitcoin-design-payment-formats</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G68" s="32" t="str">
-        <x:v>Direct edge captures the main privacy tradeoff without forcing downstream protocol-specific address schemes into prerequisites.</x:v>
+        <x:v>Direct edge keeps the concept scoped to local transaction state rather than broader relay policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="32" t="str">
-        <x:v>custody.output-labeling</x:v>
+        <x:v>protocol.transaction-relay-inv-getdata</x:v>
       </x:c>
       <x:c r="B69" s="32" t="str">
-        <x:v>custody.transaction-metadata</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="C69" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14055,21 +14204,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E69" s="32" t="str">
-        <x:v>Output labeling already introduces the idea that wallets attach their own context to payments and spendable objects, making it the cleanest direct bridge into broader transaction-level notes, contacts, and portability concerns.</x:v>
+        <x:v>This set only matters because nodes need to distinguish locally submitted transactions from those later observed through the network relay path and may retry announcing them.</x:v>
       </x:c>
       <x:c r="F69" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G69" s="32" t="str">
-        <x:v>Direct edge distinguishes wider payment-history context from narrower spend-control labels without treating them as unrelated.</x:v>
+        <x:v>Direct edge ties the mechanism to network propagation confirmation and rebroadcast attempts.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>privacy.address-reuse</x:v>
       </x:c>
       <x:c r="B70" s="32" t="str">
-        <x:v>custody.transaction-metadata</x:v>
+        <x:v>custody.human-readable-addresses</x:v>
       </x:c>
       <x:c r="C70" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14078,21 +14227,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E70" s="32" t="str">
-        <x:v>Wallet-added names, notes, and contact links matter partly because transaction history is only pseudonymous and can reveal meaningful patterns when users or tools correlate activity over time.</x:v>
+        <x:v>A major design constraint is that reusable human-readable handles can worsen privacy unless they resolve to reusable payment mechanisms or rotate safely, so learners need the address-reuse problem first.</x:v>
       </x:c>
       <x:c r="F70" s="32" t="str">
-        <x:v>source.bitcoin-design-wallet-activity</x:v>
+        <x:v>source.bitcoin-design-payment-formats</x:v>
       </x:c>
       <x:c r="G70" s="32" t="str">
-        <x:v>Direct edge keeps the node tied to the privacy and identity meaning of payment history rather than only to generic lifecycle sequencing.</x:v>
+        <x:v>Direct edge captures the main privacy tradeoff without forcing downstream protocol-specific address schemes into prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="32" t="str">
-        <x:v>custody.self-custody</x:v>
+        <x:v>custody.output-labeling</x:v>
       </x:c>
       <x:c r="B71" s="32" t="str">
-        <x:v>custody.multiple-wallets</x:v>
+        <x:v>custody.transaction-metadata</x:v>
       </x:c>
       <x:c r="C71" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14101,21 +14250,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E71" s="32" t="str">
-        <x:v>Deliberately separating funds across different wallet buckets is a custody decision, so learners need the base self-custody responsibility model before the organizational pattern makes sense.</x:v>
+        <x:v>Output labeling already introduces the idea that wallets attach their own context to payments and spendable objects, making it the cleanest direct bridge into broader transaction-level notes, contacts, and portability concerns.</x:v>
       </x:c>
       <x:c r="F71" s="32" t="str">
-        <x:v>source.bitcoin-design-multiple-wallets</x:v>
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="G71" s="32" t="str">
-        <x:v>Kept the direct parent at the responsibility-model layer; multisig, watch-only, and HD account structures remain examples or implementation details rather than prerequisites.</x:v>
+        <x:v>Direct edge distinguishes wider payment-history context from narrower spend-control labels without treating them as unrelated.</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="32" t="str">
-        <x:v>custody.hardware-wallets</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B72" s="32" t="str">
-        <x:v>custody.progressive-security</x:v>
+        <x:v>custody.transaction-metadata</x:v>
       </x:c>
       <x:c r="C72" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14124,21 +14273,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E72" s="32" t="str">
-        <x:v>One of the core upgrade steps in the reference design is moving from default low-friction storage to an external signing device, so learners need the hardware-signing model before the staged-upgrade pattern makes sense.</x:v>
+        <x:v>Wallet-added names, notes, and contact links matter partly because transaction history is only pseudonymous and can reveal meaningful patterns when users or tools correlate activity over time.</x:v>
       </x:c>
       <x:c r="F72" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoin-design-wallet-activity</x:v>
       </x:c>
       <x:c r="G72" s="32" t="str">
-        <x:v>Direct edge captures the mid-tier upgrade target without treating cloud backup itself as the core concept.</x:v>
+        <x:v>Direct edge keeps the node tied to the privacy and identity meaning of payment history rather than only to generic lifecycle sequencing.</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>custody.self-custody</x:v>
       </x:c>
       <x:c r="B73" s="32" t="str">
-        <x:v>custody.progressive-security</x:v>
+        <x:v>custody.multiple-wallets</x:v>
       </x:c>
       <x:c r="C73" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14147,21 +14296,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E73" s="32" t="str">
-        <x:v>The higher-security end of the progression moves into 2-of-3 and 3-of-5 multi-key schemes, so learners need the multisig model before they can reason about why and when a wallet should escalate there.</x:v>
+        <x:v>Deliberately separating funds across different wallet buckets is a custody decision, so learners need the base self-custody responsibility model before the organizational pattern makes sense.</x:v>
       </x:c>
       <x:c r="F73" s="32" t="str">
-        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
+        <x:v>source.bitcoin-design-multiple-wallets</x:v>
       </x:c>
       <x:c r="G73" s="32" t="str">
-        <x:v>Direct edge captures the high-assurance destination of the progression rather than a specific product flow.</x:v>
+        <x:v>Kept the direct parent at the responsibility-model layer; multisig, watch-only, and HD account structures remain examples or implementation details rather than prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="32" t="str">
-        <x:v>protocol.mempool-unbroadcast-set</x:v>
+        <x:v>custody.hardware-wallets</x:v>
       </x:c>
       <x:c r="B74" s="32" t="str">
-        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
+        <x:v>custody.progressive-security</x:v>
       </x:c>
       <x:c r="C74" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14170,21 +14319,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E74" s="32" t="str">
-        <x:v>Rebroadcast privacy builds directly on the local-node distinction between transactions merely accepted into the mempool and transactions known to have propagated, which is exactly the gap the unbroadcast set tracks.</x:v>
+        <x:v>One of the core upgrade steps in the reference design is moving from default low-friction storage to an external signing device, so learners need the hardware-signing model before the staged-upgrade pattern makes sense.</x:v>
       </x:c>
       <x:c r="F74" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="G74" s="32" t="str">
-        <x:v>Direct parent keeps the slice on the local tracking mechanism rather than reintroducing generic relay ancestors.</x:v>
+        <x:v>Direct edge captures the mid-tier upgrade target without treating cloud backup itself as the core concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="32" t="str">
-        <x:v>privacy.pseudonymity</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B75" s="32" t="str">
-        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
+        <x:v>custody.progressive-security</x:v>
       </x:c>
       <x:c r="C75" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14193,21 +14342,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E75" s="32" t="str">
-        <x:v>Different rebroadcast patterns matter because observers can correlate network behavior with public transaction history and infer likely origin, so learners need the pseudonymity and linkage problem first.</x:v>
+        <x:v>The higher-security end of the progression moves into 2-of-3 and 3-of-5 multi-key schemes, so learners need the multisig model before they can reason about why and when a wallet should escalate there.</x:v>
       </x:c>
       <x:c r="F75" s="32" t="str">
-        <x:v>source.bitcoin-core-academy-mempool</x:v>
+        <x:v>source.bitcoin-design-upgradeable-wallet</x:v>
       </x:c>
       <x:c r="G75" s="32" t="str">
-        <x:v>Direct parent keeps the node focused on why relay-side origin leakage matters, not just how rebroadcast code works.</x:v>
+        <x:v>Direct edge captures the high-assurance destination of the progression rather than a specific product flow.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="32" t="str">
-        <x:v>protocol.segregated-witness</x:v>
+        <x:v>protocol.mempool-unbroadcast-set</x:v>
       </x:c>
       <x:c r="B76" s="32" t="str">
-        <x:v>protocol.txid-vs-wtxid</x:v>
+        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
       </x:c>
       <x:c r="C76" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14216,21 +14365,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E76" s="32" t="str">
-        <x:v>The identifier split only exists because SegWit introduces a witness-inclusive serialization alongside the legacy serialization, so learners need the SegWit structure change before the two IDs make sense.</x:v>
+        <x:v>Rebroadcast privacy builds directly on the local-node distinction between transactions merely accepted into the mempool and transactions known to have propagated, which is exactly the gap the unbroadcast set tracks.</x:v>
       </x:c>
       <x:c r="F76" s="32" t="str">
         <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G76" s="32" t="str">
-        <x:v>Direct parent keeps the bridge on the serialization distinction instead of reintroducing downstream relay consequences.</x:v>
+        <x:v>Direct parent keeps the slice on the local tracking mechanism rather than reintroducing generic relay ancestors.</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="32" t="str">
-        <x:v>protocol.txid-vs-wtxid</x:v>
+        <x:v>privacy.pseudonymity</x:v>
       </x:c>
       <x:c r="B77" s="32" t="str">
-        <x:v>protocol.wtxid-relay-bip339</x:v>
+        <x:v>protocol.transaction-rebroadcast-privacy</x:v>
       </x:c>
       <x:c r="C77" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14239,21 +14388,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E77" s="32" t="str">
-        <x:v>WTXID relay is specifically the choice to announce and request witness-bearing transactions by wtxid instead of txid, so the learner should understand the two identifier forms before the relay mode change.</x:v>
+        <x:v>Different rebroadcast patterns matter because observers can correlate network behavior with public transaction history and infer likely origin, so learners need the pseudonymity and linkage problem first.</x:v>
       </x:c>
       <x:c r="F77" s="32" t="str">
         <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G77" s="32" t="str">
-        <x:v>Added as a graph bridge so the existing relay node no longer has to explain the identifier distinction internally.</x:v>
+        <x:v>Direct parent keeps the node focused on why relay-side origin leakage matters, not just how rebroadcast code works.</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="32" t="str">
-        <x:v>fundamentals.schnorr-signatures</x:v>
+        <x:v>protocol.segregated-witness</x:v>
       </x:c>
       <x:c r="B78" s="32" t="str">
-        <x:v>protocol.musig</x:v>
+        <x:v>protocol.txid-vs-wtxid</x:v>
       </x:c>
       <x:c r="C78" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14262,21 +14411,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E78" s="32" t="str">
-        <x:v>MuSig is a Schnorr aggregation protocol, so learners need the underlying Schnorr key and signature model before the combined-key protocol makes sense.</x:v>
+        <x:v>The identifier split only exists because SegWit introduces a witness-inclusive serialization alongside the legacy serialization, so learners need the SegWit structure change before the two IDs make sense.</x:v>
       </x:c>
       <x:c r="F78" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G78" s="32" t="str">
-        <x:v>Direct parent kept narrow; wallet-level multisig and Taproot remain context rather than prerequisites.</x:v>
+        <x:v>Direct parent keeps the bridge on the serialization distinction instead of reintroducing downstream relay consequences.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="32" t="str">
-        <x:v>dev.descriptors</x:v>
+        <x:v>protocol.txid-vs-wtxid</x:v>
       </x:c>
       <x:c r="B79" s="32" t="str">
-        <x:v>dev.descriptor-wallet-policies</x:v>
+        <x:v>protocol.wtxid-relay-bip339</x:v>
       </x:c>
       <x:c r="C79" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14285,21 +14434,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E79" s="32" t="str">
-        <x:v>Wallet policies are built as descriptor templates, so the base descriptor language and template structure must come first.</x:v>
+        <x:v>WTXID relay is specifically the choice to announce and request witness-bearing transactions by wtxid instead of txid, so the learner should understand the two identifier forms before the relay mode change.</x:v>
       </x:c>
       <x:c r="F79" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoin-core-academy-mempool</x:v>
       </x:c>
       <x:c r="G79" s="32" t="str">
-        <x:v>Direct parent kept above import or signer flows because the node is about the representation itself.</x:v>
+        <x:v>Added as a graph bridge so the existing relay node no longer has to explain the identifier distinction internally.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="32" t="str">
-        <x:v>dev.bip32</x:v>
+        <x:v>fundamentals.schnorr-signatures</x:v>
       </x:c>
       <x:c r="B80" s="32" t="str">
-        <x:v>dev.descriptor-wallet-policies</x:v>
+        <x:v>protocol.musig</x:v>
       </x:c>
       <x:c r="C80" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14308,13 +14457,13 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E80" s="32" t="str">
-        <x:v>BIP388 key information items package xpubs and derivation origins, so learners need the HD derivation model before the portable wallet-policy format makes sense.</x:v>
+        <x:v>MuSig is a Schnorr aggregation protocol, so learners need the underlying Schnorr key and signature model before the combined-key protocol makes sense.</x:v>
       </x:c>
       <x:c r="F80" s="32" t="str">
-        <x:v>source.bitcoinops-topics</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G80" s="32" t="str">
-        <x:v>Non-redundant alongside dev.descriptors because neither concept implies the other in the current graph.</x:v>
+        <x:v>Direct parent kept narrow; wallet-level multisig and Taproot remain context rather than prerequisites.</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -14322,7 +14471,7 @@
         <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B81" s="32" t="str">
-        <x:v>dev.descriptors-in-psbt</x:v>
+        <x:v>dev.descriptor-wallet-policies</x:v>
       </x:c>
       <x:c r="C81" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14331,21 +14480,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E81" s="32" t="str">
-        <x:v>The node is about carrying descriptor information during transaction coordination, so learners need the descriptor syntax and script-template model first.</x:v>
+        <x:v>Wallet policies are built as descriptor templates, so the base descriptor language and template structure must come first.</x:v>
       </x:c>
       <x:c r="F81" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G81" s="32" t="str">
-        <x:v>Direct parent kept at the representation layer rather than the wallet-policy or taproot-specific refinements.</x:v>
+        <x:v>Direct parent kept above import or signer flows because the node is about the representation itself.</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="32" t="str">
-        <x:v>custody.psbt</x:v>
+        <x:v>dev.bip32</x:v>
       </x:c>
       <x:c r="B82" s="32" t="str">
-        <x:v>dev.descriptors-in-psbt</x:v>
+        <x:v>dev.descriptor-wallet-policies</x:v>
       </x:c>
       <x:c r="C82" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14354,21 +14503,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E82" s="32" t="str">
-        <x:v>Descriptor-aware exchange only makes sense after the learner understands the general PSBT coordination workflow that transports signing-related data between tools.</x:v>
+        <x:v>BIP388 key information items package xpubs and derivation origins, so learners need the HD derivation model before the portable wallet-policy format makes sense.</x:v>
       </x:c>
       <x:c r="F82" s="32" t="str">
         <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G82" s="32" t="str">
-        <x:v>Direct parent kept at the base PSBT workflow level instead of requiring later version-specific extensions.</x:v>
+        <x:v>Non-redundant alongside dev.descriptors because neither concept implies the other in the current graph.</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>dev.descriptors</x:v>
       </x:c>
       <x:c r="B83" s="32" t="str">
-        <x:v>custody.degrading-multisig</x:v>
+        <x:v>dev.descriptors-in-psbt</x:v>
       </x:c>
       <x:c r="C83" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14377,21 +14526,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E83" s="32" t="str">
-        <x:v>The policy only makes sense once the learner understands ordinary multisig threshold custody and why signers can be split into live and backup sets.</x:v>
+        <x:v>The node is about carrying descriptor information during transaction coordination, so learners need the descriptor syntax and script-template model first.</x:v>
       </x:c>
       <x:c r="F83" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G83" s="32" t="str">
-        <x:v>Direct custody parent for the signer-threshold side of the construction.</x:v>
+        <x:v>Direct parent kept at the representation layer rather than the wallet-policy or taproot-specific refinements.</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="32" t="str">
-        <x:v>protocol.timelocks</x:v>
+        <x:v>custody.psbt</x:v>
       </x:c>
       <x:c r="B84" s="32" t="str">
-        <x:v>custody.degrading-multisig</x:v>
+        <x:v>dev.descriptors-in-psbt</x:v>
       </x:c>
       <x:c r="C84" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14400,21 +14549,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E84" s="32" t="str">
-        <x:v>The degrading policy activates its weaker backup path only after a timeout, so timelock semantics are a direct part of the construction.</x:v>
+        <x:v>Descriptor-aware exchange only makes sense after the learner understands the general PSBT coordination workflow that transports signing-related data between tools.</x:v>
       </x:c>
       <x:c r="F84" s="32" t="str">
-        <x:v>source.optech-schnorr-taproot-workshop</x:v>
+        <x:v>source.bitcoinops-topics</x:v>
       </x:c>
       <x:c r="G84" s="32" t="str">
-        <x:v>Needed alongside custody.multisig because the learner must understand the temporal rule, not just the signer policy.</x:v>
+        <x:v>Direct parent kept at the base PSBT workflow level instead of requiring later version-specific extensions.</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="32" t="str">
-        <x:v>protocol.block-weight-vbytes</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B85" s="32" t="str">
-        <x:v>protocol.fee-calculation</x:v>
+        <x:v>custody.degrading-multisig</x:v>
       </x:c>
       <x:c r="C85" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14423,21 +14572,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E85" s="32" t="str">
-        <x:v>Understanding whether an absolute fee is high or low requires relating it to the blockspace pricing unit, so learners need weight and virtual bytes before fee calculation is fully meaningful in practice.</x:v>
+        <x:v>The policy only makes sense once the learner understands ordinary multisig threshold custody and why signers can be split into live and backup sets.</x:v>
       </x:c>
       <x:c r="F85" s="32" t="str">
-        <x:v>source.bitcoindevs-decoding</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G85" s="32" t="str">
-        <x:v>Direct parent keeps the node at the mechanism layer without drifting into broader fee-market competition.</x:v>
+        <x:v>Direct custody parent for the signer-threshold side of the construction.</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>protocol.timelocks</x:v>
       </x:c>
       <x:c r="B86" s="32" t="str">
-        <x:v>protocol.bech32m-addresses</x:v>
+        <x:v>custody.degrading-multisig</x:v>
       </x:c>
       <x:c r="C86" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14446,21 +14595,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E86" s="32" t="str">
-        <x:v>Bech32m is an address-encoding format, so learners need the general relationship between addresses, script templates, and spendability before the newer checksum format is meaningful.</x:v>
+        <x:v>The degrading policy activates its weaker backup path only after a timeout, so timelock semantics are a direct part of the construction.</x:v>
       </x:c>
       <x:c r="F86" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.optech-schnorr-taproot-workshop</x:v>
       </x:c>
       <x:c r="G86" s="32" t="str">
-        <x:v>Direct parent keeps the node on encoding semantics rather than on raw string-format trivia.</x:v>
+        <x:v>Needed alongside custody.multisig because the learner must understand the temporal rule, not just the signer policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="32" t="str">
-        <x:v>protocol.taproot</x:v>
+        <x:v>protocol.block-weight-vbytes</x:v>
       </x:c>
       <x:c r="B87" s="32" t="str">
-        <x:v>protocol.bech32m-addresses</x:v>
+        <x:v>protocol.fee-calculation</x:v>
       </x:c>
       <x:c r="C87" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14469,21 +14618,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E87" s="32" t="str">
-        <x:v>Bech32m became necessary for witness version 1 and higher, and Taproot is the first major deployed witness-v1 use case, so learners need that upgrade context before the format distinction makes sense.</x:v>
+        <x:v>Understanding whether an absolute fee is high or low requires relating it to the blockspace pricing unit, so learners need weight and virtual bytes before fee calculation is fully meaningful in practice.</x:v>
       </x:c>
       <x:c r="F87" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.bitcoindevs-decoding</x:v>
       </x:c>
       <x:c r="G87" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored on the practical protocol transition that exposed Bech32m to users.</x:v>
+        <x:v>Direct parent keeps the node at the mechanism layer without drifting into broader fee-market competition.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="32" t="str">
-        <x:v>protocol.script</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B88" s="32" t="str">
-        <x:v>protocol.script-execution-stack</x:v>
+        <x:v>protocol.bech32m-addresses</x:v>
       </x:c>
       <x:c r="C88" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14492,21 +14641,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E88" s="32" t="str">
-        <x:v>The stack execution model is the direct mechanism by which Bitcoin Script evaluates spending conditions, so learners need the umbrella Script concept before drilling into stack behavior.</x:v>
+        <x:v>Bech32m is an address-encoding format, so learners need the general relationship between addresses, script templates, and spendability before the newer checksum format is meaningful.</x:v>
       </x:c>
       <x:c r="F88" s="32" t="str">
         <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G88" s="32" t="str">
-        <x:v>Direct parent positions the node as the conceptual middle layer between Script and opcode-specific leaves.</x:v>
+        <x:v>Direct parent keeps the node on encoding semantics rather than on raw string-format trivia.</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="32" t="str">
-        <x:v>lightning.commitment-transactions</x:v>
+        <x:v>protocol.taproot</x:v>
       </x:c>
       <x:c r="B89" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>protocol.bech32m-addresses</x:v>
       </x:c>
       <x:c r="C89" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14515,21 +14664,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E89" s="32" t="str">
-        <x:v>Per-commitment secrets are generated for each new commitment state, so learners need the commitment-transaction model before the secret-rotation mechanism makes sense.</x:v>
+        <x:v>Bech32m became necessary for witness version 1 and higher, and Taproot is the first major deployed witness-v1 use case, so learners need that upgrade context before the format distinction makes sense.</x:v>
       </x:c>
       <x:c r="F89" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G89" s="32" t="str">
-        <x:v>Direct parent keeps the node on state evolution rather than on later punishment or watchtower behavior.</x:v>
+        <x:v>Direct parent keeps the node anchored on the practical protocol transition that exposed Bech32m to users.</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="32" t="str">
-        <x:v>lightning.per-commitment-secrets</x:v>
+        <x:v>protocol.script</x:v>
       </x:c>
       <x:c r="B90" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>protocol.script-execution-stack</x:v>
       </x:c>
       <x:c r="C90" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14538,21 +14687,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E90" s="32" t="str">
-        <x:v>The to_local and to_remote scripts rely on per-state key derivation, revocation keys, and delayed-payment keys, so learners need the per-commitment secret machinery first.</x:v>
+        <x:v>The stack execution model is the direct mechanism by which Bitcoin Script evaluates spending conditions, so learners need the umbrella Script concept before drilling into stack behavior.</x:v>
       </x:c>
       <x:c r="F90" s="32" t="str">
-        <x:v>source.programming-lightning</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G90" s="32" t="str">
-        <x:v>Direct parent keeps the node at the commitment-key layer instead of collapsing back into the broader commitment-transaction overview.</x:v>
+        <x:v>Direct parent positions the node as the conceptual middle layer between Script and opcode-specific leaves.</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="32" t="str">
-        <x:v>protocol.csv-bip112</x:v>
+        <x:v>lightning.commitment-transactions</x:v>
       </x:c>
       <x:c r="B91" s="32" t="str">
-        <x:v>lightning.commitment-output-scripts</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="C91" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14561,21 +14710,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E91" s="32" t="str">
-        <x:v>The delayed to_local branch is defined by a CSV-enforced waiting period, so learners need the relative-timelock opcode before the script template makes sense.</x:v>
+        <x:v>Per-commitment secrets are generated for each new commitment state, so learners need the commitment-transaction model before the secret-rotation mechanism makes sense.</x:v>
       </x:c>
       <x:c r="F91" s="32" t="str">
         <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G91" s="32" t="str">
-        <x:v>Direct parent captures the script-mechanism side of the concept without dragging in broader force-close or HTLC timing behavior.</x:v>
+        <x:v>Direct parent keeps the node on state evolution rather than on later punishment or watchtower behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="32" t="str">
-        <x:v>protocol.difficulty-adjustment</x:v>
+        <x:v>lightning.per-commitment-secrets</x:v>
       </x:c>
       <x:c r="B92" s="32" t="str">
-        <x:v>protocol.time-warp-attack</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="C92" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14584,21 +14733,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E92" s="32" t="str">
-        <x:v>The attack only makes sense once learners understand how Bitcoin retargets mining difficulty over long block windows.</x:v>
+        <x:v>The to_local and to_remote scripts rely on per-state key derivation, revocation keys, and delayed-payment keys, so learners need the per-commitment secret machinery first.</x:v>
       </x:c>
       <x:c r="F92" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G92" s="32" t="str">
-        <x:v>Direct parent keeps the exploit tied to the retarget mechanism instead of burying it under generic mining vocabulary.</x:v>
+        <x:v>Direct parent keeps the node at the commitment-key layer instead of collapsing back into the broader commitment-transaction overview.</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="32" t="str">
-        <x:v>protocol.median-time-past</x:v>
+        <x:v>protocol.csv-bip112</x:v>
       </x:c>
       <x:c r="B93" s="32" t="str">
-        <x:v>protocol.time-warp-attack</x:v>
+        <x:v>lightning.commitment-output-scripts</x:v>
       </x:c>
       <x:c r="C93" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14607,21 +14756,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E93" s="32" t="str">
-        <x:v>Learners need the consensus timestamp constraints before they can reason about how miners manipulate time data and where the remaining attack surface lives.</x:v>
+        <x:v>The delayed to_local branch is defined by a CSV-enforced waiting period, so learners need the relative-timelock opcode before the script template makes sense.</x:v>
       </x:c>
       <x:c r="F93" s="32" t="str">
-        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
+        <x:v>source.programming-lightning</x:v>
       </x:c>
       <x:c r="G93" s="32" t="str">
-        <x:v>Direct parent captures the timestamp-boundary side of the exploit without overloading timelocks or block headers.</x:v>
+        <x:v>Direct parent captures the script-mechanism side of the concept without dragging in broader force-close or HTLC timing behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="32" t="str">
-        <x:v>fundamentals.blind-signatures</x:v>
+        <x:v>protocol.difficulty-adjustment</x:v>
       </x:c>
       <x:c r="B94" s="32" t="str">
-        <x:v>history.chaumian-ecash</x:v>
+        <x:v>protocol.time-warp-attack</x:v>
       </x:c>
       <x:c r="C94" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14630,21 +14779,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E94" s="32" t="str">
-        <x:v>Chaumian ecash is defined by using blind signatures to let a mint issue private bearer tokens without seeing the final token contents.</x:v>
+        <x:v>The attack only makes sense once learners understand how Bitcoin retargets mining difficulty over long block windows.</x:v>
       </x:c>
       <x:c r="F94" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G94" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the specific cryptographic mechanism rather than treating it as generic digital-money history.</x:v>
+        <x:v>Direct parent keeps the exploit tied to the retarget mechanism instead of burying it under generic mining vocabulary.</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="32" t="str">
-        <x:v>history.double-spend-problem</x:v>
+        <x:v>protocol.median-time-past</x:v>
       </x:c>
       <x:c r="B95" s="32" t="str">
-        <x:v>history.chaumian-ecash</x:v>
+        <x:v>protocol.time-warp-attack</x:v>
       </x:c>
       <x:c r="C95" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14653,21 +14802,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E95" s="32" t="str">
-        <x:v>Learners need the unsolved scarcity problem in digital cash before the trusted-mint tradeoff in Chaumian designs becomes meaningful.</x:v>
+        <x:v>Learners need the consensus timestamp constraints before they can reason about how miners manipulate time data and where the remaining attack surface lives.</x:v>
       </x:c>
       <x:c r="F95" s="32" t="str">
-        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
+        <x:v>source.bitcoin-dev-project-explained-posts</x:v>
       </x:c>
       <x:c r="G95" s="32" t="str">
-        <x:v>Direct parent frames why the system still needed a central operator even though it improved privacy.</x:v>
+        <x:v>Direct parent captures the timestamp-boundary side of the exploit without overloading timelocks or block headers.</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="32" t="str">
-        <x:v>economics.history-of-money</x:v>
+        <x:v>fundamentals.blind-signatures</x:v>
       </x:c>
       <x:c r="B96" s="32" t="str">
-        <x:v>privacy.secret-right-to-cash</x:v>
+        <x:v>history.chaumian-ecash</x:v>
       </x:c>
       <x:c r="C96" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14676,21 +14825,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E96" s="32" t="str">
-        <x:v>The concept depends on understanding how money moved from bearer cash toward mediated account systems, so learners need the long-run monetary history first.</x:v>
+        <x:v>Chaumian ecash is defined by using blind signatures to let a mint issue private bearer tokens without seeing the final token contents.</x:v>
       </x:c>
       <x:c r="F96" s="32" t="str">
         <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G96" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the bearer-versus-intermediated payment shift rather than drifting into generic civil-liberties framing.</x:v>
+        <x:v>Direct parent keeps the node tied to the specific cryptographic mechanism rather than treating it as generic digital-money history.</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="32" t="str">
-        <x:v>fundamentals.censorship-resistance</x:v>
+        <x:v>history.double-spend-problem</x:v>
       </x:c>
       <x:c r="B97" s="32" t="str">
-        <x:v>privacy.secret-right-to-cash</x:v>
+        <x:v>history.chaumian-ecash</x:v>
       </x:c>
       <x:c r="C97" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14699,21 +14848,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E97" s="32" t="str">
-        <x:v>Learners need the general idea that payment systems can exclude or block participants before the loss of private cash as a payment right becomes fully meaningful.</x:v>
+        <x:v>Learners need the unsolved scarcity problem in digital cash before the trusted-mint tradeoff in Chaumian designs becomes meaningful.</x:v>
       </x:c>
       <x:c r="F97" s="32" t="str">
         <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G97" s="32" t="str">
-        <x:v>Direct parent captures the exclusion-risk side of the argument without reopening broader compliance or surveillance wrappers.</x:v>
+        <x:v>Direct parent frames why the system still needed a central operator even though it improved privacy.</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="32" t="str">
-        <x:v>fundamentals.inflation</x:v>
+        <x:v>economics.history-of-money</x:v>
       </x:c>
       <x:c r="B98" s="32" t="str">
-        <x:v>economics.ideal-money</x:v>
+        <x:v>privacy.secret-right-to-cash</x:v>
       </x:c>
       <x:c r="C98" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14722,21 +14871,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E98" s="32" t="str">
-        <x:v>The concept is about minimizing monetary distortion, so learners need to understand how inflation changes purchasing power and price signals first.</x:v>
+        <x:v>The concept depends on understanding how money moved from bearer cash toward mediated account systems, so learners need the long-run monetary history first.</x:v>
       </x:c>
       <x:c r="F98" s="32" t="str">
         <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G98" s="32" t="str">
-        <x:v>Direct parent captures the measurement-distortion problem that ideal money is trying to avoid.</x:v>
+        <x:v>Direct parent keeps the node tied to the bearer-versus-intermediated payment shift rather than drifting into generic civil-liberties framing.</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="32" t="str">
-        <x:v>protocol.addresses-outputs</x:v>
+        <x:v>fundamentals.censorship-resistance</x:v>
       </x:c>
       <x:c r="B99" s="32" t="str">
-        <x:v>protocol.bitcoin-uri-bip21</x:v>
+        <x:v>privacy.secret-right-to-cash</x:v>
       </x:c>
       <x:c r="C99" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14745,21 +14894,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E99" s="32" t="str">
-        <x:v>The URI is a wrapper around a payment destination and amount, so learners need the underlying address and output model first.</x:v>
+        <x:v>Learners need the general idea that payment systems can exclude or block participants before the loss of private cash as a payment right becomes fully meaningful.</x:v>
       </x:c>
       <x:c r="F99" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G99" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the standard request format rather than collapsing it into higher-level wallet UX systems.</x:v>
+        <x:v>Direct parent captures the exclusion-risk side of the argument without reopening broader compliance or surveillance wrappers.</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="32" t="str">
-        <x:v>dev.bip32</x:v>
+        <x:v>fundamentals.inflation</x:v>
       </x:c>
       <x:c r="B100" s="32" t="str">
-        <x:v>dev.extended-keys</x:v>
+        <x:v>economics.ideal-money</x:v>
       </x:c>
       <x:c r="C100" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14768,21 +14917,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E100" s="32" t="str">
-        <x:v>Extended keys are one specific export and branch-derivation surface inside the broader BIP32 HD tree model, so learners need the base tree-derivation mechanics first.</x:v>
+        <x:v>The concept is about minimizing monetary distortion, so learners need to understand how inflation changes purchasing power and price signals first.</x:v>
       </x:c>
       <x:c r="F100" s="32" t="str">
-        <x:v>source.mastering-bitcoin-book-map</x:v>
+        <x:v>source.cypherpunk-library-bitcoin-adjacent</x:v>
       </x:c>
       <x:c r="G100" s="32" t="str">
-        <x:v>Direct parent keeps the node inside the HD derivation branch instead of treating xpub or xprv behavior as only a privacy or operational-wallet concept.</x:v>
+        <x:v>Direct parent captures the measurement-distortion problem that ideal money is trying to avoid.</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="32" t="str">
-        <x:v>dev.extended-keys</x:v>
+        <x:v>protocol.addresses-outputs</x:v>
       </x:c>
       <x:c r="B101" s="32" t="str">
-        <x:v>dev.hardened-keys</x:v>
+        <x:v>protocol.bitcoin-uri-bip21</x:v>
       </x:c>
       <x:c r="C101" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14791,21 +14940,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E101" s="32" t="str">
-        <x:v>Hardened derivation is a constraint on what an extended public key can derive and on how extended private and public key boundaries behave, so learners need the base xpub/xprv model first.</x:v>
+        <x:v>The URI is a wrapper around a payment destination and amount, so learners need the underlying address and output model first.</x:v>
       </x:c>
       <x:c r="F101" s="32" t="str">
         <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G101" s="32" t="str">
-        <x:v>Direct parent closes the previously missing branch-level bridge between BIP32 generally and hardened derivation specifically.</x:v>
+        <x:v>Direct parent keeps the node tied to the standard request format rather than collapsing it into higher-level wallet UX systems.</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="32" t="str">
-        <x:v>custody.multisig</x:v>
+        <x:v>dev.bip32</x:v>
       </x:c>
       <x:c r="B102" s="32" t="str">
-        <x:v>protocol.escrow-and-arbitration</x:v>
+        <x:v>dev.extended-keys</x:v>
       </x:c>
       <x:c r="C102" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14814,21 +14963,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E102" s="32" t="str">
-        <x:v>The escrow flow depends on understanding how multiple signers can authorize one spend and why a 2-of-3 threshold changes trust assumptions between buyer, seller, and arbitrator.</x:v>
+        <x:v>Extended keys are one specific export and branch-derivation surface inside the broader BIP32 HD tree model, so learners need the base tree-derivation mechanics first.</x:v>
       </x:c>
       <x:c r="F102" s="32" t="str">
-        <x:v>source.bitcoin-developer-guides</x:v>
+        <x:v>source.mastering-bitcoin-book-map</x:v>
       </x:c>
       <x:c r="G102" s="32" t="str">
-        <x:v>Direct parent keeps the node tied to the threshold-signing contract pattern instead of treating it as generic dispute-resolution theory.</x:v>
+        <x:v>Direct parent keeps the node inside the HD derivation branch instead of treating xpub or xprv behavior as only a privacy or operational-wallet concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="32" t="str">
-        <x:v>protocol.pay-to-script-hash</x:v>
+        <x:v>dev.extended-keys</x:v>
       </x:c>
       <x:c r="B103" s="32" t="str">
-        <x:v>protocol.escrow-and-arbitration</x:v>
+        <x:v>dev.hardened-keys</x:v>
       </x:c>
       <x:c r="C103" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14837,21 +14986,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E103" s="32" t="str">
-        <x:v>The contract uses a P2SH redeem script to hide the multisig spending conditions until spend time, so learners need the P2SH wrapper first.</x:v>
+        <x:v>Hardened derivation is a constraint on what an extended public key can derive and on how extended private and public key boundaries behave, so learners need the base xpub/xprv model first.</x:v>
       </x:c>
       <x:c r="F103" s="32" t="str">
         <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G103" s="32" t="str">
-        <x:v>Direct parent captures the on-chain contract packaging layer that makes the escrow pattern practical.</x:v>
+        <x:v>Direct parent closes the previously missing branch-level bridge between BIP32 generally and hardened derivation specifically.</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="32" t="str">
-        <x:v>fundamentals.public-private-keys</x:v>
+        <x:v>custody.multisig</x:v>
       </x:c>
       <x:c r="B104" s="32" t="str">
-        <x:v>dev.wallet-import-format-wif</x:v>
+        <x:v>protocol.escrow-and-arbitration</x:v>
       </x:c>
       <x:c r="C104" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14860,21 +15009,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E104" s="32" t="str">
-        <x:v>WIF is a serialization format for one private key, so learners need the underlying asymmetric-key concept before the network prefix, checksum, and compression flag details make sense.</x:v>
+        <x:v>The escrow flow depends on understanding how multiple signers can authorize one spend and why a 2-of-3 threshold changes trust assumptions between buyer, seller, and arbitrator.</x:v>
       </x:c>
       <x:c r="F104" s="32" t="str">
         <x:v>source.bitcoin-developer-guides</x:v>
       </x:c>
       <x:c r="G104" s="32" t="str">
-        <x:v>Direct parent keeps the node anchored on key material itself instead of overfitting it to address formats or HD wallet hierarchies.</x:v>
+        <x:v>Direct parent keeps the node tied to the threshold-signing contract pattern instead of treating it as generic dispute-resolution theory.</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="32" t="str">
-        <x:v>mining.pool-vs-solo</x:v>
+        <x:v>protocol.pay-to-script-hash</x:v>
       </x:c>
       <x:c r="B105" s="32" t="str">
-        <x:v>mining.pool-shares</x:v>
+        <x:v>protocol.escrow-and-arbitration</x:v>
       </x:c>
       <x:c r="C105" s="32" t="str">
         <x:v>prerequisite</x:v>
@@ -14883,21 +15032,21 @@
         <x:v>proposed</x:v>
       </x:c>
       <x:c r="E105" s="32" t="str">
-        <x:v>Pool shares only make sense after learners understand why pooled mining exists and why miners need a lower-variance way to prove contributed work before an actual block is found.</x:v>
+        <x:v>The contract uses a P2SH redeem script to hide the mult